<commit_message>
Auto update Combined.xlsx [Sun Sep 13 07:07:36 UTC 2026]
</commit_message>
<xml_diff>
--- a/output/Combined.xlsx
+++ b/output/Combined.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -467,48 +467,56 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Applications Invited for IMATA Conservation Fund</t>
+          <t>Application Invited For India Fund</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>About the Grant: 
-The International Marine Animal Trainers Association (IMATA) Conservation Fund was founded in 2011 to provide financial support for third-party non-profit organization projects focused on conservation-oriented issues, promoting communication, professionalism, and cooperation among those who serve marine mammal science through training, public display, research, husbandry, conservation, and education.
- Total Awarded to Date: $5,000 (cumulative across conservation projects)
- Previously Funded Projects (as in source document): 
-Marine Mammal Care Center, Manatee Rehabilitation Partnership, Pacific Marine Life Foundation, UNCW-Marine Mammal Stranding Program, Manatee Research, and Zoo to You.
- Goals 
-Make significant contributions towards marine mammal science conservation-oriented issues.
-Promote conservation efforts in the domestic and international marine animal community.
-Increase IMATA member awareness of supported issues.
-Promote the "IMATA Gives Back" philosophy.
-Expand IMATA's role and position in the conservation community.
-Increase the number of conservation-oriented IMATA members.
- Eligibility
-Applicant must be a third-party non-profit organization (not an individual).
-Project must promote communication, professionalism, and cooperation among those who serve marine mammal science through training, public display, research, husbandry, conservation, and/or education.
-Nominee must agree to IMATA's Terms of Acceptance, provide proof of the organization's non-profit status, a Statement of Organizational Support, and copies of required permits (if applicable).
- Review/Approval Process 
-The IMATA Research &amp; Conservation Committee's Conservation Fund Sub-Committee reviews all Nomination Applications for completeness and merit, making funding recommendations to the IMATA Board.
-The IMATA Board of Directors votes on whether and how much funding to award.
-Award amounts may be reduced from the requested amount to accommodate other awards or protect IMATA's fiscal solvency.
-Applicants/Project Managers notified of the Board's decision within 3 months of receiving the application.
-Award funds made available within 3 months of award notification.</t>
+          <t>About the Organization
+Paul Hamlyn Foundation was established in 1987. Since then, we have used our resources to work towards a just future in which everyone, especially young people, can realise their full potential and enjoy fulfilling and creative lives. In all of our work, including our grant-making, we are guided by six strategic priorities where we want to see change: • Investing in young people • Migration and integration • Arts access and participation • Education and learning through the arts • Nurturing ideas and people • Creating opportunities for people and communities in India
+ About the India Fund
+The India Fund supports small NGOs working with vulnerable communities in priority geographical areas of India.
+The fund is based on the principle that communities should be central to development work, with people facing disadvantage playing an important role in leading change and designing solutions to inequality.
+Strategic aims
+The fund aims to:
+Encourage NGOs to undertake community-centred development programmes.
+Enable communities to take greater control of their own development and improve their lives.
+Encourage development funding that addresses systemic change.
+Strengthen the capacity of organisations and people facilitating this work.
+ Who Can Apply?
+The fund specifically supports:
+Local Indian NGOs with FCRA registration
+This is an important eligibility requirement.
+Eligible organisations should generally be:
+Indian organisations
+Locally based in the communities they serve
+Working directly with communities
+Focused on long-term improvements in community wellbeing
+Connected with relevant panchayats in rural areas or municipalities in urban areas
+Taking steps to reduce their environmental impact
+Working to improve local ecology
+Promoting gender equality
+Supporting people of all genders to participate in change-making. 
+Important
+FCRA registration is mandatory.
+PHF explicitly states that it does not work through the FCRA prior-permission route.
+ Funding Amount
+₹10 lakh – ₹40 lakh</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>Learning</t>
+          <t>Governance</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>Sep 14, 2026</t>
+          <t>Sep 15, 2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-imata-conservation-fund-international-marine-animal-trainers-association-opg-26-00170</t>
+          <t>https://onepurpos.in/openings/grants/application-invited-for-india-fund-paul-hamlyn-foundation-opg-26-00172</t>
         </is>
       </c>
     </row>
@@ -520,24 +528,52 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>Applications Invited for the Fair Water Action Fund</t>
+          <t>RFP - Technical Consultancy for disability inclusion and livelihood initiatives</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>About the Grant:
-The Fair Water Action Fund provides financial, technical, legal, and strategic support to organisations and individuals in the Global South working to advance water justice, water security, accountability, and systemic change. The fund supports civil society, media organisations, investigative journalists, researchers, and research institutions working to hold governments, corporations, and other duty bearers accountable.
- Grant Amount
-Minimum Grant: £3,000 GBP
-Maximum Grant: £36,000 GBP per project
- Eligible Applicants
-The following applicants are eligible:
-Civil Society Organizations (CSOs)
-Media organisations
-Coalitions and networks engaged in water security activities
-Water and environmental investigative journalists
-Individual researchers
-Research institutes</t>
+          <t>Request for Proposal (RFP)
+Bids are invited for: Technical Consultancy for disability inclusion and livelihood initiatives
+Ref: AIFT/RFP/DL/2026-27/024
+Summary of Deadlines:
+Release of Request for Proposal September 8, 2026
+Bid Submission Closing Date
+  14th September 2026 (till 13:00 HRS)
+Technical Bid Submission Link
+https://forms.gle/1kyy8yKQpmsmMw4XA
+  Financial Bid Submission Link
+ https://forms.gle/PniTmy9SMBJypKuNA
+  Technical Bid Opening 14th September 2026
+Financial Bid Opening 15th September 2026 Tentative
+Finalization of Contract To be intimated to the awardee only
+Scope of work:
+Background
+Purpose of the Consultancy: The consultant will provide technical and strategic support to AIFT in strengthening the planning, implementation, monitoring and documentation of its disability inclusion and livelihood initiatives, with a focus on the ABLE and DI-verse programmes. The consultancy will provide technical inputs to the programme team, support quality implementation, strengthen stakeholder engagement, and contribute to timely and effective reporting and documentation of programme progress and outcomes.
+The American India Foundation Trust (AIFT) implements programmes aimed at promoting disability inclusion, livelihoods, employment, and equal opportunities for Persons with Disabilities (PwDs). Through initiatives such as the ABLE and DI-verse programmes, AIFT works with organisations and stakeholders to strengthen inclusive practices, build awareness and capacity, and create opportunities for greater participation of persons with disabilities.
+As these programmes involve multiple activities including organisation onboarding, assessments, certification, sensitisation, capacity building, stakeholder engagement, programme implementation, monitoring and documentation, specialised technical expertise is required to support the programme team and ensure quality and effective delivery.
+AIFT therefore seeks to engage an experienced Technical Consultant to provide technical and strategic support across the programme lifecycle, strengthen implementation and stakeholder engagement, and contribute to improved programme outcomes and documentation.
+This aligns closely with the existing SOW, which identifies the ABLE and DI-verse programmes as the focus of the consultancy.
+Objective: To engage an experienced consultant to provide technical and strategic support to AIFT in strengthening the planning, implementation, monitoring, and quality of its disability inclusion and livelihood programmes, particularly the ABLE and DI-verse programmes.
+ Scope of Services
+The selected agency shall provide the following services as mentioned below
+Consultancy period: Period of Performance: tentative Start date 17/09/2026; end dates 31/03/2027. The consultancy will be for a maximum of 60 hours per month. subject to fulfillment of deliverables and requirement.
+Applicant Eligibility Requirements
+Minimum 12–15 years of professional experience, preferably in a leadership role in workplace disability inclusion and related areas.
+Demonstrated expertise and leadership in workplace disability inclusion, disability rights, accessibility, reasonable accommodation and inclusive employment practices.
+Proven experience of direct engagement and working with Persons with Disabilities (PwDs) across employment, livelihoods, skilling and inclusion initiatives.
+Significant experience working directly with corporates and employers to advance disability-inclusive workplaces, employment practices and organisational inclusion.
+Demonstrated experience as a consultant, advisor, thought leader and/or influencer in the disability inclusion ecosystem, with the ability to shape practices and influence stakeholders.
+Strong experience in programme strategy, planning, implementation, monitoring, review and technical advisory support for disability inclusion and livelihood/employment programmes.
+Proven expertise in proposal development, concept notes, programme design, donor engagement and development of strategic programme documents.
+Demonstrated experience in designing and/or implementing disability inclusion assessments, certification programmes, sensitisation initiatives and capacity-building programmes.
+Strong track record of stakeholder engagement with PwDs, corporates, employers, NGOs, donors, implementation partners, government stakeholders and subject matter experts.
+Experience in mentoring and providing technical leadership to programme teams, including reviewing progress, strengthening implementation quality and supporting organisational processes.
+Demonstrated ability to develop and review technical reports, assessment reports, donor reports, case studies, presentations and programme documentation.
+Strong communication, facilitation, influencing and relationship-management skills, with the ability to represent the organisation in external forums and stakeholder engagements.
+Experience contributing to knowledge generation, thought leadership, advocacy, conferences, consultations, publications or sector-wide discussions on workplace disability inclusion will be an added advantage.
+Applicants should demonstrate a strong professional network and credibility within the disability inclusion, corporate/HR and employment ecosystem.
+The consultant must have the availability and capacity to provide up to 60 hours of technical and strategic support per month during the consultancy period.</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
@@ -547,12 +583,12 @@
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Sep 14, 2026</t>
+          <t>Sep 15, 2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-the-fair-water-action-fund-water-witness-international-opg-26-00171</t>
+          <t>https://onepurpos.in/openings/rfps/rfp-technical-consultancy-for-disability-inclusion-and-livelihood-initiatives-american-india-foundation-rfp-26-00352</t>
         </is>
       </c>
     </row>
@@ -564,71 +600,10 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>Application Invited For 2026 Call for Proposals Mountains ADAPT Small Grants</t>
+          <t>RFP - Engagement of Agency/Consultant for Programme Learning &amp; Ecosystem Study</t>
         </is>
       </c>
       <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-UNEP is the leading global environmental authority that sets the world's environmental agenda, promotes the coherent implementation of the environmental dimension of sustainable development within the United Nations system and serves as an authoritative advocate for the environment.
- About the Grant
-The Mountains ADAPT Small Grants Project supports community-based organizations in implementing practical solutions that help mountain communities adapt to climate change while protecting ecosystems and improving livelihoods.
-The first call will fund up to 15 projects and provides grants of up to USD 30,000 per project. Successful organizations will also receive capacity development and training support to strengthen implementation.
-The proposed solutions should have a strong focus on ecosystem-based adaptation (EbA) and/or Nature-based Solutions (NbS). Examples include:
-Ecosystem restoration
-Rainwater harvesting
-Climate-smart agriculture
-Disaster preparedness
-Livelihood diversification
-Other locally appropriate nature-based climate adaptation solutions
- Eligible Applicants
-The grant is intended for:
-Civil society organizations
-Community-based organizations
-Grassroots organizations
-Youth organizations
-Women’s organizations
-Registered NGOs working with mountain communities 
- Important eligibility requirements
-Applicants must:
-Be formally registered.
-Be locally based in an eligible mountain region.
-Have prior experience working directly with mountain communities.
-Address a mountain climate-change challenge or vulnerability.
-Use an ecosystem-based adaptation / nature-based approach.
-Demonstrate capacity to implement the proposed project.
-Submit the required organizational documentation. 
-Individuals are not eligible.</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="inlineStr">
-        <is>
-          <t>Sep 15, 2026</t>
-        </is>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/application-invited-for-2026-call-for-proposals-mountains-adapt-small-grants-united-nations-environment-programme-opg-26-00162</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="95" customHeight="1">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>RFP - Engagement of Agency/Consultant for Programme Learning &amp; Ecosystem Study</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>Request for Proposal (RFP) Bids are invited for: Engagement of Agency/Consultant for Programme Learning &amp; Ecosystem Study
 Ref: AIFT/RFP/DL/2026-27/025
@@ -666,9 +641,89 @@
 Proposals will be assessed on the ability to combine rigorous process documentation with forward-looking ecosystem analysis, and on the ability to turn research into usable strategic choices. Strong proposals should demonstrate both implementation depth and strategic breadth, with practical understanding of government-school systems, CSR partnerships, employee engagement, and AI-ready future-skills programming.</t>
         </is>
       </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Sep 15, 2026</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/rfp-engagement-of-agencyconsultant-for-programme-learning-and-ecosystem-study-american-india-foundation-rfp-26-00353</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="95" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>RFP - Selection of Agency for Conducting Street Plays for a Community Health Awareness Program</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>Request for Proposal / Quotation (RFP / RFQ)
+Selection of Agency for Conducting Street Plays for a Community Health Awareness Program
+Background
+A social impact organization is implementing a community health awareness initiative across multiple states in India. As part of the program, agencies are invited to conduct street plays (Nukkad Nataks) to promote preventive health awareness and engage communities. The program and funding partner details will be shared with the selected agency.
+Scope of Work
+The selected agency will be responsible for:
+Developing a street play script based on the communication brief provided.
+Translating/adapting the script into the local language, if required.
+Arranging artists, costumes, props, and sound system.
+Conducting rehearsals and performing street plays at designated locations.
+Engaging the audience through interactive performances.
+Providing photographs, videos, and a brief activity report after each performance.
+Tentative Locations
+State Location
+Goa Ponda, Canacona, Madgaon
+Gujarat Ahmedabad
+Uttar Pradesh Lucknow, Varanasi, Shravasti, Jhansi, GB Nagar (Noida)
+Please indicate the locations where your organization can conduct street plays.
+Proposal Submission
+Interested agencies are requested to submit:
+Technical Proposal
+Organization profile
+Relevant experience in street plays/health awareness campaigns
+Proposed approach and work plan
+Sample script and video of previous work (if available)
+Locations where services can be provided
+Financial Proposal
+Please share the budget for one street play, including:
+Script development
+Artist fees
+Rehearsals
+Travel &amp; logistics
+Props &amp; costumes
+Sound system
+Documentation
+Taxes (if applicable)
+Deliverables
+Approved street play script
+Successful execution of performances
+Audience engagement
+Photographs and videos
+Brief activity report
+Evaluation Criteria
+Proposals will be evaluated based on:
+Relevant experience
+Technical approach
+Creative concept
+Geographic coverage
+Cost-effectiveness</t>
+        </is>
+      </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>Governance</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr">
@@ -678,7 +733,7 @@
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/rfps/rfp-engagement-of-agencyconsultant-for-programme-learning-and-ecosystem-study-american-india-foundation-rfp-26-00353</t>
+          <t>https://onepurpos.in/openings/rfps/rfp-selection-of-agency-for-conducting-street-plays-for-a-community-health-awareness-program-bharatcares-rfp-26-00321</t>
         </is>
       </c>
     </row>
@@ -690,41 +745,41 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>Application Invited For India Fund</t>
+          <t>Application Invited For 2026 Call for Proposals Mountains ADAPT Small Grants</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
           <t>About the Organization
-Paul Hamlyn Foundation was established in 1987. Since then, we have used our resources to work towards a just future in which everyone, especially young people, can realise their full potential and enjoy fulfilling and creative lives. In all of our work, including our grant-making, we are guided by six strategic priorities where we want to see change: • Investing in young people • Migration and integration • Arts access and participation • Education and learning through the arts • Nurturing ideas and people • Creating opportunities for people and communities in India
- About the India Fund
-The India Fund supports small NGOs working with vulnerable communities in priority geographical areas of India.
-The fund is based on the principle that communities should be central to development work, with people facing disadvantage playing an important role in leading change and designing solutions to inequality.
-Strategic aims
-The fund aims to:
-Encourage NGOs to undertake community-centred development programmes.
-Enable communities to take greater control of their own development and improve their lives.
-Encourage development funding that addresses systemic change.
-Strengthen the capacity of organisations and people facilitating this work.
- Who Can Apply?
-The fund specifically supports:
-Local Indian NGOs with FCRA registration
-This is an important eligibility requirement.
-Eligible organisations should generally be:
-Indian organisations
-Locally based in the communities they serve
-Working directly with communities
-Focused on long-term improvements in community wellbeing
-Connected with relevant panchayats in rural areas or municipalities in urban areas
-Taking steps to reduce their environmental impact
-Working to improve local ecology
-Promoting gender equality
-Supporting people of all genders to participate in change-making. 
-Important
-FCRA registration is mandatory.
-PHF explicitly states that it does not work through the FCRA prior-permission route.
- Funding Amount
-₹10 lakh – ₹40 lakh</t>
+UNEP is the leading global environmental authority that sets the world's environmental agenda, promotes the coherent implementation of the environmental dimension of sustainable development within the United Nations system and serves as an authoritative advocate for the environment.
+ About the Grant
+The Mountains ADAPT Small Grants Project supports community-based organizations in implementing practical solutions that help mountain communities adapt to climate change while protecting ecosystems and improving livelihoods.
+The first call will fund up to 15 projects and provides grants of up to USD 30,000 per project. Successful organizations will also receive capacity development and training support to strengthen implementation.
+The proposed solutions should have a strong focus on ecosystem-based adaptation (EbA) and/or Nature-based Solutions (NbS). Examples include:
+Ecosystem restoration
+Rainwater harvesting
+Climate-smart agriculture
+Disaster preparedness
+Livelihood diversification
+Other locally appropriate nature-based climate adaptation solutions
+ Eligible Applicants
+The grant is intended for:
+Civil society organizations
+Community-based organizations
+Grassroots organizations
+Youth organizations
+Women’s organizations
+Registered NGOs working with mountain communities 
+ Important eligibility requirements
+Applicants must:
+Be formally registered.
+Be locally based in an eligible mountain region.
+Have prior experience working directly with mountain communities.
+Address a mountain climate-change challenge or vulnerability.
+Use an ecosystem-based adaptation / nature-based approach.
+Demonstrate capacity to implement the proposed project.
+Submit the required organizational documentation. 
+Individuals are not eligible.</t>
         </is>
       </c>
       <c r="D6" s="1" t="inlineStr">
@@ -739,7 +794,7 @@
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/grants/application-invited-for-india-fund-paul-hamlyn-foundation-opg-26-00172</t>
+          <t>https://onepurpos.in/openings/grants/application-invited-for-2026-call-for-proposals-mountains-adapt-small-grants-united-nations-environment-programme-opg-26-00162</t>
         </is>
       </c>
     </row>
@@ -847,52 +902,37 @@
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>RFP - Technical Consultancy for disability inclusion and livelihood initiatives</t>
+          <t>Terms of Reference TOR for Project Consultant / Organization DRE Assessment &amp; Coordination Support for Common Facility Centres CFCs</t>
         </is>
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>Request for Proposal (RFP)
-Bids are invited for: Technical Consultancy for disability inclusion and livelihood initiatives
-Ref: AIFT/RFP/DL/2026-27/024
-Summary of Deadlines:
-Release of Request for Proposal September 8, 2026
-Bid Submission Closing Date
-  14th September 2026 (till 13:00 HRS)
-Technical Bid Submission Link
-https://forms.gle/1kyy8yKQpmsmMw4XA
-  Financial Bid Submission Link
- https://forms.gle/PniTmy9SMBJypKuNA
-  Technical Bid Opening 14th September 2026
-Financial Bid Opening 15th September 2026 Tentative
-Finalization of Contract To be intimated to the awardee only
-Scope of work:
-Background
-Purpose of the Consultancy: The consultant will provide technical and strategic support to AIFT in strengthening the planning, implementation, monitoring and documentation of its disability inclusion and livelihood initiatives, with a focus on the ABLE and DI-verse programmes. The consultancy will provide technical inputs to the programme team, support quality implementation, strengthen stakeholder engagement, and contribute to timely and effective reporting and documentation of programme progress and outcomes.
-The American India Foundation Trust (AIFT) implements programmes aimed at promoting disability inclusion, livelihoods, employment, and equal opportunities for Persons with Disabilities (PwDs). Through initiatives such as the ABLE and DI-verse programmes, AIFT works with organisations and stakeholders to strengthen inclusive practices, build awareness and capacity, and create opportunities for greater participation of persons with disabilities.
-As these programmes involve multiple activities including organisation onboarding, assessments, certification, sensitisation, capacity building, stakeholder engagement, programme implementation, monitoring and documentation, specialised technical expertise is required to support the programme team and ensure quality and effective delivery.
-AIFT therefore seeks to engage an experienced Technical Consultant to provide technical and strategic support across the programme lifecycle, strengthen implementation and stakeholder engagement, and contribute to improved programme outcomes and documentation.
-This aligns closely with the existing SOW, which identifies the ABLE and DI-verse programmes as the focus of the consultancy.
-Objective: To engage an experienced consultant to provide technical and strategic support to AIFT in strengthening the planning, implementation, monitoring, and quality of its disability inclusion and livelihood programmes, particularly the ABLE and DI-verse programmes.
- Scope of Services
-The selected agency shall provide the following services as mentioned below
-Consultancy period: Period of Performance: tentative Start date 17/09/2026; end dates 31/03/2027. The consultancy will be for a maximum of 60 hours per month. subject to fulfillment of deliverables and requirement.
-Applicant Eligibility Requirements
-Minimum 12–15 years of professional experience, preferably in a leadership role in workplace disability inclusion and related areas.
-Demonstrated expertise and leadership in workplace disability inclusion, disability rights, accessibility, reasonable accommodation and inclusive employment practices.
-Proven experience of direct engagement and working with Persons with Disabilities (PwDs) across employment, livelihoods, skilling and inclusion initiatives.
-Significant experience working directly with corporates and employers to advance disability-inclusive workplaces, employment practices and organisational inclusion.
-Demonstrated experience as a consultant, advisor, thought leader and/or influencer in the disability inclusion ecosystem, with the ability to shape practices and influence stakeholders.
-Strong experience in programme strategy, planning, implementation, monitoring, review and technical advisory support for disability inclusion and livelihood/employment programmes.
-Proven expertise in proposal development, concept notes, programme design, donor engagement and development of strategic programme documents.
-Demonstrated experience in designing and/or implementing disability inclusion assessments, certification programmes, sensitisation initiatives and capacity-building programmes.
-Strong track record of stakeholder engagement with PwDs, corporates, employers, NGOs, donors, implementation partners, government stakeholders and subject matter experts.
-Experience in mentoring and providing technical leadership to programme teams, including reviewing progress, strengthening implementation quality and supporting organisational processes.
-Demonstrated ability to develop and review technical reports, assessment reports, donor reports, case studies, presentations and programme documentation.
-Strong communication, facilitation, influencing and relationship-management skills, with the ability to represent the organisation in external forums and stakeholder engagements.
-Experience contributing to knowledge generation, thought leadership, advocacy, conferences, consultations, publications or sector-wide discussions on workplace disability inclusion will be an added advantage.
-Applicants should demonstrate a strong professional network and credibility within the disability inclusion, corporate/HR and employment ecosystem.
-The consultant must have the availability and capacity to provide up to 60 hours of technical and strategic support per month during the consultancy period.</t>
+          <t>Title Project Consultant / Organization – DRE Assessment &amp; Coordination Support for Common Facility Centres (CFCs)
+Timeline
+ 6 Months
+Expected area of expertise Energy assessment, solar system sizing, documentation, and field coordination
+Apply Link
+ https://forms.gle/CTSsV4AzAAcRqmyh8
+Last Date for Apply 16th September, 2026 by 5 pm.
+About SELCO Foundation:
+SELCO Foundation is an open-source, not-for-profit organization that engages in field-based R&amp;D and ecosystem building for the deployment of clean energy solutions that alleviate poverty by improving access to sustainable energy to underserved communities in tribal, rural, and urban poor areas. The organization works in collaboration with practitioners in the social sector, energy entrepreneurs, NGOs from various developmental sectors, and educational institutions to link the benefits of sustainable energy to poverty eradication. The organization works across verticals such as energy access, health, and livelihoods. You can find more information about the SELCO Foundation on our website: http://www.selcofoundation.org/
+Summary of the Project:
+SELCO Foundation is looking to onboard a Consultant/Organization to support the assessment, documentation, and solar system sizing for 30 Common Facility Centres (CFCs) implemented by the government across Agri, animal husbandry, microbusiness, or other relevant livelihood sectors. The Consultant will also provide coordination support during implementation (carried out by a separate implementation vendor) and conduct a post-installation endline assessment.
+This is a scoped, straightforward assignment focused on assessment, standard system sizing, coordination, and endline verification — it does not include design of the overall scheme, beneficiary long-listing, or ongoing monitoring &amp; evaluation.
+Goals and Objectives
+The program's key objectives are:
+Assessing and documenting 30 Government-implemented CFCs
+Recommending standard solar system sizes/designs based on load requirements
+Coordinating with the implementation vendor and keeping CFC users updated through implementation
+Conducting a post-installation endline assessment
+Requirements
+Agency/Individual should have experience in or capacity for:
+Conducting field-based energy/load assessments and documentation.
+Solar system sizing and design recommendation based on load profiles.
+Coordinating with government departments, CFC operators, and third-party implementation vendors.
+Conducting post-installation assessments and reporting.
+Excellent written and verbal communication skills, especially for field coordination.
+Working presence across Assam, Meghalaya, and Mizoram for the duration of the agreement.</t>
         </is>
       </c>
       <c r="D8" s="1" t="inlineStr">
@@ -902,12 +942,12 @@
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>Sep 15, 2026</t>
+          <t>Sep 16, 2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/rfps/rfp-technical-consultancy-for-disability-inclusion-and-livelihood-initiatives-american-india-foundation-rfp-26-00352</t>
+          <t>https://onepurpos.in/openings/rfps/terms-of-reference-tor-for-project-consultant-organization-dre-assessment-and-coordination-support-for-common-facility-centres-cfcs-selco-foundation-rfp-26-00345</t>
         </is>
       </c>
     </row>
@@ -919,75 +959,61 @@
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
-          <t>RFP - Selection of Agency for Conducting Street Plays for a Community Health Awareness Program</t>
+          <t>ToR - Development of the WaterAid India WAI Blue Book Series Programme Implementation Guides</t>
         </is>
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>Request for Proposal / Quotation (RFP / RFQ)
-Selection of Agency for Conducting Street Plays for a Community Health Awareness Program
+          <t>Terms of Reference (ToR)
+Development of the WaterAid India (WAI) Blue Book Series – Programme Implementation Guides
+About WaterAid India
+Jal Seva Charitable Foundation (JSCF) is registered in India as a not-for-profit company under Chapter 8 of the Companies Act, 2013. JSCF, is an associate member of the WaterAid federation and uses the brand name ‘WaterAid’ in India.
+WaterAid India seeks to improve the quality of life of 5,000,000 households – with a special emphasis on the vulnerable by 2029 through the provision of climate-resilient and sustainable WASH services via demonstration, institution strengthening, and the effective utilization of public resources. We work in rural and urban areas and seek to deepen our presence in states we operate in and to work in small towns. Thanks to our amazing supporters, we have reached millions of people with these three essentials – clean water, decent toilets, and good hygiene – enabling communities to unlock their potential to break free from the cycle of poverty and to change lives for good.
+We will not stop. Not until clean water, decent toilets and good hygiene are a normal part of everyday life for everyone, everywhere.
+WaterAid India’s (WAI) country office is based in New Delhi with State Offices in Bengaluru, Bhopal, Bhubaneswar, Hyderabad, Lucknow, Patna, Kolkata and Raipur. We currently have a presence in ten states in the country.
+WAI’s Programme focus in the next five years is on ensuring access to safe and assured drinking water in the households, as well as safely managed sanitation at both the household and habitation level. Further, we seek to ensure that anganwadi’s, schools and health care facilities have adequate and appropriate water, sanitation and hygiene infrastructure. Finally, we seek to create integrated water and sanitation solutions in small towns. In all of these efforts, ensuring climate resilience of infrastructure and systems is critical. We seek to do this through demonstration and the provision of technical and knowledge support to governments at all levels who can facilitate adoption on scale. Implementation is primarily through our own field teams. Further details about WAI can be accessed at https://www.wateraid.org/in/
 Background
-A social impact organization is implementing a community health awareness initiative across multiple states in India. As part of the program, agencies are invited to conduct street plays (Nukkad Nataks) to promote preventive health awareness and engage communities. The program and funding partner details will be shared with the selected agency.
-Scope of Work
-The selected agency will be responsible for:
-Developing a street play script based on the communication brief provided.
-Translating/adapting the script into the local language, if required.
-Arranging artists, costumes, props, and sound system.
-Conducting rehearsals and performing street plays at designated locations.
-Engaging the audience through interactive performances.
-Providing photographs, videos, and a brief activity report after each performance.
-Tentative Locations
-State Location
-Goa Ponda, Canacona, Madgaon
-Gujarat Ahmedabad
-Uttar Pradesh Lucknow, Varanasi, Shravasti, Jhansi, GB Nagar (Noida)
-Please indicate the locations where your organization can conduct street plays.
+WaterAid India (WAI) implements integrated Water, Sanitation and Hygiene (WASH) programmes across multiple states through partnerships with governments, communities, civil society organizations, and development partners. Over the years, WAI has developed extensive technical expertise, programme methodologies, implementation tools, and institutional learning across diverse programme contexts.
+As WAI continues to scale its programmes, there is a need to institutionalize these experiences into a standardized implementation framework that promotes consistency, quality, accountability, and sustainability across all programme interventions.
+To address this need, WaterAid India proposes to develop the WAI Blue Book Series—the organization's programme implementation guide. The Blue Book Series will comprise six interconnected booklets that together provide end-to-end guidance for programme execution—from entering a new intervention geography and designing programmes to implementing quality WASH interventions, strengthening institutions, ensuring sustainable services, documenting evidence, and planning future programme investments.
+The Blue Book Series will establish common programme standards, implementation protocols, quality assurance mechanisms, and practical tools that can be consistently used by WaterAid India teams, partners, consultants, and other implementation stakeholders.
+Objective of the Assignment
+To develop the WAI Blue Book Series, a standardized set of programme implementation guides that establish common implementation standards, quality assurance mechanisms, operational protocols, and practical tools for delivering high-quality, inclusive, climate-resilient, and sustainable WASH programmes across WaterAid India.
+Consultant/Agency Profile
+The consultant/agency should possess:
+At least 10 years of experience in WASH, rural development, programme quality, or institutional strengthening.
+Demonstrated experience in developing implementation manuals, operational frameworks, programme standards, or quality assurance systems.
+Strong expertise in programme design, technical writing, facilitation, and organizational knowledge management.
+Experience working with government systems, development partners, and multi-state programmes.
+A multidisciplinary team with expertise in WASH programming, programme quality, safeguarding, technical writing, and graphic design will be preferred.
 Proposal Submission
-Interested agencies are requested to submit:
-Technical Proposal
-Organization profile
-Relevant experience in street plays/health awareness campaigns
-Proposed approach and work plan
-Sample script and video of previous work (if available)
-Locations where services can be provided
-Financial Proposal
-Please share the budget for one street play, including:
-Script development
-Artist fees
-Rehearsals
-Travel &amp; logistics
-Props &amp; costumes
-Sound system
-Documentation
-Taxes (if applicable)
-Deliverables
-Approved street play script
-Successful execution of performances
-Audience engagement
-Photographs and videos
-Brief activity report
+Interested consultants/agencies should submit:
+Technical proposal outlining methodology and work plan.
+Financial proposal.
+Relevant work samples (frameworks, toolkits, manuals or IEC materials).
+CVs of key personnel.
 Evaluation Criteria
-Proposals will be evaluated based on:
-Relevant experience
-Technical approach
-Creative concept
-Geographic coverage
-Cost-effectiveness</t>
+Criteria Weight
+Understanding of assignment 20%
+Proposed methodology 25%
+Relevant organisational experience 20%
+Team composition and expertise 20%
+Financial proposal 15%</t>
         </is>
       </c>
       <c r="D9" s="1" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Governance</t>
         </is>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>Sep 15, 2026</t>
+          <t>Sep 16, 2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/rfps/rfp-selection-of-agency-for-conducting-street-plays-for-a-community-health-awareness-program-bharatcares-rfp-26-00321</t>
+          <t>https://onepurpos.in/openings/rfps/tor-development-of-the-wateraid-india-wai-blue-book-series-programme-implementation-guides-wateraid-india-rfp-26-00347</t>
         </is>
       </c>
     </row>
@@ -999,10 +1025,76 @@
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
+          <t>ToR - Development of WaterAid India's Hygiene Framework Community Facilitator Toolkit Hygiene Booklet and Hygiene Calendar</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>Terms of Reference (ToR)
+Development of WaterAid India's Hygiene Framework, Community Facilitator Toolkit, Hygiene Booklet and Hygiene Calendar
+About WaterAid India
+Jal Seva Charitable Foundation (JSCF) is registered in India as a not-for-profit company under Chapter 8 of the Companies Act, 2013. JSCF, is an associate member of the WaterAid federation and uses the brand name ‘WaterAid’ in India.
+WaterAid India seeks to improve the quality of life of 5,000,000 households – with a special emphasis on the vulnerable by 2029 through the provision of climate-resilient and sustainable WASH services via demonstration, institution strengthening, and the effective utilization of public resources. We work in rural and urban areas and seek to deepen our presence in states we operate in and to work in small towns. Thanks to our amazing supporters, we have reached millions of people with these three essentials – clean water, decent toilets, and good hygiene – enabling communities to unlock their potential to break free from the cycle of poverty and to change lives for good.
+We will not stop. Not until clean water, decent toilets and good hygiene are a normal part of everyday life for everyone, everywhere.
+WaterAid India’s (WAI) country office is based in New Delhi with State Offices in Bengaluru, Bhopal, Bhubaneswar, Hyderabad, Lucknow, Patna, Kolkata and Raipur. We currently have a presence in ten states in the country.
+WAI’s Programme focus in the next five years is on ensuring access to safe and assured drinking water in the households, as well as safely managed sanitation at both the household and habitation level. Further, we seek to ensure that anganwadi’s, schools and health care facilities have adequate and appropriate water, sanitation and hygiene infrastructure. Finally, we seek to create integrated water and sanitation solutions in small towns. In all of these efforts, ensuring climate resilience of infrastructure and systems is critical. We seek to do this through demonstration and the provision of technical and knowledge support to governments at all levels who can facilitate adoption on scale. Implementation is primarily through our own field teams. Further details about WAI can be accessed at https://www.wateraid.org/in/
+Background
+WaterAid India (WAI)/ Jal Seva Charitable Foundation (JSCF) works towards achieving universal access to safe water, sanitation and hygiene (WASH), with a focus on the poorest and most marginalised communities. While access to water and sanitation infrastructure has significantly improved, sustained hygiene behaviour remains a critical determinant of health outcomes, nutrition, climate resilience and the long-term sustainability of WASH services.
+To strengthen its hygiene programming across diverse geographies, WaterAid India intends to develop a comprehensive Hygiene Framework and a set of practical implementation resources that can be used by programme teams, partner organisations and Community Facilitators (CFs). The products should adopt a life-cycle approach, integrate climate resilience and gender, and align with national programmes such as Jal Jeevan Mission, Swachh Bharat Mission (Grameen), Poshan Abhiyaan and relevant health initiatives.
+WAI/ JSCF invites proposals from experienced consultants or agencies to support the development of a comprehensive Hygiene Framework and implementation toolkit. The assignment seeks to strengthen the quality, consistency and effectiveness of hygiene programming by developing practical guidance, communication resources and facilitation tools that can be adopted across WaterAid India's programmes.
+Objective of the Assignment
+To develop a comprehensive, evidence-based and implementation-oriented Hygiene Framework and supporting tools that standardise WaterAid India's hygiene programming and enable Community Facilitators to effectively promote sustainable hygiene behaviour at the community level.
+Required Qualifications
+The consultant/agency should demonstrate:
+Minimum 8–10 years of experience in WASH, public health or behaviour change communication.
+Proven experience in developing hygiene strategies, behaviour change frameworks and community training resources.
+Experience working with government programmes such as JJM, SBM-G, NHM or ICDS.
+Strong understanding of climate-resilient WASH programming.
+Excellent technical writing, instructional design and facilitation skills.
+Experience working with national or international development organisations.
+Proposal Submission
+Interested consultants/agencies should submit:
+Technical proposal outlining methodology and work plan.
+Financial proposal.
+Relevant work samples (frameworks, toolkits, manuals or IEC materials).
+CVs of key personnel.
+Evaluation Criteria
+Criteria Weight
+Understanding of assignment 20%
+Proposed methodology 25%
+Relevant organisational experience 20%
+Team composition and expertise 20%
+Financial proposal 15%</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>Sep 16, 2026</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/tor-development-of-wateraid-indias-hygiene-framework-community-facilitator-toolkit-hygiene-booklet-and-hygiene-calendar-wateraid-india-rfp-26-00349</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="95" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
           <t>ToR - Standardisation and Development of Community Training Modules and Facilitator Manuals for WASH-Secure Communities</t>
         </is>
       </c>
-      <c r="C10" s="1" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>Terms of Reference (ToR)
 Standardisation and Development of Community Training Modules and Facilitator Manuals for WASH-Secure Communities
@@ -1071,85 +1163,19 @@
 The consultant/agency obtaining the highest combined score will be recommended for award.</t>
         </is>
       </c>
-      <c r="D10" s="1" t="inlineStr">
+      <c r="D11" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E10" s="1" t="inlineStr">
+      <c r="E11" s="1" t="inlineStr">
         <is>
           <t>Sep 16, 2026</t>
         </is>
       </c>
-      <c r="F10" s="1" t="inlineStr">
+      <c r="F11" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-standardisation-and-development-of-community-training-modules-and-facilitator-manuals-for-wash-secure-communities-wateraid-india-rfp-26-00348</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="95" customHeight="1">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="inlineStr">
-        <is>
-          <t>ToR - Development of the WaterAid India WAI Blue Book Series Programme Implementation Guides</t>
-        </is>
-      </c>
-      <c r="C11" s="1" t="inlineStr">
-        <is>
-          <t>Terms of Reference (ToR)
-Development of the WaterAid India (WAI) Blue Book Series – Programme Implementation Guides
-About WaterAid India
-Jal Seva Charitable Foundation (JSCF) is registered in India as a not-for-profit company under Chapter 8 of the Companies Act, 2013. JSCF, is an associate member of the WaterAid federation and uses the brand name ‘WaterAid’ in India.
-WaterAid India seeks to improve the quality of life of 5,000,000 households – with a special emphasis on the vulnerable by 2029 through the provision of climate-resilient and sustainable WASH services via demonstration, institution strengthening, and the effective utilization of public resources. We work in rural and urban areas and seek to deepen our presence in states we operate in and to work in small towns. Thanks to our amazing supporters, we have reached millions of people with these three essentials – clean water, decent toilets, and good hygiene – enabling communities to unlock their potential to break free from the cycle of poverty and to change lives for good.
-We will not stop. Not until clean water, decent toilets and good hygiene are a normal part of everyday life for everyone, everywhere.
-WaterAid India’s (WAI) country office is based in New Delhi with State Offices in Bengaluru, Bhopal, Bhubaneswar, Hyderabad, Lucknow, Patna, Kolkata and Raipur. We currently have a presence in ten states in the country.
-WAI’s Programme focus in the next five years is on ensuring access to safe and assured drinking water in the households, as well as safely managed sanitation at both the household and habitation level. Further, we seek to ensure that anganwadi’s, schools and health care facilities have adequate and appropriate water, sanitation and hygiene infrastructure. Finally, we seek to create integrated water and sanitation solutions in small towns. In all of these efforts, ensuring climate resilience of infrastructure and systems is critical. We seek to do this through demonstration and the provision of technical and knowledge support to governments at all levels who can facilitate adoption on scale. Implementation is primarily through our own field teams. Further details about WAI can be accessed at https://www.wateraid.org/in/
-Background
-WaterAid India (WAI) implements integrated Water, Sanitation and Hygiene (WASH) programmes across multiple states through partnerships with governments, communities, civil society organizations, and development partners. Over the years, WAI has developed extensive technical expertise, programme methodologies, implementation tools, and institutional learning across diverse programme contexts.
-As WAI continues to scale its programmes, there is a need to institutionalize these experiences into a standardized implementation framework that promotes consistency, quality, accountability, and sustainability across all programme interventions.
-To address this need, WaterAid India proposes to develop the WAI Blue Book Series—the organization's programme implementation guide. The Blue Book Series will comprise six interconnected booklets that together provide end-to-end guidance for programme execution—from entering a new intervention geography and designing programmes to implementing quality WASH interventions, strengthening institutions, ensuring sustainable services, documenting evidence, and planning future programme investments.
-The Blue Book Series will establish common programme standards, implementation protocols, quality assurance mechanisms, and practical tools that can be consistently used by WaterAid India teams, partners, consultants, and other implementation stakeholders.
-Objective of the Assignment
-To develop the WAI Blue Book Series, a standardized set of programme implementation guides that establish common implementation standards, quality assurance mechanisms, operational protocols, and practical tools for delivering high-quality, inclusive, climate-resilient, and sustainable WASH programmes across WaterAid India.
-Consultant/Agency Profile
-The consultant/agency should possess:
-At least 10 years of experience in WASH, rural development, programme quality, or institutional strengthening.
-Demonstrated experience in developing implementation manuals, operational frameworks, programme standards, or quality assurance systems.
-Strong expertise in programme design, technical writing, facilitation, and organizational knowledge management.
-Experience working with government systems, development partners, and multi-state programmes.
-A multidisciplinary team with expertise in WASH programming, programme quality, safeguarding, technical writing, and graphic design will be preferred.
-Proposal Submission
-Interested consultants/agencies should submit:
-Technical proposal outlining methodology and work plan.
-Financial proposal.
-Relevant work samples (frameworks, toolkits, manuals or IEC materials).
-CVs of key personnel.
-Evaluation Criteria
-Criteria Weight
-Understanding of assignment 20%
-Proposed methodology 25%
-Relevant organisational experience 20%
-Team composition and expertise 20%
-Financial proposal 15%</t>
-        </is>
-      </c>
-      <c r="D11" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E11" s="1" t="inlineStr">
-        <is>
-          <t>Sep 16, 2026</t>
-        </is>
-      </c>
-      <c r="F11" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/tor-development-of-the-wateraid-india-wai-blue-book-series-programme-implementation-guides-wateraid-india-rfp-26-00347</t>
         </is>
       </c>
     </row>
@@ -1161,185 +1187,10 @@
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
-          <t>Terms of Reference TOR for Project Consultant / Organization DRE Assessment &amp; Coordination Support for Common Facility Centres CFCs</t>
+          <t>SoW - Hiring an External Agency for Orientation and Capacity Building</t>
         </is>
       </c>
       <c r="C12" s="1" t="inlineStr">
-        <is>
-          <t>Title Project Consultant / Organization – DRE Assessment &amp; Coordination Support for Common Facility Centres (CFCs)
-Timeline
- 6 Months
-Expected area of expertise Energy assessment, solar system sizing, documentation, and field coordination
-Apply Link
- https://forms.gle/CTSsV4AzAAcRqmyh8
-Last Date for Apply 16th September, 2026 by 5 pm.
-About SELCO Foundation:
-SELCO Foundation is an open-source, not-for-profit organization that engages in field-based R&amp;D and ecosystem building for the deployment of clean energy solutions that alleviate poverty by improving access to sustainable energy to underserved communities in tribal, rural, and urban poor areas. The organization works in collaboration with practitioners in the social sector, energy entrepreneurs, NGOs from various developmental sectors, and educational institutions to link the benefits of sustainable energy to poverty eradication. The organization works across verticals such as energy access, health, and livelihoods. You can find more information about the SELCO Foundation on our website: http://www.selcofoundation.org/
-Summary of the Project:
-SELCO Foundation is looking to onboard a Consultant/Organization to support the assessment, documentation, and solar system sizing for 30 Common Facility Centres (CFCs) implemented by the government across Agri, animal husbandry, microbusiness, or other relevant livelihood sectors. The Consultant will also provide coordination support during implementation (carried out by a separate implementation vendor) and conduct a post-installation endline assessment.
-This is a scoped, straightforward assignment focused on assessment, standard system sizing, coordination, and endline verification — it does not include design of the overall scheme, beneficiary long-listing, or ongoing monitoring &amp; evaluation.
-Goals and Objectives
-The program's key objectives are:
-Assessing and documenting 30 Government-implemented CFCs
-Recommending standard solar system sizes/designs based on load requirements
-Coordinating with the implementation vendor and keeping CFC users updated through implementation
-Conducting a post-installation endline assessment
-Requirements
-Agency/Individual should have experience in or capacity for:
-Conducting field-based energy/load assessments and documentation.
-Solar system sizing and design recommendation based on load profiles.
-Coordinating with government departments, CFC operators, and third-party implementation vendors.
-Conducting post-installation assessments and reporting.
-Excellent written and verbal communication skills, especially for field coordination.
-Working presence across Assam, Meghalaya, and Mizoram for the duration of the agreement.</t>
-        </is>
-      </c>
-      <c r="D12" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E12" s="1" t="inlineStr">
-        <is>
-          <t>Sep 16, 2026</t>
-        </is>
-      </c>
-      <c r="F12" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/terms-of-reference-tor-for-project-consultant-organization-dre-assessment-and-coordination-support-for-common-facility-centres-cfcs-selco-foundation-rfp-26-00345</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="95" customHeight="1">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B13" s="1" t="inlineStr">
-        <is>
-          <t>ToR - Development of WaterAid India's Hygiene Framework Community Facilitator Toolkit Hygiene Booklet and Hygiene Calendar</t>
-        </is>
-      </c>
-      <c r="C13" s="1" t="inlineStr">
-        <is>
-          <t>Terms of Reference (ToR)
-Development of WaterAid India's Hygiene Framework, Community Facilitator Toolkit, Hygiene Booklet and Hygiene Calendar
-About WaterAid India
-Jal Seva Charitable Foundation (JSCF) is registered in India as a not-for-profit company under Chapter 8 of the Companies Act, 2013. JSCF, is an associate member of the WaterAid federation and uses the brand name ‘WaterAid’ in India.
-WaterAid India seeks to improve the quality of life of 5,000,000 households – with a special emphasis on the vulnerable by 2029 through the provision of climate-resilient and sustainable WASH services via demonstration, institution strengthening, and the effective utilization of public resources. We work in rural and urban areas and seek to deepen our presence in states we operate in and to work in small towns. Thanks to our amazing supporters, we have reached millions of people with these three essentials – clean water, decent toilets, and good hygiene – enabling communities to unlock their potential to break free from the cycle of poverty and to change lives for good.
-We will not stop. Not until clean water, decent toilets and good hygiene are a normal part of everyday life for everyone, everywhere.
-WaterAid India’s (WAI) country office is based in New Delhi with State Offices in Bengaluru, Bhopal, Bhubaneswar, Hyderabad, Lucknow, Patna, Kolkata and Raipur. We currently have a presence in ten states in the country.
-WAI’s Programme focus in the next five years is on ensuring access to safe and assured drinking water in the households, as well as safely managed sanitation at both the household and habitation level. Further, we seek to ensure that anganwadi’s, schools and health care facilities have adequate and appropriate water, sanitation and hygiene infrastructure. Finally, we seek to create integrated water and sanitation solutions in small towns. In all of these efforts, ensuring climate resilience of infrastructure and systems is critical. We seek to do this through demonstration and the provision of technical and knowledge support to governments at all levels who can facilitate adoption on scale. Implementation is primarily through our own field teams. Further details about WAI can be accessed at https://www.wateraid.org/in/
-Background
-WaterAid India (WAI)/ Jal Seva Charitable Foundation (JSCF) works towards achieving universal access to safe water, sanitation and hygiene (WASH), with a focus on the poorest and most marginalised communities. While access to water and sanitation infrastructure has significantly improved, sustained hygiene behaviour remains a critical determinant of health outcomes, nutrition, climate resilience and the long-term sustainability of WASH services.
-To strengthen its hygiene programming across diverse geographies, WaterAid India intends to develop a comprehensive Hygiene Framework and a set of practical implementation resources that can be used by programme teams, partner organisations and Community Facilitators (CFs). The products should adopt a life-cycle approach, integrate climate resilience and gender, and align with national programmes such as Jal Jeevan Mission, Swachh Bharat Mission (Grameen), Poshan Abhiyaan and relevant health initiatives.
-WAI/ JSCF invites proposals from experienced consultants or agencies to support the development of a comprehensive Hygiene Framework and implementation toolkit. The assignment seeks to strengthen the quality, consistency and effectiveness of hygiene programming by developing practical guidance, communication resources and facilitation tools that can be adopted across WaterAid India's programmes.
-Objective of the Assignment
-To develop a comprehensive, evidence-based and implementation-oriented Hygiene Framework and supporting tools that standardise WaterAid India's hygiene programming and enable Community Facilitators to effectively promote sustainable hygiene behaviour at the community level.
-Required Qualifications
-The consultant/agency should demonstrate:
-Minimum 8–10 years of experience in WASH, public health or behaviour change communication.
-Proven experience in developing hygiene strategies, behaviour change frameworks and community training resources.
-Experience working with government programmes such as JJM, SBM-G, NHM or ICDS.
-Strong understanding of climate-resilient WASH programming.
-Excellent technical writing, instructional design and facilitation skills.
-Experience working with national or international development organisations.
-Proposal Submission
-Interested consultants/agencies should submit:
-Technical proposal outlining methodology and work plan.
-Financial proposal.
-Relevant work samples (frameworks, toolkits, manuals or IEC materials).
-CVs of key personnel.
-Evaluation Criteria
-Criteria Weight
-Understanding of assignment 20%
-Proposed methodology 25%
-Relevant organisational experience 20%
-Team composition and expertise 20%
-Financial proposal 15%</t>
-        </is>
-      </c>
-      <c r="D13" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E13" s="1" t="inlineStr">
-        <is>
-          <t>Sep 16, 2026</t>
-        </is>
-      </c>
-      <c r="F13" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/tor-development-of-wateraid-indias-hygiene-framework-community-facilitator-toolkit-hygiene-booklet-and-hygiene-calendar-wateraid-india-rfp-26-00349</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="95" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="inlineStr">
-        <is>
-          <t>ToR - Project Consultant / Organization DRE Integration in PMFME Enterprises</t>
-        </is>
-      </c>
-      <c r="C14" s="1" t="inlineStr">
-        <is>
-          <t>Terms of Reference (TOR) for Consultancy Services
-PowerUp PMFME-DRE 
-Integrating Decentralized Renewable Energy (DRE) in PMFME Food Processing Enterprises
-Title Project Consultant / Organization – DRE Integration in PMFME Enterprises
-Location
-Karnataka and Maharashtra.
-Bidders may apply for both states as a single assignment, or as a consortium with a designated lead entity covering both.
-Timeline 6 (six) Months
-Expected area of expertise Energy assessment, project implementation, financial analysis, capacity building, post-implementation audit, and documentation
-Apply Link https://forms.gle/gAmuuSxm3MkLofpF9
-Last Date for Apply 17th Sep 2026, 5 PM
-About SELCO Foundation:
-SELCO Foundation is an open-source, not-for-profit organization that engages in field-based R&amp;D and ecosystem building for the deployment of clean energy solutions that alleviate poverty by improving access to sustainable energy to underserved communities in tribal, rural, and urban poor areas. The organization works in collaboration with practitioners in the social sector, energy entrepreneurs, NGOs from various developmental sectors, and educational institutions to link the benefits of sustainable energy to poverty eradication. The organization works across verticals such as energy access, health, and livelihoods. You can find more information about the SELCO Foundation on our website: http://www.selcofoundation.org/
-Summary of the Project:
-SELCO Foundation is working to integrate Decentralized Renewable Energy (DRE) solutions into micro food processing enterprises supported under the PM Formalisation of Micro Food Processing Enterprises (PMFME) scheme. The program aims to improve energy access and productivity for PMFME beneficiaries in Karnataka and Maharashtra, targeting a total of 500 sites for DRE integration.
-A Project Consultant/Organization may apply to coordinate and facilitate site-level implementation across these two states, ensuring interventions align with beneficiary needs and have a meaningful impact.
-Goals and Objectives
-The program's key objectives are:
-Phase 1: Designing standardized DRE system options by system size, with leverage components identified for each - validated through a preliminary long/short list and sample site visits
-Phase 2: Conducting due diligence on listed beneficiaries, energy assessments, and facilitating implementation of DRE solutions
-Phase 3: Capacity building, post-implementation audit, and documentation of program learnings.</t>
-        </is>
-      </c>
-      <c r="D14" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E14" s="1" t="inlineStr">
-        <is>
-          <t>Sep 17, 2026</t>
-        </is>
-      </c>
-      <c r="F14" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/tor-project-consultant-organization-dre-integration-in-pmfme-enterprises-selco-foundation-rfp-26-00351</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="95" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="inlineStr">
-        <is>
-          <t>SoW - Hiring an External Agency for Orientation and Capacity Building</t>
-        </is>
-      </c>
-      <c r="C15" s="1" t="inlineStr">
         <is>
           <t>Room to Read’s Foundational Literacy Program in Jharkhand: Anchoring and Delivery of Orientation Programme for Jharkhand Field Workforce
 Scope of Work (SoW)
@@ -1372,34 +1223,86 @@
 Meeting ID: 915 1781 4040</t>
         </is>
       </c>
-      <c r="D15" s="1" t="inlineStr">
+      <c r="D12" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E15" s="1" t="inlineStr">
+      <c r="E12" s="1" t="inlineStr">
         <is>
           <t>Sep 17, 2026</t>
         </is>
       </c>
-      <c r="F15" s="1" t="inlineStr">
+      <c r="F12" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/sow-hiring-an-external-agency-for-orientation-and-capacity-building-room-to-read-india-rfp-26-00346</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="95" customHeight="1">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B16" s="1" t="inlineStr">
+    <row r="13" ht="95" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>ToR - Project Consultant / Organization DRE Integration in PMFME Enterprises</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>Terms of Reference (TOR) for Consultancy Services
+PowerUp PMFME-DRE 
+Integrating Decentralized Renewable Energy (DRE) in PMFME Food Processing Enterprises
+Title Project Consultant / Organization – DRE Integration in PMFME Enterprises
+Location
+Karnataka and Maharashtra.
+Bidders may apply for both states as a single assignment, or as a consortium with a designated lead entity covering both.
+Timeline 6 (six) Months
+Expected area of expertise Energy assessment, project implementation, financial analysis, capacity building, post-implementation audit, and documentation
+Apply Link https://forms.gle/gAmuuSxm3MkLofpF9
+Last Date for Apply 17th Sep 2026, 5 PM
+About SELCO Foundation:
+SELCO Foundation is an open-source, not-for-profit organization that engages in field-based R&amp;D and ecosystem building for the deployment of clean energy solutions that alleviate poverty by improving access to sustainable energy to underserved communities in tribal, rural, and urban poor areas. The organization works in collaboration with practitioners in the social sector, energy entrepreneurs, NGOs from various developmental sectors, and educational institutions to link the benefits of sustainable energy to poverty eradication. The organization works across verticals such as energy access, health, and livelihoods. You can find more information about the SELCO Foundation on our website: http://www.selcofoundation.org/
+Summary of the Project:
+SELCO Foundation is working to integrate Decentralized Renewable Energy (DRE) solutions into micro food processing enterprises supported under the PM Formalisation of Micro Food Processing Enterprises (PMFME) scheme. The program aims to improve energy access and productivity for PMFME beneficiaries in Karnataka and Maharashtra, targeting a total of 500 sites for DRE integration.
+A Project Consultant/Organization may apply to coordinate and facilitate site-level implementation across these two states, ensuring interventions align with beneficiary needs and have a meaningful impact.
+Goals and Objectives
+The program's key objectives are:
+Phase 1: Designing standardized DRE system options by system size, with leverage components identified for each - validated through a preliminary long/short list and sample site visits
+Phase 2: Conducting due diligence on listed beneficiaries, energy assessments, and facilitating implementation of DRE solutions
+Phase 3: Capacity building, post-implementation audit, and documentation of program learnings.</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>Sep 17, 2026</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/tor-project-consultant-organization-dre-integration-in-pmfme-enterprises-selco-foundation-rfp-26-00351</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="95" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>ToR for Consultancy Service - Practitioner Knowledge Mapping Across Priority Livelihood Value Chains</t>
         </is>
       </c>
-      <c r="C16" s="1" t="inlineStr">
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>Terms of Reference (TOR) for Consultancy Services
 Title Practitioner Knowledge Mapping Across Priority Livelihood Value Chains
@@ -1434,34 +1337,34 @@
 The agency is expected to independently identify and curate knowledge resources beyond those shared by the programme team</t>
         </is>
       </c>
-      <c r="D16" s="1" t="inlineStr">
+      <c r="D14" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E16" s="1" t="inlineStr">
+      <c r="E14" s="1" t="inlineStr">
         <is>
           <t>Sep 18, 2026</t>
         </is>
       </c>
-      <c r="F16" s="1" t="inlineStr">
+      <c r="F14" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-for-consultancy-service-practitioner-knowledge-mapping-across-priority-livelihood-value-chains-selco-foundation-rfp-26-00350</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="95" customHeight="1">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B17" s="1" t="inlineStr">
+    <row r="15" ht="95" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>ToR - Behavioural Insights and Narrative Inquiry for the Climate Responsive Livelihood Programme Meghalaya</t>
         </is>
       </c>
-      <c r="C17" s="1" t="inlineStr">
+      <c r="C15" s="1" t="inlineStr">
         <is>
           <t>Title  Behavioural Insights and Narrative Inquiry for the Climate Responsive Livelihood Programme, Meghalaya
 Timeline  2 months
@@ -1479,34 +1382,34 @@
 Rather than evaluating awareness or testing communication materials, the assignment should seek to uncover deeper behavioural and social drivers that influence livelihood choices and participation. The findings will inform a narrative architecture and mobilisation approach that resonates authentically with communities across the state.</t>
         </is>
       </c>
-      <c r="D17" s="1" t="inlineStr">
+      <c r="D15" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E17" s="1" t="inlineStr">
+      <c r="E15" s="1" t="inlineStr">
         <is>
           <t>Sep 19, 2026</t>
         </is>
       </c>
-      <c r="F17" s="1" t="inlineStr">
+      <c r="F15" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-behavioural-insights-and-narrative-inquiry-for-the-climate-responsive-livelihood-programme-meghalaya-selco-foundation-rfp-26-00355</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="95" customHeight="1">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="inlineStr">
+    <row r="16" ht="95" customHeight="1">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>RFP - Agronomic Research Study For Natural Dye Crop Development</t>
         </is>
       </c>
-      <c r="C18" s="1" t="inlineStr">
+      <c r="C16" s="1" t="inlineStr">
         <is>
           <t>REǪUEST FOR PROPOSALS (RFP)
 Agronomic Research Study For Natural Dye Crop Development
@@ -1565,34 +1468,107 @@
 Experience working on natural dye</t>
         </is>
       </c>
-      <c r="D18" s="1" t="inlineStr">
+      <c r="D16" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E18" s="1" t="inlineStr">
+      <c r="E16" s="1" t="inlineStr">
         <is>
           <t>Sep 20, 2026</t>
         </is>
       </c>
-      <c r="F18" s="1" t="inlineStr">
+      <c r="F16" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfp-agronomic-research-study-for-natural-dye-crop-development-chitrika-rfp-26-00344</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="95" customHeight="1">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="inlineStr">
+    <row r="17" ht="95" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>E-Tender Request for Digital Communication Website Development and Social Media Campaign for Colors of Nature</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>REǪUEST FOR PROPOSALS (RFP)
+Digital Communication, Website Development and Social Media Campaign
+Colors of Nature Project
+Parameter Details
+Reference COLORS/DFRǪ/20260002
+Title E-Tender Request for Digital Communication, Website Development and Social Media Campaign for Colors of Nature (Activity A.2.1)
+Timeline 31st August 2026 – 31 July 2029 (3 years)
+Area of Expertise Website, Digital Marketing
+Submission Deadline 20th September 2026
+Budget Head
+5.8.4 - Website
+6.3.3 - Social Media Campaign
+Requirements Proposal for website and social media campaign to be submitted separately
+Background
+The COLORS of Nature project, co-funded by the European Union and implemented by Welthungerhilfe with partners Avani Society and Chitrika (ALAF), aims to advance circular textile production in India through plant-based dyes. The project targets 15,000 smallholder farmers and artisans across Uttarakhand, Telangana, and Andhra Pradesh (2025–2029).
+As the project progresses, there is a need to establish a strong digital identity that documents the project's journey, showcases its impact, creates awareness among consumers, and positions Colors Of Nature as a long-term knowledge and collaboration platform for natural dyes beyond the life of the project.
+Objective
+To conceptualise, design, develop and manage an integrated digital communication ecosystem for Colors Of Nature, comprising:
+Social media platforms
+Digital storytelling
+Knowledge documentation
+Consumer awareness campaigns
+Multimedia communication products
+Brand identity development
+The platform should serve not merely as a project communication tool but as a lasting digital destination for natural dyes in India.
+Specific Objectives
+The selected agency shall work towards the following objectives:
+Establish Colors Of Nature platform as a recognised digital identity for natural dyes.
+Build awareness among at least 100,000 consumers on the environmental, cultural and livelihood significance of natural dyes through planned digital campaigns.
+Ensure appropriate visibility to the European Union and Welthungerhilfe (WHH) in accordance with donor communication and visibility guidelines.
+Create opportunities for future collaborations with designers, educational institutions, buyers, researchers and sustainability practitioners.
+Build a digital footprint that continues to remain relevant beyond the project period.
+Desired Profile oF the Agency
+The project seeks to engage a young, creative and mission-driven communication agency, digital collective or social enterprise rather than a conventional large communication firm.
+Preference shall be given to agencies that:
+Demonstrate innovation, creativity and agility.
+Have experience in development communication.
+Have exposure to rural livelihoods, sustainability, crafts, agriculture or textiles.
+Are willing to mentor and build a dedicated communications team to manage website content, digital campaigns and communication products over time.
+Demonstrate strong storytelling capabilities.
+Operate through lean and cost-effective implementation models while maintaining high quality standards.
+Ready to develop a women led and based digital marketing team</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>Sep 20, 2026</t>
+        </is>
+      </c>
+      <c r="F17" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/e-tender-request-for-digital-communication-website-development-and-social-media-campaign-for-colors-of-nature-chitrika-rfp-26-00342</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="95" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>RFP - Research Collaboration For Improved Application and Processing Techniques For Natural Dyes</t>
         </is>
       </c>
-      <c r="C19" s="1" t="inlineStr">
+      <c r="C18" s="1" t="inlineStr">
         <is>
           <t>REǪUEST FOR PROPOSALS (RFP)
 Research Collaboration For Improved Application and Processing Techniques For Natural Dyes
@@ -1645,34 +1621,34 @@
 Network with dyeing units and textile industry associations</t>
         </is>
       </c>
-      <c r="D19" s="1" t="inlineStr">
+      <c r="D18" s="1" t="inlineStr">
         <is>
           <t>Climate</t>
         </is>
       </c>
-      <c r="E19" s="1" t="inlineStr">
+      <c r="E18" s="1" t="inlineStr">
         <is>
           <t>Sep 20, 2026</t>
         </is>
       </c>
-      <c r="F19" s="1" t="inlineStr">
+      <c r="F18" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfp-research-collaboration-for-improved-application-and-processing-techniques-for-natural-dyes-chitrika-rfp-26-00343</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="95" customHeight="1">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="inlineStr">
+    <row r="19" ht="95" customHeight="1">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>Expression of Interest EOI for Trade &amp; Livelihood Partners</t>
         </is>
       </c>
-      <c r="C20" s="1" t="inlineStr">
+      <c r="C19" s="1" t="inlineStr">
         <is>
           <t>Expression of Interest (EOI) for Trade &amp; Livelihood Partners
 Issued By: BharatCares
@@ -1799,107 +1775,34 @@
 Any prior work with tribal or rural communities, with references if available</t>
         </is>
       </c>
-      <c r="D20" s="1" t="inlineStr">
+      <c r="D19" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E20" s="1" t="inlineStr">
+      <c r="E19" s="1" t="inlineStr">
         <is>
           <t>Sep 20, 2026</t>
         </is>
       </c>
-      <c r="F20" s="1" t="inlineStr">
+      <c r="F19" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/expression-of-interest-eoi-for-trade-and-livelihood-partners-bharatcares-rfp-26-00340</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="95" customHeight="1">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="inlineStr">
-        <is>
-          <t>E-Tender Request for Digital Communication Website Development and Social Media Campaign for Colors of Nature</t>
-        </is>
-      </c>
-      <c r="C21" s="1" t="inlineStr">
-        <is>
-          <t>REǪUEST FOR PROPOSALS (RFP)
-Digital Communication, Website Development and Social Media Campaign
-Colors of Nature Project
-Parameter Details
-Reference COLORS/DFRǪ/20260002
-Title E-Tender Request for Digital Communication, Website Development and Social Media Campaign for Colors of Nature (Activity A.2.1)
-Timeline 31st August 2026 – 31 July 2029 (3 years)
-Area of Expertise Website, Digital Marketing
-Submission Deadline 20th September 2026
-Budget Head
-5.8.4 - Website
-6.3.3 - Social Media Campaign
-Requirements Proposal for website and social media campaign to be submitted separately
-Background
-The COLORS of Nature project, co-funded by the European Union and implemented by Welthungerhilfe with partners Avani Society and Chitrika (ALAF), aims to advance circular textile production in India through plant-based dyes. The project targets 15,000 smallholder farmers and artisans across Uttarakhand, Telangana, and Andhra Pradesh (2025–2029).
-As the project progresses, there is a need to establish a strong digital identity that documents the project's journey, showcases its impact, creates awareness among consumers, and positions Colors Of Nature as a long-term knowledge and collaboration platform for natural dyes beyond the life of the project.
-Objective
-To conceptualise, design, develop and manage an integrated digital communication ecosystem for Colors Of Nature, comprising:
-Social media platforms
-Digital storytelling
-Knowledge documentation
-Consumer awareness campaigns
-Multimedia communication products
-Brand identity development
-The platform should serve not merely as a project communication tool but as a lasting digital destination for natural dyes in India.
-Specific Objectives
-The selected agency shall work towards the following objectives:
-Establish Colors Of Nature platform as a recognised digital identity for natural dyes.
-Build awareness among at least 100,000 consumers on the environmental, cultural and livelihood significance of natural dyes through planned digital campaigns.
-Ensure appropriate visibility to the European Union and Welthungerhilfe (WHH) in accordance with donor communication and visibility guidelines.
-Create opportunities for future collaborations with designers, educational institutions, buyers, researchers and sustainability practitioners.
-Build a digital footprint that continues to remain relevant beyond the project period.
-Desired Profile oF the Agency
-The project seeks to engage a young, creative and mission-driven communication agency, digital collective or social enterprise rather than a conventional large communication firm.
-Preference shall be given to agencies that:
-Demonstrate innovation, creativity and agility.
-Have experience in development communication.
-Have exposure to rural livelihoods, sustainability, crafts, agriculture or textiles.
-Are willing to mentor and build a dedicated communications team to manage website content, digital campaigns and communication products over time.
-Demonstrate strong storytelling capabilities.
-Operate through lean and cost-effective implementation models while maintaining high quality standards.
-Ready to develop a women led and based digital marketing team</t>
-        </is>
-      </c>
-      <c r="D21" s="1" t="inlineStr">
-        <is>
-          <t>Learning</t>
-        </is>
-      </c>
-      <c r="E21" s="1" t="inlineStr">
-        <is>
-          <t>Sep 20, 2026</t>
-        </is>
-      </c>
-      <c r="F21" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/e-tender-request-for-digital-communication-website-development-and-social-media-campaign-for-colors-of-nature-chitrika-rfp-26-00342</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="95" customHeight="1">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="inlineStr">
+    <row r="20" ht="95" customHeight="1">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Wellbeing Research Grants Funding Better Evaluations of AI's Impact on Wellbeing</t>
         </is>
       </c>
-      <c r="C22" s="1" t="inlineStr">
+      <c r="C20" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We're an AI research company that builds reliable, interpretable, and steerable AI systems. Our first product is Claude, an AI assistant for tasks at any scale. Our research interests span multiple areas including natural language, human feedback, scaling laws, reinforcement learning, code generation, and interpretability. 
@@ -1918,34 +1821,34 @@
  Funding Amount: Total program pool of $5 million (individual grant sizes not specified on the page)</t>
         </is>
       </c>
-      <c r="D22" s="1" t="inlineStr">
+      <c r="D20" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E22" s="1" t="inlineStr">
+      <c r="E20" s="1" t="inlineStr">
         <is>
           <t>Sep 21, 2026</t>
         </is>
       </c>
-      <c r="F22" s="1" t="inlineStr">
+      <c r="F20" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-wellbeing-research-grants-funding-better-evaluations-of-ais-impact-on-wellbeing-anthropic-opg-26-00175</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="95" customHeight="1">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B23" s="1" t="inlineStr">
+    <row r="21" ht="95" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for GEF SGP CSO Challenge Program</t>
         </is>
       </c>
-      <c r="C23" s="1" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global Environment Facility Small Grants Programme (SGP) is a global initiative implemented by the United Nations Development Programme (UNDP) on behalf of the Global Environment Facility (GEF). Since its launch in 1992, SGP has empowered communities worldwide to take action on environmental challenges while improving livelihoods. As a GEF Corporate Programme, SGP provides direct support to civil society organisations and community-based organisations to design and implement innovative, locally driven solutions. The programme places strong emphasis on inclusion, ensuring meaningful participation of Indigenous Peoples, youth, women and girls, and other underrepresented groups.
@@ -1994,34 +1897,34 @@
 Risk management and mitigation</t>
         </is>
       </c>
-      <c r="D23" s="1" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E23" s="1" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>Sep 23, 2026</t>
         </is>
       </c>
-      <c r="F23" s="1" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-gef-sgp-cso-challenge-program-gef-small-grants-programme-sgp-opg-26-00184</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="95" customHeight="1">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B24" s="1" t="inlineStr">
+    <row r="22" ht="95" customHeight="1">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
         <is>
           <t>RFP for Impact Assessment</t>
         </is>
       </c>
-      <c r="C24" s="1" t="inlineStr">
+      <c r="C22" s="1" t="inlineStr">
         <is>
           <t>Introduction
 Titan Company Limited, a member of the Tata Group, has a long-standing commitment to Corporate Social Responsibility (CSR) in India. The company's CSR initiatives derive its philosophy from the Company’s vision statement: “We create elevating experiences for the people we touch and significantly impact the world we work in”. The initiatives are designed to promote inclusive growth, empower communities, and contribute to the country's socio-economic development. The program includes Titan’s CSR policy is governed by a dedicated CSR Committee that ensures transparency and compliance with regulatory requirements. The program includes Girl Child Education, Skill and Entrepreneurship Development, supporting Indian Heritage Arts and Crafts, Integrated Village Development Programme, Eye Care and Affirmative Action. Titan's CSR policy is governed by a dedicated CSR Committee that ensures transparency and compliance with regulatory requirements.
@@ -2055,34 +1958,86 @@
 Timeline: Proposal submission deadline: September 24, 2026</t>
         </is>
       </c>
-      <c r="D24" s="1" t="inlineStr">
+      <c r="D22" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E24" s="1" t="inlineStr">
+      <c r="E22" s="1" t="inlineStr">
         <is>
           <t>Sep 24, 2026</t>
         </is>
       </c>
-      <c r="F24" s="1" t="inlineStr">
+      <c r="F22" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfp-for-impact-assessment-titan-rfp-26-00354</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="95" customHeight="1">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B25" s="1" t="inlineStr">
+    <row r="23" ht="95" customHeight="1">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Signals of Change Shaping the Future of Sexual and Reproductive Health and Rights SRHR</t>
+        </is>
+      </c>
+      <c r="C23" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+The World Health Organization's mission: to promote health, keep the world safe, and serve the vulnerable. Working through offices in more than 150 countries, WHO staff work side by side with governments and other partners to ensure the highest attainable level of health for all people.
+ About the Opportunity
+HRP and its UN co-sponsors are leading a global Sexual and Reproductive Health and Rights (SRHR) foresight and research prioritization process for 2026–2036. This open public consultation invites diverse stakeholder input to identify "signals of change" — emerging trends, shifts, or disruptions — that could shape the future of SRHR over the next decade. The process uses foresight methodology (not prediction) to explore plausible futures and will culminate in a published report and research agenda in 2027.
+ Guiding Questions
+What future trends will shape or constrain SRHR over the next 10 years?
+What evidence and research investments are needed today to prepare SRHR for the futures we may face?
+ Scope of Submissions 
+Economic systems; social infrastructure; structural discrimination; conflict/forced migration/displacement; mega-trends (demographic shifts, climate change, digital transformation/AI, urbanization); conditions of daily life; rights/legal/governance systems; health systems; media/misinformation; and changes in the research ecosystem.
+ Who Can Participate 
+Open to individuals and organizations globally, including:
+Health workers, professional associations, clinical networks
+Civil society, community groups, youth-led organizations, rights movements
+Governments, parliamentarians, regulators, public sector bodies
+Researchers, academia, think tanks, technical experts
+UN agencies, multilateral/humanitarian/development organizations
+Funders, philanthropy, private sector, tech/innovation organizations
+Media, communications, journalism
+Anyone with relevant lived experience or perspective
+Special interest in submissions from health worker, community, youth, and rights-movement spaces not typically represented in published forums.
+ Submission Requirements: Descriptive information (name, contact email, country, sector) required alongside each submission; formal published evidence is helpful but not required — practice-based experience and field examples are also welcome. Submissions are kept confidential and anonymized before analysis.</t>
+        </is>
+      </c>
+      <c r="D23" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E23" s="1" t="inlineStr">
+        <is>
+          <t>Sep 30, 2026</t>
+        </is>
+      </c>
+      <c r="F23" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-signals-of-change-shaping-the-future-of-sexual-and-reproductive-health-and-rights-srhr-world-health-organization-opg-26-00176</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="95" customHeight="1">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
         <is>
           <t>EOI Inviting Expression of Interest-cum-Proposal for Setting Up District De-Addiction Centres under NAPDDR</t>
         </is>
       </c>
-      <c r="C25" s="1" t="inlineStr">
+      <c r="C24" s="1" t="inlineStr">
         <is>
           <t>About us
 In the year 1985-86, the erstwhile Ministry of Welfare was bifurcated into the Department of Women and Child Development and the Department of Welfare. Simultaneously, the Scheduled Castes Development Division, Tribal Development Division and the Minorities and Backward Classes Welfare Division were moved from the Ministry of Home Affairs and also the Wakf Division from the Ministry of Law to form the then Ministry of Welfare Subsequently, the name of the Ministry was changed to the Ministry of Social Justice &amp; Empowerment in May, 1998. Further, in October, 1999, the Tribal Development Division had moved out to form a separate Ministry of Tribal Affairs. In January, 2007, the Minorities Division along with Wakf Unit have been moved out of the Ministry and formed as a separate Ministry and the Child Development Division has gone to the Ministry of Women &amp; Child Development.
@@ -2122,34 +2077,34 @@
 11. Department of Social Justice and Empowerment (DoSJE) reserves the right to cancel this notice, andior invite afresh proposals with or without amendments to this document without liability or any obligation for such document, and without assigning any reason. DoSJE reserves the right to take final decision regarding selection of implementing agency or project.</t>
         </is>
       </c>
-      <c r="D25" s="1" t="inlineStr">
+      <c r="D24" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E25" s="1" t="inlineStr">
+      <c r="E24" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F25" s="1" t="inlineStr">
+      <c r="F24" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/eoi-inviting-expression-of-interest-cum-proposal-for-setting-up-district-de-addiction-centres-under-napddr-ministry-of-social-justice-and-empowerment-goi-rfp-26-00356</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="95" customHeight="1">
-      <c r="A26" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B26" s="1" t="inlineStr">
+    <row r="25" ht="95" customHeight="1">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
         <is>
           <t>Application Invited for Giving Joy Microgrant</t>
         </is>
       </c>
-      <c r="C26" s="1" t="inlineStr">
+      <c r="C25" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Giving Joy is a US-based nonprofit that strengthens and inspires women’s entrepreneurship worldwide. Through its micro-grants and mentorship program, Giving Joy helps women establish or improve their businesses and initiatives—for their benefit and the benefit of their communities. To date, Giving Joy has awarded over 88 grants to women-led initiatives in 26 countries.
@@ -2188,34 +2143,34 @@
 The grant period is six months.</t>
         </is>
       </c>
-      <c r="D26" s="1" t="inlineStr">
+      <c r="D25" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E26" s="1" t="inlineStr">
+      <c r="E25" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F26" s="1" t="inlineStr">
+      <c r="F25" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/application-invited-for-giving-joy-microgrant-giving-joy-opg-26-00185</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="95" customHeight="1">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B27" s="1" t="inlineStr">
+    <row r="26" ht="95" customHeight="1">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Setting up Viral Research and Diagnosis Laboratories VRDL in Medical Colleges/Hospitals/Medical Institutions</t>
         </is>
       </c>
-      <c r="C27" s="1" t="inlineStr">
+      <c r="C26" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The President notified the creation of the Department of Health Research under the Ministry of Health &amp; Family Welfare through an amendment to the Government of India (Allocation of Business) Rules, 1961 on the 17th September 2007. The Department of Health Research was formally launched on 5th October 2007 by the Minister for Science &amp; Technology and Earth Sciences in a function presided over by the Minister for Health &amp; Family Welfare, in the presence, inter-alia, of the Minister of State for Health &amp; Family Welfare.
@@ -2252,86 +2207,34 @@
 Private medical colleges: only top-50 NIRF-ranked institutions considered</t>
         </is>
       </c>
-      <c r="D27" s="1" t="inlineStr">
+      <c r="D26" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E27" s="1" t="inlineStr">
+      <c r="E26" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F27" s="1" t="inlineStr">
+      <c r="F26" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-setting-up-viral-research-and-diagnosis-laboratories-vrdl-in-medical-collegeshospitalsmedical-institutions-department-of-health-research-dhr-ministry-of-health-and-family-welfare-government-of-india-opg-26-00174</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="95" customHeight="1">
-      <c r="A28" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B28" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Signals of Change Shaping the Future of Sexual and Reproductive Health and Rights SRHR</t>
-        </is>
-      </c>
-      <c r="C28" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-The World Health Organization's mission: to promote health, keep the world safe, and serve the vulnerable. Working through offices in more than 150 countries, WHO staff work side by side with governments and other partners to ensure the highest attainable level of health for all people.
- About the Opportunity
-HRP and its UN co-sponsors are leading a global Sexual and Reproductive Health and Rights (SRHR) foresight and research prioritization process for 2026–2036. This open public consultation invites diverse stakeholder input to identify "signals of change" — emerging trends, shifts, or disruptions — that could shape the future of SRHR over the next decade. The process uses foresight methodology (not prediction) to explore plausible futures and will culminate in a published report and research agenda in 2027.
- Guiding Questions
-What future trends will shape or constrain SRHR over the next 10 years?
-What evidence and research investments are needed today to prepare SRHR for the futures we may face?
- Scope of Submissions 
-Economic systems; social infrastructure; structural discrimination; conflict/forced migration/displacement; mega-trends (demographic shifts, climate change, digital transformation/AI, urbanization); conditions of daily life; rights/legal/governance systems; health systems; media/misinformation; and changes in the research ecosystem.
- Who Can Participate 
-Open to individuals and organizations globally, including:
-Health workers, professional associations, clinical networks
-Civil society, community groups, youth-led organizations, rights movements
-Governments, parliamentarians, regulators, public sector bodies
-Researchers, academia, think tanks, technical experts
-UN agencies, multilateral/humanitarian/development organizations
-Funders, philanthropy, private sector, tech/innovation organizations
-Media, communications, journalism
-Anyone with relevant lived experience or perspective
-Special interest in submissions from health worker, community, youth, and rights-movement spaces not typically represented in published forums.
- Submission Requirements: Descriptive information (name, contact email, country, sector) required alongside each submission; formal published evidence is helpful but not required — practice-based experience and field examples are also welcome. Submissions are kept confidential and anonymized before analysis.</t>
-        </is>
-      </c>
-      <c r="D28" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E28" s="1" t="inlineStr">
-        <is>
-          <t>Sep 30, 2026</t>
-        </is>
-      </c>
-      <c r="F28" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-signals-of-change-shaping-the-future-of-sexual-and-reproductive-health-and-rights-srhr-world-health-organization-opg-26-00176</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="95" customHeight="1">
-      <c r="A29" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B29" s="1" t="inlineStr">
+    <row r="27" ht="95" customHeight="1">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund</t>
         </is>
       </c>
-      <c r="C29" s="1" t="inlineStr">
+      <c r="C27" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund
 Apply by: 13 October, 2026
@@ -2356,34 +2259,34 @@
  Projects should include opportunities for ServiceNow employees to volunteer in the project activation or implementation.</t>
         </is>
       </c>
-      <c r="D29" s="1" t="inlineStr">
+      <c r="D27" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E29" s="1" t="inlineStr">
+      <c r="E27" s="1" t="inlineStr">
         <is>
           <t>Oct 13, 2026</t>
         </is>
       </c>
-      <c r="F29" s="1" t="inlineStr">
+      <c r="F27" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/apply-for-the-servicenow-community-solar-fund-changex-opg-26-00186</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="95" customHeight="1">
-      <c r="A30" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B30" s="1" t="inlineStr">
+    <row r="28" ht="95" customHeight="1">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 8th Call for Proposals Small-Size Grants Global EbA Fund</t>
         </is>
       </c>
-      <c r="C30" s="1" t="inlineStr">
+      <c r="C28" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -2446,34 +2349,34 @@
 Only successful applicants will be contacted; no individual feedback provided to unsuccessful applicants</t>
         </is>
       </c>
-      <c r="D30" s="1" t="inlineStr">
+      <c r="D28" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E30" s="1" t="inlineStr">
+      <c r="E28" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F30" s="1" t="inlineStr">
+      <c r="F28" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-8th-call-for-proposals-small-size-grants-global-eba-fund-global-eba-fund-opg-26-00177</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="95" customHeight="1">
-      <c r="A31" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B31" s="1" t="inlineStr">
+    <row r="29" ht="95" customHeight="1">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIFAR Global Scholars Program 20272029 Cohort</t>
         </is>
       </c>
-      <c r="C31" s="1" t="inlineStr">
+      <c r="C29" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 CIFAR is a Canadian-based globally influential research organization that convenes the world’s most brilliant people across disciplines to advance transformative knowledge and solve humanity’s biggest problems, together. By supporting long-term interdisciplinary collaboration, CIFAR provides researchers with an unparalleled environment of trust, transparency and knowledge sharing. Our time-tested model inspires new directions of inquiry, accelerates discovery and yields breakthroughs across borders and academic disciplines. Through knowledge mobilization, we are catalysts for change in industry, government and society. Through our 15 research programs and the Pan-Canadian AI Strategy, CIFAR convenes close to 400 of the world’s top researchers from 141 institutions in 20 countries. CIFAR is generously supported by the governments of Canada, Alberta and Québec, as well as foundations, individuals, corporations and Canadian and international partner organizations.
@@ -2517,34 +2420,34 @@
  Application Deadline: November 4, 2026, 12:00 PM EST</t>
         </is>
       </c>
-      <c r="D31" s="1" t="inlineStr">
+      <c r="D29" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E31" s="1" t="inlineStr">
+      <c r="E29" s="1" t="inlineStr">
         <is>
           <t>Nov 4, 2026</t>
         </is>
       </c>
-      <c r="F31" s="1" t="inlineStr">
+      <c r="F29" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cifar-global-scholars-program-20272029-cohort-cifar-canadian-institute-for-advanced-research-opg-26-00183</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="95" customHeight="1">
-      <c r="A32" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B32" s="1" t="inlineStr">
+    <row r="30" ht="95" customHeight="1">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for IWRS Teaching Innovation Award</t>
         </is>
       </c>
-      <c r="C32" s="1" t="inlineStr">
+      <c r="C30" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
@@ -2556,34 +2459,34 @@
 Two awards of $2,000 USD are available annually.</t>
         </is>
       </c>
-      <c r="D32" s="1" t="inlineStr">
+      <c r="D30" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E32" s="1" t="inlineStr">
+      <c r="E30" s="1" t="inlineStr">
         <is>
           <t>Nov 15, 2026</t>
         </is>
       </c>
-      <c r="F32" s="1" t="inlineStr">
+      <c r="F30" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="95" customHeight="1">
-      <c r="A33" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B33" s="1" t="inlineStr">
+    <row r="31" ht="95" customHeight="1">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for IWRS Teaching Innovation Award</t>
         </is>
       </c>
-      <c r="C33" s="1" t="inlineStr">
+      <c r="C31" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Insects are one of the most numerous and diverse animal groups on Earth.
@@ -2598,34 +2501,34 @@
 IWRS staff and Advisory Group members are not eligible to apply.</t>
         </is>
       </c>
-      <c r="D33" s="1" t="inlineStr">
+      <c r="D31" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E33" s="1" t="inlineStr">
+      <c r="E31" s="1" t="inlineStr">
         <is>
           <t>Nov 15, 2026</t>
         </is>
       </c>
-      <c r="F33" s="1" t="inlineStr">
+      <c r="F31" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00166</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="95" customHeight="1">
-      <c r="A34" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B34" s="1" t="inlineStr">
+    <row r="32" ht="95" customHeight="1">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B32" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Medium-Size Grants Call for Proposals Global EbA Fund</t>
         </is>
       </c>
-      <c r="C34" s="1" t="inlineStr">
+      <c r="C32" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -2682,34 +2585,34 @@
 Applications submitted via online portal (link shared on the Medium-Size Grants webpage from Oct 12)</t>
         </is>
       </c>
-      <c r="D34" s="1" t="inlineStr">
+      <c r="D32" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E34" s="1" t="inlineStr">
+      <c r="E32" s="1" t="inlineStr">
         <is>
           <t>Nov 16, 2026</t>
         </is>
       </c>
-      <c r="F34" s="1" t="inlineStr">
+      <c r="F32" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-medium-size-grants-call-for-proposals-global-eba-fund-global-eba-fund-opg-26-00178</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="95" customHeight="1">
-      <c r="A35" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B35" s="1" t="inlineStr">
+    <row r="33" ht="95" customHeight="1">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B33" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIEIF Grant 2026 Climate Intervention Environmental Impact Fund</t>
         </is>
       </c>
-      <c r="C35" s="1" t="inlineStr">
+      <c r="C33" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Climate Intervention Environmental Impact Fund (CIEIF) is a philanthropic fund focused on supporting responsible climate intervention field tests. It provides grants for activities such as environmental impact assessment (EIA), predictive impact modelling, and engagement with potentially affected stakeholders, including local communities and government agencies.
@@ -2736,34 +2639,34 @@
 Potential for scaling the innovation to a globally relevant level</t>
         </is>
       </c>
-      <c r="D35" s="1" t="inlineStr">
+      <c r="D33" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E35" s="1" t="inlineStr">
+      <c r="E33" s="1" t="inlineStr">
         <is>
           <t>Dec 1, 2026</t>
         </is>
       </c>
-      <c r="F35" s="1" t="inlineStr">
+      <c r="F33" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cieif-grant-2026-climate-intervention-environmental-impact-fund-climate-intervention-environmental-impact-fund-opg-26-00155</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="95" customHeight="1">
-      <c r="A36" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B36" s="1" t="inlineStr">
+    <row r="34" ht="95" customHeight="1">
+      <c r="A34" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B34" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 6th Annual Seeding The Future Global Food System Challenge</t>
         </is>
       </c>
-      <c r="C36" s="1" t="inlineStr">
+      <c r="C34" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are one of the largest and most respected private organisations for development cooperation and humanitarian aid in Germany. As a politically and confessionally independent organisation, our value-oriented actions are always based on ethical principles. Our vision is clear: "Zero Hunger by 2030"
@@ -2795,34 +2698,34 @@
 Individuals with no organizational entity</t>
         </is>
       </c>
-      <c r="D36" s="1" t="inlineStr">
+      <c r="D34" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E36" s="1" t="inlineStr">
+      <c r="E34" s="1" t="inlineStr">
         <is>
           <t>Jan 1, 2027</t>
         </is>
       </c>
-      <c r="F36" s="1" t="inlineStr">
+      <c r="F34" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-6th-annual-seeding-the-future-global-food-system-challenge-welthungerhilfe-opg-26-00180</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="95" customHeight="1">
-      <c r="A37" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B37" s="1" t="inlineStr">
+    <row r="35" ht="95" customHeight="1">
+      <c r="A35" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B35" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for BES Training and Travel Grants</t>
         </is>
       </c>
-      <c r="C37" s="1" t="inlineStr">
+      <c r="C35" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are a global community of scientists shining a spotlight on the intricacy and value of our natural world, providing the evidence for better decisions. Our vision is for people and nature to thrive in a world that values ecology.
@@ -2861,17 +2764,17 @@
  Application Deadline (Round 2): Opens 30 April 2026, closes 17 May 2026</t>
         </is>
       </c>
-      <c r="D37" s="1" t="inlineStr">
+      <c r="D35" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E37" s="1" t="inlineStr">
+      <c r="E35" s="1" t="inlineStr">
         <is>
           <t>May 17, 2027</t>
         </is>
       </c>
-      <c r="F37" s="1" t="inlineStr">
+      <c r="F35" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-bes-training-and-travel-grants-british-ecological-society-opg-26-00181</t>
         </is>

</xml_diff>

<commit_message>
Auto update Combined.xlsx [Mon Sep 14 07:30:45 UTC 2026]
</commit_message>
<xml_diff>
--- a/output/Combined.xlsx
+++ b/output/Combined.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -467,568 +467,10 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Application Invited For India Fund</t>
+          <t>ToR - Development of WaterAid India's Hygiene Framework Community Facilitator Toolkit Hygiene Booklet and Hygiene Calendar</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-Paul Hamlyn Foundation was established in 1987. Since then, we have used our resources to work towards a just future in which everyone, especially young people, can realise their full potential and enjoy fulfilling and creative lives. In all of our work, including our grant-making, we are guided by six strategic priorities where we want to see change: • Investing in young people • Migration and integration • Arts access and participation • Education and learning through the arts • Nurturing ideas and people • Creating opportunities for people and communities in India
- About the India Fund
-The India Fund supports small NGOs working with vulnerable communities in priority geographical areas of India.
-The fund is based on the principle that communities should be central to development work, with people facing disadvantage playing an important role in leading change and designing solutions to inequality.
-Strategic aims
-The fund aims to:
-Encourage NGOs to undertake community-centred development programmes.
-Enable communities to take greater control of their own development and improve their lives.
-Encourage development funding that addresses systemic change.
-Strengthen the capacity of organisations and people facilitating this work.
- Who Can Apply?
-The fund specifically supports:
-Local Indian NGOs with FCRA registration
-This is an important eligibility requirement.
-Eligible organisations should generally be:
-Indian organisations
-Locally based in the communities they serve
-Working directly with communities
-Focused on long-term improvements in community wellbeing
-Connected with relevant panchayats in rural areas or municipalities in urban areas
-Taking steps to reduce their environmental impact
-Working to improve local ecology
-Promoting gender equality
-Supporting people of all genders to participate in change-making. 
-Important
-FCRA registration is mandatory.
-PHF explicitly states that it does not work through the FCRA prior-permission route.
- Funding Amount
-₹10 lakh – ₹40 lakh</t>
-        </is>
-      </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>Sep 15, 2026</t>
-        </is>
-      </c>
-      <c r="F2" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/application-invited-for-india-fund-paul-hamlyn-foundation-opg-26-00172</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="95" customHeight="1">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>RFP - Technical Consultancy for disability inclusion and livelihood initiatives</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t>Request for Proposal (RFP)
-Bids are invited for: Technical Consultancy for disability inclusion and livelihood initiatives
-Ref: AIFT/RFP/DL/2026-27/024
-Summary of Deadlines:
-Release of Request for Proposal September 8, 2026
-Bid Submission Closing Date
-  14th September 2026 (till 13:00 HRS)
-Technical Bid Submission Link
-https://forms.gle/1kyy8yKQpmsmMw4XA
-  Financial Bid Submission Link
- https://forms.gle/PniTmy9SMBJypKuNA
-  Technical Bid Opening 14th September 2026
-Financial Bid Opening 15th September 2026 Tentative
-Finalization of Contract To be intimated to the awardee only
-Scope of work:
-Background
-Purpose of the Consultancy: The consultant will provide technical and strategic support to AIFT in strengthening the planning, implementation, monitoring and documentation of its disability inclusion and livelihood initiatives, with a focus on the ABLE and DI-verse programmes. The consultancy will provide technical inputs to the programme team, support quality implementation, strengthen stakeholder engagement, and contribute to timely and effective reporting and documentation of programme progress and outcomes.
-The American India Foundation Trust (AIFT) implements programmes aimed at promoting disability inclusion, livelihoods, employment, and equal opportunities for Persons with Disabilities (PwDs). Through initiatives such as the ABLE and DI-verse programmes, AIFT works with organisations and stakeholders to strengthen inclusive practices, build awareness and capacity, and create opportunities for greater participation of persons with disabilities.
-As these programmes involve multiple activities including organisation onboarding, assessments, certification, sensitisation, capacity building, stakeholder engagement, programme implementation, monitoring and documentation, specialised technical expertise is required to support the programme team and ensure quality and effective delivery.
-AIFT therefore seeks to engage an experienced Technical Consultant to provide technical and strategic support across the programme lifecycle, strengthen implementation and stakeholder engagement, and contribute to improved programme outcomes and documentation.
-This aligns closely with the existing SOW, which identifies the ABLE and DI-verse programmes as the focus of the consultancy.
-Objective: To engage an experienced consultant to provide technical and strategic support to AIFT in strengthening the planning, implementation, monitoring, and quality of its disability inclusion and livelihood programmes, particularly the ABLE and DI-verse programmes.
- Scope of Services
-The selected agency shall provide the following services as mentioned below
-Consultancy period: Period of Performance: tentative Start date 17/09/2026; end dates 31/03/2027. The consultancy will be for a maximum of 60 hours per month. subject to fulfillment of deliverables and requirement.
-Applicant Eligibility Requirements
-Minimum 12–15 years of professional experience, preferably in a leadership role in workplace disability inclusion and related areas.
-Demonstrated expertise and leadership in workplace disability inclusion, disability rights, accessibility, reasonable accommodation and inclusive employment practices.
-Proven experience of direct engagement and working with Persons with Disabilities (PwDs) across employment, livelihoods, skilling and inclusion initiatives.
-Significant experience working directly with corporates and employers to advance disability-inclusive workplaces, employment practices and organisational inclusion.
-Demonstrated experience as a consultant, advisor, thought leader and/or influencer in the disability inclusion ecosystem, with the ability to shape practices and influence stakeholders.
-Strong experience in programme strategy, planning, implementation, monitoring, review and technical advisory support for disability inclusion and livelihood/employment programmes.
-Proven expertise in proposal development, concept notes, programme design, donor engagement and development of strategic programme documents.
-Demonstrated experience in designing and/or implementing disability inclusion assessments, certification programmes, sensitisation initiatives and capacity-building programmes.
-Strong track record of stakeholder engagement with PwDs, corporates, employers, NGOs, donors, implementation partners, government stakeholders and subject matter experts.
-Experience in mentoring and providing technical leadership to programme teams, including reviewing progress, strengthening implementation quality and supporting organisational processes.
-Demonstrated ability to develop and review technical reports, assessment reports, donor reports, case studies, presentations and programme documentation.
-Strong communication, facilitation, influencing and relationship-management skills, with the ability to represent the organisation in external forums and stakeholder engagements.
-Experience contributing to knowledge generation, thought leadership, advocacy, conferences, consultations, publications or sector-wide discussions on workplace disability inclusion will be an added advantage.
-Applicants should demonstrate a strong professional network and credibility within the disability inclusion, corporate/HR and employment ecosystem.
-The consultant must have the availability and capacity to provide up to 60 hours of technical and strategic support per month during the consultancy period.</t>
-        </is>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>Sep 15, 2026</t>
-        </is>
-      </c>
-      <c r="F3" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/rfp-technical-consultancy-for-disability-inclusion-and-livelihood-initiatives-american-india-foundation-rfp-26-00352</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="95" customHeight="1">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>RFP - Engagement of Agency/Consultant for Programme Learning &amp; Ecosystem Study</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>Request for Proposal (RFP) Bids are invited for: Engagement of Agency/Consultant for Programme Learning &amp; Ecosystem Study
-Ref: AIFT/RFP/DL/2026-27/025
-Summary of Deadlines:
-Release of Request for Proposal 8th September 2026
-Pre-bid Meeting (Online) Date 11th September 2026 (13:00 Hrs IST)
-Pre-Bid Link for Registration: https://forms.gle/eV7xmbPhUZeMgsr18
-Bid Submission Closing Date
-  15th September 2026 (till Midnight 12:00AM)
-Technical Bid Submission Link https://forms.gle/JU6sb6kxtM9M4kxt6
-Financial Bid Submission Link https://forms.gle/HY8PJXkkFYdhwk8C6
-Technical Bid Opening 16th September 2026
-Financial Bid Opening 17th September 2026 Tentative
-Finalization of Contract To be intimated to the awardee only
-Scope of Work:
-American India Foundation Trust (AIFT) seeks to engage independent consultants or agency to conduct a Study/Research which showcases 4 year implementation journey (March 2022- July’26) of EY GDS Skill Bridge Program and evaluates the wider education and future-skills ecosystem to prepare for the next phase of the programme. The assignment should generate two standalone documents: one focused on process documentation and learning from implementation, and one focused on ecosystem and sector strategy for future positioning.  Engagement period to start from tentatively from 21st September to 30th November 2026.
- Purpose of Engagement:
-The selected bidder shall produce an honest, evidence-based Learning Document that explains what the programme set out to do, how it evolved, what worked, what did not work as intended, why, and what should change in future design as Deliverable 1. The second Deliverable should produce an Ecosystem and Sector Insight Report that helps AIF and EY GDS make strategic choices on future focus areas, geographies, partnerships, government alignment, and investment priorities in light of national and state priorities around digital learning, AI, future skills, and school-to-work pathways.
- Background
-AIFT’s Digital Equalizer programme, in partnership with EY GDS Skill Bridge, has been implemented since March 2022 across Maharashtra, Haryana, Tamil Nadu, Telangana, Odisha, and Karnataka, reaching more than 240,000 students through components such as STEM, coding, financial literacy, life skills, gender awareness, and employee engagement. While the programme has generated student-level outcomes, AIF and EY GDS want an independent reflection on whether these thematic components formed a coherent learner pathway, how employee engagement contributed, and what lessons should shape future redesign.
-The broader policy and programme context has also shifted, with NEP 2020 and subsequent national directions placing stronger emphasis on computational thinking, AI literacy, digital learning, and future-ready skills in school education. There is also increasing expectation that CSR partnerships should strengthen government systems, support scalable models, and create meaningful collaboration through volunteerism, mentoring, and school-linked support rather than one-off activities.
- Overall Objectives
-The consultant or agency will be expected to:
-Reconstruct the evolution of the Skill Bridge programme from design to implementation across the six states, and capture implementation learning in a way that is useful for AIFT and EY GDS decision-making.
-Assess whether the programme’s different components operated as an integrated learner pathway or as parallel interventions, and identify missed integration points, course corrections, and design implications.
-Analyse the broader education and future-skills ecosystem to identify policy trends, peer models, promising partnerships, and practical opportunities for a more government-aligned and AI-ready future programme model.
-Translate consultations and research into actionable strategic choices, rather than producing only descriptive reporting.
- Proposal Requirements
-Interested consultants or agencies should submit:
-Organisation or consultant profile and relevant experience.
-Two or three relevant work samples.
-Team composition and CVs of key personnel.
-Technical proposal covering proposed methodology and workplan for both Deliverables.
-At least two professional references.
-Proposals will be assessed on the ability to combine rigorous process documentation with forward-looking ecosystem analysis, and on the ability to turn research into usable strategic choices. Strong proposals should demonstrate both implementation depth and strategic breadth, with practical understanding of government-school systems, CSR partnerships, employee engagement, and AI-ready future-skills programming.</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="inlineStr">
-        <is>
-          <t>Sep 15, 2026</t>
-        </is>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/rfp-engagement-of-agencyconsultant-for-programme-learning-and-ecosystem-study-american-india-foundation-rfp-26-00353</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="95" customHeight="1">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>RFP - Selection of Agency for Conducting Street Plays for a Community Health Awareness Program</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="inlineStr">
-        <is>
-          <t>Request for Proposal / Quotation (RFP / RFQ)
-Selection of Agency for Conducting Street Plays for a Community Health Awareness Program
-Background
-A social impact organization is implementing a community health awareness initiative across multiple states in India. As part of the program, agencies are invited to conduct street plays (Nukkad Nataks) to promote preventive health awareness and engage communities. The program and funding partner details will be shared with the selected agency.
-Scope of Work
-The selected agency will be responsible for:
-Developing a street play script based on the communication brief provided.
-Translating/adapting the script into the local language, if required.
-Arranging artists, costumes, props, and sound system.
-Conducting rehearsals and performing street plays at designated locations.
-Engaging the audience through interactive performances.
-Providing photographs, videos, and a brief activity report after each performance.
-Tentative Locations
-State Location
-Goa Ponda, Canacona, Madgaon
-Gujarat Ahmedabad
-Uttar Pradesh Lucknow, Varanasi, Shravasti, Jhansi, GB Nagar (Noida)
-Please indicate the locations where your organization can conduct street plays.
-Proposal Submission
-Interested agencies are requested to submit:
-Technical Proposal
-Organization profile
-Relevant experience in street plays/health awareness campaigns
-Proposed approach and work plan
-Sample script and video of previous work (if available)
-Locations where services can be provided
-Financial Proposal
-Please share the budget for one street play, including:
-Script development
-Artist fees
-Rehearsals
-Travel &amp; logistics
-Props &amp; costumes
-Sound system
-Documentation
-Taxes (if applicable)
-Deliverables
-Approved street play script
-Successful execution of performances
-Audience engagement
-Photographs and videos
-Brief activity report
-Evaluation Criteria
-Proposals will be evaluated based on:
-Relevant experience
-Technical approach
-Creative concept
-Geographic coverage
-Cost-effectiveness</t>
-        </is>
-      </c>
-      <c r="D5" s="1" t="inlineStr">
-        <is>
-          <t>Safety</t>
-        </is>
-      </c>
-      <c r="E5" s="1" t="inlineStr">
-        <is>
-          <t>Sep 15, 2026</t>
-        </is>
-      </c>
-      <c r="F5" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/rfp-selection-of-agency-for-conducting-street-plays-for-a-community-health-awareness-program-bharatcares-rfp-26-00321</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="95" customHeight="1">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>Application Invited For 2026 Call for Proposals Mountains ADAPT Small Grants</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-UNEP is the leading global environmental authority that sets the world's environmental agenda, promotes the coherent implementation of the environmental dimension of sustainable development within the United Nations system and serves as an authoritative advocate for the environment.
- About the Grant
-The Mountains ADAPT Small Grants Project supports community-based organizations in implementing practical solutions that help mountain communities adapt to climate change while protecting ecosystems and improving livelihoods.
-The first call will fund up to 15 projects and provides grants of up to USD 30,000 per project. Successful organizations will also receive capacity development and training support to strengthen implementation.
-The proposed solutions should have a strong focus on ecosystem-based adaptation (EbA) and/or Nature-based Solutions (NbS). Examples include:
-Ecosystem restoration
-Rainwater harvesting
-Climate-smart agriculture
-Disaster preparedness
-Livelihood diversification
-Other locally appropriate nature-based climate adaptation solutions
- Eligible Applicants
-The grant is intended for:
-Civil society organizations
-Community-based organizations
-Grassroots organizations
-Youth organizations
-Women’s organizations
-Registered NGOs working with mountain communities 
- Important eligibility requirements
-Applicants must:
-Be formally registered.
-Be locally based in an eligible mountain region.
-Have prior experience working directly with mountain communities.
-Address a mountain climate-change challenge or vulnerability.
-Use an ecosystem-based adaptation / nature-based approach.
-Demonstrate capacity to implement the proposed project.
-Submit the required organizational documentation. 
-Individuals are not eligible.</t>
-        </is>
-      </c>
-      <c r="D6" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E6" s="1" t="inlineStr">
-        <is>
-          <t>Sep 15, 2026</t>
-        </is>
-      </c>
-      <c r="F6" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/application-invited-for-2026-call-for-proposals-mountains-adapt-small-grants-united-nations-environment-programme-opg-26-00162</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="95" customHeight="1">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited Translation Funding Programme Grants for German-Language Literature</t>
-        </is>
-      </c>
-      <c r="C7" s="1" t="inlineStr">
-        <is>
-          <t>About us
-The Goethe-Institut is the cultural institute of the Federal Republic of Germany with a global reach. We promote knowledge of the German language abroad and foster international cultural cooperation. We convey a comprehensive image of Germany by providing information about cultural, social and political life in our nation. Our cultural and educational programmes encourage intercultural dialogue and enable cultural involvement. They strengthen the development of structures in civil society and foster worldwide mobility. With our network of Goethe-Instituts, Goethe Centres, cultural societies, reading rooms and exam and language learning centres, we have been the first point of contact for many with Germany for over sixty years. Our long-lasting partnerships with leading institutions and individuals in over ninety countries create enduring trust in Germany. We are partners for all who actively engage with Germany and its culture, working independently and without political ties.
- Conditions of Funding
-Whom we fund
-We fund international professional publishers who wish to translate German-language books. Any publishing house applying for this grant must have both well-documented experience of publishing quality literature and professional distribution channels.
-Neither translators nor authors may apply for translation subsidies through this support scheme.
- What we fund
-We fund translations of works written in the German language and published in printed form by a publisher in a German-speaking country. The translation must be made from the original German text.
-The nationality of the author is irrelevant to the application, with the restriction that applications for works of fiction by contemporary Austrian authors must be submitted to the Austrian Federal Ministry of Housing, Arts, Culture, Media and Sport (BMWKMS) and for contemporary Swiss authors to Pro Helvetia.
-The translation must not go to print before the funding agreement has been signed.
-Books from the following genres are eligible for a grant application:
-Literary fiction, poetry, picture books, comics and graphic novels for adults, children and young adults.
-Non-fiction and essays on current, social topics relevant to contemporary discourse in Germany and in the target countries.
-Scholarly works of general interest and overarching relevance to current discourses in the fields of the humanities and social sciences.
-The grant scheme aims to support the translation of contemporary works. Priority will be given to translations of the work of contemporary German authors into languages where there are no or few previous translations of that author's work or other German literature.
-Canonical literature can only be considered if the respective text has not yet been translated or if the applicant presents valid reasons for a new translation in the project justification.
-Irrespective of genre, the work for which a subsidy is being applied must be of high literary quality in terms of style, form and content. The quality of the publications to be translated will be assessed by the jury.
-Translations by translators who have relevant experience in translating from German or have completed professional training in translation will be supported. The quality of the application will also be assessed based on the following criteria concerning the applicant publisher: quality of the programme (backlist, current catalogue), quality of previously published translations, book design, distribution network, etc.
- APPLICATIONS FOR AN INDIVIDUAL SELECTION OF TEXTS (E.G. AN ANTHOLOGY)
-It is possible to apply for a text selection compiled by or for the applicant publisher.
-Additional application documents are required for this:
-Index of the selected texts, including the original German titles and bibliographic data.
-Reasons for the selection of the texts.
-Scanned copies of the included complete material.
- What we do not fund
-Light fiction, crime novels
-Specialist scholarly works (e.g. doctoral / postdoctoral theses), reference books, study materials, textbooks, commemorative publications,
-theatre texts,
-Sheet music,
-Yearbooks, books of local interest, exhibition catalogues,
-Hobby books, craft books, handbooks, cookbooks, and travel guides
-We do not fund the translation of foreign-language books into German.
- What does the funding consist of?
-If a grant application is approved, the Goethe-Institut reimburses the publisher with a share of the translation costs after publication of the translated work, usually approx. 40-60%. Full payment of translation costs or financing of licensing, printing or editorial costs is not envisaged.
-The maximum amount per book is 8,000 Euros.
-The sum applied for should correspond to the fee agreed to in the signed translation contract with the translator. The total sum of the fee must be paid to the translator, regardless of the amount that the Goethe-Institut has granted. The translator must confirm having received the full amount before a reimbursement of the grant can take place.
-The funding commitment is valid for three years, the expiry date is specified in the funding contract.
- Information about the application process
-Please apply in German or English via the Goethe-Institut’s applications portal.
-The publisher must create an account on the portal before submitting a first application. When creating an account, select the user account type “Organisation/enterprise” and not “Individual person”.
-Our calls for applications are open for a one-month period three times a year, with closing dates on 15 April, 15 September and 1 December.
-We recommend starting the application process as early as possible. The applications portal will save your information as you go, so you can complete the form at any time before submitting the application.
-If you have any questions about pending applications, please quote the application number you received upon submission.
-If your publisher wishes to apply for funding for more than one book, please submit a separate application per title. We recommend submitting no more than three applications per submission deadline.
- Required documents
-A scanned copy of the signed contract between the publishing house submitting the application and the rights holder;
-A scanned copy of the signed contract between the publishing house submitting the application and the translator;
-The publishing house's rationale for the project;
-The translator's CV comprising a list of their published translations from German, their relevant educational qualifications, professional activities, scholarships and awards;
-PDF / Word file of the original book.
-Additional information required:
-Application Form(PDF, 179 KB)
- Jury
-The translations to be funded are selected by a five-person jury made up of two literary critics, one member of staff from the Foreign Rights department of a different publishing house each year, and two members of staff from the Goethe-Institut’s Literature and Translation Funding Department.
-Currently, the jury consists of the following members:
-Katharina Teutsch is a cultural scientist and literary critic. She works for FAZ, DIE ZEIT, der Freitag and "Philosophie Magazin", among others, she produces radio features and regularly moderates “Studio LCB”.
-Michael Schmitt is a freelance literary critic and author. He worked as a literary editor for the cultural TV channel 3sat until 2025.
-Aleksandra Erakovic is Foreign Rights Manager at Kiepenheuer &amp; Witsch publishing house.
-Wolf Iro is Head of the Libraries and Literature Department at the Goethe-Institut.
-Anne-Bitt Gerecke is Head of Goethe-Institut's Litrix programme.
-Conditions for the payment of the grant
- Next application periods
-15 August to 15 September 2026 for translations going to press in December 2026 or later. The funding decision will be communicated to the applicant by email on 20 November 2026.
-1 November to 1 December 2026 for translations going to press in March 2027 or later.
-Our calls for proposals are open for a one-month period three times a year, with closing dates on 15 April, 15 September and 1 December.</t>
-        </is>
-      </c>
-      <c r="D7" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E7" s="1" t="inlineStr">
-        <is>
-          <t>Sep 15, 2026</t>
-        </is>
-      </c>
-      <c r="F7" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-translation-funding-programme-grants-for-german-language-literature-goethe-institut-indien-opg-26-00173</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="95" customHeight="1">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
-        <is>
-          <t>Terms of Reference TOR for Project Consultant / Organization DRE Assessment &amp; Coordination Support for Common Facility Centres CFCs</t>
-        </is>
-      </c>
-      <c r="C8" s="1" t="inlineStr">
-        <is>
-          <t>Title Project Consultant / Organization – DRE Assessment &amp; Coordination Support for Common Facility Centres (CFCs)
-Timeline
- 6 Months
-Expected area of expertise Energy assessment, solar system sizing, documentation, and field coordination
-Apply Link
- https://forms.gle/CTSsV4AzAAcRqmyh8
-Last Date for Apply 16th September, 2026 by 5 pm.
-About SELCO Foundation:
-SELCO Foundation is an open-source, not-for-profit organization that engages in field-based R&amp;D and ecosystem building for the deployment of clean energy solutions that alleviate poverty by improving access to sustainable energy to underserved communities in tribal, rural, and urban poor areas. The organization works in collaboration with practitioners in the social sector, energy entrepreneurs, NGOs from various developmental sectors, and educational institutions to link the benefits of sustainable energy to poverty eradication. The organization works across verticals such as energy access, health, and livelihoods. You can find more information about the SELCO Foundation on our website: http://www.selcofoundation.org/
-Summary of the Project:
-SELCO Foundation is looking to onboard a Consultant/Organization to support the assessment, documentation, and solar system sizing for 30 Common Facility Centres (CFCs) implemented by the government across Agri, animal husbandry, microbusiness, or other relevant livelihood sectors. The Consultant will also provide coordination support during implementation (carried out by a separate implementation vendor) and conduct a post-installation endline assessment.
-This is a scoped, straightforward assignment focused on assessment, standard system sizing, coordination, and endline verification — it does not include design of the overall scheme, beneficiary long-listing, or ongoing monitoring &amp; evaluation.
-Goals and Objectives
-The program's key objectives are:
-Assessing and documenting 30 Government-implemented CFCs
-Recommending standard solar system sizes/designs based on load requirements
-Coordinating with the implementation vendor and keeping CFC users updated through implementation
-Conducting a post-installation endline assessment
-Requirements
-Agency/Individual should have experience in or capacity for:
-Conducting field-based energy/load assessments and documentation.
-Solar system sizing and design recommendation based on load profiles.
-Coordinating with government departments, CFC operators, and third-party implementation vendors.
-Conducting post-installation assessments and reporting.
-Excellent written and verbal communication skills, especially for field coordination.
-Working presence across Assam, Meghalaya, and Mizoram for the duration of the agreement.</t>
-        </is>
-      </c>
-      <c r="D8" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E8" s="1" t="inlineStr">
-        <is>
-          <t>Sep 16, 2026</t>
-        </is>
-      </c>
-      <c r="F8" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/terms-of-reference-tor-for-project-consultant-organization-dre-assessment-and-coordination-support-for-common-facility-centres-cfcs-selco-foundation-rfp-26-00345</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="95" customHeight="1">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="inlineStr">
-        <is>
-          <t>ToR - Development of the WaterAid India WAI Blue Book Series Programme Implementation Guides</t>
-        </is>
-      </c>
-      <c r="C9" s="1" t="inlineStr">
-        <is>
-          <t>Terms of Reference (ToR)
-Development of the WaterAid India (WAI) Blue Book Series – Programme Implementation Guides
-About WaterAid India
-Jal Seva Charitable Foundation (JSCF) is registered in India as a not-for-profit company under Chapter 8 of the Companies Act, 2013. JSCF, is an associate member of the WaterAid federation and uses the brand name ‘WaterAid’ in India.
-WaterAid India seeks to improve the quality of life of 5,000,000 households – with a special emphasis on the vulnerable by 2029 through the provision of climate-resilient and sustainable WASH services via demonstration, institution strengthening, and the effective utilization of public resources. We work in rural and urban areas and seek to deepen our presence in states we operate in and to work in small towns. Thanks to our amazing supporters, we have reached millions of people with these three essentials – clean water, decent toilets, and good hygiene – enabling communities to unlock their potential to break free from the cycle of poverty and to change lives for good.
-We will not stop. Not until clean water, decent toilets and good hygiene are a normal part of everyday life for everyone, everywhere.
-WaterAid India’s (WAI) country office is based in New Delhi with State Offices in Bengaluru, Bhopal, Bhubaneswar, Hyderabad, Lucknow, Patna, Kolkata and Raipur. We currently have a presence in ten states in the country.
-WAI’s Programme focus in the next five years is on ensuring access to safe and assured drinking water in the households, as well as safely managed sanitation at both the household and habitation level. Further, we seek to ensure that anganwadi’s, schools and health care facilities have adequate and appropriate water, sanitation and hygiene infrastructure. Finally, we seek to create integrated water and sanitation solutions in small towns. In all of these efforts, ensuring climate resilience of infrastructure and systems is critical. We seek to do this through demonstration and the provision of technical and knowledge support to governments at all levels who can facilitate adoption on scale. Implementation is primarily through our own field teams. Further details about WAI can be accessed at https://www.wateraid.org/in/
-Background
-WaterAid India (WAI) implements integrated Water, Sanitation and Hygiene (WASH) programmes across multiple states through partnerships with governments, communities, civil society organizations, and development partners. Over the years, WAI has developed extensive technical expertise, programme methodologies, implementation tools, and institutional learning across diverse programme contexts.
-As WAI continues to scale its programmes, there is a need to institutionalize these experiences into a standardized implementation framework that promotes consistency, quality, accountability, and sustainability across all programme interventions.
-To address this need, WaterAid India proposes to develop the WAI Blue Book Series—the organization's programme implementation guide. The Blue Book Series will comprise six interconnected booklets that together provide end-to-end guidance for programme execution—from entering a new intervention geography and designing programmes to implementing quality WASH interventions, strengthening institutions, ensuring sustainable services, documenting evidence, and planning future programme investments.
-The Blue Book Series will establish common programme standards, implementation protocols, quality assurance mechanisms, and practical tools that can be consistently used by WaterAid India teams, partners, consultants, and other implementation stakeholders.
-Objective of the Assignment
-To develop the WAI Blue Book Series, a standardized set of programme implementation guides that establish common implementation standards, quality assurance mechanisms, operational protocols, and practical tools for delivering high-quality, inclusive, climate-resilient, and sustainable WASH programmes across WaterAid India.
-Consultant/Agency Profile
-The consultant/agency should possess:
-At least 10 years of experience in WASH, rural development, programme quality, or institutional strengthening.
-Demonstrated experience in developing implementation manuals, operational frameworks, programme standards, or quality assurance systems.
-Strong expertise in programme design, technical writing, facilitation, and organizational knowledge management.
-Experience working with government systems, development partners, and multi-state programmes.
-A multidisciplinary team with expertise in WASH programming, programme quality, safeguarding, technical writing, and graphic design will be preferred.
-Proposal Submission
-Interested consultants/agencies should submit:
-Technical proposal outlining methodology and work plan.
-Financial proposal.
-Relevant work samples (frameworks, toolkits, manuals or IEC materials).
-CVs of key personnel.
-Evaluation Criteria
-Criteria Weight
-Understanding of assignment 20%
-Proposed methodology 25%
-Relevant organisational experience 20%
-Team composition and expertise 20%
-Financial proposal 15%</t>
-        </is>
-      </c>
-      <c r="D9" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E9" s="1" t="inlineStr">
-        <is>
-          <t>Sep 16, 2026</t>
-        </is>
-      </c>
-      <c r="F9" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/tor-development-of-the-wateraid-india-wai-blue-book-series-programme-implementation-guides-wateraid-india-rfp-26-00347</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="95" customHeight="1">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
-        <is>
-          <t>ToR - Development of WaterAid India's Hygiene Framework Community Facilitator Toolkit Hygiene Booklet and Hygiene Calendar</t>
-        </is>
-      </c>
-      <c r="C10" s="1" t="inlineStr">
         <is>
           <t>Terms of Reference (ToR)
 Development of WaterAid India's Hygiene Framework, Community Facilitator Toolkit, Hygiene Booklet and Hygiene Calendar
@@ -1067,34 +509,34 @@
 Financial proposal 15%</t>
         </is>
       </c>
-      <c r="D10" s="1" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E10" s="1" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>Sep 16, 2026</t>
         </is>
       </c>
-      <c r="F10" s="1" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-development-of-wateraid-indias-hygiene-framework-community-facilitator-toolkit-hygiene-booklet-and-hygiene-calendar-wateraid-india-rfp-26-00349</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="95" customHeight="1">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="inlineStr">
+    <row r="3" ht="95" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>ToR - Standardisation and Development of Community Training Modules and Facilitator Manuals for WASH-Secure Communities</t>
         </is>
       </c>
-      <c r="C11" s="1" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Terms of Reference (ToR)
 Standardisation and Development of Community Training Modules and Facilitator Manuals for WASH-Secure Communities
@@ -1163,34 +605,157 @@
 The consultant/agency obtaining the highest combined score will be recommended for award.</t>
         </is>
       </c>
-      <c r="D11" s="1" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E11" s="1" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Sep 16, 2026</t>
         </is>
       </c>
-      <c r="F11" s="1" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-standardisation-and-development-of-community-training-modules-and-facilitator-manuals-for-wash-secure-communities-wateraid-india-rfp-26-00348</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="95" customHeight="1">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="inlineStr">
+    <row r="4" ht="95" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Terms of Reference TOR for Project Consultant / Organization DRE Assessment &amp; Coordination Support for Common Facility Centres CFCs</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Title Project Consultant / Organization – DRE Assessment &amp; Coordination Support for Common Facility Centres (CFCs)
+Timeline
+ 6 Months
+Expected area of expertise Energy assessment, solar system sizing, documentation, and field coordination
+Apply Link
+ https://forms.gle/CTSsV4AzAAcRqmyh8
+Last Date for Apply 16th September, 2026 by 5 pm.
+About SELCO Foundation:
+SELCO Foundation is an open-source, not-for-profit organization that engages in field-based R&amp;D and ecosystem building for the deployment of clean energy solutions that alleviate poverty by improving access to sustainable energy to underserved communities in tribal, rural, and urban poor areas. The organization works in collaboration with practitioners in the social sector, energy entrepreneurs, NGOs from various developmental sectors, and educational institutions to link the benefits of sustainable energy to poverty eradication. The organization works across verticals such as energy access, health, and livelihoods. You can find more information about the SELCO Foundation on our website: http://www.selcofoundation.org/
+Summary of the Project:
+SELCO Foundation is looking to onboard a Consultant/Organization to support the assessment, documentation, and solar system sizing for 30 Common Facility Centres (CFCs) implemented by the government across Agri, animal husbandry, microbusiness, or other relevant livelihood sectors. The Consultant will also provide coordination support during implementation (carried out by a separate implementation vendor) and conduct a post-installation endline assessment.
+This is a scoped, straightforward assignment focused on assessment, standard system sizing, coordination, and endline verification — it does not include design of the overall scheme, beneficiary long-listing, or ongoing monitoring &amp; evaluation.
+Goals and Objectives
+The program's key objectives are:
+Assessing and documenting 30 Government-implemented CFCs
+Recommending standard solar system sizes/designs based on load requirements
+Coordinating with the implementation vendor and keeping CFC users updated through implementation
+Conducting a post-installation endline assessment
+Requirements
+Agency/Individual should have experience in or capacity for:
+Conducting field-based energy/load assessments and documentation.
+Solar system sizing and design recommendation based on load profiles.
+Coordinating with government departments, CFC operators, and third-party implementation vendors.
+Conducting post-installation assessments and reporting.
+Excellent written and verbal communication skills, especially for field coordination.
+Working presence across Assam, Meghalaya, and Mizoram for the duration of the agreement.</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Sep 16, 2026</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/terms-of-reference-tor-for-project-consultant-organization-dre-assessment-and-coordination-support-for-common-facility-centres-cfcs-selco-foundation-rfp-26-00345</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="95" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>ToR - Development of the WaterAid India WAI Blue Book Series Programme Implementation Guides</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>Terms of Reference (ToR)
+Development of the WaterAid India (WAI) Blue Book Series – Programme Implementation Guides
+About WaterAid India
+Jal Seva Charitable Foundation (JSCF) is registered in India as a not-for-profit company under Chapter 8 of the Companies Act, 2013. JSCF, is an associate member of the WaterAid federation and uses the brand name ‘WaterAid’ in India.
+WaterAid India seeks to improve the quality of life of 5,000,000 households – with a special emphasis on the vulnerable by 2029 through the provision of climate-resilient and sustainable WASH services via demonstration, institution strengthening, and the effective utilization of public resources. We work in rural and urban areas and seek to deepen our presence in states we operate in and to work in small towns. Thanks to our amazing supporters, we have reached millions of people with these three essentials – clean water, decent toilets, and good hygiene – enabling communities to unlock their potential to break free from the cycle of poverty and to change lives for good.
+We will not stop. Not until clean water, decent toilets and good hygiene are a normal part of everyday life for everyone, everywhere.
+WaterAid India’s (WAI) country office is based in New Delhi with State Offices in Bengaluru, Bhopal, Bhubaneswar, Hyderabad, Lucknow, Patna, Kolkata and Raipur. We currently have a presence in ten states in the country.
+WAI’s Programme focus in the next five years is on ensuring access to safe and assured drinking water in the households, as well as safely managed sanitation at both the household and habitation level. Further, we seek to ensure that anganwadi’s, schools and health care facilities have adequate and appropriate water, sanitation and hygiene infrastructure. Finally, we seek to create integrated water and sanitation solutions in small towns. In all of these efforts, ensuring climate resilience of infrastructure and systems is critical. We seek to do this through demonstration and the provision of technical and knowledge support to governments at all levels who can facilitate adoption on scale. Implementation is primarily through our own field teams. Further details about WAI can be accessed at https://www.wateraid.org/in/
+Background
+WaterAid India (WAI) implements integrated Water, Sanitation and Hygiene (WASH) programmes across multiple states through partnerships with governments, communities, civil society organizations, and development partners. Over the years, WAI has developed extensive technical expertise, programme methodologies, implementation tools, and institutional learning across diverse programme contexts.
+As WAI continues to scale its programmes, there is a need to institutionalize these experiences into a standardized implementation framework that promotes consistency, quality, accountability, and sustainability across all programme interventions.
+To address this need, WaterAid India proposes to develop the WAI Blue Book Series—the organization's programme implementation guide. The Blue Book Series will comprise six interconnected booklets that together provide end-to-end guidance for programme execution—from entering a new intervention geography and designing programmes to implementing quality WASH interventions, strengthening institutions, ensuring sustainable services, documenting evidence, and planning future programme investments.
+The Blue Book Series will establish common programme standards, implementation protocols, quality assurance mechanisms, and practical tools that can be consistently used by WaterAid India teams, partners, consultants, and other implementation stakeholders.
+Objective of the Assignment
+To develop the WAI Blue Book Series, a standardized set of programme implementation guides that establish common implementation standards, quality assurance mechanisms, operational protocols, and practical tools for delivering high-quality, inclusive, climate-resilient, and sustainable WASH programmes across WaterAid India.
+Consultant/Agency Profile
+The consultant/agency should possess:
+At least 10 years of experience in WASH, rural development, programme quality, or institutional strengthening.
+Demonstrated experience in developing implementation manuals, operational frameworks, programme standards, or quality assurance systems.
+Strong expertise in programme design, technical writing, facilitation, and organizational knowledge management.
+Experience working with government systems, development partners, and multi-state programmes.
+A multidisciplinary team with expertise in WASH programming, programme quality, safeguarding, technical writing, and graphic design will be preferred.
+Proposal Submission
+Interested consultants/agencies should submit:
+Technical proposal outlining methodology and work plan.
+Financial proposal.
+Relevant work samples (frameworks, toolkits, manuals or IEC materials).
+CVs of key personnel.
+Evaluation Criteria
+Criteria Weight
+Understanding of assignment 20%
+Proposed methodology 25%
+Relevant organisational experience 20%
+Team composition and expertise 20%
+Financial proposal 15%</t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>Sep 16, 2026</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/tor-development-of-the-wateraid-india-wai-blue-book-series-programme-implementation-guides-wateraid-india-rfp-26-00347</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="95" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>SoW - Hiring an External Agency for Orientation and Capacity Building</t>
         </is>
       </c>
-      <c r="C12" s="1" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>Room to Read’s Foundational Literacy Program in Jharkhand: Anchoring and Delivery of Orientation Programme for Jharkhand Field Workforce
 Scope of Work (SoW)
@@ -1223,34 +788,34 @@
 Meeting ID: 915 1781 4040</t>
         </is>
       </c>
-      <c r="D12" s="1" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E12" s="1" t="inlineStr">
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>Sep 17, 2026</t>
         </is>
       </c>
-      <c r="F12" s="1" t="inlineStr">
+      <c r="F6" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/sow-hiring-an-external-agency-for-orientation-and-capacity-building-room-to-read-india-rfp-26-00346</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="95" customHeight="1">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B13" s="1" t="inlineStr">
+    <row r="7" ht="95" customHeight="1">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>ToR - Project Consultant / Organization DRE Integration in PMFME Enterprises</t>
         </is>
       </c>
-      <c r="C13" s="1" t="inlineStr">
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>Terms of Reference (TOR) for Consultancy Services
 PowerUp PMFME-DRE 
@@ -1275,34 +840,34 @@
 Phase 3: Capacity building, post-implementation audit, and documentation of program learnings.</t>
         </is>
       </c>
-      <c r="D13" s="1" t="inlineStr">
+      <c r="D7" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E13" s="1" t="inlineStr">
+      <c r="E7" s="1" t="inlineStr">
         <is>
           <t>Sep 17, 2026</t>
         </is>
       </c>
-      <c r="F13" s="1" t="inlineStr">
+      <c r="F7" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-project-consultant-organization-dre-integration-in-pmfme-enterprises-selco-foundation-rfp-26-00351</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="95" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="inlineStr">
+    <row r="8" ht="95" customHeight="1">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>ToR for Consultancy Service - Practitioner Knowledge Mapping Across Priority Livelihood Value Chains</t>
         </is>
       </c>
-      <c r="C14" s="1" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>Terms of Reference (TOR) for Consultancy Services
 Title Practitioner Knowledge Mapping Across Priority Livelihood Value Chains
@@ -1337,34 +902,34 @@
 The agency is expected to independently identify and curate knowledge resources beyond those shared by the programme team</t>
         </is>
       </c>
-      <c r="D14" s="1" t="inlineStr">
+      <c r="D8" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E14" s="1" t="inlineStr">
+      <c r="E8" s="1" t="inlineStr">
         <is>
           <t>Sep 18, 2026</t>
         </is>
       </c>
-      <c r="F14" s="1" t="inlineStr">
+      <c r="F8" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-for-consultancy-service-practitioner-knowledge-mapping-across-priority-livelihood-value-chains-selco-foundation-rfp-26-00350</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="95" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="inlineStr">
+    <row r="9" ht="95" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
         <is>
           <t>ToR - Behavioural Insights and Narrative Inquiry for the Climate Responsive Livelihood Programme Meghalaya</t>
         </is>
       </c>
-      <c r="C15" s="1" t="inlineStr">
+      <c r="C9" s="1" t="inlineStr">
         <is>
           <t>Title  Behavioural Insights and Narrative Inquiry for the Climate Responsive Livelihood Programme, Meghalaya
 Timeline  2 months
@@ -1382,120 +947,34 @@
 Rather than evaluating awareness or testing communication materials, the assignment should seek to uncover deeper behavioural and social drivers that influence livelihood choices and participation. The findings will inform a narrative architecture and mobilisation approach that resonates authentically with communities across the state.</t>
         </is>
       </c>
-      <c r="D15" s="1" t="inlineStr">
+      <c r="D9" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E15" s="1" t="inlineStr">
+      <c r="E9" s="1" t="inlineStr">
         <is>
           <t>Sep 19, 2026</t>
         </is>
       </c>
-      <c r="F15" s="1" t="inlineStr">
+      <c r="F9" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-behavioural-insights-and-narrative-inquiry-for-the-climate-responsive-livelihood-programme-meghalaya-selco-foundation-rfp-26-00355</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="95" customHeight="1">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B16" s="1" t="inlineStr">
-        <is>
-          <t>RFP - Agronomic Research Study For Natural Dye Crop Development</t>
-        </is>
-      </c>
-      <c r="C16" s="1" t="inlineStr">
-        <is>
-          <t>REǪUEST FOR PROPOSALS (RFP)
-Agronomic Research Study For Natural Dye Crop Development
-COLORS of Nature Project
-Parameter Details
-Reference COLORS/DFRǪ/20260002
-Title E-Tender Request for Agronomic Research Study for Natural Dye Crop Development (Activity A.2.1)
-Timeline 31st August 2026 – 31 July 2029 (3 years )
-Area of Expertise Agricultural   Research,   Natural    Dye   Crops,   Sustainable                       Farming Practices, Participatory Action Research
-Implementation Area
-Andhra Pradesh (Kotturu Mandal, Parvathipuram Manyam District) &amp; (Ponduru Mandal, Srikakulam District);
-Telangana (Kodangal Mandal, Vikarabad District) &amp; (Narayanpet District)
-Submission Deadline 20th September 2026
-Budget Head 5.2.6 Action research for agronomic practices for Natural Dyes Crops
-Project Overview
-The COLORS of Nature project, co-funded by the European Union and implemented by Welthungerhilfe with partners Avani Society and Chitrika (ALAF), aims to advance circular textile production in India through plant-based dyes. The project targets 15,000 smallholder farmers and artisans across Uttarakhand, Telangana, and Andhra Pradesh (2025–2029).
-Activity A.2.1 is a critical research component that will identify and validate suitable agronomic practices for natural dye crop production. This RFP seeks a qualified research institute or consultant(s) to conduct a 3-year participatory action research with 20 lighthouse farms, evaluating soil treatments, crop combinations, varieties, and harvesting protocols to optimize yield and dye quality.
- OBJECTIVES
-Overall Objective
-To develop and validate evidence-based agronomic practices for cultivating natural dye crops that improve yield, dye quality, and ecological sustainability for smallholder farmers.
- Specific Objectives
-Identify and evaluate suitable plant species/varieties for natural dye production focusing on in-demand colors (blue, red, yellow, green, black, brown, etc). This is an indicative list. Can be changed based on the agro-climatic conditions of the selected regions and the life-cycle/duration of the plan
-Develop optimal Package of Practices (PoP) for the agro - climatic conditions of the women farmers producer companies for 6 priority natural dye crops through participatory field trials.
-Determine best harvesting protocols and maturity indices for maximum dye yield and quality.
-Compare effectiveness of different organic soil management practices on crop performance.
-Assess suitability of intercropping/mixed cropping systems for natural dye crops.
- ELIGIBILITY CRITERIA
-Organizational or Individual Researchers PreFerences
-State/Central Agricultural Universities in India
-ICAR (Indian Council of Agricultural Research) Institutes
-State Agricultural Research Stations
-Reputed Agricultural NGOs with research experience
-Consultants having field experience, access to research/demo plots related to agroecology and natural dyeing
-Private agricultural research organizations
-Consortiums of the above (lead applicant must be specified)
- Mandatory Requirements:
-Legal registration in India (minimum 5 years old) in case of an institution. Not applicable for individual researchers. Instead individual researchers shall have minimum 10 years experience in agro ecology, small holder farming and organic agriculture.
-Adequate infrastructure networks for research management
- Technical Eligibility Criteria
-Essential:
-Expertise in organic/ecological agriculture projects
-Experience working with smallholder farmers in India
-Capability to conduct multi-location trials across different states
-Access to laboratory facilities for soil and plant analysis
-Experience in developing training materials/Package of Practices
-Having working knowledge of Telugu
- Desirable:
-Composition of team should have at least one researcher/professor
-Young Team Leader for the project is preferred with sufficient agro-ecology experience. Active Agro-Ecology practitioners will get additional bonus points
-Research Consultant with experience in training and building capacities around organic agriculture and agro ecology practices will be preferred.
-Prior experience with natural dye crops or Non-Timber Forest Products
-Understanding of handlooms and textile industry requirements
-Experience in Andhra Pradesh or Telangana
-Familiarity with participatory action research methodologies
-Network with agricultural universities and textile research institutions
-Experience working on natural dye</t>
-        </is>
-      </c>
-      <c r="D16" s="1" t="inlineStr">
-        <is>
-          <t>Learning</t>
-        </is>
-      </c>
-      <c r="E16" s="1" t="inlineStr">
-        <is>
-          <t>Sep 20, 2026</t>
-        </is>
-      </c>
-      <c r="F16" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/rfp-agronomic-research-study-for-natural-dye-crop-development-chitrika-rfp-26-00344</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="95" customHeight="1">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B17" s="1" t="inlineStr">
+    <row r="10" ht="95" customHeight="1">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
         <is>
           <t>E-Tender Request for Digital Communication Website Development and Social Media Campaign for Colors of Nature</t>
         </is>
       </c>
-      <c r="C17" s="1" t="inlineStr">
+      <c r="C10" s="1" t="inlineStr">
         <is>
           <t>REǪUEST FOR PROPOSALS (RFP)
 Digital Communication, Website Development and Social Media Campaign
@@ -1541,114 +1020,34 @@
 Ready to develop a women led and based digital marketing team</t>
         </is>
       </c>
-      <c r="D17" s="1" t="inlineStr">
+      <c r="D10" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E17" s="1" t="inlineStr">
+      <c r="E10" s="1" t="inlineStr">
         <is>
           <t>Sep 20, 2026</t>
         </is>
       </c>
-      <c r="F17" s="1" t="inlineStr">
+      <c r="F10" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/e-tender-request-for-digital-communication-website-development-and-social-media-campaign-for-colors-of-nature-chitrika-rfp-26-00342</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="95" customHeight="1">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="inlineStr">
-        <is>
-          <t>RFP - Research Collaboration For Improved Application and Processing Techniques For Natural Dyes</t>
-        </is>
-      </c>
-      <c r="C18" s="1" t="inlineStr">
-        <is>
-          <t>REǪUEST FOR PROPOSALS (RFP)
-Research Collaboration For Improved Application and Processing Techniques For Natural Dyes
-COLORS of Nature Project
-Parameter  Details 
-Reference COLORS/DFRǪ/20260005
-Title E-Tender Request for Research Collaboration on Improved Application and Processing Techniques for Natural Dyes (Activity A.2.3)
-Timeline 31st August 2026 – 31 July 2029 (3 years )
-Area of Expertise Textile Wet Processing &amp; Dyeing Chemistry, Natural Dye Application, Sustainable/Cleaner Textile Processing, Eco-friendly Mordanting &amp; Fixation
-Implementation Area Research institution / laboratory facilities, with pilot validation at partner dyeing unit(s) in India; coordinated with project sites in Andhra Pradesh (Parvathipuram Manyam, Srikakulam and Dr BR Ambedkar Konaseema) and Telangana (Vikarabad)
-Submission Deadline 20th September 2026
-Budget Head 5.2.8     Research on Application of Natural Dye of Textile
-Project Overview
-The COLORS of Nature project, co-funded by the European Union and implemented by Welthungerhilfe with partners Avani Society and Chitrika (ALAF), aims to advance circular textile production in India through plant-based dyes. The project targets 15,000 smallholder farmers and artisans across Uttarakhand, Telangana, and Andhra Pradesh (2025–2029).
-Activity A.2.2 and A.2.3 is a research and technology-collaboration component under Output 2 that will identify, test, and pilot improved application and processing techniques for natural dyes spanning mordanting, pre-treatment, fixation, water and energy efficiency, and residue management. This RFP seeks a qualified textile research institution or specialist consultant to conduct up to 3 years of lab-scale and mill-scale research, culminating in validated mill-ready technical guidelines.
- OBJECTIVES
-Overall Objective
-To identify, develop, and validate improved, eco-friendly application and processing techniques for natural dyes on cotton fabrics and yarn that enhance colour fastness, resource efficiency, and industrial scalability, while preserving ecological sustainability.
-Specific Objectives
-The specific objective and scope of the study may undergo changes based on the existing technology for experimentation available in India. Following are the indicative objectives subject to the availability of such a technology in India
-Identify and evaluate natural mordants and bio-based fixation/crosslinking agents that improve colour fastness and dye permanence without compromising the ecological positioning of natural dyes on cotton fabrics and yarn.
-Test and optimize pre-treatment methods on cotton fabrics and yarn.Develop and pilot water-saving dyeing strategies, including closed-loop dyeing systems.
-Evaluate energy-efficient dyeing alternativesDesign and test protocols for recycling or upcycling dye residues to support a zero-waste processing model.
-Validate the most promising techniques at pilot/mill scale in partnership with at least one dyeing unit/mill
- Currently some of the technologies are available for man-made fibers and at huge scale. Technologies suitable for handloom fabric and yarn will be the primary focus of the study
- ELIGIBILITY CRITERIA
-Eligibility
-State/Central Textile Research Associations or Institutes (e.g. South India Textile Research Association)
-National Institute of Fashion Technology (NIFT), National Institute of Design (NID), or similar design/textile institutes
-State/Central Agricultural or Technical Universities with textile chemistry departments
-Reputed textile-sector NGOs with applied research experience
-Private textile research organizations / individual textile researchers with academics from reputed organisations (NID, NIFT etc.,)
-Consortiums of the above (lead applicant must be specified)
-Individual Consultants with 10 years of experience in handlooms production
-5 years experience in working with Andhra Pradesh and Telangana Weavers
- Mandatory Organizational Requirements:
-Legal registration in India (minimum 5 years old). Not applicable to individual consultants
-Access to a testing laboratory accredited for colour-fastness and related textile testing (own or partnered)
- Technical Eligibility Criteria
-Essential:
-Experience with colour-fastness and related textile testing
-Capability to design and run both lab-scale and unit-scale (production) trials
-Prior working relationship with, or ability to secure, a commercial dyeing unit partner, weavers or dye artisans.
-Experience developing technical guidelines / SOPs for weavers or artisan use
-Desirable:
-Prior experience specifically with natural/plant-based dyes
-Familiarity with closed-loop or low-water dyeing systems
-Knowledge in eco-friendly processing certifications (e.g. GOTS, ZDHC)
-Experience in Andhra Pradesh, Telangana, or Uttarakhand
-Network with dyeing units and textile industry associations</t>
-        </is>
-      </c>
-      <c r="D18" s="1" t="inlineStr">
-        <is>
-          <t>Climate</t>
-        </is>
-      </c>
-      <c r="E18" s="1" t="inlineStr">
-        <is>
-          <t>Sep 20, 2026</t>
-        </is>
-      </c>
-      <c r="F18" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/rfp-research-collaboration-for-improved-application-and-processing-techniques-for-natural-dyes-chitrika-rfp-26-00343</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="95" customHeight="1">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="inlineStr">
+    <row r="11" ht="95" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>Expression of Interest EOI for Trade &amp; Livelihood Partners</t>
         </is>
       </c>
-      <c r="C19" s="1" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>Expression of Interest (EOI) for Trade &amp; Livelihood Partners
 Issued By: BharatCares
@@ -1775,34 +1174,200 @@
 Any prior work with tribal or rural communities, with references if available</t>
         </is>
       </c>
-      <c r="D19" s="1" t="inlineStr">
+      <c r="D11" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E19" s="1" t="inlineStr">
+      <c r="E11" s="1" t="inlineStr">
         <is>
           <t>Sep 20, 2026</t>
         </is>
       </c>
-      <c r="F19" s="1" t="inlineStr">
+      <c r="F11" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/expression-of-interest-eoi-for-trade-and-livelihood-partners-bharatcares-rfp-26-00340</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="95" customHeight="1">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="inlineStr">
+    <row r="12" ht="95" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>RFP - Agronomic Research Study For Natural Dye Crop Development</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>REǪUEST FOR PROPOSALS (RFP)
+Agronomic Research Study For Natural Dye Crop Development
+COLORS of Nature Project
+Parameter Details
+Reference COLORS/DFRǪ/20260002
+Title E-Tender Request for Agronomic Research Study for Natural Dye Crop Development (Activity A.2.1)
+Timeline 31st August 2026 – 31 July 2029 (3 years )
+Area of Expertise Agricultural   Research,   Natural    Dye   Crops,   Sustainable                       Farming Practices, Participatory Action Research
+Implementation Area
+Andhra Pradesh (Kotturu Mandal, Parvathipuram Manyam District) &amp; (Ponduru Mandal, Srikakulam District);
+Telangana (Kodangal Mandal, Vikarabad District) &amp; (Narayanpet District)
+Submission Deadline 20th September 2026
+Budget Head 5.2.6 Action research for agronomic practices for Natural Dyes Crops
+Project Overview
+The COLORS of Nature project, co-funded by the European Union and implemented by Welthungerhilfe with partners Avani Society and Chitrika (ALAF), aims to advance circular textile production in India through plant-based dyes. The project targets 15,000 smallholder farmers and artisans across Uttarakhand, Telangana, and Andhra Pradesh (2025–2029).
+Activity A.2.1 is a critical research component that will identify and validate suitable agronomic practices for natural dye crop production. This RFP seeks a qualified research institute or consultant(s) to conduct a 3-year participatory action research with 20 lighthouse farms, evaluating soil treatments, crop combinations, varieties, and harvesting protocols to optimize yield and dye quality.
+ OBJECTIVES
+Overall Objective
+To develop and validate evidence-based agronomic practices for cultivating natural dye crops that improve yield, dye quality, and ecological sustainability for smallholder farmers.
+ Specific Objectives
+Identify and evaluate suitable plant species/varieties for natural dye production focusing on in-demand colors (blue, red, yellow, green, black, brown, etc). This is an indicative list. Can be changed based on the agro-climatic conditions of the selected regions and the life-cycle/duration of the plan
+Develop optimal Package of Practices (PoP) for the agro - climatic conditions of the women farmers producer companies for 6 priority natural dye crops through participatory field trials.
+Determine best harvesting protocols and maturity indices for maximum dye yield and quality.
+Compare effectiveness of different organic soil management practices on crop performance.
+Assess suitability of intercropping/mixed cropping systems for natural dye crops.
+ ELIGIBILITY CRITERIA
+Organizational or Individual Researchers PreFerences
+State/Central Agricultural Universities in India
+ICAR (Indian Council of Agricultural Research) Institutes
+State Agricultural Research Stations
+Reputed Agricultural NGOs with research experience
+Consultants having field experience, access to research/demo plots related to agroecology and natural dyeing
+Private agricultural research organizations
+Consortiums of the above (lead applicant must be specified)
+ Mandatory Requirements:
+Legal registration in India (minimum 5 years old) in case of an institution. Not applicable for individual researchers. Instead individual researchers shall have minimum 10 years experience in agro ecology, small holder farming and organic agriculture.
+Adequate infrastructure networks for research management
+ Technical Eligibility Criteria
+Essential:
+Expertise in organic/ecological agriculture projects
+Experience working with smallholder farmers in India
+Capability to conduct multi-location trials across different states
+Access to laboratory facilities for soil and plant analysis
+Experience in developing training materials/Package of Practices
+Having working knowledge of Telugu
+ Desirable:
+Composition of team should have at least one researcher/professor
+Young Team Leader for the project is preferred with sufficient agro-ecology experience. Active Agro-Ecology practitioners will get additional bonus points
+Research Consultant with experience in training and building capacities around organic agriculture and agro ecology practices will be preferred.
+Prior experience with natural dye crops or Non-Timber Forest Products
+Understanding of handlooms and textile industry requirements
+Experience in Andhra Pradesh or Telangana
+Familiarity with participatory action research methodologies
+Network with agricultural universities and textile research institutions
+Experience working on natural dye</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>Sep 20, 2026</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/rfp-agronomic-research-study-for-natural-dye-crop-development-chitrika-rfp-26-00344</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="95" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>RFP - Research Collaboration For Improved Application and Processing Techniques For Natural Dyes</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>REǪUEST FOR PROPOSALS (RFP)
+Research Collaboration For Improved Application and Processing Techniques For Natural Dyes
+COLORS of Nature Project
+Parameter  Details 
+Reference COLORS/DFRǪ/20260005
+Title E-Tender Request for Research Collaboration on Improved Application and Processing Techniques for Natural Dyes (Activity A.2.3)
+Timeline 31st August 2026 – 31 July 2029 (3 years )
+Area of Expertise Textile Wet Processing &amp; Dyeing Chemistry, Natural Dye Application, Sustainable/Cleaner Textile Processing, Eco-friendly Mordanting &amp; Fixation
+Implementation Area Research institution / laboratory facilities, with pilot validation at partner dyeing unit(s) in India; coordinated with project sites in Andhra Pradesh (Parvathipuram Manyam, Srikakulam and Dr BR Ambedkar Konaseema) and Telangana (Vikarabad)
+Submission Deadline 20th September 2026
+Budget Head 5.2.8     Research on Application of Natural Dye of Textile
+Project Overview
+The COLORS of Nature project, co-funded by the European Union and implemented by Welthungerhilfe with partners Avani Society and Chitrika (ALAF), aims to advance circular textile production in India through plant-based dyes. The project targets 15,000 smallholder farmers and artisans across Uttarakhand, Telangana, and Andhra Pradesh (2025–2029).
+Activity A.2.2 and A.2.3 is a research and technology-collaboration component under Output 2 that will identify, test, and pilot improved application and processing techniques for natural dyes spanning mordanting, pre-treatment, fixation, water and energy efficiency, and residue management. This RFP seeks a qualified textile research institution or specialist consultant to conduct up to 3 years of lab-scale and mill-scale research, culminating in validated mill-ready technical guidelines.
+ OBJECTIVES
+Overall Objective
+To identify, develop, and validate improved, eco-friendly application and processing techniques for natural dyes on cotton fabrics and yarn that enhance colour fastness, resource efficiency, and industrial scalability, while preserving ecological sustainability.
+Specific Objectives
+The specific objective and scope of the study may undergo changes based on the existing technology for experimentation available in India. Following are the indicative objectives subject to the availability of such a technology in India
+Identify and evaluate natural mordants and bio-based fixation/crosslinking agents that improve colour fastness and dye permanence without compromising the ecological positioning of natural dyes on cotton fabrics and yarn.
+Test and optimize pre-treatment methods on cotton fabrics and yarn.Develop and pilot water-saving dyeing strategies, including closed-loop dyeing systems.
+Evaluate energy-efficient dyeing alternativesDesign and test protocols for recycling or upcycling dye residues to support a zero-waste processing model.
+Validate the most promising techniques at pilot/mill scale in partnership with at least one dyeing unit/mill
+ Currently some of the technologies are available for man-made fibers and at huge scale. Technologies suitable for handloom fabric and yarn will be the primary focus of the study
+ ELIGIBILITY CRITERIA
+Eligibility
+State/Central Textile Research Associations or Institutes (e.g. South India Textile Research Association)
+National Institute of Fashion Technology (NIFT), National Institute of Design (NID), or similar design/textile institutes
+State/Central Agricultural or Technical Universities with textile chemistry departments
+Reputed textile-sector NGOs with applied research experience
+Private textile research organizations / individual textile researchers with academics from reputed organisations (NID, NIFT etc.,)
+Consortiums of the above (lead applicant must be specified)
+Individual Consultants with 10 years of experience in handlooms production
+5 years experience in working with Andhra Pradesh and Telangana Weavers
+ Mandatory Organizational Requirements:
+Legal registration in India (minimum 5 years old). Not applicable to individual consultants
+Access to a testing laboratory accredited for colour-fastness and related textile testing (own or partnered)
+ Technical Eligibility Criteria
+Essential:
+Experience with colour-fastness and related textile testing
+Capability to design and run both lab-scale and unit-scale (production) trials
+Prior working relationship with, or ability to secure, a commercial dyeing unit partner, weavers or dye artisans.
+Experience developing technical guidelines / SOPs for weavers or artisan use
+Desirable:
+Prior experience specifically with natural/plant-based dyes
+Familiarity with closed-loop or low-water dyeing systems
+Knowledge in eco-friendly processing certifications (e.g. GOTS, ZDHC)
+Experience in Andhra Pradesh, Telangana, or Uttarakhand
+Network with dyeing units and textile industry associations</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>Climate</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>Sep 20, 2026</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/rfp-research-collaboration-for-improved-application-and-processing-techniques-for-natural-dyes-chitrika-rfp-26-00343</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="95" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Wellbeing Research Grants Funding Better Evaluations of AI's Impact on Wellbeing</t>
         </is>
       </c>
-      <c r="C20" s="1" t="inlineStr">
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We're an AI research company that builds reliable, interpretable, and steerable AI systems. Our first product is Claude, an AI assistant for tasks at any scale. Our research interests span multiple areas including natural language, human feedback, scaling laws, reinforcement learning, code generation, and interpretability. 
@@ -1821,34 +1386,34 @@
  Funding Amount: Total program pool of $5 million (individual grant sizes not specified on the page)</t>
         </is>
       </c>
-      <c r="D20" s="1" t="inlineStr">
+      <c r="D14" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E20" s="1" t="inlineStr">
+      <c r="E14" s="1" t="inlineStr">
         <is>
           <t>Sep 21, 2026</t>
         </is>
       </c>
-      <c r="F20" s="1" t="inlineStr">
+      <c r="F14" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-wellbeing-research-grants-funding-better-evaluations-of-ais-impact-on-wellbeing-anthropic-opg-26-00175</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="95" customHeight="1">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="inlineStr">
+    <row r="15" ht="95" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for GEF SGP CSO Challenge Program</t>
         </is>
       </c>
-      <c r="C21" s="1" t="inlineStr">
+      <c r="C15" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global Environment Facility Small Grants Programme (SGP) is a global initiative implemented by the United Nations Development Programme (UNDP) on behalf of the Global Environment Facility (GEF). Since its launch in 1992, SGP has empowered communities worldwide to take action on environmental challenges while improving livelihoods. As a GEF Corporate Programme, SGP provides direct support to civil society organisations and community-based organisations to design and implement innovative, locally driven solutions. The programme places strong emphasis on inclusion, ensuring meaningful participation of Indigenous Peoples, youth, women and girls, and other underrepresented groups.
@@ -1897,34 +1462,34 @@
 Risk management and mitigation</t>
         </is>
       </c>
-      <c r="D21" s="1" t="inlineStr">
+      <c r="D15" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E21" s="1" t="inlineStr">
+      <c r="E15" s="1" t="inlineStr">
         <is>
           <t>Sep 23, 2026</t>
         </is>
       </c>
-      <c r="F21" s="1" t="inlineStr">
+      <c r="F15" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-gef-sgp-cso-challenge-program-gef-small-grants-programme-sgp-opg-26-00184</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="95" customHeight="1">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="inlineStr">
+    <row r="16" ht="95" customHeight="1">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>RFP for Impact Assessment</t>
         </is>
       </c>
-      <c r="C22" s="1" t="inlineStr">
+      <c r="C16" s="1" t="inlineStr">
         <is>
           <t>Introduction
 Titan Company Limited, a member of the Tata Group, has a long-standing commitment to Corporate Social Responsibility (CSR) in India. The company's CSR initiatives derive its philosophy from the Company’s vision statement: “We create elevating experiences for the people we touch and significantly impact the world we work in”. The initiatives are designed to promote inclusive growth, empower communities, and contribute to the country's socio-economic development. The program includes Titan’s CSR policy is governed by a dedicated CSR Committee that ensures transparency and compliance with regulatory requirements. The program includes Girl Child Education, Skill and Entrepreneurship Development, supporting Indian Heritage Arts and Crafts, Integrated Village Development Programme, Eye Care and Affirmative Action. Titan's CSR policy is governed by a dedicated CSR Committee that ensures transparency and compliance with regulatory requirements.
@@ -1958,86 +1523,98 @@
 Timeline: Proposal submission deadline: September 24, 2026</t>
         </is>
       </c>
-      <c r="D22" s="1" t="inlineStr">
+      <c r="D16" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E22" s="1" t="inlineStr">
+      <c r="E16" s="1" t="inlineStr">
         <is>
           <t>Sep 24, 2026</t>
         </is>
       </c>
-      <c r="F22" s="1" t="inlineStr">
+      <c r="F16" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfp-for-impact-assessment-titan-rfp-26-00354</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="95" customHeight="1">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B23" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Signals of Change Shaping the Future of Sexual and Reproductive Health and Rights SRHR</t>
-        </is>
-      </c>
-      <c r="C23" s="1" t="inlineStr">
+    <row r="17" ht="95" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Setting up Viral Research and Diagnosis Laboratories VRDL in Medical Colleges/Hospitals/Medical Institutions</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
         <is>
           <t>About the Organization
-The World Health Organization's mission: to promote health, keep the world safe, and serve the vulnerable. Working through offices in more than 150 countries, WHO staff work side by side with governments and other partners to ensure the highest attainable level of health for all people.
- About the Opportunity
-HRP and its UN co-sponsors are leading a global Sexual and Reproductive Health and Rights (SRHR) foresight and research prioritization process for 2026–2036. This open public consultation invites diverse stakeholder input to identify "signals of change" — emerging trends, shifts, or disruptions — that could shape the future of SRHR over the next decade. The process uses foresight methodology (not prediction) to explore plausible futures and will culminate in a published report and research agenda in 2027.
- Guiding Questions
-What future trends will shape or constrain SRHR over the next 10 years?
-What evidence and research investments are needed today to prepare SRHR for the futures we may face?
- Scope of Submissions 
-Economic systems; social infrastructure; structural discrimination; conflict/forced migration/displacement; mega-trends (demographic shifts, climate change, digital transformation/AI, urbanization); conditions of daily life; rights/legal/governance systems; health systems; media/misinformation; and changes in the research ecosystem.
- Who Can Participate 
-Open to individuals and organizations globally, including:
-Health workers, professional associations, clinical networks
-Civil society, community groups, youth-led organizations, rights movements
-Governments, parliamentarians, regulators, public sector bodies
-Researchers, academia, think tanks, technical experts
-UN agencies, multilateral/humanitarian/development organizations
-Funders, philanthropy, private sector, tech/innovation organizations
-Media, communications, journalism
-Anyone with relevant lived experience or perspective
-Special interest in submissions from health worker, community, youth, and rights-movement spaces not typically represented in published forums.
- Submission Requirements: Descriptive information (name, contact email, country, sector) required alongside each submission; formal published evidence is helpful but not required — practice-based experience and field examples are also welcome. Submissions are kept confidential and anonymized before analysis.</t>
-        </is>
-      </c>
-      <c r="D23" s="1" t="inlineStr">
+The President notified the creation of the Department of Health Research under the Ministry of Health &amp; Family Welfare through an amendment to the Government of India (Allocation of Business) Rules, 1961 on the 17th September 2007. The Department of Health Research was formally launched on 5th October 2007 by the Minister for Science &amp; Technology and Earth Sciences in a function presided over by the Minister for Health &amp; Family Welfare, in the presence, inter-alia, of the Minister of State for Health &amp; Family Welfare.
+The Department became functional from November 2008 with the appointment of first Secretary of the Department The aim of the DHR is to bring modern health technologies to the people through research and innovations related to diagnosis, treatment methods and vaccines for prevention, to translate them into products and processes and, in synergy with concerned organizations, introduce these innovations into public health system.
+ About the Opportunity:
+Under DHR's scheme "Setting-up of nation-wide network of laboratories for managing epidemics and national calamities," proposals are invited from Medical Colleges/Hospitals/Research Institutions to establish a Medical College &amp; Research Institute Level – Viral Research and Diagnosis Laboratory (MCL-VRDL). The existing network comprises 167 VRDLs (11 Regional, 27 State, 129 Medical College level) across 27 states and 5 UTs, aimed at early detection of infectious pathogens, outbreak surveillance, and research on emerging/re-emerging viral diseases.
+ Objectives:
+Establish capacity for early detection of common and high-risk infectious pathogens
+Strengthen syndromic surveillance ecosystem for outbreak detection
+Undertake R&amp;D on emerging, re-emerging and novel viruses
+ Eligibility (Institution-level):
+State Government Medical Colleges
+Central Government Medical Colleges and Research Institutes
+Armed Forces Medical Institutions/Hospitals
+Railway and other Central Government health institutions
+Private medical colleges ranked in top 50 NIRF ranking
+Must have a dedicated Microbiology department with qualified faculty
+Must have &gt;200 sq.m. area available in existing building (preferably within Microbiology Dept.)
+ Funding Provision:
+Non-recurring assistance: Rs. 1.55 crore total
+Rs. 66.8 lakhs — Civil Work (infrastructure modification)
+Rs. 88.2 lakhs — Equipment (complete lab setup)
+No recurring expenditure (staff salaries, consumables, contingency) is provided — to be borne by the host institution
+ Role &amp; Responsibilities of the Lab:
+Conduct routine diagnosis of infectious pathogens
+Participate in syndromic and event-based surveillance
+Provide support during outbreaks/epidemics
+Share data with ICMR
+ Selection Criteria:
+Meeting eligibility does not guarantee selection; merit-based evaluation by a technical committee
+Preference to institutions in geographically underserved regions
+Weightage for technical strength (qualified faculty, biosafety practices, outbreak investigation experience, publications, patents, externally funded projects)
+Additional weightage for molecular diagnostics, genomic surveillance, One Health research capability, and commitment to long-term recurring support
+Private medical colleges: only top-50 NIRF-ranked institutions considered</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E23" s="1" t="inlineStr">
+      <c r="E17" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F23" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-signals-of-change-shaping-the-future-of-sexual-and-reproductive-health-and-rights-srhr-world-health-organization-opg-26-00176</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="95" customHeight="1">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B24" s="1" t="inlineStr">
+      <c r="F17" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-setting-up-viral-research-and-diagnosis-laboratories-vrdl-in-medical-collegeshospitalsmedical-institutions-department-of-health-research-dhr-ministry-of-health-and-family-welfare-government-of-india-opg-26-00174</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="95" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>EOI Inviting Expression of Interest-cum-Proposal for Setting Up District De-Addiction Centres under NAPDDR</t>
         </is>
       </c>
-      <c r="C24" s="1" t="inlineStr">
+      <c r="C18" s="1" t="inlineStr">
         <is>
           <t>About us
 In the year 1985-86, the erstwhile Ministry of Welfare was bifurcated into the Department of Women and Child Development and the Department of Welfare. Simultaneously, the Scheduled Castes Development Division, Tribal Development Division and the Minorities and Backward Classes Welfare Division were moved from the Ministry of Home Affairs and also the Wakf Division from the Ministry of Law to form the then Ministry of Welfare Subsequently, the name of the Ministry was changed to the Ministry of Social Justice &amp; Empowerment in May, 1998. Further, in October, 1999, the Tribal Development Division had moved out to form a separate Ministry of Tribal Affairs. In January, 2007, the Minorities Division along with Wakf Unit have been moved out of the Ministry and formed as a separate Ministry and the Child Development Division has gone to the Ministry of Women &amp; Child Development.
@@ -2077,34 +1654,34 @@
 11. Department of Social Justice and Empowerment (DoSJE) reserves the right to cancel this notice, andior invite afresh proposals with or without amendments to this document without liability or any obligation for such document, and without assigning any reason. DoSJE reserves the right to take final decision regarding selection of implementing agency or project.</t>
         </is>
       </c>
-      <c r="D24" s="1" t="inlineStr">
+      <c r="D18" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E24" s="1" t="inlineStr">
+      <c r="E18" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F24" s="1" t="inlineStr">
+      <c r="F18" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/eoi-inviting-expression-of-interest-cum-proposal-for-setting-up-district-de-addiction-centres-under-napddr-ministry-of-social-justice-and-empowerment-goi-rfp-26-00356</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="95" customHeight="1">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B25" s="1" t="inlineStr">
+    <row r="19" ht="95" customHeight="1">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>Application Invited for Giving Joy Microgrant</t>
         </is>
       </c>
-      <c r="C25" s="1" t="inlineStr">
+      <c r="C19" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Giving Joy is a US-based nonprofit that strengthens and inspires women’s entrepreneurship worldwide. Through its micro-grants and mentorship program, Giving Joy helps women establish or improve their businesses and initiatives—for their benefit and the benefit of their communities. To date, Giving Joy has awarded over 88 grants to women-led initiatives in 26 countries.
@@ -2143,98 +1720,86 @@
 The grant period is six months.</t>
         </is>
       </c>
-      <c r="D25" s="1" t="inlineStr">
+      <c r="D19" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E25" s="1" t="inlineStr">
+      <c r="E19" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F25" s="1" t="inlineStr">
+      <c r="F19" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/application-invited-for-giving-joy-microgrant-giving-joy-opg-26-00185</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="95" customHeight="1">
-      <c r="A26" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B26" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Setting up Viral Research and Diagnosis Laboratories VRDL in Medical Colleges/Hospitals/Medical Institutions</t>
-        </is>
-      </c>
-      <c r="C26" s="1" t="inlineStr">
+    <row r="20" ht="95" customHeight="1">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Signals of Change Shaping the Future of Sexual and Reproductive Health and Rights SRHR</t>
+        </is>
+      </c>
+      <c r="C20" s="1" t="inlineStr">
         <is>
           <t>About the Organization
-The President notified the creation of the Department of Health Research under the Ministry of Health &amp; Family Welfare through an amendment to the Government of India (Allocation of Business) Rules, 1961 on the 17th September 2007. The Department of Health Research was formally launched on 5th October 2007 by the Minister for Science &amp; Technology and Earth Sciences in a function presided over by the Minister for Health &amp; Family Welfare, in the presence, inter-alia, of the Minister of State for Health &amp; Family Welfare.
-The Department became functional from November 2008 with the appointment of first Secretary of the Department The aim of the DHR is to bring modern health technologies to the people through research and innovations related to diagnosis, treatment methods and vaccines for prevention, to translate them into products and processes and, in synergy with concerned organizations, introduce these innovations into public health system.
- About the Opportunity:
-Under DHR's scheme "Setting-up of nation-wide network of laboratories for managing epidemics and national calamities," proposals are invited from Medical Colleges/Hospitals/Research Institutions to establish a Medical College &amp; Research Institute Level – Viral Research and Diagnosis Laboratory (MCL-VRDL). The existing network comprises 167 VRDLs (11 Regional, 27 State, 129 Medical College level) across 27 states and 5 UTs, aimed at early detection of infectious pathogens, outbreak surveillance, and research on emerging/re-emerging viral diseases.
- Objectives:
-Establish capacity for early detection of common and high-risk infectious pathogens
-Strengthen syndromic surveillance ecosystem for outbreak detection
-Undertake R&amp;D on emerging, re-emerging and novel viruses
- Eligibility (Institution-level):
-State Government Medical Colleges
-Central Government Medical Colleges and Research Institutes
-Armed Forces Medical Institutions/Hospitals
-Railway and other Central Government health institutions
-Private medical colleges ranked in top 50 NIRF ranking
-Must have a dedicated Microbiology department with qualified faculty
-Must have &gt;200 sq.m. area available in existing building (preferably within Microbiology Dept.)
- Funding Provision:
-Non-recurring assistance: Rs. 1.55 crore total
-Rs. 66.8 lakhs — Civil Work (infrastructure modification)
-Rs. 88.2 lakhs — Equipment (complete lab setup)
-No recurring expenditure (staff salaries, consumables, contingency) is provided — to be borne by the host institution
- Role &amp; Responsibilities of the Lab:
-Conduct routine diagnosis of infectious pathogens
-Participate in syndromic and event-based surveillance
-Provide support during outbreaks/epidemics
-Share data with ICMR
- Selection Criteria:
-Meeting eligibility does not guarantee selection; merit-based evaluation by a technical committee
-Preference to institutions in geographically underserved regions
-Weightage for technical strength (qualified faculty, biosafety practices, outbreak investigation experience, publications, patents, externally funded projects)
-Additional weightage for molecular diagnostics, genomic surveillance, One Health research capability, and commitment to long-term recurring support
-Private medical colleges: only top-50 NIRF-ranked institutions considered</t>
-        </is>
-      </c>
-      <c r="D26" s="1" t="inlineStr">
+The World Health Organization's mission: to promote health, keep the world safe, and serve the vulnerable. Working through offices in more than 150 countries, WHO staff work side by side with governments and other partners to ensure the highest attainable level of health for all people.
+ About the Opportunity
+HRP and its UN co-sponsors are leading a global Sexual and Reproductive Health and Rights (SRHR) foresight and research prioritization process for 2026–2036. This open public consultation invites diverse stakeholder input to identify "signals of change" — emerging trends, shifts, or disruptions — that could shape the future of SRHR over the next decade. The process uses foresight methodology (not prediction) to explore plausible futures and will culminate in a published report and research agenda in 2027.
+ Guiding Questions
+What future trends will shape or constrain SRHR over the next 10 years?
+What evidence and research investments are needed today to prepare SRHR for the futures we may face?
+ Scope of Submissions 
+Economic systems; social infrastructure; structural discrimination; conflict/forced migration/displacement; mega-trends (demographic shifts, climate change, digital transformation/AI, urbanization); conditions of daily life; rights/legal/governance systems; health systems; media/misinformation; and changes in the research ecosystem.
+ Who Can Participate 
+Open to individuals and organizations globally, including:
+Health workers, professional associations, clinical networks
+Civil society, community groups, youth-led organizations, rights movements
+Governments, parliamentarians, regulators, public sector bodies
+Researchers, academia, think tanks, technical experts
+UN agencies, multilateral/humanitarian/development organizations
+Funders, philanthropy, private sector, tech/innovation organizations
+Media, communications, journalism
+Anyone with relevant lived experience or perspective
+Special interest in submissions from health worker, community, youth, and rights-movement spaces not typically represented in published forums.
+ Submission Requirements: Descriptive information (name, contact email, country, sector) required alongside each submission; formal published evidence is helpful but not required — practice-based experience and field examples are also welcome. Submissions are kept confidential and anonymized before analysis.</t>
+        </is>
+      </c>
+      <c r="D20" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E26" s="1" t="inlineStr">
+      <c r="E20" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F26" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-setting-up-viral-research-and-diagnosis-laboratories-vrdl-in-medical-collegeshospitalsmedical-institutions-department-of-health-research-dhr-ministry-of-health-and-family-welfare-government-of-india-opg-26-00174</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="95" customHeight="1">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B27" s="1" t="inlineStr">
+      <c r="F20" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-signals-of-change-shaping-the-future-of-sexual-and-reproductive-health-and-rights-srhr-world-health-organization-opg-26-00176</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="95" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund</t>
         </is>
       </c>
-      <c r="C27" s="1" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund
 Apply by: 13 October, 2026
@@ -2259,34 +1824,34 @@
  Projects should include opportunities for ServiceNow employees to volunteer in the project activation or implementation.</t>
         </is>
       </c>
-      <c r="D27" s="1" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E27" s="1" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>Oct 13, 2026</t>
         </is>
       </c>
-      <c r="F27" s="1" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/apply-for-the-servicenow-community-solar-fund-changex-opg-26-00186</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="95" customHeight="1">
-      <c r="A28" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B28" s="1" t="inlineStr">
+    <row r="22" ht="95" customHeight="1">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 8th Call for Proposals Small-Size Grants Global EbA Fund</t>
         </is>
       </c>
-      <c r="C28" s="1" t="inlineStr">
+      <c r="C22" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -2349,34 +1914,34 @@
 Only successful applicants will be contacted; no individual feedback provided to unsuccessful applicants</t>
         </is>
       </c>
-      <c r="D28" s="1" t="inlineStr">
+      <c r="D22" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E28" s="1" t="inlineStr">
+      <c r="E22" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F28" s="1" t="inlineStr">
+      <c r="F22" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-8th-call-for-proposals-small-size-grants-global-eba-fund-global-eba-fund-opg-26-00177</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="95" customHeight="1">
-      <c r="A29" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B29" s="1" t="inlineStr">
+    <row r="23" ht="95" customHeight="1">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIFAR Global Scholars Program 20272029 Cohort</t>
         </is>
       </c>
-      <c r="C29" s="1" t="inlineStr">
+      <c r="C23" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 CIFAR is a Canadian-based globally influential research organization that convenes the world’s most brilliant people across disciplines to advance transformative knowledge and solve humanity’s biggest problems, together. By supporting long-term interdisciplinary collaboration, CIFAR provides researchers with an unparalleled environment of trust, transparency and knowledge sharing. Our time-tested model inspires new directions of inquiry, accelerates discovery and yields breakthroughs across borders and academic disciplines. Through knowledge mobilization, we are catalysts for change in industry, government and society. Through our 15 research programs and the Pan-Canadian AI Strategy, CIFAR convenes close to 400 of the world’s top researchers from 141 institutions in 20 countries. CIFAR is generously supported by the governments of Canada, Alberta and Québec, as well as foundations, individuals, corporations and Canadian and international partner organizations.
@@ -2420,34 +1985,34 @@
  Application Deadline: November 4, 2026, 12:00 PM EST</t>
         </is>
       </c>
-      <c r="D29" s="1" t="inlineStr">
+      <c r="D23" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E29" s="1" t="inlineStr">
+      <c r="E23" s="1" t="inlineStr">
         <is>
           <t>Nov 4, 2026</t>
         </is>
       </c>
-      <c r="F29" s="1" t="inlineStr">
+      <c r="F23" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cifar-global-scholars-program-20272029-cohort-cifar-canadian-institute-for-advanced-research-opg-26-00183</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="95" customHeight="1">
-      <c r="A30" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B30" s="1" t="inlineStr">
+    <row r="24" ht="95" customHeight="1">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for IWRS Teaching Innovation Award</t>
         </is>
       </c>
-      <c r="C30" s="1" t="inlineStr">
+      <c r="C24" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
@@ -2459,34 +2024,34 @@
 Two awards of $2,000 USD are available annually.</t>
         </is>
       </c>
-      <c r="D30" s="1" t="inlineStr">
+      <c r="D24" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E30" s="1" t="inlineStr">
+      <c r="E24" s="1" t="inlineStr">
         <is>
           <t>Nov 15, 2026</t>
         </is>
       </c>
-      <c r="F30" s="1" t="inlineStr">
+      <c r="F24" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="95" customHeight="1">
-      <c r="A31" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B31" s="1" t="inlineStr">
+    <row r="25" ht="95" customHeight="1">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for IWRS Teaching Innovation Award</t>
         </is>
       </c>
-      <c r="C31" s="1" t="inlineStr">
+      <c r="C25" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Insects are one of the most numerous and diverse animal groups on Earth.
@@ -2501,34 +2066,34 @@
 IWRS staff and Advisory Group members are not eligible to apply.</t>
         </is>
       </c>
-      <c r="D31" s="1" t="inlineStr">
+      <c r="D25" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E31" s="1" t="inlineStr">
+      <c r="E25" s="1" t="inlineStr">
         <is>
           <t>Nov 15, 2026</t>
         </is>
       </c>
-      <c r="F31" s="1" t="inlineStr">
+      <c r="F25" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00166</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="95" customHeight="1">
-      <c r="A32" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B32" s="1" t="inlineStr">
+    <row r="26" ht="95" customHeight="1">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Medium-Size Grants Call for Proposals Global EbA Fund</t>
         </is>
       </c>
-      <c r="C32" s="1" t="inlineStr">
+      <c r="C26" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -2585,34 +2150,34 @@
 Applications submitted via online portal (link shared on the Medium-Size Grants webpage from Oct 12)</t>
         </is>
       </c>
-      <c r="D32" s="1" t="inlineStr">
+      <c r="D26" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E32" s="1" t="inlineStr">
+      <c r="E26" s="1" t="inlineStr">
         <is>
           <t>Nov 16, 2026</t>
         </is>
       </c>
-      <c r="F32" s="1" t="inlineStr">
+      <c r="F26" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-medium-size-grants-call-for-proposals-global-eba-fund-global-eba-fund-opg-26-00178</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="95" customHeight="1">
-      <c r="A33" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B33" s="1" t="inlineStr">
+    <row r="27" ht="95" customHeight="1">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIEIF Grant 2026 Climate Intervention Environmental Impact Fund</t>
         </is>
       </c>
-      <c r="C33" s="1" t="inlineStr">
+      <c r="C27" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Climate Intervention Environmental Impact Fund (CIEIF) is a philanthropic fund focused on supporting responsible climate intervention field tests. It provides grants for activities such as environmental impact assessment (EIA), predictive impact modelling, and engagement with potentially affected stakeholders, including local communities and government agencies.
@@ -2639,34 +2204,34 @@
 Potential for scaling the innovation to a globally relevant level</t>
         </is>
       </c>
-      <c r="D33" s="1" t="inlineStr">
+      <c r="D27" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E33" s="1" t="inlineStr">
+      <c r="E27" s="1" t="inlineStr">
         <is>
           <t>Dec 1, 2026</t>
         </is>
       </c>
-      <c r="F33" s="1" t="inlineStr">
+      <c r="F27" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cieif-grant-2026-climate-intervention-environmental-impact-fund-climate-intervention-environmental-impact-fund-opg-26-00155</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="95" customHeight="1">
-      <c r="A34" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B34" s="1" t="inlineStr">
+    <row r="28" ht="95" customHeight="1">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 6th Annual Seeding The Future Global Food System Challenge</t>
         </is>
       </c>
-      <c r="C34" s="1" t="inlineStr">
+      <c r="C28" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are one of the largest and most respected private organisations for development cooperation and humanitarian aid in Germany. As a politically and confessionally independent organisation, our value-oriented actions are always based on ethical principles. Our vision is clear: "Zero Hunger by 2030"
@@ -2698,34 +2263,34 @@
 Individuals with no organizational entity</t>
         </is>
       </c>
-      <c r="D34" s="1" t="inlineStr">
+      <c r="D28" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E34" s="1" t="inlineStr">
+      <c r="E28" s="1" t="inlineStr">
         <is>
           <t>Jan 1, 2027</t>
         </is>
       </c>
-      <c r="F34" s="1" t="inlineStr">
+      <c r="F28" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-6th-annual-seeding-the-future-global-food-system-challenge-welthungerhilfe-opg-26-00180</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="95" customHeight="1">
-      <c r="A35" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B35" s="1" t="inlineStr">
+    <row r="29" ht="95" customHeight="1">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for BES Training and Travel Grants</t>
         </is>
       </c>
-      <c r="C35" s="1" t="inlineStr">
+      <c r="C29" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are a global community of scientists shining a spotlight on the intricacy and value of our natural world, providing the evidence for better decisions. Our vision is for people and nature to thrive in a world that values ecology.
@@ -2764,17 +2329,17 @@
  Application Deadline (Round 2): Opens 30 April 2026, closes 17 May 2026</t>
         </is>
       </c>
-      <c r="D35" s="1" t="inlineStr">
+      <c r="D29" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E35" s="1" t="inlineStr">
+      <c r="E29" s="1" t="inlineStr">
         <is>
           <t>May 17, 2027</t>
         </is>
       </c>
-      <c r="F35" s="1" t="inlineStr">
+      <c r="F29" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-bes-training-and-travel-grants-british-ecological-society-opg-26-00181</t>
         </is>

</xml_diff>

<commit_message>
Auto update Combined.xlsx [Tue Sep 15 07:07:23 UTC 2026]
</commit_message>
<xml_diff>
--- a/output/Combined.xlsx
+++ b/output/Combined.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -467,295 +467,10 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>ToR - Development of WaterAid India's Hygiene Framework Community Facilitator Toolkit Hygiene Booklet and Hygiene Calendar</t>
+          <t>SoW - Hiring an External Agency for Orientation and Capacity Building</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
-        <is>
-          <t>Terms of Reference (ToR)
-Development of WaterAid India's Hygiene Framework, Community Facilitator Toolkit, Hygiene Booklet and Hygiene Calendar
-About WaterAid India
-Jal Seva Charitable Foundation (JSCF) is registered in India as a not-for-profit company under Chapter 8 of the Companies Act, 2013. JSCF, is an associate member of the WaterAid federation and uses the brand name ‘WaterAid’ in India.
-WaterAid India seeks to improve the quality of life of 5,000,000 households – with a special emphasis on the vulnerable by 2029 through the provision of climate-resilient and sustainable WASH services via demonstration, institution strengthening, and the effective utilization of public resources. We work in rural and urban areas and seek to deepen our presence in states we operate in and to work in small towns. Thanks to our amazing supporters, we have reached millions of people with these three essentials – clean water, decent toilets, and good hygiene – enabling communities to unlock their potential to break free from the cycle of poverty and to change lives for good.
-We will not stop. Not until clean water, decent toilets and good hygiene are a normal part of everyday life for everyone, everywhere.
-WaterAid India’s (WAI) country office is based in New Delhi with State Offices in Bengaluru, Bhopal, Bhubaneswar, Hyderabad, Lucknow, Patna, Kolkata and Raipur. We currently have a presence in ten states in the country.
-WAI’s Programme focus in the next five years is on ensuring access to safe and assured drinking water in the households, as well as safely managed sanitation at both the household and habitation level. Further, we seek to ensure that anganwadi’s, schools and health care facilities have adequate and appropriate water, sanitation and hygiene infrastructure. Finally, we seek to create integrated water and sanitation solutions in small towns. In all of these efforts, ensuring climate resilience of infrastructure and systems is critical. We seek to do this through demonstration and the provision of technical and knowledge support to governments at all levels who can facilitate adoption on scale. Implementation is primarily through our own field teams. Further details about WAI can be accessed at https://www.wateraid.org/in/
-Background
-WaterAid India (WAI)/ Jal Seva Charitable Foundation (JSCF) works towards achieving universal access to safe water, sanitation and hygiene (WASH), with a focus on the poorest and most marginalised communities. While access to water and sanitation infrastructure has significantly improved, sustained hygiene behaviour remains a critical determinant of health outcomes, nutrition, climate resilience and the long-term sustainability of WASH services.
-To strengthen its hygiene programming across diverse geographies, WaterAid India intends to develop a comprehensive Hygiene Framework and a set of practical implementation resources that can be used by programme teams, partner organisations and Community Facilitators (CFs). The products should adopt a life-cycle approach, integrate climate resilience and gender, and align with national programmes such as Jal Jeevan Mission, Swachh Bharat Mission (Grameen), Poshan Abhiyaan and relevant health initiatives.
-WAI/ JSCF invites proposals from experienced consultants or agencies to support the development of a comprehensive Hygiene Framework and implementation toolkit. The assignment seeks to strengthen the quality, consistency and effectiveness of hygiene programming by developing practical guidance, communication resources and facilitation tools that can be adopted across WaterAid India's programmes.
-Objective of the Assignment
-To develop a comprehensive, evidence-based and implementation-oriented Hygiene Framework and supporting tools that standardise WaterAid India's hygiene programming and enable Community Facilitators to effectively promote sustainable hygiene behaviour at the community level.
-Required Qualifications
-The consultant/agency should demonstrate:
-Minimum 8–10 years of experience in WASH, public health or behaviour change communication.
-Proven experience in developing hygiene strategies, behaviour change frameworks and community training resources.
-Experience working with government programmes such as JJM, SBM-G, NHM or ICDS.
-Strong understanding of climate-resilient WASH programming.
-Excellent technical writing, instructional design and facilitation skills.
-Experience working with national or international development organisations.
-Proposal Submission
-Interested consultants/agencies should submit:
-Technical proposal outlining methodology and work plan.
-Financial proposal.
-Relevant work samples (frameworks, toolkits, manuals or IEC materials).
-CVs of key personnel.
-Evaluation Criteria
-Criteria Weight
-Understanding of assignment 20%
-Proposed methodology 25%
-Relevant organisational experience 20%
-Team composition and expertise 20%
-Financial proposal 15%</t>
-        </is>
-      </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>Sep 16, 2026</t>
-        </is>
-      </c>
-      <c r="F2" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/tor-development-of-wateraid-indias-hygiene-framework-community-facilitator-toolkit-hygiene-booklet-and-hygiene-calendar-wateraid-india-rfp-26-00349</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="95" customHeight="1">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>ToR - Standardisation and Development of Community Training Modules and Facilitator Manuals for WASH-Secure Communities</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t>Terms of Reference (ToR)
-Standardisation and Development of Community Training Modules and Facilitator Manuals for WASH-Secure Communities
-About WaterAid India
-Jal Seva Charitable Foundation (JSCF) is registered in India as a not-for-profit company under Chapter 8 of the Companies Act, 2013. JSCF, is an associate member of the WaterAid federation and uses the brand name ‘WaterAid’ in India.
-WaterAid India seeks to improve the quality of life of 5,000,000 households – with a special emphasis on the vulnerable by 2029 through the provision of climate-resilient and sustainable WASH services via demonstration, institution strengthening, and the effective utilization of public resources. We work in rural and urban areas and seek to deepen our presence in states we operate in and to work in small towns. Thanks to our amazing supporters, we have reached millions of people with these three essentials – clean water, decent toilets, and good hygiene – enabling communities to unlock their potential to break free from the cycle of poverty and to change lives for good.
-We will not stop. Not until clean water, decent toilets and good hygiene are a normal part of everyday life for everyone, everywhere.
-WaterAid India’s (WAI) country office is based in New Delhi with State Offices in Bengaluru, Bhopal, Bhubaneswar, Hyderabad, Lucknow, Patna, Kolkata and Raipur. We currently have a presence in ten states in the country.
-WAI’s Programme focus in the next five years is on ensuring access to safe and assured drinking water in the households, as well as safely managed sanitation at both the household and habitation level. Further, we seek to ensure that anganwadi’s, schools and health care facilities have adequate and appropriate water, sanitation and hygiene infrastructure. Finally, we seek to create integrated water and sanitation solutions in small towns. In all of these efforts, ensuring climate resilience of infrastructure and systems is critical. We seek to do this through demonstration and the provision of technical and knowledge support to governments at all levels who can facilitate adoption on scale. Implementation is primarily through our own field teams. Further details about WAI can be accessed at https://www.wateraid.org/in/
-Background
-WaterAid India (WAI) works towards ensuring universal access to safe water, sanitation and hygiene (WASH) through strengthening community institutions, local governance systems and sustainable service delivery. Community capacity building is central to achieving sustainable WASH outcomes. Over the years, WaterAid India has developed a range of training modules, facilitation guides and learning resources for Village Water and Sanitation Committees (VWSCs), Gram Panchayats, Community Facilitators (CFs), frontline workers and community institutions.
-As WaterAid India expands its work across multiple states and programmes, there is a need to standardise these training resources into a comprehensive, high-quality learning package that reflects organisational approaches, promotes consistent delivery, incorporates climate resilience and ensures quality facilitation across all programme locations.
-WaterAid India therefore seeks the services of a competent consultant or agency to review existing learning materials and develop standardised training modules, facilitator manuals and participant handbooks for key community capacity-building interventions.
-Assignment Objective
-To review, standardise and develop a comprehensive set of community training modules and facilitator manuals that strengthen local institutions and promote sustainable, climate-resilient and inclusive WASH services leading to WASH-secure communities.
-Specific Objectives
-The assignment aims to:
-Review and consolidate existing WaterAid India training resources.
-Develop standardised, competency-based training modules for Community Facilitators.
-Produce facilitator manuals and participant handbooks that support quality and consistent delivery.
-Integrate climate resilience, inclusion, gender, safeguarding and behaviour change across all modules.
-Develop participatory learning methodologies and practical field tools.
-Pilot, validate and finalise the learning package.
-Consultant/Agency Profile
-The consultant/agency should possess:
-Minimum 10 years of experience in WASH sector programming.
-Proven experience in curriculum development and adult learning.
-Experience in developing training packages for community institutions and local governments.
-Demonstrated expertise in Jal Jeevan Mission, Swachh Bharat Mission and rural governance.
-Strong understanding of climate-resilient WASH programming.
-Experience in participatory training methodologies.
-Excellent writing, facilitation and instructional design skills.
-Proposal Submission
-Interested consultants/agencies should submit both Technical and Financial Proposals.
-A. Technical Proposal
-The technical proposal should include:
-Understanding of the assignment.
-Proposed methodology and approach.
-Detailed work plan and timeline.
-Team composition and roles.
-Relevant organisational profile.
-Experience in similar assignments.
-At least three examples of comparable assignments completed in the last three years.
-B. Financial Proposal
-The financial proposal should include:
-Professional fees.
-Applicable taxes.
-Travel and logistics (if applicable).
-Any other reimbursable costs.
-Total lump-sum cost for the assignment.
-Evaluation Criteria
-Selection will follow a Quality and Cost Based Selection (QCBS) process.
-Technical Evaluation (80 Marks)
-Criteria Marks
-Understanding of assignment 15
-Methodology and technical approach 20
-Relevant organisational experience 15
-Experience of proposed team members 20
-Quality of previous work samples 10
-Total Technical Score 80
-Only bidders scoring 60 marks or above in the technical evaluation will qualify for financial evaluation.
-Financial Evaluation (20 Marks)
-The lowest evaluated financial proposal will receive the maximum score of 20, while other proposals will be scored proportionately.
-Final Score
-Final Score = Technical Score (80%) + Financial Score (20%)
-The consultant/agency obtaining the highest combined score will be recommended for award.</t>
-        </is>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>Sep 16, 2026</t>
-        </is>
-      </c>
-      <c r="F3" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/tor-standardisation-and-development-of-community-training-modules-and-facilitator-manuals-for-wash-secure-communities-wateraid-india-rfp-26-00348</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="95" customHeight="1">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>Terms of Reference TOR for Project Consultant / Organization DRE Assessment &amp; Coordination Support for Common Facility Centres CFCs</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>Title Project Consultant / Organization – DRE Assessment &amp; Coordination Support for Common Facility Centres (CFCs)
-Timeline
- 6 Months
-Expected area of expertise Energy assessment, solar system sizing, documentation, and field coordination
-Apply Link
- https://forms.gle/CTSsV4AzAAcRqmyh8
-Last Date for Apply 16th September, 2026 by 5 pm.
-About SELCO Foundation:
-SELCO Foundation is an open-source, not-for-profit organization that engages in field-based R&amp;D and ecosystem building for the deployment of clean energy solutions that alleviate poverty by improving access to sustainable energy to underserved communities in tribal, rural, and urban poor areas. The organization works in collaboration with practitioners in the social sector, energy entrepreneurs, NGOs from various developmental sectors, and educational institutions to link the benefits of sustainable energy to poverty eradication. The organization works across verticals such as energy access, health, and livelihoods. You can find more information about the SELCO Foundation on our website: http://www.selcofoundation.org/
-Summary of the Project:
-SELCO Foundation is looking to onboard a Consultant/Organization to support the assessment, documentation, and solar system sizing for 30 Common Facility Centres (CFCs) implemented by the government across Agri, animal husbandry, microbusiness, or other relevant livelihood sectors. The Consultant will also provide coordination support during implementation (carried out by a separate implementation vendor) and conduct a post-installation endline assessment.
-This is a scoped, straightforward assignment focused on assessment, standard system sizing, coordination, and endline verification — it does not include design of the overall scheme, beneficiary long-listing, or ongoing monitoring &amp; evaluation.
-Goals and Objectives
-The program's key objectives are:
-Assessing and documenting 30 Government-implemented CFCs
-Recommending standard solar system sizes/designs based on load requirements
-Coordinating with the implementation vendor and keeping CFC users updated through implementation
-Conducting a post-installation endline assessment
-Requirements
-Agency/Individual should have experience in or capacity for:
-Conducting field-based energy/load assessments and documentation.
-Solar system sizing and design recommendation based on load profiles.
-Coordinating with government departments, CFC operators, and third-party implementation vendors.
-Conducting post-installation assessments and reporting.
-Excellent written and verbal communication skills, especially for field coordination.
-Working presence across Assam, Meghalaya, and Mizoram for the duration of the agreement.</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="inlineStr">
-        <is>
-          <t>Sep 16, 2026</t>
-        </is>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/terms-of-reference-tor-for-project-consultant-organization-dre-assessment-and-coordination-support-for-common-facility-centres-cfcs-selco-foundation-rfp-26-00345</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="95" customHeight="1">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>ToR - Development of the WaterAid India WAI Blue Book Series Programme Implementation Guides</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="inlineStr">
-        <is>
-          <t>Terms of Reference (ToR)
-Development of the WaterAid India (WAI) Blue Book Series – Programme Implementation Guides
-About WaterAid India
-Jal Seva Charitable Foundation (JSCF) is registered in India as a not-for-profit company under Chapter 8 of the Companies Act, 2013. JSCF, is an associate member of the WaterAid federation and uses the brand name ‘WaterAid’ in India.
-WaterAid India seeks to improve the quality of life of 5,000,000 households – with a special emphasis on the vulnerable by 2029 through the provision of climate-resilient and sustainable WASH services via demonstration, institution strengthening, and the effective utilization of public resources. We work in rural and urban areas and seek to deepen our presence in states we operate in and to work in small towns. Thanks to our amazing supporters, we have reached millions of people with these three essentials – clean water, decent toilets, and good hygiene – enabling communities to unlock their potential to break free from the cycle of poverty and to change lives for good.
-We will not stop. Not until clean water, decent toilets and good hygiene are a normal part of everyday life for everyone, everywhere.
-WaterAid India’s (WAI) country office is based in New Delhi with State Offices in Bengaluru, Bhopal, Bhubaneswar, Hyderabad, Lucknow, Patna, Kolkata and Raipur. We currently have a presence in ten states in the country.
-WAI’s Programme focus in the next five years is on ensuring access to safe and assured drinking water in the households, as well as safely managed sanitation at both the household and habitation level. Further, we seek to ensure that anganwadi’s, schools and health care facilities have adequate and appropriate water, sanitation and hygiene infrastructure. Finally, we seek to create integrated water and sanitation solutions in small towns. In all of these efforts, ensuring climate resilience of infrastructure and systems is critical. We seek to do this through demonstration and the provision of technical and knowledge support to governments at all levels who can facilitate adoption on scale. Implementation is primarily through our own field teams. Further details about WAI can be accessed at https://www.wateraid.org/in/
-Background
-WaterAid India (WAI) implements integrated Water, Sanitation and Hygiene (WASH) programmes across multiple states through partnerships with governments, communities, civil society organizations, and development partners. Over the years, WAI has developed extensive technical expertise, programme methodologies, implementation tools, and institutional learning across diverse programme contexts.
-As WAI continues to scale its programmes, there is a need to institutionalize these experiences into a standardized implementation framework that promotes consistency, quality, accountability, and sustainability across all programme interventions.
-To address this need, WaterAid India proposes to develop the WAI Blue Book Series—the organization's programme implementation guide. The Blue Book Series will comprise six interconnected booklets that together provide end-to-end guidance for programme execution—from entering a new intervention geography and designing programmes to implementing quality WASH interventions, strengthening institutions, ensuring sustainable services, documenting evidence, and planning future programme investments.
-The Blue Book Series will establish common programme standards, implementation protocols, quality assurance mechanisms, and practical tools that can be consistently used by WaterAid India teams, partners, consultants, and other implementation stakeholders.
-Objective of the Assignment
-To develop the WAI Blue Book Series, a standardized set of programme implementation guides that establish common implementation standards, quality assurance mechanisms, operational protocols, and practical tools for delivering high-quality, inclusive, climate-resilient, and sustainable WASH programmes across WaterAid India.
-Consultant/Agency Profile
-The consultant/agency should possess:
-At least 10 years of experience in WASH, rural development, programme quality, or institutional strengthening.
-Demonstrated experience in developing implementation manuals, operational frameworks, programme standards, or quality assurance systems.
-Strong expertise in programme design, technical writing, facilitation, and organizational knowledge management.
-Experience working with government systems, development partners, and multi-state programmes.
-A multidisciplinary team with expertise in WASH programming, programme quality, safeguarding, technical writing, and graphic design will be preferred.
-Proposal Submission
-Interested consultants/agencies should submit:
-Technical proposal outlining methodology and work plan.
-Financial proposal.
-Relevant work samples (frameworks, toolkits, manuals or IEC materials).
-CVs of key personnel.
-Evaluation Criteria
-Criteria Weight
-Understanding of assignment 20%
-Proposed methodology 25%
-Relevant organisational experience 20%
-Team composition and expertise 20%
-Financial proposal 15%</t>
-        </is>
-      </c>
-      <c r="D5" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E5" s="1" t="inlineStr">
-        <is>
-          <t>Sep 16, 2026</t>
-        </is>
-      </c>
-      <c r="F5" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/tor-development-of-the-wateraid-india-wai-blue-book-series-programme-implementation-guides-wateraid-india-rfp-26-00347</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="95" customHeight="1">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>SoW - Hiring an External Agency for Orientation and Capacity Building</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>Room to Read’s Foundational Literacy Program in Jharkhand: Anchoring and Delivery of Orientation Programme for Jharkhand Field Workforce
 Scope of Work (SoW)
@@ -788,34 +503,34 @@
 Meeting ID: 915 1781 4040</t>
         </is>
       </c>
-      <c r="D6" s="1" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E6" s="1" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>Sep 17, 2026</t>
         </is>
       </c>
-      <c r="F6" s="1" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/sow-hiring-an-external-agency-for-orientation-and-capacity-building-room-to-read-india-rfp-26-00346</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="95" customHeight="1">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
+    <row r="3" ht="95" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>ToR - Project Consultant / Organization DRE Integration in PMFME Enterprises</t>
         </is>
       </c>
-      <c r="C7" s="1" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Terms of Reference (TOR) for Consultancy Services
 PowerUp PMFME-DRE 
@@ -840,34 +555,34 @@
 Phase 3: Capacity building, post-implementation audit, and documentation of program learnings.</t>
         </is>
       </c>
-      <c r="D7" s="1" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E7" s="1" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Sep 17, 2026</t>
         </is>
       </c>
-      <c r="F7" s="1" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-project-consultant-organization-dre-integration-in-pmfme-enterprises-selco-foundation-rfp-26-00351</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="95" customHeight="1">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
+    <row r="4" ht="95" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>ToR for Consultancy Service - Practitioner Knowledge Mapping Across Priority Livelihood Value Chains</t>
         </is>
       </c>
-      <c r="C8" s="1" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>Terms of Reference (TOR) for Consultancy Services
 Title Practitioner Knowledge Mapping Across Priority Livelihood Value Chains
@@ -902,34 +617,34 @@
 The agency is expected to independently identify and curate knowledge resources beyond those shared by the programme team</t>
         </is>
       </c>
-      <c r="D8" s="1" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E8" s="1" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>Sep 18, 2026</t>
         </is>
       </c>
-      <c r="F8" s="1" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-for-consultancy-service-practitioner-knowledge-mapping-across-priority-livelihood-value-chains-selco-foundation-rfp-26-00350</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="95" customHeight="1">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="inlineStr">
+    <row r="5" ht="95" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>ToR - Behavioural Insights and Narrative Inquiry for the Climate Responsive Livelihood Programme Meghalaya</t>
         </is>
       </c>
-      <c r="C9" s="1" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>Title  Behavioural Insights and Narrative Inquiry for the Climate Responsive Livelihood Programme, Meghalaya
 Timeline  2 months
@@ -947,107 +662,34 @@
 Rather than evaluating awareness or testing communication materials, the assignment should seek to uncover deeper behavioural and social drivers that influence livelihood choices and participation. The findings will inform a narrative architecture and mobilisation approach that resonates authentically with communities across the state.</t>
         </is>
       </c>
-      <c r="D9" s="1" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E9" s="1" t="inlineStr">
+      <c r="E5" s="1" t="inlineStr">
         <is>
           <t>Sep 19, 2026</t>
         </is>
       </c>
-      <c r="F9" s="1" t="inlineStr">
+      <c r="F5" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-behavioural-insights-and-narrative-inquiry-for-the-climate-responsive-livelihood-programme-meghalaya-selco-foundation-rfp-26-00355</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="95" customHeight="1">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
-        <is>
-          <t>E-Tender Request for Digital Communication Website Development and Social Media Campaign for Colors of Nature</t>
-        </is>
-      </c>
-      <c r="C10" s="1" t="inlineStr">
-        <is>
-          <t>REǪUEST FOR PROPOSALS (RFP)
-Digital Communication, Website Development and Social Media Campaign
-Colors of Nature Project
-Parameter Details
-Reference COLORS/DFRǪ/20260002
-Title E-Tender Request for Digital Communication, Website Development and Social Media Campaign for Colors of Nature (Activity A.2.1)
-Timeline 31st August 2026 – 31 July 2029 (3 years)
-Area of Expertise Website, Digital Marketing
-Submission Deadline 20th September 2026
-Budget Head
-5.8.4 - Website
-6.3.3 - Social Media Campaign
-Requirements Proposal for website and social media campaign to be submitted separately
-Background
-The COLORS of Nature project, co-funded by the European Union and implemented by Welthungerhilfe with partners Avani Society and Chitrika (ALAF), aims to advance circular textile production in India through plant-based dyes. The project targets 15,000 smallholder farmers and artisans across Uttarakhand, Telangana, and Andhra Pradesh (2025–2029).
-As the project progresses, there is a need to establish a strong digital identity that documents the project's journey, showcases its impact, creates awareness among consumers, and positions Colors Of Nature as a long-term knowledge and collaboration platform for natural dyes beyond the life of the project.
-Objective
-To conceptualise, design, develop and manage an integrated digital communication ecosystem for Colors Of Nature, comprising:
-Social media platforms
-Digital storytelling
-Knowledge documentation
-Consumer awareness campaigns
-Multimedia communication products
-Brand identity development
-The platform should serve not merely as a project communication tool but as a lasting digital destination for natural dyes in India.
-Specific Objectives
-The selected agency shall work towards the following objectives:
-Establish Colors Of Nature platform as a recognised digital identity for natural dyes.
-Build awareness among at least 100,000 consumers on the environmental, cultural and livelihood significance of natural dyes through planned digital campaigns.
-Ensure appropriate visibility to the European Union and Welthungerhilfe (WHH) in accordance with donor communication and visibility guidelines.
-Create opportunities for future collaborations with designers, educational institutions, buyers, researchers and sustainability practitioners.
-Build a digital footprint that continues to remain relevant beyond the project period.
-Desired Profile oF the Agency
-The project seeks to engage a young, creative and mission-driven communication agency, digital collective or social enterprise rather than a conventional large communication firm.
-Preference shall be given to agencies that:
-Demonstrate innovation, creativity and agility.
-Have experience in development communication.
-Have exposure to rural livelihoods, sustainability, crafts, agriculture or textiles.
-Are willing to mentor and build a dedicated communications team to manage website content, digital campaigns and communication products over time.
-Demonstrate strong storytelling capabilities.
-Operate through lean and cost-effective implementation models while maintaining high quality standards.
-Ready to develop a women led and based digital marketing team</t>
-        </is>
-      </c>
-      <c r="D10" s="1" t="inlineStr">
-        <is>
-          <t>Learning</t>
-        </is>
-      </c>
-      <c r="E10" s="1" t="inlineStr">
-        <is>
-          <t>Sep 20, 2026</t>
-        </is>
-      </c>
-      <c r="F10" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/e-tender-request-for-digital-communication-website-development-and-social-media-campaign-for-colors-of-nature-chitrika-rfp-26-00342</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="95" customHeight="1">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="inlineStr">
+    <row r="6" ht="95" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>Expression of Interest EOI for Trade &amp; Livelihood Partners</t>
         </is>
       </c>
-      <c r="C11" s="1" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>Expression of Interest (EOI) for Trade &amp; Livelihood Partners
 Issued By: BharatCares
@@ -1174,34 +816,114 @@
 Any prior work with tribal or rural communities, with references if available</t>
         </is>
       </c>
-      <c r="D11" s="1" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E11" s="1" t="inlineStr">
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>Sep 20, 2026</t>
         </is>
       </c>
-      <c r="F11" s="1" t="inlineStr">
+      <c r="F6" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/expression-of-interest-eoi-for-trade-and-livelihood-partners-bharatcares-rfp-26-00340</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="95" customHeight="1">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="inlineStr">
+    <row r="7" ht="95" customHeight="1">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>RFP - Research Collaboration For Improved Application and Processing Techniques For Natural Dyes</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>REǪUEST FOR PROPOSALS (RFP)
+Research Collaboration For Improved Application and Processing Techniques For Natural Dyes
+COLORS of Nature Project
+Parameter  Details 
+Reference COLORS/DFRǪ/20260005
+Title E-Tender Request for Research Collaboration on Improved Application and Processing Techniques for Natural Dyes (Activity A.2.3)
+Timeline 31st August 2026 – 31 July 2029 (3 years )
+Area of Expertise Textile Wet Processing &amp; Dyeing Chemistry, Natural Dye Application, Sustainable/Cleaner Textile Processing, Eco-friendly Mordanting &amp; Fixation
+Implementation Area Research institution / laboratory facilities, with pilot validation at partner dyeing unit(s) in India; coordinated with project sites in Andhra Pradesh (Parvathipuram Manyam, Srikakulam and Dr BR Ambedkar Konaseema) and Telangana (Vikarabad)
+Submission Deadline 20th September 2026
+Budget Head 5.2.8     Research on Application of Natural Dye of Textile
+Project Overview
+The COLORS of Nature project, co-funded by the European Union and implemented by Welthungerhilfe with partners Avani Society and Chitrika (ALAF), aims to advance circular textile production in India through plant-based dyes. The project targets 15,000 smallholder farmers and artisans across Uttarakhand, Telangana, and Andhra Pradesh (2025–2029).
+Activity A.2.2 and A.2.3 is a research and technology-collaboration component under Output 2 that will identify, test, and pilot improved application and processing techniques for natural dyes spanning mordanting, pre-treatment, fixation, water and energy efficiency, and residue management. This RFP seeks a qualified textile research institution or specialist consultant to conduct up to 3 years of lab-scale and mill-scale research, culminating in validated mill-ready technical guidelines.
+ OBJECTIVES
+Overall Objective
+To identify, develop, and validate improved, eco-friendly application and processing techniques for natural dyes on cotton fabrics and yarn that enhance colour fastness, resource efficiency, and industrial scalability, while preserving ecological sustainability.
+Specific Objectives
+The specific objective and scope of the study may undergo changes based on the existing technology for experimentation available in India. Following are the indicative objectives subject to the availability of such a technology in India
+Identify and evaluate natural mordants and bio-based fixation/crosslinking agents that improve colour fastness and dye permanence without compromising the ecological positioning of natural dyes on cotton fabrics and yarn.
+Test and optimize pre-treatment methods on cotton fabrics and yarn.Develop and pilot water-saving dyeing strategies, including closed-loop dyeing systems.
+Evaluate energy-efficient dyeing alternativesDesign and test protocols for recycling or upcycling dye residues to support a zero-waste processing model.
+Validate the most promising techniques at pilot/mill scale in partnership with at least one dyeing unit/mill
+ Currently some of the technologies are available for man-made fibers and at huge scale. Technologies suitable for handloom fabric and yarn will be the primary focus of the study
+ ELIGIBILITY CRITERIA
+Eligibility
+State/Central Textile Research Associations or Institutes (e.g. South India Textile Research Association)
+National Institute of Fashion Technology (NIFT), National Institute of Design (NID), or similar design/textile institutes
+State/Central Agricultural or Technical Universities with textile chemistry departments
+Reputed textile-sector NGOs with applied research experience
+Private textile research organizations / individual textile researchers with academics from reputed organisations (NID, NIFT etc.,)
+Consortiums of the above (lead applicant must be specified)
+Individual Consultants with 10 years of experience in handlooms production
+5 years experience in working with Andhra Pradesh and Telangana Weavers
+ Mandatory Organizational Requirements:
+Legal registration in India (minimum 5 years old). Not applicable to individual consultants
+Access to a testing laboratory accredited for colour-fastness and related textile testing (own or partnered)
+ Technical Eligibility Criteria
+Essential:
+Experience with colour-fastness and related textile testing
+Capability to design and run both lab-scale and unit-scale (production) trials
+Prior working relationship with, or ability to secure, a commercial dyeing unit partner, weavers or dye artisans.
+Experience developing technical guidelines / SOPs for weavers or artisan use
+Desirable:
+Prior experience specifically with natural/plant-based dyes
+Familiarity with closed-loop or low-water dyeing systems
+Knowledge in eco-friendly processing certifications (e.g. GOTS, ZDHC)
+Experience in Andhra Pradesh, Telangana, or Uttarakhand
+Network with dyeing units and textile industry associations</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="inlineStr">
+        <is>
+          <t>Climate</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>Sep 20, 2026</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/rfp-research-collaboration-for-improved-application-and-processing-techniques-for-natural-dyes-chitrika-rfp-26-00343</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="95" customHeight="1">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>RFP - Agronomic Research Study For Natural Dye Crop Development</t>
         </is>
       </c>
-      <c r="C12" s="1" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>REǪUEST FOR PROPOSALS (RFP)
 Agronomic Research Study For Natural Dye Crop Development
@@ -1260,114 +982,107 @@
 Experience working on natural dye</t>
         </is>
       </c>
-      <c r="D12" s="1" t="inlineStr">
+      <c r="D8" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E12" s="1" t="inlineStr">
+      <c r="E8" s="1" t="inlineStr">
         <is>
           <t>Sep 20, 2026</t>
         </is>
       </c>
-      <c r="F12" s="1" t="inlineStr">
+      <c r="F8" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfp-agronomic-research-study-for-natural-dye-crop-development-chitrika-rfp-26-00344</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="95" customHeight="1">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B13" s="1" t="inlineStr">
-        <is>
-          <t>RFP - Research Collaboration For Improved Application and Processing Techniques For Natural Dyes</t>
-        </is>
-      </c>
-      <c r="C13" s="1" t="inlineStr">
+    <row r="9" ht="95" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>E-Tender Request for Digital Communication Website Development and Social Media Campaign for Colors of Nature</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
         <is>
           <t>REǪUEST FOR PROPOSALS (RFP)
-Research Collaboration For Improved Application and Processing Techniques For Natural Dyes
-COLORS of Nature Project
-Parameter  Details 
-Reference COLORS/DFRǪ/20260005
-Title E-Tender Request for Research Collaboration on Improved Application and Processing Techniques for Natural Dyes (Activity A.2.3)
-Timeline 31st August 2026 – 31 July 2029 (3 years )
-Area of Expertise Textile Wet Processing &amp; Dyeing Chemistry, Natural Dye Application, Sustainable/Cleaner Textile Processing, Eco-friendly Mordanting &amp; Fixation
-Implementation Area Research institution / laboratory facilities, with pilot validation at partner dyeing unit(s) in India; coordinated with project sites in Andhra Pradesh (Parvathipuram Manyam, Srikakulam and Dr BR Ambedkar Konaseema) and Telangana (Vikarabad)
+Digital Communication, Website Development and Social Media Campaign
+Colors of Nature Project
+Parameter Details
+Reference COLORS/DFRǪ/20260002
+Title E-Tender Request for Digital Communication, Website Development and Social Media Campaign for Colors of Nature (Activity A.2.1)
+Timeline 31st August 2026 – 31 July 2029 (3 years)
+Area of Expertise Website, Digital Marketing
 Submission Deadline 20th September 2026
-Budget Head 5.2.8     Research on Application of Natural Dye of Textile
-Project Overview
+Budget Head
+5.8.4 - Website
+6.3.3 - Social Media Campaign
+Requirements Proposal for website and social media campaign to be submitted separately
+Background
 The COLORS of Nature project, co-funded by the European Union and implemented by Welthungerhilfe with partners Avani Society and Chitrika (ALAF), aims to advance circular textile production in India through plant-based dyes. The project targets 15,000 smallholder farmers and artisans across Uttarakhand, Telangana, and Andhra Pradesh (2025–2029).
-Activity A.2.2 and A.2.3 is a research and technology-collaboration component under Output 2 that will identify, test, and pilot improved application and processing techniques for natural dyes spanning mordanting, pre-treatment, fixation, water and energy efficiency, and residue management. This RFP seeks a qualified textile research institution or specialist consultant to conduct up to 3 years of lab-scale and mill-scale research, culminating in validated mill-ready technical guidelines.
- OBJECTIVES
-Overall Objective
-To identify, develop, and validate improved, eco-friendly application and processing techniques for natural dyes on cotton fabrics and yarn that enhance colour fastness, resource efficiency, and industrial scalability, while preserving ecological sustainability.
+As the project progresses, there is a need to establish a strong digital identity that documents the project's journey, showcases its impact, creates awareness among consumers, and positions Colors Of Nature as a long-term knowledge and collaboration platform for natural dyes beyond the life of the project.
+Objective
+To conceptualise, design, develop and manage an integrated digital communication ecosystem for Colors Of Nature, comprising:
+Social media platforms
+Digital storytelling
+Knowledge documentation
+Consumer awareness campaigns
+Multimedia communication products
+Brand identity development
+The platform should serve not merely as a project communication tool but as a lasting digital destination for natural dyes in India.
 Specific Objectives
-The specific objective and scope of the study may undergo changes based on the existing technology for experimentation available in India. Following are the indicative objectives subject to the availability of such a technology in India
-Identify and evaluate natural mordants and bio-based fixation/crosslinking agents that improve colour fastness and dye permanence without compromising the ecological positioning of natural dyes on cotton fabrics and yarn.
-Test and optimize pre-treatment methods on cotton fabrics and yarn.Develop and pilot water-saving dyeing strategies, including closed-loop dyeing systems.
-Evaluate energy-efficient dyeing alternativesDesign and test protocols for recycling or upcycling dye residues to support a zero-waste processing model.
-Validate the most promising techniques at pilot/mill scale in partnership with at least one dyeing unit/mill
- Currently some of the technologies are available for man-made fibers and at huge scale. Technologies suitable for handloom fabric and yarn will be the primary focus of the study
- ELIGIBILITY CRITERIA
-Eligibility
-State/Central Textile Research Associations or Institutes (e.g. South India Textile Research Association)
-National Institute of Fashion Technology (NIFT), National Institute of Design (NID), or similar design/textile institutes
-State/Central Agricultural or Technical Universities with textile chemistry departments
-Reputed textile-sector NGOs with applied research experience
-Private textile research organizations / individual textile researchers with academics from reputed organisations (NID, NIFT etc.,)
-Consortiums of the above (lead applicant must be specified)
-Individual Consultants with 10 years of experience in handlooms production
-5 years experience in working with Andhra Pradesh and Telangana Weavers
- Mandatory Organizational Requirements:
-Legal registration in India (minimum 5 years old). Not applicable to individual consultants
-Access to a testing laboratory accredited for colour-fastness and related textile testing (own or partnered)
- Technical Eligibility Criteria
-Essential:
-Experience with colour-fastness and related textile testing
-Capability to design and run both lab-scale and unit-scale (production) trials
-Prior working relationship with, or ability to secure, a commercial dyeing unit partner, weavers or dye artisans.
-Experience developing technical guidelines / SOPs for weavers or artisan use
-Desirable:
-Prior experience specifically with natural/plant-based dyes
-Familiarity with closed-loop or low-water dyeing systems
-Knowledge in eco-friendly processing certifications (e.g. GOTS, ZDHC)
-Experience in Andhra Pradesh, Telangana, or Uttarakhand
-Network with dyeing units and textile industry associations</t>
-        </is>
-      </c>
-      <c r="D13" s="1" t="inlineStr">
-        <is>
-          <t>Climate</t>
-        </is>
-      </c>
-      <c r="E13" s="1" t="inlineStr">
+The selected agency shall work towards the following objectives:
+Establish Colors Of Nature platform as a recognised digital identity for natural dyes.
+Build awareness among at least 100,000 consumers on the environmental, cultural and livelihood significance of natural dyes through planned digital campaigns.
+Ensure appropriate visibility to the European Union and Welthungerhilfe (WHH) in accordance with donor communication and visibility guidelines.
+Create opportunities for future collaborations with designers, educational institutions, buyers, researchers and sustainability practitioners.
+Build a digital footprint that continues to remain relevant beyond the project period.
+Desired Profile oF the Agency
+The project seeks to engage a young, creative and mission-driven communication agency, digital collective or social enterprise rather than a conventional large communication firm.
+Preference shall be given to agencies that:
+Demonstrate innovation, creativity and agility.
+Have experience in development communication.
+Have exposure to rural livelihoods, sustainability, crafts, agriculture or textiles.
+Are willing to mentor and build a dedicated communications team to manage website content, digital campaigns and communication products over time.
+Demonstrate strong storytelling capabilities.
+Operate through lean and cost-effective implementation models while maintaining high quality standards.
+Ready to develop a women led and based digital marketing team</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
         <is>
           <t>Sep 20, 2026</t>
         </is>
       </c>
-      <c r="F13" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/rfp-research-collaboration-for-improved-application-and-processing-techniques-for-natural-dyes-chitrika-rfp-26-00343</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="95" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="inlineStr">
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/e-tender-request-for-digital-communication-website-development-and-social-media-campaign-for-colors-of-nature-chitrika-rfp-26-00342</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="95" customHeight="1">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Wellbeing Research Grants Funding Better Evaluations of AI's Impact on Wellbeing</t>
         </is>
       </c>
-      <c r="C14" s="1" t="inlineStr">
+      <c r="C10" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We're an AI research company that builds reliable, interpretable, and steerable AI systems. Our first product is Claude, an AI assistant for tasks at any scale. Our research interests span multiple areas including natural language, human feedback, scaling laws, reinforcement learning, code generation, and interpretability. 
@@ -1386,34 +1101,34 @@
  Funding Amount: Total program pool of $5 million (individual grant sizes not specified on the page)</t>
         </is>
       </c>
-      <c r="D14" s="1" t="inlineStr">
+      <c r="D10" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E14" s="1" t="inlineStr">
+      <c r="E10" s="1" t="inlineStr">
         <is>
           <t>Sep 21, 2026</t>
         </is>
       </c>
-      <c r="F14" s="1" t="inlineStr">
+      <c r="F10" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-wellbeing-research-grants-funding-better-evaluations-of-ais-impact-on-wellbeing-anthropic-opg-26-00175</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="95" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="inlineStr">
+    <row r="11" ht="95" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for GEF SGP CSO Challenge Program</t>
         </is>
       </c>
-      <c r="C15" s="1" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global Environment Facility Small Grants Programme (SGP) is a global initiative implemented by the United Nations Development Programme (UNDP) on behalf of the Global Environment Facility (GEF). Since its launch in 1992, SGP has empowered communities worldwide to take action on environmental challenges while improving livelihoods. As a GEF Corporate Programme, SGP provides direct support to civil society organisations and community-based organisations to design and implement innovative, locally driven solutions. The programme places strong emphasis on inclusion, ensuring meaningful participation of Indigenous Peoples, youth, women and girls, and other underrepresented groups.
@@ -1462,34 +1177,34 @@
 Risk management and mitigation</t>
         </is>
       </c>
-      <c r="D15" s="1" t="inlineStr">
+      <c r="D11" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E15" s="1" t="inlineStr">
+      <c r="E11" s="1" t="inlineStr">
         <is>
           <t>Sep 23, 2026</t>
         </is>
       </c>
-      <c r="F15" s="1" t="inlineStr">
+      <c r="F11" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-gef-sgp-cso-challenge-program-gef-small-grants-programme-sgp-opg-26-00184</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="95" customHeight="1">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B16" s="1" t="inlineStr">
+    <row r="12" ht="95" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
         <is>
           <t>RFP for Impact Assessment</t>
         </is>
       </c>
-      <c r="C16" s="1" t="inlineStr">
+      <c r="C12" s="1" t="inlineStr">
         <is>
           <t>Introduction
 Titan Company Limited, a member of the Tata Group, has a long-standing commitment to Corporate Social Responsibility (CSR) in India. The company's CSR initiatives derive its philosophy from the Company’s vision statement: “We create elevating experiences for the people we touch and significantly impact the world we work in”. The initiatives are designed to promote inclusive growth, empower communities, and contribute to the country's socio-economic development. The program includes Titan’s CSR policy is governed by a dedicated CSR Committee that ensures transparency and compliance with regulatory requirements. The program includes Girl Child Education, Skill and Entrepreneurship Development, supporting Indian Heritage Arts and Crafts, Integrated Village Development Programme, Eye Care and Affirmative Action. Titan's CSR policy is governed by a dedicated CSR Committee that ensures transparency and compliance with regulatory requirements.
@@ -1523,34 +1238,152 @@
 Timeline: Proposal submission deadline: September 24, 2026</t>
         </is>
       </c>
-      <c r="D16" s="1" t="inlineStr">
+      <c r="D12" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E16" s="1" t="inlineStr">
+      <c r="E12" s="1" t="inlineStr">
         <is>
           <t>Sep 24, 2026</t>
         </is>
       </c>
-      <c r="F16" s="1" t="inlineStr">
+      <c r="F12" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfp-for-impact-assessment-titan-rfp-26-00354</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="95" customHeight="1">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B17" s="1" t="inlineStr">
+    <row r="13" ht="95" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>Application Invited for Giving Joy Microgrant</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+Giving Joy is a US-based nonprofit that strengthens and inspires women’s entrepreneurship worldwide. Through its micro-grants and mentorship program, Giving Joy helps women establish or improve their businesses and initiatives—for their benefit and the benefit of their communities. To date, Giving Joy has awarded over 88 grants to women-led initiatives in 26 countries.
+ 2026 Grant Cycle
+Beginning in 2026, Giving Joy has moved to two global grant cycles per year.
+The organization states that this change was made after operating multiple regional rounds, with the aim of:
+Providing clearer timelines for applicants
+Increasing the quality and depth of application reviews
+Reducing administrative burden
+Improving support for grantees
+Focusing communications and fundraising more effectively
+Continuing to reach women entrepreneurs globally without dividing applications by geography
+Each cycle is open to women entrepreneurs worldwide.
+ Eligible Fields / Activities
+There is no restriction to a particular field such as health.
+Applicants can propose activities in:
+Any field
+Trade
+Occupation
+Craft
+ What Does Giving Joy Look For?
+Giving Joy prioritizes:
+Innovative ideas
+Creative ideas
+Strong potential for social impact
+Initiative
+Real community impact
+Clear economic and/or social benefits for women and girls
+ Grant Amount
+Maximum Grant
+Up to $500 USD
+The exact award amount is determined by Giving Joy based on:
+Proposed activities
+Availability of funding
+ Grant Duration
+The grant period is six months.</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>Sep 30, 2026</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/application-invited-for-giving-joy-microgrant-giving-joy-opg-26-00185</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="95" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Signals of Change Shaping the Future of Sexual and Reproductive Health and Rights SRHR</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+The World Health Organization's mission: to promote health, keep the world safe, and serve the vulnerable. Working through offices in more than 150 countries, WHO staff work side by side with governments and other partners to ensure the highest attainable level of health for all people.
+ About the Opportunity
+HRP and its UN co-sponsors are leading a global Sexual and Reproductive Health and Rights (SRHR) foresight and research prioritization process for 2026–2036. This open public consultation invites diverse stakeholder input to identify "signals of change" — emerging trends, shifts, or disruptions — that could shape the future of SRHR over the next decade. The process uses foresight methodology (not prediction) to explore plausible futures and will culminate in a published report and research agenda in 2027.
+ Guiding Questions
+What future trends will shape or constrain SRHR over the next 10 years?
+What evidence and research investments are needed today to prepare SRHR for the futures we may face?
+ Scope of Submissions 
+Economic systems; social infrastructure; structural discrimination; conflict/forced migration/displacement; mega-trends (demographic shifts, climate change, digital transformation/AI, urbanization); conditions of daily life; rights/legal/governance systems; health systems; media/misinformation; and changes in the research ecosystem.
+ Who Can Participate 
+Open to individuals and organizations globally, including:
+Health workers, professional associations, clinical networks
+Civil society, community groups, youth-led organizations, rights movements
+Governments, parliamentarians, regulators, public sector bodies
+Researchers, academia, think tanks, technical experts
+UN agencies, multilateral/humanitarian/development organizations
+Funders, philanthropy, private sector, tech/innovation organizations
+Media, communications, journalism
+Anyone with relevant lived experience or perspective
+Special interest in submissions from health worker, community, youth, and rights-movement spaces not typically represented in published forums.
+ Submission Requirements: Descriptive information (name, contact email, country, sector) required alongside each submission; formal published evidence is helpful but not required — practice-based experience and field examples are also welcome. Submissions are kept confidential and anonymized before analysis.</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>Sep 30, 2026</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-signals-of-change-shaping-the-future-of-sexual-and-reproductive-health-and-rights-srhr-world-health-organization-opg-26-00176</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="95" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Setting up Viral Research and Diagnosis Laboratories VRDL in Medical Colleges/Hospitals/Medical Institutions</t>
         </is>
       </c>
-      <c r="C17" s="1" t="inlineStr">
+      <c r="C15" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The President notified the creation of the Department of Health Research under the Ministry of Health &amp; Family Welfare through an amendment to the Government of India (Allocation of Business) Rules, 1961 on the 17th September 2007. The Department of Health Research was formally launched on 5th October 2007 by the Minister for Science &amp; Technology and Earth Sciences in a function presided over by the Minister for Health &amp; Family Welfare, in the presence, inter-alia, of the Minister of State for Health &amp; Family Welfare.
@@ -1587,34 +1420,34 @@
 Private medical colleges: only top-50 NIRF-ranked institutions considered</t>
         </is>
       </c>
-      <c r="D17" s="1" t="inlineStr">
+      <c r="D15" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E17" s="1" t="inlineStr">
+      <c r="E15" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F17" s="1" t="inlineStr">
+      <c r="F15" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-setting-up-viral-research-and-diagnosis-laboratories-vrdl-in-medical-collegeshospitalsmedical-institutions-department-of-health-research-dhr-ministry-of-health-and-family-welfare-government-of-india-opg-26-00174</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="95" customHeight="1">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="inlineStr">
+    <row r="16" ht="95" customHeight="1">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>EOI Inviting Expression of Interest-cum-Proposal for Setting Up District De-Addiction Centres under NAPDDR</t>
         </is>
       </c>
-      <c r="C18" s="1" t="inlineStr">
+      <c r="C16" s="1" t="inlineStr">
         <is>
           <t>About us
 In the year 1985-86, the erstwhile Ministry of Welfare was bifurcated into the Department of Women and Child Development and the Department of Welfare. Simultaneously, the Scheduled Castes Development Division, Tribal Development Division and the Minorities and Backward Classes Welfare Division were moved from the Ministry of Home Affairs and also the Wakf Division from the Ministry of Law to form the then Ministry of Welfare Subsequently, the name of the Ministry was changed to the Ministry of Social Justice &amp; Empowerment in May, 1998. Further, in October, 1999, the Tribal Development Division had moved out to form a separate Ministry of Tribal Affairs. In January, 2007, the Minorities Division along with Wakf Unit have been moved out of the Ministry and formed as a separate Ministry and the Child Development Division has gone to the Ministry of Women &amp; Child Development.
@@ -1654,152 +1487,34 @@
 11. Department of Social Justice and Empowerment (DoSJE) reserves the right to cancel this notice, andior invite afresh proposals with or without amendments to this document without liability or any obligation for such document, and without assigning any reason. DoSJE reserves the right to take final decision regarding selection of implementing agency or project.</t>
         </is>
       </c>
-      <c r="D18" s="1" t="inlineStr">
+      <c r="D16" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E18" s="1" t="inlineStr">
+      <c r="E16" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F18" s="1" t="inlineStr">
+      <c r="F16" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/eoi-inviting-expression-of-interest-cum-proposal-for-setting-up-district-de-addiction-centres-under-napddr-ministry-of-social-justice-and-empowerment-goi-rfp-26-00356</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="95" customHeight="1">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="inlineStr">
-        <is>
-          <t>Application Invited for Giving Joy Microgrant</t>
-        </is>
-      </c>
-      <c r="C19" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-Giving Joy is a US-based nonprofit that strengthens and inspires women’s entrepreneurship worldwide. Through its micro-grants and mentorship program, Giving Joy helps women establish or improve their businesses and initiatives—for their benefit and the benefit of their communities. To date, Giving Joy has awarded over 88 grants to women-led initiatives in 26 countries.
- 2026 Grant Cycle
-Beginning in 2026, Giving Joy has moved to two global grant cycles per year.
-The organization states that this change was made after operating multiple regional rounds, with the aim of:
-Providing clearer timelines for applicants
-Increasing the quality and depth of application reviews
-Reducing administrative burden
-Improving support for grantees
-Focusing communications and fundraising more effectively
-Continuing to reach women entrepreneurs globally without dividing applications by geography
-Each cycle is open to women entrepreneurs worldwide.
- Eligible Fields / Activities
-There is no restriction to a particular field such as health.
-Applicants can propose activities in:
-Any field
-Trade
-Occupation
-Craft
- What Does Giving Joy Look For?
-Giving Joy prioritizes:
-Innovative ideas
-Creative ideas
-Strong potential for social impact
-Initiative
-Real community impact
-Clear economic and/or social benefits for women and girls
- Grant Amount
-Maximum Grant
-Up to $500 USD
-The exact award amount is determined by Giving Joy based on:
-Proposed activities
-Availability of funding
- Grant Duration
-The grant period is six months.</t>
-        </is>
-      </c>
-      <c r="D19" s="1" t="inlineStr">
-        <is>
-          <t>Safety</t>
-        </is>
-      </c>
-      <c r="E19" s="1" t="inlineStr">
-        <is>
-          <t>Sep 30, 2026</t>
-        </is>
-      </c>
-      <c r="F19" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/application-invited-for-giving-joy-microgrant-giving-joy-opg-26-00185</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="95" customHeight="1">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Signals of Change Shaping the Future of Sexual and Reproductive Health and Rights SRHR</t>
-        </is>
-      </c>
-      <c r="C20" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-The World Health Organization's mission: to promote health, keep the world safe, and serve the vulnerable. Working through offices in more than 150 countries, WHO staff work side by side with governments and other partners to ensure the highest attainable level of health for all people.
- About the Opportunity
-HRP and its UN co-sponsors are leading a global Sexual and Reproductive Health and Rights (SRHR) foresight and research prioritization process for 2026–2036. This open public consultation invites diverse stakeholder input to identify "signals of change" — emerging trends, shifts, or disruptions — that could shape the future of SRHR over the next decade. The process uses foresight methodology (not prediction) to explore plausible futures and will culminate in a published report and research agenda in 2027.
- Guiding Questions
-What future trends will shape or constrain SRHR over the next 10 years?
-What evidence and research investments are needed today to prepare SRHR for the futures we may face?
- Scope of Submissions 
-Economic systems; social infrastructure; structural discrimination; conflict/forced migration/displacement; mega-trends (demographic shifts, climate change, digital transformation/AI, urbanization); conditions of daily life; rights/legal/governance systems; health systems; media/misinformation; and changes in the research ecosystem.
- Who Can Participate 
-Open to individuals and organizations globally, including:
-Health workers, professional associations, clinical networks
-Civil society, community groups, youth-led organizations, rights movements
-Governments, parliamentarians, regulators, public sector bodies
-Researchers, academia, think tanks, technical experts
-UN agencies, multilateral/humanitarian/development organizations
-Funders, philanthropy, private sector, tech/innovation organizations
-Media, communications, journalism
-Anyone with relevant lived experience or perspective
-Special interest in submissions from health worker, community, youth, and rights-movement spaces not typically represented in published forums.
- Submission Requirements: Descriptive information (name, contact email, country, sector) required alongside each submission; formal published evidence is helpful but not required — practice-based experience and field examples are also welcome. Submissions are kept confidential and anonymized before analysis.</t>
-        </is>
-      </c>
-      <c r="D20" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E20" s="1" t="inlineStr">
-        <is>
-          <t>Sep 30, 2026</t>
-        </is>
-      </c>
-      <c r="F20" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-signals-of-change-shaping-the-future-of-sexual-and-reproductive-health-and-rights-srhr-world-health-organization-opg-26-00176</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="95" customHeight="1">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="inlineStr">
+    <row r="17" ht="95" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund</t>
         </is>
       </c>
-      <c r="C21" s="1" t="inlineStr">
+      <c r="C17" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund
 Apply by: 13 October, 2026
@@ -1824,34 +1539,34 @@
  Projects should include opportunities for ServiceNow employees to volunteer in the project activation or implementation.</t>
         </is>
       </c>
-      <c r="D21" s="1" t="inlineStr">
+      <c r="D17" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E21" s="1" t="inlineStr">
+      <c r="E17" s="1" t="inlineStr">
         <is>
           <t>Oct 13, 2026</t>
         </is>
       </c>
-      <c r="F21" s="1" t="inlineStr">
+      <c r="F17" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/apply-for-the-servicenow-community-solar-fund-changex-opg-26-00186</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="95" customHeight="1">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="inlineStr">
+    <row r="18" ht="95" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 8th Call for Proposals Small-Size Grants Global EbA Fund</t>
         </is>
       </c>
-      <c r="C22" s="1" t="inlineStr">
+      <c r="C18" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -1914,34 +1629,74 @@
 Only successful applicants will be contacted; no individual feedback provided to unsuccessful applicants</t>
         </is>
       </c>
-      <c r="D22" s="1" t="inlineStr">
+      <c r="D18" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E22" s="1" t="inlineStr">
+      <c r="E18" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F22" s="1" t="inlineStr">
+      <c r="F18" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-8th-call-for-proposals-small-size-grants-global-eba-fund-global-eba-fund-opg-26-00177</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="95" customHeight="1">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B23" s="1" t="inlineStr">
+    <row r="19" ht="95" customHeight="1">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Whitley Award 2027</t>
+        </is>
+      </c>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>About the Grant: 
+An annual grant by the Whitley Fund for Nature (WFN) recognising grassroots conservation leaders in the Global South, providing funding to support and scale up proven, science-based solutions that deliver lasting impact for both people and nature.
+ About the Award 
+Whitley Awards support grassroots conservation leaders in the Global South. Through funding, training and profile, they help conservationists scale up effective projects that are founded in science and carried out with communities. Whitley Awards are for dynamic, mid-career conservationists who are leading vital conservation projects.
+ Grant Amount: £50,000 in project funding over one year
+ Eligibility
+Winners are nationals of the country in which they are working, seeking to scale up proven work that is embedded in the local community and would benefit from further funding, a profile boost, and international support.
+Projects must involve communities at the grassroots level and deliver practical action that is founded on science.
+You do not need to be invited or nominated to apply.</t>
+        </is>
+      </c>
+      <c r="D19" s="1" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E19" s="1" t="inlineStr">
+        <is>
+          <t>Oct 30, 2026</t>
+        </is>
+      </c>
+      <c r="F19" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-whitley-award-2027-whitley-fund-for-nature-wfn-opg-26-00153</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="95" customHeight="1">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIFAR Global Scholars Program 20272029 Cohort</t>
         </is>
       </c>
-      <c r="C23" s="1" t="inlineStr">
+      <c r="C20" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 CIFAR is a Canadian-based globally influential research organization that convenes the world’s most brilliant people across disciplines to advance transformative knowledge and solve humanity’s biggest problems, together. By supporting long-term interdisciplinary collaboration, CIFAR provides researchers with an unparalleled environment of trust, transparency and knowledge sharing. Our time-tested model inspires new directions of inquiry, accelerates discovery and yields breakthroughs across borders and academic disciplines. Through knowledge mobilization, we are catalysts for change in industry, government and society. Through our 15 research programs and the Pan-Canadian AI Strategy, CIFAR convenes close to 400 of the world’s top researchers from 141 institutions in 20 countries. CIFAR is generously supported by the governments of Canada, Alberta and Québec, as well as foundations, individuals, corporations and Canadian and international partner organizations.
@@ -1985,34 +1740,34 @@
  Application Deadline: November 4, 2026, 12:00 PM EST</t>
         </is>
       </c>
-      <c r="D23" s="1" t="inlineStr">
+      <c r="D20" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E23" s="1" t="inlineStr">
+      <c r="E20" s="1" t="inlineStr">
         <is>
           <t>Nov 4, 2026</t>
         </is>
       </c>
-      <c r="F23" s="1" t="inlineStr">
+      <c r="F20" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cifar-global-scholars-program-20272029-cohort-cifar-canadian-institute-for-advanced-research-opg-26-00183</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="95" customHeight="1">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B24" s="1" t="inlineStr">
+    <row r="21" ht="95" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for IWRS Teaching Innovation Award</t>
         </is>
       </c>
-      <c r="C24" s="1" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
@@ -2024,34 +1779,34 @@
 Two awards of $2,000 USD are available annually.</t>
         </is>
       </c>
-      <c r="D24" s="1" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E24" s="1" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>Nov 15, 2026</t>
         </is>
       </c>
-      <c r="F24" s="1" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="95" customHeight="1">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B25" s="1" t="inlineStr">
+    <row r="22" ht="95" customHeight="1">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for IWRS Teaching Innovation Award</t>
         </is>
       </c>
-      <c r="C25" s="1" t="inlineStr">
+      <c r="C22" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Insects are one of the most numerous and diverse animal groups on Earth.
@@ -2066,34 +1821,34 @@
 IWRS staff and Advisory Group members are not eligible to apply.</t>
         </is>
       </c>
-      <c r="D25" s="1" t="inlineStr">
+      <c r="D22" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E25" s="1" t="inlineStr">
+      <c r="E22" s="1" t="inlineStr">
         <is>
           <t>Nov 15, 2026</t>
         </is>
       </c>
-      <c r="F25" s="1" t="inlineStr">
+      <c r="F22" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00166</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="95" customHeight="1">
-      <c r="A26" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B26" s="1" t="inlineStr">
+    <row r="23" ht="95" customHeight="1">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Medium-Size Grants Call for Proposals Global EbA Fund</t>
         </is>
       </c>
-      <c r="C26" s="1" t="inlineStr">
+      <c r="C23" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -2150,34 +1905,34 @@
 Applications submitted via online portal (link shared on the Medium-Size Grants webpage from Oct 12)</t>
         </is>
       </c>
-      <c r="D26" s="1" t="inlineStr">
+      <c r="D23" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E26" s="1" t="inlineStr">
+      <c r="E23" s="1" t="inlineStr">
         <is>
           <t>Nov 16, 2026</t>
         </is>
       </c>
-      <c r="F26" s="1" t="inlineStr">
+      <c r="F23" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-medium-size-grants-call-for-proposals-global-eba-fund-global-eba-fund-opg-26-00178</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="95" customHeight="1">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B27" s="1" t="inlineStr">
+    <row r="24" ht="95" customHeight="1">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIEIF Grant 2026 Climate Intervention Environmental Impact Fund</t>
         </is>
       </c>
-      <c r="C27" s="1" t="inlineStr">
+      <c r="C24" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Climate Intervention Environmental Impact Fund (CIEIF) is a philanthropic fund focused on supporting responsible climate intervention field tests. It provides grants for activities such as environmental impact assessment (EIA), predictive impact modelling, and engagement with potentially affected stakeholders, including local communities and government agencies.
@@ -2204,34 +1959,34 @@
 Potential for scaling the innovation to a globally relevant level</t>
         </is>
       </c>
-      <c r="D27" s="1" t="inlineStr">
+      <c r="D24" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E27" s="1" t="inlineStr">
+      <c r="E24" s="1" t="inlineStr">
         <is>
           <t>Dec 1, 2026</t>
         </is>
       </c>
-      <c r="F27" s="1" t="inlineStr">
+      <c r="F24" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cieif-grant-2026-climate-intervention-environmental-impact-fund-climate-intervention-environmental-impact-fund-opg-26-00155</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="95" customHeight="1">
-      <c r="A28" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B28" s="1" t="inlineStr">
+    <row r="25" ht="95" customHeight="1">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 6th Annual Seeding The Future Global Food System Challenge</t>
         </is>
       </c>
-      <c r="C28" s="1" t="inlineStr">
+      <c r="C25" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are one of the largest and most respected private organisations for development cooperation and humanitarian aid in Germany. As a politically and confessionally independent organisation, our value-oriented actions are always based on ethical principles. Our vision is clear: "Zero Hunger by 2030"
@@ -2263,34 +2018,78 @@
 Individuals with no organizational entity</t>
         </is>
       </c>
-      <c r="D28" s="1" t="inlineStr">
+      <c r="D25" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E28" s="1" t="inlineStr">
+      <c r="E25" s="1" t="inlineStr">
         <is>
           <t>Jan 1, 2027</t>
         </is>
       </c>
-      <c r="F28" s="1" t="inlineStr">
+      <c r="F25" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-6th-annual-seeding-the-future-global-food-system-challenge-welthungerhilfe-opg-26-00180</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="95" customHeight="1">
-      <c r="A29" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B29" s="1" t="inlineStr">
+    <row r="26" ht="95" customHeight="1">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Microbiota &amp; Women's Health International Call for Projects</t>
+        </is>
+      </c>
+      <c r="C26" s="1" t="inlineStr">
+        <is>
+          <t>About the Grant
+An annual international research grant by the Biocodex Microbiota Foundation (BMF), rewarding research proposals on the microbiota and its implications in Women's Health and Disease. This year's theme: "Unraveling male-female genital microbiome interactions: mechanisms, transmission, and impact on vaginal dysbiosis."
+ Theme/Scope
+Proposals could include, but are not limited to, mechanistic studies elucidating how the penile microbiome contributes to the establishment, persistence, and recurrence of vaginal dysbiosis, including bacterial vaginosis. Areas of interest include microbial transmission dynamics during sexual activity, niche adaptation and persistence of BV-associated taxa in the penile environment, and the functional consequences of these interactions for vaginal community stability.
+Studies evaluating how current and emerging interventions (antibiotics, topical or systemic partner therapies, circumcision, or live biotherapeutic products) alter penile microbial ecology and influence treatment response and recurrence risk in female partners are also encouraged.
+ Purpose: From 2025, the Biocodex Microbiota Foundation rewards international research proposals involving the microbiota and its implication in Women's Health and Disease. Every year, the call for proposals covers a specific theme chosen by an International Scientific Committee. Either clinical or fundamental research proposals can be submitted. Maximum project duration: 3 years.
+ Eligibility
+Open to MDs, PhDs, or Pharm-Ds working in the subject area (gynecology, obstetrics, microbiology, infectious diseases, internal medicine, oncology, etc.).
+No geographic restrictions — all countries are eligible.
+A principal investigator who received a Women's Health International grant from BMF cannot reapply for this award for three years. However, winners of another BMF grant category can apply for this grant.
+Members of the Women's Health International Scientific Committee and their laboratory members are not allowed to apply as Principal Investigators.
+ Grant Amount
+€200,000 annually — awarded to researchers within universities, hospitals, or other research settings to finance equipment, operations, or staffing costs. Grants are NOT awarded to individuals directly (must be institutionally affiliated). Institution's overhead costs capped at 10%.</t>
+        </is>
+      </c>
+      <c r="D26" s="1" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="E26" s="1" t="inlineStr">
+        <is>
+          <t>Jan 15, 2027</t>
+        </is>
+      </c>
+      <c r="F26" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-microbiota-and-womens-health-international-call-for-projects-biocodex-microbiota-foundation-bmf-opg-26-00152</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="95" customHeight="1">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for BES Training and Travel Grants</t>
         </is>
       </c>
-      <c r="C29" s="1" t="inlineStr">
+      <c r="C27" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are a global community of scientists shining a spotlight on the intricacy and value of our natural world, providing the evidence for better decisions. Our vision is for people and nature to thrive in a world that values ecology.
@@ -2329,17 +2128,17 @@
  Application Deadline (Round 2): Opens 30 April 2026, closes 17 May 2026</t>
         </is>
       </c>
-      <c r="D29" s="1" t="inlineStr">
+      <c r="D27" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E29" s="1" t="inlineStr">
+      <c r="E27" s="1" t="inlineStr">
         <is>
           <t>May 17, 2027</t>
         </is>
       </c>
-      <c r="F29" s="1" t="inlineStr">
+      <c r="F27" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-bes-training-and-travel-grants-british-ecological-society-opg-26-00181</t>
         </is>

</xml_diff>

<commit_message>
Auto update Combined.xlsx [Wed Sep 16 07:07:51 UTC 2026]
</commit_message>
<xml_diff>
--- a/output/Combined.xlsx
+++ b/output/Combined.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -467,122 +467,10 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>SoW - Hiring an External Agency for Orientation and Capacity Building</t>
+          <t>ToR for Consultancy Service - Practitioner Knowledge Mapping Across Priority Livelihood Value Chains</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
-        <is>
-          <t>Room to Read’s Foundational Literacy Program in Jharkhand: Anchoring and Delivery of Orientation Programme for Jharkhand Field Workforce
-Scope of Work (SoW)
-for
-Hiring an External Agency for Orientation and Capacity Building
-Organizational Overview
-Founded in 2000 on the belief that World Change Starts with Educated Children®, Room to Read develops children’s foundational literacy skills, as well as life skills that promote gender equality. We nurture these essential skills in children by training and coaching educators, creating quality learning materials and spaces, strengthening education systems, and delivering programs directly and with partners – all while honouring the dignity of every child. Committed to accelerating learning outcomes for more children, more quickly, Room to Read has benefited children across 29 countries, with more than 17 million children actively benefiting from our programming in 2025 alone. Room to Read India’s literacy operations currently span across 12 states, with a focus on improving children’s reading skills, access to quality learning materials, and supportive learning environments. Room to Read envisions a world free from illiteracy and gender inequality, where all children have room to read, learn and grow. Visit us at https://www.roomtoreadindia.org/
-Jharkhand Foundational Literacy Project Overview
-Room to Read is preparing for a significant scale-up of its Foundational Literacy &amp; Numeracy initiative in Jharkhand, expanding implementation across multiple districts and requiring a substantial field workforce to support programme delivery. As Room to Read expands its field implementation in Jharkhand, a substantial number of staff will join different field-facing and supervisory roles.  As part of the planned scale-up, Room to Read expects to onboard more than 150 staff in Phase 1 across field implementation, supervisory and district-level leadership roles. A second cohort of approximately 120 additional staff is expected to be onboarded in Phase 2 as implementation expands to the remaining districts.
-Objective of the Assignment
-The overarching objective of this assignment is to ensure that over two phases 250+ team members in Jharkhand are ready for project implementation.
-Phase 1 will aim at getting all 150+ staff members ready for project implementation by March 31st, 2027.
-Phase 2 will do the same with additional 120+ team members by 30th April 2028.
-Agency Requirements &amp; Qualifications 
-The agency should preferably:
-Preferred 3 years of relevant experience in designing and delivering orientation, training or capability-building programmes for field-based teams, particularly in the education, development or government-facing sector.
-Have completed at least 2 similar assignments involving training across multiple batches, locations or large participant groups.
-Demonstrate experience in learning-needs assessment, adult-learning design, content development and participatory training methodologies.
-Demonstrate experience in developing facilitator guides, participant materials, simulations, assessments, job aids or other training resources, and provide 1-2 relevant samples where available.
-Have the ability to deliver training in Hindi and deploy an adequate pool of suitable facilitators for implementation across Jharkhand.
-Provide details and CVs of the proposed core team and key facilitators, including their qualifications, relevant experience, roles and expected level of engagement in the assignment. The agency should ensure continuity of key facilitators, with minimal changes during each phase of the assignment.
-Demonstrate experience in assessing training effectiveness through participant feedback, assessments, learning-progress tracking and/or follow-up or refresher support.
-Have established systems for project management, quality assurance, documentation, progress tracking and reporting, with the ability to maintain consistency across training cohorts.
-Provide details of at least 2 relevant past clients/assignments that may be referred to for verification of experience and performance.
-Room to Read India is inviting interesting agencies for Pre-Bid meeting on zoom as per details under:  
-Date : 14th Sep 2026
-Time: 3:00 PM to 4:00 PM -IST
-Zoom Meeting
-https://zoom.us/j/91517814040
-Meeting ID: 915 1781 4040</t>
-        </is>
-      </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>Sep 17, 2026</t>
-        </is>
-      </c>
-      <c r="F2" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/sow-hiring-an-external-agency-for-orientation-and-capacity-building-room-to-read-india-rfp-26-00346</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="95" customHeight="1">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>ToR - Project Consultant / Organization DRE Integration in PMFME Enterprises</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t>Terms of Reference (TOR) for Consultancy Services
-PowerUp PMFME-DRE 
-Integrating Decentralized Renewable Energy (DRE) in PMFME Food Processing Enterprises
-Title Project Consultant / Organization – DRE Integration in PMFME Enterprises
-Location
-Karnataka and Maharashtra.
-Bidders may apply for both states as a single assignment, or as a consortium with a designated lead entity covering both.
-Timeline 6 (six) Months
-Expected area of expertise Energy assessment, project implementation, financial analysis, capacity building, post-implementation audit, and documentation
-Apply Link https://forms.gle/gAmuuSxm3MkLofpF9
-Last Date for Apply 17th Sep 2026, 5 PM
-About SELCO Foundation:
-SELCO Foundation is an open-source, not-for-profit organization that engages in field-based R&amp;D and ecosystem building for the deployment of clean energy solutions that alleviate poverty by improving access to sustainable energy to underserved communities in tribal, rural, and urban poor areas. The organization works in collaboration with practitioners in the social sector, energy entrepreneurs, NGOs from various developmental sectors, and educational institutions to link the benefits of sustainable energy to poverty eradication. The organization works across verticals such as energy access, health, and livelihoods. You can find more information about the SELCO Foundation on our website: http://www.selcofoundation.org/
-Summary of the Project:
-SELCO Foundation is working to integrate Decentralized Renewable Energy (DRE) solutions into micro food processing enterprises supported under the PM Formalisation of Micro Food Processing Enterprises (PMFME) scheme. The program aims to improve energy access and productivity for PMFME beneficiaries in Karnataka and Maharashtra, targeting a total of 500 sites for DRE integration.
-A Project Consultant/Organization may apply to coordinate and facilitate site-level implementation across these two states, ensuring interventions align with beneficiary needs and have a meaningful impact.
-Goals and Objectives
-The program's key objectives are:
-Phase 1: Designing standardized DRE system options by system size, with leverage components identified for each - validated through a preliminary long/short list and sample site visits
-Phase 2: Conducting due diligence on listed beneficiaries, energy assessments, and facilitating implementation of DRE solutions
-Phase 3: Capacity building, post-implementation audit, and documentation of program learnings.</t>
-        </is>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>Sep 17, 2026</t>
-        </is>
-      </c>
-      <c r="F3" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/tor-project-consultant-organization-dre-integration-in-pmfme-enterprises-selco-foundation-rfp-26-00351</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="95" customHeight="1">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>ToR for Consultancy Service - Practitioner Knowledge Mapping Across Priority Livelihood Value Chains</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>Terms of Reference (TOR) for Consultancy Services
 Title Practitioner Knowledge Mapping Across Priority Livelihood Value Chains
@@ -617,34 +505,34 @@
 The agency is expected to independently identify and curate knowledge resources beyond those shared by the programme team</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>Sep 18, 2026</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-for-consultancy-service-practitioner-knowledge-mapping-across-priority-livelihood-value-chains-selco-foundation-rfp-26-00350</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="95" customHeight="1">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
+    <row r="3" ht="95" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>ToR - Behavioural Insights and Narrative Inquiry for the Climate Responsive Livelihood Programme Meghalaya</t>
         </is>
       </c>
-      <c r="C5" s="1" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Title  Behavioural Insights and Narrative Inquiry for the Climate Responsive Livelihood Programme, Meghalaya
 Timeline  2 months
@@ -662,34 +550,34 @@
 Rather than evaluating awareness or testing communication materials, the assignment should seek to uncover deeper behavioural and social drivers that influence livelihood choices and participation. The findings will inform a narrative architecture and mobilisation approach that resonates authentically with communities across the state.</t>
         </is>
       </c>
-      <c r="D5" s="1" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E5" s="1" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Sep 19, 2026</t>
         </is>
       </c>
-      <c r="F5" s="1" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-behavioural-insights-and-narrative-inquiry-for-the-climate-responsive-livelihood-programme-meghalaya-selco-foundation-rfp-26-00355</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="95" customHeight="1">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
+    <row r="4" ht="95" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>Expression of Interest EOI for Trade &amp; Livelihood Partners</t>
         </is>
       </c>
-      <c r="C6" s="1" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>Expression of Interest (EOI) for Trade &amp; Livelihood Partners
 Issued By: BharatCares
@@ -816,34 +704,34 @@
 Any prior work with tribal or rural communities, with references if available</t>
         </is>
       </c>
-      <c r="D6" s="1" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E6" s="1" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>Sep 20, 2026</t>
         </is>
       </c>
-      <c r="F6" s="1" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/expression-of-interest-eoi-for-trade-and-livelihood-partners-bharatcares-rfp-26-00340</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="95" customHeight="1">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
+    <row r="5" ht="95" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>RFP - Research Collaboration For Improved Application and Processing Techniques For Natural Dyes</t>
         </is>
       </c>
-      <c r="C7" s="1" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>REǪUEST FOR PROPOSALS (RFP)
 Research Collaboration For Improved Application and Processing Techniques For Natural Dyes
@@ -896,34 +784,34 @@
 Network with dyeing units and textile industry associations</t>
         </is>
       </c>
-      <c r="D7" s="1" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>Climate</t>
         </is>
       </c>
-      <c r="E7" s="1" t="inlineStr">
+      <c r="E5" s="1" t="inlineStr">
         <is>
           <t>Sep 20, 2026</t>
         </is>
       </c>
-      <c r="F7" s="1" t="inlineStr">
+      <c r="F5" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfp-research-collaboration-for-improved-application-and-processing-techniques-for-natural-dyes-chitrika-rfp-26-00343</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="95" customHeight="1">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
+    <row r="6" ht="95" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>RFP - Agronomic Research Study For Natural Dye Crop Development</t>
         </is>
       </c>
-      <c r="C8" s="1" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>REǪUEST FOR PROPOSALS (RFP)
 Agronomic Research Study For Natural Dye Crop Development
@@ -982,34 +870,104 @@
 Experience working on natural dye</t>
         </is>
       </c>
-      <c r="D8" s="1" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E8" s="1" t="inlineStr">
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>Sep 20, 2026</t>
         </is>
       </c>
-      <c r="F8" s="1" t="inlineStr">
+      <c r="F6" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfp-agronomic-research-study-for-natural-dye-crop-development-chitrika-rfp-26-00344</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="95" customHeight="1">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="inlineStr">
+    <row r="7" ht="95" customHeight="1">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>RFPs Invited for Using an Agent Based Model to Predict the Impact of City-Level Policies on the Adoption of Distributed Renewable Energy</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>About C40:
+C40 is a network of nearly 100 mayors of the world's leading cities working to deliver urgent climate action and create a future where everyone, everywhere, can thrive. Mayors of C40 cities are committed to using a science-based, people-focused approach to limit global heating in line with the Paris Agreement, working alongside labour, business, youth climate movement, and civil society representatives to help halve emissions by 2030.
+ Project Summary/Background:
+C40 represents 5 member cities in India (Mumbai, Ahmedabad, Bengaluru, Chennai, New Delhi) plus Karachi. C40's Research team is launching a project to accelerate Indian grid decarbonisation and improve public health, funded by the Wellcome Trust, in collaboration with Ashoka ACPET and CHART centres. The project has 3 work packages (national, urban, and rural scale); this RFP covers Work Package 2 (WP2) — the urban-scale component, led by C40, focusing on city-level interventions to accelerate distributed solar energy deployment and reduce coal dependence in Mumbai and Chennai.
+ Objective:
+Apply an Agent-Based Modelling (ABM) approach to analyse the impact of specific local policy measures on the adoption of solar and batteries by residential and commercial actors in Mumbai and Chennai. The Supplier will:
+Develop methodology, assess data needs, conduct local ground surveys, and model baseline energy consumption
+Develop/repurpose an ABM to assess how policy interventions (renewable energy mandates, metering changes, peak-hour tariff changes, etc.) impact uptake of distributed solar/batteries
+Model how changes in solar use translate to changes in capacity factors of specific coal power plants and resulting emission reductions (GHG, PM2.5, NOx)
+ Scope: Covers all energy use in the built environment and industries within Mumbai and Chennai's urban boundaries — households (owners/renters, income levels) and businesses (including industrial). Focus on distributed solar electricity generation/use and battery storage. Excludes solar thermal solutions and institutional buildings. Energy generation model covers the whole state.
+ Deliverables:
+Methodology, Local Ground Surveys &amp; Data Collection — Methodology document (20 pages max), data mapping, sample survey results, data collection documents
+Agent-Based Model of Renewable Energy Uptake — Updated methodology, ABM simulation runs, outputs report (up to 15 pages)
+Power Plant Utilisation Rate Modelling — Updated methodology, plant-level energy use files (hourly), findings report (up to 15 pages)
+ AI Use Restriction: Use of AI-supported tools must be kept to an absolute minimum; no final output (text/visuals) may be AI-produced. Any AI tool use must be justified in methodology. Results must be validated via human oversight and cross-referencing with trusted sources. C40 data is confidential and cannot be shared with AI tools.
+ Proposal Requirements: Must be under 15 pages (all-inclusive), covering: responsiveness to evaluation criteria, ABM approach &amp; survey strategy, relevant experience (with reference letters from past 3 years, not counted in page limit), risk identification/mitigation, fee justification, implementation timeline, key personnel resumes, additional support needed, and proposed working partnership structure with C40.
+ Evaluation Criteria &amp; Weighting:
+Methodology rigour and delivery clarity: 20%
+Technical Expertise (ABM, energy modelling, Indian policy context): 30%
+Project management experience: 20%
+Cost Reasonableness: 20%
+Equity and Alignment (India-based organizations strongly encouraged): 10%
+ Project Budget: USD 50,000 for all deliverables (payment per milestone approval; travel expenses included)
+ Contract Type: Professional services contract (Note: this is a contract opportunity, not a grant — organisations unable to accept professional services contracts should not apply); C40 Standard Services Contract terms are non-negotiable
+ Key Dates:
+RFP Sent: September 1, 2026
+Questions Submitted to C40: September 10, 2026
+C40 Responds to Questions: September 14, 2026
+ Deadline for Receiving Offers: 12 PM EST, 20 September 2026
+Clarification of Offers: September 25, 2026
+Evaluation of Proposals: September 28, 2026
+Interviews (if needed): September 29, 2026
+Selection Decision: September 30, 2026
+All Suppliers Notified: October 10, 2026
+ Project Delivery Timeline:
+Deliverable 1: March 30, 2026 (note: this date appears to predate the RFP issue date — likely a typo in the source document for 2027)
+Deliverable 2: May 15, 2026 (same note applies)
+Deliverable 3: June 15, 2025 (same note — likely should read 2027)
+Project runs until: June 30, 2027</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>Sep 20, 2026</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/rfps-invited-for-using-an-agent-based-model-to-predict-the-impact-of-city-level-policies-on-the-adoption-of-distributed-renewable-energy-c40-cities-rfp-26-00357</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="95" customHeight="1">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>E-Tender Request for Digital Communication Website Development and Social Media Campaign for Colors of Nature</t>
         </is>
       </c>
-      <c r="C9" s="1" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>REǪUEST FOR PROPOSALS (RFP)
 Digital Communication, Website Development and Social Media Campaign
@@ -1055,34 +1013,34 @@
 Ready to develop a women led and based digital marketing team</t>
         </is>
       </c>
-      <c r="D9" s="1" t="inlineStr">
+      <c r="D8" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E9" s="1" t="inlineStr">
+      <c r="E8" s="1" t="inlineStr">
         <is>
           <t>Sep 20, 2026</t>
         </is>
       </c>
-      <c r="F9" s="1" t="inlineStr">
+      <c r="F8" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/e-tender-request-for-digital-communication-website-development-and-social-media-campaign-for-colors-of-nature-chitrika-rfp-26-00342</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="95" customHeight="1">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
+    <row r="9" ht="95" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Wellbeing Research Grants Funding Better Evaluations of AI's Impact on Wellbeing</t>
         </is>
       </c>
-      <c r="C10" s="1" t="inlineStr">
+      <c r="C9" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We're an AI research company that builds reliable, interpretable, and steerable AI systems. Our first product is Claude, an AI assistant for tasks at any scale. Our research interests span multiple areas including natural language, human feedback, scaling laws, reinforcement learning, code generation, and interpretability. 
@@ -1101,34 +1059,34 @@
  Funding Amount: Total program pool of $5 million (individual grant sizes not specified on the page)</t>
         </is>
       </c>
-      <c r="D10" s="1" t="inlineStr">
+      <c r="D9" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E10" s="1" t="inlineStr">
+      <c r="E9" s="1" t="inlineStr">
         <is>
           <t>Sep 21, 2026</t>
         </is>
       </c>
-      <c r="F10" s="1" t="inlineStr">
+      <c r="F9" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-wellbeing-research-grants-funding-better-evaluations-of-ais-impact-on-wellbeing-anthropic-opg-26-00175</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="95" customHeight="1">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="inlineStr">
+    <row r="10" ht="95" customHeight="1">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for GEF SGP CSO Challenge Program</t>
         </is>
       </c>
-      <c r="C11" s="1" t="inlineStr">
+      <c r="C10" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global Environment Facility Small Grants Programme (SGP) is a global initiative implemented by the United Nations Development Programme (UNDP) on behalf of the Global Environment Facility (GEF). Since its launch in 1992, SGP has empowered communities worldwide to take action on environmental challenges while improving livelihoods. As a GEF Corporate Programme, SGP provides direct support to civil society organisations and community-based organisations to design and implement innovative, locally driven solutions. The programme places strong emphasis on inclusion, ensuring meaningful participation of Indigenous Peoples, youth, women and girls, and other underrepresented groups.
@@ -1177,34 +1135,34 @@
 Risk management and mitigation</t>
         </is>
       </c>
-      <c r="D11" s="1" t="inlineStr">
+      <c r="D10" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E11" s="1" t="inlineStr">
+      <c r="E10" s="1" t="inlineStr">
         <is>
           <t>Sep 23, 2026</t>
         </is>
       </c>
-      <c r="F11" s="1" t="inlineStr">
+      <c r="F10" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-gef-sgp-cso-challenge-program-gef-small-grants-programme-sgp-opg-26-00184</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="95" customHeight="1">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="inlineStr">
+    <row r="11" ht="95" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>RFP for Impact Assessment</t>
         </is>
       </c>
-      <c r="C12" s="1" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>Introduction
 Titan Company Limited, a member of the Tata Group, has a long-standing commitment to Corporate Social Responsibility (CSR) in India. The company's CSR initiatives derive its philosophy from the Company’s vision statement: “We create elevating experiences for the people we touch and significantly impact the world we work in”. The initiatives are designed to promote inclusive growth, empower communities, and contribute to the country's socio-economic development. The program includes Titan’s CSR policy is governed by a dedicated CSR Committee that ensures transparency and compliance with regulatory requirements. The program includes Girl Child Education, Skill and Entrepreneurship Development, supporting Indian Heritage Arts and Crafts, Integrated Village Development Programme, Eye Care and Affirmative Action. Titan's CSR policy is governed by a dedicated CSR Committee that ensures transparency and compliance with regulatory requirements.
@@ -1238,216 +1196,34 @@
 Timeline: Proposal submission deadline: September 24, 2026</t>
         </is>
       </c>
-      <c r="D12" s="1" t="inlineStr">
+      <c r="D11" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E12" s="1" t="inlineStr">
+      <c r="E11" s="1" t="inlineStr">
         <is>
           <t>Sep 24, 2026</t>
         </is>
       </c>
-      <c r="F12" s="1" t="inlineStr">
+      <c r="F11" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfp-for-impact-assessment-titan-rfp-26-00354</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="95" customHeight="1">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B13" s="1" t="inlineStr">
-        <is>
-          <t>Application Invited for Giving Joy Microgrant</t>
-        </is>
-      </c>
-      <c r="C13" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-Giving Joy is a US-based nonprofit that strengthens and inspires women’s entrepreneurship worldwide. Through its micro-grants and mentorship program, Giving Joy helps women establish or improve their businesses and initiatives—for their benefit and the benefit of their communities. To date, Giving Joy has awarded over 88 grants to women-led initiatives in 26 countries.
- 2026 Grant Cycle
-Beginning in 2026, Giving Joy has moved to two global grant cycles per year.
-The organization states that this change was made after operating multiple regional rounds, with the aim of:
-Providing clearer timelines for applicants
-Increasing the quality and depth of application reviews
-Reducing administrative burden
-Improving support for grantees
-Focusing communications and fundraising more effectively
-Continuing to reach women entrepreneurs globally without dividing applications by geography
-Each cycle is open to women entrepreneurs worldwide.
- Eligible Fields / Activities
-There is no restriction to a particular field such as health.
-Applicants can propose activities in:
-Any field
-Trade
-Occupation
-Craft
- What Does Giving Joy Look For?
-Giving Joy prioritizes:
-Innovative ideas
-Creative ideas
-Strong potential for social impact
-Initiative
-Real community impact
-Clear economic and/or social benefits for women and girls
- Grant Amount
-Maximum Grant
-Up to $500 USD
-The exact award amount is determined by Giving Joy based on:
-Proposed activities
-Availability of funding
- Grant Duration
-The grant period is six months.</t>
-        </is>
-      </c>
-      <c r="D13" s="1" t="inlineStr">
-        <is>
-          <t>Safety</t>
-        </is>
-      </c>
-      <c r="E13" s="1" t="inlineStr">
-        <is>
-          <t>Sep 30, 2026</t>
-        </is>
-      </c>
-      <c r="F13" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/application-invited-for-giving-joy-microgrant-giving-joy-opg-26-00185</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="95" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Signals of Change Shaping the Future of Sexual and Reproductive Health and Rights SRHR</t>
-        </is>
-      </c>
-      <c r="C14" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-The World Health Organization's mission: to promote health, keep the world safe, and serve the vulnerable. Working through offices in more than 150 countries, WHO staff work side by side with governments and other partners to ensure the highest attainable level of health for all people.
- About the Opportunity
-HRP and its UN co-sponsors are leading a global Sexual and Reproductive Health and Rights (SRHR) foresight and research prioritization process for 2026–2036. This open public consultation invites diverse stakeholder input to identify "signals of change" — emerging trends, shifts, or disruptions — that could shape the future of SRHR over the next decade. The process uses foresight methodology (not prediction) to explore plausible futures and will culminate in a published report and research agenda in 2027.
- Guiding Questions
-What future trends will shape or constrain SRHR over the next 10 years?
-What evidence and research investments are needed today to prepare SRHR for the futures we may face?
- Scope of Submissions 
-Economic systems; social infrastructure; structural discrimination; conflict/forced migration/displacement; mega-trends (demographic shifts, climate change, digital transformation/AI, urbanization); conditions of daily life; rights/legal/governance systems; health systems; media/misinformation; and changes in the research ecosystem.
- Who Can Participate 
-Open to individuals and organizations globally, including:
-Health workers, professional associations, clinical networks
-Civil society, community groups, youth-led organizations, rights movements
-Governments, parliamentarians, regulators, public sector bodies
-Researchers, academia, think tanks, technical experts
-UN agencies, multilateral/humanitarian/development organizations
-Funders, philanthropy, private sector, tech/innovation organizations
-Media, communications, journalism
-Anyone with relevant lived experience or perspective
-Special interest in submissions from health worker, community, youth, and rights-movement spaces not typically represented in published forums.
- Submission Requirements: Descriptive information (name, contact email, country, sector) required alongside each submission; formal published evidence is helpful but not required — practice-based experience and field examples are also welcome. Submissions are kept confidential and anonymized before analysis.</t>
-        </is>
-      </c>
-      <c r="D14" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E14" s="1" t="inlineStr">
-        <is>
-          <t>Sep 30, 2026</t>
-        </is>
-      </c>
-      <c r="F14" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-signals-of-change-shaping-the-future-of-sexual-and-reproductive-health-and-rights-srhr-world-health-organization-opg-26-00176</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="95" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Setting up Viral Research and Diagnosis Laboratories VRDL in Medical Colleges/Hospitals/Medical Institutions</t>
-        </is>
-      </c>
-      <c r="C15" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-The President notified the creation of the Department of Health Research under the Ministry of Health &amp; Family Welfare through an amendment to the Government of India (Allocation of Business) Rules, 1961 on the 17th September 2007. The Department of Health Research was formally launched on 5th October 2007 by the Minister for Science &amp; Technology and Earth Sciences in a function presided over by the Minister for Health &amp; Family Welfare, in the presence, inter-alia, of the Minister of State for Health &amp; Family Welfare.
-The Department became functional from November 2008 with the appointment of first Secretary of the Department The aim of the DHR is to bring modern health technologies to the people through research and innovations related to diagnosis, treatment methods and vaccines for prevention, to translate them into products and processes and, in synergy with concerned organizations, introduce these innovations into public health system.
- About the Opportunity:
-Under DHR's scheme "Setting-up of nation-wide network of laboratories for managing epidemics and national calamities," proposals are invited from Medical Colleges/Hospitals/Research Institutions to establish a Medical College &amp; Research Institute Level – Viral Research and Diagnosis Laboratory (MCL-VRDL). The existing network comprises 167 VRDLs (11 Regional, 27 State, 129 Medical College level) across 27 states and 5 UTs, aimed at early detection of infectious pathogens, outbreak surveillance, and research on emerging/re-emerging viral diseases.
- Objectives:
-Establish capacity for early detection of common and high-risk infectious pathogens
-Strengthen syndromic surveillance ecosystem for outbreak detection
-Undertake R&amp;D on emerging, re-emerging and novel viruses
- Eligibility (Institution-level):
-State Government Medical Colleges
-Central Government Medical Colleges and Research Institutes
-Armed Forces Medical Institutions/Hospitals
-Railway and other Central Government health institutions
-Private medical colleges ranked in top 50 NIRF ranking
-Must have a dedicated Microbiology department with qualified faculty
-Must have &gt;200 sq.m. area available in existing building (preferably within Microbiology Dept.)
- Funding Provision:
-Non-recurring assistance: Rs. 1.55 crore total
-Rs. 66.8 lakhs — Civil Work (infrastructure modification)
-Rs. 88.2 lakhs — Equipment (complete lab setup)
-No recurring expenditure (staff salaries, consumables, contingency) is provided — to be borne by the host institution
- Role &amp; Responsibilities of the Lab:
-Conduct routine diagnosis of infectious pathogens
-Participate in syndromic and event-based surveillance
-Provide support during outbreaks/epidemics
-Share data with ICMR
- Selection Criteria:
-Meeting eligibility does not guarantee selection; merit-based evaluation by a technical committee
-Preference to institutions in geographically underserved regions
-Weightage for technical strength (qualified faculty, biosafety practices, outbreak investigation experience, publications, patents, externally funded projects)
-Additional weightage for molecular diagnostics, genomic surveillance, One Health research capability, and commitment to long-term recurring support
-Private medical colleges: only top-50 NIRF-ranked institutions considered</t>
-        </is>
-      </c>
-      <c r="D15" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E15" s="1" t="inlineStr">
-        <is>
-          <t>Sep 30, 2026</t>
-        </is>
-      </c>
-      <c r="F15" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-setting-up-viral-research-and-diagnosis-laboratories-vrdl-in-medical-collegeshospitalsmedical-institutions-department-of-health-research-dhr-ministry-of-health-and-family-welfare-government-of-india-opg-26-00174</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="95" customHeight="1">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B16" s="1" t="inlineStr">
+    <row r="12" ht="95" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
         <is>
           <t>EOI Inviting Expression of Interest-cum-Proposal for Setting Up District De-Addiction Centres under NAPDDR</t>
         </is>
       </c>
-      <c r="C16" s="1" t="inlineStr">
+      <c r="C12" s="1" t="inlineStr">
         <is>
           <t>About us
 In the year 1985-86, the erstwhile Ministry of Welfare was bifurcated into the Department of Women and Child Development and the Department of Welfare. Simultaneously, the Scheduled Castes Development Division, Tribal Development Division and the Minorities and Backward Classes Welfare Division were moved from the Ministry of Home Affairs and also the Wakf Division from the Ministry of Law to form the then Ministry of Welfare Subsequently, the name of the Ministry was changed to the Ministry of Social Justice &amp; Empowerment in May, 1998. Further, in October, 1999, the Tribal Development Division had moved out to form a separate Ministry of Tribal Affairs. In January, 2007, the Minorities Division along with Wakf Unit have been moved out of the Ministry and formed as a separate Ministry and the Child Development Division has gone to the Ministry of Women &amp; Child Development.
@@ -1487,19 +1263,252 @@
 11. Department of Social Justice and Empowerment (DoSJE) reserves the right to cancel this notice, andior invite afresh proposals with or without amendments to this document without liability or any obligation for such document, and without assigning any reason. DoSJE reserves the right to take final decision regarding selection of implementing agency or project.</t>
         </is>
       </c>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>Sep 30, 2026</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/eoi-inviting-expression-of-interest-cum-proposal-for-setting-up-district-de-addiction-centres-under-napddr-ministry-of-social-justice-and-empowerment-goi-rfp-26-00356</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="95" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>Application Invited for Giving Joy Microgrant</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+Giving Joy is a US-based nonprofit that strengthens and inspires women’s entrepreneurship worldwide. Through its micro-grants and mentorship program, Giving Joy helps women establish or improve their businesses and initiatives—for their benefit and the benefit of their communities. To date, Giving Joy has awarded over 88 grants to women-led initiatives in 26 countries.
+ 2026 Grant Cycle
+Beginning in 2026, Giving Joy has moved to two global grant cycles per year.
+The organization states that this change was made after operating multiple regional rounds, with the aim of:
+Providing clearer timelines for applicants
+Increasing the quality and depth of application reviews
+Reducing administrative burden
+Improving support for grantees
+Focusing communications and fundraising more effectively
+Continuing to reach women entrepreneurs globally without dividing applications by geography
+Each cycle is open to women entrepreneurs worldwide.
+ Eligible Fields / Activities
+There is no restriction to a particular field such as health.
+Applicants can propose activities in:
+Any field
+Trade
+Occupation
+Craft
+ What Does Giving Joy Look For?
+Giving Joy prioritizes:
+Innovative ideas
+Creative ideas
+Strong potential for social impact
+Initiative
+Real community impact
+Clear economic and/or social benefits for women and girls
+ Grant Amount
+Maximum Grant
+Up to $500 USD
+The exact award amount is determined by Giving Joy based on:
+Proposed activities
+Availability of funding
+ Grant Duration
+The grant period is six months.</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>Sep 30, 2026</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/application-invited-for-giving-joy-microgrant-giving-joy-opg-26-00185</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="95" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Signals of Change Shaping the Future of Sexual and Reproductive Health and Rights SRHR</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+The World Health Organization's mission: to promote health, keep the world safe, and serve the vulnerable. Working through offices in more than 150 countries, WHO staff work side by side with governments and other partners to ensure the highest attainable level of health for all people.
+ About the Opportunity
+HRP and its UN co-sponsors are leading a global Sexual and Reproductive Health and Rights (SRHR) foresight and research prioritization process for 2026–2036. This open public consultation invites diverse stakeholder input to identify "signals of change" — emerging trends, shifts, or disruptions — that could shape the future of SRHR over the next decade. The process uses foresight methodology (not prediction) to explore plausible futures and will culminate in a published report and research agenda in 2027.
+ Guiding Questions
+What future trends will shape or constrain SRHR over the next 10 years?
+What evidence and research investments are needed today to prepare SRHR for the futures we may face?
+ Scope of Submissions 
+Economic systems; social infrastructure; structural discrimination; conflict/forced migration/displacement; mega-trends (demographic shifts, climate change, digital transformation/AI, urbanization); conditions of daily life; rights/legal/governance systems; health systems; media/misinformation; and changes in the research ecosystem.
+ Who Can Participate 
+Open to individuals and organizations globally, including:
+Health workers, professional associations, clinical networks
+Civil society, community groups, youth-led organizations, rights movements
+Governments, parliamentarians, regulators, public sector bodies
+Researchers, academia, think tanks, technical experts
+UN agencies, multilateral/humanitarian/development organizations
+Funders, philanthropy, private sector, tech/innovation organizations
+Media, communications, journalism
+Anyone with relevant lived experience or perspective
+Special interest in submissions from health worker, community, youth, and rights-movement spaces not typically represented in published forums.
+ Submission Requirements: Descriptive information (name, contact email, country, sector) required alongside each submission; formal published evidence is helpful but not required — practice-based experience and field examples are also welcome. Submissions are kept confidential and anonymized before analysis.</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>Sep 30, 2026</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-signals-of-change-shaping-the-future-of-sexual-and-reproductive-health-and-rights-srhr-world-health-organization-opg-26-00176</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="95" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Setting up Viral Research and Diagnosis Laboratories VRDL in Medical Colleges/Hospitals/Medical Institutions</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+The President notified the creation of the Department of Health Research under the Ministry of Health &amp; Family Welfare through an amendment to the Government of India (Allocation of Business) Rules, 1961 on the 17th September 2007. The Department of Health Research was formally launched on 5th October 2007 by the Minister for Science &amp; Technology and Earth Sciences in a function presided over by the Minister for Health &amp; Family Welfare, in the presence, inter-alia, of the Minister of State for Health &amp; Family Welfare.
+The Department became functional from November 2008 with the appointment of first Secretary of the Department The aim of the DHR is to bring modern health technologies to the people through research and innovations related to diagnosis, treatment methods and vaccines for prevention, to translate them into products and processes and, in synergy with concerned organizations, introduce these innovations into public health system.
+ About the Opportunity:
+Under DHR's scheme "Setting-up of nation-wide network of laboratories for managing epidemics and national calamities," proposals are invited from Medical Colleges/Hospitals/Research Institutions to establish a Medical College &amp; Research Institute Level – Viral Research and Diagnosis Laboratory (MCL-VRDL). The existing network comprises 167 VRDLs (11 Regional, 27 State, 129 Medical College level) across 27 states and 5 UTs, aimed at early detection of infectious pathogens, outbreak surveillance, and research on emerging/re-emerging viral diseases.
+ Objectives:
+Establish capacity for early detection of common and high-risk infectious pathogens
+Strengthen syndromic surveillance ecosystem for outbreak detection
+Undertake R&amp;D on emerging, re-emerging and novel viruses
+ Eligibility (Institution-level):
+State Government Medical Colleges
+Central Government Medical Colleges and Research Institutes
+Armed Forces Medical Institutions/Hospitals
+Railway and other Central Government health institutions
+Private medical colleges ranked in top 50 NIRF ranking
+Must have a dedicated Microbiology department with qualified faculty
+Must have &gt;200 sq.m. area available in existing building (preferably within Microbiology Dept.)
+ Funding Provision:
+Non-recurring assistance: Rs. 1.55 crore total
+Rs. 66.8 lakhs — Civil Work (infrastructure modification)
+Rs. 88.2 lakhs — Equipment (complete lab setup)
+No recurring expenditure (staff salaries, consumables, contingency) is provided — to be borne by the host institution
+ Role &amp; Responsibilities of the Lab:
+Conduct routine diagnosis of infectious pathogens
+Participate in syndromic and event-based surveillance
+Provide support during outbreaks/epidemics
+Share data with ICMR
+ Selection Criteria:
+Meeting eligibility does not guarantee selection; merit-based evaluation by a technical committee
+Preference to institutions in geographically underserved regions
+Weightage for technical strength (qualified faculty, biosafety practices, outbreak investigation experience, publications, patents, externally funded projects)
+Additional weightage for molecular diagnostics, genomic surveillance, One Health research capability, and commitment to long-term recurring support
+Private medical colleges: only top-50 NIRF-ranked institutions considered</t>
+        </is>
+      </c>
+      <c r="D15" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E15" s="1" t="inlineStr">
+        <is>
+          <t>Sep 30, 2026</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-setting-up-viral-research-and-diagnosis-laboratories-vrdl-in-medical-collegeshospitalsmedical-institutions-department-of-health-research-dhr-ministry-of-health-and-family-welfare-government-of-india-opg-26-00174</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="95" customHeight="1">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>Applications Open Draper Richards Kaplan Foundation Funding for Social Enterprises</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t>About us
+Started in 2002, Draper Richards Kaplan Foundation (DRK) is a global venture philanthropy firm supporting early stage, high impact social enterprises. Borrowed from our venture capital legacy, DRK finds, funds, and supports exceptional leaders building innovative solutions to some of the world’s most challenging social and environmental problems. Since beginning this work nearly 25 years ago, DRK has invested in more than 270 organizations that have collectively impacted over 610 million lives to date.
+Draper Richards Kaplan Foundation accepts applications for funding year-round. Completing an application is the first step of our process and allows us to get to know you and your social enterprise so we can begin assessing your organization’s alignment with our funding thesis.
+To help make this process manageable and accessible, we have designed the application to be relatively simple and minimally burdensome. The online application should take about 30-60 minutes to complete. If you would like to save your progress and resume later, please be sure to check the box at the top of the online form to save your information.
+Please upload with your application a written executive summary, pitch deck, or business plan document addressing the following topics. Please feel free to reuse or repurpose existing materials if you feel that they would provide relevant information.
+Any additional materials (e.g., financials, impact reports, etc.) are welcome, but completely optional.
+Problem and Solution
+Please succinctly describe the mission and objectives of the organization.
+Please describe the social problem your organization addresses.
+Please describe the solution your organization provides.
+Impact
+Please explain how your organization solves (or contributes to solving) the social problem in a way that improves on existing efforts.
+Please explain how your solution supports an underserved population, including the benefits that population has seen from your pilot(s).
+Please explain how your approach is unique, including in comparison to other initiatives or organizations addressing the same problem if possible/relevant.
+Please describe the organization’s tangible results to date, detailing how you plan to measure organizational outcomes and success in the future.
+Scale
+Please explain how you plan to scale the organization over time.
+Please explain the main sources of earned income that your organization will use to sustain your work over time.
+Leader
+Please attach a standard resume/CV for the entrepreneur(s) and/or key leadership team members (e.g., CEO, COO, ED, etc.). Applications with text bios for entrepreneurs or members of the leadership team will not be considered.</t>
+        </is>
+      </c>
       <c r="D16" s="1" t="inlineStr">
         <is>
-          <t>Governance</t>
+          <t>Climate</t>
         </is>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>Sep 30, 2026</t>
+          <t>Oct 10, 2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/rfps/eoi-inviting-expression-of-interest-cum-proposal-for-setting-up-district-de-addiction-centres-under-napddr-ministry-of-social-justice-and-empowerment-goi-rfp-26-00356</t>
+          <t>https://onepurpos.in/openings/grants/applications-open-draper-richards-kaplan-foundation-funding-for-social-enterprises-draper-richards-kaplan-foundation-opg-26-00188</t>
         </is>
       </c>
     </row>
@@ -1563,10 +1572,73 @@
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
+          <t>Applications Invited for Comparison of PFAS Contributions to Agricultural Systems</t>
+        </is>
+      </c>
+      <c r="C18" s="1" t="inlineStr">
+        <is>
+          <t>Project Objectives:
+Report per- and polyfluoroalkyl substance (PFAS) concentrations from a variety of agricultural inputs — animal manures, fertilizers, pesticides, composts, soil amendments, seed coatings, and biosolids-based products
+Compare the impact of various agricultural inputs on PFAS concentration in the soil profile over varying timeframes
+Evaluate the fate and transport of different inputs to PFAS contributions in agricultural systems at field-scale
+Determine relative contributions from biosolids-based products vs. other inputs to help develop/prioritize risk management strategies
+ Background/Rationale:
+Growing concern exists over human exposure to PFAS through biosolids land application on agricultural systems, with regulatory bans on biosolids land application enacted or proposed in at least 12 U.S. states. Utilities relying on land application for biosolids management are scrambling for alternative disposal pathways. The U.S. EPA's 2026 draft guidance noted its earlier 2025 draft risk assessment of PFOA/PFOS-contaminated sewage sludge lacked important contextual information (e.g., a national survey of PFOA/PFOS concentrations). Risk assessments have focused primarily on biosolids, with less attention to PFAS contributions from other sources — manures, compost, fertilizers, pesticides, seed coatings, irrigation water, farming practices, and atmospheric deposition. A Minnesota Pollution Control Agency review found 12 inert pesticide ingredients classified as PFAS. This project aims to improve understanding of PFAS risks from the wider range of agricultural inputs to support strategic resource allocation and inform policy amid surging fertilizer prices and shifts toward local circular resources.
+ Research Approach:
+Develop a baseline of knowledge on PFAS in biosolids and non-biosolids agricultural inputs via literature review, analytical methods evaluation, and examination of manufacturing/processing pathways; identify data gaps and uncertainties
+Measure/report compound-specific PFAS concentrations and profiles in agricultural inputs using standardized methods, including precursor characteristics for source attribution where possible
+Characterize PFAS contributions via literature review, data analysis, and field sampling — comparing soil profile/plant tissue composition between fields with non-biosolids inputs vs. biosolids-applied systems; study should test hypotheses on PFAS sources, transformation, retention, and mobility
+Optional additional focus areas: influence of soil/hydrologic/hydrochemistry conditions on PFAS behavior; degradation/transformation pathways; relative PFAS contributions across product lifecycle stages (manufacturing, bagging, delivery, etc.)
+Research approach should be hypothesis-driven, detailing specific end-user needs, and proposers are encouraged to leverage existing projects on PFAS plant uptake/fate/transport.
+ Expected Deliverables:
+Research report (WRF's Research Report Template) including: literature review, PFAS analysis of select products, risk management implications/prioritization recommendations, agriculture end-use guidance
+A webcast or workshop to share findings
+Optional additional deliverables: relative risk framework (mass input/fate/exposure/risk), decision support guide for farmers/regulators/utilities, plain language fact sheet, comparative PFAS mass input tool (spreadsheet/calculator)
+ Project Duration: 36 months from contract start date (longer than the other two WRF grants above, which were 24 months)
+ Eligibility to Submit:
+Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible. Not open to individuals (same structure as the two prior WRF grants).
+ Budget/Funding:
+Maximum WRF funding: $400,000 (the largest of the three WRF grants shared so far)
+Applicant must contribute at least 33% of the project award as additional resources (cost share, applicant in-kind, or third-party in-kind per 2 CFR Part 200.306)
+Proposals not meeting the 33% minimum match will not be accepted
+ Proposal Evaluation Criteria:
+Understanding the Problem and Responsiveness to RFP: 20 points
+Technical and Scientific Merit: 30 points
+Qualifications, Capabilities, and Management: 20 points
+Communication Plan, Deliverables, and Applicability: 15 points
+Budget and Schedule: 15 points
+ Compliance Standards: OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
+ Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00) — same deadline as the other two WRF grants</t>
+        </is>
+      </c>
+      <c r="D18" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E18" s="1" t="inlineStr">
+        <is>
+          <t>Oct 26, 2026</t>
+        </is>
+      </c>
+      <c r="F18" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-comparison-of-pfas-contributions-to-agricultural-systems-the-water-research-foundation-wrf-opg-26-00190</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="95" customHeight="1">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
+        <is>
           <t>Applications Invited for 8th Call for Proposals Small-Size Grants Global EbA Fund</t>
         </is>
       </c>
-      <c r="C18" s="1" t="inlineStr">
+      <c r="C19" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -1629,34 +1701,167 @@
 Only successful applicants will be contacted; no individual feedback provided to unsuccessful applicants</t>
         </is>
       </c>
-      <c r="D18" s="1" t="inlineStr">
+      <c r="D19" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E18" s="1" t="inlineStr">
+      <c r="E19" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F18" s="1" t="inlineStr">
+      <c r="F19" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-8th-call-for-proposals-small-size-grants-global-eba-fund-global-eba-fund-opg-26-00177</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="95" customHeight="1">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="inlineStr">
+    <row r="20" ht="95" customHeight="1">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Crossing the Divide Best Practices for Addressing Local and Privately-Owned Lateral Sewer Issues RFP 5419</t>
+        </is>
+      </c>
+      <c r="C20" s="1" t="inlineStr">
+        <is>
+          <t>Project Objective:
+To provide water resource recovery facilities (WRRFs) and collection system operators with an interactive manual of practice for implementing inflow and infiltration (I&amp;I) and obstruction management programs, focused on municipal and privately owned lateral sewers in complex legal, regulatory, and multi-jurisdictional environments.
+ Background/Rationale:
+Wastewater utilities face continuing challenges providing cost-effective sewer services amid rising demand, urban redevelopment, and performance disruptors (root intrusion, pipe degradation, blockages). I&amp;I and obstruction management remain persistent, costly problems without a consolidated resource to guide program design. During wet weather, peak I&amp;I flows can increase influent flows 3–5x average. Studies suggest up to 80% of I&amp;I originates on private property, and root intrusions cause over 50% of sewer blockages globally. Program effectiveness varies widely depending on statutory authority, multi-jurisdictional overlap, enforcement mechanisms, and participant willingness.
+ Central Research Questions:
+What I&amp;I and obstruction management practices are utilities using today, and how do they vary by jurisdictional/regulatory/infrastructure/environmental conditions?
+Which factors most influence successful implementation, and what barriers commonly derail programs?
+What measurable benefits (cost avoidance, capacity recovery, reduced spill risk, improved regulatory standing) have utilities realized from successful programs?
+This project extends WRF's ongoing "State-of-Practice Manual for Inflow and Infiltration Detection and Mitigation at Street and Private Lateral Levels" (Project 5365) into I&amp;I source control and obstruction management specifically.
+ Research Approach (4 Tasks):
+Literature and Regulatory Review — Comprehensive review of legal authorities/regulations in the US and comparable international jurisdictions; catalog program elements, enforcement mechanisms, incentive structures, and legal/jurisdictional barriers
+Utility Survey and Case Study Development — Broad survey across utility size/geography/system type; select at least 5 diverse in-depth case studies with quantitative results (I&amp;I reduction %, reduced bypass pumping, reduced basement backups, cost savings, recovered capacity, reduced blockage-related spills/service calls)
+Utility Workshop — At least one invitation-only workshop with utility representatives to present survey findings and gather structured feedback on draft guidance content
+Interactive Manual of Practice — Development of a decision-support tool/web-based application/interactive PDF enabling utilities to select effective I&amp;I/obstruction program elements based on their statutory authority, jurisdictional complexity, and enforcement mechanisms
+ Expected Deliverables:
+Research report (using WRF's Research Report Template) including literature/regulatory review
+Interactive manual of practice (following Technology Deliverables Guidance)
+In-depth utility survey, state-of-the-practice report, and at least 5 standalone case studies with quantitative results
+Summary documentation of the utility workshop, including feedback and how it was incorporated
+ Project Duration: 24 months from contract start date (No-Cost Extension Policy caps extensions at 9 months beyond original schedule)
+ Eligibility to Submit:
+Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible as named participants. Not open to individuals (same institutional-applicant structure as RFP 5424).
+ Budget/Funding:
+Maximum WRF funding: $250,000
+Applicant must contribute at least 33% of the project award as additional resources (cost share, applicant in-kind, or third-party in-kind per 2 CFR Part 200.306)
+Proposals not meeting the 33% minimum match will not be accepted
+ Proposal Evaluation Criteria:
+Understanding the Problem and Responsiveness to RFP: 20 points
+Technical and Scientific Merit: 30 points
+Qualifications, Capabilities, and Management: 20 points
+Communication Plan, Deliverables, and Applicability: 15 points
+Budget and Schedule: 15 points
+ Compliance Standards: OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
+ Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
+        </is>
+      </c>
+      <c r="D20" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E20" s="1" t="inlineStr">
+        <is>
+          <t>Oct 26, 2026</t>
+        </is>
+      </c>
+      <c r="F20" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-crossing-the-divide-best-practices-for-addressing-local-and-privately-owned-lateral-sewer-issues-rfp-5419-the-water-research-foundation-wrf-opg-26-00189</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="95" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Adaptive Control Frameworks to Unlock Full-Scale BNR Potential Water Research Foundation WRF</t>
+        </is>
+      </c>
+      <c r="C21" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+The Water Research Foundation (WRF) is the leading research organization advancing the science of all water to meet the evolving needs of its subscribers and the water sector. WRF is a nonprofit, charitable and educational organization which funds, manages, and publishes research on the technology, operation, and management of drinking water, wastewater, reuse, and stormwater collection, treatment and supply systems—all in pursuit of ensuring water quality and improving water services to the public.
+ Project Objectives:
+Identify and categorize dominant failure modes of current aeration and process control implementations under real-world operating conditions
+Develop guidance on data/instrumentation requirements for utilities to support adaptive control — including characterizing existing sensor infrastructure and use of soft sensors where hard sensors are limited
+Develop practical adaptive control frameworks and implementation guidance deployable without dependence on proprietary black-box tools or specialized data science expertise, including hybrid approaches augmenting conventional controls with AI/ML and digital twins for variable flow/concentration conditions
+Benchmark control performance against biological capacity indicators across multiple full-scale facilities to quantify the gap between achievable and realized Biological Nutrient Removal (BNR) performance
+ Background/Rationale:
+The water sector routinely invests in capital-intensive solutions (additional aeration, supplemental carbon systems, tertiary filtration) to address BNR shortfalls that may actually be control execution problems, not biological potential. Adaptive control strategies (e.g., ammonia-based aeration control, ammonia vs. nitrate control) frequently fail under variable influent loading or temperature swings, causing operators to revert to manual control. This project targets that execution gap using digitalization, AI/ML, and sensors. Geographic focus: United States and Canada.
+ Research Approach (flexible, proposer-defined):
+Failure-Mode Characterization
+Sensor Infrastructure Inventory and Data Quality Assessment
+Soft Sensor Development and Validation
+Adaptive Control Framework Development (hybrid rule-based + AI/ML)
+Operator Adoption and Organizational Readiness
+Multi-Facility Benchmarking
+ Expected Deliverables:
+Comprehensive literature review (including WRF's own research)
+Utility-facing implementation guidance (controller selection, sensor infrastructure, tuning, calibration, operator training, maintenance, system integration) — must include a decision framework and failure-mode catalog
+Multi-facility dataset quantifying capacity-vs-performance gap, with utility case studies across US/Canada
+Outreach (webcasts, conference presentations)
+One open-access peer-reviewed journal paper
+ Project Duration: 24 months from contract start date (No-Cost Extension Policy caps extensions at 9 months beyond original schedule)
+ Eligibility to Submit:
+Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible to be named participants.
+ Budget/Funding:
+Maximum WRF funding: $300,000
+Applicant must contribute additional resources equivalent to at least 33% of the project award (e.g., $100,000 requested → minimum $33,000 additional contribution required, via cost share, applicant in-kind, or third-party in-kind)
+Proposals not meeting the 33% minimum match will not be accepted
+ Proposal Evaluation Criteria:
+Understanding the Problem and Responsiveness to RFP: 20 points
+Technical and Scientific Merit: 30 points
+Qualifications, Capabilities, and Management: 20 points
+Communication Plan, Deliverables, and Applicability: 15 points
+Budget and Schedule: 15 points
+ Compliance Standards: Administrative, cost, and audit standards comply with OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
+Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
+        </is>
+      </c>
+      <c r="D21" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E21" s="1" t="inlineStr">
+        <is>
+          <t>Oct 26, 2026</t>
+        </is>
+      </c>
+      <c r="F21" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-adaptive-control-frameworks-to-unlock-full-scale-bnr-potential-water-research-foundation-wrf-the-water-research-foundation-wrf-opg-26-00187</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="95" customHeight="1">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Whitley Award 2027</t>
         </is>
       </c>
-      <c r="C19" s="1" t="inlineStr">
+      <c r="C22" s="1" t="inlineStr">
         <is>
           <t>About the Grant: 
 An annual grant by the Whitley Fund for Nature (WFN) recognising grassroots conservation leaders in the Global South, providing funding to support and scale up proven, science-based solutions that deliver lasting impact for both people and nature.
@@ -1669,34 +1874,34 @@
 You do not need to be invited or nominated to apply.</t>
         </is>
       </c>
-      <c r="D19" s="1" t="inlineStr">
+      <c r="D22" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E19" s="1" t="inlineStr">
+      <c r="E22" s="1" t="inlineStr">
         <is>
           <t>Oct 30, 2026</t>
         </is>
       </c>
-      <c r="F19" s="1" t="inlineStr">
+      <c r="F22" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-whitley-award-2027-whitley-fund-for-nature-wfn-opg-26-00153</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="95" customHeight="1">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="inlineStr">
+    <row r="23" ht="95" customHeight="1">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIFAR Global Scholars Program 20272029 Cohort</t>
         </is>
       </c>
-      <c r="C20" s="1" t="inlineStr">
+      <c r="C23" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 CIFAR is a Canadian-based globally influential research organization that convenes the world’s most brilliant people across disciplines to advance transformative knowledge and solve humanity’s biggest problems, together. By supporting long-term interdisciplinary collaboration, CIFAR provides researchers with an unparalleled environment of trust, transparency and knowledge sharing. Our time-tested model inspires new directions of inquiry, accelerates discovery and yields breakthroughs across borders and academic disciplines. Through knowledge mobilization, we are catalysts for change in industry, government and society. Through our 15 research programs and the Pan-Canadian AI Strategy, CIFAR convenes close to 400 of the world’s top researchers from 141 institutions in 20 countries. CIFAR is generously supported by the governments of Canada, Alberta and Québec, as well as foundations, individuals, corporations and Canadian and international partner organizations.
@@ -1740,34 +1945,34 @@
  Application Deadline: November 4, 2026, 12:00 PM EST</t>
         </is>
       </c>
-      <c r="D20" s="1" t="inlineStr">
+      <c r="D23" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E20" s="1" t="inlineStr">
+      <c r="E23" s="1" t="inlineStr">
         <is>
           <t>Nov 4, 2026</t>
         </is>
       </c>
-      <c r="F20" s="1" t="inlineStr">
+      <c r="F23" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cifar-global-scholars-program-20272029-cohort-cifar-canadian-institute-for-advanced-research-opg-26-00183</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="95" customHeight="1">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="inlineStr">
+    <row r="24" ht="95" customHeight="1">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for IWRS Teaching Innovation Award</t>
         </is>
       </c>
-      <c r="C21" s="1" t="inlineStr">
+      <c r="C24" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
@@ -1779,34 +1984,34 @@
 Two awards of $2,000 USD are available annually.</t>
         </is>
       </c>
-      <c r="D21" s="1" t="inlineStr">
+      <c r="D24" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E21" s="1" t="inlineStr">
+      <c r="E24" s="1" t="inlineStr">
         <is>
           <t>Nov 15, 2026</t>
         </is>
       </c>
-      <c r="F21" s="1" t="inlineStr">
+      <c r="F24" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="95" customHeight="1">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="inlineStr">
+    <row r="25" ht="95" customHeight="1">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for IWRS Teaching Innovation Award</t>
         </is>
       </c>
-      <c r="C22" s="1" t="inlineStr">
+      <c r="C25" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Insects are one of the most numerous and diverse animal groups on Earth.
@@ -1821,34 +2026,34 @@
 IWRS staff and Advisory Group members are not eligible to apply.</t>
         </is>
       </c>
-      <c r="D22" s="1" t="inlineStr">
+      <c r="D25" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E22" s="1" t="inlineStr">
+      <c r="E25" s="1" t="inlineStr">
         <is>
           <t>Nov 15, 2026</t>
         </is>
       </c>
-      <c r="F22" s="1" t="inlineStr">
+      <c r="F25" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00166</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="95" customHeight="1">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B23" s="1" t="inlineStr">
+    <row r="26" ht="95" customHeight="1">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Medium-Size Grants Call for Proposals Global EbA Fund</t>
         </is>
       </c>
-      <c r="C23" s="1" t="inlineStr">
+      <c r="C26" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -1905,34 +2110,34 @@
 Applications submitted via online portal (link shared on the Medium-Size Grants webpage from Oct 12)</t>
         </is>
       </c>
-      <c r="D23" s="1" t="inlineStr">
+      <c r="D26" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E23" s="1" t="inlineStr">
+      <c r="E26" s="1" t="inlineStr">
         <is>
           <t>Nov 16, 2026</t>
         </is>
       </c>
-      <c r="F23" s="1" t="inlineStr">
+      <c r="F26" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-medium-size-grants-call-for-proposals-global-eba-fund-global-eba-fund-opg-26-00178</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="95" customHeight="1">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B24" s="1" t="inlineStr">
+    <row r="27" ht="95" customHeight="1">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIEIF Grant 2026 Climate Intervention Environmental Impact Fund</t>
         </is>
       </c>
-      <c r="C24" s="1" t="inlineStr">
+      <c r="C27" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Climate Intervention Environmental Impact Fund (CIEIF) is a philanthropic fund focused on supporting responsible climate intervention field tests. It provides grants for activities such as environmental impact assessment (EIA), predictive impact modelling, and engagement with potentially affected stakeholders, including local communities and government agencies.
@@ -1959,34 +2164,34 @@
 Potential for scaling the innovation to a globally relevant level</t>
         </is>
       </c>
-      <c r="D24" s="1" t="inlineStr">
+      <c r="D27" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E24" s="1" t="inlineStr">
+      <c r="E27" s="1" t="inlineStr">
         <is>
           <t>Dec 1, 2026</t>
         </is>
       </c>
-      <c r="F24" s="1" t="inlineStr">
+      <c r="F27" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cieif-grant-2026-climate-intervention-environmental-impact-fund-climate-intervention-environmental-impact-fund-opg-26-00155</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="95" customHeight="1">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B25" s="1" t="inlineStr">
+    <row r="28" ht="95" customHeight="1">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 6th Annual Seeding The Future Global Food System Challenge</t>
         </is>
       </c>
-      <c r="C25" s="1" t="inlineStr">
+      <c r="C28" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are one of the largest and most respected private organisations for development cooperation and humanitarian aid in Germany. As a politically and confessionally independent organisation, our value-oriented actions are always based on ethical principles. Our vision is clear: "Zero Hunger by 2030"
@@ -2018,78 +2223,34 @@
 Individuals with no organizational entity</t>
         </is>
       </c>
-      <c r="D25" s="1" t="inlineStr">
+      <c r="D28" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E25" s="1" t="inlineStr">
+      <c r="E28" s="1" t="inlineStr">
         <is>
           <t>Jan 1, 2027</t>
         </is>
       </c>
-      <c r="F25" s="1" t="inlineStr">
+      <c r="F28" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-6th-annual-seeding-the-future-global-food-system-challenge-welthungerhilfe-opg-26-00180</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="95" customHeight="1">
-      <c r="A26" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B26" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Microbiota &amp; Women's Health International Call for Projects</t>
-        </is>
-      </c>
-      <c r="C26" s="1" t="inlineStr">
-        <is>
-          <t>About the Grant
-An annual international research grant by the Biocodex Microbiota Foundation (BMF), rewarding research proposals on the microbiota and its implications in Women's Health and Disease. This year's theme: "Unraveling male-female genital microbiome interactions: mechanisms, transmission, and impact on vaginal dysbiosis."
- Theme/Scope
-Proposals could include, but are not limited to, mechanistic studies elucidating how the penile microbiome contributes to the establishment, persistence, and recurrence of vaginal dysbiosis, including bacterial vaginosis. Areas of interest include microbial transmission dynamics during sexual activity, niche adaptation and persistence of BV-associated taxa in the penile environment, and the functional consequences of these interactions for vaginal community stability.
-Studies evaluating how current and emerging interventions (antibiotics, topical or systemic partner therapies, circumcision, or live biotherapeutic products) alter penile microbial ecology and influence treatment response and recurrence risk in female partners are also encouraged.
- Purpose: From 2025, the Biocodex Microbiota Foundation rewards international research proposals involving the microbiota and its implication in Women's Health and Disease. Every year, the call for proposals covers a specific theme chosen by an International Scientific Committee. Either clinical or fundamental research proposals can be submitted. Maximum project duration: 3 years.
- Eligibility
-Open to MDs, PhDs, or Pharm-Ds working in the subject area (gynecology, obstetrics, microbiology, infectious diseases, internal medicine, oncology, etc.).
-No geographic restrictions — all countries are eligible.
-A principal investigator who received a Women's Health International grant from BMF cannot reapply for this award for three years. However, winners of another BMF grant category can apply for this grant.
-Members of the Women's Health International Scientific Committee and their laboratory members are not allowed to apply as Principal Investigators.
- Grant Amount
-€200,000 annually — awarded to researchers within universities, hospitals, or other research settings to finance equipment, operations, or staffing costs. Grants are NOT awarded to individuals directly (must be institutionally affiliated). Institution's overhead costs capped at 10%.</t>
-        </is>
-      </c>
-      <c r="D26" s="1" t="inlineStr">
-        <is>
-          <t>Safety</t>
-        </is>
-      </c>
-      <c r="E26" s="1" t="inlineStr">
-        <is>
-          <t>Jan 15, 2027</t>
-        </is>
-      </c>
-      <c r="F26" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-microbiota-and-womens-health-international-call-for-projects-biocodex-microbiota-foundation-bmf-opg-26-00152</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="95" customHeight="1">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B27" s="1" t="inlineStr">
+    <row r="29" ht="95" customHeight="1">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for BES Training and Travel Grants</t>
         </is>
       </c>
-      <c r="C27" s="1" t="inlineStr">
+      <c r="C29" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are a global community of scientists shining a spotlight on the intricacy and value of our natural world, providing the evidence for better decisions. Our vision is for people and nature to thrive in a world that values ecology.
@@ -2128,17 +2289,17 @@
  Application Deadline (Round 2): Opens 30 April 2026, closes 17 May 2026</t>
         </is>
       </c>
-      <c r="D27" s="1" t="inlineStr">
+      <c r="D29" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E27" s="1" t="inlineStr">
+      <c r="E29" s="1" t="inlineStr">
         <is>
           <t>May 17, 2027</t>
         </is>
       </c>
-      <c r="F27" s="1" t="inlineStr">
+      <c r="F29" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-bes-training-and-travel-grants-british-ecological-society-opg-26-00181</t>
         </is>

</xml_diff>

<commit_message>
Auto update Combined.xlsx [Thu Sep 17 07:04:17 UTC 2026]
</commit_message>
<xml_diff>
--- a/output/Combined.xlsx
+++ b/output/Combined.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -467,72 +467,10 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>ToR for Consultancy Service - Practitioner Knowledge Mapping Across Priority Livelihood Value Chains</t>
+          <t>ToR - Behavioural Insights and Narrative Inquiry for the Climate Responsive Livelihood Programme Meghalaya</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
-        <is>
-          <t>Terms of Reference (TOR) for Consultancy Services
-Title Practitioner Knowledge Mapping Across Priority Livelihood Value Chains
-Timeline The assignment will be completed over a period of four (4) months. (September- January)
-Expected    area of expertise
- A curated digital repository comprising at least 50 high-quality knowledge resources per value chain, including technical reports, research publications, manuals, market studies, case studies and other relevant reference materials. Each resource should be accompanied by a brief annotation summarising its relevance and key insights.
-Apply Link https://forms.gle/AyXwybmyU523W7TBA
-Last    Date           for Apply 18th September 2026
-About SELCO Foundation:
-SELCO Foundation’s mission is to create a platform of solutions that uses sustainable energy as a catalyst to bridge environmental sustainability and poverty alleviation. With holistic development as the primary focus, the organization strives to create equitable societies, where services are accessed by all communities. The interventions of SELCO lead to a sustainable delivery model of essential services like livelihoods, education, and health till the last mile. (Read more about SELCO here: http://www.selcofoundation.org/)
- About the Programmes:
-The Climate Responsive Livelihood (CRL) Programme seeks to strengthen sustainable livelihoods by enabling climate resilience, entrepreneurship and local economic development through an integrated ecosystem approach. Recognising that resilient livelihoods are shaped not only by access to technology and finance, but also by institutions, market linkages, technical knowledge and local capacities, the programme aims to build an enabling ecosystem that supports communities in pursuing viable and diversified livelihood opportunities.
- Across India, numerous models of entrepreneurship, value addition, producer institutions, market engagement and enterprise development have emerged across different livelihood value chains. These experiences are often dispersed across geographies, organisations and practitioners, with valuable technical knowledge, implementation insights and business models remaining fragmented and difficult to access.
- This assignment seeks to systematically identify, document and synthesise these experiences across six priority value chains (specifically- paddy, pineapple, bamboo, turmeric, piggery and mushroom) to create a structured knowledge base that can inform programme design, enterprise incubation, capacity building and ecosystem strengthening under the Climate Responsive Livelihood Programme. The exercise will combine extensive secondary research with interviews of practitioners, entrepreneurs and technical experts from across the country to curate actionable knowledge that is relevant for adaptation within Meghalaya contexts.
- Objective:
-To develop a comprehensive evidence base on entrepreneurship opportunities, technical practices, business models and ecosystem enablers across six priority value chains by combining primary interviews with extensive secondary research.
-The assignment should identify approaches that demonstrate potential relevance to the context while also documenting the enabling conditions, risks and institutional requirements necessary for replication or adaptation.
- Scope of Work
-Secondary Research and Landscape Review
-Undertake an extensive review of literature and existing knowledge related to each value chain, including:
-Technical reports
-Research publications
-Government reports
-Market assessments
-Enterprise case studies
-Business models
-NGO and development programme documentation
-Value chain assessments
-Training manuals and technical guides
-Relevant policy and institutional documents
-The review should not be limited to Meghalaya and should draw from relevant experiences across India.
-The agency is expected to independently identify and curate knowledge resources beyond those shared by the programme team</t>
-        </is>
-      </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>Sep 18, 2026</t>
-        </is>
-      </c>
-      <c r="F2" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/tor-for-consultancy-service-practitioner-knowledge-mapping-across-priority-livelihood-value-chains-selco-foundation-rfp-26-00350</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="95" customHeight="1">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>ToR - Behavioural Insights and Narrative Inquiry for the Climate Responsive Livelihood Programme Meghalaya</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Title  Behavioural Insights and Narrative Inquiry for the Climate Responsive Livelihood Programme, Meghalaya
 Timeline  2 months
@@ -550,34 +488,34 @@
 Rather than evaluating awareness or testing communication materials, the assignment should seek to uncover deeper behavioural and social drivers that influence livelihood choices and participation. The findings will inform a narrative architecture and mobilisation approach that resonates authentically with communities across the state.</t>
         </is>
       </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>Sep 19, 2026</t>
         </is>
       </c>
-      <c r="F3" s="1" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-behavioural-insights-and-narrative-inquiry-for-the-climate-responsive-livelihood-programme-meghalaya-selco-foundation-rfp-26-00355</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="95" customHeight="1">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
+    <row r="3" ht="95" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>Expression of Interest EOI for Trade &amp; Livelihood Partners</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Expression of Interest (EOI) for Trade &amp; Livelihood Partners
 Issued By: BharatCares
@@ -704,34 +642,34 @@
 Any prior work with tribal or rural communities, with references if available</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Sep 20, 2026</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/expression-of-interest-eoi-for-trade-and-livelihood-partners-bharatcares-rfp-26-00340</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="95" customHeight="1">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
+    <row r="4" ht="95" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>RFP - Research Collaboration For Improved Application and Processing Techniques For Natural Dyes</t>
         </is>
       </c>
-      <c r="C5" s="1" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>REǪUEST FOR PROPOSALS (RFP)
 Research Collaboration For Improved Application and Processing Techniques For Natural Dyes
@@ -784,34 +722,34 @@
 Network with dyeing units and textile industry associations</t>
         </is>
       </c>
-      <c r="D5" s="1" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>Climate</t>
         </is>
       </c>
-      <c r="E5" s="1" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>Sep 20, 2026</t>
         </is>
       </c>
-      <c r="F5" s="1" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfp-research-collaboration-for-improved-application-and-processing-techniques-for-natural-dyes-chitrika-rfp-26-00343</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="95" customHeight="1">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
+    <row r="5" ht="95" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>RFP - Agronomic Research Study For Natural Dye Crop Development</t>
         </is>
       </c>
-      <c r="C6" s="1" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>REǪUEST FOR PROPOSALS (RFP)
 Agronomic Research Study For Natural Dye Crop Development
@@ -870,34 +808,34 @@
 Experience working on natural dye</t>
         </is>
       </c>
-      <c r="D6" s="1" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E6" s="1" t="inlineStr">
+      <c r="E5" s="1" t="inlineStr">
         <is>
           <t>Sep 20, 2026</t>
         </is>
       </c>
-      <c r="F6" s="1" t="inlineStr">
+      <c r="F5" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfp-agronomic-research-study-for-natural-dye-crop-development-chitrika-rfp-26-00344</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="95" customHeight="1">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
+    <row r="6" ht="95" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>RFPs Invited for Using an Agent Based Model to Predict the Impact of City-Level Policies on the Adoption of Distributed Renewable Energy</t>
         </is>
       </c>
-      <c r="C7" s="1" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>About C40:
 C40 is a network of nearly 100 mayors of the world's leading cities working to deliver urgent climate action and create a future where everyone, everywhere, can thrive. Mayors of C40 cities are committed to using a science-based, people-focused approach to limit global heating in line with the Paris Agreement, working alongside labour, business, youth climate movement, and civil society representatives to help halve emissions by 2030.
@@ -940,34 +878,34 @@
 Project runs until: June 30, 2027</t>
         </is>
       </c>
-      <c r="D7" s="1" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E7" s="1" t="inlineStr">
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>Sep 20, 2026</t>
         </is>
       </c>
-      <c r="F7" s="1" t="inlineStr">
+      <c r="F6" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfps-invited-for-using-an-agent-based-model-to-predict-the-impact-of-city-level-policies-on-the-adoption-of-distributed-renewable-energy-c40-cities-rfp-26-00357</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="95" customHeight="1">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
+    <row r="7" ht="95" customHeight="1">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>E-Tender Request for Digital Communication Website Development and Social Media Campaign for Colors of Nature</t>
         </is>
       </c>
-      <c r="C8" s="1" t="inlineStr">
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>REǪUEST FOR PROPOSALS (RFP)
 Digital Communication, Website Development and Social Media Campaign
@@ -1013,34 +951,34 @@
 Ready to develop a women led and based digital marketing team</t>
         </is>
       </c>
-      <c r="D8" s="1" t="inlineStr">
+      <c r="D7" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E8" s="1" t="inlineStr">
+      <c r="E7" s="1" t="inlineStr">
         <is>
           <t>Sep 20, 2026</t>
         </is>
       </c>
-      <c r="F8" s="1" t="inlineStr">
+      <c r="F7" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/e-tender-request-for-digital-communication-website-development-and-social-media-campaign-for-colors-of-nature-chitrika-rfp-26-00342</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="95" customHeight="1">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="inlineStr">
+    <row r="8" ht="95" customHeight="1">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Wellbeing Research Grants Funding Better Evaluations of AI's Impact on Wellbeing</t>
         </is>
       </c>
-      <c r="C9" s="1" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We're an AI research company that builds reliable, interpretable, and steerable AI systems. Our first product is Claude, an AI assistant for tasks at any scale. Our research interests span multiple areas including natural language, human feedback, scaling laws, reinforcement learning, code generation, and interpretability. 
@@ -1059,34 +997,34 @@
  Funding Amount: Total program pool of $5 million (individual grant sizes not specified on the page)</t>
         </is>
       </c>
-      <c r="D9" s="1" t="inlineStr">
+      <c r="D8" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E9" s="1" t="inlineStr">
+      <c r="E8" s="1" t="inlineStr">
         <is>
           <t>Sep 21, 2026</t>
         </is>
       </c>
-      <c r="F9" s="1" t="inlineStr">
+      <c r="F8" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-wellbeing-research-grants-funding-better-evaluations-of-ais-impact-on-wellbeing-anthropic-opg-26-00175</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="95" customHeight="1">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
+    <row r="9" ht="95" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for GEF SGP CSO Challenge Program</t>
         </is>
       </c>
-      <c r="C10" s="1" t="inlineStr">
+      <c r="C9" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global Environment Facility Small Grants Programme (SGP) is a global initiative implemented by the United Nations Development Programme (UNDP) on behalf of the Global Environment Facility (GEF). Since its launch in 1992, SGP has empowered communities worldwide to take action on environmental challenges while improving livelihoods. As a GEF Corporate Programme, SGP provides direct support to civil society organisations and community-based organisations to design and implement innovative, locally driven solutions. The programme places strong emphasis on inclusion, ensuring meaningful participation of Indigenous Peoples, youth, women and girls, and other underrepresented groups.
@@ -1135,34 +1073,34 @@
 Risk management and mitigation</t>
         </is>
       </c>
-      <c r="D10" s="1" t="inlineStr">
+      <c r="D9" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E10" s="1" t="inlineStr">
+      <c r="E9" s="1" t="inlineStr">
         <is>
           <t>Sep 23, 2026</t>
         </is>
       </c>
-      <c r="F10" s="1" t="inlineStr">
+      <c r="F9" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-gef-sgp-cso-challenge-program-gef-small-grants-programme-sgp-opg-26-00184</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="95" customHeight="1">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="inlineStr">
+    <row r="10" ht="95" customHeight="1">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
         <is>
           <t>RFP for Impact Assessment</t>
         </is>
       </c>
-      <c r="C11" s="1" t="inlineStr">
+      <c r="C10" s="1" t="inlineStr">
         <is>
           <t>Introduction
 Titan Company Limited, a member of the Tata Group, has a long-standing commitment to Corporate Social Responsibility (CSR) in India. The company's CSR initiatives derive its philosophy from the Company’s vision statement: “We create elevating experiences for the people we touch and significantly impact the world we work in”. The initiatives are designed to promote inclusive growth, empower communities, and contribute to the country's socio-economic development. The program includes Titan’s CSR policy is governed by a dedicated CSR Committee that ensures transparency and compliance with regulatory requirements. The program includes Girl Child Education, Skill and Entrepreneurship Development, supporting Indian Heritage Arts and Crafts, Integrated Village Development Programme, Eye Care and Affirmative Action. Titan's CSR policy is governed by a dedicated CSR Committee that ensures transparency and compliance with regulatory requirements.
@@ -1196,34 +1134,34 @@
 Timeline: Proposal submission deadline: September 24, 2026</t>
         </is>
       </c>
-      <c r="D11" s="1" t="inlineStr">
+      <c r="D10" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E11" s="1" t="inlineStr">
+      <c r="E10" s="1" t="inlineStr">
         <is>
           <t>Sep 24, 2026</t>
         </is>
       </c>
-      <c r="F11" s="1" t="inlineStr">
+      <c r="F10" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfp-for-impact-assessment-titan-rfp-26-00354</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="95" customHeight="1">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="inlineStr">
+    <row r="11" ht="95" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>EOI Inviting Expression of Interest-cum-Proposal for Setting Up District De-Addiction Centres under NAPDDR</t>
         </is>
       </c>
-      <c r="C12" s="1" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>About us
 In the year 1985-86, the erstwhile Ministry of Welfare was bifurcated into the Department of Women and Child Development and the Department of Welfare. Simultaneously, the Scheduled Castes Development Division, Tribal Development Division and the Minorities and Backward Classes Welfare Division were moved from the Ministry of Home Affairs and also the Wakf Division from the Ministry of Law to form the then Ministry of Welfare Subsequently, the name of the Ministry was changed to the Ministry of Social Justice &amp; Empowerment in May, 1998. Further, in October, 1999, the Tribal Development Division had moved out to form a separate Ministry of Tribal Affairs. In January, 2007, the Minorities Division along with Wakf Unit have been moved out of the Ministry and formed as a separate Ministry and the Child Development Division has gone to the Ministry of Women &amp; Child Development.
@@ -1263,6 +1201,58 @@
 11. Department of Social Justice and Empowerment (DoSJE) reserves the right to cancel this notice, andior invite afresh proposals with or without amendments to this document without liability or any obligation for such document, and without assigning any reason. DoSJE reserves the right to take final decision regarding selection of implementing agency or project.</t>
         </is>
       </c>
+      <c r="D11" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>Sep 30, 2026</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/eoi-inviting-expression-of-interest-cum-proposal-for-setting-up-district-de-addiction-centres-under-napddr-ministry-of-social-justice-and-empowerment-goi-rfp-26-00356</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="95" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Signals of Change Shaping the Future of Sexual and Reproductive Health and Rights SRHR</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+The World Health Organization's mission: to promote health, keep the world safe, and serve the vulnerable. Working through offices in more than 150 countries, WHO staff work side by side with governments and other partners to ensure the highest attainable level of health for all people.
+ About the Opportunity
+HRP and its UN co-sponsors are leading a global Sexual and Reproductive Health and Rights (SRHR) foresight and research prioritization process for 2026–2036. This open public consultation invites diverse stakeholder input to identify "signals of change" — emerging trends, shifts, or disruptions — that could shape the future of SRHR over the next decade. The process uses foresight methodology (not prediction) to explore plausible futures and will culminate in a published report and research agenda in 2027.
+ Guiding Questions
+What future trends will shape or constrain SRHR over the next 10 years?
+What evidence and research investments are needed today to prepare SRHR for the futures we may face?
+ Scope of Submissions 
+Economic systems; social infrastructure; structural discrimination; conflict/forced migration/displacement; mega-trends (demographic shifts, climate change, digital transformation/AI, urbanization); conditions of daily life; rights/legal/governance systems; health systems; media/misinformation; and changes in the research ecosystem.
+ Who Can Participate 
+Open to individuals and organizations globally, including:
+Health workers, professional associations, clinical networks
+Civil society, community groups, youth-led organizations, rights movements
+Governments, parliamentarians, regulators, public sector bodies
+Researchers, academia, think tanks, technical experts
+UN agencies, multilateral/humanitarian/development organizations
+Funders, philanthropy, private sector, tech/innovation organizations
+Media, communications, journalism
+Anyone with relevant lived experience or perspective
+Special interest in submissions from health worker, community, youth, and rights-movement spaces not typically represented in published forums.
+ Submission Requirements: Descriptive information (name, contact email, country, sector) required alongside each submission; formal published evidence is helpful but not required — practice-based experience and field examples are also welcome. Submissions are kept confidential and anonymized before analysis.</t>
+        </is>
+      </c>
       <c r="D12" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
@@ -1275,7 +1265,7 @@
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/rfps/eoi-inviting-expression-of-interest-cum-proposal-for-setting-up-district-de-addiction-centres-under-napddr-ministry-of-social-justice-and-empowerment-goi-rfp-26-00356</t>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-signals-of-change-shaping-the-future-of-sexual-and-reproductive-health-and-rights-srhr-world-health-organization-opg-26-00176</t>
         </is>
       </c>
     </row>
@@ -1287,10 +1277,74 @@
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
+          <t>Applications Invited for Setting up Viral Research and Diagnosis Laboratories VRDL in Medical Colleges/Hospitals/Medical Institutions</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+The President notified the creation of the Department of Health Research under the Ministry of Health &amp; Family Welfare through an amendment to the Government of India (Allocation of Business) Rules, 1961 on the 17th September 2007. The Department of Health Research was formally launched on 5th October 2007 by the Minister for Science &amp; Technology and Earth Sciences in a function presided over by the Minister for Health &amp; Family Welfare, in the presence, inter-alia, of the Minister of State for Health &amp; Family Welfare.
+The Department became functional from November 2008 with the appointment of first Secretary of the Department The aim of the DHR is to bring modern health technologies to the people through research and innovations related to diagnosis, treatment methods and vaccines for prevention, to translate them into products and processes and, in synergy with concerned organizations, introduce these innovations into public health system.
+ About the Opportunity:
+Under DHR's scheme "Setting-up of nation-wide network of laboratories for managing epidemics and national calamities," proposals are invited from Medical Colleges/Hospitals/Research Institutions to establish a Medical College &amp; Research Institute Level – Viral Research and Diagnosis Laboratory (MCL-VRDL). The existing network comprises 167 VRDLs (11 Regional, 27 State, 129 Medical College level) across 27 states and 5 UTs, aimed at early detection of infectious pathogens, outbreak surveillance, and research on emerging/re-emerging viral diseases.
+ Objectives:
+Establish capacity for early detection of common and high-risk infectious pathogens
+Strengthen syndromic surveillance ecosystem for outbreak detection
+Undertake R&amp;D on emerging, re-emerging and novel viruses
+ Eligibility (Institution-level):
+State Government Medical Colleges
+Central Government Medical Colleges and Research Institutes
+Armed Forces Medical Institutions/Hospitals
+Railway and other Central Government health institutions
+Private medical colleges ranked in top 50 NIRF ranking
+Must have a dedicated Microbiology department with qualified faculty
+Must have &gt;200 sq.m. area available in existing building (preferably within Microbiology Dept.)
+ Funding Provision:
+Non-recurring assistance: Rs. 1.55 crore total
+Rs. 66.8 lakhs — Civil Work (infrastructure modification)
+Rs. 88.2 lakhs — Equipment (complete lab setup)
+No recurring expenditure (staff salaries, consumables, contingency) is provided — to be borne by the host institution
+ Role &amp; Responsibilities of the Lab:
+Conduct routine diagnosis of infectious pathogens
+Participate in syndromic and event-based surveillance
+Provide support during outbreaks/epidemics
+Share data with ICMR
+ Selection Criteria:
+Meeting eligibility does not guarantee selection; merit-based evaluation by a technical committee
+Preference to institutions in geographically underserved regions
+Weightage for technical strength (qualified faculty, biosafety practices, outbreak investigation experience, publications, patents, externally funded projects)
+Additional weightage for molecular diagnostics, genomic surveillance, One Health research capability, and commitment to long-term recurring support
+Private medical colleges: only top-50 NIRF-ranked institutions considered</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>Sep 30, 2026</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-setting-up-viral-research-and-diagnosis-laboratories-vrdl-in-medical-collegeshospitalsmedical-institutions-department-of-health-research-dhr-ministry-of-health-and-family-welfare-government-of-india-opg-26-00174</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="95" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
           <t>Application Invited for Giving Joy Microgrant</t>
         </is>
       </c>
-      <c r="C13" s="1" t="inlineStr">
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Giving Joy is a US-based nonprofit that strengthens and inspires women’s entrepreneurship worldwide. Through its micro-grants and mentorship program, Giving Joy helps women establish or improve their businesses and initiatives—for their benefit and the benefit of their communities. To date, Giving Joy has awarded over 88 grants to women-led initiatives in 26 countries.
@@ -1329,71 +1383,19 @@
 The grant period is six months.</t>
         </is>
       </c>
-      <c r="D13" s="1" t="inlineStr">
+      <c r="D14" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E13" s="1" t="inlineStr">
+      <c r="E14" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F13" s="1" t="inlineStr">
+      <c r="F14" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/application-invited-for-giving-joy-microgrant-giving-joy-opg-26-00185</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="95" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Signals of Change Shaping the Future of Sexual and Reproductive Health and Rights SRHR</t>
-        </is>
-      </c>
-      <c r="C14" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-The World Health Organization's mission: to promote health, keep the world safe, and serve the vulnerable. Working through offices in more than 150 countries, WHO staff work side by side with governments and other partners to ensure the highest attainable level of health for all people.
- About the Opportunity
-HRP and its UN co-sponsors are leading a global Sexual and Reproductive Health and Rights (SRHR) foresight and research prioritization process for 2026–2036. This open public consultation invites diverse stakeholder input to identify "signals of change" — emerging trends, shifts, or disruptions — that could shape the future of SRHR over the next decade. The process uses foresight methodology (not prediction) to explore plausible futures and will culminate in a published report and research agenda in 2027.
- Guiding Questions
-What future trends will shape or constrain SRHR over the next 10 years?
-What evidence and research investments are needed today to prepare SRHR for the futures we may face?
- Scope of Submissions 
-Economic systems; social infrastructure; structural discrimination; conflict/forced migration/displacement; mega-trends (demographic shifts, climate change, digital transformation/AI, urbanization); conditions of daily life; rights/legal/governance systems; health systems; media/misinformation; and changes in the research ecosystem.
- Who Can Participate 
-Open to individuals and organizations globally, including:
-Health workers, professional associations, clinical networks
-Civil society, community groups, youth-led organizations, rights movements
-Governments, parliamentarians, regulators, public sector bodies
-Researchers, academia, think tanks, technical experts
-UN agencies, multilateral/humanitarian/development organizations
-Funders, philanthropy, private sector, tech/innovation organizations
-Media, communications, journalism
-Anyone with relevant lived experience or perspective
-Special interest in submissions from health worker, community, youth, and rights-movement spaces not typically represented in published forums.
- Submission Requirements: Descriptive information (name, contact email, country, sector) required alongside each submission; formal published evidence is helpful but not required — practice-based experience and field examples are also welcome. Submissions are kept confidential and anonymized before analysis.</t>
-        </is>
-      </c>
-      <c r="D14" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E14" s="1" t="inlineStr">
-        <is>
-          <t>Sep 30, 2026</t>
-        </is>
-      </c>
-      <c r="F14" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-signals-of-change-shaping-the-future-of-sexual-and-reproductive-health-and-rights-srhr-world-health-organization-opg-26-00176</t>
         </is>
       </c>
     </row>
@@ -1405,74 +1407,10 @@
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
-          <t>Applications Invited for Setting up Viral Research and Diagnosis Laboratories VRDL in Medical Colleges/Hospitals/Medical Institutions</t>
+          <t>Applications Open Draper Richards Kaplan Foundation Funding for Social Enterprises</t>
         </is>
       </c>
       <c r="C15" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-The President notified the creation of the Department of Health Research under the Ministry of Health &amp; Family Welfare through an amendment to the Government of India (Allocation of Business) Rules, 1961 on the 17th September 2007. The Department of Health Research was formally launched on 5th October 2007 by the Minister for Science &amp; Technology and Earth Sciences in a function presided over by the Minister for Health &amp; Family Welfare, in the presence, inter-alia, of the Minister of State for Health &amp; Family Welfare.
-The Department became functional from November 2008 with the appointment of first Secretary of the Department The aim of the DHR is to bring modern health technologies to the people through research and innovations related to diagnosis, treatment methods and vaccines for prevention, to translate them into products and processes and, in synergy with concerned organizations, introduce these innovations into public health system.
- About the Opportunity:
-Under DHR's scheme "Setting-up of nation-wide network of laboratories for managing epidemics and national calamities," proposals are invited from Medical Colleges/Hospitals/Research Institutions to establish a Medical College &amp; Research Institute Level – Viral Research and Diagnosis Laboratory (MCL-VRDL). The existing network comprises 167 VRDLs (11 Regional, 27 State, 129 Medical College level) across 27 states and 5 UTs, aimed at early detection of infectious pathogens, outbreak surveillance, and research on emerging/re-emerging viral diseases.
- Objectives:
-Establish capacity for early detection of common and high-risk infectious pathogens
-Strengthen syndromic surveillance ecosystem for outbreak detection
-Undertake R&amp;D on emerging, re-emerging and novel viruses
- Eligibility (Institution-level):
-State Government Medical Colleges
-Central Government Medical Colleges and Research Institutes
-Armed Forces Medical Institutions/Hospitals
-Railway and other Central Government health institutions
-Private medical colleges ranked in top 50 NIRF ranking
-Must have a dedicated Microbiology department with qualified faculty
-Must have &gt;200 sq.m. area available in existing building (preferably within Microbiology Dept.)
- Funding Provision:
-Non-recurring assistance: Rs. 1.55 crore total
-Rs. 66.8 lakhs — Civil Work (infrastructure modification)
-Rs. 88.2 lakhs — Equipment (complete lab setup)
-No recurring expenditure (staff salaries, consumables, contingency) is provided — to be borne by the host institution
- Role &amp; Responsibilities of the Lab:
-Conduct routine diagnosis of infectious pathogens
-Participate in syndromic and event-based surveillance
-Provide support during outbreaks/epidemics
-Share data with ICMR
- Selection Criteria:
-Meeting eligibility does not guarantee selection; merit-based evaluation by a technical committee
-Preference to institutions in geographically underserved regions
-Weightage for technical strength (qualified faculty, biosafety practices, outbreak investigation experience, publications, patents, externally funded projects)
-Additional weightage for molecular diagnostics, genomic surveillance, One Health research capability, and commitment to long-term recurring support
-Private medical colleges: only top-50 NIRF-ranked institutions considered</t>
-        </is>
-      </c>
-      <c r="D15" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E15" s="1" t="inlineStr">
-        <is>
-          <t>Sep 30, 2026</t>
-        </is>
-      </c>
-      <c r="F15" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-setting-up-viral-research-and-diagnosis-laboratories-vrdl-in-medical-collegeshospitalsmedical-institutions-department-of-health-research-dhr-ministry-of-health-and-family-welfare-government-of-india-opg-26-00174</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="95" customHeight="1">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B16" s="1" t="inlineStr">
-        <is>
-          <t>Applications Open Draper Richards Kaplan Foundation Funding for Social Enterprises</t>
-        </is>
-      </c>
-      <c r="C16" s="1" t="inlineStr">
         <is>
           <t>About us
 Started in 2002, Draper Richards Kaplan Foundation (DRK) is a global venture philanthropy firm supporting early stage, high impact social enterprises. Borrowed from our venture capital legacy, DRK finds, funds, and supports exceptional leaders building innovative solutions to some of the world’s most challenging social and environmental problems. Since beginning this work nearly 25 years ago, DRK has invested in more than 270 organizations that have collectively impacted over 610 million lives to date.
@@ -1496,34 +1434,34 @@
 Please attach a standard resume/CV for the entrepreneur(s) and/or key leadership team members (e.g., CEO, COO, ED, etc.). Applications with text bios for entrepreneurs or members of the leadership team will not be considered.</t>
         </is>
       </c>
-      <c r="D16" s="1" t="inlineStr">
+      <c r="D15" s="1" t="inlineStr">
         <is>
           <t>Climate</t>
         </is>
       </c>
-      <c r="E16" s="1" t="inlineStr">
+      <c r="E15" s="1" t="inlineStr">
         <is>
           <t>Oct 10, 2026</t>
         </is>
       </c>
-      <c r="F16" s="1" t="inlineStr">
+      <c r="F15" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-open-draper-richards-kaplan-foundation-funding-for-social-enterprises-draper-richards-kaplan-foundation-opg-26-00188</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="95" customHeight="1">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B17" s="1" t="inlineStr">
+    <row r="16" ht="95" customHeight="1">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund</t>
         </is>
       </c>
-      <c r="C17" s="1" t="inlineStr">
+      <c r="C16" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund
 Apply by: 13 October, 2026
@@ -1548,6 +1486,98 @@
  Projects should include opportunities for ServiceNow employees to volunteer in the project activation or implementation.</t>
         </is>
       </c>
+      <c r="D16" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E16" s="1" t="inlineStr">
+        <is>
+          <t>Oct 13, 2026</t>
+        </is>
+      </c>
+      <c r="F16" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/apply-for-the-servicenow-community-solar-fund-changex-opg-26-00186</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="95" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>ToR - Engagement of Consultant/Vendor Individual towards implementation of Literacy Program in Telangana State</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>ANNEX A – TERMS OF REFERENCE (ToR) 
+ Engagement of Consultant/Vendor (Individual) towards implementation of Literacy Program in Telangana State.
+ About Room to Read
+Room to Read India was established in 2003 and presently has programs in twelve states – Bihar, Chhattisgarh, Delhi, Himachal Pradesh, Jharkhand, Karnataka, Madhya Pradesh, Maharashtra, Rajasthan, Telangana, Uttarakhand, and Uttar Pradesh. Room to Read is  an organization transforming the lives of millions of children by focusing on literacy and gender equality in education. 
+ About the Program
+The Literacy Program focuses on strengthening early grade reading skills among primary school children through a comprehensive approach that includes:
+High‑quality reading materials and classroom/school libraries.
+Teacher professional development on early grade reading instruction.
+Academic mentoring, classroom observation, and supportive supervision.
+Use of reading assessments for tracking fluency and comprehension.
+System‑level technical support for government FLN implementation.
+ In Telangana, the program supports the state’s FL agenda by demonstrating effective literacy practices that can be adopted, institutionalized, and scaled within the government system.
+ Background of the Assignment
+Room to Read intends to engage a consultant – Literacy Program (Deliver Demonstration) to support hands‑on delivery, quality assurance, and field‑level demonstration of the Literacy Program in Telangana.
+This is a time‑bound consulting assignment designed to strengthen on‑ground implementation and showcase effective practices, while working closely with the State Literacy Team, Program Operations, and government counterparts.
+ Role of RtR:
+Provide the consultant with necessary data, documents, and technical inputs to support completion of assignment
+ Key Deliverables/Scope of Work/Timelines.
+Deliverable
+Timeline
+Support implementation of Literacy Program interventions in assigned mandals/districts
+Daily.
+Conduct field visits (schools, complexes, mandals, districts) with observation, feedback and mentoring
+10 to 12 visits in a month
+Demonstrate effective literacy classroom practices
+Daily
+Support planning and delivery of teacher trainings and refresher trainings
+Monthly
+Provide academic mentoring and technical support to field teams and government officials
+Daily
+Coordinate with state, district and mandal officials for program implementation and reviews
+Monthly
+Participate and support state/district review meetings and consultations
+Monthly / Quarterly
+Track program implementation and review assessment data
+Weekly requirements
+Identify quality gaps and provide actionable recommendations
+Monthly
+Submit monthly programmatic progress reports
+Monthly
+Prepare field visit observation notes with feedback
+Weekly
+Support documentation for government engagement (presentations, notes, reports).
+Monthly
+Document best practices, case studies, and field learnings.
+Quarterly
+Provide inputs on sustainability and institutionalisation of literacy practices.
+Quarterly
+Submit end-of-assignment learning and recommendation report.
+End of assignment - Yearly
+ Eligibility Criteria: - The vendor
+Master’s degree in education, Social Sciences, or a related field (bachelor’s degree with extensive relevant experience may be considered).
+Minimum 5–8 years of experience in education program implementation, preferably in literacy or FLN initiatives.
+Experience working with government education systems at state and district levels.
+Strong expertise in teacher professional development, academic mentoring, and field‑level implementation.
+Strong communication skills in English and Telugu.
+Ability to travel extensively to program locations.
+ Contract Duration:
+The duration of the assignment will be 6 months.
+Payment will be made monthly on submission of the invoice and upon delivery as per the schedule, with adjustments for any short fall in delivery, including deviations  affecting timely completion of agreed deliverables.
+Approved travel and accommodation expenses incurred for assignment-related activities shall be reimbursed by Room to Read in accordance with the consultancy reimbursement guidelines.</t>
+        </is>
+      </c>
       <c r="D17" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
@@ -1555,12 +1585,12 @@
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>Oct 13, 2026</t>
+          <t>Oct 16, 2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/grants/apply-for-the-servicenow-community-solar-fund-changex-opg-26-00186</t>
+          <t>https://onepurpos.in/openings/rfps/tor-engagement-of-consultantvendor-individual-towards-implementation-of-literacy-program-in-telangana-state-room-to-read-india-rfp-26-00360</t>
         </is>
       </c>
     </row>
@@ -1572,33 +1602,90 @@
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>Applications Invited for Comparison of PFAS Contributions to Agricultural Systems</t>
+          <t>RFPs Invited for Consultant to Develop a Technical Assistance Package for National Application of the Digital Health and AI Investment Classification Framework</t>
         </is>
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
-          <t>Project Objectives:
-Report per- and polyfluoroalkyl substance (PFAS) concentrations from a variety of agricultural inputs — animal manures, fertilizers, pesticides, composts, soil amendments, seed coatings, and biosolids-based products
-Compare the impact of various agricultural inputs on PFAS concentration in the soil profile over varying timeframes
-Evaluate the fate and transport of different inputs to PFAS contributions in agricultural systems at field-scale
-Determine relative contributions from biosolids-based products vs. other inputs to help develop/prioritize risk management strategies
+          <t>About the Organization
+We are Transform Health: a global coalition of more than 200 organisations driving the digital transformation of health to achieve universal health coverage. 
+Our focus is on strengthening the enabling environment—the  laws, regulation, policies, coordination structures and resources—that ensure the digital health transformation is equitable, inclusive and sustainable and that digital technologies are adopted responsibly, equitably, and at scale.  This means going beyond just the technologies and tools to create the conditions that enable this vision. 
+We tackle complex issues that no single organisation can resolve, leveraging the collective power and expertise of our dynamic coalition. 
+Our work is underpinned by our core values of equity, inclusion, rights, empowerment, and partnership.
+Together, we can achieve universal health coverage in the digital age.
+ About the Role:
+Transform Health is recruiting a consultant to develop a Technical Assistance (TA) approach and package that supports governments in applying the Digital Health and AI Investment Classification Framework, to aid budgeting, costing of digital health strategies/roadmaps, and analysis of digital health investment. The consultant will design the TA package and test it directly with governments in 3-4 countries, refining it based on the learnings. The work will be largely remote, with potential travel to testing countries.
+ Responsibilities:
+Deliverable 1 – Develop the TA package: Review the current draft concept note, Classification Framework, and user guide; conduct user-centric design investigation with likely TA users (government officials, technical partners); translate the three entry points for national use of the Framework into a practical, step-by-step TA delivery approach; develop supporting tools (budget/costing templates, guidance materials); consolidate into a TA package for review before country testing
+Deliverable 2 – Apply the TA package in 3-4 countries: Work with Transform Health and technical partners to identify pilot countries; support government engagement and sign-off (e.g., MoU); lead direct TA delivery in each pilot country; document the process, outputs, adaptations, and structured feedback
+Deliverable 3 – Refine the TA package: Synthesise learnings and feedback from pilot countries; produce a final, ready-to-scale TA package and tools; write a final report with recommendations; write brief case studies (~2 pages each) per pilot country; present findings to Transform Health; draft a journal article based on the process and outcomes
+ Eligibility:
+Willingness and ability to travel internationally as required
+Ability to work independently in multi-disciplinary, remote, cross-organisational teams
+ Qualification:
+Demonstrated understanding of the digital health ecosystem, particularly policy and funding landscape
+In-depth understanding of government digital health funding (national budgeting, costing of digital health strategies/frameworks)
+Familiarity with key digital health frameworks and tools
+Knowledge of national health financing systems, budget structures, and investment tracking tools (e.g., National Health Accounts)
+Strong analytical, research, and written communication skills
+Experience with user-centric/human-centred design approaches (needs assessment, prototyping, iterative refinement)
+Demonstrated experience delivering technical assistance directly to government counterparts, ideally across multiple countries
+Ability to manage multi-country consultancy engagements and coordinate with in-country focal points</t>
+        </is>
+      </c>
+      <c r="D18" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E18" s="1" t="inlineStr">
+        <is>
+          <t>Oct 23, 2026</t>
+        </is>
+      </c>
+      <c r="F18" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/rfps-invited-for-consultant-to-develop-a-technical-assistance-package-for-national-application-of-the-digital-health-and-ai-investment-classification-framework-transform-health-rfp-26-00359</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="95" customHeight="1">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Crossing the Divide Best Practices for Addressing Local and Privately-Owned Lateral Sewer Issues RFP 5419</t>
+        </is>
+      </c>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>Project Objective:
+To provide water resource recovery facilities (WRRFs) and collection system operators with an interactive manual of practice for implementing inflow and infiltration (I&amp;I) and obstruction management programs, focused on municipal and privately owned lateral sewers in complex legal, regulatory, and multi-jurisdictional environments.
  Background/Rationale:
-Growing concern exists over human exposure to PFAS through biosolids land application on agricultural systems, with regulatory bans on biosolids land application enacted or proposed in at least 12 U.S. states. Utilities relying on land application for biosolids management are scrambling for alternative disposal pathways. The U.S. EPA's 2026 draft guidance noted its earlier 2025 draft risk assessment of PFOA/PFOS-contaminated sewage sludge lacked important contextual information (e.g., a national survey of PFOA/PFOS concentrations). Risk assessments have focused primarily on biosolids, with less attention to PFAS contributions from other sources — manures, compost, fertilizers, pesticides, seed coatings, irrigation water, farming practices, and atmospheric deposition. A Minnesota Pollution Control Agency review found 12 inert pesticide ingredients classified as PFAS. This project aims to improve understanding of PFAS risks from the wider range of agricultural inputs to support strategic resource allocation and inform policy amid surging fertilizer prices and shifts toward local circular resources.
- Research Approach:
-Develop a baseline of knowledge on PFAS in biosolids and non-biosolids agricultural inputs via literature review, analytical methods evaluation, and examination of manufacturing/processing pathways; identify data gaps and uncertainties
-Measure/report compound-specific PFAS concentrations and profiles in agricultural inputs using standardized methods, including precursor characteristics for source attribution where possible
-Characterize PFAS contributions via literature review, data analysis, and field sampling — comparing soil profile/plant tissue composition between fields with non-biosolids inputs vs. biosolids-applied systems; study should test hypotheses on PFAS sources, transformation, retention, and mobility
-Optional additional focus areas: influence of soil/hydrologic/hydrochemistry conditions on PFAS behavior; degradation/transformation pathways; relative PFAS contributions across product lifecycle stages (manufacturing, bagging, delivery, etc.)
-Research approach should be hypothesis-driven, detailing specific end-user needs, and proposers are encouraged to leverage existing projects on PFAS plant uptake/fate/transport.
+Wastewater utilities face continuing challenges providing cost-effective sewer services amid rising demand, urban redevelopment, and performance disruptors (root intrusion, pipe degradation, blockages). I&amp;I and obstruction management remain persistent, costly problems without a consolidated resource to guide program design. During wet weather, peak I&amp;I flows can increase influent flows 3–5x average. Studies suggest up to 80% of I&amp;I originates on private property, and root intrusions cause over 50% of sewer blockages globally. Program effectiveness varies widely depending on statutory authority, multi-jurisdictional overlap, enforcement mechanisms, and participant willingness.
+ Central Research Questions:
+What I&amp;I and obstruction management practices are utilities using today, and how do they vary by jurisdictional/regulatory/infrastructure/environmental conditions?
+Which factors most influence successful implementation, and what barriers commonly derail programs?
+What measurable benefits (cost avoidance, capacity recovery, reduced spill risk, improved regulatory standing) have utilities realized from successful programs?
+This project extends WRF's ongoing "State-of-Practice Manual for Inflow and Infiltration Detection and Mitigation at Street and Private Lateral Levels" (Project 5365) into I&amp;I source control and obstruction management specifically.
+ Research Approach (4 Tasks):
+Literature and Regulatory Review — Comprehensive review of legal authorities/regulations in the US and comparable international jurisdictions; catalog program elements, enforcement mechanisms, incentive structures, and legal/jurisdictional barriers
+Utility Survey and Case Study Development — Broad survey across utility size/geography/system type; select at least 5 diverse in-depth case studies with quantitative results (I&amp;I reduction %, reduced bypass pumping, reduced basement backups, cost savings, recovered capacity, reduced blockage-related spills/service calls)
+Utility Workshop — At least one invitation-only workshop with utility representatives to present survey findings and gather structured feedback on draft guidance content
+Interactive Manual of Practice — Development of a decision-support tool/web-based application/interactive PDF enabling utilities to select effective I&amp;I/obstruction program elements based on their statutory authority, jurisdictional complexity, and enforcement mechanisms
  Expected Deliverables:
-Research report (WRF's Research Report Template) including: literature review, PFAS analysis of select products, risk management implications/prioritization recommendations, agriculture end-use guidance
-A webcast or workshop to share findings
-Optional additional deliverables: relative risk framework (mass input/fate/exposure/risk), decision support guide for farmers/regulators/utilities, plain language fact sheet, comparative PFAS mass input tool (spreadsheet/calculator)
- Project Duration: 36 months from contract start date (longer than the other two WRF grants above, which were 24 months)
+Research report (using WRF's Research Report Template) including literature/regulatory review
+Interactive manual of practice (following Technology Deliverables Guidance)
+In-depth utility survey, state-of-the-practice report, and at least 5 standalone case studies with quantitative results
+Summary documentation of the utility workshop, including feedback and how it was incorporated
+ Project Duration: 24 months from contract start date (No-Cost Extension Policy caps extensions at 9 months beyond original schedule)
  Eligibility to Submit:
-Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible. Not open to individuals (same structure as the two prior WRF grants).
+Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible as named participants. Not open to individuals (same institutional-applicant structure as RFP 5424).
  Budget/Funding:
-Maximum WRF funding: $400,000 (the largest of the three WRF grants shared so far)
+Maximum WRF funding: $250,000
 Applicant must contribute at least 33% of the project award as additional resources (cost share, applicant in-kind, or third-party in-kind per 2 CFR Part 200.306)
 Proposals not meeting the 33% minimum match will not be accepted
  Proposal Evaluation Criteria:
@@ -1608,37 +1695,105 @@
 Communication Plan, Deliverables, and Applicability: 15 points
 Budget and Schedule: 15 points
  Compliance Standards: OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
- Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00) — same deadline as the other two WRF grants</t>
-        </is>
-      </c>
-      <c r="D18" s="1" t="inlineStr">
+ Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
+        </is>
+      </c>
+      <c r="D19" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E18" s="1" t="inlineStr">
+      <c r="E19" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F18" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-comparison-of-pfas-contributions-to-agricultural-systems-the-water-research-foundation-wrf-opg-26-00190</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="95" customHeight="1">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="inlineStr">
+      <c r="F19" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-crossing-the-divide-best-practices-for-addressing-local-and-privately-owned-lateral-sewer-issues-rfp-5419-the-water-research-foundation-wrf-opg-26-00189</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="95" customHeight="1">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Adaptive Control Frameworks to Unlock Full-Scale BNR Potential Water Research Foundation WRF</t>
+        </is>
+      </c>
+      <c r="C20" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+The Water Research Foundation (WRF) is the leading research organization advancing the science of all water to meet the evolving needs of its subscribers and the water sector. WRF is a nonprofit, charitable and educational organization which funds, manages, and publishes research on the technology, operation, and management of drinking water, wastewater, reuse, and stormwater collection, treatment and supply systems—all in pursuit of ensuring water quality and improving water services to the public.
+ Project Objectives:
+Identify and categorize dominant failure modes of current aeration and process control implementations under real-world operating conditions
+Develop guidance on data/instrumentation requirements for utilities to support adaptive control — including characterizing existing sensor infrastructure and use of soft sensors where hard sensors are limited
+Develop practical adaptive control frameworks and implementation guidance deployable without dependence on proprietary black-box tools or specialized data science expertise, including hybrid approaches augmenting conventional controls with AI/ML and digital twins for variable flow/concentration conditions
+Benchmark control performance against biological capacity indicators across multiple full-scale facilities to quantify the gap between achievable and realized Biological Nutrient Removal (BNR) performance
+ Background/Rationale:
+The water sector routinely invests in capital-intensive solutions (additional aeration, supplemental carbon systems, tertiary filtration) to address BNR shortfalls that may actually be control execution problems, not biological potential. Adaptive control strategies (e.g., ammonia-based aeration control, ammonia vs. nitrate control) frequently fail under variable influent loading or temperature swings, causing operators to revert to manual control. This project targets that execution gap using digitalization, AI/ML, and sensors. Geographic focus: United States and Canada.
+ Research Approach (flexible, proposer-defined):
+Failure-Mode Characterization
+Sensor Infrastructure Inventory and Data Quality Assessment
+Soft Sensor Development and Validation
+Adaptive Control Framework Development (hybrid rule-based + AI/ML)
+Operator Adoption and Organizational Readiness
+Multi-Facility Benchmarking
+ Expected Deliverables:
+Comprehensive literature review (including WRF's own research)
+Utility-facing implementation guidance (controller selection, sensor infrastructure, tuning, calibration, operator training, maintenance, system integration) — must include a decision framework and failure-mode catalog
+Multi-facility dataset quantifying capacity-vs-performance gap, with utility case studies across US/Canada
+Outreach (webcasts, conference presentations)
+One open-access peer-reviewed journal paper
+ Project Duration: 24 months from contract start date (No-Cost Extension Policy caps extensions at 9 months beyond original schedule)
+ Eligibility to Submit:
+Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible to be named participants.
+ Budget/Funding:
+Maximum WRF funding: $300,000
+Applicant must contribute additional resources equivalent to at least 33% of the project award (e.g., $100,000 requested → minimum $33,000 additional contribution required, via cost share, applicant in-kind, or third-party in-kind)
+Proposals not meeting the 33% minimum match will not be accepted
+ Proposal Evaluation Criteria:
+Understanding the Problem and Responsiveness to RFP: 20 points
+Technical and Scientific Merit: 30 points
+Qualifications, Capabilities, and Management: 20 points
+Communication Plan, Deliverables, and Applicability: 15 points
+Budget and Schedule: 15 points
+ Compliance Standards: Administrative, cost, and audit standards comply with OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
+Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
+        </is>
+      </c>
+      <c r="D20" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E20" s="1" t="inlineStr">
+        <is>
+          <t>Oct 26, 2026</t>
+        </is>
+      </c>
+      <c r="F20" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-adaptive-control-frameworks-to-unlock-full-scale-bnr-potential-water-research-foundation-wrf-the-water-research-foundation-wrf-opg-26-00187</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="95" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 8th Call for Proposals Small-Size Grants Global EbA Fund</t>
         </is>
       </c>
-      <c r="C19" s="1" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -1701,59 +1856,57 @@
 Only successful applicants will be contacted; no individual feedback provided to unsuccessful applicants</t>
         </is>
       </c>
-      <c r="D19" s="1" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E19" s="1" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F19" s="1" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-8th-call-for-proposals-small-size-grants-global-eba-fund-global-eba-fund-opg-26-00177</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="95" customHeight="1">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Crossing the Divide Best Practices for Addressing Local and Privately-Owned Lateral Sewer Issues RFP 5419</t>
-        </is>
-      </c>
-      <c r="C20" s="1" t="inlineStr">
-        <is>
-          <t>Project Objective:
-To provide water resource recovery facilities (WRRFs) and collection system operators with an interactive manual of practice for implementing inflow and infiltration (I&amp;I) and obstruction management programs, focused on municipal and privately owned lateral sewers in complex legal, regulatory, and multi-jurisdictional environments.
+    <row r="22" ht="95" customHeight="1">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Comparison of PFAS Contributions to Agricultural Systems</t>
+        </is>
+      </c>
+      <c r="C22" s="1" t="inlineStr">
+        <is>
+          <t>Project Objectives:
+Report per- and polyfluoroalkyl substance (PFAS) concentrations from a variety of agricultural inputs — animal manures, fertilizers, pesticides, composts, soil amendments, seed coatings, and biosolids-based products
+Compare the impact of various agricultural inputs on PFAS concentration in the soil profile over varying timeframes
+Evaluate the fate and transport of different inputs to PFAS contributions in agricultural systems at field-scale
+Determine relative contributions from biosolids-based products vs. other inputs to help develop/prioritize risk management strategies
  Background/Rationale:
-Wastewater utilities face continuing challenges providing cost-effective sewer services amid rising demand, urban redevelopment, and performance disruptors (root intrusion, pipe degradation, blockages). I&amp;I and obstruction management remain persistent, costly problems without a consolidated resource to guide program design. During wet weather, peak I&amp;I flows can increase influent flows 3–5x average. Studies suggest up to 80% of I&amp;I originates on private property, and root intrusions cause over 50% of sewer blockages globally. Program effectiveness varies widely depending on statutory authority, multi-jurisdictional overlap, enforcement mechanisms, and participant willingness.
- Central Research Questions:
-What I&amp;I and obstruction management practices are utilities using today, and how do they vary by jurisdictional/regulatory/infrastructure/environmental conditions?
-Which factors most influence successful implementation, and what barriers commonly derail programs?
-What measurable benefits (cost avoidance, capacity recovery, reduced spill risk, improved regulatory standing) have utilities realized from successful programs?
-This project extends WRF's ongoing "State-of-Practice Manual for Inflow and Infiltration Detection and Mitigation at Street and Private Lateral Levels" (Project 5365) into I&amp;I source control and obstruction management specifically.
- Research Approach (4 Tasks):
-Literature and Regulatory Review — Comprehensive review of legal authorities/regulations in the US and comparable international jurisdictions; catalog program elements, enforcement mechanisms, incentive structures, and legal/jurisdictional barriers
-Utility Survey and Case Study Development — Broad survey across utility size/geography/system type; select at least 5 diverse in-depth case studies with quantitative results (I&amp;I reduction %, reduced bypass pumping, reduced basement backups, cost savings, recovered capacity, reduced blockage-related spills/service calls)
-Utility Workshop — At least one invitation-only workshop with utility representatives to present survey findings and gather structured feedback on draft guidance content
-Interactive Manual of Practice — Development of a decision-support tool/web-based application/interactive PDF enabling utilities to select effective I&amp;I/obstruction program elements based on their statutory authority, jurisdictional complexity, and enforcement mechanisms
+Growing concern exists over human exposure to PFAS through biosolids land application on agricultural systems, with regulatory bans on biosolids land application enacted or proposed in at least 12 U.S. states. Utilities relying on land application for biosolids management are scrambling for alternative disposal pathways. The U.S. EPA's 2026 draft guidance noted its earlier 2025 draft risk assessment of PFOA/PFOS-contaminated sewage sludge lacked important contextual information (e.g., a national survey of PFOA/PFOS concentrations). Risk assessments have focused primarily on biosolids, with less attention to PFAS contributions from other sources — manures, compost, fertilizers, pesticides, seed coatings, irrigation water, farming practices, and atmospheric deposition. A Minnesota Pollution Control Agency review found 12 inert pesticide ingredients classified as PFAS. This project aims to improve understanding of PFAS risks from the wider range of agricultural inputs to support strategic resource allocation and inform policy amid surging fertilizer prices and shifts toward local circular resources.
+ Research Approach:
+Develop a baseline of knowledge on PFAS in biosolids and non-biosolids agricultural inputs via literature review, analytical methods evaluation, and examination of manufacturing/processing pathways; identify data gaps and uncertainties
+Measure/report compound-specific PFAS concentrations and profiles in agricultural inputs using standardized methods, including precursor characteristics for source attribution where possible
+Characterize PFAS contributions via literature review, data analysis, and field sampling — comparing soil profile/plant tissue composition between fields with non-biosolids inputs vs. biosolids-applied systems; study should test hypotheses on PFAS sources, transformation, retention, and mobility
+Optional additional focus areas: influence of soil/hydrologic/hydrochemistry conditions on PFAS behavior; degradation/transformation pathways; relative PFAS contributions across product lifecycle stages (manufacturing, bagging, delivery, etc.)
+Research approach should be hypothesis-driven, detailing specific end-user needs, and proposers are encouraged to leverage existing projects on PFAS plant uptake/fate/transport.
  Expected Deliverables:
-Research report (using WRF's Research Report Template) including literature/regulatory review
-Interactive manual of practice (following Technology Deliverables Guidance)
-In-depth utility survey, state-of-the-practice report, and at least 5 standalone case studies with quantitative results
-Summary documentation of the utility workshop, including feedback and how it was incorporated
- Project Duration: 24 months from contract start date (No-Cost Extension Policy caps extensions at 9 months beyond original schedule)
+Research report (WRF's Research Report Template) including: literature review, PFAS analysis of select products, risk management implications/prioritization recommendations, agriculture end-use guidance
+A webcast or workshop to share findings
+Optional additional deliverables: relative risk framework (mass input/fate/exposure/risk), decision support guide for farmers/regulators/utilities, plain language fact sheet, comparative PFAS mass input tool (spreadsheet/calculator)
+ Project Duration: 36 months from contract start date (longer than the other two WRF grants above, which were 24 months)
  Eligibility to Submit:
-Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible as named participants. Not open to individuals (same institutional-applicant structure as RFP 5424).
+Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible. Not open to individuals (same structure as the two prior WRF grants).
  Budget/Funding:
-Maximum WRF funding: $250,000
+Maximum WRF funding: $400,000 (the largest of the three WRF grants shared so far)
 Applicant must contribute at least 33% of the project award as additional resources (cost share, applicant in-kind, or third-party in-kind per 2 CFR Part 200.306)
 Proposals not meeting the 33% minimum match will not be accepted
  Proposal Evaluation Criteria:
@@ -1763,105 +1916,37 @@
 Communication Plan, Deliverables, and Applicability: 15 points
 Budget and Schedule: 15 points
  Compliance Standards: OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
- Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
-        </is>
-      </c>
-      <c r="D20" s="1" t="inlineStr">
+ Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00) — same deadline as the other two WRF grants</t>
+        </is>
+      </c>
+      <c r="D22" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E20" s="1" t="inlineStr">
+      <c r="E22" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F20" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-crossing-the-divide-best-practices-for-addressing-local-and-privately-owned-lateral-sewer-issues-rfp-5419-the-water-research-foundation-wrf-opg-26-00189</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="95" customHeight="1">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Adaptive Control Frameworks to Unlock Full-Scale BNR Potential Water Research Foundation WRF</t>
-        </is>
-      </c>
-      <c r="C21" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-The Water Research Foundation (WRF) is the leading research organization advancing the science of all water to meet the evolving needs of its subscribers and the water sector. WRF is a nonprofit, charitable and educational organization which funds, manages, and publishes research on the technology, operation, and management of drinking water, wastewater, reuse, and stormwater collection, treatment and supply systems—all in pursuit of ensuring water quality and improving water services to the public.
- Project Objectives:
-Identify and categorize dominant failure modes of current aeration and process control implementations under real-world operating conditions
-Develop guidance on data/instrumentation requirements for utilities to support adaptive control — including characterizing existing sensor infrastructure and use of soft sensors where hard sensors are limited
-Develop practical adaptive control frameworks and implementation guidance deployable without dependence on proprietary black-box tools or specialized data science expertise, including hybrid approaches augmenting conventional controls with AI/ML and digital twins for variable flow/concentration conditions
-Benchmark control performance against biological capacity indicators across multiple full-scale facilities to quantify the gap between achievable and realized Biological Nutrient Removal (BNR) performance
- Background/Rationale:
-The water sector routinely invests in capital-intensive solutions (additional aeration, supplemental carbon systems, tertiary filtration) to address BNR shortfalls that may actually be control execution problems, not biological potential. Adaptive control strategies (e.g., ammonia-based aeration control, ammonia vs. nitrate control) frequently fail under variable influent loading or temperature swings, causing operators to revert to manual control. This project targets that execution gap using digitalization, AI/ML, and sensors. Geographic focus: United States and Canada.
- Research Approach (flexible, proposer-defined):
-Failure-Mode Characterization
-Sensor Infrastructure Inventory and Data Quality Assessment
-Soft Sensor Development and Validation
-Adaptive Control Framework Development (hybrid rule-based + AI/ML)
-Operator Adoption and Organizational Readiness
-Multi-Facility Benchmarking
- Expected Deliverables:
-Comprehensive literature review (including WRF's own research)
-Utility-facing implementation guidance (controller selection, sensor infrastructure, tuning, calibration, operator training, maintenance, system integration) — must include a decision framework and failure-mode catalog
-Multi-facility dataset quantifying capacity-vs-performance gap, with utility case studies across US/Canada
-Outreach (webcasts, conference presentations)
-One open-access peer-reviewed journal paper
- Project Duration: 24 months from contract start date (No-Cost Extension Policy caps extensions at 9 months beyond original schedule)
- Eligibility to Submit:
-Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible to be named participants.
- Budget/Funding:
-Maximum WRF funding: $300,000
-Applicant must contribute additional resources equivalent to at least 33% of the project award (e.g., $100,000 requested → minimum $33,000 additional contribution required, via cost share, applicant in-kind, or third-party in-kind)
-Proposals not meeting the 33% minimum match will not be accepted
- Proposal Evaluation Criteria:
-Understanding the Problem and Responsiveness to RFP: 20 points
-Technical and Scientific Merit: 30 points
-Qualifications, Capabilities, and Management: 20 points
-Communication Plan, Deliverables, and Applicability: 15 points
-Budget and Schedule: 15 points
- Compliance Standards: Administrative, cost, and audit standards comply with OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
-Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
-        </is>
-      </c>
-      <c r="D21" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E21" s="1" t="inlineStr">
-        <is>
-          <t>Oct 26, 2026</t>
-        </is>
-      </c>
-      <c r="F21" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-adaptive-control-frameworks-to-unlock-full-scale-bnr-potential-water-research-foundation-wrf-the-water-research-foundation-wrf-opg-26-00187</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="95" customHeight="1">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="inlineStr">
+      <c r="F22" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-comparison-of-pfas-contributions-to-agricultural-systems-the-water-research-foundation-wrf-opg-26-00190</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="95" customHeight="1">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Whitley Award 2027</t>
         </is>
       </c>
-      <c r="C22" s="1" t="inlineStr">
+      <c r="C23" s="1" t="inlineStr">
         <is>
           <t>About the Grant: 
 An annual grant by the Whitley Fund for Nature (WFN) recognising grassroots conservation leaders in the Global South, providing funding to support and scale up proven, science-based solutions that deliver lasting impact for both people and nature.
@@ -1874,34 +1959,34 @@
 You do not need to be invited or nominated to apply.</t>
         </is>
       </c>
-      <c r="D22" s="1" t="inlineStr">
+      <c r="D23" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E22" s="1" t="inlineStr">
+      <c r="E23" s="1" t="inlineStr">
         <is>
           <t>Oct 30, 2026</t>
         </is>
       </c>
-      <c r="F22" s="1" t="inlineStr">
+      <c r="F23" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-whitley-award-2027-whitley-fund-for-nature-wfn-opg-26-00153</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="95" customHeight="1">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B23" s="1" t="inlineStr">
+    <row r="24" ht="95" customHeight="1">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIFAR Global Scholars Program 20272029 Cohort</t>
         </is>
       </c>
-      <c r="C23" s="1" t="inlineStr">
+      <c r="C24" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 CIFAR is a Canadian-based globally influential research organization that convenes the world’s most brilliant people across disciplines to advance transformative knowledge and solve humanity’s biggest problems, together. By supporting long-term interdisciplinary collaboration, CIFAR provides researchers with an unparalleled environment of trust, transparency and knowledge sharing. Our time-tested model inspires new directions of inquiry, accelerates discovery and yields breakthroughs across borders and academic disciplines. Through knowledge mobilization, we are catalysts for change in industry, government and society. Through our 15 research programs and the Pan-Canadian AI Strategy, CIFAR convenes close to 400 of the world’s top researchers from 141 institutions in 20 countries. CIFAR is generously supported by the governments of Canada, Alberta and Québec, as well as foundations, individuals, corporations and Canadian and international partner organizations.
@@ -1945,58 +2030,19 @@
  Application Deadline: November 4, 2026, 12:00 PM EST</t>
         </is>
       </c>
-      <c r="D23" s="1" t="inlineStr">
+      <c r="D24" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E23" s="1" t="inlineStr">
+      <c r="E24" s="1" t="inlineStr">
         <is>
           <t>Nov 4, 2026</t>
         </is>
       </c>
-      <c r="F23" s="1" t="inlineStr">
+      <c r="F24" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cifar-global-scholars-program-20272029-cohort-cifar-canadian-institute-for-advanced-research-opg-26-00183</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="95" customHeight="1">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B24" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for IWRS Teaching Innovation Award</t>
-        </is>
-      </c>
-      <c r="C24" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
- About the Grant
-The IWRS (Insect Welfare Research Society) Teaching Innovation Award supports instructors developing new approaches to teaching insect or invertebrate biology that incorporate the 3Rs (Replacement, Reduction, and Refinement) — principles for reducing animal welfare impacts in teaching and research practices.
- Purpose
-Funds support the creation and implementation of 3Rs-driven instructional materials and pedagogical approaches. Priority is given to proposals addressing common teaching practices with substantial welfare implications.
- Grant Amount
-Two awards of $2,000 USD are available annually.</t>
-        </is>
-      </c>
-      <c r="D24" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E24" s="1" t="inlineStr">
-        <is>
-          <t>Nov 15, 2026</t>
-        </is>
-      </c>
-      <c r="F24" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
         </is>
       </c>
     </row>
@@ -2050,10 +2096,49 @@
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
+          <t>Applications Invited for IWRS Teaching Innovation Award</t>
+        </is>
+      </c>
+      <c r="C26" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
+ About the Grant
+The IWRS (Insect Welfare Research Society) Teaching Innovation Award supports instructors developing new approaches to teaching insect or invertebrate biology that incorporate the 3Rs (Replacement, Reduction, and Refinement) — principles for reducing animal welfare impacts in teaching and research practices.
+ Purpose
+Funds support the creation and implementation of 3Rs-driven instructional materials and pedagogical approaches. Priority is given to proposals addressing common teaching practices with substantial welfare implications.
+ Grant Amount
+Two awards of $2,000 USD are available annually.</t>
+        </is>
+      </c>
+      <c r="D26" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E26" s="1" t="inlineStr">
+        <is>
+          <t>Nov 15, 2026</t>
+        </is>
+      </c>
+      <c r="F26" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="95" customHeight="1">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
+        <is>
           <t>Applications Invited for Medium-Size Grants Call for Proposals Global EbA Fund</t>
         </is>
       </c>
-      <c r="C26" s="1" t="inlineStr">
+      <c r="C27" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -2110,34 +2195,34 @@
 Applications submitted via online portal (link shared on the Medium-Size Grants webpage from Oct 12)</t>
         </is>
       </c>
-      <c r="D26" s="1" t="inlineStr">
+      <c r="D27" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E26" s="1" t="inlineStr">
+      <c r="E27" s="1" t="inlineStr">
         <is>
           <t>Nov 16, 2026</t>
         </is>
       </c>
-      <c r="F26" s="1" t="inlineStr">
+      <c r="F27" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-medium-size-grants-call-for-proposals-global-eba-fund-global-eba-fund-opg-26-00178</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="95" customHeight="1">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B27" s="1" t="inlineStr">
+    <row r="28" ht="95" customHeight="1">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIEIF Grant 2026 Climate Intervention Environmental Impact Fund</t>
         </is>
       </c>
-      <c r="C27" s="1" t="inlineStr">
+      <c r="C28" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Climate Intervention Environmental Impact Fund (CIEIF) is a philanthropic fund focused on supporting responsible climate intervention field tests. It provides grants for activities such as environmental impact assessment (EIA), predictive impact modelling, and engagement with potentially affected stakeholders, including local communities and government agencies.
@@ -2164,34 +2249,34 @@
 Potential for scaling the innovation to a globally relevant level</t>
         </is>
       </c>
-      <c r="D27" s="1" t="inlineStr">
+      <c r="D28" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E27" s="1" t="inlineStr">
+      <c r="E28" s="1" t="inlineStr">
         <is>
           <t>Dec 1, 2026</t>
         </is>
       </c>
-      <c r="F27" s="1" t="inlineStr">
+      <c r="F28" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cieif-grant-2026-climate-intervention-environmental-impact-fund-climate-intervention-environmental-impact-fund-opg-26-00155</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="95" customHeight="1">
-      <c r="A28" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B28" s="1" t="inlineStr">
+    <row r="29" ht="95" customHeight="1">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 6th Annual Seeding The Future Global Food System Challenge</t>
         </is>
       </c>
-      <c r="C28" s="1" t="inlineStr">
+      <c r="C29" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are one of the largest and most respected private organisations for development cooperation and humanitarian aid in Germany. As a politically and confessionally independent organisation, our value-oriented actions are always based on ethical principles. Our vision is clear: "Zero Hunger by 2030"
@@ -2223,34 +2308,34 @@
 Individuals with no organizational entity</t>
         </is>
       </c>
-      <c r="D28" s="1" t="inlineStr">
+      <c r="D29" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E28" s="1" t="inlineStr">
+      <c r="E29" s="1" t="inlineStr">
         <is>
           <t>Jan 1, 2027</t>
         </is>
       </c>
-      <c r="F28" s="1" t="inlineStr">
+      <c r="F29" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-6th-annual-seeding-the-future-global-food-system-challenge-welthungerhilfe-opg-26-00180</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="95" customHeight="1">
-      <c r="A29" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B29" s="1" t="inlineStr">
+    <row r="30" ht="95" customHeight="1">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for BES Training and Travel Grants</t>
         </is>
       </c>
-      <c r="C29" s="1" t="inlineStr">
+      <c r="C30" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are a global community of scientists shining a spotlight on the intricacy and value of our natural world, providing the evidence for better decisions. Our vision is for people and nature to thrive in a world that values ecology.
@@ -2289,17 +2374,17 @@
  Application Deadline (Round 2): Opens 30 April 2026, closes 17 May 2026</t>
         </is>
       </c>
-      <c r="D29" s="1" t="inlineStr">
+      <c r="D30" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E29" s="1" t="inlineStr">
+      <c r="E30" s="1" t="inlineStr">
         <is>
           <t>May 17, 2027</t>
         </is>
       </c>
-      <c r="F29" s="1" t="inlineStr">
+      <c r="F30" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-bes-training-and-travel-grants-british-ecological-society-opg-26-00181</t>
         </is>

</xml_diff>

<commit_message>
Auto update Combined.xlsx [Fri Sep 18 06:59:43 UTC 2026]
</commit_message>
<xml_diff>
--- a/output/Combined.xlsx
+++ b/output/Combined.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -467,55 +467,10 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>ToR - Behavioural Insights and Narrative Inquiry for the Climate Responsive Livelihood Programme Meghalaya</t>
+          <t>Expression of Interest EOI for Trade &amp; Livelihood Partners</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
-        <is>
-          <t>Title  Behavioural Insights and Narrative Inquiry for the Climate Responsive Livelihood Programme, Meghalaya
-Timeline  2 months
-Expected    area of expertise The agency should have demonstrated expertise in behavioural science, qualitative and ethnographic research, narrative inquiry, human-centred research and community engagement, with experience in government, development or community-based programmes.
-Apply Link https://forms.gle/TFE6Nc4djRBtrdN16
-Last    Date           for Apply 19th September 2026
-About SELCO Foundation:
-SELCO Foundation’s mission is to create a platform of solutions that uses sustainable energy as a catalyst to bridge environmental sustainability and poverty alleviation. With holistic development as the primary focus, the organization strives to create equitable societies, where services are accessed by all communities. The interventions of SELCO lead to a sustainable delivery model of essential services like livelihoods, education, and health till the last mile. (Read more about SELCO here: http://www.selcofoundation.org/)
- About the Programmes:
-The Climate Responsive Livelihood (CRL) Programme seeks to strengthen livelihood resilience while enabling communities to adapt to a changing climate. As the programme evolves, there is an opportunity to understand not only the economic realities of potential participants, but also the asp irations, motivations, beliefs, identities and social norms that shape livelihood decisions.
-Experience from behavioural science suggests that participation in livelihood opportunities is influenced as much by identity, perceived opportunity, social expectations and narratives of possibility  as  by  access  to  resources  or  information.  Similarly,  narrative research demonstrates that the stories people tell about themselves and their futures influence how they engage with new opportunities and collective action.
-This assignment seeks to generate a grounded understanding of how different groups across Meghalaya perceive work, entrepreneurship, livelihoods, risk, climate, success and opportunity, and translate these insights into a compelling narrative framework that can guide future programme mobilisation, engagement and communication.
- Roles and Responsibilities
-The selected agency will undertake an exploratory behavioural and narrative inquiry across selected districts of Meghalaya to understand the motivations, aspirations and lived experiences of intended participants of the Climate Responsive Livelihood Programme.
-Rather than evaluating awareness or testing communication materials, the assignment should seek to uncover deeper behavioural and social drivers that influence livelihood choices and participation. The findings will inform a narrative architecture and mobilisation approach that resonates authentically with communities across the state.</t>
-        </is>
-      </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>Sep 19, 2026</t>
-        </is>
-      </c>
-      <c r="F2" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/tor-behavioural-insights-and-narrative-inquiry-for-the-climate-responsive-livelihood-programme-meghalaya-selco-foundation-rfp-26-00355</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="95" customHeight="1">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>Expression of Interest EOI for Trade &amp; Livelihood Partners</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Expression of Interest (EOI) for Trade &amp; Livelihood Partners
 Issued By: BharatCares
@@ -642,34 +597,34 @@
 Any prior work with tribal or rural communities, with references if available</t>
         </is>
       </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>Sep 20, 2026</t>
         </is>
       </c>
-      <c r="F3" s="1" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/expression-of-interest-eoi-for-trade-and-livelihood-partners-bharatcares-rfp-26-00340</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="95" customHeight="1">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
+    <row r="3" ht="95" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>RFP - Research Collaboration For Improved Application and Processing Techniques For Natural Dyes</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>REǪUEST FOR PROPOSALS (RFP)
 Research Collaboration For Improved Application and Processing Techniques For Natural Dyes
@@ -722,34 +677,34 @@
 Network with dyeing units and textile industry associations</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>Climate</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Sep 20, 2026</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfp-research-collaboration-for-improved-application-and-processing-techniques-for-natural-dyes-chitrika-rfp-26-00343</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="95" customHeight="1">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
+    <row r="4" ht="95" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>RFP - Agronomic Research Study For Natural Dye Crop Development</t>
         </is>
       </c>
-      <c r="C5" s="1" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>REǪUEST FOR PROPOSALS (RFP)
 Agronomic Research Study For Natural Dye Crop Development
@@ -808,34 +763,34 @@
 Experience working on natural dye</t>
         </is>
       </c>
-      <c r="D5" s="1" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E5" s="1" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>Sep 20, 2026</t>
         </is>
       </c>
-      <c r="F5" s="1" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfp-agronomic-research-study-for-natural-dye-crop-development-chitrika-rfp-26-00344</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="95" customHeight="1">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
+    <row r="5" ht="95" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>RFPs Invited for Using an Agent Based Model to Predict the Impact of City-Level Policies on the Adoption of Distributed Renewable Energy</t>
         </is>
       </c>
-      <c r="C6" s="1" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>About C40:
 C40 is a network of nearly 100 mayors of the world's leading cities working to deliver urgent climate action and create a future where everyone, everywhere, can thrive. Mayors of C40 cities are committed to using a science-based, people-focused approach to limit global heating in line with the Paris Agreement, working alongside labour, business, youth climate movement, and civil society representatives to help halve emissions by 2030.
@@ -878,34 +833,34 @@
 Project runs until: June 30, 2027</t>
         </is>
       </c>
-      <c r="D6" s="1" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E6" s="1" t="inlineStr">
+      <c r="E5" s="1" t="inlineStr">
         <is>
           <t>Sep 20, 2026</t>
         </is>
       </c>
-      <c r="F6" s="1" t="inlineStr">
+      <c r="F5" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfps-invited-for-using-an-agent-based-model-to-predict-the-impact-of-city-level-policies-on-the-adoption-of-distributed-renewable-energy-c40-cities-rfp-26-00357</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="95" customHeight="1">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
+    <row r="6" ht="95" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>E-Tender Request for Digital Communication Website Development and Social Media Campaign for Colors of Nature</t>
         </is>
       </c>
-      <c r="C7" s="1" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>REǪUEST FOR PROPOSALS (RFP)
 Digital Communication, Website Development and Social Media Campaign
@@ -951,80 +906,34 @@
 Ready to develop a women led and based digital marketing team</t>
         </is>
       </c>
-      <c r="D7" s="1" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E7" s="1" t="inlineStr">
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>Sep 20, 2026</t>
         </is>
       </c>
-      <c r="F7" s="1" t="inlineStr">
+      <c r="F6" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/e-tender-request-for-digital-communication-website-development-and-social-media-campaign-for-colors-of-nature-chitrika-rfp-26-00342</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="95" customHeight="1">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Wellbeing Research Grants Funding Better Evaluations of AI's Impact on Wellbeing</t>
-        </is>
-      </c>
-      <c r="C8" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-We're an AI research company that builds reliable, interpretable, and steerable AI systems. Our first product is Claude, an AI assistant for tasks at any scale. Our research interests span multiple areas including natural language, human feedback, scaling laws, reinforcement learning, code generation, and interpretability. 
- About the Opportunity:
-Anthropic is launching a $5 million grant program to fund independent research into how AI impacts users' wellbeing. The program will provide direct funding, access to Anthropic's models, and technical support to grantees building open-source evaluations that help the AI industry measure how models affect those who use them. Grantees will work fully independently, and will publish their work as open-source projects that any developer can make use of.
- Background/Rationale:
-AI systems have become central to how many people work, learn, and solve problems, and have also become conversational partners and sources of emotional support during difficult times, but the industry is still developing clear standards for how models should behave in such conversations — for example when a user seeks companionship or navigates a mental health crisis. Wellbeing is described as a particularly difficult area to evaluate, since assessing it requires more context than checking a single response for accuracy — the need for a cautious response may only become clear over a long conversation, and a response reasonable in one context could be harmful in another. By funding independent evaluations and benchmarks of user wellbeing, Anthropic hopes to invite more people — including clinicians, psychologists, and methodologists — to contribute to this field. 
- What They're Looking For
-Grantees should build evaluations that:
-State clearly what they are measuring (what counts as a pass or fail, and why it matters) 
-Involve clinical and subject-matter experts in the design and validation 
-Test both precautions and harms (i.e., evaluate the risk of both overcompliance and overrefusal) 
-Reflect how users actually use AI, often through multi-turn conversation scenarios where risk escalates and context shifts
-Validate their graders against real subject-matter experts 
- Eligibility/Target Applicants: Independent researchers — clinicians, psychologists, methodologists, and other subject-matter experts working on AI wellbeing evaluation/benchmarking
- Funding Amount: Total program pool of $5 million (individual grant sizes not specified on the page)</t>
-        </is>
-      </c>
-      <c r="D8" s="1" t="inlineStr">
-        <is>
-          <t>Learning</t>
-        </is>
-      </c>
-      <c r="E8" s="1" t="inlineStr">
-        <is>
-          <t>Sep 21, 2026</t>
-        </is>
-      </c>
-      <c r="F8" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-wellbeing-research-grants-funding-better-evaluations-of-ais-impact-on-wellbeing-anthropic-opg-26-00175</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="95" customHeight="1">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="inlineStr">
+    <row r="7" ht="95" customHeight="1">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for GEF SGP CSO Challenge Program</t>
         </is>
       </c>
-      <c r="C9" s="1" t="inlineStr">
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global Environment Facility Small Grants Programme (SGP) is a global initiative implemented by the United Nations Development Programme (UNDP) on behalf of the Global Environment Facility (GEF). Since its launch in 1992, SGP has empowered communities worldwide to take action on environmental challenges while improving livelihoods. As a GEF Corporate Programme, SGP provides direct support to civil society organisations and community-based organisations to design and implement innovative, locally driven solutions. The programme places strong emphasis on inclusion, ensuring meaningful participation of Indigenous Peoples, youth, women and girls, and other underrepresented groups.
@@ -1073,34 +982,34 @@
 Risk management and mitigation</t>
         </is>
       </c>
-      <c r="D9" s="1" t="inlineStr">
+      <c r="D7" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E9" s="1" t="inlineStr">
+      <c r="E7" s="1" t="inlineStr">
         <is>
           <t>Sep 23, 2026</t>
         </is>
       </c>
-      <c r="F9" s="1" t="inlineStr">
+      <c r="F7" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-gef-sgp-cso-challenge-program-gef-small-grants-programme-sgp-opg-26-00184</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="95" customHeight="1">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
+    <row r="8" ht="95" customHeight="1">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>RFP for Impact Assessment</t>
         </is>
       </c>
-      <c r="C10" s="1" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>Introduction
 Titan Company Limited, a member of the Tata Group, has a long-standing commitment to Corporate Social Responsibility (CSR) in India. The company's CSR initiatives derive its philosophy from the Company’s vision statement: “We create elevating experiences for the people we touch and significantly impact the world we work in”. The initiatives are designed to promote inclusive growth, empower communities, and contribute to the country's socio-economic development. The program includes Titan’s CSR policy is governed by a dedicated CSR Committee that ensures transparency and compliance with regulatory requirements. The program includes Girl Child Education, Skill and Entrepreneurship Development, supporting Indian Heritage Arts and Crafts, Integrated Village Development Programme, Eye Care and Affirmative Action. Titan's CSR policy is governed by a dedicated CSR Committee that ensures transparency and compliance with regulatory requirements.
@@ -1134,19 +1043,131 @@
 Timeline: Proposal submission deadline: September 24, 2026</t>
         </is>
       </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Sep 24, 2026</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/rfp-for-impact-assessment-titan-rfp-26-00354</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="95" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>ToR - Engagement of Information Design &amp; Video Production Agency / Consultant for Key Learning &amp; Dissemination Outputs</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>Terms of Reference (TOR) for Consultancy Services
+Title  Engagement of Information Design &amp; Video Production Agency / Consultant for Key Learning &amp; Dissemination Outputs
+Timeline 12 Months (1st October 2026 – 31st September 2027)
+Expected area of expertise
+ Proven experience in information design, data visualization, narrative structuring, and short-form video editing/production (preferably in the development/social sector).
+Portfolio demonstrating translation of complex, technical, or research-heavy content into engaging visual and video formats.
+Alignment with SELCO’s brand ethos and open-source dissemination principles.
+Apply Link https://forms.gle/kDNRaSdQAkqbDMrM8
+Last             Date           for Apply 28th September 2026; 5 PM
+About SELCO Foundation:
+SELCO Foundation’s mission is to create a platform of solutions that uses sustainable energy as a catalyst to bridge environmental sustainability and poverty alleviation. With holistic development as the primary focus, the organization strives to create equitable societies, where services are accessed by all communities. The interventions of SELCO lead to a sustainable delivery model of essential services like livelihoods, education, and health till the last mile. (Read more about SELCO here: http://www.selcofoundation.org/)
+About the Programmes:
+SELCO Foundation continuously generates field insights, technical frameworks, program impacts, and sectoral learnings across its core operational verticals (rural healthcare, urban livelihoods, climate adaptation, and regenerative agriculture). Effectively capturing and translating these raw research assets into accessible, high-quality public visual narratives is essential for driving ecosystem alignment and sector-wide knowledge exchange.
+Objective:
+The primary objective of this engagement is to enable SELCO Foundation to effectively capture, structure, and communicate its field insights, sectoral learnings, and program impacts. The selected Agency/Consultant (or Agencies/Consultants) will work on a monthly retainer basis to translate raw content, data, field footage, and reports provided by SELCO into high-quality, visually compelling, reader-friendly visual outputs and video assets.</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>Sep 28, 2026</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/tor-engagement-of-information-design-and-video-production-agency-consultant-for-key-learning-and-dissemination-outputs-selco-foundation-rfp-26-00362</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="95" customHeight="1">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>Application Invited for Giving Joy Microgrant</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+Giving Joy is a US-based nonprofit that strengthens and inspires women’s entrepreneurship worldwide. Through its micro-grants and mentorship program, Giving Joy helps women establish or improve their businesses and initiatives—for their benefit and the benefit of their communities. To date, Giving Joy has awarded over 88 grants to women-led initiatives in 26 countries.
+ 2026 Grant Cycle
+Beginning in 2026, Giving Joy has moved to two global grant cycles per year.
+The organization states that this change was made after operating multiple regional rounds, with the aim of:
+Providing clearer timelines for applicants
+Increasing the quality and depth of application reviews
+Reducing administrative burden
+Improving support for grantees
+Focusing communications and fundraising more effectively
+Continuing to reach women entrepreneurs globally without dividing applications by geography
+Each cycle is open to women entrepreneurs worldwide.
+ Eligible Fields / Activities
+There is no restriction to a particular field such as health.
+Applicants can propose activities in:
+Any field
+Trade
+Occupation
+Craft
+ What Does Giving Joy Look For?
+Giving Joy prioritizes:
+Innovative ideas
+Creative ideas
+Strong potential for social impact
+Initiative
+Real community impact
+Clear economic and/or social benefits for women and girls
+ Grant Amount
+Maximum Grant
+Up to $500 USD
+The exact award amount is determined by Giving Joy based on:
+Proposed activities
+Availability of funding
+ Grant Duration
+The grant period is six months.</t>
+        </is>
+      </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>Governance</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>Sep 24, 2026</t>
+          <t>Sep 30, 2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/rfps/rfp-for-impact-assessment-titan-rfp-26-00354</t>
+          <t>https://onepurpos.in/openings/grants/application-invited-for-giving-joy-microgrant-giving-joy-opg-26-00185</t>
         </is>
       </c>
     </row>
@@ -1225,32 +1246,48 @@
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
-          <t>Applications Invited for Signals of Change Shaping the Future of Sexual and Reproductive Health and Rights SRHR</t>
+          <t>RFP - Design and Delivery of an Electric Vehicle EV Skilling Programme in Karnataka</t>
         </is>
       </c>
       <c r="C12" s="1" t="inlineStr">
         <is>
           <t>About the Organization
-The World Health Organization's mission: to promote health, keep the world safe, and serve the vulnerable. Working through offices in more than 150 countries, WHO staff work side by side with governments and other partners to ensure the highest attainable level of health for all people.
- About the Opportunity
-HRP and its UN co-sponsors are leading a global Sexual and Reproductive Health and Rights (SRHR) foresight and research prioritization process for 2026–2036. This open public consultation invites diverse stakeholder input to identify "signals of change" — emerging trends, shifts, or disruptions — that could shape the future of SRHR over the next decade. The process uses foresight methodology (not prediction) to explore plausible futures and will culminate in a published report and research agenda in 2027.
- Guiding Questions
-What future trends will shape or constrain SRHR over the next 10 years?
-What evidence and research investments are needed today to prepare SRHR for the futures we may face?
- Scope of Submissions 
-Economic systems; social infrastructure; structural discrimination; conflict/forced migration/displacement; mega-trends (demographic shifts, climate change, digital transformation/AI, urbanization); conditions of daily life; rights/legal/governance systems; health systems; media/misinformation; and changes in the research ecosystem.
- Who Can Participate 
-Open to individuals and organizations globally, including:
-Health workers, professional associations, clinical networks
-Civil society, community groups, youth-led organizations, rights movements
-Governments, parliamentarians, regulators, public sector bodies
-Researchers, academia, think tanks, technical experts
-UN agencies, multilateral/humanitarian/development organizations
-Funders, philanthropy, private sector, tech/innovation organizations
-Media, communications, journalism
-Anyone with relevant lived experience or perspective
-Special interest in submissions from health worker, community, youth, and rights-movement spaces not typically represented in published forums.
- Submission Requirements: Descriptive information (name, contact email, country, sector) required alongside each submission; formal published evidence is helpful but not required — practice-based experience and field examples are also welcome. Submissions are kept confidential and anonymized before analysis.</t>
+WRI India, an independent knowledge organisation registered as the India Resources Trust, provides objective information and practical proposals to foster environmentally sound and socially equitable development. As an independent knowledge organisation, we leverage our data and expertise to catalyze change across systems like food, land and water; energy; and cities. Our work focuses on improving people’s lives, protecting and restoring nature, and addressing climate change. To enable progress at the pace and scale needed, we also engage with the economic, finance and governance systems that are key to enabling this change.
+Project background
+This work is being undertaken as part of the “Electrifying Mobility in Cities: Investing in the Transformation to Electric Mobility in India” initiative by the United Nations Environment Programme (UNEP), funded by the Global Environment Facility (GEF), guided by NITI Aayog and executed on ground by WRI India. The project workstreams focus on freight electrification, battery circularity and enabling a just and equitable transition to electric mobility in India. Under the workstream on ‘Enabling a just and equitable transition to electric mobility’, WRI India proposes targeted e-mobility skilling programmes in Karnataka, in collaboration with the Karnataka Electric Vehicle Manufacturers &amp; Dealers Association (KEVMDA) and Federation of Karnataka Chambers of Commerce and Industry (FKCCI). The proposed intervention will focus on strengthening workforce readiness in the EV repair and maintenance ecosystem, with a specific focus on women and informal workers.
+Context about the assignment 
+India’s EV penetration has crossed the double-digit mark, reaching 12.5% in June 20261 , indicating that the transition is moving from early adoption to wider market scale. As the country works towards the EV30@30 target, the sector will require a trained workforce that can safely operate, diagnose, repair and maintain EV systems across vehicle segments. This makes downstream workforce readiness particularly important. A large share of India’s automotive workforce (80.4%) is concentrated in post-manufacturing activities such as dealerships, service centers, repairs, and aftersales support2 . These segments include a significant number of informal and semi-skilled workers who may have limited access to formal training, certification, and employment pathways in the emerging EV ecosystem.
+Without targeted skilling, the EV transition may create a mismatch between market growth and repair and service capacity. This could adversely affect vehicle uptime, safety, consumer confidence, and the long-term reliability of EV adoption. Workers transitioning to EV repair and maintenance will require specialized competencies in high-voltage safety, battery systems, diagnostics, power electronics, thermal management, software-enabled fault detection, troubleshooting, etc.
+The EV transition also presents a significant opportunity to build a more gender-inclusive workforce in the automotive sector. While women's participation is gradually increasing in select parts of the EV value chain, including assembly, product development, and software roles, their presence in downstream technical occupations remains limited. Targeted training for women in EV repair and maintenance will create entry points into non-traditional automotive roles.
+Karnataka stands among India's most advanced EV markets. The state has achieved 8.5% EV penetration against a national average of 8.19% in FY20263 , recorded a 17-fold increase in EV sales between FY2021 and FY2026, and is home to approximately 8,600+ EV charging stations 4 .Under the Karnataka Clean Mobility Policy 2025-30, the state targets USD 5.2 billion in investments and the creation of 1 lakh jobs in the clean mobility sector. 
+As EV adoption and manufacturing activities scale, Karnataka will need a parallel focus on the repair and maintenance ecosystem that supports vehicle deployment, customer confidence, and long-term performance. This includes strengthening the capabilities of service technicians, informal mechanics, workshop workers, and new entrants into the EV workforce. 
+Karnataka's early-mover advantage in EV adoption, combined with an established industrial base and an active mandate for clean mobility, makes it an ideal geography to pilot targeted e-mobility skilling programmes. The proposed intervention can demonstrate a practical, industry-aligned, and inclusive skilling model for the EV repair and maintenance ecosystem, with learnings that can inform other such initiatives across Karnataka and other high-growth EV markets across India.
+Objective
+WRI India intends to engage an experienced and qualified Training Partner to design and deliver an EV skilling programme across 2-3 cities in Karnataka, including participant mobilization, classroom and practical training, on-the-job (OJT) training, assessment, certification, and placement/apprenticeship support. The proposed intervention will strengthen workforce readiness in the EV repair and maintenance ecosystem, with a focus on women and informal workers
+Scope of Work
+ The selected Training Partner will be entrusted with a range of responsibilities which includes:
+Needs assessment, mobilization and participant engagement 
+Conduct a rapid needs assessment for each selected city and/or cohort to assess participant education and prior work experience, existing technical competencies and learning needs, local EV industry requirements, employer demand, and relevant practical training and placement/ apprenticeship opportunities. Findings from the assessment shall inform the final curriculum and programme delivery approach.
+Undertake targeted, on-ground mobilization of women and informal workers in the selected cities, including existing ICE mechanics, small-garage workers, workshop assistants/helpers, and workers in unorganized workshops and informal enterprises. 
+Accompany mobilization with participant counselling on the programme structure, training and OJT requirements, available incentives/support, relevant placement/ apprenticeship opportunities, and indicative career pathways. Where relevant, counselling may also engage participants' families to support informed participation and programme retention. 
+The Training Partner shall verify participants’ identity by their government-issued identification documents, subject to obtaining necessary consent and complying with applicable privacy and data protection requirements.
+Eligibility 
+To be considered for empanelment as a Training Partner under this programme, applicants must satisfy the following criteria:
+Organizational registration
+Must be a registered firm, company, partnership, society, or trust incorporated under applicable Indian law.
+Must have been in operation for a minimum of three years as of the date of this RFP.
+Vocational training experience
+Must have a demonstrated track record of at least three years in the design and delivery of vocational or skill development training programmes.
+Certified training partners of respective Sector Skill Council (SSC) with prior experience in automotive/ EV repair and maintenance, EV-specific trainings, or related electrical/electronics and automotive trades will be preferred.
+Must provide evidence of past training projects, including programme scope, number of participants trained, certification outcomes, and placement rates.
+Experience working with government skilling schemes (e.g., Pradhan Mantri Kaushal Vikas Yojana, Deen Dayal Upadhyaya Grameen Kaushalya Yojana) or in collaboration with SSCs, National Skill Development Corporation (NSDC), or other national skilling bodies will be preferred. 
+Any awards, recognitions, or certifications received for excellence in vocational training should be highlighted. 
+Inclusive practices 
+Must demonstrate prior experience in designing and delivering training programmes specifically targeting women, informal workers, and/ or marginalized communities. 
+Must present a credible plan for mobilizing, enrolling, and supporting women and informal workers throughout the training and placement/apprenticeship cycle.
+Infrastructure and resources 
+Must possess or have access to adequate training infrastructure in Karnataka, including a well-equipped training centre with relevant tools, machinery, and a conducive learning environment. 
+Must have a team of qualified trainers and master trainers with relevant domain expertise, as well as administrative and coordination support.</t>
         </is>
       </c>
       <c r="D12" s="1" t="inlineStr">
@@ -1260,12 +1297,12 @@
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>Sep 30, 2026</t>
+          <t>Oct 5, 2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-signals-of-change-shaping-the-future-of-sexual-and-reproductive-health-and-rights-srhr-world-health-organization-opg-26-00176</t>
+          <t>https://onepurpos.in/openings/rfps/rfp-design-and-delivery-of-an-electric-vehicle-ev-skilling-programme-in-karnataka-wri-india-rfp-26-00361</t>
         </is>
       </c>
     </row>
@@ -1277,140 +1314,10 @@
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
-          <t>Applications Invited for Setting up Viral Research and Diagnosis Laboratories VRDL in Medical Colleges/Hospitals/Medical Institutions</t>
+          <t>Applications Open Draper Richards Kaplan Foundation Funding for Social Enterprises</t>
         </is>
       </c>
       <c r="C13" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-The President notified the creation of the Department of Health Research under the Ministry of Health &amp; Family Welfare through an amendment to the Government of India (Allocation of Business) Rules, 1961 on the 17th September 2007. The Department of Health Research was formally launched on 5th October 2007 by the Minister for Science &amp; Technology and Earth Sciences in a function presided over by the Minister for Health &amp; Family Welfare, in the presence, inter-alia, of the Minister of State for Health &amp; Family Welfare.
-The Department became functional from November 2008 with the appointment of first Secretary of the Department The aim of the DHR is to bring modern health technologies to the people through research and innovations related to diagnosis, treatment methods and vaccines for prevention, to translate them into products and processes and, in synergy with concerned organizations, introduce these innovations into public health system.
- About the Opportunity:
-Under DHR's scheme "Setting-up of nation-wide network of laboratories for managing epidemics and national calamities," proposals are invited from Medical Colleges/Hospitals/Research Institutions to establish a Medical College &amp; Research Institute Level – Viral Research and Diagnosis Laboratory (MCL-VRDL). The existing network comprises 167 VRDLs (11 Regional, 27 State, 129 Medical College level) across 27 states and 5 UTs, aimed at early detection of infectious pathogens, outbreak surveillance, and research on emerging/re-emerging viral diseases.
- Objectives:
-Establish capacity for early detection of common and high-risk infectious pathogens
-Strengthen syndromic surveillance ecosystem for outbreak detection
-Undertake R&amp;D on emerging, re-emerging and novel viruses
- Eligibility (Institution-level):
-State Government Medical Colleges
-Central Government Medical Colleges and Research Institutes
-Armed Forces Medical Institutions/Hospitals
-Railway and other Central Government health institutions
-Private medical colleges ranked in top 50 NIRF ranking
-Must have a dedicated Microbiology department with qualified faculty
-Must have &gt;200 sq.m. area available in existing building (preferably within Microbiology Dept.)
- Funding Provision:
-Non-recurring assistance: Rs. 1.55 crore total
-Rs. 66.8 lakhs — Civil Work (infrastructure modification)
-Rs. 88.2 lakhs — Equipment (complete lab setup)
-No recurring expenditure (staff salaries, consumables, contingency) is provided — to be borne by the host institution
- Role &amp; Responsibilities of the Lab:
-Conduct routine diagnosis of infectious pathogens
-Participate in syndromic and event-based surveillance
-Provide support during outbreaks/epidemics
-Share data with ICMR
- Selection Criteria:
-Meeting eligibility does not guarantee selection; merit-based evaluation by a technical committee
-Preference to institutions in geographically underserved regions
-Weightage for technical strength (qualified faculty, biosafety practices, outbreak investigation experience, publications, patents, externally funded projects)
-Additional weightage for molecular diagnostics, genomic surveillance, One Health research capability, and commitment to long-term recurring support
-Private medical colleges: only top-50 NIRF-ranked institutions considered</t>
-        </is>
-      </c>
-      <c r="D13" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E13" s="1" t="inlineStr">
-        <is>
-          <t>Sep 30, 2026</t>
-        </is>
-      </c>
-      <c r="F13" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-setting-up-viral-research-and-diagnosis-laboratories-vrdl-in-medical-collegeshospitalsmedical-institutions-department-of-health-research-dhr-ministry-of-health-and-family-welfare-government-of-india-opg-26-00174</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="95" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="inlineStr">
-        <is>
-          <t>Application Invited for Giving Joy Microgrant</t>
-        </is>
-      </c>
-      <c r="C14" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-Giving Joy is a US-based nonprofit that strengthens and inspires women’s entrepreneurship worldwide. Through its micro-grants and mentorship program, Giving Joy helps women establish or improve their businesses and initiatives—for their benefit and the benefit of their communities. To date, Giving Joy has awarded over 88 grants to women-led initiatives in 26 countries.
- 2026 Grant Cycle
-Beginning in 2026, Giving Joy has moved to two global grant cycles per year.
-The organization states that this change was made after operating multiple regional rounds, with the aim of:
-Providing clearer timelines for applicants
-Increasing the quality and depth of application reviews
-Reducing administrative burden
-Improving support for grantees
-Focusing communications and fundraising more effectively
-Continuing to reach women entrepreneurs globally without dividing applications by geography
-Each cycle is open to women entrepreneurs worldwide.
- Eligible Fields / Activities
-There is no restriction to a particular field such as health.
-Applicants can propose activities in:
-Any field
-Trade
-Occupation
-Craft
- What Does Giving Joy Look For?
-Giving Joy prioritizes:
-Innovative ideas
-Creative ideas
-Strong potential for social impact
-Initiative
-Real community impact
-Clear economic and/or social benefits for women and girls
- Grant Amount
-Maximum Grant
-Up to $500 USD
-The exact award amount is determined by Giving Joy based on:
-Proposed activities
-Availability of funding
- Grant Duration
-The grant period is six months.</t>
-        </is>
-      </c>
-      <c r="D14" s="1" t="inlineStr">
-        <is>
-          <t>Safety</t>
-        </is>
-      </c>
-      <c r="E14" s="1" t="inlineStr">
-        <is>
-          <t>Sep 30, 2026</t>
-        </is>
-      </c>
-      <c r="F14" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/application-invited-for-giving-joy-microgrant-giving-joy-opg-26-00185</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="95" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="inlineStr">
-        <is>
-          <t>Applications Open Draper Richards Kaplan Foundation Funding for Social Enterprises</t>
-        </is>
-      </c>
-      <c r="C15" s="1" t="inlineStr">
         <is>
           <t>About us
 Started in 2002, Draper Richards Kaplan Foundation (DRK) is a global venture philanthropy firm supporting early stage, high impact social enterprises. Borrowed from our venture capital legacy, DRK finds, funds, and supports exceptional leaders building innovative solutions to some of the world’s most challenging social and environmental problems. Since beginning this work nearly 25 years ago, DRK has invested in more than 270 organizations that have collectively impacted over 610 million lives to date.
@@ -1434,34 +1341,34 @@
 Please attach a standard resume/CV for the entrepreneur(s) and/or key leadership team members (e.g., CEO, COO, ED, etc.). Applications with text bios for entrepreneurs or members of the leadership team will not be considered.</t>
         </is>
       </c>
-      <c r="D15" s="1" t="inlineStr">
+      <c r="D13" s="1" t="inlineStr">
         <is>
           <t>Climate</t>
         </is>
       </c>
-      <c r="E15" s="1" t="inlineStr">
+      <c r="E13" s="1" t="inlineStr">
         <is>
           <t>Oct 10, 2026</t>
         </is>
       </c>
-      <c r="F15" s="1" t="inlineStr">
+      <c r="F13" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-open-draper-richards-kaplan-foundation-funding-for-social-enterprises-draper-richards-kaplan-foundation-opg-26-00188</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="95" customHeight="1">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B16" s="1" t="inlineStr">
+    <row r="14" ht="95" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund</t>
         </is>
       </c>
-      <c r="C16" s="1" t="inlineStr">
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund
 Apply by: 13 October, 2026
@@ -1486,34 +1393,34 @@
  Projects should include opportunities for ServiceNow employees to volunteer in the project activation or implementation.</t>
         </is>
       </c>
-      <c r="D16" s="1" t="inlineStr">
+      <c r="D14" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E16" s="1" t="inlineStr">
+      <c r="E14" s="1" t="inlineStr">
         <is>
           <t>Oct 13, 2026</t>
         </is>
       </c>
-      <c r="F16" s="1" t="inlineStr">
+      <c r="F14" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/apply-for-the-servicenow-community-solar-fund-changex-opg-26-00186</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="95" customHeight="1">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B17" s="1" t="inlineStr">
+    <row r="15" ht="95" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>ToR - Engagement of Consultant/Vendor Individual towards implementation of Literacy Program in Telangana State</t>
         </is>
       </c>
-      <c r="C17" s="1" t="inlineStr">
+      <c r="C15" s="1" t="inlineStr">
         <is>
           <t>ANNEX A – TERMS OF REFERENCE (ToR) 
  Engagement of Consultant/Vendor (Individual) towards implementation of Literacy Program in Telangana State.
@@ -1578,34 +1485,34 @@
 Approved travel and accommodation expenses incurred for assignment-related activities shall be reimbursed by Room to Read in accordance with the consultancy reimbursement guidelines.</t>
         </is>
       </c>
-      <c r="D17" s="1" t="inlineStr">
+      <c r="D15" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E17" s="1" t="inlineStr">
+      <c r="E15" s="1" t="inlineStr">
         <is>
           <t>Oct 16, 2026</t>
         </is>
       </c>
-      <c r="F17" s="1" t="inlineStr">
+      <c r="F15" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-engagement-of-consultantvendor-individual-towards-implementation-of-literacy-program-in-telangana-state-room-to-read-india-rfp-26-00360</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="95" customHeight="1">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="inlineStr">
+    <row r="16" ht="95" customHeight="1">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>RFPs Invited for Consultant to Develop a Technical Assistance Package for National Application of the Digital Health and AI Investment Classification Framework</t>
         </is>
       </c>
-      <c r="C18" s="1" t="inlineStr">
+      <c r="C16" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are Transform Health: a global coalition of more than 200 organisations driving the digital transformation of health to achieve universal health coverage. 
@@ -1633,59 +1540,57 @@
 Ability to manage multi-country consultancy engagements and coordinate with in-country focal points</t>
         </is>
       </c>
-      <c r="D18" s="1" t="inlineStr">
+      <c r="D16" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E18" s="1" t="inlineStr">
+      <c r="E16" s="1" t="inlineStr">
         <is>
           <t>Oct 23, 2026</t>
         </is>
       </c>
-      <c r="F18" s="1" t="inlineStr">
+      <c r="F16" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfps-invited-for-consultant-to-develop-a-technical-assistance-package-for-national-application-of-the-digital-health-and-ai-investment-classification-framework-transform-health-rfp-26-00359</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="95" customHeight="1">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Crossing the Divide Best Practices for Addressing Local and Privately-Owned Lateral Sewer Issues RFP 5419</t>
-        </is>
-      </c>
-      <c r="C19" s="1" t="inlineStr">
-        <is>
-          <t>Project Objective:
-To provide water resource recovery facilities (WRRFs) and collection system operators with an interactive manual of practice for implementing inflow and infiltration (I&amp;I) and obstruction management programs, focused on municipal and privately owned lateral sewers in complex legal, regulatory, and multi-jurisdictional environments.
+    <row r="17" ht="95" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Comparison of PFAS Contributions to Agricultural Systems</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>Project Objectives:
+Report per- and polyfluoroalkyl substance (PFAS) concentrations from a variety of agricultural inputs — animal manures, fertilizers, pesticides, composts, soil amendments, seed coatings, and biosolids-based products
+Compare the impact of various agricultural inputs on PFAS concentration in the soil profile over varying timeframes
+Evaluate the fate and transport of different inputs to PFAS contributions in agricultural systems at field-scale
+Determine relative contributions from biosolids-based products vs. other inputs to help develop/prioritize risk management strategies
  Background/Rationale:
-Wastewater utilities face continuing challenges providing cost-effective sewer services amid rising demand, urban redevelopment, and performance disruptors (root intrusion, pipe degradation, blockages). I&amp;I and obstruction management remain persistent, costly problems without a consolidated resource to guide program design. During wet weather, peak I&amp;I flows can increase influent flows 3–5x average. Studies suggest up to 80% of I&amp;I originates on private property, and root intrusions cause over 50% of sewer blockages globally. Program effectiveness varies widely depending on statutory authority, multi-jurisdictional overlap, enforcement mechanisms, and participant willingness.
- Central Research Questions:
-What I&amp;I and obstruction management practices are utilities using today, and how do they vary by jurisdictional/regulatory/infrastructure/environmental conditions?
-Which factors most influence successful implementation, and what barriers commonly derail programs?
-What measurable benefits (cost avoidance, capacity recovery, reduced spill risk, improved regulatory standing) have utilities realized from successful programs?
-This project extends WRF's ongoing "State-of-Practice Manual for Inflow and Infiltration Detection and Mitigation at Street and Private Lateral Levels" (Project 5365) into I&amp;I source control and obstruction management specifically.
- Research Approach (4 Tasks):
-Literature and Regulatory Review — Comprehensive review of legal authorities/regulations in the US and comparable international jurisdictions; catalog program elements, enforcement mechanisms, incentive structures, and legal/jurisdictional barriers
-Utility Survey and Case Study Development — Broad survey across utility size/geography/system type; select at least 5 diverse in-depth case studies with quantitative results (I&amp;I reduction %, reduced bypass pumping, reduced basement backups, cost savings, recovered capacity, reduced blockage-related spills/service calls)
-Utility Workshop — At least one invitation-only workshop with utility representatives to present survey findings and gather structured feedback on draft guidance content
-Interactive Manual of Practice — Development of a decision-support tool/web-based application/interactive PDF enabling utilities to select effective I&amp;I/obstruction program elements based on their statutory authority, jurisdictional complexity, and enforcement mechanisms
+Growing concern exists over human exposure to PFAS through biosolids land application on agricultural systems, with regulatory bans on biosolids land application enacted or proposed in at least 12 U.S. states. Utilities relying on land application for biosolids management are scrambling for alternative disposal pathways. The U.S. EPA's 2026 draft guidance noted its earlier 2025 draft risk assessment of PFOA/PFOS-contaminated sewage sludge lacked important contextual information (e.g., a national survey of PFOA/PFOS concentrations). Risk assessments have focused primarily on biosolids, with less attention to PFAS contributions from other sources — manures, compost, fertilizers, pesticides, seed coatings, irrigation water, farming practices, and atmospheric deposition. A Minnesota Pollution Control Agency review found 12 inert pesticide ingredients classified as PFAS. This project aims to improve understanding of PFAS risks from the wider range of agricultural inputs to support strategic resource allocation and inform policy amid surging fertilizer prices and shifts toward local circular resources.
+ Research Approach:
+Develop a baseline of knowledge on PFAS in biosolids and non-biosolids agricultural inputs via literature review, analytical methods evaluation, and examination of manufacturing/processing pathways; identify data gaps and uncertainties
+Measure/report compound-specific PFAS concentrations and profiles in agricultural inputs using standardized methods, including precursor characteristics for source attribution where possible
+Characterize PFAS contributions via literature review, data analysis, and field sampling — comparing soil profile/plant tissue composition between fields with non-biosolids inputs vs. biosolids-applied systems; study should test hypotheses on PFAS sources, transformation, retention, and mobility
+Optional additional focus areas: influence of soil/hydrologic/hydrochemistry conditions on PFAS behavior; degradation/transformation pathways; relative PFAS contributions across product lifecycle stages (manufacturing, bagging, delivery, etc.)
+Research approach should be hypothesis-driven, detailing specific end-user needs, and proposers are encouraged to leverage existing projects on PFAS plant uptake/fate/transport.
  Expected Deliverables:
-Research report (using WRF's Research Report Template) including literature/regulatory review
-Interactive manual of practice (following Technology Deliverables Guidance)
-In-depth utility survey, state-of-the-practice report, and at least 5 standalone case studies with quantitative results
-Summary documentation of the utility workshop, including feedback and how it was incorporated
- Project Duration: 24 months from contract start date (No-Cost Extension Policy caps extensions at 9 months beyond original schedule)
+Research report (WRF's Research Report Template) including: literature review, PFAS analysis of select products, risk management implications/prioritization recommendations, agriculture end-use guidance
+A webcast or workshop to share findings
+Optional additional deliverables: relative risk framework (mass input/fate/exposure/risk), decision support guide for farmers/regulators/utilities, plain language fact sheet, comparative PFAS mass input tool (spreadsheet/calculator)
+ Project Duration: 36 months from contract start date (longer than the other two WRF grants above, which were 24 months)
  Eligibility to Submit:
-Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible as named participants. Not open to individuals (same institutional-applicant structure as RFP 5424).
+Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible. Not open to individuals (same structure as the two prior WRF grants).
  Budget/Funding:
-Maximum WRF funding: $250,000
+Maximum WRF funding: $400,000 (the largest of the three WRF grants shared so far)
 Applicant must contribute at least 33% of the project award as additional resources (cost share, applicant in-kind, or third-party in-kind per 2 CFR Part 200.306)
 Proposals not meeting the 33% minimum match will not be accepted
  Proposal Evaluation Criteria:
@@ -1695,37 +1600,37 @@
 Communication Plan, Deliverables, and Applicability: 15 points
 Budget and Schedule: 15 points
  Compliance Standards: OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
- Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
-        </is>
-      </c>
-      <c r="D19" s="1" t="inlineStr">
+ Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00) — same deadline as the other two WRF grants</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E19" s="1" t="inlineStr">
+      <c r="E17" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F19" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-crossing-the-divide-best-practices-for-addressing-local-and-privately-owned-lateral-sewer-issues-rfp-5419-the-water-research-foundation-wrf-opg-26-00189</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="95" customHeight="1">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="inlineStr">
+      <c r="F17" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-comparison-of-pfas-contributions-to-agricultural-systems-the-water-research-foundation-wrf-opg-26-00190</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="95" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Adaptive Control Frameworks to Unlock Full-Scale BNR Potential Water Research Foundation WRF</t>
         </is>
       </c>
-      <c r="C20" s="1" t="inlineStr">
+      <c r="C18" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Water Research Foundation (WRF) is the leading research organization advancing the science of all water to meet the evolving needs of its subscribers and the water sector. WRF is a nonprofit, charitable and educational organization which funds, manages, and publishes research on the technology, operation, and management of drinking water, wastewater, reuse, and stormwater collection, treatment and supply systems—all in pursuit of ensuring water quality and improving water services to the public.
@@ -1766,147 +1671,59 @@
 Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
         </is>
       </c>
-      <c r="D20" s="1" t="inlineStr">
+      <c r="D18" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E20" s="1" t="inlineStr">
+      <c r="E18" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F20" s="1" t="inlineStr">
+      <c r="F18" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-adaptive-control-frameworks-to-unlock-full-scale-bnr-potential-water-research-foundation-wrf-the-water-research-foundation-wrf-opg-26-00187</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="95" customHeight="1">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for 8th Call for Proposals Small-Size Grants Global EbA Fund</t>
-        </is>
-      </c>
-      <c r="C21" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
- About the Opportunity:
-The Global EbA Fund invites innovative and catalytic proposals that address systemic barriers to Ecosystem-based Adaptation (EbA) scaling — by enhancing institutional and technical capacities, quality data/evidence generation, learning networks, and investment readiness. Aligned with the IKI Strategy up to 2030 (focus on socio-ecological transformation), the Fund's primary geographic focus is ODA-eligible SIDS (Small Island Developing States) and LDCs (Least Developed Countries), though other ODA-eligible countries may be considered where proposals show exceptional ambition.
- Focus Areas:
-Overcoming upstream barriers to EbA uptake/scaling (institutional &amp; technical capacity constraints, evidence generation, knowledge exchange)
-Clear adaptation chain grounded in detailed impact chain analysis (climate hazards/risks, socioeconomic/ecological sensitivity, adaptive capacity)
-Social and environmental considerations (gender responsiveness, Indigenous Peoples' rights, local participation, environmental/social safeguards, prevention of maladaptation)
-Robust sustainability and exit strategies (long-term viability, local ownership, institutional continuity)
- Encouraged Topics:
-Investment readiness and project pipeline preparation
-Innovative technologies for EbA
-Applied and functional research
-Synergies with other EbA/Nature-based Solution (NbS) initiatives
- Grant Size: Up to USD 250,000 per grant
- Project Duration: Up to 24 months
- Eligible Applicant Types:
-Non-governmental organisations (NGOs)
-International NGOs (INGOs)
-Intergovernmental organisations (IGOs)
-Community-based organisations (CBOs)
-Indigenous People's Organisations
-Universities and academic institutions
-Research institutes and think tanks
-Private sector companies (under certain conditions; no funding for sector-specific obligations, compensatory measures, or for-profit activities)
-Consortia (must designate a clear lead "Applicant Organisation"; government entities can join a consortium but cannot receive Fund money directly)
-Note: Individuals are not eligible (e.g., no PhD study funding); UNEP and IUCN offices are also not eligible to apply.
- Key Eligibility Criteria:
-Must qualify as Ecosystem-based Adaptation (EbA) per the Fund's Qualification Criteria &amp; Quality Standards
-Must have catalytic/innovative potential
-Must clearly identify climate impacts addressed
-Falls under max 1 Strategic Objective and max 2 Action Pillars of the Fund
-Global, thematic, or targets only ODA-eligible countries
-Budget up to USD 250,000; duration up to 24 months
-Must build on existing work (not standalone/field-implementation-only projects)
-Must show sustainability post-funding
-Must partner with local institutions
-Applicant &amp; partners must be legally recognized entities with relevant experience
-Must complete Due Diligence requirements
- Evaluation Criteria (weighted):
-Ecosystem-based Adaptation (EbA) approach — 30%
-Design &amp; Methodology (Theory of Change, logframe, SMART indicators, budget coherence)
-Gender &amp; Social Inclusion (participatory approach, FPIC for Indigenous Peoples' impact)
-Innovative &amp; Catalytic Contribution — 30%
-Sustainability — 20%
-Institutional Arrangements — 20%
- Reporting Requirement: Applicants must identify at least 3 indicators from the Fund's Core Indicator Framework for their project's logframe.
- Application Package Required:
-Applicant Declaration
-Co-applicant Mandate (if applicable)
-Small-Size Grants Application Form
-Project Proposal Budget Template
-Due Diligence and Financial Capacity Questionnaire (with Annexes 1(c)(i) and 1(c)(ii) at submission stage)
- Application Language: English only (organizational documents must be translated to English
- Timeline:
-Call officially launched: August 24, 2026
-Submission window: September 28 – October 26, 2026
-Applications submitted via online portal (link shared on the Small-Size Grants webpage from Sept 28)
-Only successful applicants will be contacted; no individual feedback provided to unsuccessful applicants</t>
-        </is>
-      </c>
-      <c r="D21" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E21" s="1" t="inlineStr">
-        <is>
-          <t>Oct 26, 2026</t>
-        </is>
-      </c>
-      <c r="F21" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-8th-call-for-proposals-small-size-grants-global-eba-fund-global-eba-fund-opg-26-00177</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="95" customHeight="1">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Comparison of PFAS Contributions to Agricultural Systems</t>
-        </is>
-      </c>
-      <c r="C22" s="1" t="inlineStr">
-        <is>
-          <t>Project Objectives:
-Report per- and polyfluoroalkyl substance (PFAS) concentrations from a variety of agricultural inputs — animal manures, fertilizers, pesticides, composts, soil amendments, seed coatings, and biosolids-based products
-Compare the impact of various agricultural inputs on PFAS concentration in the soil profile over varying timeframes
-Evaluate the fate and transport of different inputs to PFAS contributions in agricultural systems at field-scale
-Determine relative contributions from biosolids-based products vs. other inputs to help develop/prioritize risk management strategies
+    <row r="19" ht="95" customHeight="1">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Crossing the Divide Best Practices for Addressing Local and Privately-Owned Lateral Sewer Issues RFP 5419</t>
+        </is>
+      </c>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>Project Objective:
+To provide water resource recovery facilities (WRRFs) and collection system operators with an interactive manual of practice for implementing inflow and infiltration (I&amp;I) and obstruction management programs, focused on municipal and privately owned lateral sewers in complex legal, regulatory, and multi-jurisdictional environments.
  Background/Rationale:
-Growing concern exists over human exposure to PFAS through biosolids land application on agricultural systems, with regulatory bans on biosolids land application enacted or proposed in at least 12 U.S. states. Utilities relying on land application for biosolids management are scrambling for alternative disposal pathways. The U.S. EPA's 2026 draft guidance noted its earlier 2025 draft risk assessment of PFOA/PFOS-contaminated sewage sludge lacked important contextual information (e.g., a national survey of PFOA/PFOS concentrations). Risk assessments have focused primarily on biosolids, with less attention to PFAS contributions from other sources — manures, compost, fertilizers, pesticides, seed coatings, irrigation water, farming practices, and atmospheric deposition. A Minnesota Pollution Control Agency review found 12 inert pesticide ingredients classified as PFAS. This project aims to improve understanding of PFAS risks from the wider range of agricultural inputs to support strategic resource allocation and inform policy amid surging fertilizer prices and shifts toward local circular resources.
- Research Approach:
-Develop a baseline of knowledge on PFAS in biosolids and non-biosolids agricultural inputs via literature review, analytical methods evaluation, and examination of manufacturing/processing pathways; identify data gaps and uncertainties
-Measure/report compound-specific PFAS concentrations and profiles in agricultural inputs using standardized methods, including precursor characteristics for source attribution where possible
-Characterize PFAS contributions via literature review, data analysis, and field sampling — comparing soil profile/plant tissue composition between fields with non-biosolids inputs vs. biosolids-applied systems; study should test hypotheses on PFAS sources, transformation, retention, and mobility
-Optional additional focus areas: influence of soil/hydrologic/hydrochemistry conditions on PFAS behavior; degradation/transformation pathways; relative PFAS contributions across product lifecycle stages (manufacturing, bagging, delivery, etc.)
-Research approach should be hypothesis-driven, detailing specific end-user needs, and proposers are encouraged to leverage existing projects on PFAS plant uptake/fate/transport.
+Wastewater utilities face continuing challenges providing cost-effective sewer services amid rising demand, urban redevelopment, and performance disruptors (root intrusion, pipe degradation, blockages). I&amp;I and obstruction management remain persistent, costly problems without a consolidated resource to guide program design. During wet weather, peak I&amp;I flows can increase influent flows 3–5x average. Studies suggest up to 80% of I&amp;I originates on private property, and root intrusions cause over 50% of sewer blockages globally. Program effectiveness varies widely depending on statutory authority, multi-jurisdictional overlap, enforcement mechanisms, and participant willingness.
+ Central Research Questions:
+What I&amp;I and obstruction management practices are utilities using today, and how do they vary by jurisdictional/regulatory/infrastructure/environmental conditions?
+Which factors most influence successful implementation, and what barriers commonly derail programs?
+What measurable benefits (cost avoidance, capacity recovery, reduced spill risk, improved regulatory standing) have utilities realized from successful programs?
+This project extends WRF's ongoing "State-of-Practice Manual for Inflow and Infiltration Detection and Mitigation at Street and Private Lateral Levels" (Project 5365) into I&amp;I source control and obstruction management specifically.
+ Research Approach (4 Tasks):
+Literature and Regulatory Review — Comprehensive review of legal authorities/regulations in the US and comparable international jurisdictions; catalog program elements, enforcement mechanisms, incentive structures, and legal/jurisdictional barriers
+Utility Survey and Case Study Development — Broad survey across utility size/geography/system type; select at least 5 diverse in-depth case studies with quantitative results (I&amp;I reduction %, reduced bypass pumping, reduced basement backups, cost savings, recovered capacity, reduced blockage-related spills/service calls)
+Utility Workshop — At least one invitation-only workshop with utility representatives to present survey findings and gather structured feedback on draft guidance content
+Interactive Manual of Practice — Development of a decision-support tool/web-based application/interactive PDF enabling utilities to select effective I&amp;I/obstruction program elements based on their statutory authority, jurisdictional complexity, and enforcement mechanisms
  Expected Deliverables:
-Research report (WRF's Research Report Template) including: literature review, PFAS analysis of select products, risk management implications/prioritization recommendations, agriculture end-use guidance
-A webcast or workshop to share findings
-Optional additional deliverables: relative risk framework (mass input/fate/exposure/risk), decision support guide for farmers/regulators/utilities, plain language fact sheet, comparative PFAS mass input tool (spreadsheet/calculator)
- Project Duration: 36 months from contract start date (longer than the other two WRF grants above, which were 24 months)
+Research report (using WRF's Research Report Template) including literature/regulatory review
+Interactive manual of practice (following Technology Deliverables Guidance)
+In-depth utility survey, state-of-the-practice report, and at least 5 standalone case studies with quantitative results
+Summary documentation of the utility workshop, including feedback and how it was incorporated
+ Project Duration: 24 months from contract start date (No-Cost Extension Policy caps extensions at 9 months beyond original schedule)
  Eligibility to Submit:
-Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible. Not open to individuals (same structure as the two prior WRF grants).
+Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible as named participants. Not open to individuals (same institutional-applicant structure as RFP 5424).
  Budget/Funding:
-Maximum WRF funding: $400,000 (the largest of the three WRF grants shared so far)
+Maximum WRF funding: $250,000
 Applicant must contribute at least 33% of the project award as additional resources (cost share, applicant in-kind, or third-party in-kind per 2 CFR Part 200.306)
 Proposals not meeting the 33% minimum match will not be accepted
  Proposal Evaluation Criteria:
@@ -1916,77 +1733,37 @@
 Communication Plan, Deliverables, and Applicability: 15 points
 Budget and Schedule: 15 points
  Compliance Standards: OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
- Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00) — same deadline as the other two WRF grants</t>
-        </is>
-      </c>
-      <c r="D22" s="1" t="inlineStr">
+ Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
+        </is>
+      </c>
+      <c r="D19" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E22" s="1" t="inlineStr">
+      <c r="E19" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F22" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-comparison-of-pfas-contributions-to-agricultural-systems-the-water-research-foundation-wrf-opg-26-00190</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="95" customHeight="1">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B23" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Whitley Award 2027</t>
-        </is>
-      </c>
-      <c r="C23" s="1" t="inlineStr">
-        <is>
-          <t>About the Grant: 
-An annual grant by the Whitley Fund for Nature (WFN) recognising grassroots conservation leaders in the Global South, providing funding to support and scale up proven, science-based solutions that deliver lasting impact for both people and nature.
- About the Award 
-Whitley Awards support grassroots conservation leaders in the Global South. Through funding, training and profile, they help conservationists scale up effective projects that are founded in science and carried out with communities. Whitley Awards are for dynamic, mid-career conservationists who are leading vital conservation projects.
- Grant Amount: £50,000 in project funding over one year
- Eligibility
-Winners are nationals of the country in which they are working, seeking to scale up proven work that is embedded in the local community and would benefit from further funding, a profile boost, and international support.
-Projects must involve communities at the grassroots level and deliver practical action that is founded on science.
-You do not need to be invited or nominated to apply.</t>
-        </is>
-      </c>
-      <c r="D23" s="1" t="inlineStr">
-        <is>
-          <t>Learning</t>
-        </is>
-      </c>
-      <c r="E23" s="1" t="inlineStr">
-        <is>
-          <t>Oct 30, 2026</t>
-        </is>
-      </c>
-      <c r="F23" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-whitley-award-2027-whitley-fund-for-nature-wfn-opg-26-00153</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="95" customHeight="1">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B24" s="1" t="inlineStr">
+      <c r="F19" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-crossing-the-divide-best-practices-for-addressing-local-and-privately-owned-lateral-sewer-issues-rfp-5419-the-water-research-foundation-wrf-opg-26-00189</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="95" customHeight="1">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIFAR Global Scholars Program 20272029 Cohort</t>
         </is>
       </c>
-      <c r="C24" s="1" t="inlineStr">
+      <c r="C20" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 CIFAR is a Canadian-based globally influential research organization that convenes the world’s most brilliant people across disciplines to advance transformative knowledge and solve humanity’s biggest problems, together. By supporting long-term interdisciplinary collaboration, CIFAR provides researchers with an unparalleled environment of trust, transparency and knowledge sharing. Our time-tested model inspires new directions of inquiry, accelerates discovery and yields breakthroughs across borders and academic disciplines. Through knowledge mobilization, we are catalysts for change in industry, government and society. Through our 15 research programs and the Pan-Canadian AI Strategy, CIFAR convenes close to 400 of the world’s top researchers from 141 institutions in 20 countries. CIFAR is generously supported by the governments of Canada, Alberta and Québec, as well as foundations, individuals, corporations and Canadian and international partner organizations.
@@ -2030,115 +1807,34 @@
  Application Deadline: November 4, 2026, 12:00 PM EST</t>
         </is>
       </c>
-      <c r="D24" s="1" t="inlineStr">
+      <c r="D20" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E24" s="1" t="inlineStr">
+      <c r="E20" s="1" t="inlineStr">
         <is>
           <t>Nov 4, 2026</t>
         </is>
       </c>
-      <c r="F24" s="1" t="inlineStr">
+      <c r="F20" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cifar-global-scholars-program-20272029-cohort-cifar-canadian-institute-for-advanced-research-opg-26-00183</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="95" customHeight="1">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B25" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for IWRS Teaching Innovation Award</t>
-        </is>
-      </c>
-      <c r="C25" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-Insects are one of the most numerous and diverse animal groups on Earth.
-Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice.
-About the Award
-The IWRS Teaching Innovation Award supports instructors developing new approaches to teaching invertebrate biology that incorporate the 3Rs (replacement, reduction, and refinement). It also supports the development and implementation of any novel curricula addressing invertebrate welfare and sentience across invertebrate biology, animal welfare science, and/or veterinary medicine fields.
-Grant size
-Awards up to $2,000 USD are available for approaches requiring equipment or other materials; awards up to $1,000 USD are available otherwise. Funds may be used to support any costs associated with curriculum development and implementation, including stipends, teaching tools, and related expenses. Priority is given to proposals addressing common teaching practices with substantial welfare implications.
-Who can apply for funding?
-The applicant must be an instructor teaching content related to insect or invertebrate biology at an educational institution, scientific society or museum, field-training course, or similar educational context. If you are unsure about your eligibility, contact grants@insectwelfare.com.
-The applicant can be from any discipline, country, or institution. However, we will not pay awards to recipients located in jurisdictions, countries, or regions subject to trade restrictions, embargoes, or sanctions put in place by the United Nations or the United States of America.
-IWRS staff and Advisory Group members are not eligible to apply.</t>
-        </is>
-      </c>
-      <c r="D25" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E25" s="1" t="inlineStr">
-        <is>
-          <t>Nov 15, 2026</t>
-        </is>
-      </c>
-      <c r="F25" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00166</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="95" customHeight="1">
-      <c r="A26" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B26" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for IWRS Teaching Innovation Award</t>
-        </is>
-      </c>
-      <c r="C26" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
- About the Grant
-The IWRS (Insect Welfare Research Society) Teaching Innovation Award supports instructors developing new approaches to teaching insect or invertebrate biology that incorporate the 3Rs (Replacement, Reduction, and Refinement) — principles for reducing animal welfare impacts in teaching and research practices.
- Purpose
-Funds support the creation and implementation of 3Rs-driven instructional materials and pedagogical approaches. Priority is given to proposals addressing common teaching practices with substantial welfare implications.
- Grant Amount
-Two awards of $2,000 USD are available annually.</t>
-        </is>
-      </c>
-      <c r="D26" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E26" s="1" t="inlineStr">
-        <is>
-          <t>Nov 15, 2026</t>
-        </is>
-      </c>
-      <c r="F26" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="95" customHeight="1">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B27" s="1" t="inlineStr">
+    <row r="21" ht="95" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Medium-Size Grants Call for Proposals Global EbA Fund</t>
         </is>
       </c>
-      <c r="C27" s="1" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -2195,88 +1891,34 @@
 Applications submitted via online portal (link shared on the Medium-Size Grants webpage from Oct 12)</t>
         </is>
       </c>
-      <c r="D27" s="1" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E27" s="1" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>Nov 16, 2026</t>
         </is>
       </c>
-      <c r="F27" s="1" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-medium-size-grants-call-for-proposals-global-eba-fund-global-eba-fund-opg-26-00178</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="95" customHeight="1">
-      <c r="A28" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B28" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for CIEIF Grant 2026 Climate Intervention Environmental Impact Fund</t>
-        </is>
-      </c>
-      <c r="C28" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-Climate Intervention Environmental Impact Fund (CIEIF) is a philanthropic fund focused on supporting responsible climate intervention field tests. It provides grants for activities such as environmental impact assessment (EIA), predictive impact modelling, and engagement with potentially affected stakeholders, including local communities and government agencies.
-CIEIF aims to help climate-intervention projects better understand their potential technical, environmental, economic, social, public-health, and safety impacts before and during field testing. It also places importance on the scalability and global relevance of supported innovations and encourages publication of field-test results through peer-reviewed journals or externally peer-reviewed reports.
- About the Grant
-The Climate Intervention Environmental Impact Fund (CIEIF) Grant provides USD 75,000 to support proposed climate intervention field tests. The funding is specifically intended for Environmental Impact Assessment (EIA), predictive impact modelling, and/or engagement with potentially affected stakeholders, including local communities and government agencies.
-Applicants are expected to demonstrate the proposed field test’s technical readiness, environmental and social considerations, required government approvals, innovation and potential for globally relevant scalability. The application must include a proposed budget showing how the USD 75,000 will be used.
- Grant Objective
-The grant is intended to support proposed climate intervention field tests, particularly activities related to:
-Environmental Impact Assessment (EIA)
-Predictive impact modeling
-Engagement with potentially impacted stakeholders
-Local community and government engagement
-Understanding technical, environmental, economic, social, public-health, and safety challenges
-The proposed application must focus on at least one of these three core areas: EIA, predictive impact modeling, or stakeholder engagement.
- Eligible Project Focus
-The proposed field test should demonstrate:
-A clear climate-intervention concept
-Prior research indicating that the technology is ready for the proposed field test
-Potential for innovation and scalability
-A clear understanding of technical and environmental challenges
-Consideration of economic, social, public-health, and safety implications
-Relevant government permits and approvals
-Potential for scaling the innovation to a globally relevant level</t>
-        </is>
-      </c>
-      <c r="D28" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E28" s="1" t="inlineStr">
-        <is>
-          <t>Dec 1, 2026</t>
-        </is>
-      </c>
-      <c r="F28" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-cieif-grant-2026-climate-intervention-environmental-impact-fund-climate-intervention-environmental-impact-fund-opg-26-00155</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="95" customHeight="1">
-      <c r="A29" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B29" s="1" t="inlineStr">
+    <row r="22" ht="95" customHeight="1">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 6th Annual Seeding The Future Global Food System Challenge</t>
         </is>
       </c>
-      <c r="C29" s="1" t="inlineStr">
+      <c r="C22" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are one of the largest and most respected private organisations for development cooperation and humanitarian aid in Germany. As a politically and confessionally independent organisation, our value-oriented actions are always based on ethical principles. Our vision is clear: "Zero Hunger by 2030"
@@ -2308,34 +1950,34 @@
 Individuals with no organizational entity</t>
         </is>
       </c>
-      <c r="D29" s="1" t="inlineStr">
+      <c r="D22" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E29" s="1" t="inlineStr">
+      <c r="E22" s="1" t="inlineStr">
         <is>
           <t>Jan 1, 2027</t>
         </is>
       </c>
-      <c r="F29" s="1" t="inlineStr">
+      <c r="F22" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-6th-annual-seeding-the-future-global-food-system-challenge-welthungerhilfe-opg-26-00180</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="95" customHeight="1">
-      <c r="A30" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B30" s="1" t="inlineStr">
+    <row r="23" ht="95" customHeight="1">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for BES Training and Travel Grants</t>
         </is>
       </c>
-      <c r="C30" s="1" t="inlineStr">
+      <c r="C23" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are a global community of scientists shining a spotlight on the intricacy and value of our natural world, providing the evidence for better decisions. Our vision is for people and nature to thrive in a world that values ecology.
@@ -2374,17 +2016,17 @@
  Application Deadline (Round 2): Opens 30 April 2026, closes 17 May 2026</t>
         </is>
       </c>
-      <c r="D30" s="1" t="inlineStr">
+      <c r="D23" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E30" s="1" t="inlineStr">
+      <c r="E23" s="1" t="inlineStr">
         <is>
           <t>May 17, 2027</t>
         </is>
       </c>
-      <c r="F30" s="1" t="inlineStr">
+      <c r="F23" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-bes-training-and-travel-grants-british-ecological-society-opg-26-00181</t>
         </is>

</xml_diff>

<commit_message>
Auto update Combined.xlsx [Sat Sep 19 06:59:19 UTC 2026]
</commit_message>
<xml_diff>
--- a/output/Combined.xlsx
+++ b/output/Combined.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -467,149 +467,41 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Expression of Interest EOI for Trade &amp; Livelihood Partners</t>
+          <t>Applications Invited for Wellbeing Research Grants Funding Better Evaluations of AI's Impact on Wellbeing</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>Expression of Interest (EOI) for Trade &amp; Livelihood Partners
-Issued By: BharatCares
-Introduction
-India's rural and tribal skilling landscape holds a real opportunity: pairing structured vocational training with locally rooted crafts and livelihood traditions, so that trainees gain both immediate employability and enterprise pathways they can build on for a lifetime. The Kaushal Vikas Setu program has established Skills Academies as permanent community assets like training centers designed to expand into new trades each year, drawing on the skills, materials, and traditions already present in the communities they serve.
-Kaushal Vikas Setu is a Skill Development Program implemented by BharatCares (SMEC Trust), currently running vocational training centers at Baihar (Balaghat district, Madhya Pradesh) and Surgana (Nashik district, Maharashtra). The program trains tribal and rural youth with priority given to women across trades including Assistant Electrician, Sewing Machine Operator, and Handmade Accessories, and is designed to add new trades to its Skills Academy model over time.
-To deepen and diversify this impact, we now invite Expressions of Interest from three categories of partners: (A) bamboo-based organizations and NGOs working in the bamboo sector, (B) Warli painting artists, enthusiasts, and organizations, and (C) organizations offering high-level, advanced tailoring and garment design expertise. If your organization or you as an individual practitioner work in any of these areas, this EOI is for you.
-About the Program
-Kaushal Vikas Setu is implemented by BharatCares at two block-level Skills Academies Baihar (Balaghat, Madhya Pradesh) and Surgana (Nashik, Maharashtra) serving tribal communities including Bhil, Garasia, Bhilala, Warli, and Mahadeo Koli.
-The program is built around:
-Skills Academy model — permanent, block-level training centres offering NSQF-aligned vocational courses, designed to expand into new trades each year
-Community-rooted trades — courses selected based on local skill traditions, available materials, and market opportunity
-Women-first design — minimum 30% female participation overall, with women prioritized in trades such as Sewing Machine Operator and Handmade Accessories
-Enterprise pathway — trained participants are supported towards wage employment, self-employment, or enterprise formation, including through Hub &amp; Spoke home-based work models
-Surgana, home to the Nashik center, has a significant Warli tribal population — custodians of the Warli painting tradition. Both centers also run an existing Sewing Machine Operator / Handmade Accessories trade that we are looking to elevate into a higher-value, more market-ready tailoring offering.
-Part A — Bamboo-Based Livelihood &amp; Craft Partners             
-Why We Are Issuing This EOI
-Surgana's tribal communities carry long-standing bamboo-working knowledge, and bamboo offers a low-investment, locally sourced material base for livelihood generation. We are seeking partners who can help the Suragna Skill Centre design and deliver a structured bamboo livelihood/craft trade one that builds on existing community skill while introducing market-ready product design, quality standards, and sales linkages.
-We are looking for partners who can contribute to one or more of the following:
-Curriculum &amp; Trade Design — Developing a structured, NSQF-align able training curriculum for bamboo craft/product-making suited to the local skill base
-Trainer Deployment — Providing or training master trainers in bamboo processing, product design, and finishing techniques
-Product Development — Designing market-ready bamboo products (utility items, furniture components, décor, eco-friendly packaging) suited to urban and institutional markets
-Tools &amp; Equipment — Supporting basic processing equipment/tools for bamboo treatment and product-making
-Market Linkage — Connecting trained artisans/entrepreneurs to buyers, retailers, or export markets for bamboo products
-Objectives
-Introduce a structured bamboo livelihood trade at the center in Surgana.
-Build trainee capability from raw bamboo processing through to finished, sellable products
-Establish market linkages that make bamboo-based livelihoods sustainable beyond the training period
-Build a long-term partnership — not a one-time training that grows with the Skill Center.
-Who Can Apply
-NGOs and development organizations working in the bamboo sector or on bamboo-based livelihoods
-Bamboo cooperatives, producer companies, or enterprises with training/mentoring capacity
-Government-affiliated bamboo missions, boards, or their implementation partners
-Design studios or social enterprises with bamboo product development experience
-Eligibility Criteria
-Mandatory:
-Formally registered organization or enterprise
-Demonstrated prior work in the bamboo sector — cultivation, processing, craft, or enterprise
-Willingness to engage in a structured, time-bound collaboration with defined deliverables
-Committed to a community-first approach centring trainee ownership and livelihood outcomes
-Preferred:
-Prior experience training tribal or rural communities
-Presence or operational capacity in Maharashtra or nearby states.
-Experience in sustainable, eco-friendly bamboo product lines
-Willingness to contribute at subsidized rates or as part of a CSR/social impact mandate
-Part B — Warli Art Partners
-Why We Are Issuing This EOI
-Surgana's Warli community carries one of India's most recognized tribal art traditions, yet the shift from ancestral practice to a structured, income-generating trade needs deliberate design. We are seeking partners who can help the Surgana Skills Academy build a Warli art livelihood trade — combining respect for the tradition's cultural roots with training design that makes it commercially viable for trainees.
-We are looking for partners who can contribute to one or more of the following:
-Curriculum &amp; Trade Design — Structuring Warli art training into a teachable, skill-graded course for the Skills Academy
-Master Artisan Trainers — Deploying, or connecting us with, skilled Warli artists able to train youth in authentic technique
-Product Diversification — Adapting Warli art onto sellable formats such as textiles, home décor, stationery, wall art, and corporate gifting items
-Documentation &amp; Preservation — Documenting Warli motifs, techniques, and oral history for training material and cultural archival
-Market &amp; Exhibition Linkage — Connecting trained artists to exhibitions, retail, corporate gifting, or export opportunities
-Objectives
- Establish a structured Warli art livelihood trade at the Surgana Skills Academy
-Preserve the authenticity and cultural integrity of Warli painting while building commercial skill
-Create sustainable income pathways for Warli youth, especially women, through art-based enterprise
-Build a long-term partnership that grows with the Skills Academy — not a one-off workshop
-Who Can Apply
-Warli art organisations, collectives, or cultural preservation NGOs
-Individual master Warli artists and enthusiasts willing to train or mentor
-Design institutions or studios with craft documentation or product adaptation experience
-NGOs working in tribal art, craft-based livelihoods, or cultural heritage preservation
-Eligibility Criteria
-Mandatory:
-Demonstrated genuine practice of, or engagement with, Warli art (individuals or organisations)
-Willingness to engage in a structured, time-bound collaboration with defined deliverables
-Commitment to authenticity — training must respect and preserve traditional Warli technique and meaning
-Community-first approach, prioritising Warli artisans' ownership and livelihood outcomes
-Preferred:
-Prior experience training youth or first-time learners in Warli art
-Presence or ability to travel to Surgana, Nashik district, for on-ground engagement
-Experience adapting traditional art onto commercial products
-Willingness to contribute pro-bono or at subsidised rates as part of a CSR/social impact mandate
-Part C — High-Level Tailoring &amp; Garment Design Partners
-Why We Are Issuing This EOI
-Our existing Sewing Machine Operator and Handmade Accessories trades give trainees entry-level stitching skill, but many — especially women who complete the base course — are ready to progress into higher-value tailoring: garment construction, pattern-making, boutique-level finishing, and small-scale fashion enterprise. We are seeking partners who can help design and deliver this next tier of tailoring training at both Skills Academies.
-We are looking for partners who can contribute to one or more of the following:
-Advanced Curriculum Design — Developing a structured, higher-tier tailoring/garment construction curriculum (pattern-making, cutting, boutique stitching, finishing) that builds on the existing base-level course
-Trainer Deployment — Providing experienced tailoring/fashion trainers to deliver the advanced course
-Enterprise &amp; Boutique Readiness — Training trainees in small-batch production, costing, and boutique/home-enterprise setup
-Equipment Support — Supporting access to higher-capability machines (overlock, interlock, embroidery) beyond basic sewing machines
-Placement &amp; Market Linkage — Connecting trained tailors to boutiques, garment units, or enabling them to set up independent enterprises
-Objectives
-Establish an advanced/high-level tailoring trade as a progression pathway above the existing base-level course
-Equip trainees, particularly women, with enterprise-ready garment construction and finishing skills
-Build placement and market linkages so advanced tailoring translates into sustained income
- Build a long-term partnership that grows the tailoring trade year on year across both Skills Academies
-Who Can Apply
-Fashion and garment training institutes, and design colleges
-Boutique or fashion design studios with training/mentoring capacity
-NGOs with existing advanced tailoring, garment-making, or fashion enterprise programmes
-Sewing machine/equipment manufacturers or suppliers with a CSR or training mandate
-Eligibility Criteria
-Mandatory:
-Formally registered institution, studio, or organisation
-Demonstrated prior work in garment construction, fashion training, or advanced tailoring
-Willingness to engage in a structured, time-bound collaboration with defined deliverables
-Commitment to a trainee-first approach centred on employability and enterprise outcomes
-Preferred:
-Prior experience training rural or tribal women in tailoring/fashion skills
-Presence or operational capacity in Madhya Pradesh or Maharashtra
-Experience setting up trainees in boutique or home-based enterprise
-Willingness to contribute pro-bono or at subsidised rates as part of a CSR/social impact mandate
-What We Offer Collaborating Partners
-Access to an Active Skills Academy — two operational, block-level training centres with an existing trainee cohort and community trust already established
-Community Immersion — direct engagement with tribal and rural youth, most of them first-generation learners, in a live training environment
-Institutional Visibility — partner organisations credited in Kaushal Vikas Setu communications, training materials, and CSR reporting
-CSR &amp; Social Impact Documentation — structured impact documentation to support partners' own CSR or social impact reporting needs
-Network Access — connection to the BharatCares ecosystem of NGOs, CSR partners, and government stakeholders
-Co-creation Opportunity — a genuine role in shaping how a new trade is introduced into the Skills Academy model, from curriculum through to market linkage
-Process &amp; Next Steps
-Step 1 — EOI Submission Interested organisations or individuals submit a short EOI response covering their profile, area of interest (bamboo / Warli / tailoring), prior relevant work, and proposed collaboration model.
-Step 2 — Review &amp; Shortlisting The BharatCares programme team reviews all EOIs and shortlists partners based on relevance, capacity, and alignment with the Skills Academies' current needs. Shortlisted applicants will be contacted within 3 weeks of submission.
-Step 3 — Discovery Conversation A structured conversation between the shortlisted partner and the BharatCares team — and where possible, a visit to Baihar or Surgana — to understand the community context and co-develop the collaboration scope.
-Step 4 — Collaboration Agreement A formal Memorandum of Understanding (MOU) or collaboration agreement is signed, defining the scope, timeline, deliverables, and terms of the partnership.
-Step 5 — On-ground Engagement The collaboration begins — with the partner engaging directly with trainees and the BharatCares programme team at the relevant Skills Academy.
-Documents to Be Submitted with EOI
-Brief organisational or individual profile (2–3 pages or equivalent)
-Portfolio or work samples demonstrating relevant prior work (bamboo / Warli art / tailoring, as applicable)
-Proposed area and model of collaboration (as described in the relevant Part above)
-Names and profiles of key personnel, trainers, or artisans who would be involved
-Any prior work with tribal or rural communities, with references if available</t>
+          <t>About the Organization
+We're an AI research company that builds reliable, interpretable, and steerable AI systems. Our first product is Claude, an AI assistant for tasks at any scale. Our research interests span multiple areas including natural language, human feedback, scaling laws, reinforcement learning, code generation, and interpretability. 
+ About the Opportunity:
+Anthropic is launching a $5 million grant program to fund independent research into how AI impacts users' wellbeing. The program will provide direct funding, access to Anthropic's models, and technical support to grantees building open-source evaluations that help the AI industry measure how models affect those who use them. Grantees will work fully independently, and will publish their work as open-source projects that any developer can make use of.
+ Background/Rationale:
+AI systems have become central to how many people work, learn, and solve problems, and have also become conversational partners and sources of emotional support during difficult times, but the industry is still developing clear standards for how models should behave in such conversations — for example when a user seeks companionship or navigates a mental health crisis. Wellbeing is described as a particularly difficult area to evaluate, since assessing it requires more context than checking a single response for accuracy — the need for a cautious response may only become clear over a long conversation, and a response reasonable in one context could be harmful in another. By funding independent evaluations and benchmarks of user wellbeing, Anthropic hopes to invite more people — including clinicians, psychologists, and methodologists — to contribute to this field. 
+ What They're Looking For
+Grantees should build evaluations that:
+State clearly what they are measuring (what counts as a pass or fail, and why it matters) 
+Involve clinical and subject-matter experts in the design and validation 
+Test both precautions and harms (i.e., evaluate the risk of both overcompliance and overrefusal) 
+Reflect how users actually use AI, often through multi-turn conversation scenarios where risk escalates and context shifts
+Validate their graders against real subject-matter experts 
+ Eligibility/Target Applicants: Independent researchers — clinicians, psychologists, methodologists, and other subject-matter experts working on AI wellbeing evaluation/benchmarking
+ Funding Amount: Total program pool of $5 million (individual grant sizes not specified on the page)</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>Governance</t>
+          <t>Learning</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>Sep 20, 2026</t>
+          <t>Sep 21, 2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/rfps/expression-of-interest-eoi-for-trade-and-livelihood-partners-bharatcares-rfp-26-00340</t>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-wellbeing-research-grants-funding-better-evaluations-of-ais-impact-on-wellbeing-anthropic-opg-26-00175</t>
         </is>
       </c>
     </row>
@@ -621,75 +513,70 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>RFP - Research Collaboration For Improved Application and Processing Techniques For Natural Dyes</t>
+          <t>ToR for Stand post - Varanasi</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>REǪUEST FOR PROPOSALS (RFP)
-Research Collaboration For Improved Application and Processing Techniques For Natural Dyes
-COLORS of Nature Project
-Parameter  Details 
-Reference COLORS/DFRǪ/20260005
-Title E-Tender Request for Research Collaboration on Improved Application and Processing Techniques for Natural Dyes (Activity A.2.3)
-Timeline 31st August 2026 – 31 July 2029 (3 years )
-Area of Expertise Textile Wet Processing &amp; Dyeing Chemistry, Natural Dye Application, Sustainable/Cleaner Textile Processing, Eco-friendly Mordanting &amp; Fixation
-Implementation Area Research institution / laboratory facilities, with pilot validation at partner dyeing unit(s) in India; coordinated with project sites in Andhra Pradesh (Parvathipuram Manyam, Srikakulam and Dr BR Ambedkar Konaseema) and Telangana (Vikarabad)
-Submission Deadline 20th September 2026
-Budget Head 5.2.8     Research on Application of Natural Dye of Textile
-Project Overview
-The COLORS of Nature project, co-funded by the European Union and implemented by Welthungerhilfe with partners Avani Society and Chitrika (ALAF), aims to advance circular textile production in India through plant-based dyes. The project targets 15,000 smallholder farmers and artisans across Uttarakhand, Telangana, and Andhra Pradesh (2025–2029).
-Activity A.2.2 and A.2.3 is a research and technology-collaboration component under Output 2 that will identify, test, and pilot improved application and processing techniques for natural dyes spanning mordanting, pre-treatment, fixation, water and energy efficiency, and residue management. This RFP seeks a qualified textile research institution or specialist consultant to conduct up to 3 years of lab-scale and mill-scale research, culminating in validated mill-ready technical guidelines.
- OBJECTIVES
-Overall Objective
-To identify, develop, and validate improved, eco-friendly application and processing techniques for natural dyes on cotton fabrics and yarn that enhance colour fastness, resource efficiency, and industrial scalability, while preserving ecological sustainability.
-Specific Objectives
-The specific objective and scope of the study may undergo changes based on the existing technology for experimentation available in India. Following are the indicative objectives subject to the availability of such a technology in India
-Identify and evaluate natural mordants and bio-based fixation/crosslinking agents that improve colour fastness and dye permanence without compromising the ecological positioning of natural dyes on cotton fabrics and yarn.
-Test and optimize pre-treatment methods on cotton fabrics and yarn.Develop and pilot water-saving dyeing strategies, including closed-loop dyeing systems.
-Evaluate energy-efficient dyeing alternativesDesign and test protocols for recycling or upcycling dye residues to support a zero-waste processing model.
-Validate the most promising techniques at pilot/mill scale in partnership with at least one dyeing unit/mill
- Currently some of the technologies are available for man-made fibers and at huge scale. Technologies suitable for handloom fabric and yarn will be the primary focus of the study
- ELIGIBILITY CRITERIA
-Eligibility
-State/Central Textile Research Associations or Institutes (e.g. South India Textile Research Association)
-National Institute of Fashion Technology (NIFT), National Institute of Design (NID), or similar design/textile institutes
-State/Central Agricultural or Technical Universities with textile chemistry departments
-Reputed textile-sector NGOs with applied research experience
-Private textile research organizations / individual textile researchers with academics from reputed organisations (NID, NIFT etc.,)
-Consortiums of the above (lead applicant must be specified)
-Individual Consultants with 10 years of experience in handlooms production
-5 years experience in working with Andhra Pradesh and Telangana Weavers
- Mandatory Organizational Requirements:
-Legal registration in India (minimum 5 years old). Not applicable to individual consultants
-Access to a testing laboratory accredited for colour-fastness and related textile testing (own or partnered)
- Technical Eligibility Criteria
-Essential:
-Experience with colour-fastness and related textile testing
-Capability to design and run both lab-scale and unit-scale (production) trials
-Prior working relationship with, or ability to secure, a commercial dyeing unit partner, weavers or dye artisans.
-Experience developing technical guidelines / SOPs for weavers or artisan use
-Desirable:
-Prior experience specifically with natural/plant-based dyes
-Familiarity with closed-loop or low-water dyeing systems
-Knowledge in eco-friendly processing certifications (e.g. GOTS, ZDHC)
-Experience in Andhra Pradesh, Telangana, or Uttarakhand
-Network with dyeing units and textile industry associations</t>
+          <t>Background
+Access to safe and reliable drinking water remains a critical challenge in several habitations of Harahua Block in Varanasi District, Uttar Pradesh. Although the Government of India, through the Jal Jeevan Mission (JJM), is expanding piped water supply, many marginalized settlements continue to face inadequate access to potable water due to limited household connections, inadequate storage infrastructure, and uneven water distribution.
+ Women, children, elderly people, and socially vulnerable households are disproportionately affected, often spending considerable time and effort collecting drinking water from distant or unreliable sources. During peak summer months and periods of high demand, the availability of safe drinking water becomes even more constrained.
+ To address this challenge, installation of Ferrocement Tank Towers (Jal Minar) connected with the existing water supply system and equipped with community stand posts is proposed. Ferrocement technology offers a durable, cost-effective, low-maintenance, and climate-resilient solution for decentralized drinking water storage and distribution.
+ Project Goal:
+To improve equitable and sustainable access to safe drinking water for underserved communities in Harahua Block through the installation of Ferrocement Tank Towers (Jal Minar) with community stand posts.
+ Objectives
+Improve access to safe drinking water for underserved households.
+Reduce the distance and time spent collecting drinking water.
+Strengthen community-level drinking water infrastructure.
+Improve water security during supply interruptions and peak demand periods.
+Promote equitable access for women, children, elderly persons, and vulnerable communities.
+Support the objectives of Jal Jeevan Mission by strengthening last-mile service delivery.
+ Proposed Intervention
+The project proposes installation of Ferrocement Tank Towers (Jal Minar) at strategic community locations connected to the existing drinking water supply network.
+Each Jal Minar will include:
+Ferrocement elevated storage tank
+RCC/steel supporting tower (as per design)
+Inlet and outlet pipeline
+Community stand posts with multiple taps
+Drainage arrangement
+Platform for safe water collection
+Water quality signage
+Provision for future maintenance
+ The locations will be finalized in consultation with:
+Gram Panchayat
+Village Water &amp; Sanitation Committee (VWSC)
+Gram Pradhan
+Community representatives
+Stand post details:
+Village/Habitation
+No of Stand Post
+BhatpurwaKala
+1
+Sulemapur
+1
+Mohanpur
+1
+PalahipattiBazar
+1
+PalahipattiPrajapati Basti
+1
+Total Beneficiaries
+5</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Climate</t>
+          <t>Governance</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Sep 20, 2026</t>
+          <t>Sep 22, 2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/rfps/rfp-research-collaboration-for-improved-application-and-processing-techniques-for-natural-dyes-chitrika-rfp-26-00343</t>
+          <t>https://onepurpos.in/openings/rfps/tor-for-stand-post-varanasi-wateraid-india-rfp-26-00364</t>
         </is>
       </c>
     </row>
@@ -701,81 +588,50 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>RFP - Agronomic Research Study For Natural Dye Crop Development</t>
+          <t>SoW - Hiring an External Agency for Orientation and Capacity Building</t>
         </is>
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>REǪUEST FOR PROPOSALS (RFP)
-Agronomic Research Study For Natural Dye Crop Development
-COLORS of Nature Project
-Parameter Details
-Reference COLORS/DFRǪ/20260002
-Title E-Tender Request for Agronomic Research Study for Natural Dye Crop Development (Activity A.2.1)
-Timeline 31st August 2026 – 31 July 2029 (3 years )
-Area of Expertise Agricultural   Research,   Natural    Dye   Crops,   Sustainable                       Farming Practices, Participatory Action Research
-Implementation Area
-Andhra Pradesh (Kotturu Mandal, Parvathipuram Manyam District) &amp; (Ponduru Mandal, Srikakulam District);
-Telangana (Kodangal Mandal, Vikarabad District) &amp; (Narayanpet District)
-Submission Deadline 20th September 2026
-Budget Head 5.2.6 Action research for agronomic practices for Natural Dyes Crops
-Project Overview
-The COLORS of Nature project, co-funded by the European Union and implemented by Welthungerhilfe with partners Avani Society and Chitrika (ALAF), aims to advance circular textile production in India through plant-based dyes. The project targets 15,000 smallholder farmers and artisans across Uttarakhand, Telangana, and Andhra Pradesh (2025–2029).
-Activity A.2.1 is a critical research component that will identify and validate suitable agronomic practices for natural dye crop production. This RFP seeks a qualified research institute or consultant(s) to conduct a 3-year participatory action research with 20 lighthouse farms, evaluating soil treatments, crop combinations, varieties, and harvesting protocols to optimize yield and dye quality.
- OBJECTIVES
-Overall Objective
-To develop and validate evidence-based agronomic practices for cultivating natural dye crops that improve yield, dye quality, and ecological sustainability for smallholder farmers.
- Specific Objectives
-Identify and evaluate suitable plant species/varieties for natural dye production focusing on in-demand colors (blue, red, yellow, green, black, brown, etc). This is an indicative list. Can be changed based on the agro-climatic conditions of the selected regions and the life-cycle/duration of the plan
-Develop optimal Package of Practices (PoP) for the agro - climatic conditions of the women farmers producer companies for 6 priority natural dye crops through participatory field trials.
-Determine best harvesting protocols and maturity indices for maximum dye yield and quality.
-Compare effectiveness of different organic soil management practices on crop performance.
-Assess suitability of intercropping/mixed cropping systems for natural dye crops.
- ELIGIBILITY CRITERIA
-Organizational or Individual Researchers PreFerences
-State/Central Agricultural Universities in India
-ICAR (Indian Council of Agricultural Research) Institutes
-State Agricultural Research Stations
-Reputed Agricultural NGOs with research experience
-Consultants having field experience, access to research/demo plots related to agroecology and natural dyeing
-Private agricultural research organizations
-Consortiums of the above (lead applicant must be specified)
- Mandatory Requirements:
-Legal registration in India (minimum 5 years old) in case of an institution. Not applicable for individual researchers. Instead individual researchers shall have minimum 10 years experience in agro ecology, small holder farming and organic agriculture.
-Adequate infrastructure networks for research management
- Technical Eligibility Criteria
-Essential:
-Expertise in organic/ecological agriculture projects
-Experience working with smallholder farmers in India
-Capability to conduct multi-location trials across different states
-Access to laboratory facilities for soil and plant analysis
-Experience in developing training materials/Package of Practices
-Having working knowledge of Telugu
- Desirable:
-Composition of team should have at least one researcher/professor
-Young Team Leader for the project is preferred with sufficient agro-ecology experience. Active Agro-Ecology practitioners will get additional bonus points
-Research Consultant with experience in training and building capacities around organic agriculture and agro ecology practices will be preferred.
-Prior experience with natural dye crops or Non-Timber Forest Products
-Understanding of handlooms and textile industry requirements
-Experience in Andhra Pradesh or Telangana
-Familiarity with participatory action research methodologies
-Network with agricultural universities and textile research institutions
-Experience working on natural dye</t>
+          <t>Room to Read’s Foundational Literacy Program in Jharkhand
+Anchoring and Delivery of Orientation Programme for Jharkhand Field Workforce
+Scope of Work (SoW)
+for
+Hiring an External Agency for Orientation and Capacity Building
+Organizational Overview
+ Founded in 2000 on the belief that World Change Starts with Educated Children®, Room to Read develops children’s foundational literacy skills, as well as life skills that promote gender equality. We nurture these essential skills in children by training and coaching educators, creating quality learning materials and spaces, strengthening education systems, and delivering programs directly and with partners – all while honouring the dignity of every child. Committed to accelerating learning outcomes for more children, more quickly, Room to Read has benefited children across 29 countries, with more than 17 million children actively benefiting from our programming in 2025 alone. Room to Read India’s literacy operations currently span across 12 states, with a focus on improving children’s reading skills, access to quality learning materials, and supportive learning environments. Room to Read envisions a world free from illiteracy and gender inequality, where all children have room to read, learn and grow. Visit us at https://www.roomtoreadindia.org/
+Jharkhand Foundational Literacy Project Overview
+ Room to Read is preparing for a significant scale-up of its Foundational Literacy &amp; Numeracy initiative in Jharkhand, expanding implementation across multiple districts and requiring a substantial field workforce to support programme delivery. As Room to Read expands its field implementation in Jharkhand, a substantial number of staff will join different field-facing and supervisory roles.  As part of the planned scale-up, Room to Read expects to onboard more than 150 staff in Phase 1 across field implementation, supervisory and district-level leadership roles. A second cohort of approximately 120 additional staff is expected to be onboarded in Phase 2 as implementation expands to the remaining districts.
+ Objective of the Assignment
+The overarching objective of this assignment is to ensure that over two phases 250+ team members in Jharkhand are ready for project implementation.
+Phase 1 will aim at getting all 150+ staff members ready for project implementation by March 31st, 2027.
+Phase 2 will follow the same approach for an additional 120+ team members, with the orientation programme to be completed by 30 March 2028, followed by final review, handover and closure activities in April 2028.
+Agency Requirements &amp; Qualifications 
+The agency should preferably:
+Preferred 3 years of relevant experience in designing and delivering orientation, training or capability-building programmes for field-based teams, particularly in the education, development or government-facing sector.
+Have completed at least 2 similar assignments involving training across multiple batches, locations or large participant groups.
+Demonstrate experience in learning-needs assessment, adult-learning design, content development and participatory training methodologies.
+Demonstrate experience in developing facilitator guides, participant materials, simulations, assessments, job aids or other training resources, and provide 1-2 relevant samples where available.
+Have the ability to deliver training in Hindi and deploy an adequate pool of suitable facilitators for implementation across Jharkhand.
+Provide details and CVs of the proposed core team and key facilitators, including their qualifications, relevant experience, roles and expected level of engagement in the assignment. The agency should ensure continuity of key facilitators, with minimal changes during each phase of the assignment.
+Demonstrate experience in assessing training effectiveness through participant feedback, assessments, learning-progress tracking and/or follow-up or refresher support.
+Have established systems for project management, quality assurance, documentation, progress tracking and reporting, with the ability to maintain consistency across training cohorts.
+Provide details of at least 2 relevant past clients/assignments that may be referred to for verification of experience and performance</t>
         </is>
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>Learning</t>
+          <t>Governance</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>Sep 20, 2026</t>
+          <t>Sep 23, 2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/rfps/rfp-agronomic-research-study-for-natural-dye-crop-development-chitrika-rfp-26-00344</t>
+          <t>https://onepurpos.in/openings/rfps/sow-hiring-an-external-agency-for-orientation-and-capacity-building-room-to-read-india-rfp-26-00366</t>
         </is>
       </c>
     </row>
@@ -787,153 +643,10 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>RFPs Invited for Using an Agent Based Model to Predict the Impact of City-Level Policies on the Adoption of Distributed Renewable Energy</t>
+          <t>Applications Invited for GEF SGP CSO Challenge Program</t>
         </is>
       </c>
       <c r="C5" s="1" t="inlineStr">
-        <is>
-          <t>About C40:
-C40 is a network of nearly 100 mayors of the world's leading cities working to deliver urgent climate action and create a future where everyone, everywhere, can thrive. Mayors of C40 cities are committed to using a science-based, people-focused approach to limit global heating in line with the Paris Agreement, working alongside labour, business, youth climate movement, and civil society representatives to help halve emissions by 2030.
- Project Summary/Background:
-C40 represents 5 member cities in India (Mumbai, Ahmedabad, Bengaluru, Chennai, New Delhi) plus Karachi. C40's Research team is launching a project to accelerate Indian grid decarbonisation and improve public health, funded by the Wellcome Trust, in collaboration with Ashoka ACPET and CHART centres. The project has 3 work packages (national, urban, and rural scale); this RFP covers Work Package 2 (WP2) — the urban-scale component, led by C40, focusing on city-level interventions to accelerate distributed solar energy deployment and reduce coal dependence in Mumbai and Chennai.
- Objective:
-Apply an Agent-Based Modelling (ABM) approach to analyse the impact of specific local policy measures on the adoption of solar and batteries by residential and commercial actors in Mumbai and Chennai. The Supplier will:
-Develop methodology, assess data needs, conduct local ground surveys, and model baseline energy consumption
-Develop/repurpose an ABM to assess how policy interventions (renewable energy mandates, metering changes, peak-hour tariff changes, etc.) impact uptake of distributed solar/batteries
-Model how changes in solar use translate to changes in capacity factors of specific coal power plants and resulting emission reductions (GHG, PM2.5, NOx)
- Scope: Covers all energy use in the built environment and industries within Mumbai and Chennai's urban boundaries — households (owners/renters, income levels) and businesses (including industrial). Focus on distributed solar electricity generation/use and battery storage. Excludes solar thermal solutions and institutional buildings. Energy generation model covers the whole state.
- Deliverables:
-Methodology, Local Ground Surveys &amp; Data Collection — Methodology document (20 pages max), data mapping, sample survey results, data collection documents
-Agent-Based Model of Renewable Energy Uptake — Updated methodology, ABM simulation runs, outputs report (up to 15 pages)
-Power Plant Utilisation Rate Modelling — Updated methodology, plant-level energy use files (hourly), findings report (up to 15 pages)
- AI Use Restriction: Use of AI-supported tools must be kept to an absolute minimum; no final output (text/visuals) may be AI-produced. Any AI tool use must be justified in methodology. Results must be validated via human oversight and cross-referencing with trusted sources. C40 data is confidential and cannot be shared with AI tools.
- Proposal Requirements: Must be under 15 pages (all-inclusive), covering: responsiveness to evaluation criteria, ABM approach &amp; survey strategy, relevant experience (with reference letters from past 3 years, not counted in page limit), risk identification/mitigation, fee justification, implementation timeline, key personnel resumes, additional support needed, and proposed working partnership structure with C40.
- Evaluation Criteria &amp; Weighting:
-Methodology rigour and delivery clarity: 20%
-Technical Expertise (ABM, energy modelling, Indian policy context): 30%
-Project management experience: 20%
-Cost Reasonableness: 20%
-Equity and Alignment (India-based organizations strongly encouraged): 10%
- Project Budget: USD 50,000 for all deliverables (payment per milestone approval; travel expenses included)
- Contract Type: Professional services contract (Note: this is a contract opportunity, not a grant — organisations unable to accept professional services contracts should not apply); C40 Standard Services Contract terms are non-negotiable
- Key Dates:
-RFP Sent: September 1, 2026
-Questions Submitted to C40: September 10, 2026
-C40 Responds to Questions: September 14, 2026
- Deadline for Receiving Offers: 12 PM EST, 20 September 2026
-Clarification of Offers: September 25, 2026
-Evaluation of Proposals: September 28, 2026
-Interviews (if needed): September 29, 2026
-Selection Decision: September 30, 2026
-All Suppliers Notified: October 10, 2026
- Project Delivery Timeline:
-Deliverable 1: March 30, 2026 (note: this date appears to predate the RFP issue date — likely a typo in the source document for 2027)
-Deliverable 2: May 15, 2026 (same note applies)
-Deliverable 3: June 15, 2025 (same note — likely should read 2027)
-Project runs until: June 30, 2027</t>
-        </is>
-      </c>
-      <c r="D5" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E5" s="1" t="inlineStr">
-        <is>
-          <t>Sep 20, 2026</t>
-        </is>
-      </c>
-      <c r="F5" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/rfps-invited-for-using-an-agent-based-model-to-predict-the-impact-of-city-level-policies-on-the-adoption-of-distributed-renewable-energy-c40-cities-rfp-26-00357</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="95" customHeight="1">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>E-Tender Request for Digital Communication Website Development and Social Media Campaign for Colors of Nature</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="inlineStr">
-        <is>
-          <t>REǪUEST FOR PROPOSALS (RFP)
-Digital Communication, Website Development and Social Media Campaign
-Colors of Nature Project
-Parameter Details
-Reference COLORS/DFRǪ/20260002
-Title E-Tender Request for Digital Communication, Website Development and Social Media Campaign for Colors of Nature (Activity A.2.1)
-Timeline 31st August 2026 – 31 July 2029 (3 years)
-Area of Expertise Website, Digital Marketing
-Submission Deadline 20th September 2026
-Budget Head
-5.8.4 - Website
-6.3.3 - Social Media Campaign
-Requirements Proposal for website and social media campaign to be submitted separately
-Background
-The COLORS of Nature project, co-funded by the European Union and implemented by Welthungerhilfe with partners Avani Society and Chitrika (ALAF), aims to advance circular textile production in India through plant-based dyes. The project targets 15,000 smallholder farmers and artisans across Uttarakhand, Telangana, and Andhra Pradesh (2025–2029).
-As the project progresses, there is a need to establish a strong digital identity that documents the project's journey, showcases its impact, creates awareness among consumers, and positions Colors Of Nature as a long-term knowledge and collaboration platform for natural dyes beyond the life of the project.
-Objective
-To conceptualise, design, develop and manage an integrated digital communication ecosystem for Colors Of Nature, comprising:
-Social media platforms
-Digital storytelling
-Knowledge documentation
-Consumer awareness campaigns
-Multimedia communication products
-Brand identity development
-The platform should serve not merely as a project communication tool but as a lasting digital destination for natural dyes in India.
-Specific Objectives
-The selected agency shall work towards the following objectives:
-Establish Colors Of Nature platform as a recognised digital identity for natural dyes.
-Build awareness among at least 100,000 consumers on the environmental, cultural and livelihood significance of natural dyes through planned digital campaigns.
-Ensure appropriate visibility to the European Union and Welthungerhilfe (WHH) in accordance with donor communication and visibility guidelines.
-Create opportunities for future collaborations with designers, educational institutions, buyers, researchers and sustainability practitioners.
-Build a digital footprint that continues to remain relevant beyond the project period.
-Desired Profile oF the Agency
-The project seeks to engage a young, creative and mission-driven communication agency, digital collective or social enterprise rather than a conventional large communication firm.
-Preference shall be given to agencies that:
-Demonstrate innovation, creativity and agility.
-Have experience in development communication.
-Have exposure to rural livelihoods, sustainability, crafts, agriculture or textiles.
-Are willing to mentor and build a dedicated communications team to manage website content, digital campaigns and communication products over time.
-Demonstrate strong storytelling capabilities.
-Operate through lean and cost-effective implementation models while maintaining high quality standards.
-Ready to develop a women led and based digital marketing team</t>
-        </is>
-      </c>
-      <c r="D6" s="1" t="inlineStr">
-        <is>
-          <t>Learning</t>
-        </is>
-      </c>
-      <c r="E6" s="1" t="inlineStr">
-        <is>
-          <t>Sep 20, 2026</t>
-        </is>
-      </c>
-      <c r="F6" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/e-tender-request-for-digital-communication-website-development-and-social-media-campaign-for-colors-of-nature-chitrika-rfp-26-00342</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="95" customHeight="1">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for GEF SGP CSO Challenge Program</t>
-        </is>
-      </c>
-      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global Environment Facility Small Grants Programme (SGP) is a global initiative implemented by the United Nations Development Programme (UNDP) on behalf of the Global Environment Facility (GEF). Since its launch in 1992, SGP has empowered communities worldwide to take action on environmental challenges while improving livelihoods. As a GEF Corporate Programme, SGP provides direct support to civil society organisations and community-based organisations to design and implement innovative, locally driven solutions. The programme places strong emphasis on inclusion, ensuring meaningful participation of Indigenous Peoples, youth, women and girls, and other underrepresented groups.
@@ -982,34 +695,34 @@
 Risk management and mitigation</t>
         </is>
       </c>
-      <c r="D7" s="1" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E7" s="1" t="inlineStr">
+      <c r="E5" s="1" t="inlineStr">
         <is>
           <t>Sep 23, 2026</t>
         </is>
       </c>
-      <c r="F7" s="1" t="inlineStr">
+      <c r="F5" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-gef-sgp-cso-challenge-program-gef-small-grants-programme-sgp-opg-26-00184</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="95" customHeight="1">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
+    <row r="6" ht="95" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>RFP for Impact Assessment</t>
         </is>
       </c>
-      <c r="C8" s="1" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>Introduction
 Titan Company Limited, a member of the Tata Group, has a long-standing commitment to Corporate Social Responsibility (CSR) in India. The company's CSR initiatives derive its philosophy from the Company’s vision statement: “We create elevating experiences for the people we touch and significantly impact the world we work in”. The initiatives are designed to promote inclusive growth, empower communities, and contribute to the country's socio-economic development. The program includes Titan’s CSR policy is governed by a dedicated CSR Committee that ensures transparency and compliance with regulatory requirements. The program includes Girl Child Education, Skill and Entrepreneurship Development, supporting Indian Heritage Arts and Crafts, Integrated Village Development Programme, Eye Care and Affirmative Action. Titan's CSR policy is governed by a dedicated CSR Committee that ensures transparency and compliance with regulatory requirements.
@@ -1043,34 +756,122 @@
 Timeline: Proposal submission deadline: September 24, 2026</t>
         </is>
       </c>
-      <c r="D8" s="1" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E8" s="1" t="inlineStr">
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>Sep 24, 2026</t>
         </is>
       </c>
-      <c r="F8" s="1" t="inlineStr">
+      <c r="F6" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfp-for-impact-assessment-titan-rfp-26-00354</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="95" customHeight="1">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="inlineStr">
+    <row r="7" ht="95" customHeight="1">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>EOI- Engagement of State-Level Field Facilitation Consultants for Project Learning StudyEOI</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>Expression of Interest (EOI)
+For
+Engagement of State-Level Field Facilitation Consultants for Project Learning Study
+Publication Date: 18th September 2026 
+ 1. Assignment Objective
+The State-Level Field Facilitation Consultant will provide on-ground coordination and facilitation support to the central study agency and the organisation’s project team. The consultant will not independently conduct the research, evaluation, or learning study. Their primary responsibility will be to enable timely, smooth, ethical, and well-coordinated access to relevant stakeholders and field locations for the agency’s study activities. 
+ 2. Background
+American India Foundation Trust implemented EY Skill Bridge Project across six states (Haryana, Maharashtra, Karnataka, Telangana, Tamilnadu and Odisha) for approximately four years. Although implementation has concluded, a cross-state learning study will now be undertaken to document the project journey, assess broader outcomes, identify what worked well and what did not, and generate learning for future programming.
+ A central agency/knowledge partner will be engaged to conduct the study, including research, stakeholder consultations, field documentation, analysis, and preparation of the final learning document. Since the agency may not have established access or operational visibility at school and government levels in every state, one field facilitation consultant will be engaged in each of the six project states. Stakeholder consultation across schools, teachers, students, head teachers, and government officials is a core element of the project evaluation and learning exercises. 
+ 3. Scope of Work
+The consultant will undertake the following activities within the assigned state:
+Coordinate with AIFT’s agencies, obtain necessary background information on project locations, participating schools, key stakeholders, and available records.  
+Prepare and update field engagement plan in discussion with the agencies, including proposed school visits, stakeholder consultations, travel schedules, contact details, and required permissions. 
+Establish communication and coordinate with head teachers/principals, teachers, school management representatives, students where appropriate, and other relevant school-level stakeholders. 
+Facilitate access to identified project schools and support scheduling of visits by the central study agency. 
+Liaise with relevant government officials at district, block, cluster, or state level, as applicable, to seek appointments and enable consultations. 
+Support the central agency in organising stakeholder interviews, focus-group discussions, meetings, and field interactions according to the agency’s research plan and tools. 
+Ensure that stakeholders receive timely information about the purpose, date, time, venue, and expected duration of consultations. 
+Assist schools and local stakeholders in arranging an appropriate space and suitable time for interviews or group discussions, while ensuring minimal disruption to academic activities. 
+Support the agency in obtaining relevant non-confidential project-related records, information, or documentation available with schools and local stakeholders, subject to organisational approvals and applicable data-protection requirements. 
+Accompany or support the agency during field visits whenever required, including logistical coordination and local issue resolution. 
+Track completion of planned consultations and promptly flag delays, access constraints, cancellations, or stakeholder availability issues to the organisation and agency. 
+Maintain a concise field-visit tracker containing dates, locations, stakeholders contacted, consultations facilitated, pending actions, and key operational observations. 
+Submit brief periodic updates and a final state-level completion note to the designated project focal point. 
+This role is aligned with common education-sector consultancy practice, where field facilitators liaise with school leaders and government stakeholders, organise consultations and field visits, and document stakeholder inputs for the lead research or technical team. 
+ 4. Key Deliverables
+Each consultant will submit:
+State-level stakeholder mapping and proposed field-engagement schedule within the first week of engagement. 
+School-visit and consultation tracker, updated fortnightly. 
+Records of appointments, meetings, consultations, and field coordination completed. 
+Weekly or fortnightly progress update highlighting completed activities, upcoming engagements, challenges, and support required. 
+A final state-level completion note summarising: 
+Schools and stakeholders supported 
+Consultations facilitated 
+Key coordination challenges and resolutions 
+Pending follow-up actions, if any 
+Practical field observations relevant to the study process 
+ 5. Duration and Engagement Terms
+Number of consultants: Six consultants, one for each project state (Haryana, Maharashtra, Karnataka, Telangana, Tamil Nadu and Odisha) 
+Duration: Two months from the date of onboarding or issuance of the agreement. 
+Nature of engagement: Short-term consultancy assignment. 
+Assignment location: Respective assigned state, with travel to identified schools and government offices as required. 
+Professional fee: To be paid in INR for complete two-month assignment (Milestone), subject to satisfactory completion of agreed deliverables and compliance with organisational requirements. 
+Reporting: The consultant will report to the designated organisation focal point and work in close coordination with the centrally appointed learning-study agency. 
+6. Roles and Boundaries
+The consultant’s role is facilitative and coordination-focused. The central agency will retain responsibility for research design, tools, data collection methodology, analysis, interpretation of findings, and preparation of the final learning document. The consultant must not make commitments on behalf of the organisation, independently collect sensitive data outside the agreed process, or share stakeholder information without authorisation. 
+7. Required Competencies
+The consultant should have:
+Experience working with schools, education programmes, government systems, NGOs, CSR projects, or community-based initiatives. 
+Strong local knowledge and working relationships with school and government stakeholders in the assigned state. 
+Demonstrated ability to coordinate field visits, meetings, consultations, and logistics. 
+Good written and verbal communication skills in English and relevant local language(s). 
+Ability to travel independently within the assigned geography. 
+Professional conduct, confidentiality, responsiveness, and timely reporting discipline.  
+A strong consultant profile for this assignment combines field coordination, government liaison, stakeholder management, documentation, and support to third-party evaluation activities. 
+Scope of Information Requested
+This stage is for collecting information from interested Consultant. AIFT will review the submissions and may issue a detailed Request for Quotation (RFQ) to shortlisted consultant based on the specific assignments.</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>Sep 25, 2026</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/eoi-engagement-of-state-level-field-facilitation-consultants-for-project-learning-studyeoi-american-india-foundation-rfp-26-00367</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="95" customHeight="1">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>ToR - Engagement of Information Design &amp; Video Production Agency / Consultant for Key Learning &amp; Dissemination Outputs</t>
         </is>
       </c>
-      <c r="C9" s="1" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>Terms of Reference (TOR) for Consultancy Services
 Title  Engagement of Information Design &amp; Video Production Agency / Consultant for Key Learning &amp; Dissemination Outputs
@@ -1089,9 +890,70 @@
 The primary objective of this engagement is to enable SELCO Foundation to effectively capture, structure, and communicate its field insights, sectoral learnings, and program impacts. The selected Agency/Consultant (or Agencies/Consultants) will work on a monthly retainer basis to translate raw content, data, field footage, and reports provided by SELCO into high-quality, visually compelling, reader-friendly visual outputs and video assets.</t>
         </is>
       </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Sep 28, 2026</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/tor-engagement-of-information-design-and-video-production-agency-consultant-for-key-learning-and-dissemination-outputs-selco-foundation-rfp-26-00362</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="95" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>ToR - Video documentation of change stories on Ground water replenishment in Hyderabad and Sanga Reddy locations</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>About Jal Seva Charitable Foundation/ WaterAid India:
+Jal Seva Charitable Foundation (JSCF) is registered in India as a not-for-profit company under Chapter 8 of the Companies Act, 2013. JSCF, is an associate member of WaterAid International and uses the brand name ‘WaterAid’ in India.
+JSCF or WaterAid India seeks to improve climate resilience access to clean water, decent toilets, and good hygiene for everyone, everywhere. Our work is focused on the following themes:
+Safe, assured drinking water at a household level.
+Safely managed sanitation.
+Water, sanitation, and hygiene (WASH) in institutions (Anganwadi, schools, and health care facilities).
+Hygiene education and behaviour change.
+ WaterAid India country office is based in New Delhi with State Offices in Bengaluru, Bhopal, Bhubaneswar, Hyderabad, Lucknow, Raipur, and Patna. WaterAid India currently works in 11+ states across the country. As a direct implementing agency, WaterAid India district and block-level teams are located close to our intervention villages. Further information regarding WaterAid India can be found online;  https://www.wateraid.org/in/ 
+ Background &amp; Scope of engagement:
+Water security is a major development challenge in urban India, driven by rapid urbanization, rising water demand, declining groundwater, and climate variability. Hyderabad, one of India’s fastest-growing cities, has seen significant urban expansion, which has reduced natural recharge areas, increased surface runoff, and placed greater pressure on groundwater resources.
+The Serilingampally Zone of the Greater Hyderabad Municipal Corporation (GHMC) is especially vulnerable to groundwater depletion due to rapid development. Although municipal water supply is expanding, groundwater remains a vital supplementary source for domestic and institutional needs. Sustainable groundwater recharge and conservation are essential for long-term urban water security.
+ To address these challenges, WaterAid India, launched the Amruthvarshini Project in May 2023. The project aimed to enhance groundwater replenishment through rainwater harvesting, managed aquifer recharge, community mobilization, awareness campaigns, and institutional strengthening.
+ Over the past three years, the programme has produced increased groundwater recharge, photographs, videos, beneficiary stories, and communication materials. These now need to be converted into engaging digital content to support knowledge sharing and future urban water security initiatives.
+ In this context, Jal Seva Charitable Foundation (JSCF) seeks to engage a consultant for ‘Video Documentation of Change Stories’ as outlined in the following terms and conditions.
+ Objective of the contract:
+The objective of this assignment is to capture and document post-intervention activities of ground water replenishment in Sherlingampally Zone in Hyderabad and in Sangareddy district through video documentation.
+ Scope of assignment &amp; expected outcome:
+This assignment involves producing a 6-minute video capturing real-life change stories resulting from water-harvesting interventions.
+The assignment includes the following deliverables:
+A 6-minute, high-resolution video showcasing the impact of water-harvesting infrastructure through community testimonials. It will include interviews, relevant field visuals and a clear storyline highlighting the changes brought about by the interventions. The video will effectively capture community experiences, benefits, and key outcomes.
+ Duration of the contract: The Consultancy Agreement will be effective for a period of 20 days from the date of signing and is expected to be completed by 30 October 2026, unless extended in writing by JSCF. Any extension will be subject to additional or revised terms and conditions as mutually agreed upon in writing between the Consultant and JSCF.
+ Reporting point and Progress Report
+For matters covered by the TORs and this agreement, you will report directly to Mr Pachimadla Krishna, Program Coordinator, Telangana, JSCF, and submit reports as specified in the TORs.
+Payment Schedule Condition for Payment
+ 20%
+40%
+40%
+Upon signing of the Contract
+Upon submission of 6 Minutes of Drafted Video
+Upon completion of Assignment</t>
+        </is>
+      </c>
       <c r="D9" s="1" t="inlineStr">
         <is>
-          <t>Governance</t>
+          <t>Learning</t>
         </is>
       </c>
       <c r="E9" s="1" t="inlineStr">
@@ -1101,7 +963,7 @@
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/rfps/tor-engagement-of-information-design-and-video-production-agency-consultant-for-key-learning-and-dissemination-outputs-selco-foundation-rfp-26-00362</t>
+          <t>https://onepurpos.in/openings/rfps/tor-video-documentation-of-change-stories-on-ground-water-replenishment-in-hyderabad-and-sanga-reddy-locations-wateraid-india-rfp-26-00363</t>
         </is>
       </c>
     </row>
@@ -1113,10 +975,71 @@
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
+          <t>ToR - Video Production Storytelling and Documentation</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>Title Video Production – Storytelling and Documentation
+Timeline 3 months from the date of contracting
+Expected area of expertise Video production, documentary storytelling, interviews, field documentation, cinematography and post-production
+Apply Link https://forms.gle/qiATVNrSkDJrkNH3A
+Last      Date             for Apply 29th September 2026 by 5 PM
+About SELCO Foundation:
+SELCO Foundation’s mission is to create a platform of solutions that uses sustainable energy as a catalyst to bridge environmental sustainability and poverty alleviation. With holistic development as the primary focus, the organization strives to create equitable societies, where services are accessed by all communities. The interventions of SELCO lead to a sustainable delivery model of essential services like livelihoods, education, and health till the last mile. (Read more about SELCO here: http://www.selcofoundation.org/)
+ About the Programmes:
+SELCO Foundation is looking to engage a video production partner to develop a series of compelling videos that document and communicate stories emerging from its programmes and field interventions.
+The assignment will involve end-to-end video production, including story development, filming, interviews, visual documentation, editing and post-production. The videos will highlight people, experiences, solutions, impact and the broader context of the organisation's work.
+The final content will be used across digital platforms, social media, events, presentations, reports and other communication channels
+ Objective:
+To produce a series of compelling videos that document programme experiences, end-user journeys and solutions in a clear, engaging and accessible manner.
+The videos should move beyond activity documentation to capture the context, challenge, solution, experience and outcomes of the people and communities being documented.
+The selected partner will be expected to provide:
+Story treatment/concept notes
+Interview questions and filming plan
+Raw footage from all filming
+Edited full-length video
+Edited short version
+30-second trailer
+Subtitled versions, where required
+Final master files in agreed resolution and formats
+Social-media-ready versions, where required
+Project/source files upon completion
+ Submission Requirements:
+Interested production partners are requested to submit the following by before deadline
+Organizational/Individual Profile: Overview of your team/experience.Proposed Approach: A brief document outlining your understanding of the assignment and your proposed approach to storytelling and production.
+Relevant Portfolio: 3–5 relevant video samples demonstrating documentary, impact, social-sector, development or human-interest storytelling.Experience with Similar Assignments: Details of relevant video production and field documentation work.
+Quotation Should include all cost including Travel and Miscellaneous.</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>Sep 29, 2026</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/tor-video-production-storytelling-and-documentation-selco-foundation-rfp-26-00368</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="95" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
           <t>Application Invited for Giving Joy Microgrant</t>
         </is>
       </c>
-      <c r="C10" s="1" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Giving Joy is a US-based nonprofit that strengthens and inspires women’s entrepreneurship worldwide. Through its micro-grants and mentorship program, Giving Joy helps women establish or improve their businesses and initiatives—for their benefit and the benefit of their communities. To date, Giving Joy has awarded over 88 grants to women-led initiatives in 26 countries.
@@ -1155,34 +1078,232 @@
 The grant period is six months.</t>
         </is>
       </c>
-      <c r="D10" s="1" t="inlineStr">
+      <c r="D11" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E10" s="1" t="inlineStr">
+      <c r="E11" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F10" s="1" t="inlineStr">
+      <c r="F11" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/application-invited-for-giving-joy-microgrant-giving-joy-opg-26-00185</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="95" customHeight="1">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="inlineStr">
+    <row r="12" ht="95" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>ToR - Branding Development &amp; Design/Market Promotion Consultant Project Sashakt</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>Organisation Humana People to People India (HPPI)
+Project Sashakt – Strengthening Women-led Handloom Cooperatives in Assam (EU-funded)
+Coverage 25 women-led handloom cooperatives, ~2,500 women artisans across Kamrup, Dhubri and Chirang districts
+Location Assam-based preferred; travel to Kamrup, Dhubri and Chirang required
+Duration 12 months from date of contract signing
+Monthly Professional Fee INR 1,25,000 (all-inclusive of fees, GST, travel, workshops, design revisions and reporting)
+Total Budget INR 15,00,000 (12 months × INR 1,25,000)
+Application Deadline 30 September 2026, by 5:00 PM IST
+How to Apply Email technical and financial proposals, with a design portfolio, to careers@human-india.org, subject line “Branding &amp; Market Promotion Consultancy – Project Sashakt”
+1. Background and Purpose
+HPPI is implementing Project Sashakt, an EU-supported initiative strengthening women-led handloom cooperatives and improving livelihoods for women weavers in Assam, using a Local2Global approach to market access. HPPI is seeking an Assam-based branding and design consultant/agency to build market-ready brand identities for cooperative products and the capacity of cooperatives to use and promote them — covering brand identity, naming, logo and packaging design, brand guidelines, and capacity building — to position products for wider regional, national and international visibility and strengthen the long-term sustainability of Assam's handloom sector.
+ 2. Scope of Work
+Product Development &amp; Diversification: work hands-on with a representative sample of weavers to assess current product range, quality and design variety, and pilot feasible new designs, variants or product use-cases within existing skills, looms and materials — establishing a sufficient, market-ready product range ahead of full brand rollout.
+Brand discovery: consult HPPI, cooperatives and artisans; study existing products, weaving traditions and motifs; assess current market positioning, branding gaps and differentiation opportunities in domestic and international markets.
+Brand development: create brand concepts, positioning and identity language; develop names for cooperative brands/product lines reflecting Assamese heritage and market relevance; design logos, typography, colour palettes, motifs, packaging concepts and product labels/tags.
+Branding toolkit: produce practical, reusable guidelines and templates — logo usage, packaging, social media, product catalogues and exhibition materials — for cooperatives to apply independently.
+Capacity building: run training workshops for cooperatives on brand usage and communication, and provide hands-on implementation support and mentoring during rollout across packaging, exhibitions, social media and product communication.
+Market promotion support: develop promotional materials for exhibitions/market events; advise on digital brand presence and storytelling; support Local2Global positioning for national and international audiences.
+ 3. Deliverables and Timeline
+# Deliverable Timeline
+1 Inception report and branding strategy roadmap Month 1
+2 Product development plan and prototype products with sampled cooperatives Months 1–2
+3 Market assessment and branding gap analysis Month 2
+4 Brand concepts, names and logo options Months 3–4
+5 Finalised brand identity packages Month 5
+6 Packaging and branding templates Month 6
+7 Brand usage and communication guidelines Month 7
+8 Training workshops for cooperatives Months 8–10
+9 Handholding support for implementation Months 9–12
+10 Final report with outcomes and recommendations Month 12
+4. Required Qualifications and Experience
+Proven experience in branding, communication design and visual identity development, with a strong design portfolio.
+Experience in product or textile design/diversification support for artisan producers at a nascent or early production stage — working within existing skills, looms and materials, in addition to branding expertise.
+Prior work with handloom, handicrafts, artisan collectives, MSMEs or rural enterprises preferred; strong understanding of Assamese culture, textiles and local markets.
+Experience in packaging design, market-oriented branding, and conducting training/capacity-building workshops.
+ 5. Selection Criteria
+Criteria Weightage
+Relevant experience 30%
+Quality of portfolio 25%
+Technical approach and methodology 25%
+Understanding of Assam's handloom sector 10%
+Financial proposal 10%
+6. Proposal Submission Requirements
+Technical proposal with detailed methodology and work plan
+Portfolio of relevant assignments
+Financial proposal and CV
+References from previous assignments
+ 7. Reporting and Expected Impact
+The consultant/agency will report to HPPI's designated Project Lead, work closely with cooperative representatives, and join weekly progress review meetings. The assignment is expected to deliver a stronger market identity, greater product visibility and sales potential, enhanced entrepreneurial capacity among women weavers, and a more sustainable handloom ecosystem through strategic branding and storytelling.
+ 8. Ethics and Confidentiality
+The consultant/agency must ensure ethical, consent-based data collection with cultural sensitivity, particularly when engaging women weavers. All data and reports remain the property of HPPI and must be kept strictly confidential, with no external use.</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>Sep 30, 2026</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/tor-branding-development-and-designmarket-promotion-consultant-project-sashakt-humana-people-to-people-india-rfp-26-00365</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="95" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Signals of Change Shaping the Future of Sexual and Reproductive Health and Rights SRHR</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+The World Health Organization's mission: to promote health, keep the world safe, and serve the vulnerable. Working through offices in more than 150 countries, WHO staff work side by side with governments and other partners to ensure the highest attainable level of health for all people.
+ About the Opportunity
+HRP and its UN co-sponsors are leading a global Sexual and Reproductive Health and Rights (SRHR) foresight and research prioritization process for 2026–2036. This open public consultation invites diverse stakeholder input to identify "signals of change" — emerging trends, shifts, or disruptions — that could shape the future of SRHR over the next decade. The process uses foresight methodology (not prediction) to explore plausible futures and will culminate in a published report and research agenda in 2027.
+ Guiding Questions
+What future trends will shape or constrain SRHR over the next 10 years?
+What evidence and research investments are needed today to prepare SRHR for the futures we may face?
+ Scope of Submissions 
+Economic systems; social infrastructure; structural discrimination; conflict/forced migration/displacement; mega-trends (demographic shifts, climate change, digital transformation/AI, urbanization); conditions of daily life; rights/legal/governance systems; health systems; media/misinformation; and changes in the research ecosystem.
+ Who Can Participate 
+Open to individuals and organizations globally, including:
+Health workers, professional associations, clinical networks
+Civil society, community groups, youth-led organizations, rights movements
+Governments, parliamentarians, regulators, public sector bodies
+Researchers, academia, think tanks, technical experts
+UN agencies, multilateral/humanitarian/development organizations
+Funders, philanthropy, private sector, tech/innovation organizations
+Media, communications, journalism
+Anyone with relevant lived experience or perspective
+Special interest in submissions from health worker, community, youth, and rights-movement spaces not typically represented in published forums.
+ Submission Requirements: Descriptive information (name, contact email, country, sector) required alongside each submission; formal published evidence is helpful but not required — practice-based experience and field examples are also welcome. Submissions are kept confidential and anonymized before analysis.</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>Sep 30, 2026</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-signals-of-change-shaping-the-future-of-sexual-and-reproductive-health-and-rights-srhr-world-health-organization-opg-26-00176</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="95" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Setting up Viral Research and Diagnosis Laboratories VRDL in Medical Colleges/Hospitals/Medical Institutions</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+The President notified the creation of the Department of Health Research under the Ministry of Health &amp; Family Welfare through an amendment to the Government of India (Allocation of Business) Rules, 1961 on the 17th September 2007. The Department of Health Research was formally launched on 5th October 2007 by the Minister for Science &amp; Technology and Earth Sciences in a function presided over by the Minister for Health &amp; Family Welfare, in the presence, inter-alia, of the Minister of State for Health &amp; Family Welfare.
+The Department became functional from November 2008 with the appointment of first Secretary of the Department The aim of the DHR is to bring modern health technologies to the people through research and innovations related to diagnosis, treatment methods and vaccines for prevention, to translate them into products and processes and, in synergy with concerned organizations, introduce these innovations into public health system.
+ About the Opportunity:
+Under DHR's scheme "Setting-up of nation-wide network of laboratories for managing epidemics and national calamities," proposals are invited from Medical Colleges/Hospitals/Research Institutions to establish a Medical College &amp; Research Institute Level – Viral Research and Diagnosis Laboratory (MCL-VRDL). The existing network comprises 167 VRDLs (11 Regional, 27 State, 129 Medical College level) across 27 states and 5 UTs, aimed at early detection of infectious pathogens, outbreak surveillance, and research on emerging/re-emerging viral diseases.
+ Objectives:
+Establish capacity for early detection of common and high-risk infectious pathogens
+Strengthen syndromic surveillance ecosystem for outbreak detection
+Undertake R&amp;D on emerging, re-emerging and novel viruses
+ Eligibility (Institution-level):
+State Government Medical Colleges
+Central Government Medical Colleges and Research Institutes
+Armed Forces Medical Institutions/Hospitals
+Railway and other Central Government health institutions
+Private medical colleges ranked in top 50 NIRF ranking
+Must have a dedicated Microbiology department with qualified faculty
+Must have &gt;200 sq.m. area available in existing building (preferably within Microbiology Dept.)
+ Funding Provision:
+Non-recurring assistance: Rs. 1.55 crore total
+Rs. 66.8 lakhs — Civil Work (infrastructure modification)
+Rs. 88.2 lakhs — Equipment (complete lab setup)
+No recurring expenditure (staff salaries, consumables, contingency) is provided — to be borne by the host institution
+ Role &amp; Responsibilities of the Lab:
+Conduct routine diagnosis of infectious pathogens
+Participate in syndromic and event-based surveillance
+Provide support during outbreaks/epidemics
+Share data with ICMR
+ Selection Criteria:
+Meeting eligibility does not guarantee selection; merit-based evaluation by a technical committee
+Preference to institutions in geographically underserved regions
+Weightage for technical strength (qualified faculty, biosafety practices, outbreak investigation experience, publications, patents, externally funded projects)
+Additional weightage for molecular diagnostics, genomic surveillance, One Health research capability, and commitment to long-term recurring support
+Private medical colleges: only top-50 NIRF-ranked institutions considered</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>Sep 30, 2026</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-setting-up-viral-research-and-diagnosis-laboratories-vrdl-in-medical-collegeshospitalsmedical-institutions-department-of-health-research-dhr-ministry-of-health-and-family-welfare-government-of-india-opg-26-00174</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="95" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>EOI Inviting Expression of Interest-cum-Proposal for Setting Up District De-Addiction Centres under NAPDDR</t>
         </is>
       </c>
-      <c r="C11" s="1" t="inlineStr">
+      <c r="C15" s="1" t="inlineStr">
         <is>
           <t>About us
 In the year 1985-86, the erstwhile Ministry of Welfare was bifurcated into the Department of Women and Child Development and the Department of Welfare. Simultaneously, the Scheduled Castes Development Division, Tribal Development Division and the Minorities and Backward Classes Welfare Division were moved from the Ministry of Home Affairs and also the Wakf Division from the Ministry of Law to form the then Ministry of Welfare Subsequently, the name of the Ministry was changed to the Ministry of Social Justice &amp; Empowerment in May, 1998. Further, in October, 1999, the Tribal Development Division had moved out to form a separate Ministry of Tribal Affairs. In January, 2007, the Minorities Division along with Wakf Unit have been moved out of the Ministry and formed as a separate Ministry and the Child Development Division has gone to the Ministry of Women &amp; Child Development.
@@ -1222,34 +1343,34 @@
 11. Department of Social Justice and Empowerment (DoSJE) reserves the right to cancel this notice, andior invite afresh proposals with or without amendments to this document without liability or any obligation for such document, and without assigning any reason. DoSJE reserves the right to take final decision regarding selection of implementing agency or project.</t>
         </is>
       </c>
-      <c r="D11" s="1" t="inlineStr">
+      <c r="D15" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E11" s="1" t="inlineStr">
+      <c r="E15" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F11" s="1" t="inlineStr">
+      <c r="F15" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/eoi-inviting-expression-of-interest-cum-proposal-for-setting-up-district-de-addiction-centres-under-napddr-ministry-of-social-justice-and-empowerment-goi-rfp-26-00356</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="95" customHeight="1">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="inlineStr">
+    <row r="16" ht="95" customHeight="1">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>RFP - Design and Delivery of an Electric Vehicle EV Skilling Programme in Karnataka</t>
         </is>
       </c>
-      <c r="C12" s="1" t="inlineStr">
+      <c r="C16" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 WRI India, an independent knowledge organisation registered as the India Resources Trust, provides objective information and practical proposals to foster environmentally sound and socially equitable development. As an independent knowledge organisation, we leverage our data and expertise to catalyze change across systems like food, land and water; energy; and cities. Our work focuses on improving people’s lives, protecting and restoring nature, and addressing climate change. To enable progress at the pace and scale needed, we also engage with the economic, finance and governance systems that are key to enabling this change.
@@ -1290,34 +1411,34 @@
 Must have a team of qualified trainers and master trainers with relevant domain expertise, as well as administrative and coordination support.</t>
         </is>
       </c>
-      <c r="D12" s="1" t="inlineStr">
+      <c r="D16" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E12" s="1" t="inlineStr">
+      <c r="E16" s="1" t="inlineStr">
         <is>
           <t>Oct 5, 2026</t>
         </is>
       </c>
-      <c r="F12" s="1" t="inlineStr">
+      <c r="F16" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfp-design-and-delivery-of-an-electric-vehicle-ev-skilling-programme-in-karnataka-wri-india-rfp-26-00361</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="95" customHeight="1">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B13" s="1" t="inlineStr">
+    <row r="17" ht="95" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
         <is>
           <t>Applications Open Draper Richards Kaplan Foundation Funding for Social Enterprises</t>
         </is>
       </c>
-      <c r="C13" s="1" t="inlineStr">
+      <c r="C17" s="1" t="inlineStr">
         <is>
           <t>About us
 Started in 2002, Draper Richards Kaplan Foundation (DRK) is a global venture philanthropy firm supporting early stage, high impact social enterprises. Borrowed from our venture capital legacy, DRK finds, funds, and supports exceptional leaders building innovative solutions to some of the world’s most challenging social and environmental problems. Since beginning this work nearly 25 years ago, DRK has invested in more than 270 organizations that have collectively impacted over 610 million lives to date.
@@ -1341,34 +1462,34 @@
 Please attach a standard resume/CV for the entrepreneur(s) and/or key leadership team members (e.g., CEO, COO, ED, etc.). Applications with text bios for entrepreneurs or members of the leadership team will not be considered.</t>
         </is>
       </c>
-      <c r="D13" s="1" t="inlineStr">
+      <c r="D17" s="1" t="inlineStr">
         <is>
           <t>Climate</t>
         </is>
       </c>
-      <c r="E13" s="1" t="inlineStr">
+      <c r="E17" s="1" t="inlineStr">
         <is>
           <t>Oct 10, 2026</t>
         </is>
       </c>
-      <c r="F13" s="1" t="inlineStr">
+      <c r="F17" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-open-draper-richards-kaplan-foundation-funding-for-social-enterprises-draper-richards-kaplan-foundation-opg-26-00188</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="95" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="inlineStr">
+    <row r="18" ht="95" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund</t>
         </is>
       </c>
-      <c r="C14" s="1" t="inlineStr">
+      <c r="C18" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund
 Apply by: 13 October, 2026
@@ -1393,34 +1514,34 @@
  Projects should include opportunities for ServiceNow employees to volunteer in the project activation or implementation.</t>
         </is>
       </c>
-      <c r="D14" s="1" t="inlineStr">
+      <c r="D18" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E14" s="1" t="inlineStr">
+      <c r="E18" s="1" t="inlineStr">
         <is>
           <t>Oct 13, 2026</t>
         </is>
       </c>
-      <c r="F14" s="1" t="inlineStr">
+      <c r="F18" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/apply-for-the-servicenow-community-solar-fund-changex-opg-26-00186</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="95" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="inlineStr">
+    <row r="19" ht="95" customHeight="1">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>ToR - Engagement of Consultant/Vendor Individual towards implementation of Literacy Program in Telangana State</t>
         </is>
       </c>
-      <c r="C15" s="1" t="inlineStr">
+      <c r="C19" s="1" t="inlineStr">
         <is>
           <t>ANNEX A – TERMS OF REFERENCE (ToR) 
  Engagement of Consultant/Vendor (Individual) towards implementation of Literacy Program in Telangana State.
@@ -1485,34 +1606,34 @@
 Approved travel and accommodation expenses incurred for assignment-related activities shall be reimbursed by Room to Read in accordance with the consultancy reimbursement guidelines.</t>
         </is>
       </c>
-      <c r="D15" s="1" t="inlineStr">
+      <c r="D19" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E15" s="1" t="inlineStr">
+      <c r="E19" s="1" t="inlineStr">
         <is>
           <t>Oct 16, 2026</t>
         </is>
       </c>
-      <c r="F15" s="1" t="inlineStr">
+      <c r="F19" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-engagement-of-consultantvendor-individual-towards-implementation-of-literacy-program-in-telangana-state-room-to-read-india-rfp-26-00360</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="95" customHeight="1">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B16" s="1" t="inlineStr">
+    <row r="20" ht="95" customHeight="1">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>RFPs Invited for Consultant to Develop a Technical Assistance Package for National Application of the Digital Health and AI Investment Classification Framework</t>
         </is>
       </c>
-      <c r="C16" s="1" t="inlineStr">
+      <c r="C20" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are Transform Health: a global coalition of more than 200 organisations driving the digital transformation of health to achieve universal health coverage. 
@@ -1540,34 +1661,34 @@
 Ability to manage multi-country consultancy engagements and coordinate with in-country focal points</t>
         </is>
       </c>
-      <c r="D16" s="1" t="inlineStr">
+      <c r="D20" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E16" s="1" t="inlineStr">
+      <c r="E20" s="1" t="inlineStr">
         <is>
           <t>Oct 23, 2026</t>
         </is>
       </c>
-      <c r="F16" s="1" t="inlineStr">
+      <c r="F20" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfps-invited-for-consultant-to-develop-a-technical-assistance-package-for-national-application-of-the-digital-health-and-ai-investment-classification-framework-transform-health-rfp-26-00359</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="95" customHeight="1">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B17" s="1" t="inlineStr">
+    <row r="21" ht="95" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Comparison of PFAS Contributions to Agricultural Systems</t>
         </is>
       </c>
-      <c r="C17" s="1" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>Project Objectives:
 Report per- and polyfluoroalkyl substance (PFAS) concentrations from a variety of agricultural inputs — animal manures, fertilizers, pesticides, composts, soil amendments, seed coatings, and biosolids-based products
@@ -1603,34 +1724,124 @@
  Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00) — same deadline as the other two WRF grants</t>
         </is>
       </c>
-      <c r="D17" s="1" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E17" s="1" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F17" s="1" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-comparison-of-pfas-contributions-to-agricultural-systems-the-water-research-foundation-wrf-opg-26-00190</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="95" customHeight="1">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="inlineStr">
+    <row r="22" ht="95" customHeight="1">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for 8th Call for Proposals Small-Size Grants Global EbA Fund</t>
+        </is>
+      </c>
+      <c r="C22" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
+ About the Opportunity:
+The Global EbA Fund invites innovative and catalytic proposals that address systemic barriers to Ecosystem-based Adaptation (EbA) scaling — by enhancing institutional and technical capacities, quality data/evidence generation, learning networks, and investment readiness. Aligned with the IKI Strategy up to 2030 (focus on socio-ecological transformation), the Fund's primary geographic focus is ODA-eligible SIDS (Small Island Developing States) and LDCs (Least Developed Countries), though other ODA-eligible countries may be considered where proposals show exceptional ambition.
+ Focus Areas:
+Overcoming upstream barriers to EbA uptake/scaling (institutional &amp; technical capacity constraints, evidence generation, knowledge exchange)
+Clear adaptation chain grounded in detailed impact chain analysis (climate hazards/risks, socioeconomic/ecological sensitivity, adaptive capacity)
+Social and environmental considerations (gender responsiveness, Indigenous Peoples' rights, local participation, environmental/social safeguards, prevention of maladaptation)
+Robust sustainability and exit strategies (long-term viability, local ownership, institutional continuity)
+ Encouraged Topics:
+Investment readiness and project pipeline preparation
+Innovative technologies for EbA
+Applied and functional research
+Synergies with other EbA/Nature-based Solution (NbS) initiatives
+ Grant Size: Up to USD 250,000 per grant
+ Project Duration: Up to 24 months
+ Eligible Applicant Types:
+Non-governmental organisations (NGOs)
+International NGOs (INGOs)
+Intergovernmental organisations (IGOs)
+Community-based organisations (CBOs)
+Indigenous People's Organisations
+Universities and academic institutions
+Research institutes and think tanks
+Private sector companies (under certain conditions; no funding for sector-specific obligations, compensatory measures, or for-profit activities)
+Consortia (must designate a clear lead "Applicant Organisation"; government entities can join a consortium but cannot receive Fund money directly)
+Note: Individuals are not eligible (e.g., no PhD study funding); UNEP and IUCN offices are also not eligible to apply.
+ Key Eligibility Criteria:
+Must qualify as Ecosystem-based Adaptation (EbA) per the Fund's Qualification Criteria &amp; Quality Standards
+Must have catalytic/innovative potential
+Must clearly identify climate impacts addressed
+Falls under max 1 Strategic Objective and max 2 Action Pillars of the Fund
+Global, thematic, or targets only ODA-eligible countries
+Budget up to USD 250,000; duration up to 24 months
+Must build on existing work (not standalone/field-implementation-only projects)
+Must show sustainability post-funding
+Must partner with local institutions
+Applicant &amp; partners must be legally recognized entities with relevant experience
+Must complete Due Diligence requirements
+ Evaluation Criteria (weighted):
+Ecosystem-based Adaptation (EbA) approach — 30%
+Design &amp; Methodology (Theory of Change, logframe, SMART indicators, budget coherence)
+Gender &amp; Social Inclusion (participatory approach, FPIC for Indigenous Peoples' impact)
+Innovative &amp; Catalytic Contribution — 30%
+Sustainability — 20%
+Institutional Arrangements — 20%
+ Reporting Requirement: Applicants must identify at least 3 indicators from the Fund's Core Indicator Framework for their project's logframe.
+ Application Package Required:
+Applicant Declaration
+Co-applicant Mandate (if applicable)
+Small-Size Grants Application Form
+Project Proposal Budget Template
+Due Diligence and Financial Capacity Questionnaire (with Annexes 1(c)(i) and 1(c)(ii) at submission stage)
+ Application Language: English only (organizational documents must be translated to English
+ Timeline:
+Call officially launched: August 24, 2026
+Submission window: September 28 – October 26, 2026
+Applications submitted via online portal (link shared on the Small-Size Grants webpage from Sept 28)
+Only successful applicants will be contacted; no individual feedback provided to unsuccessful applicants</t>
+        </is>
+      </c>
+      <c r="D22" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E22" s="1" t="inlineStr">
+        <is>
+          <t>Oct 26, 2026</t>
+        </is>
+      </c>
+      <c r="F22" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-8th-call-for-proposals-small-size-grants-global-eba-fund-global-eba-fund-opg-26-00177</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="95" customHeight="1">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Adaptive Control Frameworks to Unlock Full-Scale BNR Potential Water Research Foundation WRF</t>
         </is>
       </c>
-      <c r="C18" s="1" t="inlineStr">
+      <c r="C23" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Water Research Foundation (WRF) is the leading research organization advancing the science of all water to meet the evolving needs of its subscribers and the water sector. WRF is a nonprofit, charitable and educational organization which funds, manages, and publishes research on the technology, operation, and management of drinking water, wastewater, reuse, and stormwater collection, treatment and supply systems—all in pursuit of ensuring water quality and improving water services to the public.
@@ -1671,34 +1882,34 @@
 Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
         </is>
       </c>
-      <c r="D18" s="1" t="inlineStr">
+      <c r="D23" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E18" s="1" t="inlineStr">
+      <c r="E23" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F18" s="1" t="inlineStr">
+      <c r="F23" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-adaptive-control-frameworks-to-unlock-full-scale-bnr-potential-water-research-foundation-wrf-the-water-research-foundation-wrf-opg-26-00187</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="95" customHeight="1">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="inlineStr">
+    <row r="24" ht="95" customHeight="1">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Crossing the Divide Best Practices for Addressing Local and Privately-Owned Lateral Sewer Issues RFP 5419</t>
         </is>
       </c>
-      <c r="C19" s="1" t="inlineStr">
+      <c r="C24" s="1" t="inlineStr">
         <is>
           <t>Project Objective:
 To provide water resource recovery facilities (WRRFs) and collection system operators with an interactive manual of practice for implementing inflow and infiltration (I&amp;I) and obstruction management programs, focused on municipal and privately owned lateral sewers in complex legal, regulatory, and multi-jurisdictional environments.
@@ -1736,34 +1947,74 @@
  Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
         </is>
       </c>
-      <c r="D19" s="1" t="inlineStr">
+      <c r="D24" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E19" s="1" t="inlineStr">
+      <c r="E24" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F19" s="1" t="inlineStr">
+      <c r="F24" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-crossing-the-divide-best-practices-for-addressing-local-and-privately-owned-lateral-sewer-issues-rfp-5419-the-water-research-foundation-wrf-opg-26-00189</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="95" customHeight="1">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="inlineStr">
+    <row r="25" ht="95" customHeight="1">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Whitley Award 2027</t>
+        </is>
+      </c>
+      <c r="C25" s="1" t="inlineStr">
+        <is>
+          <t>About the Grant: 
+An annual grant by the Whitley Fund for Nature (WFN) recognising grassroots conservation leaders in the Global South, providing funding to support and scale up proven, science-based solutions that deliver lasting impact for both people and nature.
+ About the Award 
+Whitley Awards support grassroots conservation leaders in the Global South. Through funding, training and profile, they help conservationists scale up effective projects that are founded in science and carried out with communities. Whitley Awards are for dynamic, mid-career conservationists who are leading vital conservation projects.
+ Grant Amount: £50,000 in project funding over one year
+ Eligibility
+Winners are nationals of the country in which they are working, seeking to scale up proven work that is embedded in the local community and would benefit from further funding, a profile boost, and international support.
+Projects must involve communities at the grassroots level and deliver practical action that is founded on science.
+You do not need to be invited or nominated to apply.</t>
+        </is>
+      </c>
+      <c r="D25" s="1" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E25" s="1" t="inlineStr">
+        <is>
+          <t>Oct 30, 2026</t>
+        </is>
+      </c>
+      <c r="F25" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-whitley-award-2027-whitley-fund-for-nature-wfn-opg-26-00153</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="95" customHeight="1">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIFAR Global Scholars Program 20272029 Cohort</t>
         </is>
       </c>
-      <c r="C20" s="1" t="inlineStr">
+      <c r="C26" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 CIFAR is a Canadian-based globally influential research organization that convenes the world’s most brilliant people across disciplines to advance transformative knowledge and solve humanity’s biggest problems, together. By supporting long-term interdisciplinary collaboration, CIFAR provides researchers with an unparalleled environment of trust, transparency and knowledge sharing. Our time-tested model inspires new directions of inquiry, accelerates discovery and yields breakthroughs across borders and academic disciplines. Through knowledge mobilization, we are catalysts for change in industry, government and society. Through our 15 research programs and the Pan-Canadian AI Strategy, CIFAR convenes close to 400 of the world’s top researchers from 141 institutions in 20 countries. CIFAR is generously supported by the governments of Canada, Alberta and Québec, as well as foundations, individuals, corporations and Canadian and international partner organizations.
@@ -1807,34 +2058,115 @@
  Application Deadline: November 4, 2026, 12:00 PM EST</t>
         </is>
       </c>
-      <c r="D20" s="1" t="inlineStr">
+      <c r="D26" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E20" s="1" t="inlineStr">
+      <c r="E26" s="1" t="inlineStr">
         <is>
           <t>Nov 4, 2026</t>
         </is>
       </c>
-      <c r="F20" s="1" t="inlineStr">
+      <c r="F26" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cifar-global-scholars-program-20272029-cohort-cifar-canadian-institute-for-advanced-research-opg-26-00183</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="95" customHeight="1">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="inlineStr">
+    <row r="27" ht="95" customHeight="1">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for IWRS Teaching Innovation Award</t>
+        </is>
+      </c>
+      <c r="C27" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+Insects are one of the most numerous and diverse animal groups on Earth.
+Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice.
+About the Award
+The IWRS Teaching Innovation Award supports instructors developing new approaches to teaching invertebrate biology that incorporate the 3Rs (replacement, reduction, and refinement). It also supports the development and implementation of any novel curricula addressing invertebrate welfare and sentience across invertebrate biology, animal welfare science, and/or veterinary medicine fields.
+Grant size
+Awards up to $2,000 USD are available for approaches requiring equipment or other materials; awards up to $1,000 USD are available otherwise. Funds may be used to support any costs associated with curriculum development and implementation, including stipends, teaching tools, and related expenses. Priority is given to proposals addressing common teaching practices with substantial welfare implications.
+Who can apply for funding?
+The applicant must be an instructor teaching content related to insect or invertebrate biology at an educational institution, scientific society or museum, field-training course, or similar educational context. If you are unsure about your eligibility, contact grants@insectwelfare.com.
+The applicant can be from any discipline, country, or institution. However, we will not pay awards to recipients located in jurisdictions, countries, or regions subject to trade restrictions, embargoes, or sanctions put in place by the United Nations or the United States of America.
+IWRS staff and Advisory Group members are not eligible to apply.</t>
+        </is>
+      </c>
+      <c r="D27" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E27" s="1" t="inlineStr">
+        <is>
+          <t>Nov 15, 2026</t>
+        </is>
+      </c>
+      <c r="F27" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00166</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="95" customHeight="1">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for IWRS Teaching Innovation Award</t>
+        </is>
+      </c>
+      <c r="C28" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
+ About the Grant
+The IWRS (Insect Welfare Research Society) Teaching Innovation Award supports instructors developing new approaches to teaching insect or invertebrate biology that incorporate the 3Rs (Replacement, Reduction, and Refinement) — principles for reducing animal welfare impacts in teaching and research practices.
+ Purpose
+Funds support the creation and implementation of 3Rs-driven instructional materials and pedagogical approaches. Priority is given to proposals addressing common teaching practices with substantial welfare implications.
+ Grant Amount
+Two awards of $2,000 USD are available annually.</t>
+        </is>
+      </c>
+      <c r="D28" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E28" s="1" t="inlineStr">
+        <is>
+          <t>Nov 15, 2026</t>
+        </is>
+      </c>
+      <c r="F28" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="95" customHeight="1">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Medium-Size Grants Call for Proposals Global EbA Fund</t>
         </is>
       </c>
-      <c r="C21" s="1" t="inlineStr">
+      <c r="C29" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -1891,34 +2223,88 @@
 Applications submitted via online portal (link shared on the Medium-Size Grants webpage from Oct 12)</t>
         </is>
       </c>
-      <c r="D21" s="1" t="inlineStr">
+      <c r="D29" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E21" s="1" t="inlineStr">
+      <c r="E29" s="1" t="inlineStr">
         <is>
           <t>Nov 16, 2026</t>
         </is>
       </c>
-      <c r="F21" s="1" t="inlineStr">
+      <c r="F29" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-medium-size-grants-call-for-proposals-global-eba-fund-global-eba-fund-opg-26-00178</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="95" customHeight="1">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="inlineStr">
+    <row r="30" ht="95" customHeight="1">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for CIEIF Grant 2026 Climate Intervention Environmental Impact Fund</t>
+        </is>
+      </c>
+      <c r="C30" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+Climate Intervention Environmental Impact Fund (CIEIF) is a philanthropic fund focused on supporting responsible climate intervention field tests. It provides grants for activities such as environmental impact assessment (EIA), predictive impact modelling, and engagement with potentially affected stakeholders, including local communities and government agencies.
+CIEIF aims to help climate-intervention projects better understand their potential technical, environmental, economic, social, public-health, and safety impacts before and during field testing. It also places importance on the scalability and global relevance of supported innovations and encourages publication of field-test results through peer-reviewed journals or externally peer-reviewed reports.
+ About the Grant
+The Climate Intervention Environmental Impact Fund (CIEIF) Grant provides USD 75,000 to support proposed climate intervention field tests. The funding is specifically intended for Environmental Impact Assessment (EIA), predictive impact modelling, and/or engagement with potentially affected stakeholders, including local communities and government agencies.
+Applicants are expected to demonstrate the proposed field test’s technical readiness, environmental and social considerations, required government approvals, innovation and potential for globally relevant scalability. The application must include a proposed budget showing how the USD 75,000 will be used.
+ Grant Objective
+The grant is intended to support proposed climate intervention field tests, particularly activities related to:
+Environmental Impact Assessment (EIA)
+Predictive impact modeling
+Engagement with potentially impacted stakeholders
+Local community and government engagement
+Understanding technical, environmental, economic, social, public-health, and safety challenges
+The proposed application must focus on at least one of these three core areas: EIA, predictive impact modeling, or stakeholder engagement.
+ Eligible Project Focus
+The proposed field test should demonstrate:
+A clear climate-intervention concept
+Prior research indicating that the technology is ready for the proposed field test
+Potential for innovation and scalability
+A clear understanding of technical and environmental challenges
+Consideration of economic, social, public-health, and safety implications
+Relevant government permits and approvals
+Potential for scaling the innovation to a globally relevant level</t>
+        </is>
+      </c>
+      <c r="D30" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E30" s="1" t="inlineStr">
+        <is>
+          <t>Dec 1, 2026</t>
+        </is>
+      </c>
+      <c r="F30" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-cieif-grant-2026-climate-intervention-environmental-impact-fund-climate-intervention-environmental-impact-fund-opg-26-00155</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="95" customHeight="1">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 6th Annual Seeding The Future Global Food System Challenge</t>
         </is>
       </c>
-      <c r="C22" s="1" t="inlineStr">
+      <c r="C31" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are one of the largest and most respected private organisations for development cooperation and humanitarian aid in Germany. As a politically and confessionally independent organisation, our value-oriented actions are always based on ethical principles. Our vision is clear: "Zero Hunger by 2030"
@@ -1950,34 +2336,34 @@
 Individuals with no organizational entity</t>
         </is>
       </c>
-      <c r="D22" s="1" t="inlineStr">
+      <c r="D31" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E22" s="1" t="inlineStr">
+      <c r="E31" s="1" t="inlineStr">
         <is>
           <t>Jan 1, 2027</t>
         </is>
       </c>
-      <c r="F22" s="1" t="inlineStr">
+      <c r="F31" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-6th-annual-seeding-the-future-global-food-system-challenge-welthungerhilfe-opg-26-00180</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="95" customHeight="1">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B23" s="1" t="inlineStr">
+    <row r="32" ht="95" customHeight="1">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B32" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for BES Training and Travel Grants</t>
         </is>
       </c>
-      <c r="C23" s="1" t="inlineStr">
+      <c r="C32" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are a global community of scientists shining a spotlight on the intricacy and value of our natural world, providing the evidence for better decisions. Our vision is for people and nature to thrive in a world that values ecology.
@@ -2016,17 +2402,17 @@
  Application Deadline (Round 2): Opens 30 April 2026, closes 17 May 2026</t>
         </is>
       </c>
-      <c r="D23" s="1" t="inlineStr">
+      <c r="D32" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E23" s="1" t="inlineStr">
+      <c r="E32" s="1" t="inlineStr">
         <is>
           <t>May 17, 2027</t>
         </is>
       </c>
-      <c r="F23" s="1" t="inlineStr">
+      <c r="F32" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-bes-training-and-travel-grants-british-ecological-society-opg-26-00181</t>
         </is>

</xml_diff>

<commit_message>
Auto update Combined.xlsx [Sun Sep 20 07:23:48 UTC 2026]
</commit_message>
<xml_diff>
--- a/output/Combined.xlsx
+++ b/output/Combined.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -467,56 +467,10 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Applications Invited for Wellbeing Research Grants Funding Better Evaluations of AI's Impact on Wellbeing</t>
+          <t>ToR for Stand post - Varanasi</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-We're an AI research company that builds reliable, interpretable, and steerable AI systems. Our first product is Claude, an AI assistant for tasks at any scale. Our research interests span multiple areas including natural language, human feedback, scaling laws, reinforcement learning, code generation, and interpretability. 
- About the Opportunity:
-Anthropic is launching a $5 million grant program to fund independent research into how AI impacts users' wellbeing. The program will provide direct funding, access to Anthropic's models, and technical support to grantees building open-source evaluations that help the AI industry measure how models affect those who use them. Grantees will work fully independently, and will publish their work as open-source projects that any developer can make use of.
- Background/Rationale:
-AI systems have become central to how many people work, learn, and solve problems, and have also become conversational partners and sources of emotional support during difficult times, but the industry is still developing clear standards for how models should behave in such conversations — for example when a user seeks companionship or navigates a mental health crisis. Wellbeing is described as a particularly difficult area to evaluate, since assessing it requires more context than checking a single response for accuracy — the need for a cautious response may only become clear over a long conversation, and a response reasonable in one context could be harmful in another. By funding independent evaluations and benchmarks of user wellbeing, Anthropic hopes to invite more people — including clinicians, psychologists, and methodologists — to contribute to this field. 
- What They're Looking For
-Grantees should build evaluations that:
-State clearly what they are measuring (what counts as a pass or fail, and why it matters) 
-Involve clinical and subject-matter experts in the design and validation 
-Test both precautions and harms (i.e., evaluate the risk of both overcompliance and overrefusal) 
-Reflect how users actually use AI, often through multi-turn conversation scenarios where risk escalates and context shifts
-Validate their graders against real subject-matter experts 
- Eligibility/Target Applicants: Independent researchers — clinicians, psychologists, methodologists, and other subject-matter experts working on AI wellbeing evaluation/benchmarking
- Funding Amount: Total program pool of $5 million (individual grant sizes not specified on the page)</t>
-        </is>
-      </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>Learning</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>Sep 21, 2026</t>
-        </is>
-      </c>
-      <c r="F2" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-wellbeing-research-grants-funding-better-evaluations-of-ais-impact-on-wellbeing-anthropic-opg-26-00175</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="95" customHeight="1">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>ToR for Stand post - Varanasi</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Background
 Access to safe and reliable drinking water remains a critical challenge in several habitations of Harahua Block in Varanasi District, Uttar Pradesh. Although the Government of India, through the Jal Jeevan Mission (JJM), is expanding piped water supply, many marginalized settlements continue to face inadequate access to potable water due to limited household connections, inadequate storage infrastructure, and uneven water distribution.
@@ -564,89 +518,34 @@
 5</t>
         </is>
       </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>Sep 22, 2026</t>
         </is>
       </c>
-      <c r="F3" s="1" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-for-stand-post-varanasi-wateraid-india-rfp-26-00364</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="95" customHeight="1">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>SoW - Hiring an External Agency for Orientation and Capacity Building</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>Room to Read’s Foundational Literacy Program in Jharkhand
-Anchoring and Delivery of Orientation Programme for Jharkhand Field Workforce
-Scope of Work (SoW)
-for
-Hiring an External Agency for Orientation and Capacity Building
-Organizational Overview
- Founded in 2000 on the belief that World Change Starts with Educated Children®, Room to Read develops children’s foundational literacy skills, as well as life skills that promote gender equality. We nurture these essential skills in children by training and coaching educators, creating quality learning materials and spaces, strengthening education systems, and delivering programs directly and with partners – all while honouring the dignity of every child. Committed to accelerating learning outcomes for more children, more quickly, Room to Read has benefited children across 29 countries, with more than 17 million children actively benefiting from our programming in 2025 alone. Room to Read India’s literacy operations currently span across 12 states, with a focus on improving children’s reading skills, access to quality learning materials, and supportive learning environments. Room to Read envisions a world free from illiteracy and gender inequality, where all children have room to read, learn and grow. Visit us at https://www.roomtoreadindia.org/
-Jharkhand Foundational Literacy Project Overview
- Room to Read is preparing for a significant scale-up of its Foundational Literacy &amp; Numeracy initiative in Jharkhand, expanding implementation across multiple districts and requiring a substantial field workforce to support programme delivery. As Room to Read expands its field implementation in Jharkhand, a substantial number of staff will join different field-facing and supervisory roles.  As part of the planned scale-up, Room to Read expects to onboard more than 150 staff in Phase 1 across field implementation, supervisory and district-level leadership roles. A second cohort of approximately 120 additional staff is expected to be onboarded in Phase 2 as implementation expands to the remaining districts.
- Objective of the Assignment
-The overarching objective of this assignment is to ensure that over two phases 250+ team members in Jharkhand are ready for project implementation.
-Phase 1 will aim at getting all 150+ staff members ready for project implementation by March 31st, 2027.
-Phase 2 will follow the same approach for an additional 120+ team members, with the orientation programme to be completed by 30 March 2028, followed by final review, handover and closure activities in April 2028.
-Agency Requirements &amp; Qualifications 
-The agency should preferably:
-Preferred 3 years of relevant experience in designing and delivering orientation, training or capability-building programmes for field-based teams, particularly in the education, development or government-facing sector.
-Have completed at least 2 similar assignments involving training across multiple batches, locations or large participant groups.
-Demonstrate experience in learning-needs assessment, adult-learning design, content development and participatory training methodologies.
-Demonstrate experience in developing facilitator guides, participant materials, simulations, assessments, job aids or other training resources, and provide 1-2 relevant samples where available.
-Have the ability to deliver training in Hindi and deploy an adequate pool of suitable facilitators for implementation across Jharkhand.
-Provide details and CVs of the proposed core team and key facilitators, including their qualifications, relevant experience, roles and expected level of engagement in the assignment. The agency should ensure continuity of key facilitators, with minimal changes during each phase of the assignment.
-Demonstrate experience in assessing training effectiveness through participant feedback, assessments, learning-progress tracking and/or follow-up or refresher support.
-Have established systems for project management, quality assurance, documentation, progress tracking and reporting, with the ability to maintain consistency across training cohorts.
-Provide details of at least 2 relevant past clients/assignments that may be referred to for verification of experience and performance</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="inlineStr">
-        <is>
-          <t>Sep 23, 2026</t>
-        </is>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/sow-hiring-an-external-agency-for-orientation-and-capacity-building-room-to-read-india-rfp-26-00366</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="95" customHeight="1">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
+    <row r="3" ht="95" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for GEF SGP CSO Challenge Program</t>
         </is>
       </c>
-      <c r="C5" s="1" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global Environment Facility Small Grants Programme (SGP) is a global initiative implemented by the United Nations Development Programme (UNDP) on behalf of the Global Environment Facility (GEF). Since its launch in 1992, SGP has empowered communities worldwide to take action on environmental challenges while improving livelihoods. As a GEF Corporate Programme, SGP provides direct support to civil society organisations and community-based organisations to design and implement innovative, locally driven solutions. The programme places strong emphasis on inclusion, ensuring meaningful participation of Indigenous Peoples, youth, women and girls, and other underrepresented groups.
@@ -695,34 +594,89 @@
 Risk management and mitigation</t>
         </is>
       </c>
-      <c r="D5" s="1" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E5" s="1" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Sep 23, 2026</t>
         </is>
       </c>
-      <c r="F5" s="1" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-gef-sgp-cso-challenge-program-gef-small-grants-programme-sgp-opg-26-00184</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="95" customHeight="1">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
+    <row r="4" ht="95" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>SoW - Hiring an External Agency for Orientation and Capacity Building</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Room to Read’s Foundational Literacy Program in Jharkhand
+Anchoring and Delivery of Orientation Programme for Jharkhand Field Workforce
+Scope of Work (SoW)
+for
+Hiring an External Agency for Orientation and Capacity Building
+Organizational Overview
+ Founded in 2000 on the belief that World Change Starts with Educated Children®, Room to Read develops children’s foundational literacy skills, as well as life skills that promote gender equality. We nurture these essential skills in children by training and coaching educators, creating quality learning materials and spaces, strengthening education systems, and delivering programs directly and with partners – all while honouring the dignity of every child. Committed to accelerating learning outcomes for more children, more quickly, Room to Read has benefited children across 29 countries, with more than 17 million children actively benefiting from our programming in 2025 alone. Room to Read India’s literacy operations currently span across 12 states, with a focus on improving children’s reading skills, access to quality learning materials, and supportive learning environments. Room to Read envisions a world free from illiteracy and gender inequality, where all children have room to read, learn and grow. Visit us at https://www.roomtoreadindia.org/
+Jharkhand Foundational Literacy Project Overview
+ Room to Read is preparing for a significant scale-up of its Foundational Literacy &amp; Numeracy initiative in Jharkhand, expanding implementation across multiple districts and requiring a substantial field workforce to support programme delivery. As Room to Read expands its field implementation in Jharkhand, a substantial number of staff will join different field-facing and supervisory roles.  As part of the planned scale-up, Room to Read expects to onboard more than 150 staff in Phase 1 across field implementation, supervisory and district-level leadership roles. A second cohort of approximately 120 additional staff is expected to be onboarded in Phase 2 as implementation expands to the remaining districts.
+ Objective of the Assignment
+The overarching objective of this assignment is to ensure that over two phases 250+ team members in Jharkhand are ready for project implementation.
+Phase 1 will aim at getting all 150+ staff members ready for project implementation by March 31st, 2027.
+Phase 2 will follow the same approach for an additional 120+ team members, with the orientation programme to be completed by 30 March 2028, followed by final review, handover and closure activities in April 2028.
+Agency Requirements &amp; Qualifications 
+The agency should preferably:
+Preferred 3 years of relevant experience in designing and delivering orientation, training or capability-building programmes for field-based teams, particularly in the education, development or government-facing sector.
+Have completed at least 2 similar assignments involving training across multiple batches, locations or large participant groups.
+Demonstrate experience in learning-needs assessment, adult-learning design, content development and participatory training methodologies.
+Demonstrate experience in developing facilitator guides, participant materials, simulations, assessments, job aids or other training resources, and provide 1-2 relevant samples where available.
+Have the ability to deliver training in Hindi and deploy an adequate pool of suitable facilitators for implementation across Jharkhand.
+Provide details and CVs of the proposed core team and key facilitators, including their qualifications, relevant experience, roles and expected level of engagement in the assignment. The agency should ensure continuity of key facilitators, with minimal changes during each phase of the assignment.
+Demonstrate experience in assessing training effectiveness through participant feedback, assessments, learning-progress tracking and/or follow-up or refresher support.
+Have established systems for project management, quality assurance, documentation, progress tracking and reporting, with the ability to maintain consistency across training cohorts.
+Provide details of at least 2 relevant past clients/assignments that may be referred to for verification of experience and performance</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Sep 23, 2026</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/sow-hiring-an-external-agency-for-orientation-and-capacity-building-room-to-read-india-rfp-26-00366</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="95" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>RFP for Impact Assessment</t>
         </is>
       </c>
-      <c r="C6" s="1" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>Introduction
 Titan Company Limited, a member of the Tata Group, has a long-standing commitment to Corporate Social Responsibility (CSR) in India. The company's CSR initiatives derive its philosophy from the Company’s vision statement: “We create elevating experiences for the people we touch and significantly impact the world we work in”. The initiatives are designed to promote inclusive growth, empower communities, and contribute to the country's socio-economic development. The program includes Titan’s CSR policy is governed by a dedicated CSR Committee that ensures transparency and compliance with regulatory requirements. The program includes Girl Child Education, Skill and Entrepreneurship Development, supporting Indian Heritage Arts and Crafts, Integrated Village Development Programme, Eye Care and Affirmative Action. Titan's CSR policy is governed by a dedicated CSR Committee that ensures transparency and compliance with regulatory requirements.
@@ -756,34 +710,34 @@
 Timeline: Proposal submission deadline: September 24, 2026</t>
         </is>
       </c>
-      <c r="D6" s="1" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E6" s="1" t="inlineStr">
+      <c r="E5" s="1" t="inlineStr">
         <is>
           <t>Sep 24, 2026</t>
         </is>
       </c>
-      <c r="F6" s="1" t="inlineStr">
+      <c r="F5" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfp-for-impact-assessment-titan-rfp-26-00354</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="95" customHeight="1">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
+    <row r="6" ht="95" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>EOI- Engagement of State-Level Field Facilitation Consultants for Project Learning StudyEOI</t>
         </is>
       </c>
-      <c r="C7" s="1" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>Expression of Interest (EOI)
 For
@@ -844,34 +798,34 @@
 This stage is for collecting information from interested Consultant. AIFT will review the submissions and may issue a detailed Request for Quotation (RFQ) to shortlisted consultant based on the specific assignments.</t>
         </is>
       </c>
-      <c r="D7" s="1" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E7" s="1" t="inlineStr">
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>Sep 25, 2026</t>
         </is>
       </c>
-      <c r="F7" s="1" t="inlineStr">
+      <c r="F6" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/eoi-engagement-of-state-level-field-facilitation-consultants-for-project-learning-studyeoi-american-india-foundation-rfp-26-00367</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="95" customHeight="1">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
+    <row r="7" ht="95" customHeight="1">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>ToR - Engagement of Information Design &amp; Video Production Agency / Consultant for Key Learning &amp; Dissemination Outputs</t>
         </is>
       </c>
-      <c r="C8" s="1" t="inlineStr">
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>Terms of Reference (TOR) for Consultancy Services
 Title  Engagement of Information Design &amp; Video Production Agency / Consultant for Key Learning &amp; Dissemination Outputs
@@ -890,34 +844,34 @@
 The primary objective of this engagement is to enable SELCO Foundation to effectively capture, structure, and communicate its field insights, sectoral learnings, and program impacts. The selected Agency/Consultant (or Agencies/Consultants) will work on a monthly retainer basis to translate raw content, data, field footage, and reports provided by SELCO into high-quality, visually compelling, reader-friendly visual outputs and video assets.</t>
         </is>
       </c>
-      <c r="D8" s="1" t="inlineStr">
+      <c r="D7" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E8" s="1" t="inlineStr">
+      <c r="E7" s="1" t="inlineStr">
         <is>
           <t>Sep 28, 2026</t>
         </is>
       </c>
-      <c r="F8" s="1" t="inlineStr">
+      <c r="F7" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-engagement-of-information-design-and-video-production-agency-consultant-for-key-learning-and-dissemination-outputs-selco-foundation-rfp-26-00362</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="95" customHeight="1">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="inlineStr">
+    <row r="8" ht="95" customHeight="1">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>ToR - Video documentation of change stories on Ground water replenishment in Hyderabad and Sanga Reddy locations</t>
         </is>
       </c>
-      <c r="C9" s="1" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>About Jal Seva Charitable Foundation/ WaterAid India:
 Jal Seva Charitable Foundation (JSCF) is registered in India as a not-for-profit company under Chapter 8 of the Companies Act, 2013. JSCF, is an associate member of WaterAid International and uses the brand name ‘WaterAid’ in India.
@@ -951,34 +905,34 @@
 Upon completion of Assignment</t>
         </is>
       </c>
-      <c r="D9" s="1" t="inlineStr">
+      <c r="D8" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E9" s="1" t="inlineStr">
+      <c r="E8" s="1" t="inlineStr">
         <is>
           <t>Sep 28, 2026</t>
         </is>
       </c>
-      <c r="F9" s="1" t="inlineStr">
+      <c r="F8" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-video-documentation-of-change-stories-on-ground-water-replenishment-in-hyderabad-and-sanga-reddy-locations-wateraid-india-rfp-26-00363</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="95" customHeight="1">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
+    <row r="9" ht="95" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
         <is>
           <t>ToR - Video Production Storytelling and Documentation</t>
         </is>
       </c>
-      <c r="C10" s="1" t="inlineStr">
+      <c r="C9" s="1" t="inlineStr">
         <is>
           <t>Title Video Production – Storytelling and Documentation
 Timeline 3 months from the date of contracting
@@ -1012,19 +966,86 @@
 Quotation Should include all cost including Travel and Miscellaneous.</t>
         </is>
       </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>Sep 29, 2026</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/tor-video-production-storytelling-and-documentation-selco-foundation-rfp-26-00368</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="95" customHeight="1">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>EOI Inviting Expression of Interest-cum-Proposal for Setting Up District De-Addiction Centres under NAPDDR</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>About us
+In the year 1985-86, the erstwhile Ministry of Welfare was bifurcated into the Department of Women and Child Development and the Department of Welfare. Simultaneously, the Scheduled Castes Development Division, Tribal Development Division and the Minorities and Backward Classes Welfare Division were moved from the Ministry of Home Affairs and also the Wakf Division from the Ministry of Law to form the then Ministry of Welfare Subsequently, the name of the Ministry was changed to the Ministry of Social Justice &amp; Empowerment in May, 1998. Further, in October, 1999, the Tribal Development Division had moved out to form a separate Ministry of Tribal Affairs. In January, 2007, the Minorities Division along with Wakf Unit have been moved out of the Ministry and formed as a separate Ministry and the Child Development Division has gone to the Ministry of Women &amp; Child Development.
+ Department of Social Justice and Empowerment invites Expression of lnterest-cum-proposal from the eligible organizations for setting up of District DeAddiction Centres under the scheme of National Action Plan for Drug Demand Reduction (NAPDDR) for 315 GAP Districts of the country (as per list attached at Annexure - l). The list of districts is subject to change (addition or deletion) time to trme by the Ministry as per requirement or need on the ground.
+ 2. Eligible NGOs may apply for setting up of DDAC provided that they have rent free accommodation for setting up of DDAC as per the standards of guideline of the NAPDDR scheme or renlfree accommodation may also be provided by the concerned District Administration. 
+ 3. Setting up and running of District De-Addiction Centres (DDACS) will be done as per the following guidelinesr. 
+ i. There will be a District De-Addiction Centre (DDAC) preferably in each district headquarter or suitably accessible place where rent free accommodation is provided by the district administration. These DDACs would provide comprehensive facilities hitherto being provided by IRCA, ODIC &amp; CPLI together. lf the district administration of identified district is not able to provide suitable rent free accommodation, then the application will be called from the eligible VOs/ NGOs, who will provide rent free accommodation for setting up of DDAC in that district.
+ ii. The functioning of DDAC will be monitored by the three tier Committees headed by the Chief Secretary, District Collector/Deputy Commissioner and Block Development Officer of the respective arealregion which have been formed under Nasha Mukt Bharat Abhiyaan (NMBA). Additionally, retired eminent personalities of the Districts, activists, Vice-Chancellor/ Head of Department (HoD)/ Principal, researcher, scholars and so on may be co-opted by Chairman as the members of the Committees. These commiftees would
+ only monitor policy related issues. Day to day and other activities relating to implementation would be the responsibility of the concerned organization/NGO approved for setting up of the DDAC. The Meetings of DDAC are to be held as per the details given below:
+ (a) State-level Steering and Monitoring Committee (High Level Task Force) - headed by Chief Secretary - to meet quarterly. (b) District-level Committee - headed by District Collector / Deputy Commissioner - to meet monthly and have mandatory inspections quarterly. (c) Block level Committee - headed by Block Development Officer - to meet &amp; have mandatory inspections monthly.
+ The Committees will also review the functioning and assess the performance of the DDAC in terms of the effectiveness of deliverables and make further suggestions to the management of DDAC. 
+ IIl t. A separate (dedicated) account will be opened for keeping funds of DDAC in the name of NGO/Organization. The account will be registered on PFMS and implemented through EAT Module. 
+ lV. For setting up of DDACs, preference would be given to those Districts, which do not have any facility of IRCA or DDAC. For this, the organization willing to work in the field of DRUGS DE-ADDICTION TREATMENT will be eligible for applying for DDAC. The priority for selection of DDAC would be: 
+a. The DDAC proposed to be run by the District administration itself. 
+b. Rent free accommodation in the district headquarter provided by the concerned DC/DM &amp; further willingness from interested NGO is sought. c, Where no proposal for rent-free accommodation is received from concerned DCiDM, interested NGO may directly apply for DDAC provided they do not seek any rent for same and only building maintenance will be given. 
+V. The details of Minimum standards like physical space and necessary amenities to be provided by District administration or NGOs are as under: 
+(a) The centre should be easily accessible and connected through public transport. 
+(b) The total built-in area of the DDAC should be at least 3000 sq,ft. in case of metros and 4000 sq.ft. in case of small towns and villages to house 15 patients and 4000 sq.ft. in case of metros and 5000 sq.ft. in case of small towns and villages to house 30 patients. This includes an area of about 2000 sq. ft. for Treatment cum Rehabilitation centre, an area of about 700 sq. ft. for Drop-ln Centre facilities and an area of about 300 sq. ft. for CPLI Centre facilities. 
+(c) The centre should be properly ventilated, well-lit and maintained in a clean manner. Water to be made available. 
+(d) Basic safety of the patients to be ensured 
+(e) Facilities at the centre - Waiting space with seating arrangements for a minimum 5 persons Cubicles / rooms for consultation for physical examination Facilities to store drugs, linen, and records of patients Facilities with privacy for providing individual counselling, group therapy, re-educative sessions, family classes. They should be airy with comfortable seating with floor mats / chairs. Blackboard, chalk and other material to be provided. Availability of recreational facilities. Separate Drop ln Facility centre with recreation room, counselling room and medical room. Project room for CPLI activities including consultation room for interviewing Vl. Standards set in the above para of the guidelines may change from time to time as and when necessary with the approval of competent authority and the stakeholders / NGOs/ VOs would be intimated of same as and when such changes happen. 
+ 4. The interested and eligible NGOs / organizations can apply through eAnudaan (https://grants-msje.gov.in/ngo-login) portal of the Ministry. The Project Screening Committee in the Ministry will select the eligible NGO(s) for establishing and running of the DDAC and recommend the release of funds in two installments. However, the organization shall be eligible for receiving GIA under the scheme from the date of approval of the competent authority. 
+ 5. ELIGIBLE ORGANIZATION: 
+Organizations which are already running MoSJE supported IRCA or State Government supported De-addiction Centre/ Government Hospital or any private run De-Addiction centre are eligible for applying for DDAC. Organization can apply only for that State/UT in which they are already running IRCA"/De-addiction Centre from the last 2 years or more from the date of call for the proposal. Condition may be relaxed for any Government run Hospitals, which are non-profitable in nature. I 
+6. Start-up consists of young persons/ professionals, who have graduated from top social institutes of lndia or abroad are also eligible to apply. However, they must have experience of 2 years in the field of Drug De-addiction TREATMENT. 7. Role and Responsibility of DDACs The main focus of the DDAC is early prevention, education, demand reduction, identification, treatment and rehabilitation services of vulnerable individuals or individuals affected by substance use disorders DDAC would: 
+a. Conduct primary prevention activities through awareness programs among the vulnerable and affected community 
+b. Engage in risk mitigation of substance use among children/ adolescenuyouth by: Preventing substance use Delaying initiation of substance use 
+c. ldentify and train selected peer educators in the community 
+d. lmplement early prevention education through life skill training led by trained peer educators 
+e. Provide awareness about referral and linkage to counseling, treatment and rehabilitation services for substance dependent adolescents identified in the community 
+f. ldentifying adolescents and other individuals subjected to substance use and facilitating their referrali admission into Rehabilitation Centers/ Drop ln Centres. 
+g. Provide a whole range of services which includes treatment, after care and rehabilitation including skill development for Whole Person Recovery (WPR) of dependents; 
+h. Undertake drug demand reduction efforts to address all forms of illicit use of any substances and ensure overall well being of humankind; 
+i. Alleviate the consequences of substance dependence amongst individuals, family and society at large 
+9. The budget details of DDAC is attached as Annexure - 
+10. The e-anudaan portal shall remain open through out the year and the recommendations from the States/UTs will be considered periodically. 
+11. Department of Social Justice and Empowerment (DoSJE) reserves the right to cancel this notice, andior invite afresh proposals with or without amendments to this document without liability or any obligation for such document, and without assigning any reason. DoSJE reserves the right to take final decision regarding selection of implementing agency or project.</t>
+        </is>
+      </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>Learning</t>
+          <t>Governance</t>
         </is>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>Sep 29, 2026</t>
+          <t>Sep 30, 2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/rfps/tor-video-production-storytelling-and-documentation-selco-foundation-rfp-26-00368</t>
+          <t>https://onepurpos.in/openings/rfps/eoi-inviting-expression-of-interest-cum-proposal-for-setting-up-district-de-addiction-centres-under-napddr-ministry-of-social-justice-and-empowerment-goi-rfp-26-00356</t>
         </is>
       </c>
     </row>
@@ -1184,193 +1205,10 @@
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
-          <t>Applications Invited for Signals of Change Shaping the Future of Sexual and Reproductive Health and Rights SRHR</t>
+          <t>RFP - Design and Delivery of an Electric Vehicle EV Skilling Programme in Karnataka</t>
         </is>
       </c>
       <c r="C13" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-The World Health Organization's mission: to promote health, keep the world safe, and serve the vulnerable. Working through offices in more than 150 countries, WHO staff work side by side with governments and other partners to ensure the highest attainable level of health for all people.
- About the Opportunity
-HRP and its UN co-sponsors are leading a global Sexual and Reproductive Health and Rights (SRHR) foresight and research prioritization process for 2026–2036. This open public consultation invites diverse stakeholder input to identify "signals of change" — emerging trends, shifts, or disruptions — that could shape the future of SRHR over the next decade. The process uses foresight methodology (not prediction) to explore plausible futures and will culminate in a published report and research agenda in 2027.
- Guiding Questions
-What future trends will shape or constrain SRHR over the next 10 years?
-What evidence and research investments are needed today to prepare SRHR for the futures we may face?
- Scope of Submissions 
-Economic systems; social infrastructure; structural discrimination; conflict/forced migration/displacement; mega-trends (demographic shifts, climate change, digital transformation/AI, urbanization); conditions of daily life; rights/legal/governance systems; health systems; media/misinformation; and changes in the research ecosystem.
- Who Can Participate 
-Open to individuals and organizations globally, including:
-Health workers, professional associations, clinical networks
-Civil society, community groups, youth-led organizations, rights movements
-Governments, parliamentarians, regulators, public sector bodies
-Researchers, academia, think tanks, technical experts
-UN agencies, multilateral/humanitarian/development organizations
-Funders, philanthropy, private sector, tech/innovation organizations
-Media, communications, journalism
-Anyone with relevant lived experience or perspective
-Special interest in submissions from health worker, community, youth, and rights-movement spaces not typically represented in published forums.
- Submission Requirements: Descriptive information (name, contact email, country, sector) required alongside each submission; formal published evidence is helpful but not required — practice-based experience and field examples are also welcome. Submissions are kept confidential and anonymized before analysis.</t>
-        </is>
-      </c>
-      <c r="D13" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E13" s="1" t="inlineStr">
-        <is>
-          <t>Sep 30, 2026</t>
-        </is>
-      </c>
-      <c r="F13" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-signals-of-change-shaping-the-future-of-sexual-and-reproductive-health-and-rights-srhr-world-health-organization-opg-26-00176</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="95" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Setting up Viral Research and Diagnosis Laboratories VRDL in Medical Colleges/Hospitals/Medical Institutions</t>
-        </is>
-      </c>
-      <c r="C14" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-The President notified the creation of the Department of Health Research under the Ministry of Health &amp; Family Welfare through an amendment to the Government of India (Allocation of Business) Rules, 1961 on the 17th September 2007. The Department of Health Research was formally launched on 5th October 2007 by the Minister for Science &amp; Technology and Earth Sciences in a function presided over by the Minister for Health &amp; Family Welfare, in the presence, inter-alia, of the Minister of State for Health &amp; Family Welfare.
-The Department became functional from November 2008 with the appointment of first Secretary of the Department The aim of the DHR is to bring modern health technologies to the people through research and innovations related to diagnosis, treatment methods and vaccines for prevention, to translate them into products and processes and, in synergy with concerned organizations, introduce these innovations into public health system.
- About the Opportunity:
-Under DHR's scheme "Setting-up of nation-wide network of laboratories for managing epidemics and national calamities," proposals are invited from Medical Colleges/Hospitals/Research Institutions to establish a Medical College &amp; Research Institute Level – Viral Research and Diagnosis Laboratory (MCL-VRDL). The existing network comprises 167 VRDLs (11 Regional, 27 State, 129 Medical College level) across 27 states and 5 UTs, aimed at early detection of infectious pathogens, outbreak surveillance, and research on emerging/re-emerging viral diseases.
- Objectives:
-Establish capacity for early detection of common and high-risk infectious pathogens
-Strengthen syndromic surveillance ecosystem for outbreak detection
-Undertake R&amp;D on emerging, re-emerging and novel viruses
- Eligibility (Institution-level):
-State Government Medical Colleges
-Central Government Medical Colleges and Research Institutes
-Armed Forces Medical Institutions/Hospitals
-Railway and other Central Government health institutions
-Private medical colleges ranked in top 50 NIRF ranking
-Must have a dedicated Microbiology department with qualified faculty
-Must have &gt;200 sq.m. area available in existing building (preferably within Microbiology Dept.)
- Funding Provision:
-Non-recurring assistance: Rs. 1.55 crore total
-Rs. 66.8 lakhs — Civil Work (infrastructure modification)
-Rs. 88.2 lakhs — Equipment (complete lab setup)
-No recurring expenditure (staff salaries, consumables, contingency) is provided — to be borne by the host institution
- Role &amp; Responsibilities of the Lab:
-Conduct routine diagnosis of infectious pathogens
-Participate in syndromic and event-based surveillance
-Provide support during outbreaks/epidemics
-Share data with ICMR
- Selection Criteria:
-Meeting eligibility does not guarantee selection; merit-based evaluation by a technical committee
-Preference to institutions in geographically underserved regions
-Weightage for technical strength (qualified faculty, biosafety practices, outbreak investigation experience, publications, patents, externally funded projects)
-Additional weightage for molecular diagnostics, genomic surveillance, One Health research capability, and commitment to long-term recurring support
-Private medical colleges: only top-50 NIRF-ranked institutions considered</t>
-        </is>
-      </c>
-      <c r="D14" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E14" s="1" t="inlineStr">
-        <is>
-          <t>Sep 30, 2026</t>
-        </is>
-      </c>
-      <c r="F14" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-setting-up-viral-research-and-diagnosis-laboratories-vrdl-in-medical-collegeshospitalsmedical-institutions-department-of-health-research-dhr-ministry-of-health-and-family-welfare-government-of-india-opg-26-00174</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="95" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="inlineStr">
-        <is>
-          <t>EOI Inviting Expression of Interest-cum-Proposal for Setting Up District De-Addiction Centres under NAPDDR</t>
-        </is>
-      </c>
-      <c r="C15" s="1" t="inlineStr">
-        <is>
-          <t>About us
-In the year 1985-86, the erstwhile Ministry of Welfare was bifurcated into the Department of Women and Child Development and the Department of Welfare. Simultaneously, the Scheduled Castes Development Division, Tribal Development Division and the Minorities and Backward Classes Welfare Division were moved from the Ministry of Home Affairs and also the Wakf Division from the Ministry of Law to form the then Ministry of Welfare Subsequently, the name of the Ministry was changed to the Ministry of Social Justice &amp; Empowerment in May, 1998. Further, in October, 1999, the Tribal Development Division had moved out to form a separate Ministry of Tribal Affairs. In January, 2007, the Minorities Division along with Wakf Unit have been moved out of the Ministry and formed as a separate Ministry and the Child Development Division has gone to the Ministry of Women &amp; Child Development.
- Department of Social Justice and Empowerment invites Expression of lnterest-cum-proposal from the eligible organizations for setting up of District DeAddiction Centres under the scheme of National Action Plan for Drug Demand Reduction (NAPDDR) for 315 GAP Districts of the country (as per list attached at Annexure - l). The list of districts is subject to change (addition or deletion) time to trme by the Ministry as per requirement or need on the ground.
- 2. Eligible NGOs may apply for setting up of DDAC provided that they have rent free accommodation for setting up of DDAC as per the standards of guideline of the NAPDDR scheme or renlfree accommodation may also be provided by the concerned District Administration. 
- 3. Setting up and running of District De-Addiction Centres (DDACS) will be done as per the following guidelinesr. 
- i. There will be a District De-Addiction Centre (DDAC) preferably in each district headquarter or suitably accessible place where rent free accommodation is provided by the district administration. These DDACs would provide comprehensive facilities hitherto being provided by IRCA, ODIC &amp; CPLI together. lf the district administration of identified district is not able to provide suitable rent free accommodation, then the application will be called from the eligible VOs/ NGOs, who will provide rent free accommodation for setting up of DDAC in that district.
- ii. The functioning of DDAC will be monitored by the three tier Committees headed by the Chief Secretary, District Collector/Deputy Commissioner and Block Development Officer of the respective arealregion which have been formed under Nasha Mukt Bharat Abhiyaan (NMBA). Additionally, retired eminent personalities of the Districts, activists, Vice-Chancellor/ Head of Department (HoD)/ Principal, researcher, scholars and so on may be co-opted by Chairman as the members of the Committees. These commiftees would
- only monitor policy related issues. Day to day and other activities relating to implementation would be the responsibility of the concerned organization/NGO approved for setting up of the DDAC. The Meetings of DDAC are to be held as per the details given below:
- (a) State-level Steering and Monitoring Committee (High Level Task Force) - headed by Chief Secretary - to meet quarterly. (b) District-level Committee - headed by District Collector / Deputy Commissioner - to meet monthly and have mandatory inspections quarterly. (c) Block level Committee - headed by Block Development Officer - to meet &amp; have mandatory inspections monthly.
- The Committees will also review the functioning and assess the performance of the DDAC in terms of the effectiveness of deliverables and make further suggestions to the management of DDAC. 
- IIl t. A separate (dedicated) account will be opened for keeping funds of DDAC in the name of NGO/Organization. The account will be registered on PFMS and implemented through EAT Module. 
- lV. For setting up of DDACs, preference would be given to those Districts, which do not have any facility of IRCA or DDAC. For this, the organization willing to work in the field of DRUGS DE-ADDICTION TREATMENT will be eligible for applying for DDAC. The priority for selection of DDAC would be: 
-a. The DDAC proposed to be run by the District administration itself. 
-b. Rent free accommodation in the district headquarter provided by the concerned DC/DM &amp; further willingness from interested NGO is sought. c, Where no proposal for rent-free accommodation is received from concerned DCiDM, interested NGO may directly apply for DDAC provided they do not seek any rent for same and only building maintenance will be given. 
-V. The details of Minimum standards like physical space and necessary amenities to be provided by District administration or NGOs are as under: 
-(a) The centre should be easily accessible and connected through public transport. 
-(b) The total built-in area of the DDAC should be at least 3000 sq,ft. in case of metros and 4000 sq.ft. in case of small towns and villages to house 15 patients and 4000 sq.ft. in case of metros and 5000 sq.ft. in case of small towns and villages to house 30 patients. This includes an area of about 2000 sq. ft. for Treatment cum Rehabilitation centre, an area of about 700 sq. ft. for Drop-ln Centre facilities and an area of about 300 sq. ft. for CPLI Centre facilities. 
-(c) The centre should be properly ventilated, well-lit and maintained in a clean manner. Water to be made available. 
-(d) Basic safety of the patients to be ensured 
-(e) Facilities at the centre - Waiting space with seating arrangements for a minimum 5 persons Cubicles / rooms for consultation for physical examination Facilities to store drugs, linen, and records of patients Facilities with privacy for providing individual counselling, group therapy, re-educative sessions, family classes. They should be airy with comfortable seating with floor mats / chairs. Blackboard, chalk and other material to be provided. Availability of recreational facilities. Separate Drop ln Facility centre with recreation room, counselling room and medical room. Project room for CPLI activities including consultation room for interviewing Vl. Standards set in the above para of the guidelines may change from time to time as and when necessary with the approval of competent authority and the stakeholders / NGOs/ VOs would be intimated of same as and when such changes happen. 
- 4. The interested and eligible NGOs / organizations can apply through eAnudaan (https://grants-msje.gov.in/ngo-login) portal of the Ministry. The Project Screening Committee in the Ministry will select the eligible NGO(s) for establishing and running of the DDAC and recommend the release of funds in two installments. However, the organization shall be eligible for receiving GIA under the scheme from the date of approval of the competent authority. 
- 5. ELIGIBLE ORGANIZATION: 
-Organizations which are already running MoSJE supported IRCA or State Government supported De-addiction Centre/ Government Hospital or any private run De-Addiction centre are eligible for applying for DDAC. Organization can apply only for that State/UT in which they are already running IRCA"/De-addiction Centre from the last 2 years or more from the date of call for the proposal. Condition may be relaxed for any Government run Hospitals, which are non-profitable in nature. I 
-6. Start-up consists of young persons/ professionals, who have graduated from top social institutes of lndia or abroad are also eligible to apply. However, they must have experience of 2 years in the field of Drug De-addiction TREATMENT. 7. Role and Responsibility of DDACs The main focus of the DDAC is early prevention, education, demand reduction, identification, treatment and rehabilitation services of vulnerable individuals or individuals affected by substance use disorders DDAC would: 
-a. Conduct primary prevention activities through awareness programs among the vulnerable and affected community 
-b. Engage in risk mitigation of substance use among children/ adolescenuyouth by: Preventing substance use Delaying initiation of substance use 
-c. ldentify and train selected peer educators in the community 
-d. lmplement early prevention education through life skill training led by trained peer educators 
-e. Provide awareness about referral and linkage to counseling, treatment and rehabilitation services for substance dependent adolescents identified in the community 
-f. ldentifying adolescents and other individuals subjected to substance use and facilitating their referrali admission into Rehabilitation Centers/ Drop ln Centres. 
-g. Provide a whole range of services which includes treatment, after care and rehabilitation including skill development for Whole Person Recovery (WPR) of dependents; 
-h. Undertake drug demand reduction efforts to address all forms of illicit use of any substances and ensure overall well being of humankind; 
-i. Alleviate the consequences of substance dependence amongst individuals, family and society at large 
-9. The budget details of DDAC is attached as Annexure - 
-10. The e-anudaan portal shall remain open through out the year and the recommendations from the States/UTs will be considered periodically. 
-11. Department of Social Justice and Empowerment (DoSJE) reserves the right to cancel this notice, andior invite afresh proposals with or without amendments to this document without liability or any obligation for such document, and without assigning any reason. DoSJE reserves the right to take final decision regarding selection of implementing agency or project.</t>
-        </is>
-      </c>
-      <c r="D15" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E15" s="1" t="inlineStr">
-        <is>
-          <t>Sep 30, 2026</t>
-        </is>
-      </c>
-      <c r="F15" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/eoi-inviting-expression-of-interest-cum-proposal-for-setting-up-district-de-addiction-centres-under-napddr-ministry-of-social-justice-and-empowerment-goi-rfp-26-00356</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="95" customHeight="1">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B16" s="1" t="inlineStr">
-        <is>
-          <t>RFP - Design and Delivery of an Electric Vehicle EV Skilling Programme in Karnataka</t>
-        </is>
-      </c>
-      <c r="C16" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 WRI India, an independent knowledge organisation registered as the India Resources Trust, provides objective information and practical proposals to foster environmentally sound and socially equitable development. As an independent knowledge organisation, we leverage our data and expertise to catalyze change across systems like food, land and water; energy; and cities. Our work focuses on improving people’s lives, protecting and restoring nature, and addressing climate change. To enable progress at the pace and scale needed, we also engage with the economic, finance and governance systems that are key to enabling this change.
@@ -1411,34 +1249,34 @@
 Must have a team of qualified trainers and master trainers with relevant domain expertise, as well as administrative and coordination support.</t>
         </is>
       </c>
-      <c r="D16" s="1" t="inlineStr">
+      <c r="D13" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E16" s="1" t="inlineStr">
+      <c r="E13" s="1" t="inlineStr">
         <is>
           <t>Oct 5, 2026</t>
         </is>
       </c>
-      <c r="F16" s="1" t="inlineStr">
+      <c r="F13" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfp-design-and-delivery-of-an-electric-vehicle-ev-skilling-programme-in-karnataka-wri-india-rfp-26-00361</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="95" customHeight="1">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B17" s="1" t="inlineStr">
+    <row r="14" ht="95" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>Applications Open Draper Richards Kaplan Foundation Funding for Social Enterprises</t>
         </is>
       </c>
-      <c r="C17" s="1" t="inlineStr">
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>About us
 Started in 2002, Draper Richards Kaplan Foundation (DRK) is a global venture philanthropy firm supporting early stage, high impact social enterprises. Borrowed from our venture capital legacy, DRK finds, funds, and supports exceptional leaders building innovative solutions to some of the world’s most challenging social and environmental problems. Since beginning this work nearly 25 years ago, DRK has invested in more than 270 organizations that have collectively impacted over 610 million lives to date.
@@ -1462,34 +1300,34 @@
 Please attach a standard resume/CV for the entrepreneur(s) and/or key leadership team members (e.g., CEO, COO, ED, etc.). Applications with text bios for entrepreneurs or members of the leadership team will not be considered.</t>
         </is>
       </c>
-      <c r="D17" s="1" t="inlineStr">
+      <c r="D14" s="1" t="inlineStr">
         <is>
           <t>Climate</t>
         </is>
       </c>
-      <c r="E17" s="1" t="inlineStr">
+      <c r="E14" s="1" t="inlineStr">
         <is>
           <t>Oct 10, 2026</t>
         </is>
       </c>
-      <c r="F17" s="1" t="inlineStr">
+      <c r="F14" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-open-draper-richards-kaplan-foundation-funding-for-social-enterprises-draper-richards-kaplan-foundation-opg-26-00188</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="95" customHeight="1">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="inlineStr">
+    <row r="15" ht="95" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund</t>
         </is>
       </c>
-      <c r="C18" s="1" t="inlineStr">
+      <c r="C15" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund
 Apply by: 13 October, 2026
@@ -1514,34 +1352,34 @@
  Projects should include opportunities for ServiceNow employees to volunteer in the project activation or implementation.</t>
         </is>
       </c>
-      <c r="D18" s="1" t="inlineStr">
+      <c r="D15" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E18" s="1" t="inlineStr">
+      <c r="E15" s="1" t="inlineStr">
         <is>
           <t>Oct 13, 2026</t>
         </is>
       </c>
-      <c r="F18" s="1" t="inlineStr">
+      <c r="F15" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/apply-for-the-servicenow-community-solar-fund-changex-opg-26-00186</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="95" customHeight="1">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="inlineStr">
+    <row r="16" ht="95" customHeight="1">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>ToR - Engagement of Consultant/Vendor Individual towards implementation of Literacy Program in Telangana State</t>
         </is>
       </c>
-      <c r="C19" s="1" t="inlineStr">
+      <c r="C16" s="1" t="inlineStr">
         <is>
           <t>ANNEX A – TERMS OF REFERENCE (ToR) 
  Engagement of Consultant/Vendor (Individual) towards implementation of Literacy Program in Telangana State.
@@ -1606,34 +1444,34 @@
 Approved travel and accommodation expenses incurred for assignment-related activities shall be reimbursed by Room to Read in accordance with the consultancy reimbursement guidelines.</t>
         </is>
       </c>
-      <c r="D19" s="1" t="inlineStr">
+      <c r="D16" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E19" s="1" t="inlineStr">
+      <c r="E16" s="1" t="inlineStr">
         <is>
           <t>Oct 16, 2026</t>
         </is>
       </c>
-      <c r="F19" s="1" t="inlineStr">
+      <c r="F16" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-engagement-of-consultantvendor-individual-towards-implementation-of-literacy-program-in-telangana-state-room-to-read-india-rfp-26-00360</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="95" customHeight="1">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="inlineStr">
+    <row r="17" ht="95" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
         <is>
           <t>RFPs Invited for Consultant to Develop a Technical Assistance Package for National Application of the Digital Health and AI Investment Classification Framework</t>
         </is>
       </c>
-      <c r="C20" s="1" t="inlineStr">
+      <c r="C17" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are Transform Health: a global coalition of more than 200 organisations driving the digital transformation of health to achieve universal health coverage. 
@@ -1661,34 +1499,34 @@
 Ability to manage multi-country consultancy engagements and coordinate with in-country focal points</t>
         </is>
       </c>
-      <c r="D20" s="1" t="inlineStr">
+      <c r="D17" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E20" s="1" t="inlineStr">
+      <c r="E17" s="1" t="inlineStr">
         <is>
           <t>Oct 23, 2026</t>
         </is>
       </c>
-      <c r="F20" s="1" t="inlineStr">
+      <c r="F17" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfps-invited-for-consultant-to-develop-a-technical-assistance-package-for-national-application-of-the-digital-health-and-ai-investment-classification-framework-transform-health-rfp-26-00359</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="95" customHeight="1">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="inlineStr">
+    <row r="18" ht="95" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Comparison of PFAS Contributions to Agricultural Systems</t>
         </is>
       </c>
-      <c r="C21" s="1" t="inlineStr">
+      <c r="C18" s="1" t="inlineStr">
         <is>
           <t>Project Objectives:
 Report per- and polyfluoroalkyl substance (PFAS) concentrations from a variety of agricultural inputs — animal manures, fertilizers, pesticides, composts, soil amendments, seed coatings, and biosolids-based products
@@ -1724,34 +1562,167 @@
  Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00) — same deadline as the other two WRF grants</t>
         </is>
       </c>
-      <c r="D21" s="1" t="inlineStr">
+      <c r="D18" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E21" s="1" t="inlineStr">
+      <c r="E18" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F21" s="1" t="inlineStr">
+      <c r="F18" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-comparison-of-pfas-contributions-to-agricultural-systems-the-water-research-foundation-wrf-opg-26-00190</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="95" customHeight="1">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="inlineStr">
+    <row r="19" ht="95" customHeight="1">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Adaptive Control Frameworks to Unlock Full-Scale BNR Potential Water Research Foundation WRF</t>
+        </is>
+      </c>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+The Water Research Foundation (WRF) is the leading research organization advancing the science of all water to meet the evolving needs of its subscribers and the water sector. WRF is a nonprofit, charitable and educational organization which funds, manages, and publishes research on the technology, operation, and management of drinking water, wastewater, reuse, and stormwater collection, treatment and supply systems—all in pursuit of ensuring water quality and improving water services to the public.
+ Project Objectives:
+Identify and categorize dominant failure modes of current aeration and process control implementations under real-world operating conditions
+Develop guidance on data/instrumentation requirements for utilities to support adaptive control — including characterizing existing sensor infrastructure and use of soft sensors where hard sensors are limited
+Develop practical adaptive control frameworks and implementation guidance deployable without dependence on proprietary black-box tools or specialized data science expertise, including hybrid approaches augmenting conventional controls with AI/ML and digital twins for variable flow/concentration conditions
+Benchmark control performance against biological capacity indicators across multiple full-scale facilities to quantify the gap between achievable and realized Biological Nutrient Removal (BNR) performance
+ Background/Rationale:
+The water sector routinely invests in capital-intensive solutions (additional aeration, supplemental carbon systems, tertiary filtration) to address BNR shortfalls that may actually be control execution problems, not biological potential. Adaptive control strategies (e.g., ammonia-based aeration control, ammonia vs. nitrate control) frequently fail under variable influent loading or temperature swings, causing operators to revert to manual control. This project targets that execution gap using digitalization, AI/ML, and sensors. Geographic focus: United States and Canada.
+ Research Approach (flexible, proposer-defined):
+Failure-Mode Characterization
+Sensor Infrastructure Inventory and Data Quality Assessment
+Soft Sensor Development and Validation
+Adaptive Control Framework Development (hybrid rule-based + AI/ML)
+Operator Adoption and Organizational Readiness
+Multi-Facility Benchmarking
+ Expected Deliverables:
+Comprehensive literature review (including WRF's own research)
+Utility-facing implementation guidance (controller selection, sensor infrastructure, tuning, calibration, operator training, maintenance, system integration) — must include a decision framework and failure-mode catalog
+Multi-facility dataset quantifying capacity-vs-performance gap, with utility case studies across US/Canada
+Outreach (webcasts, conference presentations)
+One open-access peer-reviewed journal paper
+ Project Duration: 24 months from contract start date (No-Cost Extension Policy caps extensions at 9 months beyond original schedule)
+ Eligibility to Submit:
+Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible to be named participants.
+ Budget/Funding:
+Maximum WRF funding: $300,000
+Applicant must contribute additional resources equivalent to at least 33% of the project award (e.g., $100,000 requested → minimum $33,000 additional contribution required, via cost share, applicant in-kind, or third-party in-kind)
+Proposals not meeting the 33% minimum match will not be accepted
+ Proposal Evaluation Criteria:
+Understanding the Problem and Responsiveness to RFP: 20 points
+Technical and Scientific Merit: 30 points
+Qualifications, Capabilities, and Management: 20 points
+Communication Plan, Deliverables, and Applicability: 15 points
+Budget and Schedule: 15 points
+ Compliance Standards: Administrative, cost, and audit standards comply with OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
+Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
+        </is>
+      </c>
+      <c r="D19" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E19" s="1" t="inlineStr">
+        <is>
+          <t>Oct 26, 2026</t>
+        </is>
+      </c>
+      <c r="F19" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-adaptive-control-frameworks-to-unlock-full-scale-bnr-potential-water-research-foundation-wrf-the-water-research-foundation-wrf-opg-26-00187</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="95" customHeight="1">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Crossing the Divide Best Practices for Addressing Local and Privately-Owned Lateral Sewer Issues RFP 5419</t>
+        </is>
+      </c>
+      <c r="C20" s="1" t="inlineStr">
+        <is>
+          <t>Project Objective:
+To provide water resource recovery facilities (WRRFs) and collection system operators with an interactive manual of practice for implementing inflow and infiltration (I&amp;I) and obstruction management programs, focused on municipal and privately owned lateral sewers in complex legal, regulatory, and multi-jurisdictional environments.
+ Background/Rationale:
+Wastewater utilities face continuing challenges providing cost-effective sewer services amid rising demand, urban redevelopment, and performance disruptors (root intrusion, pipe degradation, blockages). I&amp;I and obstruction management remain persistent, costly problems without a consolidated resource to guide program design. During wet weather, peak I&amp;I flows can increase influent flows 3–5x average. Studies suggest up to 80% of I&amp;I originates on private property, and root intrusions cause over 50% of sewer blockages globally. Program effectiveness varies widely depending on statutory authority, multi-jurisdictional overlap, enforcement mechanisms, and participant willingness.
+ Central Research Questions:
+What I&amp;I and obstruction management practices are utilities using today, and how do they vary by jurisdictional/regulatory/infrastructure/environmental conditions?
+Which factors most influence successful implementation, and what barriers commonly derail programs?
+What measurable benefits (cost avoidance, capacity recovery, reduced spill risk, improved regulatory standing) have utilities realized from successful programs?
+This project extends WRF's ongoing "State-of-Practice Manual for Inflow and Infiltration Detection and Mitigation at Street and Private Lateral Levels" (Project 5365) into I&amp;I source control and obstruction management specifically.
+ Research Approach (4 Tasks):
+Literature and Regulatory Review — Comprehensive review of legal authorities/regulations in the US and comparable international jurisdictions; catalog program elements, enforcement mechanisms, incentive structures, and legal/jurisdictional barriers
+Utility Survey and Case Study Development — Broad survey across utility size/geography/system type; select at least 5 diverse in-depth case studies with quantitative results (I&amp;I reduction %, reduced bypass pumping, reduced basement backups, cost savings, recovered capacity, reduced blockage-related spills/service calls)
+Utility Workshop — At least one invitation-only workshop with utility representatives to present survey findings and gather structured feedback on draft guidance content
+Interactive Manual of Practice — Development of a decision-support tool/web-based application/interactive PDF enabling utilities to select effective I&amp;I/obstruction program elements based on their statutory authority, jurisdictional complexity, and enforcement mechanisms
+ Expected Deliverables:
+Research report (using WRF's Research Report Template) including literature/regulatory review
+Interactive manual of practice (following Technology Deliverables Guidance)
+In-depth utility survey, state-of-the-practice report, and at least 5 standalone case studies with quantitative results
+Summary documentation of the utility workshop, including feedback and how it was incorporated
+ Project Duration: 24 months from contract start date (No-Cost Extension Policy caps extensions at 9 months beyond original schedule)
+ Eligibility to Submit:
+Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible as named participants. Not open to individuals (same institutional-applicant structure as RFP 5424).
+ Budget/Funding:
+Maximum WRF funding: $250,000
+Applicant must contribute at least 33% of the project award as additional resources (cost share, applicant in-kind, or third-party in-kind per 2 CFR Part 200.306)
+Proposals not meeting the 33% minimum match will not be accepted
+ Proposal Evaluation Criteria:
+Understanding the Problem and Responsiveness to RFP: 20 points
+Technical and Scientific Merit: 30 points
+Qualifications, Capabilities, and Management: 20 points
+Communication Plan, Deliverables, and Applicability: 15 points
+Budget and Schedule: 15 points
+ Compliance Standards: OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
+ Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
+        </is>
+      </c>
+      <c r="D20" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E20" s="1" t="inlineStr">
+        <is>
+          <t>Oct 26, 2026</t>
+        </is>
+      </c>
+      <c r="F20" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-crossing-the-divide-best-practices-for-addressing-local-and-privately-owned-lateral-sewer-issues-rfp-5419-the-water-research-foundation-wrf-opg-26-00189</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="95" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 8th Call for Proposals Small-Size Grants Global EbA Fund</t>
         </is>
       </c>
-      <c r="C22" s="1" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -1814,207 +1785,34 @@
 Only successful applicants will be contacted; no individual feedback provided to unsuccessful applicants</t>
         </is>
       </c>
-      <c r="D22" s="1" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E22" s="1" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F22" s="1" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-8th-call-for-proposals-small-size-grants-global-eba-fund-global-eba-fund-opg-26-00177</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="95" customHeight="1">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B23" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Adaptive Control Frameworks to Unlock Full-Scale BNR Potential Water Research Foundation WRF</t>
-        </is>
-      </c>
-      <c r="C23" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-The Water Research Foundation (WRF) is the leading research organization advancing the science of all water to meet the evolving needs of its subscribers and the water sector. WRF is a nonprofit, charitable and educational organization which funds, manages, and publishes research on the technology, operation, and management of drinking water, wastewater, reuse, and stormwater collection, treatment and supply systems—all in pursuit of ensuring water quality and improving water services to the public.
- Project Objectives:
-Identify and categorize dominant failure modes of current aeration and process control implementations under real-world operating conditions
-Develop guidance on data/instrumentation requirements for utilities to support adaptive control — including characterizing existing sensor infrastructure and use of soft sensors where hard sensors are limited
-Develop practical adaptive control frameworks and implementation guidance deployable without dependence on proprietary black-box tools or specialized data science expertise, including hybrid approaches augmenting conventional controls with AI/ML and digital twins for variable flow/concentration conditions
-Benchmark control performance against biological capacity indicators across multiple full-scale facilities to quantify the gap between achievable and realized Biological Nutrient Removal (BNR) performance
- Background/Rationale:
-The water sector routinely invests in capital-intensive solutions (additional aeration, supplemental carbon systems, tertiary filtration) to address BNR shortfalls that may actually be control execution problems, not biological potential. Adaptive control strategies (e.g., ammonia-based aeration control, ammonia vs. nitrate control) frequently fail under variable influent loading or temperature swings, causing operators to revert to manual control. This project targets that execution gap using digitalization, AI/ML, and sensors. Geographic focus: United States and Canada.
- Research Approach (flexible, proposer-defined):
-Failure-Mode Characterization
-Sensor Infrastructure Inventory and Data Quality Assessment
-Soft Sensor Development and Validation
-Adaptive Control Framework Development (hybrid rule-based + AI/ML)
-Operator Adoption and Organizational Readiness
-Multi-Facility Benchmarking
- Expected Deliverables:
-Comprehensive literature review (including WRF's own research)
-Utility-facing implementation guidance (controller selection, sensor infrastructure, tuning, calibration, operator training, maintenance, system integration) — must include a decision framework and failure-mode catalog
-Multi-facility dataset quantifying capacity-vs-performance gap, with utility case studies across US/Canada
-Outreach (webcasts, conference presentations)
-One open-access peer-reviewed journal paper
- Project Duration: 24 months from contract start date (No-Cost Extension Policy caps extensions at 9 months beyond original schedule)
- Eligibility to Submit:
-Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible to be named participants.
- Budget/Funding:
-Maximum WRF funding: $300,000
-Applicant must contribute additional resources equivalent to at least 33% of the project award (e.g., $100,000 requested → minimum $33,000 additional contribution required, via cost share, applicant in-kind, or third-party in-kind)
-Proposals not meeting the 33% minimum match will not be accepted
- Proposal Evaluation Criteria:
-Understanding the Problem and Responsiveness to RFP: 20 points
-Technical and Scientific Merit: 30 points
-Qualifications, Capabilities, and Management: 20 points
-Communication Plan, Deliverables, and Applicability: 15 points
-Budget and Schedule: 15 points
- Compliance Standards: Administrative, cost, and audit standards comply with OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
-Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
-        </is>
-      </c>
-      <c r="D23" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E23" s="1" t="inlineStr">
-        <is>
-          <t>Oct 26, 2026</t>
-        </is>
-      </c>
-      <c r="F23" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-adaptive-control-frameworks-to-unlock-full-scale-bnr-potential-water-research-foundation-wrf-the-water-research-foundation-wrf-opg-26-00187</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="95" customHeight="1">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B24" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Crossing the Divide Best Practices for Addressing Local and Privately-Owned Lateral Sewer Issues RFP 5419</t>
-        </is>
-      </c>
-      <c r="C24" s="1" t="inlineStr">
-        <is>
-          <t>Project Objective:
-To provide water resource recovery facilities (WRRFs) and collection system operators with an interactive manual of practice for implementing inflow and infiltration (I&amp;I) and obstruction management programs, focused on municipal and privately owned lateral sewers in complex legal, regulatory, and multi-jurisdictional environments.
- Background/Rationale:
-Wastewater utilities face continuing challenges providing cost-effective sewer services amid rising demand, urban redevelopment, and performance disruptors (root intrusion, pipe degradation, blockages). I&amp;I and obstruction management remain persistent, costly problems without a consolidated resource to guide program design. During wet weather, peak I&amp;I flows can increase influent flows 3–5x average. Studies suggest up to 80% of I&amp;I originates on private property, and root intrusions cause over 50% of sewer blockages globally. Program effectiveness varies widely depending on statutory authority, multi-jurisdictional overlap, enforcement mechanisms, and participant willingness.
- Central Research Questions:
-What I&amp;I and obstruction management practices are utilities using today, and how do they vary by jurisdictional/regulatory/infrastructure/environmental conditions?
-Which factors most influence successful implementation, and what barriers commonly derail programs?
-What measurable benefits (cost avoidance, capacity recovery, reduced spill risk, improved regulatory standing) have utilities realized from successful programs?
-This project extends WRF's ongoing "State-of-Practice Manual for Inflow and Infiltration Detection and Mitigation at Street and Private Lateral Levels" (Project 5365) into I&amp;I source control and obstruction management specifically.
- Research Approach (4 Tasks):
-Literature and Regulatory Review — Comprehensive review of legal authorities/regulations in the US and comparable international jurisdictions; catalog program elements, enforcement mechanisms, incentive structures, and legal/jurisdictional barriers
-Utility Survey and Case Study Development — Broad survey across utility size/geography/system type; select at least 5 diverse in-depth case studies with quantitative results (I&amp;I reduction %, reduced bypass pumping, reduced basement backups, cost savings, recovered capacity, reduced blockage-related spills/service calls)
-Utility Workshop — At least one invitation-only workshop with utility representatives to present survey findings and gather structured feedback on draft guidance content
-Interactive Manual of Practice — Development of a decision-support tool/web-based application/interactive PDF enabling utilities to select effective I&amp;I/obstruction program elements based on their statutory authority, jurisdictional complexity, and enforcement mechanisms
- Expected Deliverables:
-Research report (using WRF's Research Report Template) including literature/regulatory review
-Interactive manual of practice (following Technology Deliverables Guidance)
-In-depth utility survey, state-of-the-practice report, and at least 5 standalone case studies with quantitative results
-Summary documentation of the utility workshop, including feedback and how it was incorporated
- Project Duration: 24 months from contract start date (No-Cost Extension Policy caps extensions at 9 months beyond original schedule)
- Eligibility to Submit:
-Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible as named participants. Not open to individuals (same institutional-applicant structure as RFP 5424).
- Budget/Funding:
-Maximum WRF funding: $250,000
-Applicant must contribute at least 33% of the project award as additional resources (cost share, applicant in-kind, or third-party in-kind per 2 CFR Part 200.306)
-Proposals not meeting the 33% minimum match will not be accepted
- Proposal Evaluation Criteria:
-Understanding the Problem and Responsiveness to RFP: 20 points
-Technical and Scientific Merit: 30 points
-Qualifications, Capabilities, and Management: 20 points
-Communication Plan, Deliverables, and Applicability: 15 points
-Budget and Schedule: 15 points
- Compliance Standards: OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
- Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
-        </is>
-      </c>
-      <c r="D24" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E24" s="1" t="inlineStr">
-        <is>
-          <t>Oct 26, 2026</t>
-        </is>
-      </c>
-      <c r="F24" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-crossing-the-divide-best-practices-for-addressing-local-and-privately-owned-lateral-sewer-issues-rfp-5419-the-water-research-foundation-wrf-opg-26-00189</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="95" customHeight="1">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B25" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Whitley Award 2027</t>
-        </is>
-      </c>
-      <c r="C25" s="1" t="inlineStr">
-        <is>
-          <t>About the Grant: 
-An annual grant by the Whitley Fund for Nature (WFN) recognising grassroots conservation leaders in the Global South, providing funding to support and scale up proven, science-based solutions that deliver lasting impact for both people and nature.
- About the Award 
-Whitley Awards support grassroots conservation leaders in the Global South. Through funding, training and profile, they help conservationists scale up effective projects that are founded in science and carried out with communities. Whitley Awards are for dynamic, mid-career conservationists who are leading vital conservation projects.
- Grant Amount: £50,000 in project funding over one year
- Eligibility
-Winners are nationals of the country in which they are working, seeking to scale up proven work that is embedded in the local community and would benefit from further funding, a profile boost, and international support.
-Projects must involve communities at the grassroots level and deliver practical action that is founded on science.
-You do not need to be invited or nominated to apply.</t>
-        </is>
-      </c>
-      <c r="D25" s="1" t="inlineStr">
-        <is>
-          <t>Learning</t>
-        </is>
-      </c>
-      <c r="E25" s="1" t="inlineStr">
-        <is>
-          <t>Oct 30, 2026</t>
-        </is>
-      </c>
-      <c r="F25" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-whitley-award-2027-whitley-fund-for-nature-wfn-opg-26-00153</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="95" customHeight="1">
-      <c r="A26" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B26" s="1" t="inlineStr">
+    <row r="22" ht="95" customHeight="1">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIFAR Global Scholars Program 20272029 Cohort</t>
         </is>
       </c>
-      <c r="C26" s="1" t="inlineStr">
+      <c r="C22" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 CIFAR is a Canadian-based globally influential research organization that convenes the world’s most brilliant people across disciplines to advance transformative knowledge and solve humanity’s biggest problems, together. By supporting long-term interdisciplinary collaboration, CIFAR provides researchers with an unparalleled environment of trust, transparency and knowledge sharing. Our time-tested model inspires new directions of inquiry, accelerates discovery and yields breakthroughs across borders and academic disciplines. Through knowledge mobilization, we are catalysts for change in industry, government and society. Through our 15 research programs and the Pan-Canadian AI Strategy, CIFAR convenes close to 400 of the world’s top researchers from 141 institutions in 20 countries. CIFAR is generously supported by the governments of Canada, Alberta and Québec, as well as foundations, individuals, corporations and Canadian and international partner organizations.
@@ -2058,115 +1856,34 @@
  Application Deadline: November 4, 2026, 12:00 PM EST</t>
         </is>
       </c>
-      <c r="D26" s="1" t="inlineStr">
+      <c r="D22" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E26" s="1" t="inlineStr">
+      <c r="E22" s="1" t="inlineStr">
         <is>
           <t>Nov 4, 2026</t>
         </is>
       </c>
-      <c r="F26" s="1" t="inlineStr">
+      <c r="F22" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cifar-global-scholars-program-20272029-cohort-cifar-canadian-institute-for-advanced-research-opg-26-00183</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="95" customHeight="1">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B27" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for IWRS Teaching Innovation Award</t>
-        </is>
-      </c>
-      <c r="C27" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-Insects are one of the most numerous and diverse animal groups on Earth.
-Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice.
-About the Award
-The IWRS Teaching Innovation Award supports instructors developing new approaches to teaching invertebrate biology that incorporate the 3Rs (replacement, reduction, and refinement). It also supports the development and implementation of any novel curricula addressing invertebrate welfare and sentience across invertebrate biology, animal welfare science, and/or veterinary medicine fields.
-Grant size
-Awards up to $2,000 USD are available for approaches requiring equipment or other materials; awards up to $1,000 USD are available otherwise. Funds may be used to support any costs associated with curriculum development and implementation, including stipends, teaching tools, and related expenses. Priority is given to proposals addressing common teaching practices with substantial welfare implications.
-Who can apply for funding?
-The applicant must be an instructor teaching content related to insect or invertebrate biology at an educational institution, scientific society or museum, field-training course, or similar educational context. If you are unsure about your eligibility, contact grants@insectwelfare.com.
-The applicant can be from any discipline, country, or institution. However, we will not pay awards to recipients located in jurisdictions, countries, or regions subject to trade restrictions, embargoes, or sanctions put in place by the United Nations or the United States of America.
-IWRS staff and Advisory Group members are not eligible to apply.</t>
-        </is>
-      </c>
-      <c r="D27" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E27" s="1" t="inlineStr">
-        <is>
-          <t>Nov 15, 2026</t>
-        </is>
-      </c>
-      <c r="F27" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00166</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="95" customHeight="1">
-      <c r="A28" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B28" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for IWRS Teaching Innovation Award</t>
-        </is>
-      </c>
-      <c r="C28" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
- About the Grant
-The IWRS (Insect Welfare Research Society) Teaching Innovation Award supports instructors developing new approaches to teaching insect or invertebrate biology that incorporate the 3Rs (Replacement, Reduction, and Refinement) — principles for reducing animal welfare impacts in teaching and research practices.
- Purpose
-Funds support the creation and implementation of 3Rs-driven instructional materials and pedagogical approaches. Priority is given to proposals addressing common teaching practices with substantial welfare implications.
- Grant Amount
-Two awards of $2,000 USD are available annually.</t>
-        </is>
-      </c>
-      <c r="D28" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E28" s="1" t="inlineStr">
-        <is>
-          <t>Nov 15, 2026</t>
-        </is>
-      </c>
-      <c r="F28" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="95" customHeight="1">
-      <c r="A29" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B29" s="1" t="inlineStr">
+    <row r="23" ht="95" customHeight="1">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Medium-Size Grants Call for Proposals Global EbA Fund</t>
         </is>
       </c>
-      <c r="C29" s="1" t="inlineStr">
+      <c r="C23" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -2223,88 +1940,34 @@
 Applications submitted via online portal (link shared on the Medium-Size Grants webpage from Oct 12)</t>
         </is>
       </c>
-      <c r="D29" s="1" t="inlineStr">
+      <c r="D23" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E29" s="1" t="inlineStr">
+      <c r="E23" s="1" t="inlineStr">
         <is>
           <t>Nov 16, 2026</t>
         </is>
       </c>
-      <c r="F29" s="1" t="inlineStr">
+      <c r="F23" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-medium-size-grants-call-for-proposals-global-eba-fund-global-eba-fund-opg-26-00178</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="95" customHeight="1">
-      <c r="A30" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B30" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for CIEIF Grant 2026 Climate Intervention Environmental Impact Fund</t>
-        </is>
-      </c>
-      <c r="C30" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-Climate Intervention Environmental Impact Fund (CIEIF) is a philanthropic fund focused on supporting responsible climate intervention field tests. It provides grants for activities such as environmental impact assessment (EIA), predictive impact modelling, and engagement with potentially affected stakeholders, including local communities and government agencies.
-CIEIF aims to help climate-intervention projects better understand their potential technical, environmental, economic, social, public-health, and safety impacts before and during field testing. It also places importance on the scalability and global relevance of supported innovations and encourages publication of field-test results through peer-reviewed journals or externally peer-reviewed reports.
- About the Grant
-The Climate Intervention Environmental Impact Fund (CIEIF) Grant provides USD 75,000 to support proposed climate intervention field tests. The funding is specifically intended for Environmental Impact Assessment (EIA), predictive impact modelling, and/or engagement with potentially affected stakeholders, including local communities and government agencies.
-Applicants are expected to demonstrate the proposed field test’s technical readiness, environmental and social considerations, required government approvals, innovation and potential for globally relevant scalability. The application must include a proposed budget showing how the USD 75,000 will be used.
- Grant Objective
-The grant is intended to support proposed climate intervention field tests, particularly activities related to:
-Environmental Impact Assessment (EIA)
-Predictive impact modeling
-Engagement with potentially impacted stakeholders
-Local community and government engagement
-Understanding technical, environmental, economic, social, public-health, and safety challenges
-The proposed application must focus on at least one of these three core areas: EIA, predictive impact modeling, or stakeholder engagement.
- Eligible Project Focus
-The proposed field test should demonstrate:
-A clear climate-intervention concept
-Prior research indicating that the technology is ready for the proposed field test
-Potential for innovation and scalability
-A clear understanding of technical and environmental challenges
-Consideration of economic, social, public-health, and safety implications
-Relevant government permits and approvals
-Potential for scaling the innovation to a globally relevant level</t>
-        </is>
-      </c>
-      <c r="D30" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E30" s="1" t="inlineStr">
-        <is>
-          <t>Dec 1, 2026</t>
-        </is>
-      </c>
-      <c r="F30" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-cieif-grant-2026-climate-intervention-environmental-impact-fund-climate-intervention-environmental-impact-fund-opg-26-00155</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="95" customHeight="1">
-      <c r="A31" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B31" s="1" t="inlineStr">
+    <row r="24" ht="95" customHeight="1">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 6th Annual Seeding The Future Global Food System Challenge</t>
         </is>
       </c>
-      <c r="C31" s="1" t="inlineStr">
+      <c r="C24" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are one of the largest and most respected private organisations for development cooperation and humanitarian aid in Germany. As a politically and confessionally independent organisation, our value-oriented actions are always based on ethical principles. Our vision is clear: "Zero Hunger by 2030"
@@ -2336,34 +1999,34 @@
 Individuals with no organizational entity</t>
         </is>
       </c>
-      <c r="D31" s="1" t="inlineStr">
+      <c r="D24" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E31" s="1" t="inlineStr">
+      <c r="E24" s="1" t="inlineStr">
         <is>
           <t>Jan 1, 2027</t>
         </is>
       </c>
-      <c r="F31" s="1" t="inlineStr">
+      <c r="F24" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-6th-annual-seeding-the-future-global-food-system-challenge-welthungerhilfe-opg-26-00180</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="95" customHeight="1">
-      <c r="A32" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B32" s="1" t="inlineStr">
+    <row r="25" ht="95" customHeight="1">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for BES Training and Travel Grants</t>
         </is>
       </c>
-      <c r="C32" s="1" t="inlineStr">
+      <c r="C25" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are a global community of scientists shining a spotlight on the intricacy and value of our natural world, providing the evidence for better decisions. Our vision is for people and nature to thrive in a world that values ecology.
@@ -2402,17 +2065,17 @@
  Application Deadline (Round 2): Opens 30 April 2026, closes 17 May 2026</t>
         </is>
       </c>
-      <c r="D32" s="1" t="inlineStr">
+      <c r="D25" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E32" s="1" t="inlineStr">
+      <c r="E25" s="1" t="inlineStr">
         <is>
           <t>May 17, 2027</t>
         </is>
       </c>
-      <c r="F32" s="1" t="inlineStr">
+      <c r="F25" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-bes-training-and-travel-grants-british-ecological-society-opg-26-00181</t>
         </is>

</xml_diff>

<commit_message>
Auto update Combined.xlsx [Mon Sep 21 07:34:02 UTC 2026]
</commit_message>
<xml_diff>
--- a/output/Combined.xlsx
+++ b/output/Combined.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -467,85 +467,10 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>ToR for Stand post - Varanasi</t>
+          <t>Applications Invited for GEF SGP CSO Challenge Program</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
-        <is>
-          <t>Background
-Access to safe and reliable drinking water remains a critical challenge in several habitations of Harahua Block in Varanasi District, Uttar Pradesh. Although the Government of India, through the Jal Jeevan Mission (JJM), is expanding piped water supply, many marginalized settlements continue to face inadequate access to potable water due to limited household connections, inadequate storage infrastructure, and uneven water distribution.
- Women, children, elderly people, and socially vulnerable households are disproportionately affected, often spending considerable time and effort collecting drinking water from distant or unreliable sources. During peak summer months and periods of high demand, the availability of safe drinking water becomes even more constrained.
- To address this challenge, installation of Ferrocement Tank Towers (Jal Minar) connected with the existing water supply system and equipped with community stand posts is proposed. Ferrocement technology offers a durable, cost-effective, low-maintenance, and climate-resilient solution for decentralized drinking water storage and distribution.
- Project Goal:
-To improve equitable and sustainable access to safe drinking water for underserved communities in Harahua Block through the installation of Ferrocement Tank Towers (Jal Minar) with community stand posts.
- Objectives
-Improve access to safe drinking water for underserved households.
-Reduce the distance and time spent collecting drinking water.
-Strengthen community-level drinking water infrastructure.
-Improve water security during supply interruptions and peak demand periods.
-Promote equitable access for women, children, elderly persons, and vulnerable communities.
-Support the objectives of Jal Jeevan Mission by strengthening last-mile service delivery.
- Proposed Intervention
-The project proposes installation of Ferrocement Tank Towers (Jal Minar) at strategic community locations connected to the existing drinking water supply network.
-Each Jal Minar will include:
-Ferrocement elevated storage tank
-RCC/steel supporting tower (as per design)
-Inlet and outlet pipeline
-Community stand posts with multiple taps
-Drainage arrangement
-Platform for safe water collection
-Water quality signage
-Provision for future maintenance
- The locations will be finalized in consultation with:
-Gram Panchayat
-Village Water &amp; Sanitation Committee (VWSC)
-Gram Pradhan
-Community representatives
-Stand post details:
-Village/Habitation
-No of Stand Post
-BhatpurwaKala
-1
-Sulemapur
-1
-Mohanpur
-1
-PalahipattiBazar
-1
-PalahipattiPrajapati Basti
-1
-Total Beneficiaries
-5</t>
-        </is>
-      </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>Sep 22, 2026</t>
-        </is>
-      </c>
-      <c r="F2" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/tor-for-stand-post-varanasi-wateraid-india-rfp-26-00364</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="95" customHeight="1">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for GEF SGP CSO Challenge Program</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global Environment Facility Small Grants Programme (SGP) is a global initiative implemented by the United Nations Development Programme (UNDP) on behalf of the Global Environment Facility (GEF). Since its launch in 1992, SGP has empowered communities worldwide to take action on environmental challenges while improving livelihoods. As a GEF Corporate Programme, SGP provides direct support to civil society organisations and community-based organisations to design and implement innovative, locally driven solutions. The programme places strong emphasis on inclusion, ensuring meaningful participation of Indigenous Peoples, youth, women and girls, and other underrepresented groups.
@@ -594,34 +519,34 @@
 Risk management and mitigation</t>
         </is>
       </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>Sep 23, 2026</t>
         </is>
       </c>
-      <c r="F3" s="1" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-gef-sgp-cso-challenge-program-gef-small-grants-programme-sgp-opg-26-00184</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="95" customHeight="1">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
+    <row r="3" ht="95" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>SoW - Hiring an External Agency for Orientation and Capacity Building</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Room to Read’s Foundational Literacy Program in Jharkhand
 Anchoring and Delivery of Orientation Programme for Jharkhand Field Workforce
@@ -649,34 +574,34 @@
 Provide details of at least 2 relevant past clients/assignments that may be referred to for verification of experience and performance</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Sep 23, 2026</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/sow-hiring-an-external-agency-for-orientation-and-capacity-building-room-to-read-india-rfp-26-00366</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="95" customHeight="1">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
+    <row r="4" ht="95" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>RFP for Impact Assessment</t>
         </is>
       </c>
-      <c r="C5" s="1" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>Introduction
 Titan Company Limited, a member of the Tata Group, has a long-standing commitment to Corporate Social Responsibility (CSR) in India. The company's CSR initiatives derive its philosophy from the Company’s vision statement: “We create elevating experiences for the people we touch and significantly impact the world we work in”. The initiatives are designed to promote inclusive growth, empower communities, and contribute to the country's socio-economic development. The program includes Titan’s CSR policy is governed by a dedicated CSR Committee that ensures transparency and compliance with regulatory requirements. The program includes Girl Child Education, Skill and Entrepreneurship Development, supporting Indian Heritage Arts and Crafts, Integrated Village Development Programme, Eye Care and Affirmative Action. Titan's CSR policy is governed by a dedicated CSR Committee that ensures transparency and compliance with regulatory requirements.
@@ -710,34 +635,34 @@
 Timeline: Proposal submission deadline: September 24, 2026</t>
         </is>
       </c>
-      <c r="D5" s="1" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E5" s="1" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>Sep 24, 2026</t>
         </is>
       </c>
-      <c r="F5" s="1" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfp-for-impact-assessment-titan-rfp-26-00354</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="95" customHeight="1">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>EOI- Engagement of State-Level Field Facilitation Consultants for Project Learning StudyEOI</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="inlineStr">
+    <row r="5" ht="95" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>EOI- Engagement of State-Level Field Facilitation Consultants for Project Learning Study</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>Expression of Interest (EOI)
 For
@@ -798,34 +723,34 @@
 This stage is for collecting information from interested Consultant. AIFT will review the submissions and may issue a detailed Request for Quotation (RFQ) to shortlisted consultant based on the specific assignments.</t>
         </is>
       </c>
-      <c r="D6" s="1" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E6" s="1" t="inlineStr">
+      <c r="E5" s="1" t="inlineStr">
         <is>
           <t>Sep 25, 2026</t>
         </is>
       </c>
-      <c r="F6" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/eoi-engagement-of-state-level-field-facilitation-consultants-for-project-learning-studyeoi-american-india-foundation-rfp-26-00367</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="95" customHeight="1">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/eoi-engagement-of-state-level-field-facilitation-consultants-for-project-learning-study-american-india-foundation-rfp-26-00367</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="95" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>ToR - Engagement of Information Design &amp; Video Production Agency / Consultant for Key Learning &amp; Dissemination Outputs</t>
         </is>
       </c>
-      <c r="C7" s="1" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>Terms of Reference (TOR) for Consultancy Services
 Title  Engagement of Information Design &amp; Video Production Agency / Consultant for Key Learning &amp; Dissemination Outputs
@@ -844,34 +769,34 @@
 The primary objective of this engagement is to enable SELCO Foundation to effectively capture, structure, and communicate its field insights, sectoral learnings, and program impacts. The selected Agency/Consultant (or Agencies/Consultants) will work on a monthly retainer basis to translate raw content, data, field footage, and reports provided by SELCO into high-quality, visually compelling, reader-friendly visual outputs and video assets.</t>
         </is>
       </c>
-      <c r="D7" s="1" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E7" s="1" t="inlineStr">
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>Sep 28, 2026</t>
         </is>
       </c>
-      <c r="F7" s="1" t="inlineStr">
+      <c r="F6" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-engagement-of-information-design-and-video-production-agency-consultant-for-key-learning-and-dissemination-outputs-selco-foundation-rfp-26-00362</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="95" customHeight="1">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
+    <row r="7" ht="95" customHeight="1">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>ToR - Video documentation of change stories on Ground water replenishment in Hyderabad and Sanga Reddy locations</t>
         </is>
       </c>
-      <c r="C8" s="1" t="inlineStr">
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>About Jal Seva Charitable Foundation/ WaterAid India:
 Jal Seva Charitable Foundation (JSCF) is registered in India as a not-for-profit company under Chapter 8 of the Companies Act, 2013. JSCF, is an associate member of WaterAid International and uses the brand name ‘WaterAid’ in India.
@@ -905,34 +830,34 @@
 Upon completion of Assignment</t>
         </is>
       </c>
-      <c r="D8" s="1" t="inlineStr">
+      <c r="D7" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E8" s="1" t="inlineStr">
+      <c r="E7" s="1" t="inlineStr">
         <is>
           <t>Sep 28, 2026</t>
         </is>
       </c>
-      <c r="F8" s="1" t="inlineStr">
+      <c r="F7" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-video-documentation-of-change-stories-on-ground-water-replenishment-in-hyderabad-and-sanga-reddy-locations-wateraid-india-rfp-26-00363</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="95" customHeight="1">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="inlineStr">
+    <row r="8" ht="95" customHeight="1">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>ToR - Video Production Storytelling and Documentation</t>
         </is>
       </c>
-      <c r="C9" s="1" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>Title Video Production – Storytelling and Documentation
 Timeline 3 months from the date of contracting
@@ -966,19 +891,83 @@
 Quotation Should include all cost including Travel and Miscellaneous.</t>
         </is>
       </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Sep 29, 2026</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/tor-video-production-storytelling-and-documentation-selco-foundation-rfp-26-00368</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="95" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Setting up Viral Research and Diagnosis Laboratories VRDL in Medical Colleges/Hospitals/Medical Institutions</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+The President notified the creation of the Department of Health Research under the Ministry of Health &amp; Family Welfare through an amendment to the Government of India (Allocation of Business) Rules, 1961 on the 17th September 2007. The Department of Health Research was formally launched on 5th October 2007 by the Minister for Science &amp; Technology and Earth Sciences in a function presided over by the Minister for Health &amp; Family Welfare, in the presence, inter-alia, of the Minister of State for Health &amp; Family Welfare.
+The Department became functional from November 2008 with the appointment of first Secretary of the Department The aim of the DHR is to bring modern health technologies to the people through research and innovations related to diagnosis, treatment methods and vaccines for prevention, to translate them into products and processes and, in synergy with concerned organizations, introduce these innovations into public health system.
+ About the Opportunity:
+Under DHR's scheme "Setting-up of nation-wide network of laboratories for managing epidemics and national calamities," proposals are invited from Medical Colleges/Hospitals/Research Institutions to establish a Medical College &amp; Research Institute Level – Viral Research and Diagnosis Laboratory (MCL-VRDL). The existing network comprises 167 VRDLs (11 Regional, 27 State, 129 Medical College level) across 27 states and 5 UTs, aimed at early detection of infectious pathogens, outbreak surveillance, and research on emerging/re-emerging viral diseases.
+ Objectives:
+Establish capacity for early detection of common and high-risk infectious pathogens
+Strengthen syndromic surveillance ecosystem for outbreak detection
+Undertake R&amp;D on emerging, re-emerging and novel viruses
+ Eligibility (Institution-level):
+State Government Medical Colleges
+Central Government Medical Colleges and Research Institutes
+Armed Forces Medical Institutions/Hospitals
+Railway and other Central Government health institutions
+Private medical colleges ranked in top 50 NIRF ranking
+Must have a dedicated Microbiology department with qualified faculty
+Must have &gt;200 sq.m. area available in existing building (preferably within Microbiology Dept.)
+ Funding Provision:
+Non-recurring assistance: Rs. 1.55 crore total
+Rs. 66.8 lakhs — Civil Work (infrastructure modification)
+Rs. 88.2 lakhs — Equipment (complete lab setup)
+No recurring expenditure (staff salaries, consumables, contingency) is provided — to be borne by the host institution
+ Role &amp; Responsibilities of the Lab:
+Conduct routine diagnosis of infectious pathogens
+Participate in syndromic and event-based surveillance
+Provide support during outbreaks/epidemics
+Share data with ICMR
+ Selection Criteria:
+Meeting eligibility does not guarantee selection; merit-based evaluation by a technical committee
+Preference to institutions in geographically underserved regions
+Weightage for technical strength (qualified faculty, biosafety practices, outbreak investigation experience, publications, patents, externally funded projects)
+Additional weightage for molecular diagnostics, genomic surveillance, One Health research capability, and commitment to long-term recurring support
+Private medical colleges: only top-50 NIRF-ranked institutions considered</t>
+        </is>
+      </c>
       <c r="D9" s="1" t="inlineStr">
         <is>
-          <t>Learning</t>
+          <t>Governance</t>
         </is>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>Sep 29, 2026</t>
+          <t>Sep 30, 2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/rfps/tor-video-production-storytelling-and-documentation-selco-foundation-rfp-26-00368</t>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-setting-up-viral-research-and-diagnosis-laboratories-vrdl-in-medical-collegeshospitalsmedical-institutions-department-of-health-research-dhr-ministry-of-health-and-family-welfare-government-of-india-opg-26-00174</t>
         </is>
       </c>
     </row>
@@ -990,77 +979,10 @@
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>EOI Inviting Expression of Interest-cum-Proposal for Setting Up District De-Addiction Centres under NAPDDR</t>
+          <t>Application Invited for Giving Joy Microgrant</t>
         </is>
       </c>
       <c r="C10" s="1" t="inlineStr">
-        <is>
-          <t>About us
-In the year 1985-86, the erstwhile Ministry of Welfare was bifurcated into the Department of Women and Child Development and the Department of Welfare. Simultaneously, the Scheduled Castes Development Division, Tribal Development Division and the Minorities and Backward Classes Welfare Division were moved from the Ministry of Home Affairs and also the Wakf Division from the Ministry of Law to form the then Ministry of Welfare Subsequently, the name of the Ministry was changed to the Ministry of Social Justice &amp; Empowerment in May, 1998. Further, in October, 1999, the Tribal Development Division had moved out to form a separate Ministry of Tribal Affairs. In January, 2007, the Minorities Division along with Wakf Unit have been moved out of the Ministry and formed as a separate Ministry and the Child Development Division has gone to the Ministry of Women &amp; Child Development.
- Department of Social Justice and Empowerment invites Expression of lnterest-cum-proposal from the eligible organizations for setting up of District DeAddiction Centres under the scheme of National Action Plan for Drug Demand Reduction (NAPDDR) for 315 GAP Districts of the country (as per list attached at Annexure - l). The list of districts is subject to change (addition or deletion) time to trme by the Ministry as per requirement or need on the ground.
- 2. Eligible NGOs may apply for setting up of DDAC provided that they have rent free accommodation for setting up of DDAC as per the standards of guideline of the NAPDDR scheme or renlfree accommodation may also be provided by the concerned District Administration. 
- 3. Setting up and running of District De-Addiction Centres (DDACS) will be done as per the following guidelinesr. 
- i. There will be a District De-Addiction Centre (DDAC) preferably in each district headquarter or suitably accessible place where rent free accommodation is provided by the district administration. These DDACs would provide comprehensive facilities hitherto being provided by IRCA, ODIC &amp; CPLI together. lf the district administration of identified district is not able to provide suitable rent free accommodation, then the application will be called from the eligible VOs/ NGOs, who will provide rent free accommodation for setting up of DDAC in that district.
- ii. The functioning of DDAC will be monitored by the three tier Committees headed by the Chief Secretary, District Collector/Deputy Commissioner and Block Development Officer of the respective arealregion which have been formed under Nasha Mukt Bharat Abhiyaan (NMBA). Additionally, retired eminent personalities of the Districts, activists, Vice-Chancellor/ Head of Department (HoD)/ Principal, researcher, scholars and so on may be co-opted by Chairman as the members of the Committees. These commiftees would
- only monitor policy related issues. Day to day and other activities relating to implementation would be the responsibility of the concerned organization/NGO approved for setting up of the DDAC. The Meetings of DDAC are to be held as per the details given below:
- (a) State-level Steering and Monitoring Committee (High Level Task Force) - headed by Chief Secretary - to meet quarterly. (b) District-level Committee - headed by District Collector / Deputy Commissioner - to meet monthly and have mandatory inspections quarterly. (c) Block level Committee - headed by Block Development Officer - to meet &amp; have mandatory inspections monthly.
- The Committees will also review the functioning and assess the performance of the DDAC in terms of the effectiveness of deliverables and make further suggestions to the management of DDAC. 
- IIl t. A separate (dedicated) account will be opened for keeping funds of DDAC in the name of NGO/Organization. The account will be registered on PFMS and implemented through EAT Module. 
- lV. For setting up of DDACs, preference would be given to those Districts, which do not have any facility of IRCA or DDAC. For this, the organization willing to work in the field of DRUGS DE-ADDICTION TREATMENT will be eligible for applying for DDAC. The priority for selection of DDAC would be: 
-a. The DDAC proposed to be run by the District administration itself. 
-b. Rent free accommodation in the district headquarter provided by the concerned DC/DM &amp; further willingness from interested NGO is sought. c, Where no proposal for rent-free accommodation is received from concerned DCiDM, interested NGO may directly apply for DDAC provided they do not seek any rent for same and only building maintenance will be given. 
-V. The details of Minimum standards like physical space and necessary amenities to be provided by District administration or NGOs are as under: 
-(a) The centre should be easily accessible and connected through public transport. 
-(b) The total built-in area of the DDAC should be at least 3000 sq,ft. in case of metros and 4000 sq.ft. in case of small towns and villages to house 15 patients and 4000 sq.ft. in case of metros and 5000 sq.ft. in case of small towns and villages to house 30 patients. This includes an area of about 2000 sq. ft. for Treatment cum Rehabilitation centre, an area of about 700 sq. ft. for Drop-ln Centre facilities and an area of about 300 sq. ft. for CPLI Centre facilities. 
-(c) The centre should be properly ventilated, well-lit and maintained in a clean manner. Water to be made available. 
-(d) Basic safety of the patients to be ensured 
-(e) Facilities at the centre - Waiting space with seating arrangements for a minimum 5 persons Cubicles / rooms for consultation for physical examination Facilities to store drugs, linen, and records of patients Facilities with privacy for providing individual counselling, group therapy, re-educative sessions, family classes. They should be airy with comfortable seating with floor mats / chairs. Blackboard, chalk and other material to be provided. Availability of recreational facilities. Separate Drop ln Facility centre with recreation room, counselling room and medical room. Project room for CPLI activities including consultation room for interviewing Vl. Standards set in the above para of the guidelines may change from time to time as and when necessary with the approval of competent authority and the stakeholders / NGOs/ VOs would be intimated of same as and when such changes happen. 
- 4. The interested and eligible NGOs / organizations can apply through eAnudaan (https://grants-msje.gov.in/ngo-login) portal of the Ministry. The Project Screening Committee in the Ministry will select the eligible NGO(s) for establishing and running of the DDAC and recommend the release of funds in two installments. However, the organization shall be eligible for receiving GIA under the scheme from the date of approval of the competent authority. 
- 5. ELIGIBLE ORGANIZATION: 
-Organizations which are already running MoSJE supported IRCA or State Government supported De-addiction Centre/ Government Hospital or any private run De-Addiction centre are eligible for applying for DDAC. Organization can apply only for that State/UT in which they are already running IRCA"/De-addiction Centre from the last 2 years or more from the date of call for the proposal. Condition may be relaxed for any Government run Hospitals, which are non-profitable in nature. I 
-6. Start-up consists of young persons/ professionals, who have graduated from top social institutes of lndia or abroad are also eligible to apply. However, they must have experience of 2 years in the field of Drug De-addiction TREATMENT. 7. Role and Responsibility of DDACs The main focus of the DDAC is early prevention, education, demand reduction, identification, treatment and rehabilitation services of vulnerable individuals or individuals affected by substance use disorders DDAC would: 
-a. Conduct primary prevention activities through awareness programs among the vulnerable and affected community 
-b. Engage in risk mitigation of substance use among children/ adolescenuyouth by: Preventing substance use Delaying initiation of substance use 
-c. ldentify and train selected peer educators in the community 
-d. lmplement early prevention education through life skill training led by trained peer educators 
-e. Provide awareness about referral and linkage to counseling, treatment and rehabilitation services for substance dependent adolescents identified in the community 
-f. ldentifying adolescents and other individuals subjected to substance use and facilitating their referrali admission into Rehabilitation Centers/ Drop ln Centres. 
-g. Provide a whole range of services which includes treatment, after care and rehabilitation including skill development for Whole Person Recovery (WPR) of dependents; 
-h. Undertake drug demand reduction efforts to address all forms of illicit use of any substances and ensure overall well being of humankind; 
-i. Alleviate the consequences of substance dependence amongst individuals, family and society at large 
-9. The budget details of DDAC is attached as Annexure - 
-10. The e-anudaan portal shall remain open through out the year and the recommendations from the States/UTs will be considered periodically. 
-11. Department of Social Justice and Empowerment (DoSJE) reserves the right to cancel this notice, andior invite afresh proposals with or without amendments to this document without liability or any obligation for such document, and without assigning any reason. DoSJE reserves the right to take final decision regarding selection of implementing agency or project.</t>
-        </is>
-      </c>
-      <c r="D10" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E10" s="1" t="inlineStr">
-        <is>
-          <t>Sep 30, 2026</t>
-        </is>
-      </c>
-      <c r="F10" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/eoi-inviting-expression-of-interest-cum-proposal-for-setting-up-district-de-addiction-centres-under-napddr-ministry-of-social-justice-and-empowerment-goi-rfp-26-00356</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="95" customHeight="1">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="inlineStr">
-        <is>
-          <t>Application Invited for Giving Joy Microgrant</t>
-        </is>
-      </c>
-      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Giving Joy is a US-based nonprofit that strengthens and inspires women’s entrepreneurship worldwide. Through its micro-grants and mentorship program, Giving Joy helps women establish or improve their businesses and initiatives—for their benefit and the benefit of their communities. To date, Giving Joy has awarded over 88 grants to women-led initiatives in 26 countries.
@@ -1099,34 +1021,34 @@
 The grant period is six months.</t>
         </is>
       </c>
-      <c r="D11" s="1" t="inlineStr">
+      <c r="D10" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E11" s="1" t="inlineStr">
+      <c r="E10" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F11" s="1" t="inlineStr">
+      <c r="F10" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/application-invited-for-giving-joy-microgrant-giving-joy-opg-26-00185</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="95" customHeight="1">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="inlineStr">
+    <row r="11" ht="95" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>ToR - Branding Development &amp; Design/Market Promotion Consultant Project Sashakt</t>
         </is>
       </c>
-      <c r="C12" s="1" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>Organisation Humana People to People India (HPPI)
 Project Sashakt – Strengthening Women-led Handloom Cooperatives in Assam (EU-funded)
@@ -1181,6 +1103,58 @@
 The consultant/agency must ensure ethical, consent-based data collection with cultural sensitivity, particularly when engaging women weavers. All data and reports remain the property of HPPI and must be kept strictly confidential, with no external use.</t>
         </is>
       </c>
+      <c r="D11" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>Sep 30, 2026</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/tor-branding-development-and-designmarket-promotion-consultant-project-sashakt-humana-people-to-people-india-rfp-26-00365</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="95" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Signals of Change Shaping the Future of Sexual and Reproductive Health and Rights SRHR</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+The World Health Organization's mission: to promote health, keep the world safe, and serve the vulnerable. Working through offices in more than 150 countries, WHO staff work side by side with governments and other partners to ensure the highest attainable level of health for all people.
+ About the Opportunity
+HRP and its UN co-sponsors are leading a global Sexual and Reproductive Health and Rights (SRHR) foresight and research prioritization process for 2026–2036. This open public consultation invites diverse stakeholder input to identify "signals of change" — emerging trends, shifts, or disruptions — that could shape the future of SRHR over the next decade. The process uses foresight methodology (not prediction) to explore plausible futures and will culminate in a published report and research agenda in 2027.
+ Guiding Questions
+What future trends will shape or constrain SRHR over the next 10 years?
+What evidence and research investments are needed today to prepare SRHR for the futures we may face?
+ Scope of Submissions 
+Economic systems; social infrastructure; structural discrimination; conflict/forced migration/displacement; mega-trends (demographic shifts, climate change, digital transformation/AI, urbanization); conditions of daily life; rights/legal/governance systems; health systems; media/misinformation; and changes in the research ecosystem.
+ Who Can Participate 
+Open to individuals and organizations globally, including:
+Health workers, professional associations, clinical networks
+Civil society, community groups, youth-led organizations, rights movements
+Governments, parliamentarians, regulators, public sector bodies
+Researchers, academia, think tanks, technical experts
+UN agencies, multilateral/humanitarian/development organizations
+Funders, philanthropy, private sector, tech/innovation organizations
+Media, communications, journalism
+Anyone with relevant lived experience or perspective
+Special interest in submissions from health worker, community, youth, and rights-movement spaces not typically represented in published forums.
+ Submission Requirements: Descriptive information (name, contact email, country, sector) required alongside each submission; formal published evidence is helpful but not required — practice-based experience and field examples are also welcome. Submissions are kept confidential and anonymized before analysis.</t>
+        </is>
+      </c>
       <c r="D12" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
@@ -1193,7 +1167,7 @@
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/rfps/tor-branding-development-and-designmarket-promotion-consultant-project-sashakt-humana-people-to-people-india-rfp-26-00365</t>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-signals-of-change-shaping-the-future-of-sexual-and-reproductive-health-and-rights-srhr-world-health-organization-opg-26-00176</t>
         </is>
       </c>
     </row>
@@ -1468,261 +1442,10 @@
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>RFPs Invited for Consultant to Develop a Technical Assistance Package for National Application of the Digital Health and AI Investment Classification Framework</t>
+          <t>Applications Invited for 8th Call for Proposals Small-Size Grants Global EbA Fund</t>
         </is>
       </c>
       <c r="C17" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-We are Transform Health: a global coalition of more than 200 organisations driving the digital transformation of health to achieve universal health coverage. 
-Our focus is on strengthening the enabling environment—the  laws, regulation, policies, coordination structures and resources—that ensure the digital health transformation is equitable, inclusive and sustainable and that digital technologies are adopted responsibly, equitably, and at scale.  This means going beyond just the technologies and tools to create the conditions that enable this vision. 
-We tackle complex issues that no single organisation can resolve, leveraging the collective power and expertise of our dynamic coalition. 
-Our work is underpinned by our core values of equity, inclusion, rights, empowerment, and partnership.
-Together, we can achieve universal health coverage in the digital age.
- About the Role:
-Transform Health is recruiting a consultant to develop a Technical Assistance (TA) approach and package that supports governments in applying the Digital Health and AI Investment Classification Framework, to aid budgeting, costing of digital health strategies/roadmaps, and analysis of digital health investment. The consultant will design the TA package and test it directly with governments in 3-4 countries, refining it based on the learnings. The work will be largely remote, with potential travel to testing countries.
- Responsibilities:
-Deliverable 1 – Develop the TA package: Review the current draft concept note, Classification Framework, and user guide; conduct user-centric design investigation with likely TA users (government officials, technical partners); translate the three entry points for national use of the Framework into a practical, step-by-step TA delivery approach; develop supporting tools (budget/costing templates, guidance materials); consolidate into a TA package for review before country testing
-Deliverable 2 – Apply the TA package in 3-4 countries: Work with Transform Health and technical partners to identify pilot countries; support government engagement and sign-off (e.g., MoU); lead direct TA delivery in each pilot country; document the process, outputs, adaptations, and structured feedback
-Deliverable 3 – Refine the TA package: Synthesise learnings and feedback from pilot countries; produce a final, ready-to-scale TA package and tools; write a final report with recommendations; write brief case studies (~2 pages each) per pilot country; present findings to Transform Health; draft a journal article based on the process and outcomes
- Eligibility:
-Willingness and ability to travel internationally as required
-Ability to work independently in multi-disciplinary, remote, cross-organisational teams
- Qualification:
-Demonstrated understanding of the digital health ecosystem, particularly policy and funding landscape
-In-depth understanding of government digital health funding (national budgeting, costing of digital health strategies/frameworks)
-Familiarity with key digital health frameworks and tools
-Knowledge of national health financing systems, budget structures, and investment tracking tools (e.g., National Health Accounts)
-Strong analytical, research, and written communication skills
-Experience with user-centric/human-centred design approaches (needs assessment, prototyping, iterative refinement)
-Demonstrated experience delivering technical assistance directly to government counterparts, ideally across multiple countries
-Ability to manage multi-country consultancy engagements and coordinate with in-country focal points</t>
-        </is>
-      </c>
-      <c r="D17" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E17" s="1" t="inlineStr">
-        <is>
-          <t>Oct 23, 2026</t>
-        </is>
-      </c>
-      <c r="F17" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/rfps-invited-for-consultant-to-develop-a-technical-assistance-package-for-national-application-of-the-digital-health-and-ai-investment-classification-framework-transform-health-rfp-26-00359</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="95" customHeight="1">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Comparison of PFAS Contributions to Agricultural Systems</t>
-        </is>
-      </c>
-      <c r="C18" s="1" t="inlineStr">
-        <is>
-          <t>Project Objectives:
-Report per- and polyfluoroalkyl substance (PFAS) concentrations from a variety of agricultural inputs — animal manures, fertilizers, pesticides, composts, soil amendments, seed coatings, and biosolids-based products
-Compare the impact of various agricultural inputs on PFAS concentration in the soil profile over varying timeframes
-Evaluate the fate and transport of different inputs to PFAS contributions in agricultural systems at field-scale
-Determine relative contributions from biosolids-based products vs. other inputs to help develop/prioritize risk management strategies
- Background/Rationale:
-Growing concern exists over human exposure to PFAS through biosolids land application on agricultural systems, with regulatory bans on biosolids land application enacted or proposed in at least 12 U.S. states. Utilities relying on land application for biosolids management are scrambling for alternative disposal pathways. The U.S. EPA's 2026 draft guidance noted its earlier 2025 draft risk assessment of PFOA/PFOS-contaminated sewage sludge lacked important contextual information (e.g., a national survey of PFOA/PFOS concentrations). Risk assessments have focused primarily on biosolids, with less attention to PFAS contributions from other sources — manures, compost, fertilizers, pesticides, seed coatings, irrigation water, farming practices, and atmospheric deposition. A Minnesota Pollution Control Agency review found 12 inert pesticide ingredients classified as PFAS. This project aims to improve understanding of PFAS risks from the wider range of agricultural inputs to support strategic resource allocation and inform policy amid surging fertilizer prices and shifts toward local circular resources.
- Research Approach:
-Develop a baseline of knowledge on PFAS in biosolids and non-biosolids agricultural inputs via literature review, analytical methods evaluation, and examination of manufacturing/processing pathways; identify data gaps and uncertainties
-Measure/report compound-specific PFAS concentrations and profiles in agricultural inputs using standardized methods, including precursor characteristics for source attribution where possible
-Characterize PFAS contributions via literature review, data analysis, and field sampling — comparing soil profile/plant tissue composition between fields with non-biosolids inputs vs. biosolids-applied systems; study should test hypotheses on PFAS sources, transformation, retention, and mobility
-Optional additional focus areas: influence of soil/hydrologic/hydrochemistry conditions on PFAS behavior; degradation/transformation pathways; relative PFAS contributions across product lifecycle stages (manufacturing, bagging, delivery, etc.)
-Research approach should be hypothesis-driven, detailing specific end-user needs, and proposers are encouraged to leverage existing projects on PFAS plant uptake/fate/transport.
- Expected Deliverables:
-Research report (WRF's Research Report Template) including: literature review, PFAS analysis of select products, risk management implications/prioritization recommendations, agriculture end-use guidance
-A webcast or workshop to share findings
-Optional additional deliverables: relative risk framework (mass input/fate/exposure/risk), decision support guide for farmers/regulators/utilities, plain language fact sheet, comparative PFAS mass input tool (spreadsheet/calculator)
- Project Duration: 36 months from contract start date (longer than the other two WRF grants above, which were 24 months)
- Eligibility to Submit:
-Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible. Not open to individuals (same structure as the two prior WRF grants).
- Budget/Funding:
-Maximum WRF funding: $400,000 (the largest of the three WRF grants shared so far)
-Applicant must contribute at least 33% of the project award as additional resources (cost share, applicant in-kind, or third-party in-kind per 2 CFR Part 200.306)
-Proposals not meeting the 33% minimum match will not be accepted
- Proposal Evaluation Criteria:
-Understanding the Problem and Responsiveness to RFP: 20 points
-Technical and Scientific Merit: 30 points
-Qualifications, Capabilities, and Management: 20 points
-Communication Plan, Deliverables, and Applicability: 15 points
-Budget and Schedule: 15 points
- Compliance Standards: OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
- Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00) — same deadline as the other two WRF grants</t>
-        </is>
-      </c>
-      <c r="D18" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E18" s="1" t="inlineStr">
-        <is>
-          <t>Oct 26, 2026</t>
-        </is>
-      </c>
-      <c r="F18" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-comparison-of-pfas-contributions-to-agricultural-systems-the-water-research-foundation-wrf-opg-26-00190</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="95" customHeight="1">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Adaptive Control Frameworks to Unlock Full-Scale BNR Potential Water Research Foundation WRF</t>
-        </is>
-      </c>
-      <c r="C19" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-The Water Research Foundation (WRF) is the leading research organization advancing the science of all water to meet the evolving needs of its subscribers and the water sector. WRF is a nonprofit, charitable and educational organization which funds, manages, and publishes research on the technology, operation, and management of drinking water, wastewater, reuse, and stormwater collection, treatment and supply systems—all in pursuit of ensuring water quality and improving water services to the public.
- Project Objectives:
-Identify and categorize dominant failure modes of current aeration and process control implementations under real-world operating conditions
-Develop guidance on data/instrumentation requirements for utilities to support adaptive control — including characterizing existing sensor infrastructure and use of soft sensors where hard sensors are limited
-Develop practical adaptive control frameworks and implementation guidance deployable without dependence on proprietary black-box tools or specialized data science expertise, including hybrid approaches augmenting conventional controls with AI/ML and digital twins for variable flow/concentration conditions
-Benchmark control performance against biological capacity indicators across multiple full-scale facilities to quantify the gap between achievable and realized Biological Nutrient Removal (BNR) performance
- Background/Rationale:
-The water sector routinely invests in capital-intensive solutions (additional aeration, supplemental carbon systems, tertiary filtration) to address BNR shortfalls that may actually be control execution problems, not biological potential. Adaptive control strategies (e.g., ammonia-based aeration control, ammonia vs. nitrate control) frequently fail under variable influent loading or temperature swings, causing operators to revert to manual control. This project targets that execution gap using digitalization, AI/ML, and sensors. Geographic focus: United States and Canada.
- Research Approach (flexible, proposer-defined):
-Failure-Mode Characterization
-Sensor Infrastructure Inventory and Data Quality Assessment
-Soft Sensor Development and Validation
-Adaptive Control Framework Development (hybrid rule-based + AI/ML)
-Operator Adoption and Organizational Readiness
-Multi-Facility Benchmarking
- Expected Deliverables:
-Comprehensive literature review (including WRF's own research)
-Utility-facing implementation guidance (controller selection, sensor infrastructure, tuning, calibration, operator training, maintenance, system integration) — must include a decision framework and failure-mode catalog
-Multi-facility dataset quantifying capacity-vs-performance gap, with utility case studies across US/Canada
-Outreach (webcasts, conference presentations)
-One open-access peer-reviewed journal paper
- Project Duration: 24 months from contract start date (No-Cost Extension Policy caps extensions at 9 months beyond original schedule)
- Eligibility to Submit:
-Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible to be named participants.
- Budget/Funding:
-Maximum WRF funding: $300,000
-Applicant must contribute additional resources equivalent to at least 33% of the project award (e.g., $100,000 requested → minimum $33,000 additional contribution required, via cost share, applicant in-kind, or third-party in-kind)
-Proposals not meeting the 33% minimum match will not be accepted
- Proposal Evaluation Criteria:
-Understanding the Problem and Responsiveness to RFP: 20 points
-Technical and Scientific Merit: 30 points
-Qualifications, Capabilities, and Management: 20 points
-Communication Plan, Deliverables, and Applicability: 15 points
-Budget and Schedule: 15 points
- Compliance Standards: Administrative, cost, and audit standards comply with OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
-Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
-        </is>
-      </c>
-      <c r="D19" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E19" s="1" t="inlineStr">
-        <is>
-          <t>Oct 26, 2026</t>
-        </is>
-      </c>
-      <c r="F19" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-adaptive-control-frameworks-to-unlock-full-scale-bnr-potential-water-research-foundation-wrf-the-water-research-foundation-wrf-opg-26-00187</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="95" customHeight="1">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Crossing the Divide Best Practices for Addressing Local and Privately-Owned Lateral Sewer Issues RFP 5419</t>
-        </is>
-      </c>
-      <c r="C20" s="1" t="inlineStr">
-        <is>
-          <t>Project Objective:
-To provide water resource recovery facilities (WRRFs) and collection system operators with an interactive manual of practice for implementing inflow and infiltration (I&amp;I) and obstruction management programs, focused on municipal and privately owned lateral sewers in complex legal, regulatory, and multi-jurisdictional environments.
- Background/Rationale:
-Wastewater utilities face continuing challenges providing cost-effective sewer services amid rising demand, urban redevelopment, and performance disruptors (root intrusion, pipe degradation, blockages). I&amp;I and obstruction management remain persistent, costly problems without a consolidated resource to guide program design. During wet weather, peak I&amp;I flows can increase influent flows 3–5x average. Studies suggest up to 80% of I&amp;I originates on private property, and root intrusions cause over 50% of sewer blockages globally. Program effectiveness varies widely depending on statutory authority, multi-jurisdictional overlap, enforcement mechanisms, and participant willingness.
- Central Research Questions:
-What I&amp;I and obstruction management practices are utilities using today, and how do they vary by jurisdictional/regulatory/infrastructure/environmental conditions?
-Which factors most influence successful implementation, and what barriers commonly derail programs?
-What measurable benefits (cost avoidance, capacity recovery, reduced spill risk, improved regulatory standing) have utilities realized from successful programs?
-This project extends WRF's ongoing "State-of-Practice Manual for Inflow and Infiltration Detection and Mitigation at Street and Private Lateral Levels" (Project 5365) into I&amp;I source control and obstruction management specifically.
- Research Approach (4 Tasks):
-Literature and Regulatory Review — Comprehensive review of legal authorities/regulations in the US and comparable international jurisdictions; catalog program elements, enforcement mechanisms, incentive structures, and legal/jurisdictional barriers
-Utility Survey and Case Study Development — Broad survey across utility size/geography/system type; select at least 5 diverse in-depth case studies with quantitative results (I&amp;I reduction %, reduced bypass pumping, reduced basement backups, cost savings, recovered capacity, reduced blockage-related spills/service calls)
-Utility Workshop — At least one invitation-only workshop with utility representatives to present survey findings and gather structured feedback on draft guidance content
-Interactive Manual of Practice — Development of a decision-support tool/web-based application/interactive PDF enabling utilities to select effective I&amp;I/obstruction program elements based on their statutory authority, jurisdictional complexity, and enforcement mechanisms
- Expected Deliverables:
-Research report (using WRF's Research Report Template) including literature/regulatory review
-Interactive manual of practice (following Technology Deliverables Guidance)
-In-depth utility survey, state-of-the-practice report, and at least 5 standalone case studies with quantitative results
-Summary documentation of the utility workshop, including feedback and how it was incorporated
- Project Duration: 24 months from contract start date (No-Cost Extension Policy caps extensions at 9 months beyond original schedule)
- Eligibility to Submit:
-Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible as named participants. Not open to individuals (same institutional-applicant structure as RFP 5424).
- Budget/Funding:
-Maximum WRF funding: $250,000
-Applicant must contribute at least 33% of the project award as additional resources (cost share, applicant in-kind, or third-party in-kind per 2 CFR Part 200.306)
-Proposals not meeting the 33% minimum match will not be accepted
- Proposal Evaluation Criteria:
-Understanding the Problem and Responsiveness to RFP: 20 points
-Technical and Scientific Merit: 30 points
-Qualifications, Capabilities, and Management: 20 points
-Communication Plan, Deliverables, and Applicability: 15 points
-Budget and Schedule: 15 points
- Compliance Standards: OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
- Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
-        </is>
-      </c>
-      <c r="D20" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E20" s="1" t="inlineStr">
-        <is>
-          <t>Oct 26, 2026</t>
-        </is>
-      </c>
-      <c r="F20" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-crossing-the-divide-best-practices-for-addressing-local-and-privately-owned-lateral-sewer-issues-rfp-5419-the-water-research-foundation-wrf-opg-26-00189</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="95" customHeight="1">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for 8th Call for Proposals Small-Size Grants Global EbA Fund</t>
-        </is>
-      </c>
-      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -1785,19 +1508,255 @@
 Only successful applicants will be contacted; no individual feedback provided to unsuccessful applicants</t>
         </is>
       </c>
+      <c r="D17" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>Oct 26, 2026</t>
+        </is>
+      </c>
+      <c r="F17" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-8th-call-for-proposals-small-size-grants-global-eba-fund-global-eba-fund-opg-26-00177</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="95" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Adaptive Control Frameworks to Unlock Full-Scale BNR Potential Water Research Foundation WRF</t>
+        </is>
+      </c>
+      <c r="C18" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+The Water Research Foundation (WRF) is the leading research organization advancing the science of all water to meet the evolving needs of its subscribers and the water sector. WRF is a nonprofit, charitable and educational organization which funds, manages, and publishes research on the technology, operation, and management of drinking water, wastewater, reuse, and stormwater collection, treatment and supply systems—all in pursuit of ensuring water quality and improving water services to the public.
+ Project Objectives:
+Identify and categorize dominant failure modes of current aeration and process control implementations under real-world operating conditions
+Develop guidance on data/instrumentation requirements for utilities to support adaptive control — including characterizing existing sensor infrastructure and use of soft sensors where hard sensors are limited
+Develop practical adaptive control frameworks and implementation guidance deployable without dependence on proprietary black-box tools or specialized data science expertise, including hybrid approaches augmenting conventional controls with AI/ML and digital twins for variable flow/concentration conditions
+Benchmark control performance against biological capacity indicators across multiple full-scale facilities to quantify the gap between achievable and realized Biological Nutrient Removal (BNR) performance
+ Background/Rationale:
+The water sector routinely invests in capital-intensive solutions (additional aeration, supplemental carbon systems, tertiary filtration) to address BNR shortfalls that may actually be control execution problems, not biological potential. Adaptive control strategies (e.g., ammonia-based aeration control, ammonia vs. nitrate control) frequently fail under variable influent loading or temperature swings, causing operators to revert to manual control. This project targets that execution gap using digitalization, AI/ML, and sensors. Geographic focus: United States and Canada.
+ Research Approach (flexible, proposer-defined):
+Failure-Mode Characterization
+Sensor Infrastructure Inventory and Data Quality Assessment
+Soft Sensor Development and Validation
+Adaptive Control Framework Development (hybrid rule-based + AI/ML)
+Operator Adoption and Organizational Readiness
+Multi-Facility Benchmarking
+ Expected Deliverables:
+Comprehensive literature review (including WRF's own research)
+Utility-facing implementation guidance (controller selection, sensor infrastructure, tuning, calibration, operator training, maintenance, system integration) — must include a decision framework and failure-mode catalog
+Multi-facility dataset quantifying capacity-vs-performance gap, with utility case studies across US/Canada
+Outreach (webcasts, conference presentations)
+One open-access peer-reviewed journal paper
+ Project Duration: 24 months from contract start date (No-Cost Extension Policy caps extensions at 9 months beyond original schedule)
+ Eligibility to Submit:
+Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible to be named participants.
+ Budget/Funding:
+Maximum WRF funding: $300,000
+Applicant must contribute additional resources equivalent to at least 33% of the project award (e.g., $100,000 requested → minimum $33,000 additional contribution required, via cost share, applicant in-kind, or third-party in-kind)
+Proposals not meeting the 33% minimum match will not be accepted
+ Proposal Evaluation Criteria:
+Understanding the Problem and Responsiveness to RFP: 20 points
+Technical and Scientific Merit: 30 points
+Qualifications, Capabilities, and Management: 20 points
+Communication Plan, Deliverables, and Applicability: 15 points
+Budget and Schedule: 15 points
+ Compliance Standards: Administrative, cost, and audit standards comply with OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
+Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
+        </is>
+      </c>
+      <c r="D18" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E18" s="1" t="inlineStr">
+        <is>
+          <t>Oct 26, 2026</t>
+        </is>
+      </c>
+      <c r="F18" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-adaptive-control-frameworks-to-unlock-full-scale-bnr-potential-water-research-foundation-wrf-the-water-research-foundation-wrf-opg-26-00187</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="95" customHeight="1">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Crossing the Divide Best Practices for Addressing Local and Privately-Owned Lateral Sewer Issues RFP 5419</t>
+        </is>
+      </c>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>Project Objective:
+To provide water resource recovery facilities (WRRFs) and collection system operators with an interactive manual of practice for implementing inflow and infiltration (I&amp;I) and obstruction management programs, focused on municipal and privately owned lateral sewers in complex legal, regulatory, and multi-jurisdictional environments.
+ Background/Rationale:
+Wastewater utilities face continuing challenges providing cost-effective sewer services amid rising demand, urban redevelopment, and performance disruptors (root intrusion, pipe degradation, blockages). I&amp;I and obstruction management remain persistent, costly problems without a consolidated resource to guide program design. During wet weather, peak I&amp;I flows can increase influent flows 3–5x average. Studies suggest up to 80% of I&amp;I originates on private property, and root intrusions cause over 50% of sewer blockages globally. Program effectiveness varies widely depending on statutory authority, multi-jurisdictional overlap, enforcement mechanisms, and participant willingness.
+ Central Research Questions:
+What I&amp;I and obstruction management practices are utilities using today, and how do they vary by jurisdictional/regulatory/infrastructure/environmental conditions?
+Which factors most influence successful implementation, and what barriers commonly derail programs?
+What measurable benefits (cost avoidance, capacity recovery, reduced spill risk, improved regulatory standing) have utilities realized from successful programs?
+This project extends WRF's ongoing "State-of-Practice Manual for Inflow and Infiltration Detection and Mitigation at Street and Private Lateral Levels" (Project 5365) into I&amp;I source control and obstruction management specifically.
+ Research Approach (4 Tasks):
+Literature and Regulatory Review — Comprehensive review of legal authorities/regulations in the US and comparable international jurisdictions; catalog program elements, enforcement mechanisms, incentive structures, and legal/jurisdictional barriers
+Utility Survey and Case Study Development — Broad survey across utility size/geography/system type; select at least 5 diverse in-depth case studies with quantitative results (I&amp;I reduction %, reduced bypass pumping, reduced basement backups, cost savings, recovered capacity, reduced blockage-related spills/service calls)
+Utility Workshop — At least one invitation-only workshop with utility representatives to present survey findings and gather structured feedback on draft guidance content
+Interactive Manual of Practice — Development of a decision-support tool/web-based application/interactive PDF enabling utilities to select effective I&amp;I/obstruction program elements based on their statutory authority, jurisdictional complexity, and enforcement mechanisms
+ Expected Deliverables:
+Research report (using WRF's Research Report Template) including literature/regulatory review
+Interactive manual of practice (following Technology Deliverables Guidance)
+In-depth utility survey, state-of-the-practice report, and at least 5 standalone case studies with quantitative results
+Summary documentation of the utility workshop, including feedback and how it was incorporated
+ Project Duration: 24 months from contract start date (No-Cost Extension Policy caps extensions at 9 months beyond original schedule)
+ Eligibility to Submit:
+Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible as named participants. Not open to individuals (same institutional-applicant structure as RFP 5424).
+ Budget/Funding:
+Maximum WRF funding: $250,000
+Applicant must contribute at least 33% of the project award as additional resources (cost share, applicant in-kind, or third-party in-kind per 2 CFR Part 200.306)
+Proposals not meeting the 33% minimum match will not be accepted
+ Proposal Evaluation Criteria:
+Understanding the Problem and Responsiveness to RFP: 20 points
+Technical and Scientific Merit: 30 points
+Qualifications, Capabilities, and Management: 20 points
+Communication Plan, Deliverables, and Applicability: 15 points
+Budget and Schedule: 15 points
+ Compliance Standards: OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
+ Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
+        </is>
+      </c>
+      <c r="D19" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E19" s="1" t="inlineStr">
+        <is>
+          <t>Oct 26, 2026</t>
+        </is>
+      </c>
+      <c r="F19" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-crossing-the-divide-best-practices-for-addressing-local-and-privately-owned-lateral-sewer-issues-rfp-5419-the-water-research-foundation-wrf-opg-26-00189</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="95" customHeight="1">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Comparison of PFAS Contributions to Agricultural Systems</t>
+        </is>
+      </c>
+      <c r="C20" s="1" t="inlineStr">
+        <is>
+          <t>Project Objectives:
+Report per- and polyfluoroalkyl substance (PFAS) concentrations from a variety of agricultural inputs — animal manures, fertilizers, pesticides, composts, soil amendments, seed coatings, and biosolids-based products
+Compare the impact of various agricultural inputs on PFAS concentration in the soil profile over varying timeframes
+Evaluate the fate and transport of different inputs to PFAS contributions in agricultural systems at field-scale
+Determine relative contributions from biosolids-based products vs. other inputs to help develop/prioritize risk management strategies
+ Background/Rationale:
+Growing concern exists over human exposure to PFAS through biosolids land application on agricultural systems, with regulatory bans on biosolids land application enacted or proposed in at least 12 U.S. states. Utilities relying on land application for biosolids management are scrambling for alternative disposal pathways. The U.S. EPA's 2026 draft guidance noted its earlier 2025 draft risk assessment of PFOA/PFOS-contaminated sewage sludge lacked important contextual information (e.g., a national survey of PFOA/PFOS concentrations). Risk assessments have focused primarily on biosolids, with less attention to PFAS contributions from other sources — manures, compost, fertilizers, pesticides, seed coatings, irrigation water, farming practices, and atmospheric deposition. A Minnesota Pollution Control Agency review found 12 inert pesticide ingredients classified as PFAS. This project aims to improve understanding of PFAS risks from the wider range of agricultural inputs to support strategic resource allocation and inform policy amid surging fertilizer prices and shifts toward local circular resources.
+ Research Approach:
+Develop a baseline of knowledge on PFAS in biosolids and non-biosolids agricultural inputs via literature review, analytical methods evaluation, and examination of manufacturing/processing pathways; identify data gaps and uncertainties
+Measure/report compound-specific PFAS concentrations and profiles in agricultural inputs using standardized methods, including precursor characteristics for source attribution where possible
+Characterize PFAS contributions via literature review, data analysis, and field sampling — comparing soil profile/plant tissue composition between fields with non-biosolids inputs vs. biosolids-applied systems; study should test hypotheses on PFAS sources, transformation, retention, and mobility
+Optional additional focus areas: influence of soil/hydrologic/hydrochemistry conditions on PFAS behavior; degradation/transformation pathways; relative PFAS contributions across product lifecycle stages (manufacturing, bagging, delivery, etc.)
+Research approach should be hypothesis-driven, detailing specific end-user needs, and proposers are encouraged to leverage existing projects on PFAS plant uptake/fate/transport.
+ Expected Deliverables:
+Research report (WRF's Research Report Template) including: literature review, PFAS analysis of select products, risk management implications/prioritization recommendations, agriculture end-use guidance
+A webcast or workshop to share findings
+Optional additional deliverables: relative risk framework (mass input/fate/exposure/risk), decision support guide for farmers/regulators/utilities, plain language fact sheet, comparative PFAS mass input tool (spreadsheet/calculator)
+ Project Duration: 36 months from contract start date (longer than the other two WRF grants above, which were 24 months)
+ Eligibility to Submit:
+Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible. Not open to individuals (same structure as the two prior WRF grants).
+ Budget/Funding:
+Maximum WRF funding: $400,000 (the largest of the three WRF grants shared so far)
+Applicant must contribute at least 33% of the project award as additional resources (cost share, applicant in-kind, or third-party in-kind per 2 CFR Part 200.306)
+Proposals not meeting the 33% minimum match will not be accepted
+ Proposal Evaluation Criteria:
+Understanding the Problem and Responsiveness to RFP: 20 points
+Technical and Scientific Merit: 30 points
+Qualifications, Capabilities, and Management: 20 points
+Communication Plan, Deliverables, and Applicability: 15 points
+Budget and Schedule: 15 points
+ Compliance Standards: OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
+ Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00) — same deadline as the other two WRF grants</t>
+        </is>
+      </c>
+      <c r="D20" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E20" s="1" t="inlineStr">
+        <is>
+          <t>Oct 26, 2026</t>
+        </is>
+      </c>
+      <c r="F20" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-comparison-of-pfas-contributions-to-agricultural-systems-the-water-research-foundation-wrf-opg-26-00190</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="95" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Whitley Award 2027</t>
+        </is>
+      </c>
+      <c r="C21" s="1" t="inlineStr">
+        <is>
+          <t>About the Grant: 
+An annual grant by the Whitley Fund for Nature (WFN) recognising grassroots conservation leaders in the Global South, providing funding to support and scale up proven, science-based solutions that deliver lasting impact for both people and nature.
+ About the Award 
+Whitley Awards support grassroots conservation leaders in the Global South. Through funding, training and profile, they help conservationists scale up effective projects that are founded in science and carried out with communities. Whitley Awards are for dynamic, mid-career conservationists who are leading vital conservation projects.
+ Grant Amount: £50,000 in project funding over one year
+ Eligibility
+Winners are nationals of the country in which they are working, seeking to scale up proven work that is embedded in the local community and would benefit from further funding, a profile boost, and international support.
+Projects must involve communities at the grassroots level and deliver practical action that is founded on science.
+You do not need to be invited or nominated to apply.</t>
+        </is>
+      </c>
       <c r="D21" s="1" t="inlineStr">
         <is>
-          <t>Governance</t>
+          <t>Learning</t>
         </is>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>Oct 26, 2026</t>
+          <t>Oct 30, 2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-8th-call-for-proposals-small-size-grants-global-eba-fund-global-eba-fund-opg-26-00177</t>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-whitley-award-2027-whitley-fund-for-nature-wfn-opg-26-00153</t>
         </is>
       </c>
     </row>
@@ -1880,10 +1839,91 @@
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
+          <t>Applications Invited for IWRS Teaching Innovation Award</t>
+        </is>
+      </c>
+      <c r="C23" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+Insects are one of the most numerous and diverse animal groups on Earth.
+Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice.
+About the Award
+The IWRS Teaching Innovation Award supports instructors developing new approaches to teaching invertebrate biology that incorporate the 3Rs (replacement, reduction, and refinement). It also supports the development and implementation of any novel curricula addressing invertebrate welfare and sentience across invertebrate biology, animal welfare science, and/or veterinary medicine fields.
+Grant size
+Awards up to $2,000 USD are available for approaches requiring equipment or other materials; awards up to $1,000 USD are available otherwise. Funds may be used to support any costs associated with curriculum development and implementation, including stipends, teaching tools, and related expenses. Priority is given to proposals addressing common teaching practices with substantial welfare implications.
+Who can apply for funding?
+The applicant must be an instructor teaching content related to insect or invertebrate biology at an educational institution, scientific society or museum, field-training course, or similar educational context. If you are unsure about your eligibility, contact grants@insectwelfare.com.
+The applicant can be from any discipline, country, or institution. However, we will not pay awards to recipients located in jurisdictions, countries, or regions subject to trade restrictions, embargoes, or sanctions put in place by the United Nations or the United States of America.
+IWRS staff and Advisory Group members are not eligible to apply.</t>
+        </is>
+      </c>
+      <c r="D23" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E23" s="1" t="inlineStr">
+        <is>
+          <t>Nov 15, 2026</t>
+        </is>
+      </c>
+      <c r="F23" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00166</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="95" customHeight="1">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for IWRS Teaching Innovation Award</t>
+        </is>
+      </c>
+      <c r="C24" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
+ About the Grant
+The IWRS (Insect Welfare Research Society) Teaching Innovation Award supports instructors developing new approaches to teaching insect or invertebrate biology that incorporate the 3Rs (Replacement, Reduction, and Refinement) — principles for reducing animal welfare impacts in teaching and research practices.
+ Purpose
+Funds support the creation and implementation of 3Rs-driven instructional materials and pedagogical approaches. Priority is given to proposals addressing common teaching practices with substantial welfare implications.
+ Grant Amount
+Two awards of $2,000 USD are available annually.</t>
+        </is>
+      </c>
+      <c r="D24" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E24" s="1" t="inlineStr">
+        <is>
+          <t>Nov 15, 2026</t>
+        </is>
+      </c>
+      <c r="F24" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="95" customHeight="1">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
+        <is>
           <t>Applications Invited for Medium-Size Grants Call for Proposals Global EbA Fund</t>
         </is>
       </c>
-      <c r="C23" s="1" t="inlineStr">
+      <c r="C25" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -1940,34 +1980,88 @@
 Applications submitted via online portal (link shared on the Medium-Size Grants webpage from Oct 12)</t>
         </is>
       </c>
-      <c r="D23" s="1" t="inlineStr">
+      <c r="D25" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E23" s="1" t="inlineStr">
+      <c r="E25" s="1" t="inlineStr">
         <is>
           <t>Nov 16, 2026</t>
         </is>
       </c>
-      <c r="F23" s="1" t="inlineStr">
+      <c r="F25" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-medium-size-grants-call-for-proposals-global-eba-fund-global-eba-fund-opg-26-00178</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="95" customHeight="1">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B24" s="1" t="inlineStr">
+    <row r="26" ht="95" customHeight="1">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for CIEIF Grant 2026 Climate Intervention Environmental Impact Fund</t>
+        </is>
+      </c>
+      <c r="C26" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+Climate Intervention Environmental Impact Fund (CIEIF) is a philanthropic fund focused on supporting responsible climate intervention field tests. It provides grants for activities such as environmental impact assessment (EIA), predictive impact modelling, and engagement with potentially affected stakeholders, including local communities and government agencies.
+CIEIF aims to help climate-intervention projects better understand their potential technical, environmental, economic, social, public-health, and safety impacts before and during field testing. It also places importance on the scalability and global relevance of supported innovations and encourages publication of field-test results through peer-reviewed journals or externally peer-reviewed reports.
+ About the Grant
+The Climate Intervention Environmental Impact Fund (CIEIF) Grant provides USD 75,000 to support proposed climate intervention field tests. The funding is specifically intended for Environmental Impact Assessment (EIA), predictive impact modelling, and/or engagement with potentially affected stakeholders, including local communities and government agencies.
+Applicants are expected to demonstrate the proposed field test’s technical readiness, environmental and social considerations, required government approvals, innovation and potential for globally relevant scalability. The application must include a proposed budget showing how the USD 75,000 will be used.
+ Grant Objective
+The grant is intended to support proposed climate intervention field tests, particularly activities related to:
+Environmental Impact Assessment (EIA)
+Predictive impact modeling
+Engagement with potentially impacted stakeholders
+Local community and government engagement
+Understanding technical, environmental, economic, social, public-health, and safety challenges
+The proposed application must focus on at least one of these three core areas: EIA, predictive impact modeling, or stakeholder engagement.
+ Eligible Project Focus
+The proposed field test should demonstrate:
+A clear climate-intervention concept
+Prior research indicating that the technology is ready for the proposed field test
+Potential for innovation and scalability
+A clear understanding of technical and environmental challenges
+Consideration of economic, social, public-health, and safety implications
+Relevant government permits and approvals
+Potential for scaling the innovation to a globally relevant level</t>
+        </is>
+      </c>
+      <c r="D26" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E26" s="1" t="inlineStr">
+        <is>
+          <t>Dec 1, 2026</t>
+        </is>
+      </c>
+      <c r="F26" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-cieif-grant-2026-climate-intervention-environmental-impact-fund-climate-intervention-environmental-impact-fund-opg-26-00155</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="95" customHeight="1">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 6th Annual Seeding The Future Global Food System Challenge</t>
         </is>
       </c>
-      <c r="C24" s="1" t="inlineStr">
+      <c r="C27" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are one of the largest and most respected private organisations for development cooperation and humanitarian aid in Germany. As a politically and confessionally independent organisation, our value-oriented actions are always based on ethical principles. Our vision is clear: "Zero Hunger by 2030"
@@ -1999,34 +2093,34 @@
 Individuals with no organizational entity</t>
         </is>
       </c>
-      <c r="D24" s="1" t="inlineStr">
+      <c r="D27" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E24" s="1" t="inlineStr">
+      <c r="E27" s="1" t="inlineStr">
         <is>
           <t>Jan 1, 2027</t>
         </is>
       </c>
-      <c r="F24" s="1" t="inlineStr">
+      <c r="F27" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-6th-annual-seeding-the-future-global-food-system-challenge-welthungerhilfe-opg-26-00180</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="95" customHeight="1">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B25" s="1" t="inlineStr">
+    <row r="28" ht="95" customHeight="1">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for BES Training and Travel Grants</t>
         </is>
       </c>
-      <c r="C25" s="1" t="inlineStr">
+      <c r="C28" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are a global community of scientists shining a spotlight on the intricacy and value of our natural world, providing the evidence for better decisions. Our vision is for people and nature to thrive in a world that values ecology.
@@ -2065,17 +2159,17 @@
  Application Deadline (Round 2): Opens 30 April 2026, closes 17 May 2026</t>
         </is>
       </c>
-      <c r="D25" s="1" t="inlineStr">
+      <c r="D28" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E25" s="1" t="inlineStr">
+      <c r="E28" s="1" t="inlineStr">
         <is>
           <t>May 17, 2027</t>
         </is>
       </c>
-      <c r="F25" s="1" t="inlineStr">
+      <c r="F28" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-bes-training-and-travel-grants-british-ecological-society-opg-26-00181</t>
         </is>

</xml_diff>

<commit_message>
Auto update Combined.xlsx [Tue Sep 22 07:14:08 UTC 2026]
</commit_message>
<xml_diff>
--- a/output/Combined.xlsx
+++ b/output/Combined.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -467,141 +467,10 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Applications Invited for GEF SGP CSO Challenge Program</t>
+          <t>RFP for Impact Assessment</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-The Global Environment Facility Small Grants Programme (SGP) is a global initiative implemented by the United Nations Development Programme (UNDP) on behalf of the Global Environment Facility (GEF). Since its launch in 1992, SGP has empowered communities worldwide to take action on environmental challenges while improving livelihoods. As a GEF Corporate Programme, SGP provides direct support to civil society organisations and community-based organisations to design and implement innovative, locally driven solutions. The programme places strong emphasis on inclusion, ensuring meaningful participation of Indigenous Peoples, youth, women and girls, and other underrepresented groups.
- About the Opportunity:
-The GEF SGP CSO Challenge Program is a new global program that seeks to identify, reward, support, and scale up high-impact innovative environmental solutions from civil society organizations (CSOs). Selected CSOs receive up to $300,000 USD in direct grants, along with demand-driven capacity building and support to strengthen impact and share good practices. This is part of the GEF's broader Small Grants Program (SGP) — active since 1992, having delivered over $838 million in project funding to nearly 30,000 community-based projects across 136 countries. The Challenge Program specifically uses larger grants (vs. the $75k cap of the Core SGP), a global open call (vs. national-level calls), and offers tailored program-level support.
- Program Objectives:
-Recognize and support high-impact CSO-led initiatives addressing global environmental challenges
-Enhance CSO capacity to design, implement, and scale innovative environmental solutions
-Foster knowledge creation, peer-to-peer learning, and partnerships among CSOs, governments, donors, and the private sector
-Support inclusion of under-represented groups (women, youth, Indigenous Peoples, local communities) in CSO-led conservation
- Grant Use — Grants support CSOs in:
-Replicating proven models in new communities/contexts/locations
-Adapting existing solutions to local conditions
-Testing scaling approaches for promising innovations
- Non-Financial Support Provided:
-Organizational capacity building (green entrepreneurship, financial management, leadership, policy influencing, communications, proposal development, innovation/risk management)
-Technical training on IUCN tools for assessing/strengthening/monitoring conservation work (threatened ecosystems, biodiversity, protected areas, agricultural landscapes, urban environments)
-Visibility and networking opportunities via peer-learning platforms, global/regional knowledge exchange workshops, and communities of practice
-Runners-up (non-winning finalists) receive recognition + access to capacity-development support and networks (though not direct grant funding)
- Eligibility:
-Proponents/initiatives must be based in GEF recipient countries (list: https://www.thegef.org/projects-operations/recipient-countries)
-Must be a Civil Society Organization (CSO) with legal entity status and a bank account in the organization's name
-Project must be a replication/scaling of already-tested initiatives or work under implementation (not just a concept)
-Project must align with at least 1 of 5 SGP 2.0 priority areas:
-Community-based management of threatened ecosystems and species
-Sustainable agriculture and fisheries, and food security
-Low-carbon energy access and co-benefits
-Local to global coalitions for chemicals and waste management
-Catalyzing sustainable urban solutions
-Proposals can be subnational, national, regional, or global in scope
-Special encouragement for proposals from/with extensive participation of youth, women, Indigenous Peoples, and local communities
- Grant Amount: Up to $300,000 USD per organization
- Selection Criteria (13 categories):
-Alignment with SGP 2.0 priority areas
-Impact potential (global environmental benefits)
-Alignment/support to countries delivering on national MEA commitments (CBD, UNFCCC, UNCCD, GBF, etc.)
-Scalability
-Inclusivity (diversity of stakeholders, youth/women/Indigenous-led networks)
-Innovation (technological, finance, business models, policy, institutional)
-Robust Theory of Change and Logical Framework
-Technical competency of proponent
-Financial viability (budget + co-financing adequacy, cost efficiency)
-Sustainability beyond project end
-Partnerships and cooperation with key stakeholders
-Commitment to knowledge sharing and learning
-Risk management and mitigation</t>
-        </is>
-      </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>Sep 23, 2026</t>
-        </is>
-      </c>
-      <c r="F2" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-gef-sgp-cso-challenge-program-gef-small-grants-programme-sgp-opg-26-00184</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="95" customHeight="1">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>SoW - Hiring an External Agency for Orientation and Capacity Building</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t>Room to Read’s Foundational Literacy Program in Jharkhand
-Anchoring and Delivery of Orientation Programme for Jharkhand Field Workforce
-Scope of Work (SoW)
-for
-Hiring an External Agency for Orientation and Capacity Building
-Organizational Overview
- Founded in 2000 on the belief that World Change Starts with Educated Children®, Room to Read develops children’s foundational literacy skills, as well as life skills that promote gender equality. We nurture these essential skills in children by training and coaching educators, creating quality learning materials and spaces, strengthening education systems, and delivering programs directly and with partners – all while honouring the dignity of every child. Committed to accelerating learning outcomes for more children, more quickly, Room to Read has benefited children across 29 countries, with more than 17 million children actively benefiting from our programming in 2025 alone. Room to Read India’s literacy operations currently span across 12 states, with a focus on improving children’s reading skills, access to quality learning materials, and supportive learning environments. Room to Read envisions a world free from illiteracy and gender inequality, where all children have room to read, learn and grow. Visit us at https://www.roomtoreadindia.org/
-Jharkhand Foundational Literacy Project Overview
- Room to Read is preparing for a significant scale-up of its Foundational Literacy &amp; Numeracy initiative in Jharkhand, expanding implementation across multiple districts and requiring a substantial field workforce to support programme delivery. As Room to Read expands its field implementation in Jharkhand, a substantial number of staff will join different field-facing and supervisory roles.  As part of the planned scale-up, Room to Read expects to onboard more than 150 staff in Phase 1 across field implementation, supervisory and district-level leadership roles. A second cohort of approximately 120 additional staff is expected to be onboarded in Phase 2 as implementation expands to the remaining districts.
- Objective of the Assignment
-The overarching objective of this assignment is to ensure that over two phases 250+ team members in Jharkhand are ready for project implementation.
-Phase 1 will aim at getting all 150+ staff members ready for project implementation by March 31st, 2027.
-Phase 2 will follow the same approach for an additional 120+ team members, with the orientation programme to be completed by 30 March 2028, followed by final review, handover and closure activities in April 2028.
-Agency Requirements &amp; Qualifications 
-The agency should preferably:
-Preferred 3 years of relevant experience in designing and delivering orientation, training or capability-building programmes for field-based teams, particularly in the education, development or government-facing sector.
-Have completed at least 2 similar assignments involving training across multiple batches, locations or large participant groups.
-Demonstrate experience in learning-needs assessment, adult-learning design, content development and participatory training methodologies.
-Demonstrate experience in developing facilitator guides, participant materials, simulations, assessments, job aids or other training resources, and provide 1-2 relevant samples where available.
-Have the ability to deliver training in Hindi and deploy an adequate pool of suitable facilitators for implementation across Jharkhand.
-Provide details and CVs of the proposed core team and key facilitators, including their qualifications, relevant experience, roles and expected level of engagement in the assignment. The agency should ensure continuity of key facilitators, with minimal changes during each phase of the assignment.
-Demonstrate experience in assessing training effectiveness through participant feedback, assessments, learning-progress tracking and/or follow-up or refresher support.
-Have established systems for project management, quality assurance, documentation, progress tracking and reporting, with the ability to maintain consistency across training cohorts.
-Provide details of at least 2 relevant past clients/assignments that may be referred to for verification of experience and performance</t>
-        </is>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>Sep 23, 2026</t>
-        </is>
-      </c>
-      <c r="F3" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/sow-hiring-an-external-agency-for-orientation-and-capacity-building-room-to-read-india-rfp-26-00366</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="95" customHeight="1">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>RFP for Impact Assessment</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>Introduction
 Titan Company Limited, a member of the Tata Group, has a long-standing commitment to Corporate Social Responsibility (CSR) in India. The company's CSR initiatives derive its philosophy from the Company’s vision statement: “We create elevating experiences for the people we touch and significantly impact the world we work in”. The initiatives are designed to promote inclusive growth, empower communities, and contribute to the country's socio-economic development. The program includes Titan’s CSR policy is governed by a dedicated CSR Committee that ensures transparency and compliance with regulatory requirements. The program includes Girl Child Education, Skill and Entrepreneurship Development, supporting Indian Heritage Arts and Crafts, Integrated Village Development Programme, Eye Care and Affirmative Action. Titan's CSR policy is governed by a dedicated CSR Committee that ensures transparency and compliance with regulatory requirements.
@@ -635,34 +504,34 @@
 Timeline: Proposal submission deadline: September 24, 2026</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>Sep 24, 2026</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfp-for-impact-assessment-titan-rfp-26-00354</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="95" customHeight="1">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
+    <row r="3" ht="95" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>EOI- Engagement of State-Level Field Facilitation Consultants for Project Learning Study</t>
         </is>
       </c>
-      <c r="C5" s="1" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Expression of Interest (EOI)
 For
@@ -723,34 +592,34 @@
 This stage is for collecting information from interested Consultant. AIFT will review the submissions and may issue a detailed Request for Quotation (RFQ) to shortlisted consultant based on the specific assignments.</t>
         </is>
       </c>
-      <c r="D5" s="1" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E5" s="1" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Sep 25, 2026</t>
         </is>
       </c>
-      <c r="F5" s="1" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/eoi-engagement-of-state-level-field-facilitation-consultants-for-project-learning-study-american-india-foundation-rfp-26-00367</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="95" customHeight="1">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
+    <row r="4" ht="95" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>ToR - Engagement of Information Design &amp; Video Production Agency / Consultant for Key Learning &amp; Dissemination Outputs</t>
         </is>
       </c>
-      <c r="C6" s="1" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>Terms of Reference (TOR) for Consultancy Services
 Title  Engagement of Information Design &amp; Video Production Agency / Consultant for Key Learning &amp; Dissemination Outputs
@@ -769,34 +638,34 @@
 The primary objective of this engagement is to enable SELCO Foundation to effectively capture, structure, and communicate its field insights, sectoral learnings, and program impacts. The selected Agency/Consultant (or Agencies/Consultants) will work on a monthly retainer basis to translate raw content, data, field footage, and reports provided by SELCO into high-quality, visually compelling, reader-friendly visual outputs and video assets.</t>
         </is>
       </c>
-      <c r="D6" s="1" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E6" s="1" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>Sep 28, 2026</t>
         </is>
       </c>
-      <c r="F6" s="1" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-engagement-of-information-design-and-video-production-agency-consultant-for-key-learning-and-dissemination-outputs-selco-foundation-rfp-26-00362</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="95" customHeight="1">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
+    <row r="5" ht="95" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>ToR - Video documentation of change stories on Ground water replenishment in Hyderabad and Sanga Reddy locations</t>
         </is>
       </c>
-      <c r="C7" s="1" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>About Jal Seva Charitable Foundation/ WaterAid India:
 Jal Seva Charitable Foundation (JSCF) is registered in India as a not-for-profit company under Chapter 8 of the Companies Act, 2013. JSCF, is an associate member of WaterAid International and uses the brand name ‘WaterAid’ in India.
@@ -830,34 +699,34 @@
 Upon completion of Assignment</t>
         </is>
       </c>
-      <c r="D7" s="1" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E7" s="1" t="inlineStr">
+      <c r="E5" s="1" t="inlineStr">
         <is>
           <t>Sep 28, 2026</t>
         </is>
       </c>
-      <c r="F7" s="1" t="inlineStr">
+      <c r="F5" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-video-documentation-of-change-stories-on-ground-water-replenishment-in-hyderabad-and-sanga-reddy-locations-wateraid-india-rfp-26-00363</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="95" customHeight="1">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
+    <row r="6" ht="95" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>ToR - Video Production Storytelling and Documentation</t>
         </is>
       </c>
-      <c r="C8" s="1" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>Title Video Production – Storytelling and Documentation
 Timeline 3 months from the date of contracting
@@ -891,98 +760,101 @@
 Quotation Should include all cost including Travel and Miscellaneous.</t>
         </is>
       </c>
-      <c r="D8" s="1" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E8" s="1" t="inlineStr">
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>Sep 29, 2026</t>
         </is>
       </c>
-      <c r="F8" s="1" t="inlineStr">
+      <c r="F6" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-video-production-storytelling-and-documentation-selco-foundation-rfp-26-00368</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="95" customHeight="1">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Setting up Viral Research and Diagnosis Laboratories VRDL in Medical Colleges/Hospitals/Medical Institutions</t>
-        </is>
-      </c>
-      <c r="C9" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-The President notified the creation of the Department of Health Research under the Ministry of Health &amp; Family Welfare through an amendment to the Government of India (Allocation of Business) Rules, 1961 on the 17th September 2007. The Department of Health Research was formally launched on 5th October 2007 by the Minister for Science &amp; Technology and Earth Sciences in a function presided over by the Minister for Health &amp; Family Welfare, in the presence, inter-alia, of the Minister of State for Health &amp; Family Welfare.
-The Department became functional from November 2008 with the appointment of first Secretary of the Department The aim of the DHR is to bring modern health technologies to the people through research and innovations related to diagnosis, treatment methods and vaccines for prevention, to translate them into products and processes and, in synergy with concerned organizations, introduce these innovations into public health system.
- About the Opportunity:
-Under DHR's scheme "Setting-up of nation-wide network of laboratories for managing epidemics and national calamities," proposals are invited from Medical Colleges/Hospitals/Research Institutions to establish a Medical College &amp; Research Institute Level – Viral Research and Diagnosis Laboratory (MCL-VRDL). The existing network comprises 167 VRDLs (11 Regional, 27 State, 129 Medical College level) across 27 states and 5 UTs, aimed at early detection of infectious pathogens, outbreak surveillance, and research on emerging/re-emerging viral diseases.
- Objectives:
-Establish capacity for early detection of common and high-risk infectious pathogens
-Strengthen syndromic surveillance ecosystem for outbreak detection
-Undertake R&amp;D on emerging, re-emerging and novel viruses
- Eligibility (Institution-level):
-State Government Medical Colleges
-Central Government Medical Colleges and Research Institutes
-Armed Forces Medical Institutions/Hospitals
-Railway and other Central Government health institutions
-Private medical colleges ranked in top 50 NIRF ranking
-Must have a dedicated Microbiology department with qualified faculty
-Must have &gt;200 sq.m. area available in existing building (preferably within Microbiology Dept.)
- Funding Provision:
-Non-recurring assistance: Rs. 1.55 crore total
-Rs. 66.8 lakhs — Civil Work (infrastructure modification)
-Rs. 88.2 lakhs — Equipment (complete lab setup)
-No recurring expenditure (staff salaries, consumables, contingency) is provided — to be borne by the host institution
- Role &amp; Responsibilities of the Lab:
-Conduct routine diagnosis of infectious pathogens
-Participate in syndromic and event-based surveillance
-Provide support during outbreaks/epidemics
-Share data with ICMR
- Selection Criteria:
-Meeting eligibility does not guarantee selection; merit-based evaluation by a technical committee
-Preference to institutions in geographically underserved regions
-Weightage for technical strength (qualified faculty, biosafety practices, outbreak investigation experience, publications, patents, externally funded projects)
-Additional weightage for molecular diagnostics, genomic surveillance, One Health research capability, and commitment to long-term recurring support
-Private medical colleges: only top-50 NIRF-ranked institutions considered</t>
-        </is>
-      </c>
-      <c r="D9" s="1" t="inlineStr">
+    <row r="7" ht="95" customHeight="1">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>EOI Inviting Expression of Interest-cum-Proposal for Setting Up District De-Addiction Centres under NAPDDR</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>About us
+In the year 1985-86, the erstwhile Ministry of Welfare was bifurcated into the Department of Women and Child Development and the Department of Welfare. Simultaneously, the Scheduled Castes Development Division, Tribal Development Division and the Minorities and Backward Classes Welfare Division were moved from the Ministry of Home Affairs and also the Wakf Division from the Ministry of Law to form the then Ministry of Welfare Subsequently, the name of the Ministry was changed to the Ministry of Social Justice &amp; Empowerment in May, 1998. Further, in October, 1999, the Tribal Development Division had moved out to form a separate Ministry of Tribal Affairs. In January, 2007, the Minorities Division along with Wakf Unit have been moved out of the Ministry and formed as a separate Ministry and the Child Development Division has gone to the Ministry of Women &amp; Child Development.
+ Department of Social Justice and Empowerment invites Expression of lnterest-cum-proposal from the eligible organizations for setting up of District DeAddiction Centres under the scheme of National Action Plan for Drug Demand Reduction (NAPDDR) for 315 GAP Districts of the country (as per list attached at Annexure - l). The list of districts is subject to change (addition or deletion) time to trme by the Ministry as per requirement or need on the ground.
+ 2. Eligible NGOs may apply for setting up of DDAC provided that they have rent free accommodation for setting up of DDAC as per the standards of guideline of the NAPDDR scheme or renlfree accommodation may also be provided by the concerned District Administration. 
+ 3. Setting up and running of District De-Addiction Centres (DDACS) will be done as per the following guidelinesr. 
+ i. There will be a District De-Addiction Centre (DDAC) preferably in each district headquarter or suitably accessible place where rent free accommodation is provided by the district administration. These DDACs would provide comprehensive facilities hitherto being provided by IRCA, ODIC &amp; CPLI together. lf the district administration of identified district is not able to provide suitable rent free accommodation, then the application will be called from the eligible VOs/ NGOs, who will provide rent free accommodation for setting up of DDAC in that district.
+ ii. The functioning of DDAC will be monitored by the three tier Committees headed by the Chief Secretary, District Collector/Deputy Commissioner and Block Development Officer of the respective arealregion which have been formed under Nasha Mukt Bharat Abhiyaan (NMBA). Additionally, retired eminent personalities of the Districts, activists, Vice-Chancellor/ Head of Department (HoD)/ Principal, researcher, scholars and so on may be co-opted by Chairman as the members of the Committees. These commiftees would
+ only monitor policy related issues. Day to day and other activities relating to implementation would be the responsibility of the concerned organization/NGO approved for setting up of the DDAC. The Meetings of DDAC are to be held as per the details given below:
+ (a) State-level Steering and Monitoring Committee (High Level Task Force) - headed by Chief Secretary - to meet quarterly. (b) District-level Committee - headed by District Collector / Deputy Commissioner - to meet monthly and have mandatory inspections quarterly. (c) Block level Committee - headed by Block Development Officer - to meet &amp; have mandatory inspections monthly.
+ The Committees will also review the functioning and assess the performance of the DDAC in terms of the effectiveness of deliverables and make further suggestions to the management of DDAC. 
+ IIl t. A separate (dedicated) account will be opened for keeping funds of DDAC in the name of NGO/Organization. The account will be registered on PFMS and implemented through EAT Module. 
+ lV. For setting up of DDACs, preference would be given to those Districts, which do not have any facility of IRCA or DDAC. For this, the organization willing to work in the field of DRUGS DE-ADDICTION TREATMENT will be eligible for applying for DDAC. The priority for selection of DDAC would be: 
+a. The DDAC proposed to be run by the District administration itself. 
+b. Rent free accommodation in the district headquarter provided by the concerned DC/DM &amp; further willingness from interested NGO is sought. c, Where no proposal for rent-free accommodation is received from concerned DCiDM, interested NGO may directly apply for DDAC provided they do not seek any rent for same and only building maintenance will be given. 
+V. The details of Minimum standards like physical space and necessary amenities to be provided by District administration or NGOs are as under: 
+(a) The centre should be easily accessible and connected through public transport. 
+(b) The total built-in area of the DDAC should be at least 3000 sq,ft. in case of metros and 4000 sq.ft. in case of small towns and villages to house 15 patients and 4000 sq.ft. in case of metros and 5000 sq.ft. in case of small towns and villages to house 30 patients. This includes an area of about 2000 sq. ft. for Treatment cum Rehabilitation centre, an area of about 700 sq. ft. for Drop-ln Centre facilities and an area of about 300 sq. ft. for CPLI Centre facilities. 
+(c) The centre should be properly ventilated, well-lit and maintained in a clean manner. Water to be made available. 
+(d) Basic safety of the patients to be ensured 
+(e) Facilities at the centre - Waiting space with seating arrangements for a minimum 5 persons Cubicles / rooms for consultation for physical examination Facilities to store drugs, linen, and records of patients Facilities with privacy for providing individual counselling, group therapy, re-educative sessions, family classes. They should be airy with comfortable seating with floor mats / chairs. Blackboard, chalk and other material to be provided. Availability of recreational facilities. Separate Drop ln Facility centre with recreation room, counselling room and medical room. Project room for CPLI activities including consultation room for interviewing Vl. Standards set in the above para of the guidelines may change from time to time as and when necessary with the approval of competent authority and the stakeholders / NGOs/ VOs would be intimated of same as and when such changes happen. 
+ 4. The interested and eligible NGOs / organizations can apply through eAnudaan (https://grants-msje.gov.in/ngo-login) portal of the Ministry. The Project Screening Committee in the Ministry will select the eligible NGO(s) for establishing and running of the DDAC and recommend the release of funds in two installments. However, the organization shall be eligible for receiving GIA under the scheme from the date of approval of the competent authority. 
+ 5. ELIGIBLE ORGANIZATION: 
+Organizations which are already running MoSJE supported IRCA or State Government supported De-addiction Centre/ Government Hospital or any private run De-Addiction centre are eligible for applying for DDAC. Organization can apply only for that State/UT in which they are already running IRCA"/De-addiction Centre from the last 2 years or more from the date of call for the proposal. Condition may be relaxed for any Government run Hospitals, which are non-profitable in nature. I 
+6. Start-up consists of young persons/ professionals, who have graduated from top social institutes of lndia or abroad are also eligible to apply. However, they must have experience of 2 years in the field of Drug De-addiction TREATMENT. 7. Role and Responsibility of DDACs The main focus of the DDAC is early prevention, education, demand reduction, identification, treatment and rehabilitation services of vulnerable individuals or individuals affected by substance use disorders DDAC would: 
+a. Conduct primary prevention activities through awareness programs among the vulnerable and affected community 
+b. Engage in risk mitigation of substance use among children/ adolescenuyouth by: Preventing substance use Delaying initiation of substance use 
+c. ldentify and train selected peer educators in the community 
+d. lmplement early prevention education through life skill training led by trained peer educators 
+e. Provide awareness about referral and linkage to counseling, treatment and rehabilitation services for substance dependent adolescents identified in the community 
+f. ldentifying adolescents and other individuals subjected to substance use and facilitating their referrali admission into Rehabilitation Centers/ Drop ln Centres. 
+g. Provide a whole range of services which includes treatment, after care and rehabilitation including skill development for Whole Person Recovery (WPR) of dependents; 
+h. Undertake drug demand reduction efforts to address all forms of illicit use of any substances and ensure overall well being of humankind; 
+i. Alleviate the consequences of substance dependence amongst individuals, family and society at large 
+9. The budget details of DDAC is attached as Annexure - 
+10. The e-anudaan portal shall remain open through out the year and the recommendations from the States/UTs will be considered periodically. 
+11. Department of Social Justice and Empowerment (DoSJE) reserves the right to cancel this notice, andior invite afresh proposals with or without amendments to this document without liability or any obligation for such document, and without assigning any reason. DoSJE reserves the right to take final decision regarding selection of implementing agency or project.</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E9" s="1" t="inlineStr">
+      <c r="E7" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F9" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-setting-up-viral-research-and-diagnosis-laboratories-vrdl-in-medical-collegeshospitalsmedical-institutions-department-of-health-research-dhr-ministry-of-health-and-family-welfare-government-of-india-opg-26-00174</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="95" customHeight="1">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/eoi-inviting-expression-of-interest-cum-proposal-for-setting-up-district-de-addiction-centres-under-napddr-ministry-of-social-justice-and-empowerment-goi-rfp-26-00356</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="95" customHeight="1">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>Application Invited for Giving Joy Microgrant</t>
         </is>
       </c>
-      <c r="C10" s="1" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Giving Joy is a US-based nonprofit that strengthens and inspires women’s entrepreneurship worldwide. Through its micro-grants and mentorship program, Giving Joy helps women establish or improve their businesses and initiatives—for their benefit and the benefit of their communities. To date, Giving Joy has awarded over 88 grants to women-led initiatives in 26 countries.
@@ -1021,34 +893,34 @@
 The grant period is six months.</t>
         </is>
       </c>
-      <c r="D10" s="1" t="inlineStr">
+      <c r="D8" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E10" s="1" t="inlineStr">
+      <c r="E8" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F10" s="1" t="inlineStr">
+      <c r="F8" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/application-invited-for-giving-joy-microgrant-giving-joy-opg-26-00185</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="95" customHeight="1">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="inlineStr">
+    <row r="9" ht="95" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
         <is>
           <t>ToR - Branding Development &amp; Design/Market Promotion Consultant Project Sashakt</t>
         </is>
       </c>
-      <c r="C11" s="1" t="inlineStr">
+      <c r="C9" s="1" t="inlineStr">
         <is>
           <t>Organisation Humana People to People India (HPPI)
 Project Sashakt – Strengthening Women-led Handloom Cooperatives in Assam (EU-funded)
@@ -1103,34 +975,34 @@
 The consultant/agency must ensure ethical, consent-based data collection with cultural sensitivity, particularly when engaging women weavers. All data and reports remain the property of HPPI and must be kept strictly confidential, with no external use.</t>
         </is>
       </c>
-      <c r="D11" s="1" t="inlineStr">
+      <c r="D9" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E11" s="1" t="inlineStr">
+      <c r="E9" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F11" s="1" t="inlineStr">
+      <c r="F9" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-branding-development-and-designmarket-promotion-consultant-project-sashakt-humana-people-to-people-india-rfp-26-00365</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="95" customHeight="1">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="inlineStr">
+    <row r="10" ht="95" customHeight="1">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Signals of Change Shaping the Future of Sexual and Reproductive Health and Rights SRHR</t>
         </is>
       </c>
-      <c r="C12" s="1" t="inlineStr">
+      <c r="C10" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The World Health Organization's mission: to promote health, keep the world safe, and serve the vulnerable. Working through offices in more than 150 countries, WHO staff work side by side with governments and other partners to ensure the highest attainable level of health for all people.
@@ -1155,34 +1027,98 @@
  Submission Requirements: Descriptive information (name, contact email, country, sector) required alongside each submission; formal published evidence is helpful but not required — practice-based experience and field examples are also welcome. Submissions are kept confidential and anonymized before analysis.</t>
         </is>
       </c>
-      <c r="D12" s="1" t="inlineStr">
+      <c r="D10" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E12" s="1" t="inlineStr">
+      <c r="E10" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F12" s="1" t="inlineStr">
+      <c r="F10" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-signals-of-change-shaping-the-future-of-sexual-and-reproductive-health-and-rights-srhr-world-health-organization-opg-26-00176</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="95" customHeight="1">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B13" s="1" t="inlineStr">
+    <row r="11" ht="95" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Setting up Viral Research and Diagnosis Laboratories VRDL in Medical Colleges/Hospitals/Medical Institutions</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+The President notified the creation of the Department of Health Research under the Ministry of Health &amp; Family Welfare through an amendment to the Government of India (Allocation of Business) Rules, 1961 on the 17th September 2007. The Department of Health Research was formally launched on 5th October 2007 by the Minister for Science &amp; Technology and Earth Sciences in a function presided over by the Minister for Health &amp; Family Welfare, in the presence, inter-alia, of the Minister of State for Health &amp; Family Welfare.
+The Department became functional from November 2008 with the appointment of first Secretary of the Department The aim of the DHR is to bring modern health technologies to the people through research and innovations related to diagnosis, treatment methods and vaccines for prevention, to translate them into products and processes and, in synergy with concerned organizations, introduce these innovations into public health system.
+ About the Opportunity:
+Under DHR's scheme "Setting-up of nation-wide network of laboratories for managing epidemics and national calamities," proposals are invited from Medical Colleges/Hospitals/Research Institutions to establish a Medical College &amp; Research Institute Level – Viral Research and Diagnosis Laboratory (MCL-VRDL). The existing network comprises 167 VRDLs (11 Regional, 27 State, 129 Medical College level) across 27 states and 5 UTs, aimed at early detection of infectious pathogens, outbreak surveillance, and research on emerging/re-emerging viral diseases.
+ Objectives:
+Establish capacity for early detection of common and high-risk infectious pathogens
+Strengthen syndromic surveillance ecosystem for outbreak detection
+Undertake R&amp;D on emerging, re-emerging and novel viruses
+ Eligibility (Institution-level):
+State Government Medical Colleges
+Central Government Medical Colleges and Research Institutes
+Armed Forces Medical Institutions/Hospitals
+Railway and other Central Government health institutions
+Private medical colleges ranked in top 50 NIRF ranking
+Must have a dedicated Microbiology department with qualified faculty
+Must have &gt;200 sq.m. area available in existing building (preferably within Microbiology Dept.)
+ Funding Provision:
+Non-recurring assistance: Rs. 1.55 crore total
+Rs. 66.8 lakhs — Civil Work (infrastructure modification)
+Rs. 88.2 lakhs — Equipment (complete lab setup)
+No recurring expenditure (staff salaries, consumables, contingency) is provided — to be borne by the host institution
+ Role &amp; Responsibilities of the Lab:
+Conduct routine diagnosis of infectious pathogens
+Participate in syndromic and event-based surveillance
+Provide support during outbreaks/epidemics
+Share data with ICMR
+ Selection Criteria:
+Meeting eligibility does not guarantee selection; merit-based evaluation by a technical committee
+Preference to institutions in geographically underserved regions
+Weightage for technical strength (qualified faculty, biosafety practices, outbreak investigation experience, publications, patents, externally funded projects)
+Additional weightage for molecular diagnostics, genomic surveillance, One Health research capability, and commitment to long-term recurring support
+Private medical colleges: only top-50 NIRF-ranked institutions considered</t>
+        </is>
+      </c>
+      <c r="D11" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>Sep 30, 2026</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-setting-up-viral-research-and-diagnosis-laboratories-vrdl-in-medical-collegeshospitalsmedical-institutions-department-of-health-research-dhr-ministry-of-health-and-family-welfare-government-of-india-opg-26-00174</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="95" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
         <is>
           <t>RFP - Design and Delivery of an Electric Vehicle EV Skilling Programme in Karnataka</t>
         </is>
       </c>
-      <c r="C13" s="1" t="inlineStr">
+      <c r="C12" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 WRI India, an independent knowledge organisation registered as the India Resources Trust, provides objective information and practical proposals to foster environmentally sound and socially equitable development. As an independent knowledge organisation, we leverage our data and expertise to catalyze change across systems like food, land and water; energy; and cities. Our work focuses on improving people’s lives, protecting and restoring nature, and addressing climate change. To enable progress at the pace and scale needed, we also engage with the economic, finance and governance systems that are key to enabling this change.
@@ -1223,6 +1159,59 @@
 Must have a team of qualified trainers and master trainers with relevant domain expertise, as well as administrative and coordination support.</t>
         </is>
       </c>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>Oct 5, 2026</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/rfp-design-and-delivery-of-an-electric-vehicle-ev-skilling-programme-in-karnataka-wri-india-rfp-26-00361</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="95" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>RFPs Invited for Engagement of a Manpower Agency for Providing Subject Matter Specialists/Experts for the Cluster Development Programme</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>About the RFP
+National Horticulture Board (NHB), an autonomous organization under the Ministry of Agriculture and Farmers' Welfare, Government of India, invites bids from eligible manpower agencies for engagement to recruit, deploy, and manage qualified personnel supporting NHB's Cluster Development Programme (CDP) — a Central Sector Scheme promoting integrated, market-led horticulture cluster development. The engaged agency will provide three types of Subject Matter Experts per Cluster and additional consultants/manpower as required by NHB from time to time.
+ Scope of Personnel to be Provided:
+Subject Matter Expert – Horticulture/Agribusiness
+Monitoring &amp; Evaluation Expert
+Infrastructure Expert
+Additional consultants/experts/manpower as requisitioned by NHB from time to time
+ Eligibility (for Bidding Agency):
+Must be an Indian entity registered under applicable law (Company/Society/Trust/Partnership/LLP/Sole Proprietorship)
+Must be operational in India, engaged in manpower outsourcing, staffing, recruitment, deployment of professional/technical manpower, or similar services
+Valid registrations required: PAN, GST, EPF, ESI (wherever applicable)
+Valid labour licence under the Contract Labour (Regulation &amp; Abolition) Act, 1970 (wherever applicable)
+Must have completed/initiated at least 3 similar assignments in the last 5 years for Central/State Government Departments, PSUs, Autonomous Bodies, or Statutory Authorities
+Minimum value of similar services in last 7 financial years: 3 services of ≥₹1.44 crore each, OR 2 services of ≥₹1.80 crore each, OR 1 service of ≥₹2.88 crore
+Annual average turnover of at least ₹10.80 crore (F.Y. 2023-24, 2024-25 &amp; 2025-26)
+Positive net worth as on last financial year-end
+Must not be blacklisted/debarred by any Government/PSU in India
+ Qualification: N/A (agency-level eligibility, not individual — see above)
+ Experience Bracket: Agency must have 5+ years of relevant institutional experience (per similar-services criteria above)
+ Application Deadline: 6 October 2026, 5:00 PM (Bid Due Date)
+ State: Pan-India (Authority based in Haryana)
+ District: Gurugram, Haryana (NHB Head Office)</t>
+        </is>
+      </c>
       <c r="D13" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
@@ -1230,12 +1219,12 @@
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>Oct 5, 2026</t>
+          <t>Oct 6, 2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/rfps/rfp-design-and-delivery-of-an-electric-vehicle-ev-skilling-programme-in-karnataka-wri-india-rfp-26-00361</t>
+          <t>https://onepurpos.in/openings/rfps/rfps-invited-for-engagement-of-a-manpower-agency-for-providing-subject-matter-specialistsexperts-for-the-cluster-development-programme-national-horticulture-board-nhb-rfp-26-00370</t>
         </is>
       </c>
     </row>
@@ -1442,10 +1431,115 @@
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
+          <t>RFPs Invited for Consultant to Develop a Technical Assistance Package for National Application of the Digital Health and AI Investment Classification Framework</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+We are Transform Health: a global coalition of more than 200 organisations driving the digital transformation of health to achieve universal health coverage. 
+Our focus is on strengthening the enabling environment—the  laws, regulation, policies, coordination structures and resources—that ensure the digital health transformation is equitable, inclusive and sustainable and that digital technologies are adopted responsibly, equitably, and at scale.  This means going beyond just the technologies and tools to create the conditions that enable this vision. 
+We tackle complex issues that no single organisation can resolve, leveraging the collective power and expertise of our dynamic coalition. 
+Our work is underpinned by our core values of equity, inclusion, rights, empowerment, and partnership.
+Together, we can achieve universal health coverage in the digital age.
+ About the Role:
+Transform Health is recruiting a consultant to develop a Technical Assistance (TA) approach and package that supports governments in applying the Digital Health and AI Investment Classification Framework, to aid budgeting, costing of digital health strategies/roadmaps, and analysis of digital health investment. The consultant will design the TA package and test it directly with governments in 3-4 countries, refining it based on the learnings. The work will be largely remote, with potential travel to testing countries.
+ Responsibilities:
+Deliverable 1 – Develop the TA package: Review the current draft concept note, Classification Framework, and user guide; conduct user-centric design investigation with likely TA users (government officials, technical partners); translate the three entry points for national use of the Framework into a practical, step-by-step TA delivery approach; develop supporting tools (budget/costing templates, guidance materials); consolidate into a TA package for review before country testing
+Deliverable 2 – Apply the TA package in 3-4 countries: Work with Transform Health and technical partners to identify pilot countries; support government engagement and sign-off (e.g., MoU); lead direct TA delivery in each pilot country; document the process, outputs, adaptations, and structured feedback
+Deliverable 3 – Refine the TA package: Synthesise learnings and feedback from pilot countries; produce a final, ready-to-scale TA package and tools; write a final report with recommendations; write brief case studies (~2 pages each) per pilot country; present findings to Transform Health; draft a journal article based on the process and outcomes
+ Eligibility:
+Willingness and ability to travel internationally as required
+Ability to work independently in multi-disciplinary, remote, cross-organisational teams
+ Qualification:
+Demonstrated understanding of the digital health ecosystem, particularly policy and funding landscape
+In-depth understanding of government digital health funding (national budgeting, costing of digital health strategies/frameworks)
+Familiarity with key digital health frameworks and tools
+Knowledge of national health financing systems, budget structures, and investment tracking tools (e.g., National Health Accounts)
+Strong analytical, research, and written communication skills
+Experience with user-centric/human-centred design approaches (needs assessment, prototyping, iterative refinement)
+Demonstrated experience delivering technical assistance directly to government counterparts, ideally across multiple countries
+Ability to manage multi-country consultancy engagements and coordinate with in-country focal points</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>Oct 23, 2026</t>
+        </is>
+      </c>
+      <c r="F17" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/rfps-invited-for-consultant-to-develop-a-technical-assistance-package-for-national-application-of-the-digital-health-and-ai-investment-classification-framework-transform-health-rfp-26-00359</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="95" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for D-Prize Global Competition Seed Funding for New Poverty-Solution Distribution Organizations</t>
+        </is>
+      </c>
+      <c r="C18" s="1" t="inlineStr">
+        <is>
+          <t>About the Grant:
+D-Prize seeds new organizations that distribute proven poverty solutions at the "last mile," with the aim of scaling impact. Applicants select from a range of evidence-based interventions (health, agriculture, education, water, safety, transparency, and more) and propose how they would launch or grow an organization to distribute that intervention. Top entrepreneurs receive up to $20,000 in seed funding to run a pilot and build an organization capable of scaling to reach thousands, even millions of people.
+ Intervention Areas (sample — 20+ tracks available):
+Health: Childhood Diarrhea Treatment, DMPA-SC (contraceptive) initiatives, Reading Glasses, Kangaroo Care, Oxygen access, Maternal Health, Child Immunization, Prevention of Mother-to-Child HIV Transmission, Patient Identification
+Education: Teaching at the Right Level, ConnectEd Phone-based Tutoring, Sugar Daddy Awareness
+Agriculture: Post-Harvest Support, Quality Inputs, Water Filters, custom agriculture proposals
+Livelihoods/Governance: Poverty Graduation, Government Transparency, Road Safety, Childcare
+"Propose Your Own": pitch a distribution model for any credible, evidence-based poverty intervention not listed
+ Eligibility:
+New organizations only — most awardees are first-time entrepreneurs who have not yet launched or raised outside funding
+Applicants from low- and middle-income countries especially encouraged
+Organizations with more than 18 months of full-time operations or more than $30,000 USD already raised are typically not supported
+Existing organizations considered only if their core focus is distributing an existing, evidence-based poverty intervention
+ Qualification: Not specified (open to entrepreneurs of any background; evaluated on quality of distribution concept and execution ability)
+ Experience Bracket: Early-stage/first-time entrepreneurs preferred; not aimed at established organizations
+ Application Deadline:
+Early Submission: 25 October 2026, midnight PT
+Regular Submission: 15 November 2026, midnight PT
+Extension Deadline: 6 December 2026, midnight PT (extension registration required)</t>
+        </is>
+      </c>
+      <c r="D18" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E18" s="1" t="inlineStr">
+        <is>
+          <t>Oct 25, 2026</t>
+        </is>
+      </c>
+      <c r="F18" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-d-prize-global-competition-seed-funding-for-new-poverty-solution-distribution-organizations-d-prize-opg-26-00191</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="95" customHeight="1">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
+        <is>
           <t>Applications Invited for 8th Call for Proposals Small-Size Grants Global EbA Fund</t>
         </is>
       </c>
-      <c r="C17" s="1" t="inlineStr">
+      <c r="C19" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -1508,34 +1602,34 @@
 Only successful applicants will be contacted; no individual feedback provided to unsuccessful applicants</t>
         </is>
       </c>
-      <c r="D17" s="1" t="inlineStr">
+      <c r="D19" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E17" s="1" t="inlineStr">
+      <c r="E19" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F17" s="1" t="inlineStr">
+      <c r="F19" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-8th-call-for-proposals-small-size-grants-global-eba-fund-global-eba-fund-opg-26-00177</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="95" customHeight="1">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="inlineStr">
+    <row r="20" ht="95" customHeight="1">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Adaptive Control Frameworks to Unlock Full-Scale BNR Potential Water Research Foundation WRF</t>
         </is>
       </c>
-      <c r="C18" s="1" t="inlineStr">
+      <c r="C20" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Water Research Foundation (WRF) is the leading research organization advancing the science of all water to meet the evolving needs of its subscribers and the water sector. WRF is a nonprofit, charitable and educational organization which funds, manages, and publishes research on the technology, operation, and management of drinking water, wastewater, reuse, and stormwater collection, treatment and supply systems—all in pursuit of ensuring water quality and improving water services to the public.
@@ -1576,34 +1670,34 @@
 Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
         </is>
       </c>
-      <c r="D18" s="1" t="inlineStr">
+      <c r="D20" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E18" s="1" t="inlineStr">
+      <c r="E20" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F18" s="1" t="inlineStr">
+      <c r="F20" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-adaptive-control-frameworks-to-unlock-full-scale-bnr-potential-water-research-foundation-wrf-the-water-research-foundation-wrf-opg-26-00187</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="95" customHeight="1">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="inlineStr">
+    <row r="21" ht="95" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Crossing the Divide Best Practices for Addressing Local and Privately-Owned Lateral Sewer Issues RFP 5419</t>
         </is>
       </c>
-      <c r="C19" s="1" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>Project Objective:
 To provide water resource recovery facilities (WRRFs) and collection system operators with an interactive manual of practice for implementing inflow and infiltration (I&amp;I) and obstruction management programs, focused on municipal and privately owned lateral sewers in complex legal, regulatory, and multi-jurisdictional environments.
@@ -1641,34 +1735,34 @@
  Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
         </is>
       </c>
-      <c r="D19" s="1" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E19" s="1" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F19" s="1" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-crossing-the-divide-best-practices-for-addressing-local-and-privately-owned-lateral-sewer-issues-rfp-5419-the-water-research-foundation-wrf-opg-26-00189</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="95" customHeight="1">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="inlineStr">
+    <row r="22" ht="95" customHeight="1">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Comparison of PFAS Contributions to Agricultural Systems</t>
         </is>
       </c>
-      <c r="C20" s="1" t="inlineStr">
+      <c r="C22" s="1" t="inlineStr">
         <is>
           <t>Project Objectives:
 Report per- and polyfluoroalkyl substance (PFAS) concentrations from a variety of agricultural inputs — animal manures, fertilizers, pesticides, composts, soil amendments, seed coatings, and biosolids-based products
@@ -1704,34 +1798,34 @@
  Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00) — same deadline as the other two WRF grants</t>
         </is>
       </c>
-      <c r="D20" s="1" t="inlineStr">
+      <c r="D22" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E20" s="1" t="inlineStr">
+      <c r="E22" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F20" s="1" t="inlineStr">
+      <c r="F22" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-comparison-of-pfas-contributions-to-agricultural-systems-the-water-research-foundation-wrf-opg-26-00190</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="95" customHeight="1">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="inlineStr">
+    <row r="23" ht="95" customHeight="1">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Whitley Award 2027</t>
         </is>
       </c>
-      <c r="C21" s="1" t="inlineStr">
+      <c r="C23" s="1" t="inlineStr">
         <is>
           <t>About the Grant: 
 An annual grant by the Whitley Fund for Nature (WFN) recognising grassroots conservation leaders in the Global South, providing funding to support and scale up proven, science-based solutions that deliver lasting impact for both people and nature.
@@ -1744,34 +1838,34 @@
 You do not need to be invited or nominated to apply.</t>
         </is>
       </c>
-      <c r="D21" s="1" t="inlineStr">
+      <c r="D23" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E21" s="1" t="inlineStr">
+      <c r="E23" s="1" t="inlineStr">
         <is>
           <t>Oct 30, 2026</t>
         </is>
       </c>
-      <c r="F21" s="1" t="inlineStr">
+      <c r="F23" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-whitley-award-2027-whitley-fund-for-nature-wfn-opg-26-00153</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="95" customHeight="1">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="inlineStr">
+    <row r="24" ht="95" customHeight="1">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIFAR Global Scholars Program 20272029 Cohort</t>
         </is>
       </c>
-      <c r="C22" s="1" t="inlineStr">
+      <c r="C24" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 CIFAR is a Canadian-based globally influential research organization that convenes the world’s most brilliant people across disciplines to advance transformative knowledge and solve humanity’s biggest problems, together. By supporting long-term interdisciplinary collaboration, CIFAR provides researchers with an unparalleled environment of trust, transparency and knowledge sharing. Our time-tested model inspires new directions of inquiry, accelerates discovery and yields breakthroughs across borders and academic disciplines. Through knowledge mobilization, we are catalysts for change in industry, government and society. Through our 15 research programs and the Pan-Canadian AI Strategy, CIFAR convenes close to 400 of the world’s top researchers from 141 institutions in 20 countries. CIFAR is generously supported by the governments of Canada, Alberta and Québec, as well as foundations, individuals, corporations and Canadian and international partner organizations.
@@ -1815,34 +1909,34 @@
  Application Deadline: November 4, 2026, 12:00 PM EST</t>
         </is>
       </c>
-      <c r="D22" s="1" t="inlineStr">
+      <c r="D24" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E22" s="1" t="inlineStr">
+      <c r="E24" s="1" t="inlineStr">
         <is>
           <t>Nov 4, 2026</t>
         </is>
       </c>
-      <c r="F22" s="1" t="inlineStr">
+      <c r="F24" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cifar-global-scholars-program-20272029-cohort-cifar-canadian-institute-for-advanced-research-opg-26-00183</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="95" customHeight="1">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B23" s="1" t="inlineStr">
+    <row r="25" ht="95" customHeight="1">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for IWRS Teaching Innovation Award</t>
         </is>
       </c>
-      <c r="C23" s="1" t="inlineStr">
+      <c r="C25" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Insects are one of the most numerous and diverse animal groups on Earth.
@@ -1857,34 +1951,34 @@
 IWRS staff and Advisory Group members are not eligible to apply.</t>
         </is>
       </c>
-      <c r="D23" s="1" t="inlineStr">
+      <c r="D25" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E23" s="1" t="inlineStr">
+      <c r="E25" s="1" t="inlineStr">
         <is>
           <t>Nov 15, 2026</t>
         </is>
       </c>
-      <c r="F23" s="1" t="inlineStr">
+      <c r="F25" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00166</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="95" customHeight="1">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B24" s="1" t="inlineStr">
+    <row r="26" ht="95" customHeight="1">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for IWRS Teaching Innovation Award</t>
         </is>
       </c>
-      <c r="C24" s="1" t="inlineStr">
+      <c r="C26" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
@@ -1896,34 +1990,34 @@
 Two awards of $2,000 USD are available annually.</t>
         </is>
       </c>
-      <c r="D24" s="1" t="inlineStr">
+      <c r="D26" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E24" s="1" t="inlineStr">
+      <c r="E26" s="1" t="inlineStr">
         <is>
           <t>Nov 15, 2026</t>
         </is>
       </c>
-      <c r="F24" s="1" t="inlineStr">
+      <c r="F26" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="95" customHeight="1">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B25" s="1" t="inlineStr">
+    <row r="27" ht="95" customHeight="1">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Medium-Size Grants Call for Proposals Global EbA Fund</t>
         </is>
       </c>
-      <c r="C25" s="1" t="inlineStr">
+      <c r="C27" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -1980,34 +2074,34 @@
 Applications submitted via online portal (link shared on the Medium-Size Grants webpage from Oct 12)</t>
         </is>
       </c>
-      <c r="D25" s="1" t="inlineStr">
+      <c r="D27" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E25" s="1" t="inlineStr">
+      <c r="E27" s="1" t="inlineStr">
         <is>
           <t>Nov 16, 2026</t>
         </is>
       </c>
-      <c r="F25" s="1" t="inlineStr">
+      <c r="F27" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-medium-size-grants-call-for-proposals-global-eba-fund-global-eba-fund-opg-26-00178</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="95" customHeight="1">
-      <c r="A26" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B26" s="1" t="inlineStr">
+    <row r="28" ht="95" customHeight="1">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIEIF Grant 2026 Climate Intervention Environmental Impact Fund</t>
         </is>
       </c>
-      <c r="C26" s="1" t="inlineStr">
+      <c r="C28" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Climate Intervention Environmental Impact Fund (CIEIF) is a philanthropic fund focused on supporting responsible climate intervention field tests. It provides grants for activities such as environmental impact assessment (EIA), predictive impact modelling, and engagement with potentially affected stakeholders, including local communities and government agencies.
@@ -2034,34 +2128,34 @@
 Potential for scaling the innovation to a globally relevant level</t>
         </is>
       </c>
-      <c r="D26" s="1" t="inlineStr">
+      <c r="D28" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E26" s="1" t="inlineStr">
+      <c r="E28" s="1" t="inlineStr">
         <is>
           <t>Dec 1, 2026</t>
         </is>
       </c>
-      <c r="F26" s="1" t="inlineStr">
+      <c r="F28" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cieif-grant-2026-climate-intervention-environmental-impact-fund-climate-intervention-environmental-impact-fund-opg-26-00155</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="95" customHeight="1">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B27" s="1" t="inlineStr">
+    <row r="29" ht="95" customHeight="1">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 6th Annual Seeding The Future Global Food System Challenge</t>
         </is>
       </c>
-      <c r="C27" s="1" t="inlineStr">
+      <c r="C29" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are one of the largest and most respected private organisations for development cooperation and humanitarian aid in Germany. As a politically and confessionally independent organisation, our value-oriented actions are always based on ethical principles. Our vision is clear: "Zero Hunger by 2030"
@@ -2093,34 +2187,34 @@
 Individuals with no organizational entity</t>
         </is>
       </c>
-      <c r="D27" s="1" t="inlineStr">
+      <c r="D29" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E27" s="1" t="inlineStr">
+      <c r="E29" s="1" t="inlineStr">
         <is>
           <t>Jan 1, 2027</t>
         </is>
       </c>
-      <c r="F27" s="1" t="inlineStr">
+      <c r="F29" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-6th-annual-seeding-the-future-global-food-system-challenge-welthungerhilfe-opg-26-00180</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="95" customHeight="1">
-      <c r="A28" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B28" s="1" t="inlineStr">
+    <row r="30" ht="95" customHeight="1">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for BES Training and Travel Grants</t>
         </is>
       </c>
-      <c r="C28" s="1" t="inlineStr">
+      <c r="C30" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are a global community of scientists shining a spotlight on the intricacy and value of our natural world, providing the evidence for better decisions. Our vision is for people and nature to thrive in a world that values ecology.
@@ -2159,17 +2253,17 @@
  Application Deadline (Round 2): Opens 30 April 2026, closes 17 May 2026</t>
         </is>
       </c>
-      <c r="D28" s="1" t="inlineStr">
+      <c r="D30" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E28" s="1" t="inlineStr">
+      <c r="E30" s="1" t="inlineStr">
         <is>
           <t>May 17, 2027</t>
         </is>
       </c>
-      <c r="F28" s="1" t="inlineStr">
+      <c r="F30" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-bes-training-and-travel-grants-british-ecological-society-opg-26-00181</t>
         </is>

</xml_diff>

<commit_message>
Auto update Combined.xlsx [Wed Sep 23 07:12:30 UTC 2026]
</commit_message>
<xml_diff>
--- a/output/Combined.xlsx
+++ b/output/Combined.xlsx
@@ -467,71 +467,10 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>RFP for Impact Assessment</t>
+          <t>EOI- Engagement of State-Level Field Facilitation Consultants for Project Learning Study</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
-        <is>
-          <t>Introduction
-Titan Company Limited, a member of the Tata Group, has a long-standing commitment to Corporate Social Responsibility (CSR) in India. The company's CSR initiatives derive its philosophy from the Company’s vision statement: “We create elevating experiences for the people we touch and significantly impact the world we work in”. The initiatives are designed to promote inclusive growth, empower communities, and contribute to the country's socio-economic development. The program includes Titan’s CSR policy is governed by a dedicated CSR Committee that ensures transparency and compliance with regulatory requirements. The program includes Girl Child Education, Skill and Entrepreneurship Development, supporting Indian Heritage Arts and Crafts, Integrated Village Development Programme, Eye Care and Affirmative Action. Titan's CSR policy is governed by a dedicated CSR Committee that ensures transparency and compliance with regulatory requirements.
-Objectives of the Assignment
-The primary purpose of this Impact Assessment is to generate credible, third-party evidence on the relevance, efficiency, effectiveness, impact, and sustainability of interventions for FY 2025-2026. A detailed scope is given below.
-Scope of Work
-Key questions to be answered:
-Relevance and Alignment: The programs are aligned with community needs, national priorities, and Titan’s CSR policy.
-Outcomes and Impact: Direct and indirect outcomes of the interventions and their contribution to long-term change at the individual, household, and community levels.
-Efficiency and Resource Utilization: Cost-effectiveness of the interventions.
-Understand Sustainability and Scalability
-Enable Learning and Improvement
-Eligibility Criteria for DIM and DIA
-Prior experience in conducting similar assessments for Corporates/Foundations/Institutional Grantees on Social Entrepreneurship/Enterprises initiatives, incubation support, startup ecosystem.
-Water &amp; Sustainability: Understanding of water conservation, access, usage, and scalable sustainability solutions.
-Design-Led Innovation: Awareness of how design approaches and creative problem-solving can drive social change.
-Members of Evaluation Team should have:
-Master's degree in any relevant discipline (Tech Innovation/Social Entrepreneurship) Excellent analytical skills.
-At least 5 years of relevant working experience in research, monitoring and evaluation, and assessments. Excellent communication and drafting skills for effective reporting.
-Team members should have relevant experience working on water conservation initiatives, tech driven community development program.
-Eligibility Criteria for Tarasha
-The agency should have prior experience of atleast 3-4 years in conducting similar assessments for Corporates/Foundations/Institutional Grantees on Artisan livelihoods, Handicrafts and creative enterprises, Entrepreneurship development programs, Livelihood and value-chain development projects.
-Members of Evaluation Team should have:
-Master's degree in any relevant discipline (MSW/Population Studies/Statistics/Sociology)
-Strong expertise in qualitative and quantitative research methods, survey design, sampling, data analysis, and impact measurement.
-Excellent communication, stakeholder engagement, and report-writing skills.
-Experience working across multiple states and engaging with diverse artisan communities.
-At least 5 years of relevant working experience in research, monitoring and evaluation, assessments.
-Excellent communication and drafting skills for effective reporting.
-Team members should have relevant experience working on Artisan livelihoods, Handicrafts and creative enterprises, Entrepreneurship development programs, Livelihood and value-chain development projects.
-Timeline: Proposal submission deadline: September 24, 2026</t>
-        </is>
-      </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>Sep 24, 2026</t>
-        </is>
-      </c>
-      <c r="F2" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/rfp-for-impact-assessment-titan-rfp-26-00354</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="95" customHeight="1">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>EOI- Engagement of State-Level Field Facilitation Consultants for Project Learning Study</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Expression of Interest (EOI)
 For
@@ -592,34 +531,34 @@
 This stage is for collecting information from interested Consultant. AIFT will review the submissions and may issue a detailed Request for Quotation (RFQ) to shortlisted consultant based on the specific assignments.</t>
         </is>
       </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>Sep 25, 2026</t>
         </is>
       </c>
-      <c r="F3" s="1" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/eoi-engagement-of-state-level-field-facilitation-consultants-for-project-learning-study-american-india-foundation-rfp-26-00367</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="95" customHeight="1">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
+    <row r="3" ht="95" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>ToR - Engagement of Information Design &amp; Video Production Agency / Consultant for Key Learning &amp; Dissemination Outputs</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Terms of Reference (TOR) for Consultancy Services
 Title  Engagement of Information Design &amp; Video Production Agency / Consultant for Key Learning &amp; Dissemination Outputs
@@ -638,34 +577,34 @@
 The primary objective of this engagement is to enable SELCO Foundation to effectively capture, structure, and communicate its field insights, sectoral learnings, and program impacts. The selected Agency/Consultant (or Agencies/Consultants) will work on a monthly retainer basis to translate raw content, data, field footage, and reports provided by SELCO into high-quality, visually compelling, reader-friendly visual outputs and video assets.</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Sep 28, 2026</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-engagement-of-information-design-and-video-production-agency-consultant-for-key-learning-and-dissemination-outputs-selco-foundation-rfp-26-00362</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="95" customHeight="1">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
+    <row r="4" ht="95" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>ToR - Video documentation of change stories on Ground water replenishment in Hyderabad and Sanga Reddy locations</t>
         </is>
       </c>
-      <c r="C5" s="1" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>About Jal Seva Charitable Foundation/ WaterAid India:
 Jal Seva Charitable Foundation (JSCF) is registered in India as a not-for-profit company under Chapter 8 of the Companies Act, 2013. JSCF, is an associate member of WaterAid International and uses the brand name ‘WaterAid’ in India.
@@ -699,34 +638,34 @@
 Upon completion of Assignment</t>
         </is>
       </c>
-      <c r="D5" s="1" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E5" s="1" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>Sep 28, 2026</t>
         </is>
       </c>
-      <c r="F5" s="1" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-video-documentation-of-change-stories-on-ground-water-replenishment-in-hyderabad-and-sanga-reddy-locations-wateraid-india-rfp-26-00363</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="95" customHeight="1">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
+    <row r="5" ht="95" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>ToR - Video Production Storytelling and Documentation</t>
         </is>
       </c>
-      <c r="C6" s="1" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>Title Video Production – Storytelling and Documentation
 Timeline 3 months from the date of contracting
@@ -760,34 +699,34 @@
 Quotation Should include all cost including Travel and Miscellaneous.</t>
         </is>
       </c>
-      <c r="D6" s="1" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E6" s="1" t="inlineStr">
+      <c r="E5" s="1" t="inlineStr">
         <is>
           <t>Sep 29, 2026</t>
         </is>
       </c>
-      <c r="F6" s="1" t="inlineStr">
+      <c r="F5" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-video-production-storytelling-and-documentation-selco-foundation-rfp-26-00368</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="95" customHeight="1">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
+    <row r="6" ht="95" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>EOI Inviting Expression of Interest-cum-Proposal for Setting Up District De-Addiction Centres under NAPDDR</t>
         </is>
       </c>
-      <c r="C7" s="1" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>About us
 In the year 1985-86, the erstwhile Ministry of Welfare was bifurcated into the Department of Women and Child Development and the Department of Welfare. Simultaneously, the Scheduled Castes Development Division, Tribal Development Division and the Minorities and Backward Classes Welfare Division were moved from the Ministry of Home Affairs and also the Wakf Division from the Ministry of Law to form the then Ministry of Welfare Subsequently, the name of the Ministry was changed to the Ministry of Social Justice &amp; Empowerment in May, 1998. Further, in October, 1999, the Tribal Development Division had moved out to form a separate Ministry of Tribal Affairs. In January, 2007, the Minorities Division along with Wakf Unit have been moved out of the Ministry and formed as a separate Ministry and the Child Development Division has gone to the Ministry of Women &amp; Child Development.
@@ -827,34 +766,34 @@
 11. Department of Social Justice and Empowerment (DoSJE) reserves the right to cancel this notice, andior invite afresh proposals with or without amendments to this document without liability or any obligation for such document, and without assigning any reason. DoSJE reserves the right to take final decision regarding selection of implementing agency or project.</t>
         </is>
       </c>
-      <c r="D7" s="1" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E7" s="1" t="inlineStr">
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F7" s="1" t="inlineStr">
+      <c r="F6" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/eoi-inviting-expression-of-interest-cum-proposal-for-setting-up-district-de-addiction-centres-under-napddr-ministry-of-social-justice-and-empowerment-goi-rfp-26-00356</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="95" customHeight="1">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
+    <row r="7" ht="95" customHeight="1">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>Application Invited for Giving Joy Microgrant</t>
         </is>
       </c>
-      <c r="C8" s="1" t="inlineStr">
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Giving Joy is a US-based nonprofit that strengthens and inspires women’s entrepreneurship worldwide. Through its micro-grants and mentorship program, Giving Joy helps women establish or improve their businesses and initiatives—for their benefit and the benefit of their communities. To date, Giving Joy has awarded over 88 grants to women-led initiatives in 26 countries.
@@ -893,34 +832,34 @@
 The grant period is six months.</t>
         </is>
       </c>
-      <c r="D8" s="1" t="inlineStr">
+      <c r="D7" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E8" s="1" t="inlineStr">
+      <c r="E7" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F8" s="1" t="inlineStr">
+      <c r="F7" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/application-invited-for-giving-joy-microgrant-giving-joy-opg-26-00185</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="95" customHeight="1">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="inlineStr">
+    <row r="8" ht="95" customHeight="1">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>ToR - Branding Development &amp; Design/Market Promotion Consultant Project Sashakt</t>
         </is>
       </c>
-      <c r="C9" s="1" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>Organisation Humana People to People India (HPPI)
 Project Sashakt – Strengthening Women-led Handloom Cooperatives in Assam (EU-funded)
@@ -975,34 +914,34 @@
 The consultant/agency must ensure ethical, consent-based data collection with cultural sensitivity, particularly when engaging women weavers. All data and reports remain the property of HPPI and must be kept strictly confidential, with no external use.</t>
         </is>
       </c>
-      <c r="D9" s="1" t="inlineStr">
+      <c r="D8" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E9" s="1" t="inlineStr">
+      <c r="E8" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F9" s="1" t="inlineStr">
+      <c r="F8" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-branding-development-and-designmarket-promotion-consultant-project-sashakt-humana-people-to-people-india-rfp-26-00365</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="95" customHeight="1">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
+    <row r="9" ht="95" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Signals of Change Shaping the Future of Sexual and Reproductive Health and Rights SRHR</t>
         </is>
       </c>
-      <c r="C10" s="1" t="inlineStr">
+      <c r="C9" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The World Health Organization's mission: to promote health, keep the world safe, and serve the vulnerable. Working through offices in more than 150 countries, WHO staff work side by side with governments and other partners to ensure the highest attainable level of health for all people.
@@ -1027,34 +966,34 @@
  Submission Requirements: Descriptive information (name, contact email, country, sector) required alongside each submission; formal published evidence is helpful but not required — practice-based experience and field examples are also welcome. Submissions are kept confidential and anonymized before analysis.</t>
         </is>
       </c>
-      <c r="D10" s="1" t="inlineStr">
+      <c r="D9" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E10" s="1" t="inlineStr">
+      <c r="E9" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F10" s="1" t="inlineStr">
+      <c r="F9" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-signals-of-change-shaping-the-future-of-sexual-and-reproductive-health-and-rights-srhr-world-health-organization-opg-26-00176</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="95" customHeight="1">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="inlineStr">
+    <row r="10" ht="95" customHeight="1">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Setting up Viral Research and Diagnosis Laboratories VRDL in Medical Colleges/Hospitals/Medical Institutions</t>
         </is>
       </c>
-      <c r="C11" s="1" t="inlineStr">
+      <c r="C10" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The President notified the creation of the Department of Health Research under the Ministry of Health &amp; Family Welfare through an amendment to the Government of India (Allocation of Business) Rules, 1961 on the 17th September 2007. The Department of Health Research was formally launched on 5th October 2007 by the Minister for Science &amp; Technology and Earth Sciences in a function presided over by the Minister for Health &amp; Family Welfare, in the presence, inter-alia, of the Minister of State for Health &amp; Family Welfare.
@@ -1091,34 +1030,34 @@
 Private medical colleges: only top-50 NIRF-ranked institutions considered</t>
         </is>
       </c>
-      <c r="D11" s="1" t="inlineStr">
+      <c r="D10" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E11" s="1" t="inlineStr">
+      <c r="E10" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F11" s="1" t="inlineStr">
+      <c r="F10" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-setting-up-viral-research-and-diagnosis-laboratories-vrdl-in-medical-collegeshospitalsmedical-institutions-department-of-health-research-dhr-ministry-of-health-and-family-welfare-government-of-india-opg-26-00174</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="95" customHeight="1">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="inlineStr">
+    <row r="11" ht="95" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>RFP - Design and Delivery of an Electric Vehicle EV Skilling Programme in Karnataka</t>
         </is>
       </c>
-      <c r="C12" s="1" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 WRI India, an independent knowledge organisation registered as the India Resources Trust, provides objective information and practical proposals to foster environmentally sound and socially equitable development. As an independent knowledge organisation, we leverage our data and expertise to catalyze change across systems like food, land and water; energy; and cities. Our work focuses on improving people’s lives, protecting and restoring nature, and addressing climate change. To enable progress at the pace and scale needed, we also engage with the economic, finance and governance systems that are key to enabling this change.
@@ -1159,34 +1098,34 @@
 Must have a team of qualified trainers and master trainers with relevant domain expertise, as well as administrative and coordination support.</t>
         </is>
       </c>
-      <c r="D12" s="1" t="inlineStr">
+      <c r="D11" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E12" s="1" t="inlineStr">
+      <c r="E11" s="1" t="inlineStr">
         <is>
           <t>Oct 5, 2026</t>
         </is>
       </c>
-      <c r="F12" s="1" t="inlineStr">
+      <c r="F11" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfp-design-and-delivery-of-an-electric-vehicle-ev-skilling-programme-in-karnataka-wri-india-rfp-26-00361</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="95" customHeight="1">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B13" s="1" t="inlineStr">
+    <row r="12" ht="95" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
         <is>
           <t>RFPs Invited for Engagement of a Manpower Agency for Providing Subject Matter Specialists/Experts for the Cluster Development Programme</t>
         </is>
       </c>
-      <c r="C13" s="1" t="inlineStr">
+      <c r="C12" s="1" t="inlineStr">
         <is>
           <t>About the RFP
 National Horticulture Board (NHB), an autonomous organization under the Ministry of Agriculture and Farmers' Welfare, Government of India, invites bids from eligible manpower agencies for engagement to recruit, deploy, and manage qualified personnel supporting NHB's Cluster Development Programme (CDP) — a Central Sector Scheme promoting integrated, market-led horticulture cluster development. The engaged agency will provide three types of Subject Matter Experts per Cluster and additional consultants/manpower as required by NHB from time to time.
@@ -1212,34 +1151,34 @@
  District: Gurugram, Haryana (NHB Head Office)</t>
         </is>
       </c>
-      <c r="D13" s="1" t="inlineStr">
+      <c r="D12" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E13" s="1" t="inlineStr">
+      <c r="E12" s="1" t="inlineStr">
         <is>
           <t>Oct 6, 2026</t>
         </is>
       </c>
-      <c r="F13" s="1" t="inlineStr">
+      <c r="F12" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfps-invited-for-engagement-of-a-manpower-agency-for-providing-subject-matter-specialistsexperts-for-the-cluster-development-programme-national-horticulture-board-nhb-rfp-26-00370</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="95" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="inlineStr">
+    <row r="13" ht="95" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
         <is>
           <t>Applications Open Draper Richards Kaplan Foundation Funding for Social Enterprises</t>
         </is>
       </c>
-      <c r="C14" s="1" t="inlineStr">
+      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>About us
 Started in 2002, Draper Richards Kaplan Foundation (DRK) is a global venture philanthropy firm supporting early stage, high impact social enterprises. Borrowed from our venture capital legacy, DRK finds, funds, and supports exceptional leaders building innovative solutions to some of the world’s most challenging social and environmental problems. Since beginning this work nearly 25 years ago, DRK has invested in more than 270 organizations that have collectively impacted over 610 million lives to date.
@@ -1263,34 +1202,34 @@
 Please attach a standard resume/CV for the entrepreneur(s) and/or key leadership team members (e.g., CEO, COO, ED, etc.). Applications with text bios for entrepreneurs or members of the leadership team will not be considered.</t>
         </is>
       </c>
-      <c r="D14" s="1" t="inlineStr">
+      <c r="D13" s="1" t="inlineStr">
         <is>
           <t>Climate</t>
         </is>
       </c>
-      <c r="E14" s="1" t="inlineStr">
+      <c r="E13" s="1" t="inlineStr">
         <is>
           <t>Oct 10, 2026</t>
         </is>
       </c>
-      <c r="F14" s="1" t="inlineStr">
+      <c r="F13" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-open-draper-richards-kaplan-foundation-funding-for-social-enterprises-draper-richards-kaplan-foundation-opg-26-00188</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="95" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="inlineStr">
+    <row r="14" ht="95" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund</t>
         </is>
       </c>
-      <c r="C15" s="1" t="inlineStr">
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund
 Apply by: 13 October, 2026
@@ -1315,34 +1254,34 @@
  Projects should include opportunities for ServiceNow employees to volunteer in the project activation or implementation.</t>
         </is>
       </c>
-      <c r="D15" s="1" t="inlineStr">
+      <c r="D14" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E15" s="1" t="inlineStr">
+      <c r="E14" s="1" t="inlineStr">
         <is>
           <t>Oct 13, 2026</t>
         </is>
       </c>
-      <c r="F15" s="1" t="inlineStr">
+      <c r="F14" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/apply-for-the-servicenow-community-solar-fund-changex-opg-26-00186</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="95" customHeight="1">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B16" s="1" t="inlineStr">
+    <row r="15" ht="95" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>ToR - Engagement of Consultant/Vendor Individual towards implementation of Literacy Program in Telangana State</t>
         </is>
       </c>
-      <c r="C16" s="1" t="inlineStr">
+      <c r="C15" s="1" t="inlineStr">
         <is>
           <t>ANNEX A – TERMS OF REFERENCE (ToR) 
  Engagement of Consultant/Vendor (Individual) towards implementation of Literacy Program in Telangana State.
@@ -1407,6 +1346,55 @@
 Approved travel and accommodation expenses incurred for assignment-related activities shall be reimbursed by Room to Read in accordance with the consultancy reimbursement guidelines.</t>
         </is>
       </c>
+      <c r="D15" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E15" s="1" t="inlineStr">
+        <is>
+          <t>Oct 16, 2026</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/tor-engagement-of-consultantvendor-individual-towards-implementation-of-literacy-program-in-telangana-state-room-to-read-india-rfp-26-00360</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="95" customHeight="1">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>RFPs Invited for Empanelment of Publishers for Procurement of E-Books for Rashtriya e-Pustakalaya National Book Trust India</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t>About the RFP:
+Rashtriya e-Pustakalaya, a free National Digital Library for children and adolescents — an initiative of the Department of School Education &amp; Literacy, Ministry of Education, Government of India, implemented by the National Book Trust (NBT), India — invites Expression of Interest (EoI) for the empanelment of publishers for the selection and procurement of e-books, with the objective of enriching the platform's book collection. NBT is an autonomous body under the Ministry of Education, established in 1957 to promote literacy and reading culture in India.
+ Scope of Work:
+Provide acceptable, age-appropriate e-books for ages 8–11, 11–14, and 14+ (Young Adults) across genres like Classics, Mystery, Thriller, Historical, Fiction, Science &amp; Technology, Sports &amp; Fitness, Adventure, etc., with special emphasis on promoting the Indian Knowledge System, history, traditions, and achievements of India
+Provide e-books in specified formats (ePUB / searchable PDF) accessible on the Rashtriya e-Pustakalaya app
+Ensure all necessary consents/approvals from authors, illustrators, artists, translators, or legal owners as per the Copyright Act, 1957 and Copyright Rules, 2013
+Ensure necessary licensing agreements and adherence to copyright laws for uninterrupted hosting
+Ensure content relevance to specific age groups and target audience
+Provide content with valid ISBN/RNI registration only
+Provide metadata of e-books in the specified format with periodic updates
+ Eligibility (for Publishers):
+Must be a registered legal entity: Company (Companies Act, 2013) / LLP (LLP Act, 2008) / Trust (Indian Trusts Act, 1882) / Society (Societies Registration Act, 1860) / Partnership firm (Indian Partnership Act, 1932) / Proprietorship firm (registered under Shops &amp; Establishment Act/Labour Department/GST/other statutory department)
+Must hold valid ISBN/RNI registration
+Must have GST Registration (if applicable), PAN, and Aadhar Card (if applicable)
+Must not be blacklisted by the Government of India, any State/UT Government, or their agencies for corrupt/fraudulent/unfair trade practices, or for backing out of a contract after award
+Publisher, directors, and officers must not have been convicted of any criminal offence related to their professional conduct or false statements/misrepresentation in the last 3 years, or otherwise debarred
+No conflict of interest in the empanelment process
+Must indemnify Rashtriya e-Pustakalaya/NBT-India for any IP-related claims from authors/illustrators/translators/legal owners</t>
+        </is>
+      </c>
       <c r="D16" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
@@ -1419,7 +1407,7 @@
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/rfps/tor-engagement-of-consultantvendor-individual-towards-implementation-of-literacy-program-in-telangana-state-room-to-read-india-rfp-26-00360</t>
+          <t>https://onepurpos.in/openings/rfps/rfps-invited-for-empanelment-of-publishers-for-procurement-of-e-books-for-rashtriya-e-pustakalaya-national-book-trust-india-national-book-trust-nbt-india-rfp-26-00371</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update Combined.xlsx [Thu Sep 24 07:06:21 UTC 2026]
</commit_message>
<xml_diff>
--- a/output/Combined.xlsx
+++ b/output/Combined.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -467,98 +467,10 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>EOI- Engagement of State-Level Field Facilitation Consultants for Project Learning Study</t>
+          <t>ToR - Engagement of Information Design &amp; Video Production Agency / Consultant for Key Learning &amp; Dissemination Outputs</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
-        <is>
-          <t>Expression of Interest (EOI)
-For
-Engagement of State-Level Field Facilitation Consultants for Project Learning Study
-Publication Date: 18th September 2026 
- 1. Assignment Objective
-The State-Level Field Facilitation Consultant will provide on-ground coordination and facilitation support to the central study agency and the organisation’s project team. The consultant will not independently conduct the research, evaluation, or learning study. Their primary responsibility will be to enable timely, smooth, ethical, and well-coordinated access to relevant stakeholders and field locations for the agency’s study activities. 
- 2. Background
-American India Foundation Trust implemented EY Skill Bridge Project across six states (Haryana, Maharashtra, Karnataka, Telangana, Tamilnadu and Odisha) for approximately four years. Although implementation has concluded, a cross-state learning study will now be undertaken to document the project journey, assess broader outcomes, identify what worked well and what did not, and generate learning for future programming.
- A central agency/knowledge partner will be engaged to conduct the study, including research, stakeholder consultations, field documentation, analysis, and preparation of the final learning document. Since the agency may not have established access or operational visibility at school and government levels in every state, one field facilitation consultant will be engaged in each of the six project states. Stakeholder consultation across schools, teachers, students, head teachers, and government officials is a core element of the project evaluation and learning exercises. 
- 3. Scope of Work
-The consultant will undertake the following activities within the assigned state:
-Coordinate with AIFT’s agencies, obtain necessary background information on project locations, participating schools, key stakeholders, and available records.  
-Prepare and update field engagement plan in discussion with the agencies, including proposed school visits, stakeholder consultations, travel schedules, contact details, and required permissions. 
-Establish communication and coordinate with head teachers/principals, teachers, school management representatives, students where appropriate, and other relevant school-level stakeholders. 
-Facilitate access to identified project schools and support scheduling of visits by the central study agency. 
-Liaise with relevant government officials at district, block, cluster, or state level, as applicable, to seek appointments and enable consultations. 
-Support the central agency in organising stakeholder interviews, focus-group discussions, meetings, and field interactions according to the agency’s research plan and tools. 
-Ensure that stakeholders receive timely information about the purpose, date, time, venue, and expected duration of consultations. 
-Assist schools and local stakeholders in arranging an appropriate space and suitable time for interviews or group discussions, while ensuring minimal disruption to academic activities. 
-Support the agency in obtaining relevant non-confidential project-related records, information, or documentation available with schools and local stakeholders, subject to organisational approvals and applicable data-protection requirements. 
-Accompany or support the agency during field visits whenever required, including logistical coordination and local issue resolution. 
-Track completion of planned consultations and promptly flag delays, access constraints, cancellations, or stakeholder availability issues to the organisation and agency. 
-Maintain a concise field-visit tracker containing dates, locations, stakeholders contacted, consultations facilitated, pending actions, and key operational observations. 
-Submit brief periodic updates and a final state-level completion note to the designated project focal point. 
-This role is aligned with common education-sector consultancy practice, where field facilitators liaise with school leaders and government stakeholders, organise consultations and field visits, and document stakeholder inputs for the lead research or technical team. 
- 4. Key Deliverables
-Each consultant will submit:
-State-level stakeholder mapping and proposed field-engagement schedule within the first week of engagement. 
-School-visit and consultation tracker, updated fortnightly. 
-Records of appointments, meetings, consultations, and field coordination completed. 
-Weekly or fortnightly progress update highlighting completed activities, upcoming engagements, challenges, and support required. 
-A final state-level completion note summarising: 
-Schools and stakeholders supported 
-Consultations facilitated 
-Key coordination challenges and resolutions 
-Pending follow-up actions, if any 
-Practical field observations relevant to the study process 
- 5. Duration and Engagement Terms
-Number of consultants: Six consultants, one for each project state (Haryana, Maharashtra, Karnataka, Telangana, Tamil Nadu and Odisha) 
-Duration: Two months from the date of onboarding or issuance of the agreement. 
-Nature of engagement: Short-term consultancy assignment. 
-Assignment location: Respective assigned state, with travel to identified schools and government offices as required. 
-Professional fee: To be paid in INR for complete two-month assignment (Milestone), subject to satisfactory completion of agreed deliverables and compliance with organisational requirements. 
-Reporting: The consultant will report to the designated organisation focal point and work in close coordination with the centrally appointed learning-study agency. 
-6. Roles and Boundaries
-The consultant’s role is facilitative and coordination-focused. The central agency will retain responsibility for research design, tools, data collection methodology, analysis, interpretation of findings, and preparation of the final learning document. The consultant must not make commitments on behalf of the organisation, independently collect sensitive data outside the agreed process, or share stakeholder information without authorisation. 
-7. Required Competencies
-The consultant should have:
-Experience working with schools, education programmes, government systems, NGOs, CSR projects, or community-based initiatives. 
-Strong local knowledge and working relationships with school and government stakeholders in the assigned state. 
-Demonstrated ability to coordinate field visits, meetings, consultations, and logistics. 
-Good written and verbal communication skills in English and relevant local language(s). 
-Ability to travel independently within the assigned geography. 
-Professional conduct, confidentiality, responsiveness, and timely reporting discipline.  
-A strong consultant profile for this assignment combines field coordination, government liaison, stakeholder management, documentation, and support to third-party evaluation activities. 
-Scope of Information Requested
-This stage is for collecting information from interested Consultant. AIFT will review the submissions and may issue a detailed Request for Quotation (RFQ) to shortlisted consultant based on the specific assignments.</t>
-        </is>
-      </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>Sep 25, 2026</t>
-        </is>
-      </c>
-      <c r="F2" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/eoi-engagement-of-state-level-field-facilitation-consultants-for-project-learning-study-american-india-foundation-rfp-26-00367</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="95" customHeight="1">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>ToR - Engagement of Information Design &amp; Video Production Agency / Consultant for Key Learning &amp; Dissemination Outputs</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Terms of Reference (TOR) for Consultancy Services
 Title  Engagement of Information Design &amp; Video Production Agency / Consultant for Key Learning &amp; Dissemination Outputs
@@ -577,34 +489,34 @@
 The primary objective of this engagement is to enable SELCO Foundation to effectively capture, structure, and communicate its field insights, sectoral learnings, and program impacts. The selected Agency/Consultant (or Agencies/Consultants) will work on a monthly retainer basis to translate raw content, data, field footage, and reports provided by SELCO into high-quality, visually compelling, reader-friendly visual outputs and video assets.</t>
         </is>
       </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>Sep 28, 2026</t>
         </is>
       </c>
-      <c r="F3" s="1" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-engagement-of-information-design-and-video-production-agency-consultant-for-key-learning-and-dissemination-outputs-selco-foundation-rfp-26-00362</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="95" customHeight="1">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
+    <row r="3" ht="95" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>ToR - Video documentation of change stories on Ground water replenishment in Hyderabad and Sanga Reddy locations</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>About Jal Seva Charitable Foundation/ WaterAid India:
 Jal Seva Charitable Foundation (JSCF) is registered in India as a not-for-profit company under Chapter 8 of the Companies Act, 2013. JSCF, is an associate member of WaterAid International and uses the brand name ‘WaterAid’ in India.
@@ -638,19 +550,113 @@
 Upon completion of Assignment</t>
         </is>
       </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Sep 28, 2026</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/tor-video-documentation-of-change-stories-on-ground-water-replenishment-in-hyderabad-and-sanga-reddy-locations-wateraid-india-rfp-26-00363</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="95" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>RFP - Engagement of Agency for Development of MIS Dashboard and Mobile-based Application for Adolescent Mental Health</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Release of Request for Proposal
+23rd September 2026
+Pre-bid Meeting (Online) Date
+25th September 2026 
+Pre-Bid Link for Registration: 
+ Pre-Bid Meeting date and time
+25.9.26 @ 5:30 PM
+https://forms.gle/DiwgwoKZzwzYHAsL7
+ Pre-bid Meeting Link
+meet.google.com/dgb-mjez-wam
+  Bid Submission Closing Date
+29th September 2026 (23:59 Hrs. IST)
+Please submit proposals
+ in the following respective Google Forms -
+Technical: https://forms.gle/96REn8vzjEJ7uEPp6
+Financial: https://forms.gle/Hz7pLBp7iS86Eovu9
+Technical Bid Opening
+30th September 2026
+Financial Bid Opening
+  Finalization of Contract
+TBD
+(to be intimated to the awardee only)
+Scope of Work:
+Terms of Reference for Development of MIS Dashboard and Android-based Mobile Application for Adolescent Mental Health Programme in Madhya Pradesh
+ For the Adolescent Mental Health and Well-being Programme, AIFT requires the development of a new Android-based mobile application and a web-based Management Information System (MIS) dashboard. The mobile application will enable adolescents to access age-appropriate learning modules, undertake mental health screening, and connect with mental health support services, wherever required. The MIS dashboard will support programme implementation by enabling counsellors and project staff to record programme activities, monitor school-based interventions, and generate implementation reports.
+ THE AMERICAN INDIA FOUNDATION TRUST (AIFT) intends to engage an agency to design, develop, test and deploy the mobile application and the MIS dashboard as per the requirements shared by AIFT. As this is a time-sensitive requirement, preference will be given to agencies that already have a working application and dashboard of this kind, which can be customized and deployed quickly. The scope of work will include requirement assessment and design, end-to-end development of the application and dashboard, testing and piloting, deployment and handover, training of users, and, after go-live, maintenance, technical support, data support and documentation to facilitate effective implementation and scale-up of the intervention.
+ The selected agency shall design, develop and deploy the mobile application and MIS dashboard, and thereafter provide maintenance, technical and operational support till 30th September 2029, subject to fulfilment of the conditions of the bid and the funding for the programme.
+ Proposal Requirement:
+The technical proposal should cover at least below areas:
+ Applicant eligibility requirement(s):
+The bidder organization should be registered as a legal entity for doing business in India.
+The applicant must have demonstrated ability to provide expert advice and should have at least 3 years of experience in custom software development, or relevant experience in developing a similar mental health application.
+The bidder must have demonstrated experience in designing, developing and deploying mobile applications in the field of adolescent mental health, with at least one similar application developed and implemented within the last three years.
+Preference will be given to bidders who already have a working adolescent mental health mobile application and MIS dashboard that can be customized and deployed for AIFT within a short time, as this is a time-sensitive requirement.
+The bidder should have experience in designing and developing web-based Management Information System (MIS) dashboards for programme monitoring, reporting and data management, preferably for health or social sector programmes.
+The mobile application to be developed must support multilingual functionality (at minimum Hindi and English), and the bidder should have prior experience in developing multilingual mobile applications.
+The bidder should have proven experience across the full development cycle (requirement analysis, UI/UX design, development, testing and deployment), as well as post-deployment maintenance and technical support for mobile applications and dashboards.
+Preference will be given to agencies with prior experience of working with Government departments, development partners, NGOs, or international organizations in implementing digital health or mental health programmes.
+ Technical Requirements:
+The bidder should provide information in English language on overall qualifications, including:
+Profile of organization
+Past experience, clients handled and completed assignments.
+Services and support available post-delivery of Services
+Technical Proposal covering the proposed approach, technical architecture, technology stack and time required to go-live (maximum limit of 10-12 pages)
+Details of the bidder’s existing adolescent mental health mobile application and MIS dashboard (key features, screenshots, demo link/credentials and current deployments), along with confirmation of availability for a live demonstration
+At least two references of clients (contact email id/ phone)
+Views on the RFP requirements – Agreement and suggestions to the scope of work outlined in Section III (not more than 5 pages)
+Profile of team members proposed for the project (not more than 2 pages)
+Any other relevant information (not more than 1 page)
+Only for-profit entities can apply. Nonprofit entities (NGO) are not eligible to apply under this bid.
+ Attachments/ Enclosures for Technical Bid:
+Bid must be submitted in English language only and should contain:
+Covering letter with reference to all enclosures or attachments.
+Copy of registration documents/ certificate and most recent renewal as a legal entity.
+License or permission if any for doing business with computers.
+Copy of PAN &amp; TAN.
+Copy of GST Registration.
+Copy of MSME registration certificate (if registered)
+Copies of last three years ITR. (exempted for startup raised within last two year)
+All Bid must contain the complete address of firm, including contact number/ email ID of the person who is authorized to submit the bid under their signatures.
+Technical bid form as per Annexure I
+ Financial Bid
+It is to be submitted separately as per Annexure II. No conditional price is to be quoted.</t>
+        </is>
+      </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>Learning</t>
+          <t>Governance</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>Sep 28, 2026</t>
+          <t>Sep 29, 2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/rfps/tor-video-documentation-of-change-stories-on-ground-water-replenishment-in-hyderabad-and-sanga-reddy-locations-wateraid-india-rfp-26-00363</t>
+          <t>https://onepurpos.in/openings/rfps/rfp-engagement-of-agency-for-development-of-mis-dashboard-and-mobile-based-application-for-adolescent-mental-health-american-india-foundation-rfp-26-00372</t>
         </is>
       </c>
     </row>
@@ -790,51 +796,49 @@
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>Application Invited for Giving Joy Microgrant</t>
+          <t>Applications Invited for Setting up Viral Research and Diagnosis Laboratories VRDL in Medical Colleges/Hospitals/Medical Institutions</t>
         </is>
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
           <t>About the Organization
-Giving Joy is a US-based nonprofit that strengthens and inspires women’s entrepreneurship worldwide. Through its micro-grants and mentorship program, Giving Joy helps women establish or improve their businesses and initiatives—for their benefit and the benefit of their communities. To date, Giving Joy has awarded over 88 grants to women-led initiatives in 26 countries.
- 2026 Grant Cycle
-Beginning in 2026, Giving Joy has moved to two global grant cycles per year.
-The organization states that this change was made after operating multiple regional rounds, with the aim of:
-Providing clearer timelines for applicants
-Increasing the quality and depth of application reviews
-Reducing administrative burden
-Improving support for grantees
-Focusing communications and fundraising more effectively
-Continuing to reach women entrepreneurs globally without dividing applications by geography
-Each cycle is open to women entrepreneurs worldwide.
- Eligible Fields / Activities
-There is no restriction to a particular field such as health.
-Applicants can propose activities in:
-Any field
-Trade
-Occupation
-Craft
- What Does Giving Joy Look For?
-Giving Joy prioritizes:
-Innovative ideas
-Creative ideas
-Strong potential for social impact
-Initiative
-Real community impact
-Clear economic and/or social benefits for women and girls
- Grant Amount
-Maximum Grant
-Up to $500 USD
-The exact award amount is determined by Giving Joy based on:
-Proposed activities
-Availability of funding
- Grant Duration
-The grant period is six months.</t>
+The President notified the creation of the Department of Health Research under the Ministry of Health &amp; Family Welfare through an amendment to the Government of India (Allocation of Business) Rules, 1961 on the 17th September 2007. The Department of Health Research was formally launched on 5th October 2007 by the Minister for Science &amp; Technology and Earth Sciences in a function presided over by the Minister for Health &amp; Family Welfare, in the presence, inter-alia, of the Minister of State for Health &amp; Family Welfare.
+The Department became functional from November 2008 with the appointment of first Secretary of the Department The aim of the DHR is to bring modern health technologies to the people through research and innovations related to diagnosis, treatment methods and vaccines for prevention, to translate them into products and processes and, in synergy with concerned organizations, introduce these innovations into public health system.
+ About the Opportunity:
+Under DHR's scheme "Setting-up of nation-wide network of laboratories for managing epidemics and national calamities," proposals are invited from Medical Colleges/Hospitals/Research Institutions to establish a Medical College &amp; Research Institute Level – Viral Research and Diagnosis Laboratory (MCL-VRDL). The existing network comprises 167 VRDLs (11 Regional, 27 State, 129 Medical College level) across 27 states and 5 UTs, aimed at early detection of infectious pathogens, outbreak surveillance, and research on emerging/re-emerging viral diseases.
+ Objectives:
+Establish capacity for early detection of common and high-risk infectious pathogens
+Strengthen syndromic surveillance ecosystem for outbreak detection
+Undertake R&amp;D on emerging, re-emerging and novel viruses
+ Eligibility (Institution-level):
+State Government Medical Colleges
+Central Government Medical Colleges and Research Institutes
+Armed Forces Medical Institutions/Hospitals
+Railway and other Central Government health institutions
+Private medical colleges ranked in top 50 NIRF ranking
+Must have a dedicated Microbiology department with qualified faculty
+Must have &gt;200 sq.m. area available in existing building (preferably within Microbiology Dept.)
+ Funding Provision:
+Non-recurring assistance: Rs. 1.55 crore total
+Rs. 66.8 lakhs — Civil Work (infrastructure modification)
+Rs. 88.2 lakhs — Equipment (complete lab setup)
+No recurring expenditure (staff salaries, consumables, contingency) is provided — to be borne by the host institution
+ Role &amp; Responsibilities of the Lab:
+Conduct routine diagnosis of infectious pathogens
+Participate in syndromic and event-based surveillance
+Provide support during outbreaks/epidemics
+Share data with ICMR
+ Selection Criteria:
+Meeting eligibility does not guarantee selection; merit-based evaluation by a technical committee
+Preference to institutions in geographically underserved regions
+Weightage for technical strength (qualified faculty, biosafety practices, outbreak investigation experience, publications, patents, externally funded projects)
+Additional weightage for molecular diagnostics, genomic surveillance, One Health research capability, and commitment to long-term recurring support
+Private medical colleges: only top-50 NIRF-ranked institutions considered</t>
         </is>
       </c>
       <c r="D7" s="1" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Governance</t>
         </is>
       </c>
       <c r="E7" s="1" t="inlineStr">
@@ -844,7 +848,7 @@
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/grants/application-invited-for-giving-joy-microgrant-giving-joy-opg-26-00185</t>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-setting-up-viral-research-and-diagnosis-laboratories-vrdl-in-medical-collegeshospitalsmedical-institutions-department-of-health-research-dhr-ministry-of-health-and-family-welfare-government-of-india-opg-26-00174</t>
         </is>
       </c>
     </row>
@@ -856,10 +860,62 @@
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
+          <t>Applications Invited for Signals of Change Shaping the Future of Sexual and Reproductive Health and Rights SRHR</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+The World Health Organization's mission: to promote health, keep the world safe, and serve the vulnerable. Working through offices in more than 150 countries, WHO staff work side by side with governments and other partners to ensure the highest attainable level of health for all people.
+ About the Opportunity
+HRP and its UN co-sponsors are leading a global Sexual and Reproductive Health and Rights (SRHR) foresight and research prioritization process for 2026–2036. This open public consultation invites diverse stakeholder input to identify "signals of change" — emerging trends, shifts, or disruptions — that could shape the future of SRHR over the next decade. The process uses foresight methodology (not prediction) to explore plausible futures and will culminate in a published report and research agenda in 2027.
+ Guiding Questions
+What future trends will shape or constrain SRHR over the next 10 years?
+What evidence and research investments are needed today to prepare SRHR for the futures we may face?
+ Scope of Submissions 
+Economic systems; social infrastructure; structural discrimination; conflict/forced migration/displacement; mega-trends (demographic shifts, climate change, digital transformation/AI, urbanization); conditions of daily life; rights/legal/governance systems; health systems; media/misinformation; and changes in the research ecosystem.
+ Who Can Participate 
+Open to individuals and organizations globally, including:
+Health workers, professional associations, clinical networks
+Civil society, community groups, youth-led organizations, rights movements
+Governments, parliamentarians, regulators, public sector bodies
+Researchers, academia, think tanks, technical experts
+UN agencies, multilateral/humanitarian/development organizations
+Funders, philanthropy, private sector, tech/innovation organizations
+Media, communications, journalism
+Anyone with relevant lived experience or perspective
+Special interest in submissions from health worker, community, youth, and rights-movement spaces not typically represented in published forums.
+ Submission Requirements: Descriptive information (name, contact email, country, sector) required alongside each submission; formal published evidence is helpful but not required — practice-based experience and field examples are also welcome. Submissions are kept confidential and anonymized before analysis.</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Sep 30, 2026</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-signals-of-change-shaping-the-future-of-sexual-and-reproductive-health-and-rights-srhr-world-health-organization-opg-26-00176</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="95" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
           <t>ToR - Branding Development &amp; Design/Market Promotion Consultant Project Sashakt</t>
         </is>
       </c>
-      <c r="C8" s="1" t="inlineStr">
+      <c r="C9" s="1" t="inlineStr">
         <is>
           <t>Organisation Humana People to People India (HPPI)
 Project Sashakt – Strengthening Women-led Handloom Cooperatives in Assam (EU-funded)
@@ -914,71 +970,19 @@
 The consultant/agency must ensure ethical, consent-based data collection with cultural sensitivity, particularly when engaging women weavers. All data and reports remain the property of HPPI and must be kept strictly confidential, with no external use.</t>
         </is>
       </c>
-      <c r="D8" s="1" t="inlineStr">
+      <c r="D9" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E8" s="1" t="inlineStr">
+      <c r="E9" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F8" s="1" t="inlineStr">
+      <c r="F9" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-branding-development-and-designmarket-promotion-consultant-project-sashakt-humana-people-to-people-india-rfp-26-00365</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="95" customHeight="1">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Signals of Change Shaping the Future of Sexual and Reproductive Health and Rights SRHR</t>
-        </is>
-      </c>
-      <c r="C9" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-The World Health Organization's mission: to promote health, keep the world safe, and serve the vulnerable. Working through offices in more than 150 countries, WHO staff work side by side with governments and other partners to ensure the highest attainable level of health for all people.
- About the Opportunity
-HRP and its UN co-sponsors are leading a global Sexual and Reproductive Health and Rights (SRHR) foresight and research prioritization process for 2026–2036. This open public consultation invites diverse stakeholder input to identify "signals of change" — emerging trends, shifts, or disruptions — that could shape the future of SRHR over the next decade. The process uses foresight methodology (not prediction) to explore plausible futures and will culminate in a published report and research agenda in 2027.
- Guiding Questions
-What future trends will shape or constrain SRHR over the next 10 years?
-What evidence and research investments are needed today to prepare SRHR for the futures we may face?
- Scope of Submissions 
-Economic systems; social infrastructure; structural discrimination; conflict/forced migration/displacement; mega-trends (demographic shifts, climate change, digital transformation/AI, urbanization); conditions of daily life; rights/legal/governance systems; health systems; media/misinformation; and changes in the research ecosystem.
- Who Can Participate 
-Open to individuals and organizations globally, including:
-Health workers, professional associations, clinical networks
-Civil society, community groups, youth-led organizations, rights movements
-Governments, parliamentarians, regulators, public sector bodies
-Researchers, academia, think tanks, technical experts
-UN agencies, multilateral/humanitarian/development organizations
-Funders, philanthropy, private sector, tech/innovation organizations
-Media, communications, journalism
-Anyone with relevant lived experience or perspective
-Special interest in submissions from health worker, community, youth, and rights-movement spaces not typically represented in published forums.
- Submission Requirements: Descriptive information (name, contact email, country, sector) required alongside each submission; formal published evidence is helpful but not required — practice-based experience and field examples are also welcome. Submissions are kept confidential and anonymized before analysis.</t>
-        </is>
-      </c>
-      <c r="D9" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E9" s="1" t="inlineStr">
-        <is>
-          <t>Sep 30, 2026</t>
-        </is>
-      </c>
-      <c r="F9" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-signals-of-change-shaping-the-future-of-sexual-and-reproductive-health-and-rights-srhr-world-health-organization-opg-26-00176</t>
         </is>
       </c>
     </row>
@@ -990,49 +994,51 @@
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>Applications Invited for Setting up Viral Research and Diagnosis Laboratories VRDL in Medical Colleges/Hospitals/Medical Institutions</t>
+          <t>Application Invited for Giving Joy Microgrant</t>
         </is>
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
           <t>About the Organization
-The President notified the creation of the Department of Health Research under the Ministry of Health &amp; Family Welfare through an amendment to the Government of India (Allocation of Business) Rules, 1961 on the 17th September 2007. The Department of Health Research was formally launched on 5th October 2007 by the Minister for Science &amp; Technology and Earth Sciences in a function presided over by the Minister for Health &amp; Family Welfare, in the presence, inter-alia, of the Minister of State for Health &amp; Family Welfare.
-The Department became functional from November 2008 with the appointment of first Secretary of the Department The aim of the DHR is to bring modern health technologies to the people through research and innovations related to diagnosis, treatment methods and vaccines for prevention, to translate them into products and processes and, in synergy with concerned organizations, introduce these innovations into public health system.
- About the Opportunity:
-Under DHR's scheme "Setting-up of nation-wide network of laboratories for managing epidemics and national calamities," proposals are invited from Medical Colleges/Hospitals/Research Institutions to establish a Medical College &amp; Research Institute Level – Viral Research and Diagnosis Laboratory (MCL-VRDL). The existing network comprises 167 VRDLs (11 Regional, 27 State, 129 Medical College level) across 27 states and 5 UTs, aimed at early detection of infectious pathogens, outbreak surveillance, and research on emerging/re-emerging viral diseases.
- Objectives:
-Establish capacity for early detection of common and high-risk infectious pathogens
-Strengthen syndromic surveillance ecosystem for outbreak detection
-Undertake R&amp;D on emerging, re-emerging and novel viruses
- Eligibility (Institution-level):
-State Government Medical Colleges
-Central Government Medical Colleges and Research Institutes
-Armed Forces Medical Institutions/Hospitals
-Railway and other Central Government health institutions
-Private medical colleges ranked in top 50 NIRF ranking
-Must have a dedicated Microbiology department with qualified faculty
-Must have &gt;200 sq.m. area available in existing building (preferably within Microbiology Dept.)
- Funding Provision:
-Non-recurring assistance: Rs. 1.55 crore total
-Rs. 66.8 lakhs — Civil Work (infrastructure modification)
-Rs. 88.2 lakhs — Equipment (complete lab setup)
-No recurring expenditure (staff salaries, consumables, contingency) is provided — to be borne by the host institution
- Role &amp; Responsibilities of the Lab:
-Conduct routine diagnosis of infectious pathogens
-Participate in syndromic and event-based surveillance
-Provide support during outbreaks/epidemics
-Share data with ICMR
- Selection Criteria:
-Meeting eligibility does not guarantee selection; merit-based evaluation by a technical committee
-Preference to institutions in geographically underserved regions
-Weightage for technical strength (qualified faculty, biosafety practices, outbreak investigation experience, publications, patents, externally funded projects)
-Additional weightage for molecular diagnostics, genomic surveillance, One Health research capability, and commitment to long-term recurring support
-Private medical colleges: only top-50 NIRF-ranked institutions considered</t>
+Giving Joy is a US-based nonprofit that strengthens and inspires women’s entrepreneurship worldwide. Through its micro-grants and mentorship program, Giving Joy helps women establish or improve their businesses and initiatives—for their benefit and the benefit of their communities. To date, Giving Joy has awarded over 88 grants to women-led initiatives in 26 countries.
+ 2026 Grant Cycle
+Beginning in 2026, Giving Joy has moved to two global grant cycles per year.
+The organization states that this change was made after operating multiple regional rounds, with the aim of:
+Providing clearer timelines for applicants
+Increasing the quality and depth of application reviews
+Reducing administrative burden
+Improving support for grantees
+Focusing communications and fundraising more effectively
+Continuing to reach women entrepreneurs globally without dividing applications by geography
+Each cycle is open to women entrepreneurs worldwide.
+ Eligible Fields / Activities
+There is no restriction to a particular field such as health.
+Applicants can propose activities in:
+Any field
+Trade
+Occupation
+Craft
+ What Does Giving Joy Look For?
+Giving Joy prioritizes:
+Innovative ideas
+Creative ideas
+Strong potential for social impact
+Initiative
+Real community impact
+Clear economic and/or social benefits for women and girls
+ Grant Amount
+Maximum Grant
+Up to $500 USD
+The exact award amount is determined by Giving Joy based on:
+Proposed activities
+Availability of funding
+ Grant Duration
+The grant period is six months.</t>
         </is>
       </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>Governance</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="E10" s="1" t="inlineStr">
@@ -1042,7 +1048,7 @@
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-setting-up-viral-research-and-diagnosis-laboratories-vrdl-in-medical-collegeshospitalsmedical-institutions-department-of-health-research-dhr-ministry-of-health-and-family-welfare-government-of-india-opg-26-00174</t>
+          <t>https://onepurpos.in/openings/grants/application-invited-for-giving-joy-microgrant-giving-joy-opg-26-00185</t>
         </is>
       </c>
     </row>
@@ -1122,10 +1128,71 @@
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
+          <t>ToR for Onboarding of consultant/agency for Innovating &amp; Scaling Reproductive Maternal Newborn and Child Health Solutions in the Last-Mile</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>Title Terms of Reference for Onboarding of consultant/agency for Innovating &amp; Scaling Reproductive, Maternal, Newborn and Child Health Solutions in the Last-Mile
+Timeline September 2026 to February 2027
+Scope of Work
+• Outreach and program visibility
+• Application design, launch, review, shortlisting, and due diligence
+• Stakeholder engagement and coordination
+• Knowledge materials and document learnings and insights
+Application Link https://forms.gle/jsngbAREkYmgK7cB6
+Last Date to Apply 5th October, 5 PM
+About SELCO Foundation:
+SELCO Foundation's mission is to create a platform of solutions that uses sustainable energy as a catalyst to bridge environmental sustainability and poverty alleviation. With holistic development as the primary focus, the organization strives to create equitable societies, where services are accessed by all communities. The interventions of SELCO lead to a sustainable delivery model of essential services like livelihoods, education, and health till the last mile.
+(Read more about SELCO here: https://selcofoundation.org/)
+ About the Program
+The program aims to catalyse the development, adoption, and scale of innovative solutions that contribute to improved maternal and child health outcomes. It seeks to build an ecosystem where enterprises and innovators can develop and strengthen technology and technology-allied solutions that enable more accessible, quality, efficient, affordable, and continuous maternal and child health services, particularly across last-mile health facilities and underserved communities.
+The program envisions a future where innovation, technology, and enterprise-led solutions are meaningfully integrated into maternal and child health delivery, enabling health systems, facilities, and frontline health workers to deliver better services to women and children.
+The initiative will bring together enterprises, innovators, health facilities, frontline health workers, institutions, and other ecosystem stakeholders to co-create, test, deploy, and scale solutions with the potential to transform maternal and child health delivery. The focus will be on enabling promising solutions to move beyond individual deployments towards sustainable models of adoption, replication, and scale.
+For the same, we are looking to partner with a like-minded organization that shares this vision and can play an integral role in designing and implementing the initiative. The partner will support enterprise identification and engagement, solution assessment, co-creation, health-system linkages, implementation, stakeholder coordination, evidence generation, and pathways to scale, contributing to more resilient, responsive, and equitable maternal and child health services for women and children.
+ Geography
+Primary Focus: Maharashtra, Karnataka, Odisha, Meghalaya, Mizoram, Nagaland
+Secondary Focus: Other states
+ Selection Criteria
+Applicants should meet the following criteria for being a part of the evaluation:
+Demonstrated experience working with vendors, enterprises, innovators, or solution providers, along with an understanding of grassroots and last-mile contexts and user needs
+Ability to assess enterprise and solution needs and curate tailored mentorship, technical assistance, health-system linkages, and implementation support
+Demonstrated experience in program design, planning, implementation, and management of multi-stakeholder initiatives, preferably in health, maternal and child health, technology, or last-mile service delivery
+Proven ability to manage end-to-end application, assessment, screening, shortlisting, and due diligence processes for a portfolio of enterprises or innovators
+Experience in communication, outreach, stakeholder engagement, and facilitating collaboration between solution providers and health-system stakeholders
+Capability to develop documentation and knowledge products that capture program processes, solution performance, outcomes, implementation models, and learnings for scale and replication
+Prior experience working with development sector organisations, NGOs, health systems, technology providers, enterprises, or think tanks will be considered an added advantage
+The agency will be selected on a combined technical and financial evaluation. Proposals must score a minimum of 70% on the technical components (1–5 below) to be considered for financial evaluation.</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>Oct 5, 2026</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/tor-for-onboarding-of-consultantagency-for-innovating-and-scaling-reproductive-maternal-newborn-and-child-health-solutions-in-the-last-mile-selco-foundation-rfp-26-00373</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="95" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
           <t>RFPs Invited for Engagement of a Manpower Agency for Providing Subject Matter Specialists/Experts for the Cluster Development Programme</t>
         </is>
       </c>
-      <c r="C12" s="1" t="inlineStr">
+      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>About the RFP
 National Horticulture Board (NHB), an autonomous organization under the Ministry of Agriculture and Farmers' Welfare, Government of India, invites bids from eligible manpower agencies for engagement to recruit, deploy, and manage qualified personnel supporting NHB's Cluster Development Programme (CDP) — a Central Sector Scheme promoting integrated, market-led horticulture cluster development. The engaged agency will provide three types of Subject Matter Experts per Cluster and additional consultants/manpower as required by NHB from time to time.
@@ -1151,34 +1218,34 @@
  District: Gurugram, Haryana (NHB Head Office)</t>
         </is>
       </c>
-      <c r="D12" s="1" t="inlineStr">
+      <c r="D13" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E12" s="1" t="inlineStr">
+      <c r="E13" s="1" t="inlineStr">
         <is>
           <t>Oct 6, 2026</t>
         </is>
       </c>
-      <c r="F12" s="1" t="inlineStr">
+      <c r="F13" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfps-invited-for-engagement-of-a-manpower-agency-for-providing-subject-matter-specialistsexperts-for-the-cluster-development-programme-national-horticulture-board-nhb-rfp-26-00370</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="95" customHeight="1">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B13" s="1" t="inlineStr">
+    <row r="14" ht="95" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>Applications Open Draper Richards Kaplan Foundation Funding for Social Enterprises</t>
         </is>
       </c>
-      <c r="C13" s="1" t="inlineStr">
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>About us
 Started in 2002, Draper Richards Kaplan Foundation (DRK) is a global venture philanthropy firm supporting early stage, high impact social enterprises. Borrowed from our venture capital legacy, DRK finds, funds, and supports exceptional leaders building innovative solutions to some of the world’s most challenging social and environmental problems. Since beginning this work nearly 25 years ago, DRK has invested in more than 270 organizations that have collectively impacted over 610 million lives to date.
@@ -1202,34 +1269,34 @@
 Please attach a standard resume/CV for the entrepreneur(s) and/or key leadership team members (e.g., CEO, COO, ED, etc.). Applications with text bios for entrepreneurs or members of the leadership team will not be considered.</t>
         </is>
       </c>
-      <c r="D13" s="1" t="inlineStr">
+      <c r="D14" s="1" t="inlineStr">
         <is>
           <t>Climate</t>
         </is>
       </c>
-      <c r="E13" s="1" t="inlineStr">
+      <c r="E14" s="1" t="inlineStr">
         <is>
           <t>Oct 10, 2026</t>
         </is>
       </c>
-      <c r="F13" s="1" t="inlineStr">
+      <c r="F14" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-open-draper-richards-kaplan-foundation-funding-for-social-enterprises-draper-richards-kaplan-foundation-opg-26-00188</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="95" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="inlineStr">
+    <row r="15" ht="95" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund</t>
         </is>
       </c>
-      <c r="C14" s="1" t="inlineStr">
+      <c r="C15" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund
 Apply by: 13 October, 2026
@@ -1254,34 +1321,83 @@
  Projects should include opportunities for ServiceNow employees to volunteer in the project activation or implementation.</t>
         </is>
       </c>
-      <c r="D14" s="1" t="inlineStr">
+      <c r="D15" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E14" s="1" t="inlineStr">
+      <c r="E15" s="1" t="inlineStr">
         <is>
           <t>Oct 13, 2026</t>
         </is>
       </c>
-      <c r="F14" s="1" t="inlineStr">
+      <c r="F15" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/apply-for-the-servicenow-community-solar-fund-changex-opg-26-00186</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="95" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="inlineStr">
+    <row r="16" ht="95" customHeight="1">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>RFPs Invited for Empanelment of Publishers for Procurement of E-Books for Rashtriya e-Pustakalaya National Book Trust India</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t>About the RFP:
+Rashtriya e-Pustakalaya, a free National Digital Library for children and adolescents — an initiative of the Department of School Education &amp; Literacy, Ministry of Education, Government of India, implemented by the National Book Trust (NBT), India — invites Expression of Interest (EoI) for the empanelment of publishers for the selection and procurement of e-books, with the objective of enriching the platform's book collection. NBT is an autonomous body under the Ministry of Education, established in 1957 to promote literacy and reading culture in India.
+ Scope of Work:
+Provide acceptable, age-appropriate e-books for ages 8–11, 11–14, and 14+ (Young Adults) across genres like Classics, Mystery, Thriller, Historical, Fiction, Science &amp; Technology, Sports &amp; Fitness, Adventure, etc., with special emphasis on promoting the Indian Knowledge System, history, traditions, and achievements of India
+Provide e-books in specified formats (ePUB / searchable PDF) accessible on the Rashtriya e-Pustakalaya app
+Ensure all necessary consents/approvals from authors, illustrators, artists, translators, or legal owners as per the Copyright Act, 1957 and Copyright Rules, 2013
+Ensure necessary licensing agreements and adherence to copyright laws for uninterrupted hosting
+Ensure content relevance to specific age groups and target audience
+Provide content with valid ISBN/RNI registration only
+Provide metadata of e-books in the specified format with periodic updates
+ Eligibility (for Publishers):
+Must be a registered legal entity: Company (Companies Act, 2013) / LLP (LLP Act, 2008) / Trust (Indian Trusts Act, 1882) / Society (Societies Registration Act, 1860) / Partnership firm (Indian Partnership Act, 1932) / Proprietorship firm (registered under Shops &amp; Establishment Act/Labour Department/GST/other statutory department)
+Must hold valid ISBN/RNI registration
+Must have GST Registration (if applicable), PAN, and Aadhar Card (if applicable)
+Must not be blacklisted by the Government of India, any State/UT Government, or their agencies for corrupt/fraudulent/unfair trade practices, or for backing out of a contract after award
+Publisher, directors, and officers must not have been convicted of any criminal offence related to their professional conduct or false statements/misrepresentation in the last 3 years, or otherwise debarred
+No conflict of interest in the empanelment process
+Must indemnify Rashtriya e-Pustakalaya/NBT-India for any IP-related claims from authors/illustrators/translators/legal owners</t>
+        </is>
+      </c>
+      <c r="D16" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E16" s="1" t="inlineStr">
+        <is>
+          <t>Oct 16, 2026</t>
+        </is>
+      </c>
+      <c r="F16" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/rfps-invited-for-empanelment-of-publishers-for-procurement-of-e-books-for-rashtriya-e-pustakalaya-national-book-trust-india-national-book-trust-nbt-india-rfp-26-00371</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="95" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
         <is>
           <t>ToR - Engagement of Consultant/Vendor Individual towards implementation of Literacy Program in Telangana State</t>
         </is>
       </c>
-      <c r="C15" s="1" t="inlineStr">
+      <c r="C17" s="1" t="inlineStr">
         <is>
           <t>ANNEX A – TERMS OF REFERENCE (ToR) 
  Engagement of Consultant/Vendor (Individual) towards implementation of Literacy Program in Telangana State.
@@ -1346,83 +1462,34 @@
 Approved travel and accommodation expenses incurred for assignment-related activities shall be reimbursed by Room to Read in accordance with the consultancy reimbursement guidelines.</t>
         </is>
       </c>
-      <c r="D15" s="1" t="inlineStr">
+      <c r="D17" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E15" s="1" t="inlineStr">
+      <c r="E17" s="1" t="inlineStr">
         <is>
           <t>Oct 16, 2026</t>
         </is>
       </c>
-      <c r="F15" s="1" t="inlineStr">
+      <c r="F17" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-engagement-of-consultantvendor-individual-towards-implementation-of-literacy-program-in-telangana-state-room-to-read-india-rfp-26-00360</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="95" customHeight="1">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B16" s="1" t="inlineStr">
-        <is>
-          <t>RFPs Invited for Empanelment of Publishers for Procurement of E-Books for Rashtriya e-Pustakalaya National Book Trust India</t>
-        </is>
-      </c>
-      <c r="C16" s="1" t="inlineStr">
-        <is>
-          <t>About the RFP:
-Rashtriya e-Pustakalaya, a free National Digital Library for children and adolescents — an initiative of the Department of School Education &amp; Literacy, Ministry of Education, Government of India, implemented by the National Book Trust (NBT), India — invites Expression of Interest (EoI) for the empanelment of publishers for the selection and procurement of e-books, with the objective of enriching the platform's book collection. NBT is an autonomous body under the Ministry of Education, established in 1957 to promote literacy and reading culture in India.
- Scope of Work:
-Provide acceptable, age-appropriate e-books for ages 8–11, 11–14, and 14+ (Young Adults) across genres like Classics, Mystery, Thriller, Historical, Fiction, Science &amp; Technology, Sports &amp; Fitness, Adventure, etc., with special emphasis on promoting the Indian Knowledge System, history, traditions, and achievements of India
-Provide e-books in specified formats (ePUB / searchable PDF) accessible on the Rashtriya e-Pustakalaya app
-Ensure all necessary consents/approvals from authors, illustrators, artists, translators, or legal owners as per the Copyright Act, 1957 and Copyright Rules, 2013
-Ensure necessary licensing agreements and adherence to copyright laws for uninterrupted hosting
-Ensure content relevance to specific age groups and target audience
-Provide content with valid ISBN/RNI registration only
-Provide metadata of e-books in the specified format with periodic updates
- Eligibility (for Publishers):
-Must be a registered legal entity: Company (Companies Act, 2013) / LLP (LLP Act, 2008) / Trust (Indian Trusts Act, 1882) / Society (Societies Registration Act, 1860) / Partnership firm (Indian Partnership Act, 1932) / Proprietorship firm (registered under Shops &amp; Establishment Act/Labour Department/GST/other statutory department)
-Must hold valid ISBN/RNI registration
-Must have GST Registration (if applicable), PAN, and Aadhar Card (if applicable)
-Must not be blacklisted by the Government of India, any State/UT Government, or their agencies for corrupt/fraudulent/unfair trade practices, or for backing out of a contract after award
-Publisher, directors, and officers must not have been convicted of any criminal offence related to their professional conduct or false statements/misrepresentation in the last 3 years, or otherwise debarred
-No conflict of interest in the empanelment process
-Must indemnify Rashtriya e-Pustakalaya/NBT-India for any IP-related claims from authors/illustrators/translators/legal owners</t>
-        </is>
-      </c>
-      <c r="D16" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E16" s="1" t="inlineStr">
-        <is>
-          <t>Oct 16, 2026</t>
-        </is>
-      </c>
-      <c r="F16" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/rfps-invited-for-empanelment-of-publishers-for-procurement-of-e-books-for-rashtriya-e-pustakalaya-national-book-trust-india-national-book-trust-nbt-india-rfp-26-00371</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="95" customHeight="1">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B17" s="1" t="inlineStr">
+    <row r="18" ht="95" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>RFPs Invited for Consultant to Develop a Technical Assistance Package for National Application of the Digital Health and AI Investment Classification Framework</t>
         </is>
       </c>
-      <c r="C17" s="1" t="inlineStr">
+      <c r="C18" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are Transform Health: a global coalition of more than 200 organisations driving the digital transformation of health to achieve universal health coverage. 
@@ -1450,34 +1517,34 @@
 Ability to manage multi-country consultancy engagements and coordinate with in-country focal points</t>
         </is>
       </c>
-      <c r="D17" s="1" t="inlineStr">
+      <c r="D18" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E17" s="1" t="inlineStr">
+      <c r="E18" s="1" t="inlineStr">
         <is>
           <t>Oct 23, 2026</t>
         </is>
       </c>
-      <c r="F17" s="1" t="inlineStr">
+      <c r="F18" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfps-invited-for-consultant-to-develop-a-technical-assistance-package-for-national-application-of-the-digital-health-and-ai-investment-classification-framework-transform-health-rfp-26-00359</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="95" customHeight="1">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="inlineStr">
+    <row r="19" ht="95" customHeight="1">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for D-Prize Global Competition Seed Funding for New Poverty-Solution Distribution Organizations</t>
         </is>
       </c>
-      <c r="C18" s="1" t="inlineStr">
+      <c r="C19" s="1" t="inlineStr">
         <is>
           <t>About the Grant:
 D-Prize seeds new organizations that distribute proven poverty solutions at the "last mile," with the aim of scaling impact. Applicants select from a range of evidence-based interventions (health, agriculture, education, water, safety, transparency, and more) and propose how they would launch or grow an organization to distribute that intervention. Top entrepreneurs receive up to $20,000 in seed funding to run a pilot and build an organization capable of scaling to reach thousands, even millions of people.
@@ -1500,34 +1567,34 @@
 Extension Deadline: 6 December 2026, midnight PT (extension registration required)</t>
         </is>
       </c>
-      <c r="D18" s="1" t="inlineStr">
+      <c r="D19" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E18" s="1" t="inlineStr">
+      <c r="E19" s="1" t="inlineStr">
         <is>
           <t>Oct 25, 2026</t>
         </is>
       </c>
-      <c r="F18" s="1" t="inlineStr">
+      <c r="F19" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-d-prize-global-competition-seed-funding-for-new-poverty-solution-distribution-organizations-d-prize-opg-26-00191</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="95" customHeight="1">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="inlineStr">
+    <row r="20" ht="95" customHeight="1">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 8th Call for Proposals Small-Size Grants Global EbA Fund</t>
         </is>
       </c>
-      <c r="C19" s="1" t="inlineStr">
+      <c r="C20" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -1590,34 +1657,34 @@
 Only successful applicants will be contacted; no individual feedback provided to unsuccessful applicants</t>
         </is>
       </c>
-      <c r="D19" s="1" t="inlineStr">
+      <c r="D20" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E19" s="1" t="inlineStr">
+      <c r="E20" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F19" s="1" t="inlineStr">
+      <c r="F20" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-8th-call-for-proposals-small-size-grants-global-eba-fund-global-eba-fund-opg-26-00177</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="95" customHeight="1">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="inlineStr">
+    <row r="21" ht="95" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Adaptive Control Frameworks to Unlock Full-Scale BNR Potential Water Research Foundation WRF</t>
         </is>
       </c>
-      <c r="C20" s="1" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Water Research Foundation (WRF) is the leading research organization advancing the science of all water to meet the evolving needs of its subscribers and the water sector. WRF is a nonprofit, charitable and educational organization which funds, manages, and publishes research on the technology, operation, and management of drinking water, wastewater, reuse, and stormwater collection, treatment and supply systems—all in pursuit of ensuring water quality and improving water services to the public.
@@ -1658,34 +1725,34 @@
 Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
         </is>
       </c>
-      <c r="D20" s="1" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E20" s="1" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F20" s="1" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-adaptive-control-frameworks-to-unlock-full-scale-bnr-potential-water-research-foundation-wrf-the-water-research-foundation-wrf-opg-26-00187</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="95" customHeight="1">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="inlineStr">
+    <row r="22" ht="95" customHeight="1">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Crossing the Divide Best Practices for Addressing Local and Privately-Owned Lateral Sewer Issues RFP 5419</t>
         </is>
       </c>
-      <c r="C21" s="1" t="inlineStr">
+      <c r="C22" s="1" t="inlineStr">
         <is>
           <t>Project Objective:
 To provide water resource recovery facilities (WRRFs) and collection system operators with an interactive manual of practice for implementing inflow and infiltration (I&amp;I) and obstruction management programs, focused on municipal and privately owned lateral sewers in complex legal, regulatory, and multi-jurisdictional environments.
@@ -1723,34 +1790,34 @@
  Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
         </is>
       </c>
-      <c r="D21" s="1" t="inlineStr">
+      <c r="D22" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E21" s="1" t="inlineStr">
+      <c r="E22" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F21" s="1" t="inlineStr">
+      <c r="F22" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-crossing-the-divide-best-practices-for-addressing-local-and-privately-owned-lateral-sewer-issues-rfp-5419-the-water-research-foundation-wrf-opg-26-00189</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="95" customHeight="1">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="inlineStr">
+    <row r="23" ht="95" customHeight="1">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Comparison of PFAS Contributions to Agricultural Systems</t>
         </is>
       </c>
-      <c r="C22" s="1" t="inlineStr">
+      <c r="C23" s="1" t="inlineStr">
         <is>
           <t>Project Objectives:
 Report per- and polyfluoroalkyl substance (PFAS) concentrations from a variety of agricultural inputs — animal manures, fertilizers, pesticides, composts, soil amendments, seed coatings, and biosolids-based products
@@ -1786,34 +1853,34 @@
  Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00) — same deadline as the other two WRF grants</t>
         </is>
       </c>
-      <c r="D22" s="1" t="inlineStr">
+      <c r="D23" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E22" s="1" t="inlineStr">
+      <c r="E23" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F22" s="1" t="inlineStr">
+      <c r="F23" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-comparison-of-pfas-contributions-to-agricultural-systems-the-water-research-foundation-wrf-opg-26-00190</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="95" customHeight="1">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B23" s="1" t="inlineStr">
+    <row r="24" ht="95" customHeight="1">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Whitley Award 2027</t>
         </is>
       </c>
-      <c r="C23" s="1" t="inlineStr">
+      <c r="C24" s="1" t="inlineStr">
         <is>
           <t>About the Grant: 
 An annual grant by the Whitley Fund for Nature (WFN) recognising grassroots conservation leaders in the Global South, providing funding to support and scale up proven, science-based solutions that deliver lasting impact for both people and nature.
@@ -1826,34 +1893,34 @@
 You do not need to be invited or nominated to apply.</t>
         </is>
       </c>
-      <c r="D23" s="1" t="inlineStr">
+      <c r="D24" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E23" s="1" t="inlineStr">
+      <c r="E24" s="1" t="inlineStr">
         <is>
           <t>Oct 30, 2026</t>
         </is>
       </c>
-      <c r="F23" s="1" t="inlineStr">
+      <c r="F24" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-whitley-award-2027-whitley-fund-for-nature-wfn-opg-26-00153</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="95" customHeight="1">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B24" s="1" t="inlineStr">
+    <row r="25" ht="95" customHeight="1">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIFAR Global Scholars Program 20272029 Cohort</t>
         </is>
       </c>
-      <c r="C24" s="1" t="inlineStr">
+      <c r="C25" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 CIFAR is a Canadian-based globally influential research organization that convenes the world’s most brilliant people across disciplines to advance transformative knowledge and solve humanity’s biggest problems, together. By supporting long-term interdisciplinary collaboration, CIFAR provides researchers with an unparalleled environment of trust, transparency and knowledge sharing. Our time-tested model inspires new directions of inquiry, accelerates discovery and yields breakthroughs across borders and academic disciplines. Through knowledge mobilization, we are catalysts for change in industry, government and society. Through our 15 research programs and the Pan-Canadian AI Strategy, CIFAR convenes close to 400 of the world’s top researchers from 141 institutions in 20 countries. CIFAR is generously supported by the governments of Canada, Alberta and Québec, as well as foundations, individuals, corporations and Canadian and international partner organizations.
@@ -1897,34 +1964,73 @@
  Application Deadline: November 4, 2026, 12:00 PM EST</t>
         </is>
       </c>
-      <c r="D24" s="1" t="inlineStr">
+      <c r="D25" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E24" s="1" t="inlineStr">
+      <c r="E25" s="1" t="inlineStr">
         <is>
           <t>Nov 4, 2026</t>
         </is>
       </c>
-      <c r="F24" s="1" t="inlineStr">
+      <c r="F25" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cifar-global-scholars-program-20272029-cohort-cifar-canadian-institute-for-advanced-research-opg-26-00183</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="95" customHeight="1">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B25" s="1" t="inlineStr">
+    <row r="26" ht="95" customHeight="1">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for IWRS Teaching Innovation Award</t>
         </is>
       </c>
-      <c r="C25" s="1" t="inlineStr">
+      <c r="C26" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
+ About the Grant
+The IWRS (Insect Welfare Research Society) Teaching Innovation Award supports instructors developing new approaches to teaching insect or invertebrate biology that incorporate the 3Rs (Replacement, Reduction, and Refinement) — principles for reducing animal welfare impacts in teaching and research practices.
+ Purpose
+Funds support the creation and implementation of 3Rs-driven instructional materials and pedagogical approaches. Priority is given to proposals addressing common teaching practices with substantial welfare implications.
+ Grant Amount
+Two awards of $2,000 USD are available annually.</t>
+        </is>
+      </c>
+      <c r="D26" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E26" s="1" t="inlineStr">
+        <is>
+          <t>Nov 15, 2026</t>
+        </is>
+      </c>
+      <c r="F26" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="95" customHeight="1">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for IWRS Teaching Innovation Award</t>
+        </is>
+      </c>
+      <c r="C27" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Insects are one of the most numerous and diverse animal groups on Earth.
@@ -1939,73 +2045,34 @@
 IWRS staff and Advisory Group members are not eligible to apply.</t>
         </is>
       </c>
-      <c r="D25" s="1" t="inlineStr">
+      <c r="D27" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E25" s="1" t="inlineStr">
+      <c r="E27" s="1" t="inlineStr">
         <is>
           <t>Nov 15, 2026</t>
         </is>
       </c>
-      <c r="F25" s="1" t="inlineStr">
+      <c r="F27" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00166</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="95" customHeight="1">
-      <c r="A26" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B26" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for IWRS Teaching Innovation Award</t>
-        </is>
-      </c>
-      <c r="C26" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
- About the Grant
-The IWRS (Insect Welfare Research Society) Teaching Innovation Award supports instructors developing new approaches to teaching insect or invertebrate biology that incorporate the 3Rs (Replacement, Reduction, and Refinement) — principles for reducing animal welfare impacts in teaching and research practices.
- Purpose
-Funds support the creation and implementation of 3Rs-driven instructional materials and pedagogical approaches. Priority is given to proposals addressing common teaching practices with substantial welfare implications.
- Grant Amount
-Two awards of $2,000 USD are available annually.</t>
-        </is>
-      </c>
-      <c r="D26" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E26" s="1" t="inlineStr">
-        <is>
-          <t>Nov 15, 2026</t>
-        </is>
-      </c>
-      <c r="F26" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="95" customHeight="1">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B27" s="1" t="inlineStr">
+    <row r="28" ht="95" customHeight="1">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Medium-Size Grants Call for Proposals Global EbA Fund</t>
         </is>
       </c>
-      <c r="C27" s="1" t="inlineStr">
+      <c r="C28" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -2062,34 +2129,34 @@
 Applications submitted via online portal (link shared on the Medium-Size Grants webpage from Oct 12)</t>
         </is>
       </c>
-      <c r="D27" s="1" t="inlineStr">
+      <c r="D28" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E27" s="1" t="inlineStr">
+      <c r="E28" s="1" t="inlineStr">
         <is>
           <t>Nov 16, 2026</t>
         </is>
       </c>
-      <c r="F27" s="1" t="inlineStr">
+      <c r="F28" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-medium-size-grants-call-for-proposals-global-eba-fund-global-eba-fund-opg-26-00178</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="95" customHeight="1">
-      <c r="A28" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B28" s="1" t="inlineStr">
+    <row r="29" ht="95" customHeight="1">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIEIF Grant 2026 Climate Intervention Environmental Impact Fund</t>
         </is>
       </c>
-      <c r="C28" s="1" t="inlineStr">
+      <c r="C29" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Climate Intervention Environmental Impact Fund (CIEIF) is a philanthropic fund focused on supporting responsible climate intervention field tests. It provides grants for activities such as environmental impact assessment (EIA), predictive impact modelling, and engagement with potentially affected stakeholders, including local communities and government agencies.
@@ -2116,34 +2183,34 @@
 Potential for scaling the innovation to a globally relevant level</t>
         </is>
       </c>
-      <c r="D28" s="1" t="inlineStr">
+      <c r="D29" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E28" s="1" t="inlineStr">
+      <c r="E29" s="1" t="inlineStr">
         <is>
           <t>Dec 1, 2026</t>
         </is>
       </c>
-      <c r="F28" s="1" t="inlineStr">
+      <c r="F29" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cieif-grant-2026-climate-intervention-environmental-impact-fund-climate-intervention-environmental-impact-fund-opg-26-00155</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="95" customHeight="1">
-      <c r="A29" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B29" s="1" t="inlineStr">
+    <row r="30" ht="95" customHeight="1">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 6th Annual Seeding The Future Global Food System Challenge</t>
         </is>
       </c>
-      <c r="C29" s="1" t="inlineStr">
+      <c r="C30" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are one of the largest and most respected private organisations for development cooperation and humanitarian aid in Germany. As a politically and confessionally independent organisation, our value-oriented actions are always based on ethical principles. Our vision is clear: "Zero Hunger by 2030"
@@ -2175,34 +2242,78 @@
 Individuals with no organizational entity</t>
         </is>
       </c>
-      <c r="D29" s="1" t="inlineStr">
+      <c r="D30" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E29" s="1" t="inlineStr">
+      <c r="E30" s="1" t="inlineStr">
         <is>
           <t>Jan 1, 2027</t>
         </is>
       </c>
-      <c r="F29" s="1" t="inlineStr">
+      <c r="F30" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-6th-annual-seeding-the-future-global-food-system-challenge-welthungerhilfe-opg-26-00180</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="95" customHeight="1">
-      <c r="A30" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B30" s="1" t="inlineStr">
+    <row r="31" ht="95" customHeight="1">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Microbiota &amp; Women's Health International Call for Projects</t>
+        </is>
+      </c>
+      <c r="C31" s="1" t="inlineStr">
+        <is>
+          <t>About the Grant
+An annual international research grant by the Biocodex Microbiota Foundation (BMF), rewarding research proposals on the microbiota and its implications in Women's Health and Disease. This year's theme: "Unraveling male-female genital microbiome interactions: mechanisms, transmission, and impact on vaginal dysbiosis."
+ Theme/Scope
+Proposals could include, but are not limited to, mechanistic studies elucidating how the penile microbiome contributes to the establishment, persistence, and recurrence of vaginal dysbiosis, including bacterial vaginosis. Areas of interest include microbial transmission dynamics during sexual activity, niche adaptation and persistence of BV-associated taxa in the penile environment, and the functional consequences of these interactions for vaginal community stability.
+Studies evaluating how current and emerging interventions (antibiotics, topical or systemic partner therapies, circumcision, or live biotherapeutic products) alter penile microbial ecology and influence treatment response and recurrence risk in female partners are also encouraged.
+ Purpose: From 2025, the Biocodex Microbiota Foundation rewards international research proposals involving the microbiota and its implication in Women's Health and Disease. Every year, the call for proposals covers a specific theme chosen by an International Scientific Committee. Either clinical or fundamental research proposals can be submitted. Maximum project duration: 3 years.
+ Eligibility
+Open to MDs, PhDs, or Pharm-Ds working in the subject area (gynecology, obstetrics, microbiology, infectious diseases, internal medicine, oncology, etc.).
+No geographic restrictions — all countries are eligible.
+A principal investigator who received a Women's Health International grant from BMF cannot reapply for this award for three years. However, winners of another BMF grant category can apply for this grant.
+Members of the Women's Health International Scientific Committee and their laboratory members are not allowed to apply as Principal Investigators.
+ Grant Amount
+€200,000 annually — awarded to researchers within universities, hospitals, or other research settings to finance equipment, operations, or staffing costs. Grants are NOT awarded to individuals directly (must be institutionally affiliated). Institution's overhead costs capped at 10%.</t>
+        </is>
+      </c>
+      <c r="D31" s="1" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="E31" s="1" t="inlineStr">
+        <is>
+          <t>Jan 15, 2027</t>
+        </is>
+      </c>
+      <c r="F31" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-microbiota-and-womens-health-international-call-for-projects-biocodex-microbiota-foundation-bmf-opg-26-00152</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="95" customHeight="1">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B32" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for BES Training and Travel Grants</t>
         </is>
       </c>
-      <c r="C30" s="1" t="inlineStr">
+      <c r="C32" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are a global community of scientists shining a spotlight on the intricacy and value of our natural world, providing the evidence for better decisions. Our vision is for people and nature to thrive in a world that values ecology.
@@ -2241,17 +2352,17 @@
  Application Deadline (Round 2): Opens 30 April 2026, closes 17 May 2026</t>
         </is>
       </c>
-      <c r="D30" s="1" t="inlineStr">
+      <c r="D32" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E30" s="1" t="inlineStr">
+      <c r="E32" s="1" t="inlineStr">
         <is>
           <t>May 17, 2027</t>
         </is>
       </c>
-      <c r="F30" s="1" t="inlineStr">
+      <c r="F32" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-bes-training-and-travel-grants-british-ecological-society-opg-26-00181</t>
         </is>

</xml_diff>

<commit_message>
Auto update Combined.xlsx [Fri Sep 25 07:02:19 UTC 2026]
</commit_message>
<xml_diff>
--- a/output/Combined.xlsx
+++ b/output/Combined.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1060,10 +1060,129 @@
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
+          <t>EOI - Engagement of Agencies for HR Recruitment Services</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>The American India Foundation Trust (AIFT) seeks to engage an experienced recruitment agency to provide end-to-end recruitment and talent acquisition services for identified positions across its offices, programmes, and functions in India.
+The selected agency shall support AIFT in sourcing, screening, shortlisting, interview coordination, candidate engagement, offer management, and recruitment closure, in accordance with the requirements, timelines, and service levels agreed with AIFT.
+The agency shall ensure access to a relevant, qualified, and diverse pool of candidates while maintaining confidentiality, professionalism, and compliance with applicable laws and AIFT's requirements. Engagement period to start tentatively from 1st October 2026 to 30th September 2027.
+Scope of Services
+Understanding of Recruitment Requirements
+The agency shall:
+Understand the manpower requirement, role profile, reporting structure, location, compensation range, experience requirements, and other specifications shared by AIFT.
+Seek clarification from AIFT wherever required before initiating the recruitment process.
+Develop an appropriate recruitment/search strategy based on the nature and seniority of the position.
+Maintain confidentiality of all information shared by AIFT.
+Candidate Sourcing and Vacancy Posting
+The agency shall undertake proactive candidate sourcing through appropriate channels, including:
+Relevant online job portals and professional networks;
+Social media and sector-specific platforms;
+Existing/internal candidate databases;
+Professional networks and referrals;
+Targeted sourcing/headhunting for senior or specialised positions; and
+Other appropriate sourcing channels.
+For each shortlisted candidate, the agency shall provide a structured candidate summary containing, at minimum:
+Current/most recent designation and organisation;
+Total and relevant experience;
+Educational qualifications;
+Current and expected CTC;
+Notice period/availability;
+Current location and preferred location;
+Key strengths/relevance to the role; and
+Any other information specifically requested by AIFT.</t>
+        </is>
+      </c>
+      <c r="D11" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>Oct 4, 2026</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/eoi-engagement-of-agencies-for-hr-recruitment-services-american-india-foundation-rfp-26-00375</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="95" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>ToR for Onboarding of consultant/agency for Innovating &amp; Scaling Reproductive Maternal Newborn and Child Health Solutions in the Last-Mile</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>Title Terms of Reference for Onboarding of consultant/agency for Innovating &amp; Scaling Reproductive, Maternal, Newborn and Child Health Solutions in the Last-Mile
+Timeline September 2026 to February 2027
+Scope of Work
+• Outreach and program visibility
+• Application design, launch, review, shortlisting, and due diligence
+• Stakeholder engagement and coordination
+• Knowledge materials and document learnings and insights
+Application Link https://forms.gle/jsngbAREkYmgK7cB6
+Last Date to Apply 5th October, 5 PM
+About SELCO Foundation:
+SELCO Foundation's mission is to create a platform of solutions that uses sustainable energy as a catalyst to bridge environmental sustainability and poverty alleviation. With holistic development as the primary focus, the organization strives to create equitable societies, where services are accessed by all communities. The interventions of SELCO lead to a sustainable delivery model of essential services like livelihoods, education, and health till the last mile.
+(Read more about SELCO here: https://selcofoundation.org/)
+ About the Program
+The program aims to catalyse the development, adoption, and scale of innovative solutions that contribute to improved maternal and child health outcomes. It seeks to build an ecosystem where enterprises and innovators can develop and strengthen technology and technology-allied solutions that enable more accessible, quality, efficient, affordable, and continuous maternal and child health services, particularly across last-mile health facilities and underserved communities.
+The program envisions a future where innovation, technology, and enterprise-led solutions are meaningfully integrated into maternal and child health delivery, enabling health systems, facilities, and frontline health workers to deliver better services to women and children.
+The initiative will bring together enterprises, innovators, health facilities, frontline health workers, institutions, and other ecosystem stakeholders to co-create, test, deploy, and scale solutions with the potential to transform maternal and child health delivery. The focus will be on enabling promising solutions to move beyond individual deployments towards sustainable models of adoption, replication, and scale.
+For the same, we are looking to partner with a like-minded organization that shares this vision and can play an integral role in designing and implementing the initiative. The partner will support enterprise identification and engagement, solution assessment, co-creation, health-system linkages, implementation, stakeholder coordination, evidence generation, and pathways to scale, contributing to more resilient, responsive, and equitable maternal and child health services for women and children.
+ Geography
+Primary Focus: Maharashtra, Karnataka, Odisha, Meghalaya, Mizoram, Nagaland
+Secondary Focus: Other states
+ Selection Criteria
+Applicants should meet the following criteria for being a part of the evaluation:
+Demonstrated experience working with vendors, enterprises, innovators, or solution providers, along with an understanding of grassroots and last-mile contexts and user needs
+Ability to assess enterprise and solution needs and curate tailored mentorship, technical assistance, health-system linkages, and implementation support
+Demonstrated experience in program design, planning, implementation, and management of multi-stakeholder initiatives, preferably in health, maternal and child health, technology, or last-mile service delivery
+Proven ability to manage end-to-end application, assessment, screening, shortlisting, and due diligence processes for a portfolio of enterprises or innovators
+Experience in communication, outreach, stakeholder engagement, and facilitating collaboration between solution providers and health-system stakeholders
+Capability to develop documentation and knowledge products that capture program processes, solution performance, outcomes, implementation models, and learnings for scale and replication
+Prior experience working with development sector organisations, NGOs, health systems, technology providers, enterprises, or think tanks will be considered an added advantage
+The agency will be selected on a combined technical and financial evaluation. Proposals must score a minimum of 70% on the technical components (1–5 below) to be considered for financial evaluation.</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>Oct 5, 2026</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/tor-for-onboarding-of-consultantagency-for-innovating-and-scaling-reproductive-maternal-newborn-and-child-health-solutions-in-the-last-mile-selco-foundation-rfp-26-00373</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="95" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
           <t>RFP - Design and Delivery of an Electric Vehicle EV Skilling Programme in Karnataka</t>
         </is>
       </c>
-      <c r="C11" s="1" t="inlineStr">
+      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 WRI India, an independent knowledge organisation registered as the India Resources Trust, provides objective information and practical proposals to foster environmentally sound and socially equitable development. As an independent knowledge organisation, we leverage our data and expertise to catalyze change across systems like food, land and water; energy; and cities. Our work focuses on improving people’s lives, protecting and restoring nature, and addressing climate change. To enable progress at the pace and scale needed, we also engage with the economic, finance and governance systems that are key to enabling this change.
@@ -1104,95 +1223,34 @@
 Must have a team of qualified trainers and master trainers with relevant domain expertise, as well as administrative and coordination support.</t>
         </is>
       </c>
-      <c r="D11" s="1" t="inlineStr">
+      <c r="D13" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E11" s="1" t="inlineStr">
+      <c r="E13" s="1" t="inlineStr">
         <is>
           <t>Oct 5, 2026</t>
         </is>
       </c>
-      <c r="F11" s="1" t="inlineStr">
+      <c r="F13" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfp-design-and-delivery-of-an-electric-vehicle-ev-skilling-programme-in-karnataka-wri-india-rfp-26-00361</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="95" customHeight="1">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="inlineStr">
-        <is>
-          <t>ToR for Onboarding of consultant/agency for Innovating &amp; Scaling Reproductive Maternal Newborn and Child Health Solutions in the Last-Mile</t>
-        </is>
-      </c>
-      <c r="C12" s="1" t="inlineStr">
-        <is>
-          <t>Title Terms of Reference for Onboarding of consultant/agency for Innovating &amp; Scaling Reproductive, Maternal, Newborn and Child Health Solutions in the Last-Mile
-Timeline September 2026 to February 2027
-Scope of Work
-• Outreach and program visibility
-• Application design, launch, review, shortlisting, and due diligence
-• Stakeholder engagement and coordination
-• Knowledge materials and document learnings and insights
-Application Link https://forms.gle/jsngbAREkYmgK7cB6
-Last Date to Apply 5th October, 5 PM
-About SELCO Foundation:
-SELCO Foundation's mission is to create a platform of solutions that uses sustainable energy as a catalyst to bridge environmental sustainability and poverty alleviation. With holistic development as the primary focus, the organization strives to create equitable societies, where services are accessed by all communities. The interventions of SELCO lead to a sustainable delivery model of essential services like livelihoods, education, and health till the last mile.
-(Read more about SELCO here: https://selcofoundation.org/)
- About the Program
-The program aims to catalyse the development, adoption, and scale of innovative solutions that contribute to improved maternal and child health outcomes. It seeks to build an ecosystem where enterprises and innovators can develop and strengthen technology and technology-allied solutions that enable more accessible, quality, efficient, affordable, and continuous maternal and child health services, particularly across last-mile health facilities and underserved communities.
-The program envisions a future where innovation, technology, and enterprise-led solutions are meaningfully integrated into maternal and child health delivery, enabling health systems, facilities, and frontline health workers to deliver better services to women and children.
-The initiative will bring together enterprises, innovators, health facilities, frontline health workers, institutions, and other ecosystem stakeholders to co-create, test, deploy, and scale solutions with the potential to transform maternal and child health delivery. The focus will be on enabling promising solutions to move beyond individual deployments towards sustainable models of adoption, replication, and scale.
-For the same, we are looking to partner with a like-minded organization that shares this vision and can play an integral role in designing and implementing the initiative. The partner will support enterprise identification and engagement, solution assessment, co-creation, health-system linkages, implementation, stakeholder coordination, evidence generation, and pathways to scale, contributing to more resilient, responsive, and equitable maternal and child health services for women and children.
- Geography
-Primary Focus: Maharashtra, Karnataka, Odisha, Meghalaya, Mizoram, Nagaland
-Secondary Focus: Other states
- Selection Criteria
-Applicants should meet the following criteria for being a part of the evaluation:
-Demonstrated experience working with vendors, enterprises, innovators, or solution providers, along with an understanding of grassroots and last-mile contexts and user needs
-Ability to assess enterprise and solution needs and curate tailored mentorship, technical assistance, health-system linkages, and implementation support
-Demonstrated experience in program design, planning, implementation, and management of multi-stakeholder initiatives, preferably in health, maternal and child health, technology, or last-mile service delivery
-Proven ability to manage end-to-end application, assessment, screening, shortlisting, and due diligence processes for a portfolio of enterprises or innovators
-Experience in communication, outreach, stakeholder engagement, and facilitating collaboration between solution providers and health-system stakeholders
-Capability to develop documentation and knowledge products that capture program processes, solution performance, outcomes, implementation models, and learnings for scale and replication
-Prior experience working with development sector organisations, NGOs, health systems, technology providers, enterprises, or think tanks will be considered an added advantage
-The agency will be selected on a combined technical and financial evaluation. Proposals must score a minimum of 70% on the technical components (1–5 below) to be considered for financial evaluation.</t>
-        </is>
-      </c>
-      <c r="D12" s="1" t="inlineStr">
-        <is>
-          <t>Learning</t>
-        </is>
-      </c>
-      <c r="E12" s="1" t="inlineStr">
-        <is>
-          <t>Oct 5, 2026</t>
-        </is>
-      </c>
-      <c r="F12" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/tor-for-onboarding-of-consultantagency-for-innovating-and-scaling-reproductive-maternal-newborn-and-child-health-solutions-in-the-last-mile-selco-foundation-rfp-26-00373</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="95" customHeight="1">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B13" s="1" t="inlineStr">
+    <row r="14" ht="95" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>RFPs Invited for Engagement of a Manpower Agency for Providing Subject Matter Specialists/Experts for the Cluster Development Programme</t>
         </is>
       </c>
-      <c r="C13" s="1" t="inlineStr">
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>About the RFP
 National Horticulture Board (NHB), an autonomous organization under the Ministry of Agriculture and Farmers' Welfare, Government of India, invites bids from eligible manpower agencies for engagement to recruit, deploy, and manage qualified personnel supporting NHB's Cluster Development Programme (CDP) — a Central Sector Scheme promoting integrated, market-led horticulture cluster development. The engaged agency will provide three types of Subject Matter Experts per Cluster and additional consultants/manpower as required by NHB from time to time.
@@ -1218,34 +1276,34 @@
  District: Gurugram, Haryana (NHB Head Office)</t>
         </is>
       </c>
-      <c r="D13" s="1" t="inlineStr">
+      <c r="D14" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E13" s="1" t="inlineStr">
+      <c r="E14" s="1" t="inlineStr">
         <is>
           <t>Oct 6, 2026</t>
         </is>
       </c>
-      <c r="F13" s="1" t="inlineStr">
+      <c r="F14" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfps-invited-for-engagement-of-a-manpower-agency-for-providing-subject-matter-specialistsexperts-for-the-cluster-development-programme-national-horticulture-board-nhb-rfp-26-00370</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="95" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="inlineStr">
+    <row r="15" ht="95" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>Applications Open Draper Richards Kaplan Foundation Funding for Social Enterprises</t>
         </is>
       </c>
-      <c r="C14" s="1" t="inlineStr">
+      <c r="C15" s="1" t="inlineStr">
         <is>
           <t>About us
 Started in 2002, Draper Richards Kaplan Foundation (DRK) is a global venture philanthropy firm supporting early stage, high impact social enterprises. Borrowed from our venture capital legacy, DRK finds, funds, and supports exceptional leaders building innovative solutions to some of the world’s most challenging social and environmental problems. Since beginning this work nearly 25 years ago, DRK has invested in more than 270 organizations that have collectively impacted over 610 million lives to date.
@@ -1269,34 +1327,34 @@
 Please attach a standard resume/CV for the entrepreneur(s) and/or key leadership team members (e.g., CEO, COO, ED, etc.). Applications with text bios for entrepreneurs or members of the leadership team will not be considered.</t>
         </is>
       </c>
-      <c r="D14" s="1" t="inlineStr">
+      <c r="D15" s="1" t="inlineStr">
         <is>
           <t>Climate</t>
         </is>
       </c>
-      <c r="E14" s="1" t="inlineStr">
+      <c r="E15" s="1" t="inlineStr">
         <is>
           <t>Oct 10, 2026</t>
         </is>
       </c>
-      <c r="F14" s="1" t="inlineStr">
+      <c r="F15" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-open-draper-richards-kaplan-foundation-funding-for-social-enterprises-draper-richards-kaplan-foundation-opg-26-00188</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="95" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="inlineStr">
+    <row r="16" ht="95" customHeight="1">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund</t>
         </is>
       </c>
-      <c r="C15" s="1" t="inlineStr">
+      <c r="C16" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund
 Apply by: 13 October, 2026
@@ -1321,34 +1379,34 @@
  Projects should include opportunities for ServiceNow employees to volunteer in the project activation or implementation.</t>
         </is>
       </c>
-      <c r="D15" s="1" t="inlineStr">
+      <c r="D16" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E15" s="1" t="inlineStr">
+      <c r="E16" s="1" t="inlineStr">
         <is>
           <t>Oct 13, 2026</t>
         </is>
       </c>
-      <c r="F15" s="1" t="inlineStr">
+      <c r="F16" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/apply-for-the-servicenow-community-solar-fund-changex-opg-26-00186</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="95" customHeight="1">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B16" s="1" t="inlineStr">
+    <row r="17" ht="95" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
         <is>
           <t>RFPs Invited for Empanelment of Publishers for Procurement of E-Books for Rashtriya e-Pustakalaya National Book Trust India</t>
         </is>
       </c>
-      <c r="C16" s="1" t="inlineStr">
+      <c r="C17" s="1" t="inlineStr">
         <is>
           <t>About the RFP:
 Rashtriya e-Pustakalaya, a free National Digital Library for children and adolescents — an initiative of the Department of School Education &amp; Literacy, Ministry of Education, Government of India, implemented by the National Book Trust (NBT), India — invites Expression of Interest (EoI) for the empanelment of publishers for the selection and procurement of e-books, with the objective of enriching the platform's book collection. NBT is an autonomous body under the Ministry of Education, established in 1957 to promote literacy and reading culture in India.
@@ -1370,34 +1428,34 @@
 Must indemnify Rashtriya e-Pustakalaya/NBT-India for any IP-related claims from authors/illustrators/translators/legal owners</t>
         </is>
       </c>
-      <c r="D16" s="1" t="inlineStr">
+      <c r="D17" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E16" s="1" t="inlineStr">
+      <c r="E17" s="1" t="inlineStr">
         <is>
           <t>Oct 16, 2026</t>
         </is>
       </c>
-      <c r="F16" s="1" t="inlineStr">
+      <c r="F17" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfps-invited-for-empanelment-of-publishers-for-procurement-of-e-books-for-rashtriya-e-pustakalaya-national-book-trust-india-national-book-trust-nbt-india-rfp-26-00371</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="95" customHeight="1">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B17" s="1" t="inlineStr">
+    <row r="18" ht="95" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>ToR - Engagement of Consultant/Vendor Individual towards implementation of Literacy Program in Telangana State</t>
         </is>
       </c>
-      <c r="C17" s="1" t="inlineStr">
+      <c r="C18" s="1" t="inlineStr">
         <is>
           <t>ANNEX A – TERMS OF REFERENCE (ToR) 
  Engagement of Consultant/Vendor (Individual) towards implementation of Literacy Program in Telangana State.
@@ -1462,34 +1520,34 @@
 Approved travel and accommodation expenses incurred for assignment-related activities shall be reimbursed by Room to Read in accordance with the consultancy reimbursement guidelines.</t>
         </is>
       </c>
-      <c r="D17" s="1" t="inlineStr">
+      <c r="D18" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E17" s="1" t="inlineStr">
+      <c r="E18" s="1" t="inlineStr">
         <is>
           <t>Oct 16, 2026</t>
         </is>
       </c>
-      <c r="F17" s="1" t="inlineStr">
+      <c r="F18" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-engagement-of-consultantvendor-individual-towards-implementation-of-literacy-program-in-telangana-state-room-to-read-india-rfp-26-00360</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="95" customHeight="1">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="inlineStr">
+    <row r="19" ht="95" customHeight="1">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>RFPs Invited for Consultant to Develop a Technical Assistance Package for National Application of the Digital Health and AI Investment Classification Framework</t>
         </is>
       </c>
-      <c r="C18" s="1" t="inlineStr">
+      <c r="C19" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are Transform Health: a global coalition of more than 200 organisations driving the digital transformation of health to achieve universal health coverage. 
@@ -1517,34 +1575,34 @@
 Ability to manage multi-country consultancy engagements and coordinate with in-country focal points</t>
         </is>
       </c>
-      <c r="D18" s="1" t="inlineStr">
+      <c r="D19" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E18" s="1" t="inlineStr">
+      <c r="E19" s="1" t="inlineStr">
         <is>
           <t>Oct 23, 2026</t>
         </is>
       </c>
-      <c r="F18" s="1" t="inlineStr">
+      <c r="F19" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfps-invited-for-consultant-to-develop-a-technical-assistance-package-for-national-application-of-the-digital-health-and-ai-investment-classification-framework-transform-health-rfp-26-00359</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="95" customHeight="1">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="inlineStr">
+    <row r="20" ht="95" customHeight="1">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for D-Prize Global Competition Seed Funding for New Poverty-Solution Distribution Organizations</t>
         </is>
       </c>
-      <c r="C19" s="1" t="inlineStr">
+      <c r="C20" s="1" t="inlineStr">
         <is>
           <t>About the Grant:
 D-Prize seeds new organizations that distribute proven poverty solutions at the "last mile," with the aim of scaling impact. Applicants select from a range of evidence-based interventions (health, agriculture, education, water, safety, transparency, and more) and propose how they would launch or grow an organization to distribute that intervention. Top entrepreneurs receive up to $20,000 in seed funding to run a pilot and build an organization capable of scaling to reach thousands, even millions of people.
@@ -1567,34 +1625,34 @@
 Extension Deadline: 6 December 2026, midnight PT (extension registration required)</t>
         </is>
       </c>
-      <c r="D19" s="1" t="inlineStr">
+      <c r="D20" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E19" s="1" t="inlineStr">
+      <c r="E20" s="1" t="inlineStr">
         <is>
           <t>Oct 25, 2026</t>
         </is>
       </c>
-      <c r="F19" s="1" t="inlineStr">
+      <c r="F20" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-d-prize-global-competition-seed-funding-for-new-poverty-solution-distribution-organizations-d-prize-opg-26-00191</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="95" customHeight="1">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="inlineStr">
+    <row r="21" ht="95" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 8th Call for Proposals Small-Size Grants Global EbA Fund</t>
         </is>
       </c>
-      <c r="C20" s="1" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -1657,34 +1715,34 @@
 Only successful applicants will be contacted; no individual feedback provided to unsuccessful applicants</t>
         </is>
       </c>
-      <c r="D20" s="1" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E20" s="1" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F20" s="1" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-8th-call-for-proposals-small-size-grants-global-eba-fund-global-eba-fund-opg-26-00177</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="95" customHeight="1">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="inlineStr">
+    <row r="22" ht="95" customHeight="1">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Adaptive Control Frameworks to Unlock Full-Scale BNR Potential Water Research Foundation WRF</t>
         </is>
       </c>
-      <c r="C21" s="1" t="inlineStr">
+      <c r="C22" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Water Research Foundation (WRF) is the leading research organization advancing the science of all water to meet the evolving needs of its subscribers and the water sector. WRF is a nonprofit, charitable and educational organization which funds, manages, and publishes research on the technology, operation, and management of drinking water, wastewater, reuse, and stormwater collection, treatment and supply systems—all in pursuit of ensuring water quality and improving water services to the public.
@@ -1725,34 +1783,34 @@
 Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
         </is>
       </c>
-      <c r="D21" s="1" t="inlineStr">
+      <c r="D22" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E21" s="1" t="inlineStr">
+      <c r="E22" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F21" s="1" t="inlineStr">
+      <c r="F22" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-adaptive-control-frameworks-to-unlock-full-scale-bnr-potential-water-research-foundation-wrf-the-water-research-foundation-wrf-opg-26-00187</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="95" customHeight="1">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="inlineStr">
+    <row r="23" ht="95" customHeight="1">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Crossing the Divide Best Practices for Addressing Local and Privately-Owned Lateral Sewer Issues RFP 5419</t>
         </is>
       </c>
-      <c r="C22" s="1" t="inlineStr">
+      <c r="C23" s="1" t="inlineStr">
         <is>
           <t>Project Objective:
 To provide water resource recovery facilities (WRRFs) and collection system operators with an interactive manual of practice for implementing inflow and infiltration (I&amp;I) and obstruction management programs, focused on municipal and privately owned lateral sewers in complex legal, regulatory, and multi-jurisdictional environments.
@@ -1790,34 +1848,34 @@
  Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
         </is>
       </c>
-      <c r="D22" s="1" t="inlineStr">
+      <c r="D23" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E22" s="1" t="inlineStr">
+      <c r="E23" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F22" s="1" t="inlineStr">
+      <c r="F23" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-crossing-the-divide-best-practices-for-addressing-local-and-privately-owned-lateral-sewer-issues-rfp-5419-the-water-research-foundation-wrf-opg-26-00189</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="95" customHeight="1">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B23" s="1" t="inlineStr">
+    <row r="24" ht="95" customHeight="1">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Comparison of PFAS Contributions to Agricultural Systems</t>
         </is>
       </c>
-      <c r="C23" s="1" t="inlineStr">
+      <c r="C24" s="1" t="inlineStr">
         <is>
           <t>Project Objectives:
 Report per- and polyfluoroalkyl substance (PFAS) concentrations from a variety of agricultural inputs — animal manures, fertilizers, pesticides, composts, soil amendments, seed coatings, and biosolids-based products
@@ -1853,34 +1911,34 @@
  Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00) — same deadline as the other two WRF grants</t>
         </is>
       </c>
-      <c r="D23" s="1" t="inlineStr">
+      <c r="D24" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E23" s="1" t="inlineStr">
+      <c r="E24" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F23" s="1" t="inlineStr">
+      <c r="F24" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-comparison-of-pfas-contributions-to-agricultural-systems-the-water-research-foundation-wrf-opg-26-00190</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="95" customHeight="1">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B24" s="1" t="inlineStr">
+    <row r="25" ht="95" customHeight="1">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Whitley Award 2027</t>
         </is>
       </c>
-      <c r="C24" s="1" t="inlineStr">
+      <c r="C25" s="1" t="inlineStr">
         <is>
           <t>About the Grant: 
 An annual grant by the Whitley Fund for Nature (WFN) recognising grassroots conservation leaders in the Global South, providing funding to support and scale up proven, science-based solutions that deliver lasting impact for both people and nature.
@@ -1893,34 +1951,34 @@
 You do not need to be invited or nominated to apply.</t>
         </is>
       </c>
-      <c r="D24" s="1" t="inlineStr">
+      <c r="D25" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E24" s="1" t="inlineStr">
+      <c r="E25" s="1" t="inlineStr">
         <is>
           <t>Oct 30, 2026</t>
         </is>
       </c>
-      <c r="F24" s="1" t="inlineStr">
+      <c r="F25" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-whitley-award-2027-whitley-fund-for-nature-wfn-opg-26-00153</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="95" customHeight="1">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B25" s="1" t="inlineStr">
+    <row r="26" ht="95" customHeight="1">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIFAR Global Scholars Program 20272029 Cohort</t>
         </is>
       </c>
-      <c r="C25" s="1" t="inlineStr">
+      <c r="C26" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 CIFAR is a Canadian-based globally influential research organization that convenes the world’s most brilliant people across disciplines to advance transformative knowledge and solve humanity’s biggest problems, together. By supporting long-term interdisciplinary collaboration, CIFAR provides researchers with an unparalleled environment of trust, transparency and knowledge sharing. Our time-tested model inspires new directions of inquiry, accelerates discovery and yields breakthroughs across borders and academic disciplines. Through knowledge mobilization, we are catalysts for change in industry, government and society. Through our 15 research programs and the Pan-Canadian AI Strategy, CIFAR convenes close to 400 of the world’s top researchers from 141 institutions in 20 countries. CIFAR is generously supported by the governments of Canada, Alberta and Québec, as well as foundations, individuals, corporations and Canadian and international partner organizations.
@@ -1964,34 +2022,34 @@
  Application Deadline: November 4, 2026, 12:00 PM EST</t>
         </is>
       </c>
-      <c r="D25" s="1" t="inlineStr">
+      <c r="D26" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E25" s="1" t="inlineStr">
+      <c r="E26" s="1" t="inlineStr">
         <is>
           <t>Nov 4, 2026</t>
         </is>
       </c>
-      <c r="F25" s="1" t="inlineStr">
+      <c r="F26" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cifar-global-scholars-program-20272029-cohort-cifar-canadian-institute-for-advanced-research-opg-26-00183</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="95" customHeight="1">
-      <c r="A26" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B26" s="1" t="inlineStr">
+    <row r="27" ht="95" customHeight="1">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for IWRS Teaching Innovation Award</t>
         </is>
       </c>
-      <c r="C26" s="1" t="inlineStr">
+      <c r="C27" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
@@ -2003,34 +2061,34 @@
 Two awards of $2,000 USD are available annually.</t>
         </is>
       </c>
-      <c r="D26" s="1" t="inlineStr">
+      <c r="D27" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E26" s="1" t="inlineStr">
+      <c r="E27" s="1" t="inlineStr">
         <is>
           <t>Nov 15, 2026</t>
         </is>
       </c>
-      <c r="F26" s="1" t="inlineStr">
+      <c r="F27" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="95" customHeight="1">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B27" s="1" t="inlineStr">
+    <row r="28" ht="95" customHeight="1">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for IWRS Teaching Innovation Award</t>
         </is>
       </c>
-      <c r="C27" s="1" t="inlineStr">
+      <c r="C28" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Insects are one of the most numerous and diverse animal groups on Earth.
@@ -2045,34 +2103,34 @@
 IWRS staff and Advisory Group members are not eligible to apply.</t>
         </is>
       </c>
-      <c r="D27" s="1" t="inlineStr">
+      <c r="D28" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E27" s="1" t="inlineStr">
+      <c r="E28" s="1" t="inlineStr">
         <is>
           <t>Nov 15, 2026</t>
         </is>
       </c>
-      <c r="F27" s="1" t="inlineStr">
+      <c r="F28" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00166</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="95" customHeight="1">
-      <c r="A28" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B28" s="1" t="inlineStr">
+    <row r="29" ht="95" customHeight="1">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Medium-Size Grants Call for Proposals Global EbA Fund</t>
         </is>
       </c>
-      <c r="C28" s="1" t="inlineStr">
+      <c r="C29" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -2129,34 +2187,34 @@
 Applications submitted via online portal (link shared on the Medium-Size Grants webpage from Oct 12)</t>
         </is>
       </c>
-      <c r="D28" s="1" t="inlineStr">
+      <c r="D29" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E28" s="1" t="inlineStr">
+      <c r="E29" s="1" t="inlineStr">
         <is>
           <t>Nov 16, 2026</t>
         </is>
       </c>
-      <c r="F28" s="1" t="inlineStr">
+      <c r="F29" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-medium-size-grants-call-for-proposals-global-eba-fund-global-eba-fund-opg-26-00178</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="95" customHeight="1">
-      <c r="A29" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B29" s="1" t="inlineStr">
+    <row r="30" ht="95" customHeight="1">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIEIF Grant 2026 Climate Intervention Environmental Impact Fund</t>
         </is>
       </c>
-      <c r="C29" s="1" t="inlineStr">
+      <c r="C30" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Climate Intervention Environmental Impact Fund (CIEIF) is a philanthropic fund focused on supporting responsible climate intervention field tests. It provides grants for activities such as environmental impact assessment (EIA), predictive impact modelling, and engagement with potentially affected stakeholders, including local communities and government agencies.
@@ -2183,34 +2241,34 @@
 Potential for scaling the innovation to a globally relevant level</t>
         </is>
       </c>
-      <c r="D29" s="1" t="inlineStr">
+      <c r="D30" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E29" s="1" t="inlineStr">
+      <c r="E30" s="1" t="inlineStr">
         <is>
           <t>Dec 1, 2026</t>
         </is>
       </c>
-      <c r="F29" s="1" t="inlineStr">
+      <c r="F30" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cieif-grant-2026-climate-intervention-environmental-impact-fund-climate-intervention-environmental-impact-fund-opg-26-00155</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="95" customHeight="1">
-      <c r="A30" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B30" s="1" t="inlineStr">
+    <row r="31" ht="95" customHeight="1">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 6th Annual Seeding The Future Global Food System Challenge</t>
         </is>
       </c>
-      <c r="C30" s="1" t="inlineStr">
+      <c r="C31" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are one of the largest and most respected private organisations for development cooperation and humanitarian aid in Germany. As a politically and confessionally independent organisation, our value-oriented actions are always based on ethical principles. Our vision is clear: "Zero Hunger by 2030"
@@ -2242,34 +2300,34 @@
 Individuals with no organizational entity</t>
         </is>
       </c>
-      <c r="D30" s="1" t="inlineStr">
+      <c r="D31" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E30" s="1" t="inlineStr">
+      <c r="E31" s="1" t="inlineStr">
         <is>
           <t>Jan 1, 2027</t>
         </is>
       </c>
-      <c r="F30" s="1" t="inlineStr">
+      <c r="F31" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-6th-annual-seeding-the-future-global-food-system-challenge-welthungerhilfe-opg-26-00180</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="95" customHeight="1">
-      <c r="A31" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B31" s="1" t="inlineStr">
+    <row r="32" ht="95" customHeight="1">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B32" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Microbiota &amp; Women's Health International Call for Projects</t>
         </is>
       </c>
-      <c r="C31" s="1" t="inlineStr">
+      <c r="C32" s="1" t="inlineStr">
         <is>
           <t>About the Grant
 An annual international research grant by the Biocodex Microbiota Foundation (BMF), rewarding research proposals on the microbiota and its implications in Women's Health and Disease. This year's theme: "Unraveling male-female genital microbiome interactions: mechanisms, transmission, and impact on vaginal dysbiosis."
@@ -2286,34 +2344,34 @@
 €200,000 annually — awarded to researchers within universities, hospitals, or other research settings to finance equipment, operations, or staffing costs. Grants are NOT awarded to individuals directly (must be institutionally affiliated). Institution's overhead costs capped at 10%.</t>
         </is>
       </c>
-      <c r="D31" s="1" t="inlineStr">
+      <c r="D32" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E31" s="1" t="inlineStr">
+      <c r="E32" s="1" t="inlineStr">
         <is>
           <t>Jan 15, 2027</t>
         </is>
       </c>
-      <c r="F31" s="1" t="inlineStr">
+      <c r="F32" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-microbiota-and-womens-health-international-call-for-projects-biocodex-microbiota-foundation-bmf-opg-26-00152</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="95" customHeight="1">
-      <c r="A32" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B32" s="1" t="inlineStr">
+    <row r="33" ht="95" customHeight="1">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B33" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for BES Training and Travel Grants</t>
         </is>
       </c>
-      <c r="C32" s="1" t="inlineStr">
+      <c r="C33" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are a global community of scientists shining a spotlight on the intricacy and value of our natural world, providing the evidence for better decisions. Our vision is for people and nature to thrive in a world that values ecology.
@@ -2352,17 +2410,17 @@
  Application Deadline (Round 2): Opens 30 April 2026, closes 17 May 2026</t>
         </is>
       </c>
-      <c r="D32" s="1" t="inlineStr">
+      <c r="D33" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E32" s="1" t="inlineStr">
+      <c r="E33" s="1" t="inlineStr">
         <is>
           <t>May 17, 2027</t>
         </is>
       </c>
-      <c r="F32" s="1" t="inlineStr">
+      <c r="F33" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-bes-training-and-travel-grants-british-ecological-society-opg-26-00181</t>
         </is>

</xml_diff>

<commit_message>
Auto update Combined.xlsx [Sat Sep 26 07:01:01 UTC 2026]
</commit_message>
<xml_diff>
--- a/output/Combined.xlsx
+++ b/output/Combined.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -462,15 +462,43 @@
     <row r="2" ht="95" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>onepurpos</t>
+          <t>ESTM</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
+          <t>District Coordination Associate</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>No description available</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr"/>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>10/10/2026, 03:59 AM</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>https://estm.fa.em2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1/job/37155/?location=India&amp;locationId=300000000440677&amp;locationLevel=country&amp;mode=location</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="95" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
           <t>ToR - Engagement of Information Design &amp; Video Production Agency / Consultant for Key Learning &amp; Dissemination Outputs</t>
         </is>
       </c>
-      <c r="C2" s="1" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Terms of Reference (TOR) for Consultancy Services
 Title  Engagement of Information Design &amp; Video Production Agency / Consultant for Key Learning &amp; Dissemination Outputs
@@ -489,34 +517,34 @@
 The primary objective of this engagement is to enable SELCO Foundation to effectively capture, structure, and communicate its field insights, sectoral learnings, and program impacts. The selected Agency/Consultant (or Agencies/Consultants) will work on a monthly retainer basis to translate raw content, data, field footage, and reports provided by SELCO into high-quality, visually compelling, reader-friendly visual outputs and video assets.</t>
         </is>
       </c>
-      <c r="D2" s="1" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E2" s="1" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Sep 28, 2026</t>
         </is>
       </c>
-      <c r="F2" s="1" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-engagement-of-information-design-and-video-production-agency-consultant-for-key-learning-and-dissemination-outputs-selco-foundation-rfp-26-00362</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="95" customHeight="1">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
+    <row r="4" ht="95" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>ToR - Video documentation of change stories on Ground water replenishment in Hyderabad and Sanga Reddy locations</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>About Jal Seva Charitable Foundation/ WaterAid India:
 Jal Seva Charitable Foundation (JSCF) is registered in India as a not-for-profit company under Chapter 8 of the Companies Act, 2013. JSCF, is an associate member of WaterAid International and uses the brand name ‘WaterAid’ in India.
@@ -550,34 +578,95 @@
 Upon completion of Assignment</t>
         </is>
       </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>Sep 28, 2026</t>
         </is>
       </c>
-      <c r="F3" s="1" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-video-documentation-of-change-stories-on-ground-water-replenishment-in-hyderabad-and-sanga-reddy-locations-wateraid-india-rfp-26-00363</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="95" customHeight="1">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
+    <row r="5" ht="95" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>ToR - Video Production Storytelling and Documentation</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>Title Video Production – Storytelling and Documentation
+Timeline 3 months from the date of contracting
+Expected area of expertise Video production, documentary storytelling, interviews, field documentation, cinematography and post-production
+Apply Link https://forms.gle/qiATVNrSkDJrkNH3A
+Last      Date             for Apply 29th September 2026 by 5 PM
+About SELCO Foundation:
+SELCO Foundation’s mission is to create a platform of solutions that uses sustainable energy as a catalyst to bridge environmental sustainability and poverty alleviation. With holistic development as the primary focus, the organization strives to create equitable societies, where services are accessed by all communities. The interventions of SELCO lead to a sustainable delivery model of essential services like livelihoods, education, and health till the last mile. (Read more about SELCO here: http://www.selcofoundation.org/)
+ About the Programmes:
+SELCO Foundation is looking to engage a video production partner to develop a series of compelling videos that document and communicate stories emerging from its programmes and field interventions.
+The assignment will involve end-to-end video production, including story development, filming, interviews, visual documentation, editing and post-production. The videos will highlight people, experiences, solutions, impact and the broader context of the organisation's work.
+The final content will be used across digital platforms, social media, events, presentations, reports and other communication channels
+ Objective:
+To produce a series of compelling videos that document programme experiences, end-user journeys and solutions in a clear, engaging and accessible manner.
+The videos should move beyond activity documentation to capture the context, challenge, solution, experience and outcomes of the people and communities being documented.
+The selected partner will be expected to provide:
+Story treatment/concept notes
+Interview questions and filming plan
+Raw footage from all filming
+Edited full-length video
+Edited short version
+30-second trailer
+Subtitled versions, where required
+Final master files in agreed resolution and formats
+Social-media-ready versions, where required
+Project/source files upon completion
+ Submission Requirements:
+Interested production partners are requested to submit the following by before deadline
+Organizational/Individual Profile: Overview of your team/experience.Proposed Approach: A brief document outlining your understanding of the assignment and your proposed approach to storytelling and production.
+Relevant Portfolio: 3–5 relevant video samples demonstrating documentary, impact, social-sector, development or human-interest storytelling.Experience with Similar Assignments: Details of relevant video production and field documentation work.
+Quotation Should include all cost including Travel and Miscellaneous.</t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>Sep 29, 2026</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/tor-video-production-storytelling-and-documentation-selco-foundation-rfp-26-00368</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="95" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>RFP - Engagement of Agency for Development of MIS Dashboard and Mobile-based Application for Adolescent Mental Health</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>Release of Request for Proposal
 23rd September 2026
@@ -644,147 +733,19 @@
 It is to be submitted separately as per Annexure II. No conditional price is to be quoted.</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>Sep 29, 2026</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="F6" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfp-engagement-of-agency-for-development-of-mis-dashboard-and-mobile-based-application-for-adolescent-mental-health-american-india-foundation-rfp-26-00372</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="95" customHeight="1">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>ToR - Video Production Storytelling and Documentation</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="inlineStr">
-        <is>
-          <t>Title Video Production – Storytelling and Documentation
-Timeline 3 months from the date of contracting
-Expected area of expertise Video production, documentary storytelling, interviews, field documentation, cinematography and post-production
-Apply Link https://forms.gle/qiATVNrSkDJrkNH3A
-Last      Date             for Apply 29th September 2026 by 5 PM
-About SELCO Foundation:
-SELCO Foundation’s mission is to create a platform of solutions that uses sustainable energy as a catalyst to bridge environmental sustainability and poverty alleviation. With holistic development as the primary focus, the organization strives to create equitable societies, where services are accessed by all communities. The interventions of SELCO lead to a sustainable delivery model of essential services like livelihoods, education, and health till the last mile. (Read more about SELCO here: http://www.selcofoundation.org/)
- About the Programmes:
-SELCO Foundation is looking to engage a video production partner to develop a series of compelling videos that document and communicate stories emerging from its programmes and field interventions.
-The assignment will involve end-to-end video production, including story development, filming, interviews, visual documentation, editing and post-production. The videos will highlight people, experiences, solutions, impact and the broader context of the organisation's work.
-The final content will be used across digital platforms, social media, events, presentations, reports and other communication channels
- Objective:
-To produce a series of compelling videos that document programme experiences, end-user journeys and solutions in a clear, engaging and accessible manner.
-The videos should move beyond activity documentation to capture the context, challenge, solution, experience and outcomes of the people and communities being documented.
-The selected partner will be expected to provide:
-Story treatment/concept notes
-Interview questions and filming plan
-Raw footage from all filming
-Edited full-length video
-Edited short version
-30-second trailer
-Subtitled versions, where required
-Final master files in agreed resolution and formats
-Social-media-ready versions, where required
-Project/source files upon completion
- Submission Requirements:
-Interested production partners are requested to submit the following by before deadline
-Organizational/Individual Profile: Overview of your team/experience.Proposed Approach: A brief document outlining your understanding of the assignment and your proposed approach to storytelling and production.
-Relevant Portfolio: 3–5 relevant video samples demonstrating documentary, impact, social-sector, development or human-interest storytelling.Experience with Similar Assignments: Details of relevant video production and field documentation work.
-Quotation Should include all cost including Travel and Miscellaneous.</t>
-        </is>
-      </c>
-      <c r="D5" s="1" t="inlineStr">
-        <is>
-          <t>Learning</t>
-        </is>
-      </c>
-      <c r="E5" s="1" t="inlineStr">
-        <is>
-          <t>Sep 29, 2026</t>
-        </is>
-      </c>
-      <c r="F5" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/tor-video-production-storytelling-and-documentation-selco-foundation-rfp-26-00368</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="95" customHeight="1">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>EOI Inviting Expression of Interest-cum-Proposal for Setting Up District De-Addiction Centres under NAPDDR</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="inlineStr">
-        <is>
-          <t>About us
-In the year 1985-86, the erstwhile Ministry of Welfare was bifurcated into the Department of Women and Child Development and the Department of Welfare. Simultaneously, the Scheduled Castes Development Division, Tribal Development Division and the Minorities and Backward Classes Welfare Division were moved from the Ministry of Home Affairs and also the Wakf Division from the Ministry of Law to form the then Ministry of Welfare Subsequently, the name of the Ministry was changed to the Ministry of Social Justice &amp; Empowerment in May, 1998. Further, in October, 1999, the Tribal Development Division had moved out to form a separate Ministry of Tribal Affairs. In January, 2007, the Minorities Division along with Wakf Unit have been moved out of the Ministry and formed as a separate Ministry and the Child Development Division has gone to the Ministry of Women &amp; Child Development.
- Department of Social Justice and Empowerment invites Expression of lnterest-cum-proposal from the eligible organizations for setting up of District DeAddiction Centres under the scheme of National Action Plan for Drug Demand Reduction (NAPDDR) for 315 GAP Districts of the country (as per list attached at Annexure - l). The list of districts is subject to change (addition or deletion) time to trme by the Ministry as per requirement or need on the ground.
- 2. Eligible NGOs may apply for setting up of DDAC provided that they have rent free accommodation for setting up of DDAC as per the standards of guideline of the NAPDDR scheme or renlfree accommodation may also be provided by the concerned District Administration. 
- 3. Setting up and running of District De-Addiction Centres (DDACS) will be done as per the following guidelinesr. 
- i. There will be a District De-Addiction Centre (DDAC) preferably in each district headquarter or suitably accessible place where rent free accommodation is provided by the district administration. These DDACs would provide comprehensive facilities hitherto being provided by IRCA, ODIC &amp; CPLI together. lf the district administration of identified district is not able to provide suitable rent free accommodation, then the application will be called from the eligible VOs/ NGOs, who will provide rent free accommodation for setting up of DDAC in that district.
- ii. The functioning of DDAC will be monitored by the three tier Committees headed by the Chief Secretary, District Collector/Deputy Commissioner and Block Development Officer of the respective arealregion which have been formed under Nasha Mukt Bharat Abhiyaan (NMBA). Additionally, retired eminent personalities of the Districts, activists, Vice-Chancellor/ Head of Department (HoD)/ Principal, researcher, scholars and so on may be co-opted by Chairman as the members of the Committees. These commiftees would
- only monitor policy related issues. Day to day and other activities relating to implementation would be the responsibility of the concerned organization/NGO approved for setting up of the DDAC. The Meetings of DDAC are to be held as per the details given below:
- (a) State-level Steering and Monitoring Committee (High Level Task Force) - headed by Chief Secretary - to meet quarterly. (b) District-level Committee - headed by District Collector / Deputy Commissioner - to meet monthly and have mandatory inspections quarterly. (c) Block level Committee - headed by Block Development Officer - to meet &amp; have mandatory inspections monthly.
- The Committees will also review the functioning and assess the performance of the DDAC in terms of the effectiveness of deliverables and make further suggestions to the management of DDAC. 
- IIl t. A separate (dedicated) account will be opened for keeping funds of DDAC in the name of NGO/Organization. The account will be registered on PFMS and implemented through EAT Module. 
- lV. For setting up of DDACs, preference would be given to those Districts, which do not have any facility of IRCA or DDAC. For this, the organization willing to work in the field of DRUGS DE-ADDICTION TREATMENT will be eligible for applying for DDAC. The priority for selection of DDAC would be: 
-a. The DDAC proposed to be run by the District administration itself. 
-b. Rent free accommodation in the district headquarter provided by the concerned DC/DM &amp; further willingness from interested NGO is sought. c, Where no proposal for rent-free accommodation is received from concerned DCiDM, interested NGO may directly apply for DDAC provided they do not seek any rent for same and only building maintenance will be given. 
-V. The details of Minimum standards like physical space and necessary amenities to be provided by District administration or NGOs are as under: 
-(a) The centre should be easily accessible and connected through public transport. 
-(b) The total built-in area of the DDAC should be at least 3000 sq,ft. in case of metros and 4000 sq.ft. in case of small towns and villages to house 15 patients and 4000 sq.ft. in case of metros and 5000 sq.ft. in case of small towns and villages to house 30 patients. This includes an area of about 2000 sq. ft. for Treatment cum Rehabilitation centre, an area of about 700 sq. ft. for Drop-ln Centre facilities and an area of about 300 sq. ft. for CPLI Centre facilities. 
-(c) The centre should be properly ventilated, well-lit and maintained in a clean manner. Water to be made available. 
-(d) Basic safety of the patients to be ensured 
-(e) Facilities at the centre - Waiting space with seating arrangements for a minimum 5 persons Cubicles / rooms for consultation for physical examination Facilities to store drugs, linen, and records of patients Facilities with privacy for providing individual counselling, group therapy, re-educative sessions, family classes. They should be airy with comfortable seating with floor mats / chairs. Blackboard, chalk and other material to be provided. Availability of recreational facilities. Separate Drop ln Facility centre with recreation room, counselling room and medical room. Project room for CPLI activities including consultation room for interviewing Vl. Standards set in the above para of the guidelines may change from time to time as and when necessary with the approval of competent authority and the stakeholders / NGOs/ VOs would be intimated of same as and when such changes happen. 
- 4. The interested and eligible NGOs / organizations can apply through eAnudaan (https://grants-msje.gov.in/ngo-login) portal of the Ministry. The Project Screening Committee in the Ministry will select the eligible NGO(s) for establishing and running of the DDAC and recommend the release of funds in two installments. However, the organization shall be eligible for receiving GIA under the scheme from the date of approval of the competent authority. 
- 5. ELIGIBLE ORGANIZATION: 
-Organizations which are already running MoSJE supported IRCA or State Government supported De-addiction Centre/ Government Hospital or any private run De-Addiction centre are eligible for applying for DDAC. Organization can apply only for that State/UT in which they are already running IRCA"/De-addiction Centre from the last 2 years or more from the date of call for the proposal. Condition may be relaxed for any Government run Hospitals, which are non-profitable in nature. I 
-6. Start-up consists of young persons/ professionals, who have graduated from top social institutes of lndia or abroad are also eligible to apply. However, they must have experience of 2 years in the field of Drug De-addiction TREATMENT. 7. Role and Responsibility of DDACs The main focus of the DDAC is early prevention, education, demand reduction, identification, treatment and rehabilitation services of vulnerable individuals or individuals affected by substance use disorders DDAC would: 
-a. Conduct primary prevention activities through awareness programs among the vulnerable and affected community 
-b. Engage in risk mitigation of substance use among children/ adolescenuyouth by: Preventing substance use Delaying initiation of substance use 
-c. ldentify and train selected peer educators in the community 
-d. lmplement early prevention education through life skill training led by trained peer educators 
-e. Provide awareness about referral and linkage to counseling, treatment and rehabilitation services for substance dependent adolescents identified in the community 
-f. ldentifying adolescents and other individuals subjected to substance use and facilitating their referrali admission into Rehabilitation Centers/ Drop ln Centres. 
-g. Provide a whole range of services which includes treatment, after care and rehabilitation including skill development for Whole Person Recovery (WPR) of dependents; 
-h. Undertake drug demand reduction efforts to address all forms of illicit use of any substances and ensure overall well being of humankind; 
-i. Alleviate the consequences of substance dependence amongst individuals, family and society at large 
-9. The budget details of DDAC is attached as Annexure - 
-10. The e-anudaan portal shall remain open through out the year and the recommendations from the States/UTs will be considered periodically. 
-11. Department of Social Justice and Empowerment (DoSJE) reserves the right to cancel this notice, andior invite afresh proposals with or without amendments to this document without liability or any obligation for such document, and without assigning any reason. DoSJE reserves the right to take final decision regarding selection of implementing agency or project.</t>
-        </is>
-      </c>
-      <c r="D6" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E6" s="1" t="inlineStr">
-        <is>
-          <t>Sep 30, 2026</t>
-        </is>
-      </c>
-      <c r="F6" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/eoi-inviting-expression-of-interest-cum-proposal-for-setting-up-district-de-addiction-centres-under-napddr-ministry-of-social-justice-and-empowerment-goi-rfp-26-00356</t>
         </is>
       </c>
     </row>
@@ -994,10 +955,77 @@
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
+          <t>EOI Inviting Expression of Interest-cum-Proposal for Setting Up District De-Addiction Centres under NAPDDR</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>About us
+In the year 1985-86, the erstwhile Ministry of Welfare was bifurcated into the Department of Women and Child Development and the Department of Welfare. Simultaneously, the Scheduled Castes Development Division, Tribal Development Division and the Minorities and Backward Classes Welfare Division were moved from the Ministry of Home Affairs and also the Wakf Division from the Ministry of Law to form the then Ministry of Welfare Subsequently, the name of the Ministry was changed to the Ministry of Social Justice &amp; Empowerment in May, 1998. Further, in October, 1999, the Tribal Development Division had moved out to form a separate Ministry of Tribal Affairs. In January, 2007, the Minorities Division along with Wakf Unit have been moved out of the Ministry and formed as a separate Ministry and the Child Development Division has gone to the Ministry of Women &amp; Child Development.
+ Department of Social Justice and Empowerment invites Expression of lnterest-cum-proposal from the eligible organizations for setting up of District DeAddiction Centres under the scheme of National Action Plan for Drug Demand Reduction (NAPDDR) for 315 GAP Districts of the country (as per list attached at Annexure - l). The list of districts is subject to change (addition or deletion) time to trme by the Ministry as per requirement or need on the ground.
+ 2. Eligible NGOs may apply for setting up of DDAC provided that they have rent free accommodation for setting up of DDAC as per the standards of guideline of the NAPDDR scheme or renlfree accommodation may also be provided by the concerned District Administration. 
+ 3. Setting up and running of District De-Addiction Centres (DDACS) will be done as per the following guidelinesr. 
+ i. There will be a District De-Addiction Centre (DDAC) preferably in each district headquarter or suitably accessible place where rent free accommodation is provided by the district administration. These DDACs would provide comprehensive facilities hitherto being provided by IRCA, ODIC &amp; CPLI together. lf the district administration of identified district is not able to provide suitable rent free accommodation, then the application will be called from the eligible VOs/ NGOs, who will provide rent free accommodation for setting up of DDAC in that district.
+ ii. The functioning of DDAC will be monitored by the three tier Committees headed by the Chief Secretary, District Collector/Deputy Commissioner and Block Development Officer of the respective arealregion which have been formed under Nasha Mukt Bharat Abhiyaan (NMBA). Additionally, retired eminent personalities of the Districts, activists, Vice-Chancellor/ Head of Department (HoD)/ Principal, researcher, scholars and so on may be co-opted by Chairman as the members of the Committees. These commiftees would
+ only monitor policy related issues. Day to day and other activities relating to implementation would be the responsibility of the concerned organization/NGO approved for setting up of the DDAC. The Meetings of DDAC are to be held as per the details given below:
+ (a) State-level Steering and Monitoring Committee (High Level Task Force) - headed by Chief Secretary - to meet quarterly. (b) District-level Committee - headed by District Collector / Deputy Commissioner - to meet monthly and have mandatory inspections quarterly. (c) Block level Committee - headed by Block Development Officer - to meet &amp; have mandatory inspections monthly.
+ The Committees will also review the functioning and assess the performance of the DDAC in terms of the effectiveness of deliverables and make further suggestions to the management of DDAC. 
+ IIl t. A separate (dedicated) account will be opened for keeping funds of DDAC in the name of NGO/Organization. The account will be registered on PFMS and implemented through EAT Module. 
+ lV. For setting up of DDACs, preference would be given to those Districts, which do not have any facility of IRCA or DDAC. For this, the organization willing to work in the field of DRUGS DE-ADDICTION TREATMENT will be eligible for applying for DDAC. The priority for selection of DDAC would be: 
+a. The DDAC proposed to be run by the District administration itself. 
+b. Rent free accommodation in the district headquarter provided by the concerned DC/DM &amp; further willingness from interested NGO is sought. c, Where no proposal for rent-free accommodation is received from concerned DCiDM, interested NGO may directly apply for DDAC provided they do not seek any rent for same and only building maintenance will be given. 
+V. The details of Minimum standards like physical space and necessary amenities to be provided by District administration or NGOs are as under: 
+(a) The centre should be easily accessible and connected through public transport. 
+(b) The total built-in area of the DDAC should be at least 3000 sq,ft. in case of metros and 4000 sq.ft. in case of small towns and villages to house 15 patients and 4000 sq.ft. in case of metros and 5000 sq.ft. in case of small towns and villages to house 30 patients. This includes an area of about 2000 sq. ft. for Treatment cum Rehabilitation centre, an area of about 700 sq. ft. for Drop-ln Centre facilities and an area of about 300 sq. ft. for CPLI Centre facilities. 
+(c) The centre should be properly ventilated, well-lit and maintained in a clean manner. Water to be made available. 
+(d) Basic safety of the patients to be ensured 
+(e) Facilities at the centre - Waiting space with seating arrangements for a minimum 5 persons Cubicles / rooms for consultation for physical examination Facilities to store drugs, linen, and records of patients Facilities with privacy for providing individual counselling, group therapy, re-educative sessions, family classes. They should be airy with comfortable seating with floor mats / chairs. Blackboard, chalk and other material to be provided. Availability of recreational facilities. Separate Drop ln Facility centre with recreation room, counselling room and medical room. Project room for CPLI activities including consultation room for interviewing Vl. Standards set in the above para of the guidelines may change from time to time as and when necessary with the approval of competent authority and the stakeholders / NGOs/ VOs would be intimated of same as and when such changes happen. 
+ 4. The interested and eligible NGOs / organizations can apply through eAnudaan (https://grants-msje.gov.in/ngo-login) portal of the Ministry. The Project Screening Committee in the Ministry will select the eligible NGO(s) for establishing and running of the DDAC and recommend the release of funds in two installments. However, the organization shall be eligible for receiving GIA under the scheme from the date of approval of the competent authority. 
+ 5. ELIGIBLE ORGANIZATION: 
+Organizations which are already running MoSJE supported IRCA or State Government supported De-addiction Centre/ Government Hospital or any private run De-Addiction centre are eligible for applying for DDAC. Organization can apply only for that State/UT in which they are already running IRCA"/De-addiction Centre from the last 2 years or more from the date of call for the proposal. Condition may be relaxed for any Government run Hospitals, which are non-profitable in nature. I 
+6. Start-up consists of young persons/ professionals, who have graduated from top social institutes of lndia or abroad are also eligible to apply. However, they must have experience of 2 years in the field of Drug De-addiction TREATMENT. 7. Role and Responsibility of DDACs The main focus of the DDAC is early prevention, education, demand reduction, identification, treatment and rehabilitation services of vulnerable individuals or individuals affected by substance use disorders DDAC would: 
+a. Conduct primary prevention activities through awareness programs among the vulnerable and affected community 
+b. Engage in risk mitigation of substance use among children/ adolescenuyouth by: Preventing substance use Delaying initiation of substance use 
+c. ldentify and train selected peer educators in the community 
+d. lmplement early prevention education through life skill training led by trained peer educators 
+e. Provide awareness about referral and linkage to counseling, treatment and rehabilitation services for substance dependent adolescents identified in the community 
+f. ldentifying adolescents and other individuals subjected to substance use and facilitating their referrali admission into Rehabilitation Centers/ Drop ln Centres. 
+g. Provide a whole range of services which includes treatment, after care and rehabilitation including skill development for Whole Person Recovery (WPR) of dependents; 
+h. Undertake drug demand reduction efforts to address all forms of illicit use of any substances and ensure overall well being of humankind; 
+i. Alleviate the consequences of substance dependence amongst individuals, family and society at large 
+9. The budget details of DDAC is attached as Annexure - 
+10. The e-anudaan portal shall remain open through out the year and the recommendations from the States/UTs will be considered periodically. 
+11. Department of Social Justice and Empowerment (DoSJE) reserves the right to cancel this notice, andior invite afresh proposals with or without amendments to this document without liability or any obligation for such document, and without assigning any reason. DoSJE reserves the right to take final decision regarding selection of implementing agency or project.</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>Sep 30, 2026</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/eoi-inviting-expression-of-interest-cum-proposal-for-setting-up-district-de-addiction-centres-under-napddr-ministry-of-social-justice-and-empowerment-goi-rfp-26-00356</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="95" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
           <t>Application Invited for Giving Joy Microgrant</t>
         </is>
       </c>
-      <c r="C10" s="1" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Giving Joy is a US-based nonprofit that strengthens and inspires women’s entrepreneurship worldwide. Through its micro-grants and mentorship program, Giving Joy helps women establish or improve their businesses and initiatives—for their benefit and the benefit of their communities. To date, Giving Joy has awarded over 88 grants to women-led initiatives in 26 countries.
@@ -1036,34 +1064,102 @@
 The grant period is six months.</t>
         </is>
       </c>
-      <c r="D10" s="1" t="inlineStr">
+      <c r="D11" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E10" s="1" t="inlineStr">
+      <c r="E11" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F10" s="1" t="inlineStr">
+      <c r="F11" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/application-invited-for-giving-joy-microgrant-giving-joy-opg-26-00185</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="95" customHeight="1">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="inlineStr">
+    <row r="12" ht="95" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>ToR - Project Management Unit Solarization of Women-led Livelihoods in Maharashtra MAVIMSELCO Foundation Short Duration Project</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>Title Project Management Unit – Solarization of Women-led Livelihoods in Maharashtra (MAVIM–SELCO Foundation Short Duration Project)
+Timeline 6 Months (Oct – Mar)
+Expected area of expertise Enterprise profiling &amp; energy assessment, field mobilization &amp; outreach, due diligence, stakeholder coordination, installation facilitation and site validation
+Geographical Scope 5–6 districts of Maharashtra (to be finalized in consultation with MAVIM)
+Apply Link https://forms.gle/ntigMBJ8PDzNPSJ58 
+Last Date for Apply 03rd October 2026 by 5 pm. 
+About SELCO Foundation:
+SELCO Foundation is an open-source, not-for-profit organization that engages in field-based R&amp;D and ecosystem building for the deployment of clean energy solutions that alleviate poverty by improving access to sustainable energy to underserved communities in tribal, rural, and urban poor areas. The organization works in collaboration with practitioners in the social sector, energy entrepreneurs, NGOs from various developmental sectors, and educational institutions to link the benefits of sustainable energy to poverty eradication. The organization works across verticals such as energy access, health, and livelihoods. You can find more information about the SELCO Foundation on our website: http://www.selcofoundation.org/
+ Summary of the Project:
+While access to decentralized renewable energy (DRE) can help nano/micro-entrepreneurs upscale, improve productivity, and increase income, its adoption remains sub-optimal due to limited awareness, lack of access to a supportive ecosystem, and high initial capital requirements.
+ SELCO Foundation is working with the Maharashtra Mahila Aarthik Vikas Mahamandal (MAVIM) to co-design a short duration project aimed at solarizing the livelihoods of 1000 women nano/micro-entrepreneurs. These women, drawn from the network of Self-Help Groups (SHGs) supported by MAVIM, work in the streams of food processing, value-added food products, and non-food manufacturing through home-based or dedicated facility-based setups. Eligible entrepreneurs will be supported under this initiative through the installation of off-grid solar systems, across 5–6 districts of Maharashtra to be selected in consultation with MAVIM, over a 6-month duration.
+A consultant (individual or organization) working as a Project Management Unit (PMU) is being onboarded by SELCO Foundation to lead field-level implementation of the project — from enterprise profiling and energy assessment, through mobilization, due diligence and shortlisting, to installation coordination and site validation.
+ Goals and Objectives:
+The engagement's key objectives are:
+Facilitate the solarization of 1000 women-led nano/micro-enterprises drawn from MAVIM's SHG network, across 5–6 districts of Maharashtra.
+Assess energy requirements for enterprises based on their occupational profile.
+Mobilize and engage entrepreneurs from the longlist shared by MAVIM, and build a verified shortlist of eligible, willing participants through due diligence and documentation.
+Coordinate closely with MAVIM's district and sub-district cadre to ensure proper engagement and participation of women entrepreneurs throughout the project.
+Facilitate timely, quality installation of solar systems in coordination with the technology vendor and validate proper installation at each site.
+ Requirements
+Agency/Individual should have experience in or capacity for:
+Project management and field-level implementation, specifically in livelihood and enterprise support.
+Field-based enterprise profiling, ideally within micro-enterprise/livelihood contexts (food processing, non-food manufacturing, or similar).
+Community mobilization and outreach, including working with women's Self-Help Group (SHG) networks.
+Conducting due diligence and basic documentation of prospective beneficiaries.
+Coordinating with government/semi-government bodies (such as MAVIM) at district and sub-district levels.
+Coordinating with technology vendors for timely and quality installation and validating site-level installation.
+Monitoring and documentation, including maintaining trackers and status reports.
+Excellent written and verbal communication skills, especially for field- and stakeholder-level coordination.
+The PMU (agency/individual) will need to be based in or have a strong field presence across Maharashtra throughout the duration of the engagement.
+ Submission Requirements
+Interested agencies/consultants are requested to submit:
+A detailed proposal outlining approach, methodology, and timelines for each phase of the scope of work.
+Team composition, roles, and CVs with relevant experience.
+Organizational profile.
+A financial quote with a breakdown of costs, split by phase/deliverable wherever possible.
+Examples of similar past projects, particularly involving SHG networks, livelihood programs, or energy access.</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>Oct 3, 2026</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/tor-project-management-unit-solarization-of-women-led-livelihoods-in-maharashtra-mavimselco-foundation-short-duration-project-selco-foundation-rfp-26-00374</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="95" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
         <is>
           <t>EOI - Engagement of Agencies for HR Recruitment Services</t>
         </is>
       </c>
-      <c r="C11" s="1" t="inlineStr">
+      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>The American India Foundation Trust (AIFT) seeks to engage an experienced recruitment agency to provide end-to-end recruitment and talent acquisition services for identified positions across its offices, programmes, and functions in India.
 The selected agency shall support AIFT in sourcing, screening, shortlisting, interview coordination, candidate engagement, offer management, and recruitment closure, in accordance with the requirements, timelines, and service levels agreed with AIFT.
@@ -1094,95 +1190,34 @@
 Any other information specifically requested by AIFT.</t>
         </is>
       </c>
-      <c r="D11" s="1" t="inlineStr">
+      <c r="D13" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E11" s="1" t="inlineStr">
+      <c r="E13" s="1" t="inlineStr">
         <is>
           <t>Oct 4, 2026</t>
         </is>
       </c>
-      <c r="F11" s="1" t="inlineStr">
+      <c r="F13" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/eoi-engagement-of-agencies-for-hr-recruitment-services-american-india-foundation-rfp-26-00375</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="95" customHeight="1">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="inlineStr">
-        <is>
-          <t>ToR for Onboarding of consultant/agency for Innovating &amp; Scaling Reproductive Maternal Newborn and Child Health Solutions in the Last-Mile</t>
-        </is>
-      </c>
-      <c r="C12" s="1" t="inlineStr">
-        <is>
-          <t>Title Terms of Reference for Onboarding of consultant/agency for Innovating &amp; Scaling Reproductive, Maternal, Newborn and Child Health Solutions in the Last-Mile
-Timeline September 2026 to February 2027
-Scope of Work
-• Outreach and program visibility
-• Application design, launch, review, shortlisting, and due diligence
-• Stakeholder engagement and coordination
-• Knowledge materials and document learnings and insights
-Application Link https://forms.gle/jsngbAREkYmgK7cB6
-Last Date to Apply 5th October, 5 PM
-About SELCO Foundation:
-SELCO Foundation's mission is to create a platform of solutions that uses sustainable energy as a catalyst to bridge environmental sustainability and poverty alleviation. With holistic development as the primary focus, the organization strives to create equitable societies, where services are accessed by all communities. The interventions of SELCO lead to a sustainable delivery model of essential services like livelihoods, education, and health till the last mile.
-(Read more about SELCO here: https://selcofoundation.org/)
- About the Program
-The program aims to catalyse the development, adoption, and scale of innovative solutions that contribute to improved maternal and child health outcomes. It seeks to build an ecosystem where enterprises and innovators can develop and strengthen technology and technology-allied solutions that enable more accessible, quality, efficient, affordable, and continuous maternal and child health services, particularly across last-mile health facilities and underserved communities.
-The program envisions a future where innovation, technology, and enterprise-led solutions are meaningfully integrated into maternal and child health delivery, enabling health systems, facilities, and frontline health workers to deliver better services to women and children.
-The initiative will bring together enterprises, innovators, health facilities, frontline health workers, institutions, and other ecosystem stakeholders to co-create, test, deploy, and scale solutions with the potential to transform maternal and child health delivery. The focus will be on enabling promising solutions to move beyond individual deployments towards sustainable models of adoption, replication, and scale.
-For the same, we are looking to partner with a like-minded organization that shares this vision and can play an integral role in designing and implementing the initiative. The partner will support enterprise identification and engagement, solution assessment, co-creation, health-system linkages, implementation, stakeholder coordination, evidence generation, and pathways to scale, contributing to more resilient, responsive, and equitable maternal and child health services for women and children.
- Geography
-Primary Focus: Maharashtra, Karnataka, Odisha, Meghalaya, Mizoram, Nagaland
-Secondary Focus: Other states
- Selection Criteria
-Applicants should meet the following criteria for being a part of the evaluation:
-Demonstrated experience working with vendors, enterprises, innovators, or solution providers, along with an understanding of grassroots and last-mile contexts and user needs
-Ability to assess enterprise and solution needs and curate tailored mentorship, technical assistance, health-system linkages, and implementation support
-Demonstrated experience in program design, planning, implementation, and management of multi-stakeholder initiatives, preferably in health, maternal and child health, technology, or last-mile service delivery
-Proven ability to manage end-to-end application, assessment, screening, shortlisting, and due diligence processes for a portfolio of enterprises or innovators
-Experience in communication, outreach, stakeholder engagement, and facilitating collaboration between solution providers and health-system stakeholders
-Capability to develop documentation and knowledge products that capture program processes, solution performance, outcomes, implementation models, and learnings for scale and replication
-Prior experience working with development sector organisations, NGOs, health systems, technology providers, enterprises, or think tanks will be considered an added advantage
-The agency will be selected on a combined technical and financial evaluation. Proposals must score a minimum of 70% on the technical components (1–5 below) to be considered for financial evaluation.</t>
-        </is>
-      </c>
-      <c r="D12" s="1" t="inlineStr">
-        <is>
-          <t>Learning</t>
-        </is>
-      </c>
-      <c r="E12" s="1" t="inlineStr">
-        <is>
-          <t>Oct 5, 2026</t>
-        </is>
-      </c>
-      <c r="F12" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/tor-for-onboarding-of-consultantagency-for-innovating-and-scaling-reproductive-maternal-newborn-and-child-health-solutions-in-the-last-mile-selco-foundation-rfp-26-00373</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="95" customHeight="1">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B13" s="1" t="inlineStr">
+    <row r="14" ht="95" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>RFP - Design and Delivery of an Electric Vehicle EV Skilling Programme in Karnataka</t>
         </is>
       </c>
-      <c r="C13" s="1" t="inlineStr">
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 WRI India, an independent knowledge organisation registered as the India Resources Trust, provides objective information and practical proposals to foster environmentally sound and socially equitable development. As an independent knowledge organisation, we leverage our data and expertise to catalyze change across systems like food, land and water; energy; and cities. Our work focuses on improving people’s lives, protecting and restoring nature, and addressing climate change. To enable progress at the pace and scale needed, we also engage with the economic, finance and governance systems that are key to enabling this change.
@@ -1223,34 +1258,95 @@
 Must have a team of qualified trainers and master trainers with relevant domain expertise, as well as administrative and coordination support.</t>
         </is>
       </c>
-      <c r="D13" s="1" t="inlineStr">
+      <c r="D14" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E13" s="1" t="inlineStr">
+      <c r="E14" s="1" t="inlineStr">
         <is>
           <t>Oct 5, 2026</t>
         </is>
       </c>
-      <c r="F13" s="1" t="inlineStr">
+      <c r="F14" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfp-design-and-delivery-of-an-electric-vehicle-ev-skilling-programme-in-karnataka-wri-india-rfp-26-00361</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="95" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="inlineStr">
+    <row r="15" ht="95" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>ToR for Onboarding of consultant/agency for Innovating &amp; Scaling Reproductive Maternal Newborn and Child Health Solutions in the Last-Mile</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>Title Terms of Reference for Onboarding of consultant/agency for Innovating &amp; Scaling Reproductive, Maternal, Newborn and Child Health Solutions in the Last-Mile
+Timeline September 2026 to February 2027
+Scope of Work
+• Outreach and program visibility
+• Application design, launch, review, shortlisting, and due diligence
+• Stakeholder engagement and coordination
+• Knowledge materials and document learnings and insights
+Application Link https://forms.gle/jsngbAREkYmgK7cB6
+Last Date to Apply 5th October, 5 PM
+About SELCO Foundation:
+SELCO Foundation's mission is to create a platform of solutions that uses sustainable energy as a catalyst to bridge environmental sustainability and poverty alleviation. With holistic development as the primary focus, the organization strives to create equitable societies, where services are accessed by all communities. The interventions of SELCO lead to a sustainable delivery model of essential services like livelihoods, education, and health till the last mile.
+(Read more about SELCO here: https://selcofoundation.org/)
+ About the Program
+The program aims to catalyse the development, adoption, and scale of innovative solutions that contribute to improved maternal and child health outcomes. It seeks to build an ecosystem where enterprises and innovators can develop and strengthen technology and technology-allied solutions that enable more accessible, quality, efficient, affordable, and continuous maternal and child health services, particularly across last-mile health facilities and underserved communities.
+The program envisions a future where innovation, technology, and enterprise-led solutions are meaningfully integrated into maternal and child health delivery, enabling health systems, facilities, and frontline health workers to deliver better services to women and children.
+The initiative will bring together enterprises, innovators, health facilities, frontline health workers, institutions, and other ecosystem stakeholders to co-create, test, deploy, and scale solutions with the potential to transform maternal and child health delivery. The focus will be on enabling promising solutions to move beyond individual deployments towards sustainable models of adoption, replication, and scale.
+For the same, we are looking to partner with a like-minded organization that shares this vision and can play an integral role in designing and implementing the initiative. The partner will support enterprise identification and engagement, solution assessment, co-creation, health-system linkages, implementation, stakeholder coordination, evidence generation, and pathways to scale, contributing to more resilient, responsive, and equitable maternal and child health services for women and children.
+ Geography
+Primary Focus: Maharashtra, Karnataka, Odisha, Meghalaya, Mizoram, Nagaland
+Secondary Focus: Other states
+ Selection Criteria
+Applicants should meet the following criteria for being a part of the evaluation:
+Demonstrated experience working with vendors, enterprises, innovators, or solution providers, along with an understanding of grassroots and last-mile contexts and user needs
+Ability to assess enterprise and solution needs and curate tailored mentorship, technical assistance, health-system linkages, and implementation support
+Demonstrated experience in program design, planning, implementation, and management of multi-stakeholder initiatives, preferably in health, maternal and child health, technology, or last-mile service delivery
+Proven ability to manage end-to-end application, assessment, screening, shortlisting, and due diligence processes for a portfolio of enterprises or innovators
+Experience in communication, outreach, stakeholder engagement, and facilitating collaboration between solution providers and health-system stakeholders
+Capability to develop documentation and knowledge products that capture program processes, solution performance, outcomes, implementation models, and learnings for scale and replication
+Prior experience working with development sector organisations, NGOs, health systems, technology providers, enterprises, or think tanks will be considered an added advantage
+The agency will be selected on a combined technical and financial evaluation. Proposals must score a minimum of 70% on the technical components (1–5 below) to be considered for financial evaluation.</t>
+        </is>
+      </c>
+      <c r="D15" s="1" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E15" s="1" t="inlineStr">
+        <is>
+          <t>Oct 5, 2026</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/tor-for-onboarding-of-consultantagency-for-innovating-and-scaling-reproductive-maternal-newborn-and-child-health-solutions-in-the-last-mile-selco-foundation-rfp-26-00373</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="95" customHeight="1">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>RFPs Invited for Engagement of a Manpower Agency for Providing Subject Matter Specialists/Experts for the Cluster Development Programme</t>
         </is>
       </c>
-      <c r="C14" s="1" t="inlineStr">
+      <c r="C16" s="1" t="inlineStr">
         <is>
           <t>About the RFP
 National Horticulture Board (NHB), an autonomous organization under the Ministry of Agriculture and Farmers' Welfare, Government of India, invites bids from eligible manpower agencies for engagement to recruit, deploy, and manage qualified personnel supporting NHB's Cluster Development Programme (CDP) — a Central Sector Scheme promoting integrated, market-led horticulture cluster development. The engaged agency will provide three types of Subject Matter Experts per Cluster and additional consultants/manpower as required by NHB from time to time.
@@ -1276,34 +1372,34 @@
  District: Gurugram, Haryana (NHB Head Office)</t>
         </is>
       </c>
-      <c r="D14" s="1" t="inlineStr">
+      <c r="D16" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E14" s="1" t="inlineStr">
+      <c r="E16" s="1" t="inlineStr">
         <is>
           <t>Oct 6, 2026</t>
         </is>
       </c>
-      <c r="F14" s="1" t="inlineStr">
+      <c r="F16" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfps-invited-for-engagement-of-a-manpower-agency-for-providing-subject-matter-specialistsexperts-for-the-cluster-development-programme-national-horticulture-board-nhb-rfp-26-00370</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="95" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="inlineStr">
+    <row r="17" ht="95" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
         <is>
           <t>Applications Open Draper Richards Kaplan Foundation Funding for Social Enterprises</t>
         </is>
       </c>
-      <c r="C15" s="1" t="inlineStr">
+      <c r="C17" s="1" t="inlineStr">
         <is>
           <t>About us
 Started in 2002, Draper Richards Kaplan Foundation (DRK) is a global venture philanthropy firm supporting early stage, high impact social enterprises. Borrowed from our venture capital legacy, DRK finds, funds, and supports exceptional leaders building innovative solutions to some of the world’s most challenging social and environmental problems. Since beginning this work nearly 25 years ago, DRK has invested in more than 270 organizations that have collectively impacted over 610 million lives to date.
@@ -1327,34 +1423,34 @@
 Please attach a standard resume/CV for the entrepreneur(s) and/or key leadership team members (e.g., CEO, COO, ED, etc.). Applications with text bios for entrepreneurs or members of the leadership team will not be considered.</t>
         </is>
       </c>
-      <c r="D15" s="1" t="inlineStr">
+      <c r="D17" s="1" t="inlineStr">
         <is>
           <t>Climate</t>
         </is>
       </c>
-      <c r="E15" s="1" t="inlineStr">
+      <c r="E17" s="1" t="inlineStr">
         <is>
           <t>Oct 10, 2026</t>
         </is>
       </c>
-      <c r="F15" s="1" t="inlineStr">
+      <c r="F17" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-open-draper-richards-kaplan-foundation-funding-for-social-enterprises-draper-richards-kaplan-foundation-opg-26-00188</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="95" customHeight="1">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B16" s="1" t="inlineStr">
+    <row r="18" ht="95" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund</t>
         </is>
       </c>
-      <c r="C16" s="1" t="inlineStr">
+      <c r="C18" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund
 Apply by: 13 October, 2026
@@ -1379,34 +1475,34 @@
  Projects should include opportunities for ServiceNow employees to volunteer in the project activation or implementation.</t>
         </is>
       </c>
-      <c r="D16" s="1" t="inlineStr">
+      <c r="D18" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E16" s="1" t="inlineStr">
+      <c r="E18" s="1" t="inlineStr">
         <is>
           <t>Oct 13, 2026</t>
         </is>
       </c>
-      <c r="F16" s="1" t="inlineStr">
+      <c r="F18" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/apply-for-the-servicenow-community-solar-fund-changex-opg-26-00186</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="95" customHeight="1">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B17" s="1" t="inlineStr">
+    <row r="19" ht="95" customHeight="1">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>RFPs Invited for Empanelment of Publishers for Procurement of E-Books for Rashtriya e-Pustakalaya National Book Trust India</t>
         </is>
       </c>
-      <c r="C17" s="1" t="inlineStr">
+      <c r="C19" s="1" t="inlineStr">
         <is>
           <t>About the RFP:
 Rashtriya e-Pustakalaya, a free National Digital Library for children and adolescents — an initiative of the Department of School Education &amp; Literacy, Ministry of Education, Government of India, implemented by the National Book Trust (NBT), India — invites Expression of Interest (EoI) for the empanelment of publishers for the selection and procurement of e-books, with the objective of enriching the platform's book collection. NBT is an autonomous body under the Ministry of Education, established in 1957 to promote literacy and reading culture in India.
@@ -1428,34 +1524,34 @@
 Must indemnify Rashtriya e-Pustakalaya/NBT-India for any IP-related claims from authors/illustrators/translators/legal owners</t>
         </is>
       </c>
-      <c r="D17" s="1" t="inlineStr">
+      <c r="D19" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E17" s="1" t="inlineStr">
+      <c r="E19" s="1" t="inlineStr">
         <is>
           <t>Oct 16, 2026</t>
         </is>
       </c>
-      <c r="F17" s="1" t="inlineStr">
+      <c r="F19" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfps-invited-for-empanelment-of-publishers-for-procurement-of-e-books-for-rashtriya-e-pustakalaya-national-book-trust-india-national-book-trust-nbt-india-rfp-26-00371</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="95" customHeight="1">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="inlineStr">
+    <row r="20" ht="95" customHeight="1">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>ToR - Engagement of Consultant/Vendor Individual towards implementation of Literacy Program in Telangana State</t>
         </is>
       </c>
-      <c r="C18" s="1" t="inlineStr">
+      <c r="C20" s="1" t="inlineStr">
         <is>
           <t>ANNEX A – TERMS OF REFERENCE (ToR) 
  Engagement of Consultant/Vendor (Individual) towards implementation of Literacy Program in Telangana State.
@@ -1520,34 +1616,34 @@
 Approved travel and accommodation expenses incurred for assignment-related activities shall be reimbursed by Room to Read in accordance with the consultancy reimbursement guidelines.</t>
         </is>
       </c>
-      <c r="D18" s="1" t="inlineStr">
+      <c r="D20" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E18" s="1" t="inlineStr">
+      <c r="E20" s="1" t="inlineStr">
         <is>
           <t>Oct 16, 2026</t>
         </is>
       </c>
-      <c r="F18" s="1" t="inlineStr">
+      <c r="F20" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-engagement-of-consultantvendor-individual-towards-implementation-of-literacy-program-in-telangana-state-room-to-read-india-rfp-26-00360</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="95" customHeight="1">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="inlineStr">
+    <row r="21" ht="95" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>RFPs Invited for Consultant to Develop a Technical Assistance Package for National Application of the Digital Health and AI Investment Classification Framework</t>
         </is>
       </c>
-      <c r="C19" s="1" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are Transform Health: a global coalition of more than 200 organisations driving the digital transformation of health to achieve universal health coverage. 
@@ -1575,34 +1671,34 @@
 Ability to manage multi-country consultancy engagements and coordinate with in-country focal points</t>
         </is>
       </c>
-      <c r="D19" s="1" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E19" s="1" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>Oct 23, 2026</t>
         </is>
       </c>
-      <c r="F19" s="1" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfps-invited-for-consultant-to-develop-a-technical-assistance-package-for-national-application-of-the-digital-health-and-ai-investment-classification-framework-transform-health-rfp-26-00359</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="95" customHeight="1">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="inlineStr">
+    <row r="22" ht="95" customHeight="1">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for D-Prize Global Competition Seed Funding for New Poverty-Solution Distribution Organizations</t>
         </is>
       </c>
-      <c r="C20" s="1" t="inlineStr">
+      <c r="C22" s="1" t="inlineStr">
         <is>
           <t>About the Grant:
 D-Prize seeds new organizations that distribute proven poverty solutions at the "last mile," with the aim of scaling impact. Applicants select from a range of evidence-based interventions (health, agriculture, education, water, safety, transparency, and more) and propose how they would launch or grow an organization to distribute that intervention. Top entrepreneurs receive up to $20,000 in seed funding to run a pilot and build an organization capable of scaling to reach thousands, even millions of people.
@@ -1625,34 +1721,34 @@
 Extension Deadline: 6 December 2026, midnight PT (extension registration required)</t>
         </is>
       </c>
-      <c r="D20" s="1" t="inlineStr">
+      <c r="D22" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E20" s="1" t="inlineStr">
+      <c r="E22" s="1" t="inlineStr">
         <is>
           <t>Oct 25, 2026</t>
         </is>
       </c>
-      <c r="F20" s="1" t="inlineStr">
+      <c r="F22" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-d-prize-global-competition-seed-funding-for-new-poverty-solution-distribution-organizations-d-prize-opg-26-00191</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="95" customHeight="1">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="inlineStr">
+    <row r="23" ht="95" customHeight="1">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 8th Call for Proposals Small-Size Grants Global EbA Fund</t>
         </is>
       </c>
-      <c r="C21" s="1" t="inlineStr">
+      <c r="C23" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -1715,34 +1811,34 @@
 Only successful applicants will be contacted; no individual feedback provided to unsuccessful applicants</t>
         </is>
       </c>
-      <c r="D21" s="1" t="inlineStr">
+      <c r="D23" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E21" s="1" t="inlineStr">
+      <c r="E23" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F21" s="1" t="inlineStr">
+      <c r="F23" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-8th-call-for-proposals-small-size-grants-global-eba-fund-global-eba-fund-opg-26-00177</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="95" customHeight="1">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="inlineStr">
+    <row r="24" ht="95" customHeight="1">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Adaptive Control Frameworks to Unlock Full-Scale BNR Potential Water Research Foundation WRF</t>
         </is>
       </c>
-      <c r="C22" s="1" t="inlineStr">
+      <c r="C24" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Water Research Foundation (WRF) is the leading research organization advancing the science of all water to meet the evolving needs of its subscribers and the water sector. WRF is a nonprofit, charitable and educational organization which funds, manages, and publishes research on the technology, operation, and management of drinking water, wastewater, reuse, and stormwater collection, treatment and supply systems—all in pursuit of ensuring water quality and improving water services to the public.
@@ -1783,34 +1879,34 @@
 Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
         </is>
       </c>
-      <c r="D22" s="1" t="inlineStr">
+      <c r="D24" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E22" s="1" t="inlineStr">
+      <c r="E24" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F22" s="1" t="inlineStr">
+      <c r="F24" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-adaptive-control-frameworks-to-unlock-full-scale-bnr-potential-water-research-foundation-wrf-the-water-research-foundation-wrf-opg-26-00187</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="95" customHeight="1">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B23" s="1" t="inlineStr">
+    <row r="25" ht="95" customHeight="1">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Crossing the Divide Best Practices for Addressing Local and Privately-Owned Lateral Sewer Issues RFP 5419</t>
         </is>
       </c>
-      <c r="C23" s="1" t="inlineStr">
+      <c r="C25" s="1" t="inlineStr">
         <is>
           <t>Project Objective:
 To provide water resource recovery facilities (WRRFs) and collection system operators with an interactive manual of practice for implementing inflow and infiltration (I&amp;I) and obstruction management programs, focused on municipal and privately owned lateral sewers in complex legal, regulatory, and multi-jurisdictional environments.
@@ -1848,34 +1944,34 @@
  Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
         </is>
       </c>
-      <c r="D23" s="1" t="inlineStr">
+      <c r="D25" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E23" s="1" t="inlineStr">
+      <c r="E25" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F23" s="1" t="inlineStr">
+      <c r="F25" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-crossing-the-divide-best-practices-for-addressing-local-and-privately-owned-lateral-sewer-issues-rfp-5419-the-water-research-foundation-wrf-opg-26-00189</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="95" customHeight="1">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B24" s="1" t="inlineStr">
+    <row r="26" ht="95" customHeight="1">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Comparison of PFAS Contributions to Agricultural Systems</t>
         </is>
       </c>
-      <c r="C24" s="1" t="inlineStr">
+      <c r="C26" s="1" t="inlineStr">
         <is>
           <t>Project Objectives:
 Report per- and polyfluoroalkyl substance (PFAS) concentrations from a variety of agricultural inputs — animal manures, fertilizers, pesticides, composts, soil amendments, seed coatings, and biosolids-based products
@@ -1911,34 +2007,34 @@
  Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00) — same deadline as the other two WRF grants</t>
         </is>
       </c>
-      <c r="D24" s="1" t="inlineStr">
+      <c r="D26" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E24" s="1" t="inlineStr">
+      <c r="E26" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F24" s="1" t="inlineStr">
+      <c r="F26" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-comparison-of-pfas-contributions-to-agricultural-systems-the-water-research-foundation-wrf-opg-26-00190</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="95" customHeight="1">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B25" s="1" t="inlineStr">
+    <row r="27" ht="95" customHeight="1">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Whitley Award 2027</t>
         </is>
       </c>
-      <c r="C25" s="1" t="inlineStr">
+      <c r="C27" s="1" t="inlineStr">
         <is>
           <t>About the Grant: 
 An annual grant by the Whitley Fund for Nature (WFN) recognising grassroots conservation leaders in the Global South, providing funding to support and scale up proven, science-based solutions that deliver lasting impact for both people and nature.
@@ -1951,34 +2047,34 @@
 You do not need to be invited or nominated to apply.</t>
         </is>
       </c>
-      <c r="D25" s="1" t="inlineStr">
+      <c r="D27" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E25" s="1" t="inlineStr">
+      <c r="E27" s="1" t="inlineStr">
         <is>
           <t>Oct 30, 2026</t>
         </is>
       </c>
-      <c r="F25" s="1" t="inlineStr">
+      <c r="F27" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-whitley-award-2027-whitley-fund-for-nature-wfn-opg-26-00153</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="95" customHeight="1">
-      <c r="A26" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B26" s="1" t="inlineStr">
+    <row r="28" ht="95" customHeight="1">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIFAR Global Scholars Program 20272029 Cohort</t>
         </is>
       </c>
-      <c r="C26" s="1" t="inlineStr">
+      <c r="C28" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 CIFAR is a Canadian-based globally influential research organization that convenes the world’s most brilliant people across disciplines to advance transformative knowledge and solve humanity’s biggest problems, together. By supporting long-term interdisciplinary collaboration, CIFAR provides researchers with an unparalleled environment of trust, transparency and knowledge sharing. Our time-tested model inspires new directions of inquiry, accelerates discovery and yields breakthroughs across borders and academic disciplines. Through knowledge mobilization, we are catalysts for change in industry, government and society. Through our 15 research programs and the Pan-Canadian AI Strategy, CIFAR convenes close to 400 of the world’s top researchers from 141 institutions in 20 countries. CIFAR is generously supported by the governments of Canada, Alberta and Québec, as well as foundations, individuals, corporations and Canadian and international partner organizations.
@@ -2022,73 +2118,34 @@
  Application Deadline: November 4, 2026, 12:00 PM EST</t>
         </is>
       </c>
-      <c r="D26" s="1" t="inlineStr">
+      <c r="D28" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E26" s="1" t="inlineStr">
+      <c r="E28" s="1" t="inlineStr">
         <is>
           <t>Nov 4, 2026</t>
         </is>
       </c>
-      <c r="F26" s="1" t="inlineStr">
+      <c r="F28" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cifar-global-scholars-program-20272029-cohort-cifar-canadian-institute-for-advanced-research-opg-26-00183</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="95" customHeight="1">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B27" s="1" t="inlineStr">
+    <row r="29" ht="95" customHeight="1">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for IWRS Teaching Innovation Award</t>
         </is>
       </c>
-      <c r="C27" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
- About the Grant
-The IWRS (Insect Welfare Research Society) Teaching Innovation Award supports instructors developing new approaches to teaching insect or invertebrate biology that incorporate the 3Rs (Replacement, Reduction, and Refinement) — principles for reducing animal welfare impacts in teaching and research practices.
- Purpose
-Funds support the creation and implementation of 3Rs-driven instructional materials and pedagogical approaches. Priority is given to proposals addressing common teaching practices with substantial welfare implications.
- Grant Amount
-Two awards of $2,000 USD are available annually.</t>
-        </is>
-      </c>
-      <c r="D27" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E27" s="1" t="inlineStr">
-        <is>
-          <t>Nov 15, 2026</t>
-        </is>
-      </c>
-      <c r="F27" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="95" customHeight="1">
-      <c r="A28" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B28" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for IWRS Teaching Innovation Award</t>
-        </is>
-      </c>
-      <c r="C28" s="1" t="inlineStr">
+      <c r="C29" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Insects are one of the most numerous and diverse animal groups on Earth.
@@ -2103,34 +2160,73 @@
 IWRS staff and Advisory Group members are not eligible to apply.</t>
         </is>
       </c>
-      <c r="D28" s="1" t="inlineStr">
+      <c r="D29" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E28" s="1" t="inlineStr">
+      <c r="E29" s="1" t="inlineStr">
         <is>
           <t>Nov 15, 2026</t>
         </is>
       </c>
-      <c r="F28" s="1" t="inlineStr">
+      <c r="F29" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00166</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="95" customHeight="1">
-      <c r="A29" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B29" s="1" t="inlineStr">
+    <row r="30" ht="95" customHeight="1">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for IWRS Teaching Innovation Award</t>
+        </is>
+      </c>
+      <c r="C30" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
+ About the Grant
+The IWRS (Insect Welfare Research Society) Teaching Innovation Award supports instructors developing new approaches to teaching insect or invertebrate biology that incorporate the 3Rs (Replacement, Reduction, and Refinement) — principles for reducing animal welfare impacts in teaching and research practices.
+ Purpose
+Funds support the creation and implementation of 3Rs-driven instructional materials and pedagogical approaches. Priority is given to proposals addressing common teaching practices with substantial welfare implications.
+ Grant Amount
+Two awards of $2,000 USD are available annually.</t>
+        </is>
+      </c>
+      <c r="D30" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E30" s="1" t="inlineStr">
+        <is>
+          <t>Nov 15, 2026</t>
+        </is>
+      </c>
+      <c r="F30" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="95" customHeight="1">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Medium-Size Grants Call for Proposals Global EbA Fund</t>
         </is>
       </c>
-      <c r="C29" s="1" t="inlineStr">
+      <c r="C31" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -2187,34 +2283,34 @@
 Applications submitted via online portal (link shared on the Medium-Size Grants webpage from Oct 12)</t>
         </is>
       </c>
-      <c r="D29" s="1" t="inlineStr">
+      <c r="D31" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E29" s="1" t="inlineStr">
+      <c r="E31" s="1" t="inlineStr">
         <is>
           <t>Nov 16, 2026</t>
         </is>
       </c>
-      <c r="F29" s="1" t="inlineStr">
+      <c r="F31" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-medium-size-grants-call-for-proposals-global-eba-fund-global-eba-fund-opg-26-00178</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="95" customHeight="1">
-      <c r="A30" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B30" s="1" t="inlineStr">
+    <row r="32" ht="95" customHeight="1">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B32" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIEIF Grant 2026 Climate Intervention Environmental Impact Fund</t>
         </is>
       </c>
-      <c r="C30" s="1" t="inlineStr">
+      <c r="C32" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Climate Intervention Environmental Impact Fund (CIEIF) is a philanthropic fund focused on supporting responsible climate intervention field tests. It provides grants for activities such as environmental impact assessment (EIA), predictive impact modelling, and engagement with potentially affected stakeholders, including local communities and government agencies.
@@ -2241,34 +2337,34 @@
 Potential for scaling the innovation to a globally relevant level</t>
         </is>
       </c>
-      <c r="D30" s="1" t="inlineStr">
+      <c r="D32" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E30" s="1" t="inlineStr">
+      <c r="E32" s="1" t="inlineStr">
         <is>
           <t>Dec 1, 2026</t>
         </is>
       </c>
-      <c r="F30" s="1" t="inlineStr">
+      <c r="F32" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cieif-grant-2026-climate-intervention-environmental-impact-fund-climate-intervention-environmental-impact-fund-opg-26-00155</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="95" customHeight="1">
-      <c r="A31" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B31" s="1" t="inlineStr">
+    <row r="33" ht="95" customHeight="1">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B33" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 6th Annual Seeding The Future Global Food System Challenge</t>
         </is>
       </c>
-      <c r="C31" s="1" t="inlineStr">
+      <c r="C33" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are one of the largest and most respected private organisations for development cooperation and humanitarian aid in Germany. As a politically and confessionally independent organisation, our value-oriented actions are always based on ethical principles. Our vision is clear: "Zero Hunger by 2030"
@@ -2300,34 +2396,34 @@
 Individuals with no organizational entity</t>
         </is>
       </c>
-      <c r="D31" s="1" t="inlineStr">
+      <c r="D33" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E31" s="1" t="inlineStr">
+      <c r="E33" s="1" t="inlineStr">
         <is>
           <t>Jan 1, 2027</t>
         </is>
       </c>
-      <c r="F31" s="1" t="inlineStr">
+      <c r="F33" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-6th-annual-seeding-the-future-global-food-system-challenge-welthungerhilfe-opg-26-00180</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="95" customHeight="1">
-      <c r="A32" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B32" s="1" t="inlineStr">
+    <row r="34" ht="95" customHeight="1">
+      <c r="A34" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B34" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Microbiota &amp; Women's Health International Call for Projects</t>
         </is>
       </c>
-      <c r="C32" s="1" t="inlineStr">
+      <c r="C34" s="1" t="inlineStr">
         <is>
           <t>About the Grant
 An annual international research grant by the Biocodex Microbiota Foundation (BMF), rewarding research proposals on the microbiota and its implications in Women's Health and Disease. This year's theme: "Unraveling male-female genital microbiome interactions: mechanisms, transmission, and impact on vaginal dysbiosis."
@@ -2344,34 +2440,34 @@
 €200,000 annually — awarded to researchers within universities, hospitals, or other research settings to finance equipment, operations, or staffing costs. Grants are NOT awarded to individuals directly (must be institutionally affiliated). Institution's overhead costs capped at 10%.</t>
         </is>
       </c>
-      <c r="D32" s="1" t="inlineStr">
+      <c r="D34" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E32" s="1" t="inlineStr">
+      <c r="E34" s="1" t="inlineStr">
         <is>
           <t>Jan 15, 2027</t>
         </is>
       </c>
-      <c r="F32" s="1" t="inlineStr">
+      <c r="F34" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-microbiota-and-womens-health-international-call-for-projects-biocodex-microbiota-foundation-bmf-opg-26-00152</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="95" customHeight="1">
-      <c r="A33" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B33" s="1" t="inlineStr">
+    <row r="35" ht="95" customHeight="1">
+      <c r="A35" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B35" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for BES Training and Travel Grants</t>
         </is>
       </c>
-      <c r="C33" s="1" t="inlineStr">
+      <c r="C35" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are a global community of scientists shining a spotlight on the intricacy and value of our natural world, providing the evidence for better decisions. Our vision is for people and nature to thrive in a world that values ecology.
@@ -2410,17 +2506,17 @@
  Application Deadline (Round 2): Opens 30 April 2026, closes 17 May 2026</t>
         </is>
       </c>
-      <c r="D33" s="1" t="inlineStr">
+      <c r="D35" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E33" s="1" t="inlineStr">
+      <c r="E35" s="1" t="inlineStr">
         <is>
           <t>May 17, 2027</t>
         </is>
       </c>
-      <c r="F33" s="1" t="inlineStr">
+      <c r="F35" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-bes-training-and-travel-grants-british-ecological-society-opg-26-00181</t>
         </is>

</xml_diff>

<commit_message>
Auto update Combined.xlsx [Sun Sep 27 07:30:40 UTC 2026]
</commit_message>
<xml_diff>
--- a/output/Combined.xlsx
+++ b/output/Combined.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -495,178 +495,10 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>ToR - Engagement of Information Design &amp; Video Production Agency / Consultant for Key Learning &amp; Dissemination Outputs</t>
+          <t>RFP - Engagement of Agency for Development of MIS Dashboard and Mobile-based Application for Adolescent Mental Health</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t>Terms of Reference (TOR) for Consultancy Services
-Title  Engagement of Information Design &amp; Video Production Agency / Consultant for Key Learning &amp; Dissemination Outputs
-Timeline 12 Months (1st October 2026 – 31st September 2027)
-Expected area of expertise
- Proven experience in information design, data visualization, narrative structuring, and short-form video editing/production (preferably in the development/social sector).
-Portfolio demonstrating translation of complex, technical, or research-heavy content into engaging visual and video formats.
-Alignment with SELCO’s brand ethos and open-source dissemination principles.
-Apply Link https://forms.gle/kDNRaSdQAkqbDMrM8
-Last             Date           for Apply 28th September 2026; 5 PM
-About SELCO Foundation:
-SELCO Foundation’s mission is to create a platform of solutions that uses sustainable energy as a catalyst to bridge environmental sustainability and poverty alleviation. With holistic development as the primary focus, the organization strives to create equitable societies, where services are accessed by all communities. The interventions of SELCO lead to a sustainable delivery model of essential services like livelihoods, education, and health till the last mile. (Read more about SELCO here: http://www.selcofoundation.org/)
-About the Programmes:
-SELCO Foundation continuously generates field insights, technical frameworks, program impacts, and sectoral learnings across its core operational verticals (rural healthcare, urban livelihoods, climate adaptation, and regenerative agriculture). Effectively capturing and translating these raw research assets into accessible, high-quality public visual narratives is essential for driving ecosystem alignment and sector-wide knowledge exchange.
-Objective:
-The primary objective of this engagement is to enable SELCO Foundation to effectively capture, structure, and communicate its field insights, sectoral learnings, and program impacts. The selected Agency/Consultant (or Agencies/Consultants) will work on a monthly retainer basis to translate raw content, data, field footage, and reports provided by SELCO into high-quality, visually compelling, reader-friendly visual outputs and video assets.</t>
-        </is>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>Sep 28, 2026</t>
-        </is>
-      </c>
-      <c r="F3" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/tor-engagement-of-information-design-and-video-production-agency-consultant-for-key-learning-and-dissemination-outputs-selco-foundation-rfp-26-00362</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="95" customHeight="1">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>ToR - Video documentation of change stories on Ground water replenishment in Hyderabad and Sanga Reddy locations</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>About Jal Seva Charitable Foundation/ WaterAid India:
-Jal Seva Charitable Foundation (JSCF) is registered in India as a not-for-profit company under Chapter 8 of the Companies Act, 2013. JSCF, is an associate member of WaterAid International and uses the brand name ‘WaterAid’ in India.
-JSCF or WaterAid India seeks to improve climate resilience access to clean water, decent toilets, and good hygiene for everyone, everywhere. Our work is focused on the following themes:
-Safe, assured drinking water at a household level.
-Safely managed sanitation.
-Water, sanitation, and hygiene (WASH) in institutions (Anganwadi, schools, and health care facilities).
-Hygiene education and behaviour change.
- WaterAid India country office is based in New Delhi with State Offices in Bengaluru, Bhopal, Bhubaneswar, Hyderabad, Lucknow, Raipur, and Patna. WaterAid India currently works in 11+ states across the country. As a direct implementing agency, WaterAid India district and block-level teams are located close to our intervention villages. Further information regarding WaterAid India can be found online;  https://www.wateraid.org/in/ 
- Background &amp; Scope of engagement:
-Water security is a major development challenge in urban India, driven by rapid urbanization, rising water demand, declining groundwater, and climate variability. Hyderabad, one of India’s fastest-growing cities, has seen significant urban expansion, which has reduced natural recharge areas, increased surface runoff, and placed greater pressure on groundwater resources.
-The Serilingampally Zone of the Greater Hyderabad Municipal Corporation (GHMC) is especially vulnerable to groundwater depletion due to rapid development. Although municipal water supply is expanding, groundwater remains a vital supplementary source for domestic and institutional needs. Sustainable groundwater recharge and conservation are essential for long-term urban water security.
- To address these challenges, WaterAid India, launched the Amruthvarshini Project in May 2023. The project aimed to enhance groundwater replenishment through rainwater harvesting, managed aquifer recharge, community mobilization, awareness campaigns, and institutional strengthening.
- Over the past three years, the programme has produced increased groundwater recharge, photographs, videos, beneficiary stories, and communication materials. These now need to be converted into engaging digital content to support knowledge sharing and future urban water security initiatives.
- In this context, Jal Seva Charitable Foundation (JSCF) seeks to engage a consultant for ‘Video Documentation of Change Stories’ as outlined in the following terms and conditions.
- Objective of the contract:
-The objective of this assignment is to capture and document post-intervention activities of ground water replenishment in Sherlingampally Zone in Hyderabad and in Sangareddy district through video documentation.
- Scope of assignment &amp; expected outcome:
-This assignment involves producing a 6-minute video capturing real-life change stories resulting from water-harvesting interventions.
-The assignment includes the following deliverables:
-A 6-minute, high-resolution video showcasing the impact of water-harvesting infrastructure through community testimonials. It will include interviews, relevant field visuals and a clear storyline highlighting the changes brought about by the interventions. The video will effectively capture community experiences, benefits, and key outcomes.
- Duration of the contract: The Consultancy Agreement will be effective for a period of 20 days from the date of signing and is expected to be completed by 30 October 2026, unless extended in writing by JSCF. Any extension will be subject to additional or revised terms and conditions as mutually agreed upon in writing between the Consultant and JSCF.
- Reporting point and Progress Report
-For matters covered by the TORs and this agreement, you will report directly to Mr Pachimadla Krishna, Program Coordinator, Telangana, JSCF, and submit reports as specified in the TORs.
-Payment Schedule Condition for Payment
- 20%
-40%
-40%
-Upon signing of the Contract
-Upon submission of 6 Minutes of Drafted Video
-Upon completion of Assignment</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>Learning</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="inlineStr">
-        <is>
-          <t>Sep 28, 2026</t>
-        </is>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/tor-video-documentation-of-change-stories-on-ground-water-replenishment-in-hyderabad-and-sanga-reddy-locations-wateraid-india-rfp-26-00363</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="95" customHeight="1">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>ToR - Video Production Storytelling and Documentation</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="inlineStr">
-        <is>
-          <t>Title Video Production – Storytelling and Documentation
-Timeline 3 months from the date of contracting
-Expected area of expertise Video production, documentary storytelling, interviews, field documentation, cinematography and post-production
-Apply Link https://forms.gle/qiATVNrSkDJrkNH3A
-Last      Date             for Apply 29th September 2026 by 5 PM
-About SELCO Foundation:
-SELCO Foundation’s mission is to create a platform of solutions that uses sustainable energy as a catalyst to bridge environmental sustainability and poverty alleviation. With holistic development as the primary focus, the organization strives to create equitable societies, where services are accessed by all communities. The interventions of SELCO lead to a sustainable delivery model of essential services like livelihoods, education, and health till the last mile. (Read more about SELCO here: http://www.selcofoundation.org/)
- About the Programmes:
-SELCO Foundation is looking to engage a video production partner to develop a series of compelling videos that document and communicate stories emerging from its programmes and field interventions.
-The assignment will involve end-to-end video production, including story development, filming, interviews, visual documentation, editing and post-production. The videos will highlight people, experiences, solutions, impact and the broader context of the organisation's work.
-The final content will be used across digital platforms, social media, events, presentations, reports and other communication channels
- Objective:
-To produce a series of compelling videos that document programme experiences, end-user journeys and solutions in a clear, engaging and accessible manner.
-The videos should move beyond activity documentation to capture the context, challenge, solution, experience and outcomes of the people and communities being documented.
-The selected partner will be expected to provide:
-Story treatment/concept notes
-Interview questions and filming plan
-Raw footage from all filming
-Edited full-length video
-Edited short version
-30-second trailer
-Subtitled versions, where required
-Final master files in agreed resolution and formats
-Social-media-ready versions, where required
-Project/source files upon completion
- Submission Requirements:
-Interested production partners are requested to submit the following by before deadline
-Organizational/Individual Profile: Overview of your team/experience.Proposed Approach: A brief document outlining your understanding of the assignment and your proposed approach to storytelling and production.
-Relevant Portfolio: 3–5 relevant video samples demonstrating documentary, impact, social-sector, development or human-interest storytelling.Experience with Similar Assignments: Details of relevant video production and field documentation work.
-Quotation Should include all cost including Travel and Miscellaneous.</t>
-        </is>
-      </c>
-      <c r="D5" s="1" t="inlineStr">
-        <is>
-          <t>Learning</t>
-        </is>
-      </c>
-      <c r="E5" s="1" t="inlineStr">
-        <is>
-          <t>Sep 29, 2026</t>
-        </is>
-      </c>
-      <c r="F5" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/tor-video-production-storytelling-and-documentation-selco-foundation-rfp-26-00368</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="95" customHeight="1">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>RFP - Engagement of Agency for Development of MIS Dashboard and Mobile-based Application for Adolescent Mental Health</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>Release of Request for Proposal
 23rd September 2026
@@ -733,34 +565,162 @@
 It is to be submitted separately as per Annexure II. No conditional price is to be quoted.</t>
         </is>
       </c>
-      <c r="D6" s="1" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E6" s="1" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Sep 29, 2026</t>
         </is>
       </c>
-      <c r="F6" s="1" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfp-engagement-of-agency-for-development-of-mis-dashboard-and-mobile-based-application-for-adolescent-mental-health-american-india-foundation-rfp-26-00372</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="95" customHeight="1">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
+    <row r="4" ht="95" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>ToR - Video Production Storytelling and Documentation</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Title Video Production – Storytelling and Documentation
+Timeline 3 months from the date of contracting
+Expected area of expertise Video production, documentary storytelling, interviews, field documentation, cinematography and post-production
+Apply Link https://forms.gle/qiATVNrSkDJrkNH3A
+Last      Date             for Apply 29th September 2026 by 5 PM
+About SELCO Foundation:
+SELCO Foundation’s mission is to create a platform of solutions that uses sustainable energy as a catalyst to bridge environmental sustainability and poverty alleviation. With holistic development as the primary focus, the organization strives to create equitable societies, where services are accessed by all communities. The interventions of SELCO lead to a sustainable delivery model of essential services like livelihoods, education, and health till the last mile. (Read more about SELCO here: http://www.selcofoundation.org/)
+ About the Programmes:
+SELCO Foundation is looking to engage a video production partner to develop a series of compelling videos that document and communicate stories emerging from its programmes and field interventions.
+The assignment will involve end-to-end video production, including story development, filming, interviews, visual documentation, editing and post-production. The videos will highlight people, experiences, solutions, impact and the broader context of the organisation's work.
+The final content will be used across digital platforms, social media, events, presentations, reports and other communication channels
+ Objective:
+To produce a series of compelling videos that document programme experiences, end-user journeys and solutions in a clear, engaging and accessible manner.
+The videos should move beyond activity documentation to capture the context, challenge, solution, experience and outcomes of the people and communities being documented.
+The selected partner will be expected to provide:
+Story treatment/concept notes
+Interview questions and filming plan
+Raw footage from all filming
+Edited full-length video
+Edited short version
+30-second trailer
+Subtitled versions, where required
+Final master files in agreed resolution and formats
+Social-media-ready versions, where required
+Project/source files upon completion
+ Submission Requirements:
+Interested production partners are requested to submit the following by before deadline
+Organizational/Individual Profile: Overview of your team/experience.Proposed Approach: A brief document outlining your understanding of the assignment and your proposed approach to storytelling and production.
+Relevant Portfolio: 3–5 relevant video samples demonstrating documentary, impact, social-sector, development or human-interest storytelling.Experience with Similar Assignments: Details of relevant video production and field documentation work.
+Quotation Should include all cost including Travel and Miscellaneous.</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Sep 29, 2026</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/tor-video-production-storytelling-and-documentation-selco-foundation-rfp-26-00368</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="95" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>EOI Inviting Expression of Interest-cum-Proposal for Setting Up District De-Addiction Centres under NAPDDR</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>About us
+In the year 1985-86, the erstwhile Ministry of Welfare was bifurcated into the Department of Women and Child Development and the Department of Welfare. Simultaneously, the Scheduled Castes Development Division, Tribal Development Division and the Minorities and Backward Classes Welfare Division were moved from the Ministry of Home Affairs and also the Wakf Division from the Ministry of Law to form the then Ministry of Welfare Subsequently, the name of the Ministry was changed to the Ministry of Social Justice &amp; Empowerment in May, 1998. Further, in October, 1999, the Tribal Development Division had moved out to form a separate Ministry of Tribal Affairs. In January, 2007, the Minorities Division along with Wakf Unit have been moved out of the Ministry and formed as a separate Ministry and the Child Development Division has gone to the Ministry of Women &amp; Child Development.
+ Department of Social Justice and Empowerment invites Expression of lnterest-cum-proposal from the eligible organizations for setting up of District DeAddiction Centres under the scheme of National Action Plan for Drug Demand Reduction (NAPDDR) for 315 GAP Districts of the country (as per list attached at Annexure - l). The list of districts is subject to change (addition or deletion) time to trme by the Ministry as per requirement or need on the ground.
+ 2. Eligible NGOs may apply for setting up of DDAC provided that they have rent free accommodation for setting up of DDAC as per the standards of guideline of the NAPDDR scheme or renlfree accommodation may also be provided by the concerned District Administration. 
+ 3. Setting up and running of District De-Addiction Centres (DDACS) will be done as per the following guidelinesr. 
+ i. There will be a District De-Addiction Centre (DDAC) preferably in each district headquarter or suitably accessible place where rent free accommodation is provided by the district administration. These DDACs would provide comprehensive facilities hitherto being provided by IRCA, ODIC &amp; CPLI together. lf the district administration of identified district is not able to provide suitable rent free accommodation, then the application will be called from the eligible VOs/ NGOs, who will provide rent free accommodation for setting up of DDAC in that district.
+ ii. The functioning of DDAC will be monitored by the three tier Committees headed by the Chief Secretary, District Collector/Deputy Commissioner and Block Development Officer of the respective arealregion which have been formed under Nasha Mukt Bharat Abhiyaan (NMBA). Additionally, retired eminent personalities of the Districts, activists, Vice-Chancellor/ Head of Department (HoD)/ Principal, researcher, scholars and so on may be co-opted by Chairman as the members of the Committees. These commiftees would
+ only monitor policy related issues. Day to day and other activities relating to implementation would be the responsibility of the concerned organization/NGO approved for setting up of the DDAC. The Meetings of DDAC are to be held as per the details given below:
+ (a) State-level Steering and Monitoring Committee (High Level Task Force) - headed by Chief Secretary - to meet quarterly. (b) District-level Committee - headed by District Collector / Deputy Commissioner - to meet monthly and have mandatory inspections quarterly. (c) Block level Committee - headed by Block Development Officer - to meet &amp; have mandatory inspections monthly.
+ The Committees will also review the functioning and assess the performance of the DDAC in terms of the effectiveness of deliverables and make further suggestions to the management of DDAC. 
+ IIl t. A separate (dedicated) account will be opened for keeping funds of DDAC in the name of NGO/Organization. The account will be registered on PFMS and implemented through EAT Module. 
+ lV. For setting up of DDACs, preference would be given to those Districts, which do not have any facility of IRCA or DDAC. For this, the organization willing to work in the field of DRUGS DE-ADDICTION TREATMENT will be eligible for applying for DDAC. The priority for selection of DDAC would be: 
+a. The DDAC proposed to be run by the District administration itself. 
+b. Rent free accommodation in the district headquarter provided by the concerned DC/DM &amp; further willingness from interested NGO is sought. c, Where no proposal for rent-free accommodation is received from concerned DCiDM, interested NGO may directly apply for DDAC provided they do not seek any rent for same and only building maintenance will be given. 
+V. The details of Minimum standards like physical space and necessary amenities to be provided by District administration or NGOs are as under: 
+(a) The centre should be easily accessible and connected through public transport. 
+(b) The total built-in area of the DDAC should be at least 3000 sq,ft. in case of metros and 4000 sq.ft. in case of small towns and villages to house 15 patients and 4000 sq.ft. in case of metros and 5000 sq.ft. in case of small towns and villages to house 30 patients. This includes an area of about 2000 sq. ft. for Treatment cum Rehabilitation centre, an area of about 700 sq. ft. for Drop-ln Centre facilities and an area of about 300 sq. ft. for CPLI Centre facilities. 
+(c) The centre should be properly ventilated, well-lit and maintained in a clean manner. Water to be made available. 
+(d) Basic safety of the patients to be ensured 
+(e) Facilities at the centre - Waiting space with seating arrangements for a minimum 5 persons Cubicles / rooms for consultation for physical examination Facilities to store drugs, linen, and records of patients Facilities with privacy for providing individual counselling, group therapy, re-educative sessions, family classes. They should be airy with comfortable seating with floor mats / chairs. Blackboard, chalk and other material to be provided. Availability of recreational facilities. Separate Drop ln Facility centre with recreation room, counselling room and medical room. Project room for CPLI activities including consultation room for interviewing Vl. Standards set in the above para of the guidelines may change from time to time as and when necessary with the approval of competent authority and the stakeholders / NGOs/ VOs would be intimated of same as and when such changes happen. 
+ 4. The interested and eligible NGOs / organizations can apply through eAnudaan (https://grants-msje.gov.in/ngo-login) portal of the Ministry. The Project Screening Committee in the Ministry will select the eligible NGO(s) for establishing and running of the DDAC and recommend the release of funds in two installments. However, the organization shall be eligible for receiving GIA under the scheme from the date of approval of the competent authority. 
+ 5. ELIGIBLE ORGANIZATION: 
+Organizations which are already running MoSJE supported IRCA or State Government supported De-addiction Centre/ Government Hospital or any private run De-Addiction centre are eligible for applying for DDAC. Organization can apply only for that State/UT in which they are already running IRCA"/De-addiction Centre from the last 2 years or more from the date of call for the proposal. Condition may be relaxed for any Government run Hospitals, which are non-profitable in nature. I 
+6. Start-up consists of young persons/ professionals, who have graduated from top social institutes of lndia or abroad are also eligible to apply. However, they must have experience of 2 years in the field of Drug De-addiction TREATMENT. 7. Role and Responsibility of DDACs The main focus of the DDAC is early prevention, education, demand reduction, identification, treatment and rehabilitation services of vulnerable individuals or individuals affected by substance use disorders DDAC would: 
+a. Conduct primary prevention activities through awareness programs among the vulnerable and affected community 
+b. Engage in risk mitigation of substance use among children/ adolescenuyouth by: Preventing substance use Delaying initiation of substance use 
+c. ldentify and train selected peer educators in the community 
+d. lmplement early prevention education through life skill training led by trained peer educators 
+e. Provide awareness about referral and linkage to counseling, treatment and rehabilitation services for substance dependent adolescents identified in the community 
+f. ldentifying adolescents and other individuals subjected to substance use and facilitating their referrali admission into Rehabilitation Centers/ Drop ln Centres. 
+g. Provide a whole range of services which includes treatment, after care and rehabilitation including skill development for Whole Person Recovery (WPR) of dependents; 
+h. Undertake drug demand reduction efforts to address all forms of illicit use of any substances and ensure overall well being of humankind; 
+i. Alleviate the consequences of substance dependence amongst individuals, family and society at large 
+9. The budget details of DDAC is attached as Annexure - 
+10. The e-anudaan portal shall remain open through out the year and the recommendations from the States/UTs will be considered periodically. 
+11. Department of Social Justice and Empowerment (DoSJE) reserves the right to cancel this notice, andior invite afresh proposals with or without amendments to this document without liability or any obligation for such document, and without assigning any reason. DoSJE reserves the right to take final decision regarding selection of implementing agency or project.</t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>Sep 30, 2026</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/eoi-inviting-expression-of-interest-cum-proposal-for-setting-up-district-de-addiction-centres-under-napddr-ministry-of-social-justice-and-empowerment-goi-rfp-26-00356</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="95" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Setting up Viral Research and Diagnosis Laboratories VRDL in Medical Colleges/Hospitals/Medical Institutions</t>
         </is>
       </c>
-      <c r="C7" s="1" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The President notified the creation of the Department of Health Research under the Ministry of Health &amp; Family Welfare through an amendment to the Government of India (Allocation of Business) Rules, 1961 on the 17th September 2007. The Department of Health Research was formally launched on 5th October 2007 by the Minister for Science &amp; Technology and Earth Sciences in a function presided over by the Minister for Health &amp; Family Welfare, in the presence, inter-alia, of the Minister of State for Health &amp; Family Welfare.
@@ -797,34 +757,34 @@
 Private medical colleges: only top-50 NIRF-ranked institutions considered</t>
         </is>
       </c>
-      <c r="D7" s="1" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E7" s="1" t="inlineStr">
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F7" s="1" t="inlineStr">
+      <c r="F6" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-setting-up-viral-research-and-diagnosis-laboratories-vrdl-in-medical-collegeshospitalsmedical-institutions-department-of-health-research-dhr-ministry-of-health-and-family-welfare-government-of-india-opg-26-00174</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="95" customHeight="1">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
+    <row r="7" ht="95" customHeight="1">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Signals of Change Shaping the Future of Sexual and Reproductive Health and Rights SRHR</t>
         </is>
       </c>
-      <c r="C8" s="1" t="inlineStr">
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The World Health Organization's mission: to promote health, keep the world safe, and serve the vulnerable. Working through offices in more than 150 countries, WHO staff work side by side with governments and other partners to ensure the highest attainable level of health for all people.
@@ -849,34 +809,34 @@
  Submission Requirements: Descriptive information (name, contact email, country, sector) required alongside each submission; formal published evidence is helpful but not required — practice-based experience and field examples are also welcome. Submissions are kept confidential and anonymized before analysis.</t>
         </is>
       </c>
-      <c r="D8" s="1" t="inlineStr">
+      <c r="D7" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E8" s="1" t="inlineStr">
+      <c r="E7" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F8" s="1" t="inlineStr">
+      <c r="F7" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-signals-of-change-shaping-the-future-of-sexual-and-reproductive-health-and-rights-srhr-world-health-organization-opg-26-00176</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="95" customHeight="1">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="inlineStr">
+    <row r="8" ht="95" customHeight="1">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>ToR - Branding Development &amp; Design/Market Promotion Consultant Project Sashakt</t>
         </is>
       </c>
-      <c r="C9" s="1" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>Organisation Humana People to People India (HPPI)
 Project Sashakt – Strengthening Women-led Handloom Cooperatives in Assam (EU-funded)
@@ -931,101 +891,34 @@
 The consultant/agency must ensure ethical, consent-based data collection with cultural sensitivity, particularly when engaging women weavers. All data and reports remain the property of HPPI and must be kept strictly confidential, with no external use.</t>
         </is>
       </c>
-      <c r="D9" s="1" t="inlineStr">
+      <c r="D8" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E9" s="1" t="inlineStr">
+      <c r="E8" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F9" s="1" t="inlineStr">
+      <c r="F8" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-branding-development-and-designmarket-promotion-consultant-project-sashakt-humana-people-to-people-india-rfp-26-00365</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="95" customHeight="1">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
-        <is>
-          <t>EOI Inviting Expression of Interest-cum-Proposal for Setting Up District De-Addiction Centres under NAPDDR</t>
-        </is>
-      </c>
-      <c r="C10" s="1" t="inlineStr">
-        <is>
-          <t>About us
-In the year 1985-86, the erstwhile Ministry of Welfare was bifurcated into the Department of Women and Child Development and the Department of Welfare. Simultaneously, the Scheduled Castes Development Division, Tribal Development Division and the Minorities and Backward Classes Welfare Division were moved from the Ministry of Home Affairs and also the Wakf Division from the Ministry of Law to form the then Ministry of Welfare Subsequently, the name of the Ministry was changed to the Ministry of Social Justice &amp; Empowerment in May, 1998. Further, in October, 1999, the Tribal Development Division had moved out to form a separate Ministry of Tribal Affairs. In January, 2007, the Minorities Division along with Wakf Unit have been moved out of the Ministry and formed as a separate Ministry and the Child Development Division has gone to the Ministry of Women &amp; Child Development.
- Department of Social Justice and Empowerment invites Expression of lnterest-cum-proposal from the eligible organizations for setting up of District DeAddiction Centres under the scheme of National Action Plan for Drug Demand Reduction (NAPDDR) for 315 GAP Districts of the country (as per list attached at Annexure - l). The list of districts is subject to change (addition or deletion) time to trme by the Ministry as per requirement or need on the ground.
- 2. Eligible NGOs may apply for setting up of DDAC provided that they have rent free accommodation for setting up of DDAC as per the standards of guideline of the NAPDDR scheme or renlfree accommodation may also be provided by the concerned District Administration. 
- 3. Setting up and running of District De-Addiction Centres (DDACS) will be done as per the following guidelinesr. 
- i. There will be a District De-Addiction Centre (DDAC) preferably in each district headquarter or suitably accessible place where rent free accommodation is provided by the district administration. These DDACs would provide comprehensive facilities hitherto being provided by IRCA, ODIC &amp; CPLI together. lf the district administration of identified district is not able to provide suitable rent free accommodation, then the application will be called from the eligible VOs/ NGOs, who will provide rent free accommodation for setting up of DDAC in that district.
- ii. The functioning of DDAC will be monitored by the three tier Committees headed by the Chief Secretary, District Collector/Deputy Commissioner and Block Development Officer of the respective arealregion which have been formed under Nasha Mukt Bharat Abhiyaan (NMBA). Additionally, retired eminent personalities of the Districts, activists, Vice-Chancellor/ Head of Department (HoD)/ Principal, researcher, scholars and so on may be co-opted by Chairman as the members of the Committees. These commiftees would
- only monitor policy related issues. Day to day and other activities relating to implementation would be the responsibility of the concerned organization/NGO approved for setting up of the DDAC. The Meetings of DDAC are to be held as per the details given below:
- (a) State-level Steering and Monitoring Committee (High Level Task Force) - headed by Chief Secretary - to meet quarterly. (b) District-level Committee - headed by District Collector / Deputy Commissioner - to meet monthly and have mandatory inspections quarterly. (c) Block level Committee - headed by Block Development Officer - to meet &amp; have mandatory inspections monthly.
- The Committees will also review the functioning and assess the performance of the DDAC in terms of the effectiveness of deliverables and make further suggestions to the management of DDAC. 
- IIl t. A separate (dedicated) account will be opened for keeping funds of DDAC in the name of NGO/Organization. The account will be registered on PFMS and implemented through EAT Module. 
- lV. For setting up of DDACs, preference would be given to those Districts, which do not have any facility of IRCA or DDAC. For this, the organization willing to work in the field of DRUGS DE-ADDICTION TREATMENT will be eligible for applying for DDAC. The priority for selection of DDAC would be: 
-a. The DDAC proposed to be run by the District administration itself. 
-b. Rent free accommodation in the district headquarter provided by the concerned DC/DM &amp; further willingness from interested NGO is sought. c, Where no proposal for rent-free accommodation is received from concerned DCiDM, interested NGO may directly apply for DDAC provided they do not seek any rent for same and only building maintenance will be given. 
-V. The details of Minimum standards like physical space and necessary amenities to be provided by District administration or NGOs are as under: 
-(a) The centre should be easily accessible and connected through public transport. 
-(b) The total built-in area of the DDAC should be at least 3000 sq,ft. in case of metros and 4000 sq.ft. in case of small towns and villages to house 15 patients and 4000 sq.ft. in case of metros and 5000 sq.ft. in case of small towns and villages to house 30 patients. This includes an area of about 2000 sq. ft. for Treatment cum Rehabilitation centre, an area of about 700 sq. ft. for Drop-ln Centre facilities and an area of about 300 sq. ft. for CPLI Centre facilities. 
-(c) The centre should be properly ventilated, well-lit and maintained in a clean manner. Water to be made available. 
-(d) Basic safety of the patients to be ensured 
-(e) Facilities at the centre - Waiting space with seating arrangements for a minimum 5 persons Cubicles / rooms for consultation for physical examination Facilities to store drugs, linen, and records of patients Facilities with privacy for providing individual counselling, group therapy, re-educative sessions, family classes. They should be airy with comfortable seating with floor mats / chairs. Blackboard, chalk and other material to be provided. Availability of recreational facilities. Separate Drop ln Facility centre with recreation room, counselling room and medical room. Project room for CPLI activities including consultation room for interviewing Vl. Standards set in the above para of the guidelines may change from time to time as and when necessary with the approval of competent authority and the stakeholders / NGOs/ VOs would be intimated of same as and when such changes happen. 
- 4. The interested and eligible NGOs / organizations can apply through eAnudaan (https://grants-msje.gov.in/ngo-login) portal of the Ministry. The Project Screening Committee in the Ministry will select the eligible NGO(s) for establishing and running of the DDAC and recommend the release of funds in two installments. However, the organization shall be eligible for receiving GIA under the scheme from the date of approval of the competent authority. 
- 5. ELIGIBLE ORGANIZATION: 
-Organizations which are already running MoSJE supported IRCA or State Government supported De-addiction Centre/ Government Hospital or any private run De-Addiction centre are eligible for applying for DDAC. Organization can apply only for that State/UT in which they are already running IRCA"/De-addiction Centre from the last 2 years or more from the date of call for the proposal. Condition may be relaxed for any Government run Hospitals, which are non-profitable in nature. I 
-6. Start-up consists of young persons/ professionals, who have graduated from top social institutes of lndia or abroad are also eligible to apply. However, they must have experience of 2 years in the field of Drug De-addiction TREATMENT. 7. Role and Responsibility of DDACs The main focus of the DDAC is early prevention, education, demand reduction, identification, treatment and rehabilitation services of vulnerable individuals or individuals affected by substance use disorders DDAC would: 
-a. Conduct primary prevention activities through awareness programs among the vulnerable and affected community 
-b. Engage in risk mitigation of substance use among children/ adolescenuyouth by: Preventing substance use Delaying initiation of substance use 
-c. ldentify and train selected peer educators in the community 
-d. lmplement early prevention education through life skill training led by trained peer educators 
-e. Provide awareness about referral and linkage to counseling, treatment and rehabilitation services for substance dependent adolescents identified in the community 
-f. ldentifying adolescents and other individuals subjected to substance use and facilitating their referrali admission into Rehabilitation Centers/ Drop ln Centres. 
-g. Provide a whole range of services which includes treatment, after care and rehabilitation including skill development for Whole Person Recovery (WPR) of dependents; 
-h. Undertake drug demand reduction efforts to address all forms of illicit use of any substances and ensure overall well being of humankind; 
-i. Alleviate the consequences of substance dependence amongst individuals, family and society at large 
-9. The budget details of DDAC is attached as Annexure - 
-10. The e-anudaan portal shall remain open through out the year and the recommendations from the States/UTs will be considered periodically. 
-11. Department of Social Justice and Empowerment (DoSJE) reserves the right to cancel this notice, andior invite afresh proposals with or without amendments to this document without liability or any obligation for such document, and without assigning any reason. DoSJE reserves the right to take final decision regarding selection of implementing agency or project.</t>
-        </is>
-      </c>
-      <c r="D10" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E10" s="1" t="inlineStr">
-        <is>
-          <t>Sep 30, 2026</t>
-        </is>
-      </c>
-      <c r="F10" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/eoi-inviting-expression-of-interest-cum-proposal-for-setting-up-district-de-addiction-centres-under-napddr-ministry-of-social-justice-and-empowerment-goi-rfp-26-00356</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="95" customHeight="1">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="inlineStr">
+    <row r="9" ht="95" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
         <is>
           <t>Application Invited for Giving Joy Microgrant</t>
         </is>
       </c>
-      <c r="C11" s="1" t="inlineStr">
+      <c r="C9" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Giving Joy is a US-based nonprofit that strengthens and inspires women’s entrepreneurship worldwide. Through its micro-grants and mentorship program, Giving Joy helps women establish or improve their businesses and initiatives—for their benefit and the benefit of their communities. To date, Giving Joy has awarded over 88 grants to women-led initiatives in 26 countries.
@@ -1064,34 +957,34 @@
 The grant period is six months.</t>
         </is>
       </c>
-      <c r="D11" s="1" t="inlineStr">
+      <c r="D9" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E11" s="1" t="inlineStr">
+      <c r="E9" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F11" s="1" t="inlineStr">
+      <c r="F9" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/application-invited-for-giving-joy-microgrant-giving-joy-opg-26-00185</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="95" customHeight="1">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="inlineStr">
+    <row r="10" ht="95" customHeight="1">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
         <is>
           <t>ToR - Project Management Unit Solarization of Women-led Livelihoods in Maharashtra MAVIMSELCO Foundation Short Duration Project</t>
         </is>
       </c>
-      <c r="C12" s="1" t="inlineStr">
+      <c r="C10" s="1" t="inlineStr">
         <is>
           <t>Title Project Management Unit – Solarization of Women-led Livelihoods in Maharashtra (MAVIM–SELCO Foundation Short Duration Project)
 Timeline 6 Months (Oct – Mar)
@@ -1132,34 +1025,34 @@
 Examples of similar past projects, particularly involving SHG networks, livelihood programs, or energy access.</t>
         </is>
       </c>
-      <c r="D12" s="1" t="inlineStr">
+      <c r="D10" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E12" s="1" t="inlineStr">
+      <c r="E10" s="1" t="inlineStr">
         <is>
           <t>Oct 3, 2026</t>
         </is>
       </c>
-      <c r="F12" s="1" t="inlineStr">
+      <c r="F10" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-project-management-unit-solarization-of-women-led-livelihoods-in-maharashtra-mavimselco-foundation-short-duration-project-selco-foundation-rfp-26-00374</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="95" customHeight="1">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B13" s="1" t="inlineStr">
+    <row r="11" ht="95" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>EOI - Engagement of Agencies for HR Recruitment Services</t>
         </is>
       </c>
-      <c r="C13" s="1" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>The American India Foundation Trust (AIFT) seeks to engage an experienced recruitment agency to provide end-to-end recruitment and talent acquisition services for identified positions across its offices, programmes, and functions in India.
 The selected agency shall support AIFT in sourcing, screening, shortlisting, interview coordination, candidate engagement, offer management, and recruitment closure, in accordance with the requirements, timelines, and service levels agreed with AIFT.
@@ -1190,34 +1083,95 @@
 Any other information specifically requested by AIFT.</t>
         </is>
       </c>
-      <c r="D13" s="1" t="inlineStr">
+      <c r="D11" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E13" s="1" t="inlineStr">
+      <c r="E11" s="1" t="inlineStr">
         <is>
           <t>Oct 4, 2026</t>
         </is>
       </c>
-      <c r="F13" s="1" t="inlineStr">
+      <c r="F11" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/eoi-engagement-of-agencies-for-hr-recruitment-services-american-india-foundation-rfp-26-00375</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="95" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="inlineStr">
+    <row r="12" ht="95" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>ToR for Onboarding of consultant/agency for Innovating &amp; Scaling Reproductive Maternal Newborn and Child Health Solutions in the Last-Mile</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>Title Terms of Reference for Onboarding of consultant/agency for Innovating &amp; Scaling Reproductive, Maternal, Newborn and Child Health Solutions in the Last-Mile
+Timeline September 2026 to February 2027
+Scope of Work
+• Outreach and program visibility
+• Application design, launch, review, shortlisting, and due diligence
+• Stakeholder engagement and coordination
+• Knowledge materials and document learnings and insights
+Application Link https://forms.gle/jsngbAREkYmgK7cB6
+Last Date to Apply 5th October, 5 PM
+About SELCO Foundation:
+SELCO Foundation's mission is to create a platform of solutions that uses sustainable energy as a catalyst to bridge environmental sustainability and poverty alleviation. With holistic development as the primary focus, the organization strives to create equitable societies, where services are accessed by all communities. The interventions of SELCO lead to a sustainable delivery model of essential services like livelihoods, education, and health till the last mile.
+(Read more about SELCO here: https://selcofoundation.org/)
+ About the Program
+The program aims to catalyse the development, adoption, and scale of innovative solutions that contribute to improved maternal and child health outcomes. It seeks to build an ecosystem where enterprises and innovators can develop and strengthen technology and technology-allied solutions that enable more accessible, quality, efficient, affordable, and continuous maternal and child health services, particularly across last-mile health facilities and underserved communities.
+The program envisions a future where innovation, technology, and enterprise-led solutions are meaningfully integrated into maternal and child health delivery, enabling health systems, facilities, and frontline health workers to deliver better services to women and children.
+The initiative will bring together enterprises, innovators, health facilities, frontline health workers, institutions, and other ecosystem stakeholders to co-create, test, deploy, and scale solutions with the potential to transform maternal and child health delivery. The focus will be on enabling promising solutions to move beyond individual deployments towards sustainable models of adoption, replication, and scale.
+For the same, we are looking to partner with a like-minded organization that shares this vision and can play an integral role in designing and implementing the initiative. The partner will support enterprise identification and engagement, solution assessment, co-creation, health-system linkages, implementation, stakeholder coordination, evidence generation, and pathways to scale, contributing to more resilient, responsive, and equitable maternal and child health services for women and children.
+ Geography
+Primary Focus: Maharashtra, Karnataka, Odisha, Meghalaya, Mizoram, Nagaland
+Secondary Focus: Other states
+ Selection Criteria
+Applicants should meet the following criteria for being a part of the evaluation:
+Demonstrated experience working with vendors, enterprises, innovators, or solution providers, along with an understanding of grassroots and last-mile contexts and user needs
+Ability to assess enterprise and solution needs and curate tailored mentorship, technical assistance, health-system linkages, and implementation support
+Demonstrated experience in program design, planning, implementation, and management of multi-stakeholder initiatives, preferably in health, maternal and child health, technology, or last-mile service delivery
+Proven ability to manage end-to-end application, assessment, screening, shortlisting, and due diligence processes for a portfolio of enterprises or innovators
+Experience in communication, outreach, stakeholder engagement, and facilitating collaboration between solution providers and health-system stakeholders
+Capability to develop documentation and knowledge products that capture program processes, solution performance, outcomes, implementation models, and learnings for scale and replication
+Prior experience working with development sector organisations, NGOs, health systems, technology providers, enterprises, or think tanks will be considered an added advantage
+The agency will be selected on a combined technical and financial evaluation. Proposals must score a minimum of 70% on the technical components (1–5 below) to be considered for financial evaluation.</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>Oct 5, 2026</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/tor-for-onboarding-of-consultantagency-for-innovating-and-scaling-reproductive-maternal-newborn-and-child-health-solutions-in-the-last-mile-selco-foundation-rfp-26-00373</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="95" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
         <is>
           <t>RFP - Design and Delivery of an Electric Vehicle EV Skilling Programme in Karnataka</t>
         </is>
       </c>
-      <c r="C14" s="1" t="inlineStr">
+      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 WRI India, an independent knowledge organisation registered as the India Resources Trust, provides objective information and practical proposals to foster environmentally sound and socially equitable development. As an independent knowledge organisation, we leverage our data and expertise to catalyze change across systems like food, land and water; energy; and cities. Our work focuses on improving people’s lives, protecting and restoring nature, and addressing climate change. To enable progress at the pace and scale needed, we also engage with the economic, finance and governance systems that are key to enabling this change.
@@ -1258,95 +1212,34 @@
 Must have a team of qualified trainers and master trainers with relevant domain expertise, as well as administrative and coordination support.</t>
         </is>
       </c>
-      <c r="D14" s="1" t="inlineStr">
+      <c r="D13" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E14" s="1" t="inlineStr">
+      <c r="E13" s="1" t="inlineStr">
         <is>
           <t>Oct 5, 2026</t>
         </is>
       </c>
-      <c r="F14" s="1" t="inlineStr">
+      <c r="F13" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfp-design-and-delivery-of-an-electric-vehicle-ev-skilling-programme-in-karnataka-wri-india-rfp-26-00361</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="95" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="inlineStr">
-        <is>
-          <t>ToR for Onboarding of consultant/agency for Innovating &amp; Scaling Reproductive Maternal Newborn and Child Health Solutions in the Last-Mile</t>
-        </is>
-      </c>
-      <c r="C15" s="1" t="inlineStr">
-        <is>
-          <t>Title Terms of Reference for Onboarding of consultant/agency for Innovating &amp; Scaling Reproductive, Maternal, Newborn and Child Health Solutions in the Last-Mile
-Timeline September 2026 to February 2027
-Scope of Work
-• Outreach and program visibility
-• Application design, launch, review, shortlisting, and due diligence
-• Stakeholder engagement and coordination
-• Knowledge materials and document learnings and insights
-Application Link https://forms.gle/jsngbAREkYmgK7cB6
-Last Date to Apply 5th October, 5 PM
-About SELCO Foundation:
-SELCO Foundation's mission is to create a platform of solutions that uses sustainable energy as a catalyst to bridge environmental sustainability and poverty alleviation. With holistic development as the primary focus, the organization strives to create equitable societies, where services are accessed by all communities. The interventions of SELCO lead to a sustainable delivery model of essential services like livelihoods, education, and health till the last mile.
-(Read more about SELCO here: https://selcofoundation.org/)
- About the Program
-The program aims to catalyse the development, adoption, and scale of innovative solutions that contribute to improved maternal and child health outcomes. It seeks to build an ecosystem where enterprises and innovators can develop and strengthen technology and technology-allied solutions that enable more accessible, quality, efficient, affordable, and continuous maternal and child health services, particularly across last-mile health facilities and underserved communities.
-The program envisions a future where innovation, technology, and enterprise-led solutions are meaningfully integrated into maternal and child health delivery, enabling health systems, facilities, and frontline health workers to deliver better services to women and children.
-The initiative will bring together enterprises, innovators, health facilities, frontline health workers, institutions, and other ecosystem stakeholders to co-create, test, deploy, and scale solutions with the potential to transform maternal and child health delivery. The focus will be on enabling promising solutions to move beyond individual deployments towards sustainable models of adoption, replication, and scale.
-For the same, we are looking to partner with a like-minded organization that shares this vision and can play an integral role in designing and implementing the initiative. The partner will support enterprise identification and engagement, solution assessment, co-creation, health-system linkages, implementation, stakeholder coordination, evidence generation, and pathways to scale, contributing to more resilient, responsive, and equitable maternal and child health services for women and children.
- Geography
-Primary Focus: Maharashtra, Karnataka, Odisha, Meghalaya, Mizoram, Nagaland
-Secondary Focus: Other states
- Selection Criteria
-Applicants should meet the following criteria for being a part of the evaluation:
-Demonstrated experience working with vendors, enterprises, innovators, or solution providers, along with an understanding of grassroots and last-mile contexts and user needs
-Ability to assess enterprise and solution needs and curate tailored mentorship, technical assistance, health-system linkages, and implementation support
-Demonstrated experience in program design, planning, implementation, and management of multi-stakeholder initiatives, preferably in health, maternal and child health, technology, or last-mile service delivery
-Proven ability to manage end-to-end application, assessment, screening, shortlisting, and due diligence processes for a portfolio of enterprises or innovators
-Experience in communication, outreach, stakeholder engagement, and facilitating collaboration between solution providers and health-system stakeholders
-Capability to develop documentation and knowledge products that capture program processes, solution performance, outcomes, implementation models, and learnings for scale and replication
-Prior experience working with development sector organisations, NGOs, health systems, technology providers, enterprises, or think tanks will be considered an added advantage
-The agency will be selected on a combined technical and financial evaluation. Proposals must score a minimum of 70% on the technical components (1–5 below) to be considered for financial evaluation.</t>
-        </is>
-      </c>
-      <c r="D15" s="1" t="inlineStr">
-        <is>
-          <t>Learning</t>
-        </is>
-      </c>
-      <c r="E15" s="1" t="inlineStr">
-        <is>
-          <t>Oct 5, 2026</t>
-        </is>
-      </c>
-      <c r="F15" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/tor-for-onboarding-of-consultantagency-for-innovating-and-scaling-reproductive-maternal-newborn-and-child-health-solutions-in-the-last-mile-selco-foundation-rfp-26-00373</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="95" customHeight="1">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B16" s="1" t="inlineStr">
+    <row r="14" ht="95" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>RFPs Invited for Engagement of a Manpower Agency for Providing Subject Matter Specialists/Experts for the Cluster Development Programme</t>
         </is>
       </c>
-      <c r="C16" s="1" t="inlineStr">
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>About the RFP
 National Horticulture Board (NHB), an autonomous organization under the Ministry of Agriculture and Farmers' Welfare, Government of India, invites bids from eligible manpower agencies for engagement to recruit, deploy, and manage qualified personnel supporting NHB's Cluster Development Programme (CDP) — a Central Sector Scheme promoting integrated, market-led horticulture cluster development. The engaged agency will provide three types of Subject Matter Experts per Cluster and additional consultants/manpower as required by NHB from time to time.
@@ -1372,34 +1265,34 @@
  District: Gurugram, Haryana (NHB Head Office)</t>
         </is>
       </c>
-      <c r="D16" s="1" t="inlineStr">
+      <c r="D14" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E16" s="1" t="inlineStr">
+      <c r="E14" s="1" t="inlineStr">
         <is>
           <t>Oct 6, 2026</t>
         </is>
       </c>
-      <c r="F16" s="1" t="inlineStr">
+      <c r="F14" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfps-invited-for-engagement-of-a-manpower-agency-for-providing-subject-matter-specialistsexperts-for-the-cluster-development-programme-national-horticulture-board-nhb-rfp-26-00370</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="95" customHeight="1">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B17" s="1" t="inlineStr">
+    <row r="15" ht="95" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>Applications Open Draper Richards Kaplan Foundation Funding for Social Enterprises</t>
         </is>
       </c>
-      <c r="C17" s="1" t="inlineStr">
+      <c r="C15" s="1" t="inlineStr">
         <is>
           <t>About us
 Started in 2002, Draper Richards Kaplan Foundation (DRK) is a global venture philanthropy firm supporting early stage, high impact social enterprises. Borrowed from our venture capital legacy, DRK finds, funds, and supports exceptional leaders building innovative solutions to some of the world’s most challenging social and environmental problems. Since beginning this work nearly 25 years ago, DRK has invested in more than 270 organizations that have collectively impacted over 610 million lives to date.
@@ -1423,34 +1316,34 @@
 Please attach a standard resume/CV for the entrepreneur(s) and/or key leadership team members (e.g., CEO, COO, ED, etc.). Applications with text bios for entrepreneurs or members of the leadership team will not be considered.</t>
         </is>
       </c>
-      <c r="D17" s="1" t="inlineStr">
+      <c r="D15" s="1" t="inlineStr">
         <is>
           <t>Climate</t>
         </is>
       </c>
-      <c r="E17" s="1" t="inlineStr">
+      <c r="E15" s="1" t="inlineStr">
         <is>
           <t>Oct 10, 2026</t>
         </is>
       </c>
-      <c r="F17" s="1" t="inlineStr">
+      <c r="F15" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-open-draper-richards-kaplan-foundation-funding-for-social-enterprises-draper-richards-kaplan-foundation-opg-26-00188</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="95" customHeight="1">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="inlineStr">
+    <row r="16" ht="95" customHeight="1">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund</t>
         </is>
       </c>
-      <c r="C18" s="1" t="inlineStr">
+      <c r="C16" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund
 Apply by: 13 October, 2026
@@ -1475,34 +1368,34 @@
  Projects should include opportunities for ServiceNow employees to volunteer in the project activation or implementation.</t>
         </is>
       </c>
-      <c r="D18" s="1" t="inlineStr">
+      <c r="D16" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E18" s="1" t="inlineStr">
+      <c r="E16" s="1" t="inlineStr">
         <is>
           <t>Oct 13, 2026</t>
         </is>
       </c>
-      <c r="F18" s="1" t="inlineStr">
+      <c r="F16" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/apply-for-the-servicenow-community-solar-fund-changex-opg-26-00186</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="95" customHeight="1">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="inlineStr">
+    <row r="17" ht="95" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
         <is>
           <t>RFPs Invited for Empanelment of Publishers for Procurement of E-Books for Rashtriya e-Pustakalaya National Book Trust India</t>
         </is>
       </c>
-      <c r="C19" s="1" t="inlineStr">
+      <c r="C17" s="1" t="inlineStr">
         <is>
           <t>About the RFP:
 Rashtriya e-Pustakalaya, a free National Digital Library for children and adolescents — an initiative of the Department of School Education &amp; Literacy, Ministry of Education, Government of India, implemented by the National Book Trust (NBT), India — invites Expression of Interest (EoI) for the empanelment of publishers for the selection and procurement of e-books, with the objective of enriching the platform's book collection. NBT is an autonomous body under the Ministry of Education, established in 1957 to promote literacy and reading culture in India.
@@ -1524,34 +1417,34 @@
 Must indemnify Rashtriya e-Pustakalaya/NBT-India for any IP-related claims from authors/illustrators/translators/legal owners</t>
         </is>
       </c>
-      <c r="D19" s="1" t="inlineStr">
+      <c r="D17" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E19" s="1" t="inlineStr">
+      <c r="E17" s="1" t="inlineStr">
         <is>
           <t>Oct 16, 2026</t>
         </is>
       </c>
-      <c r="F19" s="1" t="inlineStr">
+      <c r="F17" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfps-invited-for-empanelment-of-publishers-for-procurement-of-e-books-for-rashtriya-e-pustakalaya-national-book-trust-india-national-book-trust-nbt-india-rfp-26-00371</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="95" customHeight="1">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="inlineStr">
+    <row r="18" ht="95" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>ToR - Engagement of Consultant/Vendor Individual towards implementation of Literacy Program in Telangana State</t>
         </is>
       </c>
-      <c r="C20" s="1" t="inlineStr">
+      <c r="C18" s="1" t="inlineStr">
         <is>
           <t>ANNEX A – TERMS OF REFERENCE (ToR) 
  Engagement of Consultant/Vendor (Individual) towards implementation of Literacy Program in Telangana State.
@@ -1616,34 +1509,34 @@
 Approved travel and accommodation expenses incurred for assignment-related activities shall be reimbursed by Room to Read in accordance with the consultancy reimbursement guidelines.</t>
         </is>
       </c>
-      <c r="D20" s="1" t="inlineStr">
+      <c r="D18" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E20" s="1" t="inlineStr">
+      <c r="E18" s="1" t="inlineStr">
         <is>
           <t>Oct 16, 2026</t>
         </is>
       </c>
-      <c r="F20" s="1" t="inlineStr">
+      <c r="F18" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-engagement-of-consultantvendor-individual-towards-implementation-of-literacy-program-in-telangana-state-room-to-read-india-rfp-26-00360</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="95" customHeight="1">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="inlineStr">
+    <row r="19" ht="95" customHeight="1">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>RFPs Invited for Consultant to Develop a Technical Assistance Package for National Application of the Digital Health and AI Investment Classification Framework</t>
         </is>
       </c>
-      <c r="C21" s="1" t="inlineStr">
+      <c r="C19" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are Transform Health: a global coalition of more than 200 organisations driving the digital transformation of health to achieve universal health coverage. 
@@ -1671,34 +1564,34 @@
 Ability to manage multi-country consultancy engagements and coordinate with in-country focal points</t>
         </is>
       </c>
-      <c r="D21" s="1" t="inlineStr">
+      <c r="D19" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E21" s="1" t="inlineStr">
+      <c r="E19" s="1" t="inlineStr">
         <is>
           <t>Oct 23, 2026</t>
         </is>
       </c>
-      <c r="F21" s="1" t="inlineStr">
+      <c r="F19" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfps-invited-for-consultant-to-develop-a-technical-assistance-package-for-national-application-of-the-digital-health-and-ai-investment-classification-framework-transform-health-rfp-26-00359</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="95" customHeight="1">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="inlineStr">
+    <row r="20" ht="95" customHeight="1">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for D-Prize Global Competition Seed Funding for New Poverty-Solution Distribution Organizations</t>
         </is>
       </c>
-      <c r="C22" s="1" t="inlineStr">
+      <c r="C20" s="1" t="inlineStr">
         <is>
           <t>About the Grant:
 D-Prize seeds new organizations that distribute proven poverty solutions at the "last mile," with the aim of scaling impact. Applicants select from a range of evidence-based interventions (health, agriculture, education, water, safety, transparency, and more) and propose how they would launch or grow an organization to distribute that intervention. Top entrepreneurs receive up to $20,000 in seed funding to run a pilot and build an organization capable of scaling to reach thousands, even millions of people.
@@ -1721,34 +1614,34 @@
 Extension Deadline: 6 December 2026, midnight PT (extension registration required)</t>
         </is>
       </c>
-      <c r="D22" s="1" t="inlineStr">
+      <c r="D20" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E22" s="1" t="inlineStr">
+      <c r="E20" s="1" t="inlineStr">
         <is>
           <t>Oct 25, 2026</t>
         </is>
       </c>
-      <c r="F22" s="1" t="inlineStr">
+      <c r="F20" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-d-prize-global-competition-seed-funding-for-new-poverty-solution-distribution-organizations-d-prize-opg-26-00191</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="95" customHeight="1">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B23" s="1" t="inlineStr">
+    <row r="21" ht="95" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 8th Call for Proposals Small-Size Grants Global EbA Fund</t>
         </is>
       </c>
-      <c r="C23" s="1" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -1811,34 +1704,34 @@
 Only successful applicants will be contacted; no individual feedback provided to unsuccessful applicants</t>
         </is>
       </c>
-      <c r="D23" s="1" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E23" s="1" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F23" s="1" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-8th-call-for-proposals-small-size-grants-global-eba-fund-global-eba-fund-opg-26-00177</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="95" customHeight="1">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B24" s="1" t="inlineStr">
+    <row r="22" ht="95" customHeight="1">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Adaptive Control Frameworks to Unlock Full-Scale BNR Potential Water Research Foundation WRF</t>
         </is>
       </c>
-      <c r="C24" s="1" t="inlineStr">
+      <c r="C22" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Water Research Foundation (WRF) is the leading research organization advancing the science of all water to meet the evolving needs of its subscribers and the water sector. WRF is a nonprofit, charitable and educational organization which funds, manages, and publishes research on the technology, operation, and management of drinking water, wastewater, reuse, and stormwater collection, treatment and supply systems—all in pursuit of ensuring water quality and improving water services to the public.
@@ -1879,34 +1772,34 @@
 Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
         </is>
       </c>
-      <c r="D24" s="1" t="inlineStr">
+      <c r="D22" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E24" s="1" t="inlineStr">
+      <c r="E22" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F24" s="1" t="inlineStr">
+      <c r="F22" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-adaptive-control-frameworks-to-unlock-full-scale-bnr-potential-water-research-foundation-wrf-the-water-research-foundation-wrf-opg-26-00187</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="95" customHeight="1">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B25" s="1" t="inlineStr">
+    <row r="23" ht="95" customHeight="1">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Crossing the Divide Best Practices for Addressing Local and Privately-Owned Lateral Sewer Issues RFP 5419</t>
         </is>
       </c>
-      <c r="C25" s="1" t="inlineStr">
+      <c r="C23" s="1" t="inlineStr">
         <is>
           <t>Project Objective:
 To provide water resource recovery facilities (WRRFs) and collection system operators with an interactive manual of practice for implementing inflow and infiltration (I&amp;I) and obstruction management programs, focused on municipal and privately owned lateral sewers in complex legal, regulatory, and multi-jurisdictional environments.
@@ -1944,34 +1837,34 @@
  Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
         </is>
       </c>
-      <c r="D25" s="1" t="inlineStr">
+      <c r="D23" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E25" s="1" t="inlineStr">
+      <c r="E23" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F25" s="1" t="inlineStr">
+      <c r="F23" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-crossing-the-divide-best-practices-for-addressing-local-and-privately-owned-lateral-sewer-issues-rfp-5419-the-water-research-foundation-wrf-opg-26-00189</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="95" customHeight="1">
-      <c r="A26" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B26" s="1" t="inlineStr">
+    <row r="24" ht="95" customHeight="1">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Comparison of PFAS Contributions to Agricultural Systems</t>
         </is>
       </c>
-      <c r="C26" s="1" t="inlineStr">
+      <c r="C24" s="1" t="inlineStr">
         <is>
           <t>Project Objectives:
 Report per- and polyfluoroalkyl substance (PFAS) concentrations from a variety of agricultural inputs — animal manures, fertilizers, pesticides, composts, soil amendments, seed coatings, and biosolids-based products
@@ -2007,34 +1900,34 @@
  Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00) — same deadline as the other two WRF grants</t>
         </is>
       </c>
-      <c r="D26" s="1" t="inlineStr">
+      <c r="D24" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E26" s="1" t="inlineStr">
+      <c r="E24" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F26" s="1" t="inlineStr">
+      <c r="F24" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-comparison-of-pfas-contributions-to-agricultural-systems-the-water-research-foundation-wrf-opg-26-00190</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="95" customHeight="1">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B27" s="1" t="inlineStr">
+    <row r="25" ht="95" customHeight="1">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Whitley Award 2027</t>
         </is>
       </c>
-      <c r="C27" s="1" t="inlineStr">
+      <c r="C25" s="1" t="inlineStr">
         <is>
           <t>About the Grant: 
 An annual grant by the Whitley Fund for Nature (WFN) recognising grassroots conservation leaders in the Global South, providing funding to support and scale up proven, science-based solutions that deliver lasting impact for both people and nature.
@@ -2047,34 +1940,34 @@
 You do not need to be invited or nominated to apply.</t>
         </is>
       </c>
-      <c r="D27" s="1" t="inlineStr">
+      <c r="D25" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E27" s="1" t="inlineStr">
+      <c r="E25" s="1" t="inlineStr">
         <is>
           <t>Oct 30, 2026</t>
         </is>
       </c>
-      <c r="F27" s="1" t="inlineStr">
+      <c r="F25" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-whitley-award-2027-whitley-fund-for-nature-wfn-opg-26-00153</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="95" customHeight="1">
-      <c r="A28" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B28" s="1" t="inlineStr">
+    <row r="26" ht="95" customHeight="1">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIFAR Global Scholars Program 20272029 Cohort</t>
         </is>
       </c>
-      <c r="C28" s="1" t="inlineStr">
+      <c r="C26" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 CIFAR is a Canadian-based globally influential research organization that convenes the world’s most brilliant people across disciplines to advance transformative knowledge and solve humanity’s biggest problems, together. By supporting long-term interdisciplinary collaboration, CIFAR provides researchers with an unparalleled environment of trust, transparency and knowledge sharing. Our time-tested model inspires new directions of inquiry, accelerates discovery and yields breakthroughs across borders and academic disciplines. Through knowledge mobilization, we are catalysts for change in industry, government and society. Through our 15 research programs and the Pan-Canadian AI Strategy, CIFAR convenes close to 400 of the world’s top researchers from 141 institutions in 20 countries. CIFAR is generously supported by the governments of Canada, Alberta and Québec, as well as foundations, individuals, corporations and Canadian and international partner organizations.
@@ -2118,34 +2011,73 @@
  Application Deadline: November 4, 2026, 12:00 PM EST</t>
         </is>
       </c>
-      <c r="D28" s="1" t="inlineStr">
+      <c r="D26" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E28" s="1" t="inlineStr">
+      <c r="E26" s="1" t="inlineStr">
         <is>
           <t>Nov 4, 2026</t>
         </is>
       </c>
-      <c r="F28" s="1" t="inlineStr">
+      <c r="F26" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cifar-global-scholars-program-20272029-cohort-cifar-canadian-institute-for-advanced-research-opg-26-00183</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="95" customHeight="1">
-      <c r="A29" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B29" s="1" t="inlineStr">
+    <row r="27" ht="95" customHeight="1">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for IWRS Teaching Innovation Award</t>
         </is>
       </c>
-      <c r="C29" s="1" t="inlineStr">
+      <c r="C27" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
+ About the Grant
+The IWRS (Insect Welfare Research Society) Teaching Innovation Award supports instructors developing new approaches to teaching insect or invertebrate biology that incorporate the 3Rs (Replacement, Reduction, and Refinement) — principles for reducing animal welfare impacts in teaching and research practices.
+ Purpose
+Funds support the creation and implementation of 3Rs-driven instructional materials and pedagogical approaches. Priority is given to proposals addressing common teaching practices with substantial welfare implications.
+ Grant Amount
+Two awards of $2,000 USD are available annually.</t>
+        </is>
+      </c>
+      <c r="D27" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E27" s="1" t="inlineStr">
+        <is>
+          <t>Nov 15, 2026</t>
+        </is>
+      </c>
+      <c r="F27" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="95" customHeight="1">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for IWRS Teaching Innovation Award</t>
+        </is>
+      </c>
+      <c r="C28" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Insects are one of the most numerous and diverse animal groups on Earth.
@@ -2160,73 +2092,34 @@
 IWRS staff and Advisory Group members are not eligible to apply.</t>
         </is>
       </c>
-      <c r="D29" s="1" t="inlineStr">
+      <c r="D28" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E29" s="1" t="inlineStr">
+      <c r="E28" s="1" t="inlineStr">
         <is>
           <t>Nov 15, 2026</t>
         </is>
       </c>
-      <c r="F29" s="1" t="inlineStr">
+      <c r="F28" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00166</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="95" customHeight="1">
-      <c r="A30" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B30" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for IWRS Teaching Innovation Award</t>
-        </is>
-      </c>
-      <c r="C30" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
- About the Grant
-The IWRS (Insect Welfare Research Society) Teaching Innovation Award supports instructors developing new approaches to teaching insect or invertebrate biology that incorporate the 3Rs (Replacement, Reduction, and Refinement) — principles for reducing animal welfare impacts in teaching and research practices.
- Purpose
-Funds support the creation and implementation of 3Rs-driven instructional materials and pedagogical approaches. Priority is given to proposals addressing common teaching practices with substantial welfare implications.
- Grant Amount
-Two awards of $2,000 USD are available annually.</t>
-        </is>
-      </c>
-      <c r="D30" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E30" s="1" t="inlineStr">
-        <is>
-          <t>Nov 15, 2026</t>
-        </is>
-      </c>
-      <c r="F30" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="95" customHeight="1">
-      <c r="A31" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B31" s="1" t="inlineStr">
+    <row r="29" ht="95" customHeight="1">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Medium-Size Grants Call for Proposals Global EbA Fund</t>
         </is>
       </c>
-      <c r="C31" s="1" t="inlineStr">
+      <c r="C29" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -2283,34 +2176,34 @@
 Applications submitted via online portal (link shared on the Medium-Size Grants webpage from Oct 12)</t>
         </is>
       </c>
-      <c r="D31" s="1" t="inlineStr">
+      <c r="D29" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E31" s="1" t="inlineStr">
+      <c r="E29" s="1" t="inlineStr">
         <is>
           <t>Nov 16, 2026</t>
         </is>
       </c>
-      <c r="F31" s="1" t="inlineStr">
+      <c r="F29" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-medium-size-grants-call-for-proposals-global-eba-fund-global-eba-fund-opg-26-00178</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="95" customHeight="1">
-      <c r="A32" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B32" s="1" t="inlineStr">
+    <row r="30" ht="95" customHeight="1">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIEIF Grant 2026 Climate Intervention Environmental Impact Fund</t>
         </is>
       </c>
-      <c r="C32" s="1" t="inlineStr">
+      <c r="C30" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Climate Intervention Environmental Impact Fund (CIEIF) is a philanthropic fund focused on supporting responsible climate intervention field tests. It provides grants for activities such as environmental impact assessment (EIA), predictive impact modelling, and engagement with potentially affected stakeholders, including local communities and government agencies.
@@ -2337,34 +2230,34 @@
 Potential for scaling the innovation to a globally relevant level</t>
         </is>
       </c>
-      <c r="D32" s="1" t="inlineStr">
+      <c r="D30" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E32" s="1" t="inlineStr">
+      <c r="E30" s="1" t="inlineStr">
         <is>
           <t>Dec 1, 2026</t>
         </is>
       </c>
-      <c r="F32" s="1" t="inlineStr">
+      <c r="F30" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cieif-grant-2026-climate-intervention-environmental-impact-fund-climate-intervention-environmental-impact-fund-opg-26-00155</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="95" customHeight="1">
-      <c r="A33" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B33" s="1" t="inlineStr">
+    <row r="31" ht="95" customHeight="1">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 6th Annual Seeding The Future Global Food System Challenge</t>
         </is>
       </c>
-      <c r="C33" s="1" t="inlineStr">
+      <c r="C31" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are one of the largest and most respected private organisations for development cooperation and humanitarian aid in Germany. As a politically and confessionally independent organisation, our value-oriented actions are always based on ethical principles. Our vision is clear: "Zero Hunger by 2030"
@@ -2396,34 +2289,34 @@
 Individuals with no organizational entity</t>
         </is>
       </c>
-      <c r="D33" s="1" t="inlineStr">
+      <c r="D31" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E33" s="1" t="inlineStr">
+      <c r="E31" s="1" t="inlineStr">
         <is>
           <t>Jan 1, 2027</t>
         </is>
       </c>
-      <c r="F33" s="1" t="inlineStr">
+      <c r="F31" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-6th-annual-seeding-the-future-global-food-system-challenge-welthungerhilfe-opg-26-00180</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="95" customHeight="1">
-      <c r="A34" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B34" s="1" t="inlineStr">
+    <row r="32" ht="95" customHeight="1">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B32" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Microbiota &amp; Women's Health International Call for Projects</t>
         </is>
       </c>
-      <c r="C34" s="1" t="inlineStr">
+      <c r="C32" s="1" t="inlineStr">
         <is>
           <t>About the Grant
 An annual international research grant by the Biocodex Microbiota Foundation (BMF), rewarding research proposals on the microbiota and its implications in Women's Health and Disease. This year's theme: "Unraveling male-female genital microbiome interactions: mechanisms, transmission, and impact on vaginal dysbiosis."
@@ -2440,34 +2333,34 @@
 €200,000 annually — awarded to researchers within universities, hospitals, or other research settings to finance equipment, operations, or staffing costs. Grants are NOT awarded to individuals directly (must be institutionally affiliated). Institution's overhead costs capped at 10%.</t>
         </is>
       </c>
-      <c r="D34" s="1" t="inlineStr">
+      <c r="D32" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E34" s="1" t="inlineStr">
+      <c r="E32" s="1" t="inlineStr">
         <is>
           <t>Jan 15, 2027</t>
         </is>
       </c>
-      <c r="F34" s="1" t="inlineStr">
+      <c r="F32" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-microbiota-and-womens-health-international-call-for-projects-biocodex-microbiota-foundation-bmf-opg-26-00152</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="95" customHeight="1">
-      <c r="A35" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B35" s="1" t="inlineStr">
+    <row r="33" ht="95" customHeight="1">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B33" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for BES Training and Travel Grants</t>
         </is>
       </c>
-      <c r="C35" s="1" t="inlineStr">
+      <c r="C33" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are a global community of scientists shining a spotlight on the intricacy and value of our natural world, providing the evidence for better decisions. Our vision is for people and nature to thrive in a world that values ecology.
@@ -2506,17 +2399,17 @@
  Application Deadline (Round 2): Opens 30 April 2026, closes 17 May 2026</t>
         </is>
       </c>
-      <c r="D35" s="1" t="inlineStr">
+      <c r="D33" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E35" s="1" t="inlineStr">
+      <c r="E33" s="1" t="inlineStr">
         <is>
           <t>May 17, 2027</t>
         </is>
       </c>
-      <c r="F35" s="1" t="inlineStr">
+      <c r="F33" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-bes-training-and-travel-grants-british-ecological-society-opg-26-00181</t>
         </is>

</xml_diff>

<commit_message>
Auto update Combined.xlsx [Mon Sep 28 08:08:09 UTC 2026]
</commit_message>
<xml_diff>
--- a/output/Combined.xlsx
+++ b/output/Combined.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>District Coordination Associate</t>
+          <t>State Project Coordinator</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
@@ -478,12 +478,12 @@
       <c r="D2" s="1" t="inlineStr"/>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>10/10/2026, 03:59 AM</t>
+          <t>10/12/2026, 03:59 AM</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://estm.fa.em2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1/job/37155/?location=India&amp;locationId=300000000440677&amp;locationLevel=country&amp;mode=location</t>
+          <t>https://estm.fa.em2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1/job/37164/?location=India&amp;locationId=300000000440677&amp;locationLevel=country&amp;mode=location</t>
         </is>
       </c>
     </row>
@@ -495,165 +495,10 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>RFP - Engagement of Agency for Development of MIS Dashboard and Mobile-based Application for Adolescent Mental Health</t>
+          <t>EOI Inviting Expression of Interest-cum-Proposal for Setting Up District De-Addiction Centres under NAPDDR</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t>Release of Request for Proposal
-23rd September 2026
-Pre-bid Meeting (Online) Date
-25th September 2026 
-Pre-Bid Link for Registration: 
- Pre-Bid Meeting date and time
-25.9.26 @ 5:30 PM
-https://forms.gle/DiwgwoKZzwzYHAsL7
- Pre-bid Meeting Link
-meet.google.com/dgb-mjez-wam
-  Bid Submission Closing Date
-29th September 2026 (23:59 Hrs. IST)
-Please submit proposals
- in the following respective Google Forms -
-Technical: https://forms.gle/96REn8vzjEJ7uEPp6
-Financial: https://forms.gle/Hz7pLBp7iS86Eovu9
-Technical Bid Opening
-30th September 2026
-Financial Bid Opening
-  Finalization of Contract
-TBD
-(to be intimated to the awardee only)
-Scope of Work:
-Terms of Reference for Development of MIS Dashboard and Android-based Mobile Application for Adolescent Mental Health Programme in Madhya Pradesh
- For the Adolescent Mental Health and Well-being Programme, AIFT requires the development of a new Android-based mobile application and a web-based Management Information System (MIS) dashboard. The mobile application will enable adolescents to access age-appropriate learning modules, undertake mental health screening, and connect with mental health support services, wherever required. The MIS dashboard will support programme implementation by enabling counsellors and project staff to record programme activities, monitor school-based interventions, and generate implementation reports.
- THE AMERICAN INDIA FOUNDATION TRUST (AIFT) intends to engage an agency to design, develop, test and deploy the mobile application and the MIS dashboard as per the requirements shared by AIFT. As this is a time-sensitive requirement, preference will be given to agencies that already have a working application and dashboard of this kind, which can be customized and deployed quickly. The scope of work will include requirement assessment and design, end-to-end development of the application and dashboard, testing and piloting, deployment and handover, training of users, and, after go-live, maintenance, technical support, data support and documentation to facilitate effective implementation and scale-up of the intervention.
- The selected agency shall design, develop and deploy the mobile application and MIS dashboard, and thereafter provide maintenance, technical and operational support till 30th September 2029, subject to fulfilment of the conditions of the bid and the funding for the programme.
- Proposal Requirement:
-The technical proposal should cover at least below areas:
- Applicant eligibility requirement(s):
-The bidder organization should be registered as a legal entity for doing business in India.
-The applicant must have demonstrated ability to provide expert advice and should have at least 3 years of experience in custom software development, or relevant experience in developing a similar mental health application.
-The bidder must have demonstrated experience in designing, developing and deploying mobile applications in the field of adolescent mental health, with at least one similar application developed and implemented within the last three years.
-Preference will be given to bidders who already have a working adolescent mental health mobile application and MIS dashboard that can be customized and deployed for AIFT within a short time, as this is a time-sensitive requirement.
-The bidder should have experience in designing and developing web-based Management Information System (MIS) dashboards for programme monitoring, reporting and data management, preferably for health or social sector programmes.
-The mobile application to be developed must support multilingual functionality (at minimum Hindi and English), and the bidder should have prior experience in developing multilingual mobile applications.
-The bidder should have proven experience across the full development cycle (requirement analysis, UI/UX design, development, testing and deployment), as well as post-deployment maintenance and technical support for mobile applications and dashboards.
-Preference will be given to agencies with prior experience of working with Government departments, development partners, NGOs, or international organizations in implementing digital health or mental health programmes.
- Technical Requirements:
-The bidder should provide information in English language on overall qualifications, including:
-Profile of organization
-Past experience, clients handled and completed assignments.
-Services and support available post-delivery of Services
-Technical Proposal covering the proposed approach, technical architecture, technology stack and time required to go-live (maximum limit of 10-12 pages)
-Details of the bidder’s existing adolescent mental health mobile application and MIS dashboard (key features, screenshots, demo link/credentials and current deployments), along with confirmation of availability for a live demonstration
-At least two references of clients (contact email id/ phone)
-Views on the RFP requirements – Agreement and suggestions to the scope of work outlined in Section III (not more than 5 pages)
-Profile of team members proposed for the project (not more than 2 pages)
-Any other relevant information (not more than 1 page)
-Only for-profit entities can apply. Nonprofit entities (NGO) are not eligible to apply under this bid.
- Attachments/ Enclosures for Technical Bid:
-Bid must be submitted in English language only and should contain:
-Covering letter with reference to all enclosures or attachments.
-Copy of registration documents/ certificate and most recent renewal as a legal entity.
-License or permission if any for doing business with computers.
-Copy of PAN &amp; TAN.
-Copy of GST Registration.
-Copy of MSME registration certificate (if registered)
-Copies of last three years ITR. (exempted for startup raised within last two year)
-All Bid must contain the complete address of firm, including contact number/ email ID of the person who is authorized to submit the bid under their signatures.
-Technical bid form as per Annexure I
- Financial Bid
-It is to be submitted separately as per Annexure II. No conditional price is to be quoted.</t>
-        </is>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>Sep 29, 2026</t>
-        </is>
-      </c>
-      <c r="F3" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/rfp-engagement-of-agency-for-development-of-mis-dashboard-and-mobile-based-application-for-adolescent-mental-health-american-india-foundation-rfp-26-00372</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="95" customHeight="1">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>ToR - Video Production Storytelling and Documentation</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>Title Video Production – Storytelling and Documentation
-Timeline 3 months from the date of contracting
-Expected area of expertise Video production, documentary storytelling, interviews, field documentation, cinematography and post-production
-Apply Link https://forms.gle/qiATVNrSkDJrkNH3A
-Last      Date             for Apply 29th September 2026 by 5 PM
-About SELCO Foundation:
-SELCO Foundation’s mission is to create a platform of solutions that uses sustainable energy as a catalyst to bridge environmental sustainability and poverty alleviation. With holistic development as the primary focus, the organization strives to create equitable societies, where services are accessed by all communities. The interventions of SELCO lead to a sustainable delivery model of essential services like livelihoods, education, and health till the last mile. (Read more about SELCO here: http://www.selcofoundation.org/)
- About the Programmes:
-SELCO Foundation is looking to engage a video production partner to develop a series of compelling videos that document and communicate stories emerging from its programmes and field interventions.
-The assignment will involve end-to-end video production, including story development, filming, interviews, visual documentation, editing and post-production. The videos will highlight people, experiences, solutions, impact and the broader context of the organisation's work.
-The final content will be used across digital platforms, social media, events, presentations, reports and other communication channels
- Objective:
-To produce a series of compelling videos that document programme experiences, end-user journeys and solutions in a clear, engaging and accessible manner.
-The videos should move beyond activity documentation to capture the context, challenge, solution, experience and outcomes of the people and communities being documented.
-The selected partner will be expected to provide:
-Story treatment/concept notes
-Interview questions and filming plan
-Raw footage from all filming
-Edited full-length video
-Edited short version
-30-second trailer
-Subtitled versions, where required
-Final master files in agreed resolution and formats
-Social-media-ready versions, where required
-Project/source files upon completion
- Submission Requirements:
-Interested production partners are requested to submit the following by before deadline
-Organizational/Individual Profile: Overview of your team/experience.Proposed Approach: A brief document outlining your understanding of the assignment and your proposed approach to storytelling and production.
-Relevant Portfolio: 3–5 relevant video samples demonstrating documentary, impact, social-sector, development or human-interest storytelling.Experience with Similar Assignments: Details of relevant video production and field documentation work.
-Quotation Should include all cost including Travel and Miscellaneous.</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>Learning</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="inlineStr">
-        <is>
-          <t>Sep 29, 2026</t>
-        </is>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/tor-video-production-storytelling-and-documentation-selco-foundation-rfp-26-00368</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="95" customHeight="1">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>EOI Inviting Expression of Interest-cum-Proposal for Setting Up District De-Addiction Centres under NAPDDR</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>About us
 In the year 1985-86, the erstwhile Ministry of Welfare was bifurcated into the Department of Women and Child Development and the Department of Welfare. Simultaneously, the Scheduled Castes Development Division, Tribal Development Division and the Minorities and Backward Classes Welfare Division were moved from the Ministry of Home Affairs and also the Wakf Division from the Ministry of Law to form the then Ministry of Welfare Subsequently, the name of the Ministry was changed to the Ministry of Social Justice &amp; Empowerment in May, 1998. Further, in October, 1999, the Tribal Development Division had moved out to form a separate Ministry of Tribal Affairs. In January, 2007, the Minorities Division along with Wakf Unit have been moved out of the Ministry and formed as a separate Ministry and the Child Development Division has gone to the Ministry of Women &amp; Child Development.
@@ -693,150 +538,34 @@
 11. Department of Social Justice and Empowerment (DoSJE) reserves the right to cancel this notice, andior invite afresh proposals with or without amendments to this document without liability or any obligation for such document, and without assigning any reason. DoSJE reserves the right to take final decision regarding selection of implementing agency or project.</t>
         </is>
       </c>
-      <c r="D5" s="1" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E5" s="1" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F5" s="1" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/eoi-inviting-expression-of-interest-cum-proposal-for-setting-up-district-de-addiction-centres-under-napddr-ministry-of-social-justice-and-empowerment-goi-rfp-26-00356</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="95" customHeight="1">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Setting up Viral Research and Diagnosis Laboratories VRDL in Medical Colleges/Hospitals/Medical Institutions</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-The President notified the creation of the Department of Health Research under the Ministry of Health &amp; Family Welfare through an amendment to the Government of India (Allocation of Business) Rules, 1961 on the 17th September 2007. The Department of Health Research was formally launched on 5th October 2007 by the Minister for Science &amp; Technology and Earth Sciences in a function presided over by the Minister for Health &amp; Family Welfare, in the presence, inter-alia, of the Minister of State for Health &amp; Family Welfare.
-The Department became functional from November 2008 with the appointment of first Secretary of the Department The aim of the DHR is to bring modern health technologies to the people through research and innovations related to diagnosis, treatment methods and vaccines for prevention, to translate them into products and processes and, in synergy with concerned organizations, introduce these innovations into public health system.
- About the Opportunity:
-Under DHR's scheme "Setting-up of nation-wide network of laboratories for managing epidemics and national calamities," proposals are invited from Medical Colleges/Hospitals/Research Institutions to establish a Medical College &amp; Research Institute Level – Viral Research and Diagnosis Laboratory (MCL-VRDL). The existing network comprises 167 VRDLs (11 Regional, 27 State, 129 Medical College level) across 27 states and 5 UTs, aimed at early detection of infectious pathogens, outbreak surveillance, and research on emerging/re-emerging viral diseases.
- Objectives:
-Establish capacity for early detection of common and high-risk infectious pathogens
-Strengthen syndromic surveillance ecosystem for outbreak detection
-Undertake R&amp;D on emerging, re-emerging and novel viruses
- Eligibility (Institution-level):
-State Government Medical Colleges
-Central Government Medical Colleges and Research Institutes
-Armed Forces Medical Institutions/Hospitals
-Railway and other Central Government health institutions
-Private medical colleges ranked in top 50 NIRF ranking
-Must have a dedicated Microbiology department with qualified faculty
-Must have &gt;200 sq.m. area available in existing building (preferably within Microbiology Dept.)
- Funding Provision:
-Non-recurring assistance: Rs. 1.55 crore total
-Rs. 66.8 lakhs — Civil Work (infrastructure modification)
-Rs. 88.2 lakhs — Equipment (complete lab setup)
-No recurring expenditure (staff salaries, consumables, contingency) is provided — to be borne by the host institution
- Role &amp; Responsibilities of the Lab:
-Conduct routine diagnosis of infectious pathogens
-Participate in syndromic and event-based surveillance
-Provide support during outbreaks/epidemics
-Share data with ICMR
- Selection Criteria:
-Meeting eligibility does not guarantee selection; merit-based evaluation by a technical committee
-Preference to institutions in geographically underserved regions
-Weightage for technical strength (qualified faculty, biosafety practices, outbreak investigation experience, publications, patents, externally funded projects)
-Additional weightage for molecular diagnostics, genomic surveillance, One Health research capability, and commitment to long-term recurring support
-Private medical colleges: only top-50 NIRF-ranked institutions considered</t>
-        </is>
-      </c>
-      <c r="D6" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E6" s="1" t="inlineStr">
-        <is>
-          <t>Sep 30, 2026</t>
-        </is>
-      </c>
-      <c r="F6" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-setting-up-viral-research-and-diagnosis-laboratories-vrdl-in-medical-collegeshospitalsmedical-institutions-department-of-health-research-dhr-ministry-of-health-and-family-welfare-government-of-india-opg-26-00174</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="95" customHeight="1">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Signals of Change Shaping the Future of Sexual and Reproductive Health and Rights SRHR</t>
-        </is>
-      </c>
-      <c r="C7" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-The World Health Organization's mission: to promote health, keep the world safe, and serve the vulnerable. Working through offices in more than 150 countries, WHO staff work side by side with governments and other partners to ensure the highest attainable level of health for all people.
- About the Opportunity
-HRP and its UN co-sponsors are leading a global Sexual and Reproductive Health and Rights (SRHR) foresight and research prioritization process for 2026–2036. This open public consultation invites diverse stakeholder input to identify "signals of change" — emerging trends, shifts, or disruptions — that could shape the future of SRHR over the next decade. The process uses foresight methodology (not prediction) to explore plausible futures and will culminate in a published report and research agenda in 2027.
- Guiding Questions
-What future trends will shape or constrain SRHR over the next 10 years?
-What evidence and research investments are needed today to prepare SRHR for the futures we may face?
- Scope of Submissions 
-Economic systems; social infrastructure; structural discrimination; conflict/forced migration/displacement; mega-trends (demographic shifts, climate change, digital transformation/AI, urbanization); conditions of daily life; rights/legal/governance systems; health systems; media/misinformation; and changes in the research ecosystem.
- Who Can Participate 
-Open to individuals and organizations globally, including:
-Health workers, professional associations, clinical networks
-Civil society, community groups, youth-led organizations, rights movements
-Governments, parliamentarians, regulators, public sector bodies
-Researchers, academia, think tanks, technical experts
-UN agencies, multilateral/humanitarian/development organizations
-Funders, philanthropy, private sector, tech/innovation organizations
-Media, communications, journalism
-Anyone with relevant lived experience or perspective
-Special interest in submissions from health worker, community, youth, and rights-movement spaces not typically represented in published forums.
- Submission Requirements: Descriptive information (name, contact email, country, sector) required alongside each submission; formal published evidence is helpful but not required — practice-based experience and field examples are also welcome. Submissions are kept confidential and anonymized before analysis.</t>
-        </is>
-      </c>
-      <c r="D7" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E7" s="1" t="inlineStr">
-        <is>
-          <t>Sep 30, 2026</t>
-        </is>
-      </c>
-      <c r="F7" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-signals-of-change-shaping-the-future-of-sexual-and-reproductive-health-and-rights-srhr-world-health-organization-opg-26-00176</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="95" customHeight="1">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
+    <row r="4" ht="95" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>ToR - Branding Development &amp; Design/Market Promotion Consultant Project Sashakt</t>
         </is>
       </c>
-      <c r="C8" s="1" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>Organisation Humana People to People India (HPPI)
 Project Sashakt – Strengthening Women-led Handloom Cooperatives in Assam (EU-funded)
@@ -891,34 +620,34 @@
 The consultant/agency must ensure ethical, consent-based data collection with cultural sensitivity, particularly when engaging women weavers. All data and reports remain the property of HPPI and must be kept strictly confidential, with no external use.</t>
         </is>
       </c>
-      <c r="D8" s="1" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E8" s="1" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F8" s="1" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-branding-development-and-designmarket-promotion-consultant-project-sashakt-humana-people-to-people-india-rfp-26-00365</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="95" customHeight="1">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="inlineStr">
+    <row r="5" ht="95" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>Application Invited for Giving Joy Microgrant</t>
         </is>
       </c>
-      <c r="C9" s="1" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Giving Joy is a US-based nonprofit that strengthens and inspires women’s entrepreneurship worldwide. Through its micro-grants and mentorship program, Giving Joy helps women establish or improve their businesses and initiatives—for their benefit and the benefit of their communities. To date, Giving Joy has awarded over 88 grants to women-led initiatives in 26 countries.
@@ -957,34 +686,150 @@
 The grant period is six months.</t>
         </is>
       </c>
-      <c r="D9" s="1" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E9" s="1" t="inlineStr">
+      <c r="E5" s="1" t="inlineStr">
         <is>
           <t>Sep 30, 2026</t>
         </is>
       </c>
-      <c r="F9" s="1" t="inlineStr">
+      <c r="F5" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/application-invited-for-giving-joy-microgrant-giving-joy-opg-26-00185</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="95" customHeight="1">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
+    <row r="6" ht="95" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Signals of Change Shaping the Future of Sexual and Reproductive Health and Rights SRHR</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+The World Health Organization's mission: to promote health, keep the world safe, and serve the vulnerable. Working through offices in more than 150 countries, WHO staff work side by side with governments and other partners to ensure the highest attainable level of health for all people.
+ About the Opportunity
+HRP and its UN co-sponsors are leading a global Sexual and Reproductive Health and Rights (SRHR) foresight and research prioritization process for 2026–2036. This open public consultation invites diverse stakeholder input to identify "signals of change" — emerging trends, shifts, or disruptions — that could shape the future of SRHR over the next decade. The process uses foresight methodology (not prediction) to explore plausible futures and will culminate in a published report and research agenda in 2027.
+ Guiding Questions
+What future trends will shape or constrain SRHR over the next 10 years?
+What evidence and research investments are needed today to prepare SRHR for the futures we may face?
+ Scope of Submissions 
+Economic systems; social infrastructure; structural discrimination; conflict/forced migration/displacement; mega-trends (demographic shifts, climate change, digital transformation/AI, urbanization); conditions of daily life; rights/legal/governance systems; health systems; media/misinformation; and changes in the research ecosystem.
+ Who Can Participate 
+Open to individuals and organizations globally, including:
+Health workers, professional associations, clinical networks
+Civil society, community groups, youth-led organizations, rights movements
+Governments, parliamentarians, regulators, public sector bodies
+Researchers, academia, think tanks, technical experts
+UN agencies, multilateral/humanitarian/development organizations
+Funders, philanthropy, private sector, tech/innovation organizations
+Media, communications, journalism
+Anyone with relevant lived experience or perspective
+Special interest in submissions from health worker, community, youth, and rights-movement spaces not typically represented in published forums.
+ Submission Requirements: Descriptive information (name, contact email, country, sector) required alongside each submission; formal published evidence is helpful but not required — practice-based experience and field examples are also welcome. Submissions are kept confidential and anonymized before analysis.</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>Sep 30, 2026</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-signals-of-change-shaping-the-future-of-sexual-and-reproductive-health-and-rights-srhr-world-health-organization-opg-26-00176</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="95" customHeight="1">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Setting up Viral Research and Diagnosis Laboratories VRDL in Medical Colleges/Hospitals/Medical Institutions</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+The President notified the creation of the Department of Health Research under the Ministry of Health &amp; Family Welfare through an amendment to the Government of India (Allocation of Business) Rules, 1961 on the 17th September 2007. The Department of Health Research was formally launched on 5th October 2007 by the Minister for Science &amp; Technology and Earth Sciences in a function presided over by the Minister for Health &amp; Family Welfare, in the presence, inter-alia, of the Minister of State for Health &amp; Family Welfare.
+The Department became functional from November 2008 with the appointment of first Secretary of the Department The aim of the DHR is to bring modern health technologies to the people through research and innovations related to diagnosis, treatment methods and vaccines for prevention, to translate them into products and processes and, in synergy with concerned organizations, introduce these innovations into public health system.
+ About the Opportunity:
+Under DHR's scheme "Setting-up of nation-wide network of laboratories for managing epidemics and national calamities," proposals are invited from Medical Colleges/Hospitals/Research Institutions to establish a Medical College &amp; Research Institute Level – Viral Research and Diagnosis Laboratory (MCL-VRDL). The existing network comprises 167 VRDLs (11 Regional, 27 State, 129 Medical College level) across 27 states and 5 UTs, aimed at early detection of infectious pathogens, outbreak surveillance, and research on emerging/re-emerging viral diseases.
+ Objectives:
+Establish capacity for early detection of common and high-risk infectious pathogens
+Strengthen syndromic surveillance ecosystem for outbreak detection
+Undertake R&amp;D on emerging, re-emerging and novel viruses
+ Eligibility (Institution-level):
+State Government Medical Colleges
+Central Government Medical Colleges and Research Institutes
+Armed Forces Medical Institutions/Hospitals
+Railway and other Central Government health institutions
+Private medical colleges ranked in top 50 NIRF ranking
+Must have a dedicated Microbiology department with qualified faculty
+Must have &gt;200 sq.m. area available in existing building (preferably within Microbiology Dept.)
+ Funding Provision:
+Non-recurring assistance: Rs. 1.55 crore total
+Rs. 66.8 lakhs — Civil Work (infrastructure modification)
+Rs. 88.2 lakhs — Equipment (complete lab setup)
+No recurring expenditure (staff salaries, consumables, contingency) is provided — to be borne by the host institution
+ Role &amp; Responsibilities of the Lab:
+Conduct routine diagnosis of infectious pathogens
+Participate in syndromic and event-based surveillance
+Provide support during outbreaks/epidemics
+Share data with ICMR
+ Selection Criteria:
+Meeting eligibility does not guarantee selection; merit-based evaluation by a technical committee
+Preference to institutions in geographically underserved regions
+Weightage for technical strength (qualified faculty, biosafety practices, outbreak investigation experience, publications, patents, externally funded projects)
+Additional weightage for molecular diagnostics, genomic surveillance, One Health research capability, and commitment to long-term recurring support
+Private medical colleges: only top-50 NIRF-ranked institutions considered</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>Sep 30, 2026</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-setting-up-viral-research-and-diagnosis-laboratories-vrdl-in-medical-collegeshospitalsmedical-institutions-department-of-health-research-dhr-ministry-of-health-and-family-welfare-government-of-india-opg-26-00174</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="95" customHeight="1">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>ToR - Project Management Unit Solarization of Women-led Livelihoods in Maharashtra MAVIMSELCO Foundation Short Duration Project</t>
         </is>
       </c>
-      <c r="C10" s="1" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>Title Project Management Unit – Solarization of Women-led Livelihoods in Maharashtra (MAVIM–SELCO Foundation Short Duration Project)
 Timeline 6 Months (Oct – Mar)
@@ -1025,34 +870,34 @@
 Examples of similar past projects, particularly involving SHG networks, livelihood programs, or energy access.</t>
         </is>
       </c>
-      <c r="D10" s="1" t="inlineStr">
+      <c r="D8" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E10" s="1" t="inlineStr">
+      <c r="E8" s="1" t="inlineStr">
         <is>
           <t>Oct 3, 2026</t>
         </is>
       </c>
-      <c r="F10" s="1" t="inlineStr">
+      <c r="F8" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-project-management-unit-solarization-of-women-led-livelihoods-in-maharashtra-mavimselco-foundation-short-duration-project-selco-foundation-rfp-26-00374</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="95" customHeight="1">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="inlineStr">
+    <row r="9" ht="95" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
         <is>
           <t>EOI - Engagement of Agencies for HR Recruitment Services</t>
         </is>
       </c>
-      <c r="C11" s="1" t="inlineStr">
+      <c r="C9" s="1" t="inlineStr">
         <is>
           <t>The American India Foundation Trust (AIFT) seeks to engage an experienced recruitment agency to provide end-to-end recruitment and talent acquisition services for identified positions across its offices, programmes, and functions in India.
 The selected agency shall support AIFT in sourcing, screening, shortlisting, interview coordination, candidate engagement, offer management, and recruitment closure, in accordance with the requirements, timelines, and service levels agreed with AIFT.
@@ -1083,95 +928,73 @@
 Any other information specifically requested by AIFT.</t>
         </is>
       </c>
-      <c r="D11" s="1" t="inlineStr">
+      <c r="D9" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E11" s="1" t="inlineStr">
+      <c r="E9" s="1" t="inlineStr">
         <is>
           <t>Oct 4, 2026</t>
         </is>
       </c>
-      <c r="F11" s="1" t="inlineStr">
+      <c r="F9" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/eoi-engagement-of-agencies-for-hr-recruitment-services-american-india-foundation-rfp-26-00375</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="95" customHeight="1">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="inlineStr">
-        <is>
-          <t>ToR for Onboarding of consultant/agency for Innovating &amp; Scaling Reproductive Maternal Newborn and Child Health Solutions in the Last-Mile</t>
-        </is>
-      </c>
-      <c r="C12" s="1" t="inlineStr">
-        <is>
-          <t>Title Terms of Reference for Onboarding of consultant/agency for Innovating &amp; Scaling Reproductive, Maternal, Newborn and Child Health Solutions in the Last-Mile
-Timeline September 2026 to February 2027
-Scope of Work
-• Outreach and program visibility
-• Application design, launch, review, shortlisting, and due diligence
-• Stakeholder engagement and coordination
-• Knowledge materials and document learnings and insights
-Application Link https://forms.gle/jsngbAREkYmgK7cB6
-Last Date to Apply 5th October, 5 PM
-About SELCO Foundation:
-SELCO Foundation's mission is to create a platform of solutions that uses sustainable energy as a catalyst to bridge environmental sustainability and poverty alleviation. With holistic development as the primary focus, the organization strives to create equitable societies, where services are accessed by all communities. The interventions of SELCO lead to a sustainable delivery model of essential services like livelihoods, education, and health till the last mile.
-(Read more about SELCO here: https://selcofoundation.org/)
- About the Program
-The program aims to catalyse the development, adoption, and scale of innovative solutions that contribute to improved maternal and child health outcomes. It seeks to build an ecosystem where enterprises and innovators can develop and strengthen technology and technology-allied solutions that enable more accessible, quality, efficient, affordable, and continuous maternal and child health services, particularly across last-mile health facilities and underserved communities.
-The program envisions a future where innovation, technology, and enterprise-led solutions are meaningfully integrated into maternal and child health delivery, enabling health systems, facilities, and frontline health workers to deliver better services to women and children.
-The initiative will bring together enterprises, innovators, health facilities, frontline health workers, institutions, and other ecosystem stakeholders to co-create, test, deploy, and scale solutions with the potential to transform maternal and child health delivery. The focus will be on enabling promising solutions to move beyond individual deployments towards sustainable models of adoption, replication, and scale.
-For the same, we are looking to partner with a like-minded organization that shares this vision and can play an integral role in designing and implementing the initiative. The partner will support enterprise identification and engagement, solution assessment, co-creation, health-system linkages, implementation, stakeholder coordination, evidence generation, and pathways to scale, contributing to more resilient, responsive, and equitable maternal and child health services for women and children.
- Geography
-Primary Focus: Maharashtra, Karnataka, Odisha, Meghalaya, Mizoram, Nagaland
-Secondary Focus: Other states
- Selection Criteria
-Applicants should meet the following criteria for being a part of the evaluation:
-Demonstrated experience working with vendors, enterprises, innovators, or solution providers, along with an understanding of grassroots and last-mile contexts and user needs
-Ability to assess enterprise and solution needs and curate tailored mentorship, technical assistance, health-system linkages, and implementation support
-Demonstrated experience in program design, planning, implementation, and management of multi-stakeholder initiatives, preferably in health, maternal and child health, technology, or last-mile service delivery
-Proven ability to manage end-to-end application, assessment, screening, shortlisting, and due diligence processes for a portfolio of enterprises or innovators
-Experience in communication, outreach, stakeholder engagement, and facilitating collaboration between solution providers and health-system stakeholders
-Capability to develop documentation and knowledge products that capture program processes, solution performance, outcomes, implementation models, and learnings for scale and replication
-Prior experience working with development sector organisations, NGOs, health systems, technology providers, enterprises, or think tanks will be considered an added advantage
-The agency will be selected on a combined technical and financial evaluation. Proposals must score a minimum of 70% on the technical components (1–5 below) to be considered for financial evaluation.</t>
-        </is>
-      </c>
-      <c r="D12" s="1" t="inlineStr">
-        <is>
-          <t>Learning</t>
-        </is>
-      </c>
-      <c r="E12" s="1" t="inlineStr">
-        <is>
-          <t>Oct 5, 2026</t>
-        </is>
-      </c>
-      <c r="F12" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/tor-for-onboarding-of-consultantagency-for-innovating-and-scaling-reproductive-maternal-newborn-and-child-health-solutions-in-the-last-mile-selco-foundation-rfp-26-00373</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="95" customHeight="1">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B13" s="1" t="inlineStr">
+    <row r="10" ht="95" customHeight="1">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>ToR - Landscape Study for Foundational Literacy and Numeracy FLN Program Six Districts-Jharkhand</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>Organizational Overview
+Founded in 2000 on the belief that World Change Starts with Educated Children®, Room to Read develops children’s foundational literacy skills, as well as life skills that promote gender equality. We nurture these essential skills in children by training and coaching educators, creating quality learning materials and spaces, strengthening education systems, and delivering programs directly and with partners – all while honouring the dignity of every child. Committed to accelerating learning outcomes for more children, more quickly, Room to Read has benefited children across 29 countries, with more than 17 million children actively benefiting from our programming in 2025 alone. Room to Read India’s literacy operations currently span across 12 states, with a focus on improving children’s reading skills, access to quality learning materials, and supportive learning environments. Room to Read envisions a world free from illiteracy and gender inequality, where all children have room to read, learn and grow. Visit us at https://www.roomtoreadindia.org/
+ Study Overview
+About the Project
+This project is Room to Read India's initiative to extend its comprehensive FLN approach in Jharkhand - to six additional districts. The program aims to strengthen Grade 1 and Grade 2 foundational literacy and numeracy outcomes in government schools through structured pedagogy, teacher capacity building, and supportive supervision, in close partnership with state and district government systems.
+ Before finalizing program design for the six districts, Room to Read seeks to commission a Landscape Study to build a rigorous, evidence-based understanding of the current status of foundational literacy and numeracy, the readiness and capacity of the government education system, and district-specific realities and constraints in each district. The study will generate a strategic, decision-ready document - including a consolidated cross-district synthesis and individual district profiles - to guide program design, process adoption and contextualization of Room to Read's FLN approach across the six districts.
+ Purpose of the Study
+This Landscape Study is being commissioned to build a clear, evidence-based understanding of the current FLN landscape - government systems, school-level realities, and district context - across the six districts, ahead of program design and roll-out. Its purpose is to ensure that the design and contextualization of the program in each district is grounded in accurate, on-the-ground evidence</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>Oct 4, 2026</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/tor-landscape-study-for-foundational-literacy-and-numeracy-fln-program-six-districts-jharkhand-room-to-read-india-rfp-26-00376</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="95" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>RFP - Design and Delivery of an Electric Vehicle EV Skilling Programme in Karnataka</t>
         </is>
       </c>
-      <c r="C13" s="1" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 WRI India, an independent knowledge organisation registered as the India Resources Trust, provides objective information and practical proposals to foster environmentally sound and socially equitable development. As an independent knowledge organisation, we leverage our data and expertise to catalyze change across systems like food, land and water; energy; and cities. Our work focuses on improving people’s lives, protecting and restoring nature, and addressing climate change. To enable progress at the pace and scale needed, we also engage with the economic, finance and governance systems that are key to enabling this change.
@@ -1212,34 +1035,95 @@
 Must have a team of qualified trainers and master trainers with relevant domain expertise, as well as administrative and coordination support.</t>
         </is>
       </c>
-      <c r="D13" s="1" t="inlineStr">
+      <c r="D11" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E13" s="1" t="inlineStr">
+      <c r="E11" s="1" t="inlineStr">
         <is>
           <t>Oct 5, 2026</t>
         </is>
       </c>
-      <c r="F13" s="1" t="inlineStr">
+      <c r="F11" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfp-design-and-delivery-of-an-electric-vehicle-ev-skilling-programme-in-karnataka-wri-india-rfp-26-00361</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="95" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="inlineStr">
+    <row r="12" ht="95" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>ToR for Onboarding of consultant/agency for Innovating &amp; Scaling Reproductive Maternal Newborn and Child Health Solutions in the Last-Mile</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>Title Terms of Reference for Onboarding of consultant/agency for Innovating &amp; Scaling Reproductive, Maternal, Newborn and Child Health Solutions in the Last-Mile
+Timeline September 2026 to February 2027
+Scope of Work
+• Outreach and program visibility
+• Application design, launch, review, shortlisting, and due diligence
+• Stakeholder engagement and coordination
+• Knowledge materials and document learnings and insights
+Application Link https://forms.gle/jsngbAREkYmgK7cB6
+Last Date to Apply 5th October, 5 PM
+About SELCO Foundation:
+SELCO Foundation's mission is to create a platform of solutions that uses sustainable energy as a catalyst to bridge environmental sustainability and poverty alleviation. With holistic development as the primary focus, the organization strives to create equitable societies, where services are accessed by all communities. The interventions of SELCO lead to a sustainable delivery model of essential services like livelihoods, education, and health till the last mile.
+(Read more about SELCO here: https://selcofoundation.org/)
+ About the Program
+The program aims to catalyse the development, adoption, and scale of innovative solutions that contribute to improved maternal and child health outcomes. It seeks to build an ecosystem where enterprises and innovators can develop and strengthen technology and technology-allied solutions that enable more accessible, quality, efficient, affordable, and continuous maternal and child health services, particularly across last-mile health facilities and underserved communities.
+The program envisions a future where innovation, technology, and enterprise-led solutions are meaningfully integrated into maternal and child health delivery, enabling health systems, facilities, and frontline health workers to deliver better services to women and children.
+The initiative will bring together enterprises, innovators, health facilities, frontline health workers, institutions, and other ecosystem stakeholders to co-create, test, deploy, and scale solutions with the potential to transform maternal and child health delivery. The focus will be on enabling promising solutions to move beyond individual deployments towards sustainable models of adoption, replication, and scale.
+For the same, we are looking to partner with a like-minded organization that shares this vision and can play an integral role in designing and implementing the initiative. The partner will support enterprise identification and engagement, solution assessment, co-creation, health-system linkages, implementation, stakeholder coordination, evidence generation, and pathways to scale, contributing to more resilient, responsive, and equitable maternal and child health services for women and children.
+ Geography
+Primary Focus: Maharashtra, Karnataka, Odisha, Meghalaya, Mizoram, Nagaland
+Secondary Focus: Other states
+ Selection Criteria
+Applicants should meet the following criteria for being a part of the evaluation:
+Demonstrated experience working with vendors, enterprises, innovators, or solution providers, along with an understanding of grassroots and last-mile contexts and user needs
+Ability to assess enterprise and solution needs and curate tailored mentorship, technical assistance, health-system linkages, and implementation support
+Demonstrated experience in program design, planning, implementation, and management of multi-stakeholder initiatives, preferably in health, maternal and child health, technology, or last-mile service delivery
+Proven ability to manage end-to-end application, assessment, screening, shortlisting, and due diligence processes for a portfolio of enterprises or innovators
+Experience in communication, outreach, stakeholder engagement, and facilitating collaboration between solution providers and health-system stakeholders
+Capability to develop documentation and knowledge products that capture program processes, solution performance, outcomes, implementation models, and learnings for scale and replication
+Prior experience working with development sector organisations, NGOs, health systems, technology providers, enterprises, or think tanks will be considered an added advantage
+The agency will be selected on a combined technical and financial evaluation. Proposals must score a minimum of 70% on the technical components (1–5 below) to be considered for financial evaluation.</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>Oct 5, 2026</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/tor-for-onboarding-of-consultantagency-for-innovating-and-scaling-reproductive-maternal-newborn-and-child-health-solutions-in-the-last-mile-selco-foundation-rfp-26-00373</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="95" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
         <is>
           <t>RFPs Invited for Engagement of a Manpower Agency for Providing Subject Matter Specialists/Experts for the Cluster Development Programme</t>
         </is>
       </c>
-      <c r="C14" s="1" t="inlineStr">
+      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>About the RFP
 National Horticulture Board (NHB), an autonomous organization under the Ministry of Agriculture and Farmers' Welfare, Government of India, invites bids from eligible manpower agencies for engagement to recruit, deploy, and manage qualified personnel supporting NHB's Cluster Development Programme (CDP) — a Central Sector Scheme promoting integrated, market-led horticulture cluster development. The engaged agency will provide three types of Subject Matter Experts per Cluster and additional consultants/manpower as required by NHB from time to time.
@@ -1265,34 +1149,34 @@
  District: Gurugram, Haryana (NHB Head Office)</t>
         </is>
       </c>
-      <c r="D14" s="1" t="inlineStr">
+      <c r="D13" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E14" s="1" t="inlineStr">
+      <c r="E13" s="1" t="inlineStr">
         <is>
           <t>Oct 6, 2026</t>
         </is>
       </c>
-      <c r="F14" s="1" t="inlineStr">
+      <c r="F13" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfps-invited-for-engagement-of-a-manpower-agency-for-providing-subject-matter-specialistsexperts-for-the-cluster-development-programme-national-horticulture-board-nhb-rfp-26-00370</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="95" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="inlineStr">
+    <row r="14" ht="95" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>Applications Open Draper Richards Kaplan Foundation Funding for Social Enterprises</t>
         </is>
       </c>
-      <c r="C15" s="1" t="inlineStr">
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>About us
 Started in 2002, Draper Richards Kaplan Foundation (DRK) is a global venture philanthropy firm supporting early stage, high impact social enterprises. Borrowed from our venture capital legacy, DRK finds, funds, and supports exceptional leaders building innovative solutions to some of the world’s most challenging social and environmental problems. Since beginning this work nearly 25 years ago, DRK has invested in more than 270 organizations that have collectively impacted over 610 million lives to date.
@@ -1316,34 +1200,34 @@
 Please attach a standard resume/CV for the entrepreneur(s) and/or key leadership team members (e.g., CEO, COO, ED, etc.). Applications with text bios for entrepreneurs or members of the leadership team will not be considered.</t>
         </is>
       </c>
-      <c r="D15" s="1" t="inlineStr">
+      <c r="D14" s="1" t="inlineStr">
         <is>
           <t>Climate</t>
         </is>
       </c>
-      <c r="E15" s="1" t="inlineStr">
+      <c r="E14" s="1" t="inlineStr">
         <is>
           <t>Oct 10, 2026</t>
         </is>
       </c>
-      <c r="F15" s="1" t="inlineStr">
+      <c r="F14" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-open-draper-richards-kaplan-foundation-funding-for-social-enterprises-draper-richards-kaplan-foundation-opg-26-00188</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="95" customHeight="1">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B16" s="1" t="inlineStr">
+    <row r="15" ht="95" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund</t>
         </is>
       </c>
-      <c r="C16" s="1" t="inlineStr">
+      <c r="C15" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund
 Apply by: 13 October, 2026
@@ -1368,83 +1252,34 @@
  Projects should include opportunities for ServiceNow employees to volunteer in the project activation or implementation.</t>
         </is>
       </c>
-      <c r="D16" s="1" t="inlineStr">
+      <c r="D15" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E16" s="1" t="inlineStr">
+      <c r="E15" s="1" t="inlineStr">
         <is>
           <t>Oct 13, 2026</t>
         </is>
       </c>
-      <c r="F16" s="1" t="inlineStr">
+      <c r="F15" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/apply-for-the-servicenow-community-solar-fund-changex-opg-26-00186</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="95" customHeight="1">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B17" s="1" t="inlineStr">
-        <is>
-          <t>RFPs Invited for Empanelment of Publishers for Procurement of E-Books for Rashtriya e-Pustakalaya National Book Trust India</t>
-        </is>
-      </c>
-      <c r="C17" s="1" t="inlineStr">
-        <is>
-          <t>About the RFP:
-Rashtriya e-Pustakalaya, a free National Digital Library for children and adolescents — an initiative of the Department of School Education &amp; Literacy, Ministry of Education, Government of India, implemented by the National Book Trust (NBT), India — invites Expression of Interest (EoI) for the empanelment of publishers for the selection and procurement of e-books, with the objective of enriching the platform's book collection. NBT is an autonomous body under the Ministry of Education, established in 1957 to promote literacy and reading culture in India.
- Scope of Work:
-Provide acceptable, age-appropriate e-books for ages 8–11, 11–14, and 14+ (Young Adults) across genres like Classics, Mystery, Thriller, Historical, Fiction, Science &amp; Technology, Sports &amp; Fitness, Adventure, etc., with special emphasis on promoting the Indian Knowledge System, history, traditions, and achievements of India
-Provide e-books in specified formats (ePUB / searchable PDF) accessible on the Rashtriya e-Pustakalaya app
-Ensure all necessary consents/approvals from authors, illustrators, artists, translators, or legal owners as per the Copyright Act, 1957 and Copyright Rules, 2013
-Ensure necessary licensing agreements and adherence to copyright laws for uninterrupted hosting
-Ensure content relevance to specific age groups and target audience
-Provide content with valid ISBN/RNI registration only
-Provide metadata of e-books in the specified format with periodic updates
- Eligibility (for Publishers):
-Must be a registered legal entity: Company (Companies Act, 2013) / LLP (LLP Act, 2008) / Trust (Indian Trusts Act, 1882) / Society (Societies Registration Act, 1860) / Partnership firm (Indian Partnership Act, 1932) / Proprietorship firm (registered under Shops &amp; Establishment Act/Labour Department/GST/other statutory department)
-Must hold valid ISBN/RNI registration
-Must have GST Registration (if applicable), PAN, and Aadhar Card (if applicable)
-Must not be blacklisted by the Government of India, any State/UT Government, or their agencies for corrupt/fraudulent/unfair trade practices, or for backing out of a contract after award
-Publisher, directors, and officers must not have been convicted of any criminal offence related to their professional conduct or false statements/misrepresentation in the last 3 years, or otherwise debarred
-No conflict of interest in the empanelment process
-Must indemnify Rashtriya e-Pustakalaya/NBT-India for any IP-related claims from authors/illustrators/translators/legal owners</t>
-        </is>
-      </c>
-      <c r="D17" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E17" s="1" t="inlineStr">
-        <is>
-          <t>Oct 16, 2026</t>
-        </is>
-      </c>
-      <c r="F17" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/rfps-invited-for-empanelment-of-publishers-for-procurement-of-e-books-for-rashtriya-e-pustakalaya-national-book-trust-india-national-book-trust-nbt-india-rfp-26-00371</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="95" customHeight="1">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="inlineStr">
+    <row r="16" ht="95" customHeight="1">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>ToR - Engagement of Consultant/Vendor Individual towards implementation of Literacy Program in Telangana State</t>
         </is>
       </c>
-      <c r="C18" s="1" t="inlineStr">
+      <c r="C16" s="1" t="inlineStr">
         <is>
           <t>ANNEX A – TERMS OF REFERENCE (ToR) 
  Engagement of Consultant/Vendor (Individual) towards implementation of Literacy Program in Telangana State.
@@ -1509,34 +1344,83 @@
 Approved travel and accommodation expenses incurred for assignment-related activities shall be reimbursed by Room to Read in accordance with the consultancy reimbursement guidelines.</t>
         </is>
       </c>
-      <c r="D18" s="1" t="inlineStr">
+      <c r="D16" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E18" s="1" t="inlineStr">
+      <c r="E16" s="1" t="inlineStr">
         <is>
           <t>Oct 16, 2026</t>
         </is>
       </c>
-      <c r="F18" s="1" t="inlineStr">
+      <c r="F16" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-engagement-of-consultantvendor-individual-towards-implementation-of-literacy-program-in-telangana-state-room-to-read-india-rfp-26-00360</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="95" customHeight="1">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="inlineStr">
+    <row r="17" ht="95" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>RFPs Invited for Empanelment of Publishers for Procurement of E-Books for Rashtriya e-Pustakalaya National Book Trust India</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>About the RFP:
+Rashtriya e-Pustakalaya, a free National Digital Library for children and adolescents — an initiative of the Department of School Education &amp; Literacy, Ministry of Education, Government of India, implemented by the National Book Trust (NBT), India — invites Expression of Interest (EoI) for the empanelment of publishers for the selection and procurement of e-books, with the objective of enriching the platform's book collection. NBT is an autonomous body under the Ministry of Education, established in 1957 to promote literacy and reading culture in India.
+ Scope of Work:
+Provide acceptable, age-appropriate e-books for ages 8–11, 11–14, and 14+ (Young Adults) across genres like Classics, Mystery, Thriller, Historical, Fiction, Science &amp; Technology, Sports &amp; Fitness, Adventure, etc., with special emphasis on promoting the Indian Knowledge System, history, traditions, and achievements of India
+Provide e-books in specified formats (ePUB / searchable PDF) accessible on the Rashtriya e-Pustakalaya app
+Ensure all necessary consents/approvals from authors, illustrators, artists, translators, or legal owners as per the Copyright Act, 1957 and Copyright Rules, 2013
+Ensure necessary licensing agreements and adherence to copyright laws for uninterrupted hosting
+Ensure content relevance to specific age groups and target audience
+Provide content with valid ISBN/RNI registration only
+Provide metadata of e-books in the specified format with periodic updates
+ Eligibility (for Publishers):
+Must be a registered legal entity: Company (Companies Act, 2013) / LLP (LLP Act, 2008) / Trust (Indian Trusts Act, 1882) / Society (Societies Registration Act, 1860) / Partnership firm (Indian Partnership Act, 1932) / Proprietorship firm (registered under Shops &amp; Establishment Act/Labour Department/GST/other statutory department)
+Must hold valid ISBN/RNI registration
+Must have GST Registration (if applicable), PAN, and Aadhar Card (if applicable)
+Must not be blacklisted by the Government of India, any State/UT Government, or their agencies for corrupt/fraudulent/unfair trade practices, or for backing out of a contract after award
+Publisher, directors, and officers must not have been convicted of any criminal offence related to their professional conduct or false statements/misrepresentation in the last 3 years, or otherwise debarred
+No conflict of interest in the empanelment process
+Must indemnify Rashtriya e-Pustakalaya/NBT-India for any IP-related claims from authors/illustrators/translators/legal owners</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>Oct 16, 2026</t>
+        </is>
+      </c>
+      <c r="F17" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/rfps-invited-for-empanelment-of-publishers-for-procurement-of-e-books-for-rashtriya-e-pustakalaya-national-book-trust-india-national-book-trust-nbt-india-rfp-26-00371</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="95" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>RFPs Invited for Consultant to Develop a Technical Assistance Package for National Application of the Digital Health and AI Investment Classification Framework</t>
         </is>
       </c>
-      <c r="C19" s="1" t="inlineStr">
+      <c r="C18" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are Transform Health: a global coalition of more than 200 organisations driving the digital transformation of health to achieve universal health coverage. 
@@ -1564,34 +1448,34 @@
 Ability to manage multi-country consultancy engagements and coordinate with in-country focal points</t>
         </is>
       </c>
-      <c r="D19" s="1" t="inlineStr">
+      <c r="D18" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E19" s="1" t="inlineStr">
+      <c r="E18" s="1" t="inlineStr">
         <is>
           <t>Oct 23, 2026</t>
         </is>
       </c>
-      <c r="F19" s="1" t="inlineStr">
+      <c r="F18" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfps-invited-for-consultant-to-develop-a-technical-assistance-package-for-national-application-of-the-digital-health-and-ai-investment-classification-framework-transform-health-rfp-26-00359</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="95" customHeight="1">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="inlineStr">
+    <row r="19" ht="95" customHeight="1">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for D-Prize Global Competition Seed Funding for New Poverty-Solution Distribution Organizations</t>
         </is>
       </c>
-      <c r="C20" s="1" t="inlineStr">
+      <c r="C19" s="1" t="inlineStr">
         <is>
           <t>About the Grant:
 D-Prize seeds new organizations that distribute proven poverty solutions at the "last mile," with the aim of scaling impact. Applicants select from a range of evidence-based interventions (health, agriculture, education, water, safety, transparency, and more) and propose how they would launch or grow an organization to distribute that intervention. Top entrepreneurs receive up to $20,000 in seed funding to run a pilot and build an organization capable of scaling to reach thousands, even millions of people.
@@ -1614,34 +1498,34 @@
 Extension Deadline: 6 December 2026, midnight PT (extension registration required)</t>
         </is>
       </c>
-      <c r="D20" s="1" t="inlineStr">
+      <c r="D19" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E20" s="1" t="inlineStr">
+      <c r="E19" s="1" t="inlineStr">
         <is>
           <t>Oct 25, 2026</t>
         </is>
       </c>
-      <c r="F20" s="1" t="inlineStr">
+      <c r="F19" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-d-prize-global-competition-seed-funding-for-new-poverty-solution-distribution-organizations-d-prize-opg-26-00191</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="95" customHeight="1">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="inlineStr">
+    <row r="20" ht="95" customHeight="1">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 8th Call for Proposals Small-Size Grants Global EbA Fund</t>
         </is>
       </c>
-      <c r="C21" s="1" t="inlineStr">
+      <c r="C20" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -1704,34 +1588,34 @@
 Only successful applicants will be contacted; no individual feedback provided to unsuccessful applicants</t>
         </is>
       </c>
-      <c r="D21" s="1" t="inlineStr">
+      <c r="D20" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E21" s="1" t="inlineStr">
+      <c r="E20" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F21" s="1" t="inlineStr">
+      <c r="F20" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-8th-call-for-proposals-small-size-grants-global-eba-fund-global-eba-fund-opg-26-00177</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="95" customHeight="1">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="inlineStr">
+    <row r="21" ht="95" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Adaptive Control Frameworks to Unlock Full-Scale BNR Potential Water Research Foundation WRF</t>
         </is>
       </c>
-      <c r="C22" s="1" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Water Research Foundation (WRF) is the leading research organization advancing the science of all water to meet the evolving needs of its subscribers and the water sector. WRF is a nonprofit, charitable and educational organization which funds, manages, and publishes research on the technology, operation, and management of drinking water, wastewater, reuse, and stormwater collection, treatment and supply systems—all in pursuit of ensuring water quality and improving water services to the public.
@@ -1772,34 +1656,34 @@
 Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
         </is>
       </c>
-      <c r="D22" s="1" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E22" s="1" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F22" s="1" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-adaptive-control-frameworks-to-unlock-full-scale-bnr-potential-water-research-foundation-wrf-the-water-research-foundation-wrf-opg-26-00187</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="95" customHeight="1">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B23" s="1" t="inlineStr">
+    <row r="22" ht="95" customHeight="1">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Crossing the Divide Best Practices for Addressing Local and Privately-Owned Lateral Sewer Issues RFP 5419</t>
         </is>
       </c>
-      <c r="C23" s="1" t="inlineStr">
+      <c r="C22" s="1" t="inlineStr">
         <is>
           <t>Project Objective:
 To provide water resource recovery facilities (WRRFs) and collection system operators with an interactive manual of practice for implementing inflow and infiltration (I&amp;I) and obstruction management programs, focused on municipal and privately owned lateral sewers in complex legal, regulatory, and multi-jurisdictional environments.
@@ -1837,34 +1721,34 @@
  Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
         </is>
       </c>
-      <c r="D23" s="1" t="inlineStr">
+      <c r="D22" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E23" s="1" t="inlineStr">
+      <c r="E22" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F23" s="1" t="inlineStr">
+      <c r="F22" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-crossing-the-divide-best-practices-for-addressing-local-and-privately-owned-lateral-sewer-issues-rfp-5419-the-water-research-foundation-wrf-opg-26-00189</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="95" customHeight="1">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B24" s="1" t="inlineStr">
+    <row r="23" ht="95" customHeight="1">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Comparison of PFAS Contributions to Agricultural Systems</t>
         </is>
       </c>
-      <c r="C24" s="1" t="inlineStr">
+      <c r="C23" s="1" t="inlineStr">
         <is>
           <t>Project Objectives:
 Report per- and polyfluoroalkyl substance (PFAS) concentrations from a variety of agricultural inputs — animal manures, fertilizers, pesticides, composts, soil amendments, seed coatings, and biosolids-based products
@@ -1900,34 +1784,34 @@
  Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00) — same deadline as the other two WRF grants</t>
         </is>
       </c>
-      <c r="D24" s="1" t="inlineStr">
+      <c r="D23" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E24" s="1" t="inlineStr">
+      <c r="E23" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F24" s="1" t="inlineStr">
+      <c r="F23" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-comparison-of-pfas-contributions-to-agricultural-systems-the-water-research-foundation-wrf-opg-26-00190</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="95" customHeight="1">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B25" s="1" t="inlineStr">
+    <row r="24" ht="95" customHeight="1">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Whitley Award 2027</t>
         </is>
       </c>
-      <c r="C25" s="1" t="inlineStr">
+      <c r="C24" s="1" t="inlineStr">
         <is>
           <t>About the Grant: 
 An annual grant by the Whitley Fund for Nature (WFN) recognising grassroots conservation leaders in the Global South, providing funding to support and scale up proven, science-based solutions that deliver lasting impact for both people and nature.
@@ -1940,34 +1824,34 @@
 You do not need to be invited or nominated to apply.</t>
         </is>
       </c>
-      <c r="D25" s="1" t="inlineStr">
+      <c r="D24" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E25" s="1" t="inlineStr">
+      <c r="E24" s="1" t="inlineStr">
         <is>
           <t>Oct 30, 2026</t>
         </is>
       </c>
-      <c r="F25" s="1" t="inlineStr">
+      <c r="F24" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-whitley-award-2027-whitley-fund-for-nature-wfn-opg-26-00153</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="95" customHeight="1">
-      <c r="A26" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B26" s="1" t="inlineStr">
+    <row r="25" ht="95" customHeight="1">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIFAR Global Scholars Program 20272029 Cohort</t>
         </is>
       </c>
-      <c r="C26" s="1" t="inlineStr">
+      <c r="C25" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 CIFAR is a Canadian-based globally influential research organization that convenes the world’s most brilliant people across disciplines to advance transformative knowledge and solve humanity’s biggest problems, together. By supporting long-term interdisciplinary collaboration, CIFAR provides researchers with an unparalleled environment of trust, transparency and knowledge sharing. Our time-tested model inspires new directions of inquiry, accelerates discovery and yields breakthroughs across borders and academic disciplines. Through knowledge mobilization, we are catalysts for change in industry, government and society. Through our 15 research programs and the Pan-Canadian AI Strategy, CIFAR convenes close to 400 of the world’s top researchers from 141 institutions in 20 countries. CIFAR is generously supported by the governments of Canada, Alberta and Québec, as well as foundations, individuals, corporations and Canadian and international partner organizations.
@@ -2011,73 +1895,34 @@
  Application Deadline: November 4, 2026, 12:00 PM EST</t>
         </is>
       </c>
-      <c r="D26" s="1" t="inlineStr">
+      <c r="D25" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E26" s="1" t="inlineStr">
+      <c r="E25" s="1" t="inlineStr">
         <is>
           <t>Nov 4, 2026</t>
         </is>
       </c>
-      <c r="F26" s="1" t="inlineStr">
+      <c r="F25" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cifar-global-scholars-program-20272029-cohort-cifar-canadian-institute-for-advanced-research-opg-26-00183</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="95" customHeight="1">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B27" s="1" t="inlineStr">
+    <row r="26" ht="95" customHeight="1">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for IWRS Teaching Innovation Award</t>
         </is>
       </c>
-      <c r="C27" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
- About the Grant
-The IWRS (Insect Welfare Research Society) Teaching Innovation Award supports instructors developing new approaches to teaching insect or invertebrate biology that incorporate the 3Rs (Replacement, Reduction, and Refinement) — principles for reducing animal welfare impacts in teaching and research practices.
- Purpose
-Funds support the creation and implementation of 3Rs-driven instructional materials and pedagogical approaches. Priority is given to proposals addressing common teaching practices with substantial welfare implications.
- Grant Amount
-Two awards of $2,000 USD are available annually.</t>
-        </is>
-      </c>
-      <c r="D27" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E27" s="1" t="inlineStr">
-        <is>
-          <t>Nov 15, 2026</t>
-        </is>
-      </c>
-      <c r="F27" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="95" customHeight="1">
-      <c r="A28" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B28" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for IWRS Teaching Innovation Award</t>
-        </is>
-      </c>
-      <c r="C28" s="1" t="inlineStr">
+      <c r="C26" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Insects are one of the most numerous and diverse animal groups on Earth.
@@ -2092,34 +1937,73 @@
 IWRS staff and Advisory Group members are not eligible to apply.</t>
         </is>
       </c>
-      <c r="D28" s="1" t="inlineStr">
+      <c r="D26" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E28" s="1" t="inlineStr">
+      <c r="E26" s="1" t="inlineStr">
         <is>
           <t>Nov 15, 2026</t>
         </is>
       </c>
-      <c r="F28" s="1" t="inlineStr">
+      <c r="F26" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00166</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="95" customHeight="1">
-      <c r="A29" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B29" s="1" t="inlineStr">
+    <row r="27" ht="95" customHeight="1">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for IWRS Teaching Innovation Award</t>
+        </is>
+      </c>
+      <c r="C27" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
+ About the Grant
+The IWRS (Insect Welfare Research Society) Teaching Innovation Award supports instructors developing new approaches to teaching insect or invertebrate biology that incorporate the 3Rs (Replacement, Reduction, and Refinement) — principles for reducing animal welfare impacts in teaching and research practices.
+ Purpose
+Funds support the creation and implementation of 3Rs-driven instructional materials and pedagogical approaches. Priority is given to proposals addressing common teaching practices with substantial welfare implications.
+ Grant Amount
+Two awards of $2,000 USD are available annually.</t>
+        </is>
+      </c>
+      <c r="D27" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E27" s="1" t="inlineStr">
+        <is>
+          <t>Nov 15, 2026</t>
+        </is>
+      </c>
+      <c r="F27" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="95" customHeight="1">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Medium-Size Grants Call for Proposals Global EbA Fund</t>
         </is>
       </c>
-      <c r="C29" s="1" t="inlineStr">
+      <c r="C28" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -2176,34 +2060,34 @@
 Applications submitted via online portal (link shared on the Medium-Size Grants webpage from Oct 12)</t>
         </is>
       </c>
-      <c r="D29" s="1" t="inlineStr">
+      <c r="D28" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E29" s="1" t="inlineStr">
+      <c r="E28" s="1" t="inlineStr">
         <is>
           <t>Nov 16, 2026</t>
         </is>
       </c>
-      <c r="F29" s="1" t="inlineStr">
+      <c r="F28" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-medium-size-grants-call-for-proposals-global-eba-fund-global-eba-fund-opg-26-00178</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="95" customHeight="1">
-      <c r="A30" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B30" s="1" t="inlineStr">
+    <row r="29" ht="95" customHeight="1">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIEIF Grant 2026 Climate Intervention Environmental Impact Fund</t>
         </is>
       </c>
-      <c r="C30" s="1" t="inlineStr">
+      <c r="C29" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Climate Intervention Environmental Impact Fund (CIEIF) is a philanthropic fund focused on supporting responsible climate intervention field tests. It provides grants for activities such as environmental impact assessment (EIA), predictive impact modelling, and engagement with potentially affected stakeholders, including local communities and government agencies.
@@ -2230,34 +2114,34 @@
 Potential for scaling the innovation to a globally relevant level</t>
         </is>
       </c>
-      <c r="D30" s="1" t="inlineStr">
+      <c r="D29" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E30" s="1" t="inlineStr">
+      <c r="E29" s="1" t="inlineStr">
         <is>
           <t>Dec 1, 2026</t>
         </is>
       </c>
-      <c r="F30" s="1" t="inlineStr">
+      <c r="F29" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cieif-grant-2026-climate-intervention-environmental-impact-fund-climate-intervention-environmental-impact-fund-opg-26-00155</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="95" customHeight="1">
-      <c r="A31" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B31" s="1" t="inlineStr">
+    <row r="30" ht="95" customHeight="1">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 6th Annual Seeding The Future Global Food System Challenge</t>
         </is>
       </c>
-      <c r="C31" s="1" t="inlineStr">
+      <c r="C30" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are one of the largest and most respected private organisations for development cooperation and humanitarian aid in Germany. As a politically and confessionally independent organisation, our value-oriented actions are always based on ethical principles. Our vision is clear: "Zero Hunger by 2030"
@@ -2289,34 +2173,34 @@
 Individuals with no organizational entity</t>
         </is>
       </c>
-      <c r="D31" s="1" t="inlineStr">
+      <c r="D30" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E31" s="1" t="inlineStr">
+      <c r="E30" s="1" t="inlineStr">
         <is>
           <t>Jan 1, 2027</t>
         </is>
       </c>
-      <c r="F31" s="1" t="inlineStr">
+      <c r="F30" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-6th-annual-seeding-the-future-global-food-system-challenge-welthungerhilfe-opg-26-00180</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="95" customHeight="1">
-      <c r="A32" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B32" s="1" t="inlineStr">
+    <row r="31" ht="95" customHeight="1">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Microbiota &amp; Women's Health International Call for Projects</t>
         </is>
       </c>
-      <c r="C32" s="1" t="inlineStr">
+      <c r="C31" s="1" t="inlineStr">
         <is>
           <t>About the Grant
 An annual international research grant by the Biocodex Microbiota Foundation (BMF), rewarding research proposals on the microbiota and its implications in Women's Health and Disease. This year's theme: "Unraveling male-female genital microbiome interactions: mechanisms, transmission, and impact on vaginal dysbiosis."
@@ -2333,34 +2217,34 @@
 €200,000 annually — awarded to researchers within universities, hospitals, or other research settings to finance equipment, operations, or staffing costs. Grants are NOT awarded to individuals directly (must be institutionally affiliated). Institution's overhead costs capped at 10%.</t>
         </is>
       </c>
-      <c r="D32" s="1" t="inlineStr">
+      <c r="D31" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E32" s="1" t="inlineStr">
+      <c r="E31" s="1" t="inlineStr">
         <is>
           <t>Jan 15, 2027</t>
         </is>
       </c>
-      <c r="F32" s="1" t="inlineStr">
+      <c r="F31" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-microbiota-and-womens-health-international-call-for-projects-biocodex-microbiota-foundation-bmf-opg-26-00152</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="95" customHeight="1">
-      <c r="A33" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B33" s="1" t="inlineStr">
+    <row r="32" ht="95" customHeight="1">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B32" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for BES Training and Travel Grants</t>
         </is>
       </c>
-      <c r="C33" s="1" t="inlineStr">
+      <c r="C32" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are a global community of scientists shining a spotlight on the intricacy and value of our natural world, providing the evidence for better decisions. Our vision is for people and nature to thrive in a world that values ecology.
@@ -2399,17 +2283,17 @@
  Application Deadline (Round 2): Opens 30 April 2026, closes 17 May 2026</t>
         </is>
       </c>
-      <c r="D33" s="1" t="inlineStr">
+      <c r="D32" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E33" s="1" t="inlineStr">
+      <c r="E32" s="1" t="inlineStr">
         <is>
           <t>May 17, 2027</t>
         </is>
       </c>
-      <c r="F33" s="1" t="inlineStr">
+      <c r="F32" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-bes-training-and-travel-grants-british-ecological-society-opg-26-00181</t>
         </is>

</xml_diff>

<commit_message>
Auto update Combined.xlsx [Tue Sep 29 07:49:10 UTC 2026]
</commit_message>
<xml_diff>
--- a/output/Combined.xlsx
+++ b/output/Combined.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -495,341 +495,10 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>EOI Inviting Expression of Interest-cum-Proposal for Setting Up District De-Addiction Centres under NAPDDR</t>
+          <t>ToR - Project Management Unit Solarization of Women-led Livelihoods in Maharashtra MAVIMSELCO Foundation Short Duration Project</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t>About us
-In the year 1985-86, the erstwhile Ministry of Welfare was bifurcated into the Department of Women and Child Development and the Department of Welfare. Simultaneously, the Scheduled Castes Development Division, Tribal Development Division and the Minorities and Backward Classes Welfare Division were moved from the Ministry of Home Affairs and also the Wakf Division from the Ministry of Law to form the then Ministry of Welfare Subsequently, the name of the Ministry was changed to the Ministry of Social Justice &amp; Empowerment in May, 1998. Further, in October, 1999, the Tribal Development Division had moved out to form a separate Ministry of Tribal Affairs. In January, 2007, the Minorities Division along with Wakf Unit have been moved out of the Ministry and formed as a separate Ministry and the Child Development Division has gone to the Ministry of Women &amp; Child Development.
- Department of Social Justice and Empowerment invites Expression of lnterest-cum-proposal from the eligible organizations for setting up of District DeAddiction Centres under the scheme of National Action Plan for Drug Demand Reduction (NAPDDR) for 315 GAP Districts of the country (as per list attached at Annexure - l). The list of districts is subject to change (addition or deletion) time to trme by the Ministry as per requirement or need on the ground.
- 2. Eligible NGOs may apply for setting up of DDAC provided that they have rent free accommodation for setting up of DDAC as per the standards of guideline of the NAPDDR scheme or renlfree accommodation may also be provided by the concerned District Administration. 
- 3. Setting up and running of District De-Addiction Centres (DDACS) will be done as per the following guidelinesr. 
- i. There will be a District De-Addiction Centre (DDAC) preferably in each district headquarter or suitably accessible place where rent free accommodation is provided by the district administration. These DDACs would provide comprehensive facilities hitherto being provided by IRCA, ODIC &amp; CPLI together. lf the district administration of identified district is not able to provide suitable rent free accommodation, then the application will be called from the eligible VOs/ NGOs, who will provide rent free accommodation for setting up of DDAC in that district.
- ii. The functioning of DDAC will be monitored by the three tier Committees headed by the Chief Secretary, District Collector/Deputy Commissioner and Block Development Officer of the respective arealregion which have been formed under Nasha Mukt Bharat Abhiyaan (NMBA). Additionally, retired eminent personalities of the Districts, activists, Vice-Chancellor/ Head of Department (HoD)/ Principal, researcher, scholars and so on may be co-opted by Chairman as the members of the Committees. These commiftees would
- only monitor policy related issues. Day to day and other activities relating to implementation would be the responsibility of the concerned organization/NGO approved for setting up of the DDAC. The Meetings of DDAC are to be held as per the details given below:
- (a) State-level Steering and Monitoring Committee (High Level Task Force) - headed by Chief Secretary - to meet quarterly. (b) District-level Committee - headed by District Collector / Deputy Commissioner - to meet monthly and have mandatory inspections quarterly. (c) Block level Committee - headed by Block Development Officer - to meet &amp; have mandatory inspections monthly.
- The Committees will also review the functioning and assess the performance of the DDAC in terms of the effectiveness of deliverables and make further suggestions to the management of DDAC. 
- IIl t. A separate (dedicated) account will be opened for keeping funds of DDAC in the name of NGO/Organization. The account will be registered on PFMS and implemented through EAT Module. 
- lV. For setting up of DDACs, preference would be given to those Districts, which do not have any facility of IRCA or DDAC. For this, the organization willing to work in the field of DRUGS DE-ADDICTION TREATMENT will be eligible for applying for DDAC. The priority for selection of DDAC would be: 
-a. The DDAC proposed to be run by the District administration itself. 
-b. Rent free accommodation in the district headquarter provided by the concerned DC/DM &amp; further willingness from interested NGO is sought. c, Where no proposal for rent-free accommodation is received from concerned DCiDM, interested NGO may directly apply for DDAC provided they do not seek any rent for same and only building maintenance will be given. 
-V. The details of Minimum standards like physical space and necessary amenities to be provided by District administration or NGOs are as under: 
-(a) The centre should be easily accessible and connected through public transport. 
-(b) The total built-in area of the DDAC should be at least 3000 sq,ft. in case of metros and 4000 sq.ft. in case of small towns and villages to house 15 patients and 4000 sq.ft. in case of metros and 5000 sq.ft. in case of small towns and villages to house 30 patients. This includes an area of about 2000 sq. ft. for Treatment cum Rehabilitation centre, an area of about 700 sq. ft. for Drop-ln Centre facilities and an area of about 300 sq. ft. for CPLI Centre facilities. 
-(c) The centre should be properly ventilated, well-lit and maintained in a clean manner. Water to be made available. 
-(d) Basic safety of the patients to be ensured 
-(e) Facilities at the centre - Waiting space with seating arrangements for a minimum 5 persons Cubicles / rooms for consultation for physical examination Facilities to store drugs, linen, and records of patients Facilities with privacy for providing individual counselling, group therapy, re-educative sessions, family classes. They should be airy with comfortable seating with floor mats / chairs. Blackboard, chalk and other material to be provided. Availability of recreational facilities. Separate Drop ln Facility centre with recreation room, counselling room and medical room. Project room for CPLI activities including consultation room for interviewing Vl. Standards set in the above para of the guidelines may change from time to time as and when necessary with the approval of competent authority and the stakeholders / NGOs/ VOs would be intimated of same as and when such changes happen. 
- 4. The interested and eligible NGOs / organizations can apply through eAnudaan (https://grants-msje.gov.in/ngo-login) portal of the Ministry. The Project Screening Committee in the Ministry will select the eligible NGO(s) for establishing and running of the DDAC and recommend the release of funds in two installments. However, the organization shall be eligible for receiving GIA under the scheme from the date of approval of the competent authority. 
- 5. ELIGIBLE ORGANIZATION: 
-Organizations which are already running MoSJE supported IRCA or State Government supported De-addiction Centre/ Government Hospital or any private run De-Addiction centre are eligible for applying for DDAC. Organization can apply only for that State/UT in which they are already running IRCA"/De-addiction Centre from the last 2 years or more from the date of call for the proposal. Condition may be relaxed for any Government run Hospitals, which are non-profitable in nature. I 
-6. Start-up consists of young persons/ professionals, who have graduated from top social institutes of lndia or abroad are also eligible to apply. However, they must have experience of 2 years in the field of Drug De-addiction TREATMENT. 7. Role and Responsibility of DDACs The main focus of the DDAC is early prevention, education, demand reduction, identification, treatment and rehabilitation services of vulnerable individuals or individuals affected by substance use disorders DDAC would: 
-a. Conduct primary prevention activities through awareness programs among the vulnerable and affected community 
-b. Engage in risk mitigation of substance use among children/ adolescenuyouth by: Preventing substance use Delaying initiation of substance use 
-c. ldentify and train selected peer educators in the community 
-d. lmplement early prevention education through life skill training led by trained peer educators 
-e. Provide awareness about referral and linkage to counseling, treatment and rehabilitation services for substance dependent adolescents identified in the community 
-f. ldentifying adolescents and other individuals subjected to substance use and facilitating their referrali admission into Rehabilitation Centers/ Drop ln Centres. 
-g. Provide a whole range of services which includes treatment, after care and rehabilitation including skill development for Whole Person Recovery (WPR) of dependents; 
-h. Undertake drug demand reduction efforts to address all forms of illicit use of any substances and ensure overall well being of humankind; 
-i. Alleviate the consequences of substance dependence amongst individuals, family and society at large 
-9. The budget details of DDAC is attached as Annexure - 
-10. The e-anudaan portal shall remain open through out the year and the recommendations from the States/UTs will be considered periodically. 
-11. Department of Social Justice and Empowerment (DoSJE) reserves the right to cancel this notice, andior invite afresh proposals with or without amendments to this document without liability or any obligation for such document, and without assigning any reason. DoSJE reserves the right to take final decision regarding selection of implementing agency or project.</t>
-        </is>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>Sep 30, 2026</t>
-        </is>
-      </c>
-      <c r="F3" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/eoi-inviting-expression-of-interest-cum-proposal-for-setting-up-district-de-addiction-centres-under-napddr-ministry-of-social-justice-and-empowerment-goi-rfp-26-00356</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="95" customHeight="1">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>ToR - Branding Development &amp; Design/Market Promotion Consultant Project Sashakt</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>Organisation Humana People to People India (HPPI)
-Project Sashakt – Strengthening Women-led Handloom Cooperatives in Assam (EU-funded)
-Coverage 25 women-led handloom cooperatives, ~2,500 women artisans across Kamrup, Dhubri and Chirang districts
-Location Assam-based preferred; travel to Kamrup, Dhubri and Chirang required
-Duration 12 months from date of contract signing
-Monthly Professional Fee INR 1,25,000 (all-inclusive of fees, GST, travel, workshops, design revisions and reporting)
-Total Budget INR 15,00,000 (12 months × INR 1,25,000)
-Application Deadline 30 September 2026, by 5:00 PM IST
-How to Apply Email technical and financial proposals, with a design portfolio, to careers@human-india.org, subject line “Branding &amp; Market Promotion Consultancy – Project Sashakt”
-1. Background and Purpose
-HPPI is implementing Project Sashakt, an EU-supported initiative strengthening women-led handloom cooperatives and improving livelihoods for women weavers in Assam, using a Local2Global approach to market access. HPPI is seeking an Assam-based branding and design consultant/agency to build market-ready brand identities for cooperative products and the capacity of cooperatives to use and promote them — covering brand identity, naming, logo and packaging design, brand guidelines, and capacity building — to position products for wider regional, national and international visibility and strengthen the long-term sustainability of Assam's handloom sector.
- 2. Scope of Work
-Product Development &amp; Diversification: work hands-on with a representative sample of weavers to assess current product range, quality and design variety, and pilot feasible new designs, variants or product use-cases within existing skills, looms and materials — establishing a sufficient, market-ready product range ahead of full brand rollout.
-Brand discovery: consult HPPI, cooperatives and artisans; study existing products, weaving traditions and motifs; assess current market positioning, branding gaps and differentiation opportunities in domestic and international markets.
-Brand development: create brand concepts, positioning and identity language; develop names for cooperative brands/product lines reflecting Assamese heritage and market relevance; design logos, typography, colour palettes, motifs, packaging concepts and product labels/tags.
-Branding toolkit: produce practical, reusable guidelines and templates — logo usage, packaging, social media, product catalogues and exhibition materials — for cooperatives to apply independently.
-Capacity building: run training workshops for cooperatives on brand usage and communication, and provide hands-on implementation support and mentoring during rollout across packaging, exhibitions, social media and product communication.
-Market promotion support: develop promotional materials for exhibitions/market events; advise on digital brand presence and storytelling; support Local2Global positioning for national and international audiences.
- 3. Deliverables and Timeline
-# Deliverable Timeline
-1 Inception report and branding strategy roadmap Month 1
-2 Product development plan and prototype products with sampled cooperatives Months 1–2
-3 Market assessment and branding gap analysis Month 2
-4 Brand concepts, names and logo options Months 3–4
-5 Finalised brand identity packages Month 5
-6 Packaging and branding templates Month 6
-7 Brand usage and communication guidelines Month 7
-8 Training workshops for cooperatives Months 8–10
-9 Handholding support for implementation Months 9–12
-10 Final report with outcomes and recommendations Month 12
-4. Required Qualifications and Experience
-Proven experience in branding, communication design and visual identity development, with a strong design portfolio.
-Experience in product or textile design/diversification support for artisan producers at a nascent or early production stage — working within existing skills, looms and materials, in addition to branding expertise.
-Prior work with handloom, handicrafts, artisan collectives, MSMEs or rural enterprises preferred; strong understanding of Assamese culture, textiles and local markets.
-Experience in packaging design, market-oriented branding, and conducting training/capacity-building workshops.
- 5. Selection Criteria
-Criteria Weightage
-Relevant experience 30%
-Quality of portfolio 25%
-Technical approach and methodology 25%
-Understanding of Assam's handloom sector 10%
-Financial proposal 10%
-6. Proposal Submission Requirements
-Technical proposal with detailed methodology and work plan
-Portfolio of relevant assignments
-Financial proposal and CV
-References from previous assignments
- 7. Reporting and Expected Impact
-The consultant/agency will report to HPPI's designated Project Lead, work closely with cooperative representatives, and join weekly progress review meetings. The assignment is expected to deliver a stronger market identity, greater product visibility and sales potential, enhanced entrepreneurial capacity among women weavers, and a more sustainable handloom ecosystem through strategic branding and storytelling.
- 8. Ethics and Confidentiality
-The consultant/agency must ensure ethical, consent-based data collection with cultural sensitivity, particularly when engaging women weavers. All data and reports remain the property of HPPI and must be kept strictly confidential, with no external use.</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="inlineStr">
-        <is>
-          <t>Sep 30, 2026</t>
-        </is>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/tor-branding-development-and-designmarket-promotion-consultant-project-sashakt-humana-people-to-people-india-rfp-26-00365</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="95" customHeight="1">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>Application Invited for Giving Joy Microgrant</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-Giving Joy is a US-based nonprofit that strengthens and inspires women’s entrepreneurship worldwide. Through its micro-grants and mentorship program, Giving Joy helps women establish or improve their businesses and initiatives—for their benefit and the benefit of their communities. To date, Giving Joy has awarded over 88 grants to women-led initiatives in 26 countries.
- 2026 Grant Cycle
-Beginning in 2026, Giving Joy has moved to two global grant cycles per year.
-The organization states that this change was made after operating multiple regional rounds, with the aim of:
-Providing clearer timelines for applicants
-Increasing the quality and depth of application reviews
-Reducing administrative burden
-Improving support for grantees
-Focusing communications and fundraising more effectively
-Continuing to reach women entrepreneurs globally without dividing applications by geography
-Each cycle is open to women entrepreneurs worldwide.
- Eligible Fields / Activities
-There is no restriction to a particular field such as health.
-Applicants can propose activities in:
-Any field
-Trade
-Occupation
-Craft
- What Does Giving Joy Look For?
-Giving Joy prioritizes:
-Innovative ideas
-Creative ideas
-Strong potential for social impact
-Initiative
-Real community impact
-Clear economic and/or social benefits for women and girls
- Grant Amount
-Maximum Grant
-Up to $500 USD
-The exact award amount is determined by Giving Joy based on:
-Proposed activities
-Availability of funding
- Grant Duration
-The grant period is six months.</t>
-        </is>
-      </c>
-      <c r="D5" s="1" t="inlineStr">
-        <is>
-          <t>Safety</t>
-        </is>
-      </c>
-      <c r="E5" s="1" t="inlineStr">
-        <is>
-          <t>Sep 30, 2026</t>
-        </is>
-      </c>
-      <c r="F5" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/application-invited-for-giving-joy-microgrant-giving-joy-opg-26-00185</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="95" customHeight="1">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Signals of Change Shaping the Future of Sexual and Reproductive Health and Rights SRHR</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-The World Health Organization's mission: to promote health, keep the world safe, and serve the vulnerable. Working through offices in more than 150 countries, WHO staff work side by side with governments and other partners to ensure the highest attainable level of health for all people.
- About the Opportunity
-HRP and its UN co-sponsors are leading a global Sexual and Reproductive Health and Rights (SRHR) foresight and research prioritization process for 2026–2036. This open public consultation invites diverse stakeholder input to identify "signals of change" — emerging trends, shifts, or disruptions — that could shape the future of SRHR over the next decade. The process uses foresight methodology (not prediction) to explore plausible futures and will culminate in a published report and research agenda in 2027.
- Guiding Questions
-What future trends will shape or constrain SRHR over the next 10 years?
-What evidence and research investments are needed today to prepare SRHR for the futures we may face?
- Scope of Submissions 
-Economic systems; social infrastructure; structural discrimination; conflict/forced migration/displacement; mega-trends (demographic shifts, climate change, digital transformation/AI, urbanization); conditions of daily life; rights/legal/governance systems; health systems; media/misinformation; and changes in the research ecosystem.
- Who Can Participate 
-Open to individuals and organizations globally, including:
-Health workers, professional associations, clinical networks
-Civil society, community groups, youth-led organizations, rights movements
-Governments, parliamentarians, regulators, public sector bodies
-Researchers, academia, think tanks, technical experts
-UN agencies, multilateral/humanitarian/development organizations
-Funders, philanthropy, private sector, tech/innovation organizations
-Media, communications, journalism
-Anyone with relevant lived experience or perspective
-Special interest in submissions from health worker, community, youth, and rights-movement spaces not typically represented in published forums.
- Submission Requirements: Descriptive information (name, contact email, country, sector) required alongside each submission; formal published evidence is helpful but not required — practice-based experience and field examples are also welcome. Submissions are kept confidential and anonymized before analysis.</t>
-        </is>
-      </c>
-      <c r="D6" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E6" s="1" t="inlineStr">
-        <is>
-          <t>Sep 30, 2026</t>
-        </is>
-      </c>
-      <c r="F6" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-signals-of-change-shaping-the-future-of-sexual-and-reproductive-health-and-rights-srhr-world-health-organization-opg-26-00176</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="95" customHeight="1">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Setting up Viral Research and Diagnosis Laboratories VRDL in Medical Colleges/Hospitals/Medical Institutions</t>
-        </is>
-      </c>
-      <c r="C7" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-The President notified the creation of the Department of Health Research under the Ministry of Health &amp; Family Welfare through an amendment to the Government of India (Allocation of Business) Rules, 1961 on the 17th September 2007. The Department of Health Research was formally launched on 5th October 2007 by the Minister for Science &amp; Technology and Earth Sciences in a function presided over by the Minister for Health &amp; Family Welfare, in the presence, inter-alia, of the Minister of State for Health &amp; Family Welfare.
-The Department became functional from November 2008 with the appointment of first Secretary of the Department The aim of the DHR is to bring modern health technologies to the people through research and innovations related to diagnosis, treatment methods and vaccines for prevention, to translate them into products and processes and, in synergy with concerned organizations, introduce these innovations into public health system.
- About the Opportunity:
-Under DHR's scheme "Setting-up of nation-wide network of laboratories for managing epidemics and national calamities," proposals are invited from Medical Colleges/Hospitals/Research Institutions to establish a Medical College &amp; Research Institute Level – Viral Research and Diagnosis Laboratory (MCL-VRDL). The existing network comprises 167 VRDLs (11 Regional, 27 State, 129 Medical College level) across 27 states and 5 UTs, aimed at early detection of infectious pathogens, outbreak surveillance, and research on emerging/re-emerging viral diseases.
- Objectives:
-Establish capacity for early detection of common and high-risk infectious pathogens
-Strengthen syndromic surveillance ecosystem for outbreak detection
-Undertake R&amp;D on emerging, re-emerging and novel viruses
- Eligibility (Institution-level):
-State Government Medical Colleges
-Central Government Medical Colleges and Research Institutes
-Armed Forces Medical Institutions/Hospitals
-Railway and other Central Government health institutions
-Private medical colleges ranked in top 50 NIRF ranking
-Must have a dedicated Microbiology department with qualified faculty
-Must have &gt;200 sq.m. area available in existing building (preferably within Microbiology Dept.)
- Funding Provision:
-Non-recurring assistance: Rs. 1.55 crore total
-Rs. 66.8 lakhs — Civil Work (infrastructure modification)
-Rs. 88.2 lakhs — Equipment (complete lab setup)
-No recurring expenditure (staff salaries, consumables, contingency) is provided — to be borne by the host institution
- Role &amp; Responsibilities of the Lab:
-Conduct routine diagnosis of infectious pathogens
-Participate in syndromic and event-based surveillance
-Provide support during outbreaks/epidemics
-Share data with ICMR
- Selection Criteria:
-Meeting eligibility does not guarantee selection; merit-based evaluation by a technical committee
-Preference to institutions in geographically underserved regions
-Weightage for technical strength (qualified faculty, biosafety practices, outbreak investigation experience, publications, patents, externally funded projects)
-Additional weightage for molecular diagnostics, genomic surveillance, One Health research capability, and commitment to long-term recurring support
-Private medical colleges: only top-50 NIRF-ranked institutions considered</t>
-        </is>
-      </c>
-      <c r="D7" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E7" s="1" t="inlineStr">
-        <is>
-          <t>Sep 30, 2026</t>
-        </is>
-      </c>
-      <c r="F7" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-setting-up-viral-research-and-diagnosis-laboratories-vrdl-in-medical-collegeshospitalsmedical-institutions-department-of-health-research-dhr-ministry-of-health-and-family-welfare-government-of-india-opg-26-00174</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="95" customHeight="1">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
-        <is>
-          <t>ToR - Project Management Unit Solarization of Women-led Livelihoods in Maharashtra MAVIMSELCO Foundation Short Duration Project</t>
-        </is>
-      </c>
-      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>Title Project Management Unit – Solarization of Women-led Livelihoods in Maharashtra (MAVIM–SELCO Foundation Short Duration Project)
 Timeline 6 Months (Oct – Mar)
@@ -870,34 +539,34 @@
 Examples of similar past projects, particularly involving SHG networks, livelihood programs, or energy access.</t>
         </is>
       </c>
-      <c r="D8" s="1" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E8" s="1" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Oct 3, 2026</t>
         </is>
       </c>
-      <c r="F8" s="1" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-project-management-unit-solarization-of-women-led-livelihoods-in-maharashtra-mavimselco-foundation-short-duration-project-selco-foundation-rfp-26-00374</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="95" customHeight="1">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="inlineStr">
+    <row r="4" ht="95" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>EOI - Engagement of Agencies for HR Recruitment Services</t>
         </is>
       </c>
-      <c r="C9" s="1" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>The American India Foundation Trust (AIFT) seeks to engage an experienced recruitment agency to provide end-to-end recruitment and talent acquisition services for identified positions across its offices, programmes, and functions in India.
 The selected agency shall support AIFT in sourcing, screening, shortlisting, interview coordination, candidate engagement, offer management, and recruitment closure, in accordance with the requirements, timelines, and service levels agreed with AIFT.
@@ -928,34 +597,34 @@
 Any other information specifically requested by AIFT.</t>
         </is>
       </c>
-      <c r="D9" s="1" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E9" s="1" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>Oct 4, 2026</t>
         </is>
       </c>
-      <c r="F9" s="1" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/eoi-engagement-of-agencies-for-hr-recruitment-services-american-india-foundation-rfp-26-00375</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="95" customHeight="1">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
+    <row r="5" ht="95" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>ToR - Landscape Study for Foundational Literacy and Numeracy FLN Program Six Districts-Jharkhand</t>
         </is>
       </c>
-      <c r="C10" s="1" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>Organizational Overview
 Founded in 2000 on the belief that World Change Starts with Educated Children®, Room to Read develops children’s foundational literacy skills, as well as life skills that promote gender equality. We nurture these essential skills in children by training and coaching educators, creating quality learning materials and spaces, strengthening education systems, and delivering programs directly and with partners – all while honouring the dignity of every child. Committed to accelerating learning outcomes for more children, more quickly, Room to Read has benefited children across 29 countries, with more than 17 million children actively benefiting from our programming in 2025 alone. Room to Read India’s literacy operations currently span across 12 states, with a focus on improving children’s reading skills, access to quality learning materials, and supportive learning environments. Room to Read envisions a world free from illiteracy and gender inequality, where all children have room to read, learn and grow. Visit us at https://www.roomtoreadindia.org/
@@ -967,34 +636,34 @@
 This Landscape Study is being commissioned to build a clear, evidence-based understanding of the current FLN landscape - government systems, school-level realities, and district context - across the six districts, ahead of program design and roll-out. Its purpose is to ensure that the design and contextualization of the program in each district is grounded in accurate, on-the-ground evidence</t>
         </is>
       </c>
-      <c r="D10" s="1" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E10" s="1" t="inlineStr">
+      <c r="E5" s="1" t="inlineStr">
         <is>
           <t>Oct 4, 2026</t>
         </is>
       </c>
-      <c r="F10" s="1" t="inlineStr">
+      <c r="F5" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-landscape-study-for-foundational-literacy-and-numeracy-fln-program-six-districts-jharkhand-room-to-read-india-rfp-26-00376</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="95" customHeight="1">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="inlineStr">
+    <row r="6" ht="95" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>RFP - Design and Delivery of an Electric Vehicle EV Skilling Programme in Karnataka</t>
         </is>
       </c>
-      <c r="C11" s="1" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 WRI India, an independent knowledge organisation registered as the India Resources Trust, provides objective information and practical proposals to foster environmentally sound and socially equitable development. As an independent knowledge organisation, we leverage our data and expertise to catalyze change across systems like food, land and water; energy; and cities. Our work focuses on improving people’s lives, protecting and restoring nature, and addressing climate change. To enable progress at the pace and scale needed, we also engage with the economic, finance and governance systems that are key to enabling this change.
@@ -1035,34 +704,34 @@
 Must have a team of qualified trainers and master trainers with relevant domain expertise, as well as administrative and coordination support.</t>
         </is>
       </c>
-      <c r="D11" s="1" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E11" s="1" t="inlineStr">
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>Oct 5, 2026</t>
         </is>
       </c>
-      <c r="F11" s="1" t="inlineStr">
+      <c r="F6" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfp-design-and-delivery-of-an-electric-vehicle-ev-skilling-programme-in-karnataka-wri-india-rfp-26-00361</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="95" customHeight="1">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="inlineStr">
+    <row r="7" ht="95" customHeight="1">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>ToR for Onboarding of consultant/agency for Innovating &amp; Scaling Reproductive Maternal Newborn and Child Health Solutions in the Last-Mile</t>
         </is>
       </c>
-      <c r="C12" s="1" t="inlineStr">
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>Title Terms of Reference for Onboarding of consultant/agency for Innovating &amp; Scaling Reproductive, Maternal, Newborn and Child Health Solutions in the Last-Mile
 Timeline September 2026 to February 2027
@@ -1096,34 +765,34 @@
 The agency will be selected on a combined technical and financial evaluation. Proposals must score a minimum of 70% on the technical components (1–5 below) to be considered for financial evaluation.</t>
         </is>
       </c>
-      <c r="D12" s="1" t="inlineStr">
+      <c r="D7" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E12" s="1" t="inlineStr">
+      <c r="E7" s="1" t="inlineStr">
         <is>
           <t>Oct 5, 2026</t>
         </is>
       </c>
-      <c r="F12" s="1" t="inlineStr">
+      <c r="F7" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-for-onboarding-of-consultantagency-for-innovating-and-scaling-reproductive-maternal-newborn-and-child-health-solutions-in-the-last-mile-selco-foundation-rfp-26-00373</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="95" customHeight="1">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B13" s="1" t="inlineStr">
+    <row r="8" ht="95" customHeight="1">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>RFPs Invited for Engagement of a Manpower Agency for Providing Subject Matter Specialists/Experts for the Cluster Development Programme</t>
         </is>
       </c>
-      <c r="C13" s="1" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>About the RFP
 National Horticulture Board (NHB), an autonomous organization under the Ministry of Agriculture and Farmers' Welfare, Government of India, invites bids from eligible manpower agencies for engagement to recruit, deploy, and manage qualified personnel supporting NHB's Cluster Development Programme (CDP) — a Central Sector Scheme promoting integrated, market-led horticulture cluster development. The engaged agency will provide three types of Subject Matter Experts per Cluster and additional consultants/manpower as required by NHB from time to time.
@@ -1149,34 +818,159 @@
  District: Gurugram, Haryana (NHB Head Office)</t>
         </is>
       </c>
-      <c r="D13" s="1" t="inlineStr">
+      <c r="D8" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E13" s="1" t="inlineStr">
+      <c r="E8" s="1" t="inlineStr">
         <is>
           <t>Oct 6, 2026</t>
         </is>
       </c>
-      <c r="F13" s="1" t="inlineStr">
+      <c r="F8" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfps-invited-for-engagement-of-a-manpower-agency-for-providing-subject-matter-specialistsexperts-for-the-cluster-development-programme-national-horticulture-board-nhb-rfp-26-00370</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="95" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="inlineStr">
+    <row r="9" ht="95" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>Application Invited GFF x CIVIC VOICES Call for Proposals</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>About us
+PATH is a global nonprofit that turns innovation into better health. For nearly 50 years, PATH has worked with countries, communities, health workers, researchers, governments, and partners to develop and deliver health innovations, from vaccines and diagnostics to strong health systems and more accessible care. By bringing together expertise in science, economics, technology, advocacy, and other fields, PATH develops and scales innovative solutions to the world’s most pressing health challenges. *PATH has become aware of scams involving false job offers.* Please advise: - PATH will never ask for a fee during any stage of the recruitment process. - All active jobs are advertised directly on our careers page: https://path.silkroad.com/epostings/. - Official PATH emails will always arrive from an @path.org address Please report any suspicious communications to careersitehelp@path.org.
+  Civil society and youth-led organizations are essential partners in improving health and nutrition outcomes for women, children, and adolescents. Yet too often, barriers to participation limit their influence.
+The World Bank Group’s GFF × CIVIC partnership—a joint initiative of the Global Financing Facility for Women, Children and Adolescents (GFF) and the CIVIC: The Civil Society and Social Innovation Alliance—works to help close that gap.
+Through its first pillar, the initiative is supporting a consortium led by PATH—in partnership with the African Institute for Development Policy (AFIDEP) and the Organisation of African Youth (OAY), working together as VOICES (Voices Organizing for Inclusive Civic Engagement and Sustainability)—to strengthen civil society engagement, coalition-building, and youth leadership around domestic resource mobilization for women’s, children’s and adolescent health and nutrition. To advance these objectives, the VOICES consortium will award subgrants to local CSOs and youth-led organizations in up to 22 African countries.
+Funding opportunity
+Up to USD 3,350,000 in financial support will be awarded across up to 22 African countries.
+Recipients must be local CSOs or youth-led organizations and/or community-based organizations.
+Each partnership must include at least 2 and no more than 3 organizations, with at least 1 being a youth-led organization.
+Up to 18-month grants, along with advocacy training, budget analysis technical assistance, and mentorship.
+ Application deadline
+Applications close Wednesday, October 7th, 2026 at 23:59 East Africa Time. For more information, including submission details and launch event materials, visit our resource page.
+Call for proposals</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>Oct 7, 2026</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/application-invited-gff-x-civic-voices-call-for-proposals-path-opg-26-00192</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="95" customHeight="1">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>Request for Quotation RfQ for Purchase of Laptops</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>Reference No.: PR_CO_G_2026_162                                                                                            Dated: 28th Sep’ 2026
+ Request for Quotation (RfQ)
+Room to Read India Trust invites electronic quotations from registered Vendors, Suppliers, OEMs and OEM-authorized dealers for the supply of 217 laptops as per the technical specifications and terms specified in this RFQ
+ ABOUT ROOM TO READ INDIA TRUST
+Room to Read India Trust was established in 2003 and today reaches children across twelve states — Bihar, Chhattisgarh, Delhi NCR, Himachal Pradesh Jharkhand, Karnataka, Madhya Pradesh, Maharashtra, Rajasthan, Telangana, Uttarakhand and Uttar Pradesh. As part of the global Room to Read network founded in 2000 on the belief that World Change Starts with Educated Children®, we assist in the development of foundational literacy skills and life skills that promote gender equality. We achieve this by training and coaching educators, creating child‑friendly libraries and learning materials, and partnering with state education systems to ensure sustainable impact. To date, over eighteen million children in India have benefited from our programs. Room to Read envisions a world free from illiteracy and gender inequality, where every child has room to read, learn and grow.
+ OBEJECTIVE
+The objective of this procurement is to procure 217 laptops, meeting the specified technical requirements, while ensuring:
+Compliance with the required technical specifications;
+Quality and authenticity of the equipment;
+Timely delivery and installation;
+Cost-effective procurement for Room to Read India Trust.
+IMPORTANT DATES
+RFQ Issue Date 28th Sep 2026
+Deadline for Submission of Queries 1st Oct 2026
+Deadline for Submission of Quotations 8th Oct 2026
+Bid Opening Date 9th Oct 2026
+SCOPE OF WORK
+The selected vendor must ensure compliance with the SOW requirements, including but not limited to those specified in this document
+ Technical Specifications &amp; Standardization
+The selected vendor shall be responsible for ensuring that all laptops supplied are fully compliant with the Technical Specifications and Standardization guidelines as specified by Room To Read India Trust, with no deviations
+Delivery, Installation &amp; Supply of Hardware
+The selected vendor needs to ensure to deliver the laptop as per the agreed timeline, instruction and location mentioned in RFQ (part delivery, if required).
+The vendor needs to ensure that unboxing, installation, and configuration (OS setup, drivers, connecting to domain/network if applicable) .
+The vendor needs to provide basic testing/demo to confirm proper functioning before handover (if applicable).
+The vendor needs to ensure that all equipment must be brand new, genuine, and unused (no refurbished/reconditioned units)
+Provide part delivery, if required by Room to Read India Trust
+Coordinate with the designated Room to Read India Trust contact for delivery and handover.
+Pre-loaded Software
+The selected vendors need to supply genuine, licensed Operating System (e.g., Windows11 Pro) and other pre-installed software as specified
+Warranty &amp; Support
+The selected vendor needs to ensure that Laptops details must be reflected on the OEM Official website within 7 days post-delivery.
+Damage, Defective or non-conforming units
+The selected vendor needs to ensure that in case any laptop found to be damaged, defective or non-conforming at the time of delivery, inspection or acceptance, shall be replaced/exchanged at no additional cost.
+ MANDATORY DOCUMENTS
+All Bidders need to submit the following mandatory documents along with the Quotation:
+Company profile GST Registration Certificate
+PAN Card of the Organization
+PAN Card of the Owner/Management team
+MSME Certificate, if applicable
+OEM Authorization Certificate, where applicable
+Financial Proposal as per Annexure A
+Cancel Cheque of the Organization only
+* Room to Read India Trust may reject or exclude a quotation that does not contain the required mandatory documents.
+ EVALUATION PARAMETERS
+Proposals/Quotations will be evaluated based on the following parameters:
+Compliance with Technical Specifications
+Commercial/Price Competitiveness
+Delivery Timeline
+Compliance with Eligibility and Mandatory Documentation Requirements
+*Room to Read India Trust reserves the right to seek supporting documents to verify the above eligibility requirements.</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>Oct 8, 2026</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/request-for-quotation-rfq-for-purchase-of-laptops-room-to-read-india-rfp-26-00377</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="95" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>Applications Open Draper Richards Kaplan Foundation Funding for Social Enterprises</t>
         </is>
       </c>
-      <c r="C14" s="1" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>About us
 Started in 2002, Draper Richards Kaplan Foundation (DRK) is a global venture philanthropy firm supporting early stage, high impact social enterprises. Borrowed from our venture capital legacy, DRK finds, funds, and supports exceptional leaders building innovative solutions to some of the world’s most challenging social and environmental problems. Since beginning this work nearly 25 years ago, DRK has invested in more than 270 organizations that have collectively impacted over 610 million lives to date.
@@ -1200,34 +994,189 @@
 Please attach a standard resume/CV for the entrepreneur(s) and/or key leadership team members (e.g., CEO, COO, ED, etc.). Applications with text bios for entrepreneurs or members of the leadership team will not be considered.</t>
         </is>
       </c>
-      <c r="D14" s="1" t="inlineStr">
+      <c r="D11" s="1" t="inlineStr">
         <is>
           <t>Climate</t>
         </is>
       </c>
-      <c r="E14" s="1" t="inlineStr">
+      <c r="E11" s="1" t="inlineStr">
         <is>
           <t>Oct 10, 2026</t>
         </is>
       </c>
-      <c r="F14" s="1" t="inlineStr">
+      <c r="F11" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-open-draper-richards-kaplan-foundation-funding-for-social-enterprises-draper-richards-kaplan-foundation-opg-26-00188</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="95" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="inlineStr">
+    <row r="12" ht="95" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>RFP for Endline Assessment of Digital Equalizer DE Program - RIST</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>Request for Proposal (RFP) Bids are invited By The American India Foundation Trust for Endline Assessment of Digital Equalizer (DE) Program - RIST
+Ref: AIFT/RFP/DL/2026-27/26
+Summary of Deadlines:
+Release of Request for Proposal 28th September 2026
+ Pre-Bid Meeting Registration –
+Prebid Meeting Date &amp; Time: -
+5th Oct-2026 at 4:00 PM to 4:30 PM
+   https://forms.gle/8VbvjgLTmY6xQaXY6
+Prebid Meeting Link
+https://meet.google.com/wzs-qzpj-fii
+  Bid Submission Closing Date
+10th October 2026 (23:59 Hrs. IST)
+Link for submission of proposals:
+Technical:
+https://forms.gle/5DZ6pcFiDxDMGEvw5  
+Financial:
+https://forms.gle/77KuEFkQwiEvqvXD9
+Technical Bid Opening 12th October 2026
+Financial Bid Opening TBD
+Finalization of Contract
+TBD
+(to be intimated to the awardee only)
+ABOUT THE PROJECT
+AIF's implementation strategy aligns with the National Education Policy (NEP) 2020 and is anchored in strategic partnerships and close collaboration with the Government of Uttarakhand. Digital Equalizer 2.0 is a       initiative that aims to improve learning outcomes and strengthen STEM readiness among students in Grades 6–12, with a particular focus on girls. The project also seeks to prepare students for competitive examinations and facilitate their transition to STEM-focused higher education.      
+The overarching goal of the project is to “bridge the gender divide in the workforce by promoting STEM careers among underprivileged girls.” T     he project has been implemented across 40 schools in five districts of Uttarakhand—Almora, Champawat, Dehradun, Udham Singh Nagar, and Pauri Garhwal—with eight schools covered in each district.
+ Specific objectives of the Project
+Strengthening STEM School Education in Rural Government Schools
+Improved performance of underprivileged girls' students from govt schools in competitive examination
+Building Institutional Capacity of 05 DIET on STEM Learning, Techno pedagogy, and preparing Students for the competitive exam.      
+Institutionalized best practices for sustainability through the creation of a playbook in partnership with the Government and sharing evidence of the same
+ SCOPE OF WORK
+The American India Foundation Trust (AIF) seeks to engage an evaluation agency to conduct the endline evaluation of the Digital Equalizer 2.0 project across 5 (five) intervention districts in Uttarakhand. The study will assess the effectiveness of the project’s intervention model and its key components in generating cumulative gains in students’ learning outcomes and STEM readiness, through both curriculum-aligned and competitive examination-focused interventions.
+The endline evaluation will generate robust evidence on the project’s contribution to student learning outcomes and assess changes across the intervention and comparison groups.</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>Oct 10, 2026</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/rfp-for-endline-assessment-of-digital-equalizer-de-program-rist-american-india-foundation-rfp-26-00378</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="95" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>ToR - Catalyse Tech Reproductive Maternal Newborn &amp; Child Health</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>Terms of Reference (TOR) for Call for Applications
+Title
+Catalyse Tech: Reproductive, Maternal, Newborn &amp; Child Health
+Strengthening Maternal, Newborn and Child Health Outcomes Through Certified MedTech and Technology-Enabled Solutions
+Timeline 4-month program from onboarding (November 2026 to February 2027)
+Expected area of expertise
+ Certified MedTech, hardware and/or phygital solutions for Reproductive, Maternal, Newborn &amp; Child Health (RMNCH) – medical devices, diagnostics, screening, monitoring systems, digital health platforms and technology-enabled care models
+Apply Link https://forms.gle/btqACyds77XjfC4j7
+Last     Date             for Apply 10th October 2026 @ 5 pm.
+About SELCO Foundation:
+SELCO Foundation’s mission is to create a platform of solutions that uses sustainable energy as a catalyst to bridge environmental sustainability and poverty alleviation. With holistic development as the primary focus, the organization strives to create equitable societies, where services are accessed by all communities. The interventions of SELCO lead to a sustainable delivery model of essential services like livelihoods, education, and health till the last mile. (Read more about SELCO here: http://www.selcofoundation.org/)
+Objective:
+Enable certified MedTech and technology-enabled RMNCH solutions to move from development to field validation, and from pilot implementation to large-scale adoption in public healthcare systems
+Provide strategic financial support, mentorship and field-testing opportunities to selected innovators/solution providers
+Strengthen implementation capacity, generate evidence of impact, and build pathways for adoption, replication and scale of certified solutions
+Advance inclusive, hardware-led and phygital R&amp;D that strengthens last-mile maternal, newborn and child health service delivery, particularly in underserved and resource-constrained settings
+Scope of Work
+Shortlisted innovators/solution providers may choose to work on all or a part of the activities listed below:
+Technology piloting and field validation of certified solutions
+Implementation strengthening, user feedback and solution refinement based on field learning
+Deployment and scaling of certified maternal and child health technologies in public healthcare systems
+Unlocking relevant schemes and finance
+Conducting research, evidence generation and documentation
+Creating training modules for frontline workers and healthcare providers
+Conducting awareness and orientation workshops with end users, frontline workers, healthcare providers, financial institutions and NGOs
+Documentation of certification/regulatory approvals and empanelment of technologies
+Demonstration of technology at end-user sites/centres
+Demonstration videos and case documentation, and documents for stakeholders
+Selection Criteria:
+In addition to the filled application form, SELCO Foundation will evaluate the applications based on the following criteria:
+Solutions addressing a clearly defined and significant maternal, newborn or child health challenge within the program's focus areas
+Required certification / regulatory approval: the certification(s), regulatory approval(s) or other applicable statutory authorization required for the MedTech product in its intended use and market. Evidence will be required during selection and due diligence
+Technological innovation: a technological component that is original and/or addresses a gap in maternal and child health, with potential for meaningful, real-world impact
+Hardware / phygital integration: hardware, medical devices or phygital elements where relevant to deliver tangible, on-ground solutions; digital-only solutions may be considered where they clearly enable field-level impact
+Impact on women and children: measurable and observable benefits for women, newborns and/or children, either directly or through stronger health-service delivery
+Problem–solution readiness: a clearly defined maternal or child health problem and a developed, certified solution that is ready for implementation, field validation, adoption or scale
+Implementation readiness: the team, operational capacity and partnerships required to deploy, test, refine or scale the certified solution within the program period
+Potential for adoption, replication and scale, particularly in underserved and resource-constrained settings, while improving access, quality, efficiency, safety or health outcomes
+For solutions at the Scale stage: technically sound and well-functioning certified solutions with evidence of use, and intent for post-installation servicing of technologies
+Who can apply:
+Innovators/solution providers that innovate/develop/supply/integrate certified MedTech and technology-enabled solutions for reproductive, maternal, newborn and child health
+Innovators with a certified solution that has been developed and is ready for implementation, or solution providers with a certified solution already being implemented, piloted or deployed with evidence of use
+Innovators/solution providers seeking to test and/or deploy the certified MedTech technologies for field validation and evidence building
+Innovators/solution providers catering to women, newborns, children, caregivers, frontline workers and health systems, particularly in underserved and resource-constrained settings
+Innovators/solution providers looking at working closely with stakeholders such as NGOs/govt. institutes/public health systems/financial institutions for scaling their technologies
+Applicants may collaborate with other entities where this strengthens the solution or its implementation capacity. Ongoing projects and multiple entries are welcome, provided each solution independently meets the eligibility criteria, including the applicable certification/approval requirement
+*Geography – Pan India
+*Early-stage concepts (Ideator category) are not eligible. Applicants must have a developed solution with the required certification/approval.
+Minimum eligibility (screening – pass/fail):
+Applicant is an innovator or solution provider that innovates, develops, supplies or integrates a certified MedTech or technology-enabled solution for reproductive, maternal, newborn or child health (individuals with early-stage/Ideator-category concepts are not eligible)
+Solution holds the required certification(s), regulatory approval(s) or statutory authorization applicable to its intended use and market
+Applicant is based in, or the solution is deployable across, Pan-India geography
+Applicants may collaborate with other entities where this strengthens the solution or its implementation capacity; ongoing projects and multiple entries are welcome, provided each solution independently meets the eligibility criteria
+Submission Requirements:
+Interested innovators/solution providers are requested to submit the following before the deadline:
+Organizational Profile: Overview of the organization and its team.
+Proposed Approach: A clear problem statement, certified solution description, and the Scope of Work activities the applicant proposes to undertake.
+Certification/Regulatory Evidence: Documentary evidence of the certification(s)/regulatory approval(s) applicable to the solution.
+Relevant Portfolio: Evidence of the solution's maturity level and intended impact, including prior deployment/pilot data where applicable (Scale-stage applicants).
+Financial Proposal: Requested budget breakdown for the execution of the proposed Scope of Work activities.</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>Oct 10, 2026</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/tor-catalyse-tech-reproductive-maternal-newborn-and-child-health-selco-foundation-rfp-26-00379</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="95" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund</t>
         </is>
       </c>
-      <c r="C15" s="1" t="inlineStr">
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund
 Apply by: 13 October, 2026
@@ -1252,6 +1201,55 @@
  Projects should include opportunities for ServiceNow employees to volunteer in the project activation or implementation.</t>
         </is>
       </c>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>Oct 13, 2026</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/apply-for-the-servicenow-community-solar-fund-changex-opg-26-00186</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="95" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>RFPs Invited for Empanelment of Publishers for Procurement of E-Books for Rashtriya e-Pustakalaya National Book Trust India</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>About the RFP:
+Rashtriya e-Pustakalaya, a free National Digital Library for children and adolescents — an initiative of the Department of School Education &amp; Literacy, Ministry of Education, Government of India, implemented by the National Book Trust (NBT), India — invites Expression of Interest (EoI) for the empanelment of publishers for the selection and procurement of e-books, with the objective of enriching the platform's book collection. NBT is an autonomous body under the Ministry of Education, established in 1957 to promote literacy and reading culture in India.
+ Scope of Work:
+Provide acceptable, age-appropriate e-books for ages 8–11, 11–14, and 14+ (Young Adults) across genres like Classics, Mystery, Thriller, Historical, Fiction, Science &amp; Technology, Sports &amp; Fitness, Adventure, etc., with special emphasis on promoting the Indian Knowledge System, history, traditions, and achievements of India
+Provide e-books in specified formats (ePUB / searchable PDF) accessible on the Rashtriya e-Pustakalaya app
+Ensure all necessary consents/approvals from authors, illustrators, artists, translators, or legal owners as per the Copyright Act, 1957 and Copyright Rules, 2013
+Ensure necessary licensing agreements and adherence to copyright laws for uninterrupted hosting
+Ensure content relevance to specific age groups and target audience
+Provide content with valid ISBN/RNI registration only
+Provide metadata of e-books in the specified format with periodic updates
+ Eligibility (for Publishers):
+Must be a registered legal entity: Company (Companies Act, 2013) / LLP (LLP Act, 2008) / Trust (Indian Trusts Act, 1882) / Society (Societies Registration Act, 1860) / Partnership firm (Indian Partnership Act, 1932) / Proprietorship firm (registered under Shops &amp; Establishment Act/Labour Department/GST/other statutory department)
+Must hold valid ISBN/RNI registration
+Must have GST Registration (if applicable), PAN, and Aadhar Card (if applicable)
+Must not be blacklisted by the Government of India, any State/UT Government, or their agencies for corrupt/fraudulent/unfair trade practices, or for backing out of a contract after award
+Publisher, directors, and officers must not have been convicted of any criminal offence related to their professional conduct or false statements/misrepresentation in the last 3 years, or otherwise debarred
+No conflict of interest in the empanelment process
+Must indemnify Rashtriya e-Pustakalaya/NBT-India for any IP-related claims from authors/illustrators/translators/legal owners</t>
+        </is>
+      </c>
       <c r="D15" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
@@ -1259,12 +1257,12 @@
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>Oct 13, 2026</t>
+          <t>Oct 16, 2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/grants/apply-for-the-servicenow-community-solar-fund-changex-opg-26-00186</t>
+          <t>https://onepurpos.in/openings/rfps/rfps-invited-for-empanelment-of-publishers-for-procurement-of-e-books-for-rashtriya-e-pustakalaya-national-book-trust-india-national-book-trust-nbt-india-rfp-26-00371</t>
         </is>
       </c>
     </row>
@@ -1368,59 +1366,10 @@
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>RFPs Invited for Empanelment of Publishers for Procurement of E-Books for Rashtriya e-Pustakalaya National Book Trust India</t>
+          <t>RFPs Invited for Consultant to Develop a Technical Assistance Package for National Application of the Digital Health and AI Investment Classification Framework</t>
         </is>
       </c>
       <c r="C17" s="1" t="inlineStr">
-        <is>
-          <t>About the RFP:
-Rashtriya e-Pustakalaya, a free National Digital Library for children and adolescents — an initiative of the Department of School Education &amp; Literacy, Ministry of Education, Government of India, implemented by the National Book Trust (NBT), India — invites Expression of Interest (EoI) for the empanelment of publishers for the selection and procurement of e-books, with the objective of enriching the platform's book collection. NBT is an autonomous body under the Ministry of Education, established in 1957 to promote literacy and reading culture in India.
- Scope of Work:
-Provide acceptable, age-appropriate e-books for ages 8–11, 11–14, and 14+ (Young Adults) across genres like Classics, Mystery, Thriller, Historical, Fiction, Science &amp; Technology, Sports &amp; Fitness, Adventure, etc., with special emphasis on promoting the Indian Knowledge System, history, traditions, and achievements of India
-Provide e-books in specified formats (ePUB / searchable PDF) accessible on the Rashtriya e-Pustakalaya app
-Ensure all necessary consents/approvals from authors, illustrators, artists, translators, or legal owners as per the Copyright Act, 1957 and Copyright Rules, 2013
-Ensure necessary licensing agreements and adherence to copyright laws for uninterrupted hosting
-Ensure content relevance to specific age groups and target audience
-Provide content with valid ISBN/RNI registration only
-Provide metadata of e-books in the specified format with periodic updates
- Eligibility (for Publishers):
-Must be a registered legal entity: Company (Companies Act, 2013) / LLP (LLP Act, 2008) / Trust (Indian Trusts Act, 1882) / Society (Societies Registration Act, 1860) / Partnership firm (Indian Partnership Act, 1932) / Proprietorship firm (registered under Shops &amp; Establishment Act/Labour Department/GST/other statutory department)
-Must hold valid ISBN/RNI registration
-Must have GST Registration (if applicable), PAN, and Aadhar Card (if applicable)
-Must not be blacklisted by the Government of India, any State/UT Government, or their agencies for corrupt/fraudulent/unfair trade practices, or for backing out of a contract after award
-Publisher, directors, and officers must not have been convicted of any criminal offence related to their professional conduct or false statements/misrepresentation in the last 3 years, or otherwise debarred
-No conflict of interest in the empanelment process
-Must indemnify Rashtriya e-Pustakalaya/NBT-India for any IP-related claims from authors/illustrators/translators/legal owners</t>
-        </is>
-      </c>
-      <c r="D17" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E17" s="1" t="inlineStr">
-        <is>
-          <t>Oct 16, 2026</t>
-        </is>
-      </c>
-      <c r="F17" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/rfps-invited-for-empanelment-of-publishers-for-procurement-of-e-books-for-rashtriya-e-pustakalaya-national-book-trust-india-national-book-trust-nbt-india-rfp-26-00371</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="95" customHeight="1">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="inlineStr">
-        <is>
-          <t>RFPs Invited for Consultant to Develop a Technical Assistance Package for National Application of the Digital Health and AI Investment Classification Framework</t>
-        </is>
-      </c>
-      <c r="C18" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are Transform Health: a global coalition of more than 200 organisations driving the digital transformation of health to achieve universal health coverage. 
@@ -1448,34 +1397,34 @@
 Ability to manage multi-country consultancy engagements and coordinate with in-country focal points</t>
         </is>
       </c>
-      <c r="D18" s="1" t="inlineStr">
+      <c r="D17" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E18" s="1" t="inlineStr">
+      <c r="E17" s="1" t="inlineStr">
         <is>
           <t>Oct 23, 2026</t>
         </is>
       </c>
-      <c r="F18" s="1" t="inlineStr">
+      <c r="F17" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfps-invited-for-consultant-to-develop-a-technical-assistance-package-for-national-application-of-the-digital-health-and-ai-investment-classification-framework-transform-health-rfp-26-00359</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="95" customHeight="1">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="inlineStr">
+    <row r="18" ht="95" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for D-Prize Global Competition Seed Funding for New Poverty-Solution Distribution Organizations</t>
         </is>
       </c>
-      <c r="C19" s="1" t="inlineStr">
+      <c r="C18" s="1" t="inlineStr">
         <is>
           <t>About the Grant:
 D-Prize seeds new organizations that distribute proven poverty solutions at the "last mile," with the aim of scaling impact. Applicants select from a range of evidence-based interventions (health, agriculture, education, water, safety, transparency, and more) and propose how they would launch or grow an organization to distribute that intervention. Top entrepreneurs receive up to $20,000 in seed funding to run a pilot and build an organization capable of scaling to reach thousands, even millions of people.
@@ -1498,34 +1447,34 @@
 Extension Deadline: 6 December 2026, midnight PT (extension registration required)</t>
         </is>
       </c>
-      <c r="D19" s="1" t="inlineStr">
+      <c r="D18" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E19" s="1" t="inlineStr">
+      <c r="E18" s="1" t="inlineStr">
         <is>
           <t>Oct 25, 2026</t>
         </is>
       </c>
-      <c r="F19" s="1" t="inlineStr">
+      <c r="F18" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-d-prize-global-competition-seed-funding-for-new-poverty-solution-distribution-organizations-d-prize-opg-26-00191</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="95" customHeight="1">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="inlineStr">
+    <row r="19" ht="95" customHeight="1">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 8th Call for Proposals Small-Size Grants Global EbA Fund</t>
         </is>
       </c>
-      <c r="C20" s="1" t="inlineStr">
+      <c r="C19" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -1588,34 +1537,34 @@
 Only successful applicants will be contacted; no individual feedback provided to unsuccessful applicants</t>
         </is>
       </c>
-      <c r="D20" s="1" t="inlineStr">
+      <c r="D19" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E20" s="1" t="inlineStr">
+      <c r="E19" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F20" s="1" t="inlineStr">
+      <c r="F19" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-8th-call-for-proposals-small-size-grants-global-eba-fund-global-eba-fund-opg-26-00177</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="95" customHeight="1">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="inlineStr">
+    <row r="20" ht="95" customHeight="1">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Adaptive Control Frameworks to Unlock Full-Scale BNR Potential Water Research Foundation WRF</t>
         </is>
       </c>
-      <c r="C21" s="1" t="inlineStr">
+      <c r="C20" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Water Research Foundation (WRF) is the leading research organization advancing the science of all water to meet the evolving needs of its subscribers and the water sector. WRF is a nonprofit, charitable and educational organization which funds, manages, and publishes research on the technology, operation, and management of drinking water, wastewater, reuse, and stormwater collection, treatment and supply systems—all in pursuit of ensuring water quality and improving water services to the public.
@@ -1656,34 +1605,34 @@
 Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
         </is>
       </c>
-      <c r="D21" s="1" t="inlineStr">
+      <c r="D20" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E21" s="1" t="inlineStr">
+      <c r="E20" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F21" s="1" t="inlineStr">
+      <c r="F20" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-adaptive-control-frameworks-to-unlock-full-scale-bnr-potential-water-research-foundation-wrf-the-water-research-foundation-wrf-opg-26-00187</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="95" customHeight="1">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="inlineStr">
+    <row r="21" ht="95" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Crossing the Divide Best Practices for Addressing Local and Privately-Owned Lateral Sewer Issues RFP 5419</t>
         </is>
       </c>
-      <c r="C22" s="1" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>Project Objective:
 To provide water resource recovery facilities (WRRFs) and collection system operators with an interactive manual of practice for implementing inflow and infiltration (I&amp;I) and obstruction management programs, focused on municipal and privately owned lateral sewers in complex legal, regulatory, and multi-jurisdictional environments.
@@ -1721,34 +1670,34 @@
  Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
         </is>
       </c>
-      <c r="D22" s="1" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E22" s="1" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F22" s="1" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-crossing-the-divide-best-practices-for-addressing-local-and-privately-owned-lateral-sewer-issues-rfp-5419-the-water-research-foundation-wrf-opg-26-00189</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="95" customHeight="1">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B23" s="1" t="inlineStr">
+    <row r="22" ht="95" customHeight="1">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Comparison of PFAS Contributions to Agricultural Systems</t>
         </is>
       </c>
-      <c r="C23" s="1" t="inlineStr">
+      <c r="C22" s="1" t="inlineStr">
         <is>
           <t>Project Objectives:
 Report per- and polyfluoroalkyl substance (PFAS) concentrations from a variety of agricultural inputs — animal manures, fertilizers, pesticides, composts, soil amendments, seed coatings, and biosolids-based products
@@ -1784,34 +1733,34 @@
  Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00) — same deadline as the other two WRF grants</t>
         </is>
       </c>
-      <c r="D23" s="1" t="inlineStr">
+      <c r="D22" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E23" s="1" t="inlineStr">
+      <c r="E22" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F23" s="1" t="inlineStr">
+      <c r="F22" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-comparison-of-pfas-contributions-to-agricultural-systems-the-water-research-foundation-wrf-opg-26-00190</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="95" customHeight="1">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B24" s="1" t="inlineStr">
+    <row r="23" ht="95" customHeight="1">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Whitley Award 2027</t>
         </is>
       </c>
-      <c r="C24" s="1" t="inlineStr">
+      <c r="C23" s="1" t="inlineStr">
         <is>
           <t>About the Grant: 
 An annual grant by the Whitley Fund for Nature (WFN) recognising grassroots conservation leaders in the Global South, providing funding to support and scale up proven, science-based solutions that deliver lasting impact for both people and nature.
@@ -1824,34 +1773,34 @@
 You do not need to be invited or nominated to apply.</t>
         </is>
       </c>
-      <c r="D24" s="1" t="inlineStr">
+      <c r="D23" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E24" s="1" t="inlineStr">
+      <c r="E23" s="1" t="inlineStr">
         <is>
           <t>Oct 30, 2026</t>
         </is>
       </c>
-      <c r="F24" s="1" t="inlineStr">
+      <c r="F23" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-whitley-award-2027-whitley-fund-for-nature-wfn-opg-26-00153</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="95" customHeight="1">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B25" s="1" t="inlineStr">
+    <row r="24" ht="95" customHeight="1">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIFAR Global Scholars Program 20272029 Cohort</t>
         </is>
       </c>
-      <c r="C25" s="1" t="inlineStr">
+      <c r="C24" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 CIFAR is a Canadian-based globally influential research organization that convenes the world’s most brilliant people across disciplines to advance transformative knowledge and solve humanity’s biggest problems, together. By supporting long-term interdisciplinary collaboration, CIFAR provides researchers with an unparalleled environment of trust, transparency and knowledge sharing. Our time-tested model inspires new directions of inquiry, accelerates discovery and yields breakthroughs across borders and academic disciplines. Through knowledge mobilization, we are catalysts for change in industry, government and society. Through our 15 research programs and the Pan-Canadian AI Strategy, CIFAR convenes close to 400 of the world’s top researchers from 141 institutions in 20 countries. CIFAR is generously supported by the governments of Canada, Alberta and Québec, as well as foundations, individuals, corporations and Canadian and international partner organizations.
@@ -1895,6 +1844,45 @@
  Application Deadline: November 4, 2026, 12:00 PM EST</t>
         </is>
       </c>
+      <c r="D24" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E24" s="1" t="inlineStr">
+        <is>
+          <t>Nov 4, 2026</t>
+        </is>
+      </c>
+      <c r="F24" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-cifar-global-scholars-program-20272029-cohort-cifar-canadian-institute-for-advanced-research-opg-26-00183</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="95" customHeight="1">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for IWRS Teaching Innovation Award</t>
+        </is>
+      </c>
+      <c r="C25" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
+ About the Grant
+The IWRS (Insect Welfare Research Society) Teaching Innovation Award supports instructors developing new approaches to teaching insect or invertebrate biology that incorporate the 3Rs (Replacement, Reduction, and Refinement) — principles for reducing animal welfare impacts in teaching and research practices.
+ Purpose
+Funds support the creation and implementation of 3Rs-driven instructional materials and pedagogical approaches. Priority is given to proposals addressing common teaching practices with substantial welfare implications.
+ Grant Amount
+Two awards of $2,000 USD are available annually.</t>
+        </is>
+      </c>
       <c r="D25" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
@@ -1902,12 +1890,12 @@
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>Nov 4, 2026</t>
+          <t>Nov 15, 2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-cifar-global-scholars-program-20272029-cohort-cifar-canadian-institute-for-advanced-research-opg-26-00183</t>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
         </is>
       </c>
     </row>
@@ -1961,49 +1949,10 @@
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
-          <t>Applications Invited for IWRS Teaching Innovation Award</t>
+          <t>Applications Invited for Medium-Size Grants Call for Proposals Global EbA Fund</t>
         </is>
       </c>
       <c r="C27" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
- About the Grant
-The IWRS (Insect Welfare Research Society) Teaching Innovation Award supports instructors developing new approaches to teaching insect or invertebrate biology that incorporate the 3Rs (Replacement, Reduction, and Refinement) — principles for reducing animal welfare impacts in teaching and research practices.
- Purpose
-Funds support the creation and implementation of 3Rs-driven instructional materials and pedagogical approaches. Priority is given to proposals addressing common teaching practices with substantial welfare implications.
- Grant Amount
-Two awards of $2,000 USD are available annually.</t>
-        </is>
-      </c>
-      <c r="D27" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E27" s="1" t="inlineStr">
-        <is>
-          <t>Nov 15, 2026</t>
-        </is>
-      </c>
-      <c r="F27" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="95" customHeight="1">
-      <c r="A28" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B28" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Medium-Size Grants Call for Proposals Global EbA Fund</t>
-        </is>
-      </c>
-      <c r="C28" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -2060,34 +2009,34 @@
 Applications submitted via online portal (link shared on the Medium-Size Grants webpage from Oct 12)</t>
         </is>
       </c>
-      <c r="D28" s="1" t="inlineStr">
+      <c r="D27" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E28" s="1" t="inlineStr">
+      <c r="E27" s="1" t="inlineStr">
         <is>
           <t>Nov 16, 2026</t>
         </is>
       </c>
-      <c r="F28" s="1" t="inlineStr">
+      <c r="F27" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-medium-size-grants-call-for-proposals-global-eba-fund-global-eba-fund-opg-26-00178</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="95" customHeight="1">
-      <c r="A29" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B29" s="1" t="inlineStr">
+    <row r="28" ht="95" customHeight="1">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIEIF Grant 2026 Climate Intervention Environmental Impact Fund</t>
         </is>
       </c>
-      <c r="C29" s="1" t="inlineStr">
+      <c r="C28" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Climate Intervention Environmental Impact Fund (CIEIF) is a philanthropic fund focused on supporting responsible climate intervention field tests. It provides grants for activities such as environmental impact assessment (EIA), predictive impact modelling, and engagement with potentially affected stakeholders, including local communities and government agencies.
@@ -2114,34 +2063,34 @@
 Potential for scaling the innovation to a globally relevant level</t>
         </is>
       </c>
-      <c r="D29" s="1" t="inlineStr">
+      <c r="D28" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E29" s="1" t="inlineStr">
+      <c r="E28" s="1" t="inlineStr">
         <is>
           <t>Dec 1, 2026</t>
         </is>
       </c>
-      <c r="F29" s="1" t="inlineStr">
+      <c r="F28" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cieif-grant-2026-climate-intervention-environmental-impact-fund-climate-intervention-environmental-impact-fund-opg-26-00155</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="95" customHeight="1">
-      <c r="A30" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B30" s="1" t="inlineStr">
+    <row r="29" ht="95" customHeight="1">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 6th Annual Seeding The Future Global Food System Challenge</t>
         </is>
       </c>
-      <c r="C30" s="1" t="inlineStr">
+      <c r="C29" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are one of the largest and most respected private organisations for development cooperation and humanitarian aid in Germany. As a politically and confessionally independent organisation, our value-oriented actions are always based on ethical principles. Our vision is clear: "Zero Hunger by 2030"
@@ -2173,78 +2122,34 @@
 Individuals with no organizational entity</t>
         </is>
       </c>
-      <c r="D30" s="1" t="inlineStr">
+      <c r="D29" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E30" s="1" t="inlineStr">
+      <c r="E29" s="1" t="inlineStr">
         <is>
           <t>Jan 1, 2027</t>
         </is>
       </c>
-      <c r="F30" s="1" t="inlineStr">
+      <c r="F29" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-6th-annual-seeding-the-future-global-food-system-challenge-welthungerhilfe-opg-26-00180</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="95" customHeight="1">
-      <c r="A31" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B31" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Microbiota &amp; Women's Health International Call for Projects</t>
-        </is>
-      </c>
-      <c r="C31" s="1" t="inlineStr">
-        <is>
-          <t>About the Grant
-An annual international research grant by the Biocodex Microbiota Foundation (BMF), rewarding research proposals on the microbiota and its implications in Women's Health and Disease. This year's theme: "Unraveling male-female genital microbiome interactions: mechanisms, transmission, and impact on vaginal dysbiosis."
- Theme/Scope
-Proposals could include, but are not limited to, mechanistic studies elucidating how the penile microbiome contributes to the establishment, persistence, and recurrence of vaginal dysbiosis, including bacterial vaginosis. Areas of interest include microbial transmission dynamics during sexual activity, niche adaptation and persistence of BV-associated taxa in the penile environment, and the functional consequences of these interactions for vaginal community stability.
-Studies evaluating how current and emerging interventions (antibiotics, topical or systemic partner therapies, circumcision, or live biotherapeutic products) alter penile microbial ecology and influence treatment response and recurrence risk in female partners are also encouraged.
- Purpose: From 2025, the Biocodex Microbiota Foundation rewards international research proposals involving the microbiota and its implication in Women's Health and Disease. Every year, the call for proposals covers a specific theme chosen by an International Scientific Committee. Either clinical or fundamental research proposals can be submitted. Maximum project duration: 3 years.
- Eligibility
-Open to MDs, PhDs, or Pharm-Ds working in the subject area (gynecology, obstetrics, microbiology, infectious diseases, internal medicine, oncology, etc.).
-No geographic restrictions — all countries are eligible.
-A principal investigator who received a Women's Health International grant from BMF cannot reapply for this award for three years. However, winners of another BMF grant category can apply for this grant.
-Members of the Women's Health International Scientific Committee and their laboratory members are not allowed to apply as Principal Investigators.
- Grant Amount
-€200,000 annually — awarded to researchers within universities, hospitals, or other research settings to finance equipment, operations, or staffing costs. Grants are NOT awarded to individuals directly (must be institutionally affiliated). Institution's overhead costs capped at 10%.</t>
-        </is>
-      </c>
-      <c r="D31" s="1" t="inlineStr">
-        <is>
-          <t>Safety</t>
-        </is>
-      </c>
-      <c r="E31" s="1" t="inlineStr">
-        <is>
-          <t>Jan 15, 2027</t>
-        </is>
-      </c>
-      <c r="F31" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-microbiota-and-womens-health-international-call-for-projects-biocodex-microbiota-foundation-bmf-opg-26-00152</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="95" customHeight="1">
-      <c r="A32" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B32" s="1" t="inlineStr">
+    <row r="30" ht="95" customHeight="1">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for BES Training and Travel Grants</t>
         </is>
       </c>
-      <c r="C32" s="1" t="inlineStr">
+      <c r="C30" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are a global community of scientists shining a spotlight on the intricacy and value of our natural world, providing the evidence for better decisions. Our vision is for people and nature to thrive in a world that values ecology.
@@ -2283,17 +2188,17 @@
  Application Deadline (Round 2): Opens 30 April 2026, closes 17 May 2026</t>
         </is>
       </c>
-      <c r="D32" s="1" t="inlineStr">
+      <c r="D30" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E32" s="1" t="inlineStr">
+      <c r="E30" s="1" t="inlineStr">
         <is>
           <t>May 17, 2027</t>
         </is>
       </c>
-      <c r="F32" s="1" t="inlineStr">
+      <c r="F30" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-bes-training-and-travel-grants-british-ecological-society-opg-26-00181</t>
         </is>

</xml_diff>

<commit_message>
Auto update Combined.xlsx [Wed Sep 30 07:52:15 UTC 2026]
</commit_message>
<xml_diff>
--- a/output/Combined.xlsx
+++ b/output/Combined.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1225,10 +1225,118 @@
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
+          <t>EOI invited for Consultant Road Safety Expert / Technical</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>Position Consultant – Road Safety Expert / Technical
+Function Road Safety &amp; Technical Projects
+Base location Delhi NCR preferred, with travel to Project Sites as per requirement 
+Experience Minimum 7 years (candidates with 7–12 years are the primary target; more senior applicants are welcome)
+Engagement Independent consultancy – deliverable-based and non-exclusive
+Who can apply Individual consultants
+Coordination &amp; Reporting To Project Manager
+Last date to apply 15 October 2026
+About the Assignment
+Bharatcares is a CSR implementation organisation based in Ahmedabad, working with corporate, government and community partners across road safety, women’s entrepreneurship, Health Care, Livelihoods, Environment and skill development. As its road safety portfolio grows, Bharatcares is seeking an experienced independent consultant (individual) to lead the engineering side of multi-location road safety projects. 
+ The Consultant will provide end-to-end technical support across road safety audits, post-audit implementation, civil and engineering interventions, technical specifications, quality assurance, documentation and government coordination. The role is the technical link between the project team, engineering and civil vendors, other consultants and government stakeholders, ensuring that proposed and implemented interventions are technically appropriate, standards-compliant, feasible and properly documented.
+ 2. Scope of Work
+A. Road Safety Audit &amp; Technical Assessment
+Conduct and/or lead Road Safety Audits (RSA) for road stretches, intersections, blackspots, school zones and other high-risk locations.
+Undertake site reconnaissance covering road geometry, traffic and pedestrian movement, signage, markings, visibility, road condition, drainage, conflict points and existing safety infrastructure.
+Review crash and blackspot data (police records, iRAD/eDAR where available) with field observations; support GIS-based mapping of risk locations.
+Prepare audit reports with risk observations, photographs, GPS/location references and prioritised countermeasures.
+Conduct pre- and post-implementation assessments, including before/after comparison of risk and, where data permits, crash outcomes.
+B. Engineering &amp; Infrastructure Interventions
+Translate audit findings into location-specific, executable engineering interventions.
+Develop/review technical specifications for: road signage, sign supports and retro-reflective systems; road markings and thermoplastic applications; rumble strips and speed-calming measures; pedestrian crossings and school-zone infrastructure; bollards, barricades, guardrails and road furniture; median/road-edge treatments and railings; reflective safety infrastructure and lighting; other civil/road safety interventions as required.
+Define material specifications, dimensions, grades, thickness, reflectivity, fixing methods and installation requirements.
+Prepare and/or review BoQs, cost estimates, technical drawings, layouts, material samples and vendor technical proposals.
+Ensure alignment with applicable IRC, MoRTH, BIS and state/local standards (for example IRC:SP:88 for RSA, and the relevant IRC codes for signs, markings, traffic calming and pedestrian facilities).
+C. Post-Audit Implementation &amp; Quality Control
+Convert approved audit recommendations into practical implementation packages and provide technical inputs during procurement and vendor finalisation.
+Inspect sites during implementation to verify materials, dimensions, placement, workmanship and technical compliance, including review of test certificates and retro-reflectivity/third-party test results where applicable.
+Check that traffic management and worker safety arrangements are in place during works.
+Identify deviations, recommend corrective actions and recommend rejection of non-conforming materials or work.
+Verify completed works against approved specifications and audit recommendations; support technical sign-off, completion, handover and defect-liability/warranty documentation.
+D. Government Coordination &amp; Permissions
+Coordinate with relevant stakeholders including the Transport Department, RTOs, Traffic Police, Municipal Corporations, PWD, NHAI and other authorities, identifying the road-owning agency for each location.
+Prepare/review technical documents for submissions and permissions: audit reports, drawings, BoQs, site photographs, technical notes and intervention proposals.
+Facilitate technical discussions and joint site visits, address queries, incorporate required modifications, and track approvals and follow-ups so that permissions are in place before implementation.
+E. Technical Documentation &amp; Reporting
+Prepare/review RSA and post-audit reports; technical assessment reports; specifications and BoQs; drawings and intervention plans; government submission documents; site inspection and quality reports; and completion, handover and post-implementation reports.
+Maintain traceability from audit findings → approved interventions → BoQ → actual implementation → post-implementation verification.
+Contribute technical inputs, photo-documented progress and outcome indicators to BHARATCARES’s funder and stakeholder reports.
+Develop standardised technical templates and checklists for multi-location projects.
+3. Independence &amp; Working Arrangements
+The Consultant works as an independent professional or firm and is not an employee of BHARATCARES. The Consultant plans site visits and work schedules in agreement with project timelines and coordinates with the BHARATCARES Project Manager on scope, access and reporting.
+The engagement is non-exclusive: the Consultant may take other assignments, provided there is no conflict of interest with BHARATCARES projects, clients or funders, and that agreed deadlines are met.
+Technical recommendations are made by the Consultant; final technical sign-off rests with Project Manager. Vendor selection and contracting decisions remain with BHARATCARES; the Consultant provides technical evaluation and may flag deviations and recommend rejection of non-conforming work.
+Where required by the client or road-owning agency, BHARATCARES will separate the audit, design and final verification roles for a location. 
+4. Key Deliverables
+# Deliverable
+1 Location-specific Road Safety Audit reports
+2 Technical intervention designs and recommendations
+3 Technical specifications, BoQs and material standards
+4 Technical review of drawings and vendor proposals
+5 Government submission and permission documentation
+6 Site inspection and quality assurance reports
+7 Post-implementation technical assessment
+8 Completion, handover and technical compliance documentation
+9 Standardised technical templates and checklists for multi-location projects
+5. Qualifications &amp; Experience
+Essential
+B.E./B.Tech in Civil Engineering, Transportation Engineering, Highway Engineering or a related discipline.
+Minimum 7 years of relevant experience in road safety, highway/traffic engineering, civil infrastructure or related projects.
+Formal training or certification in Road Safety Audit, with demonstrated experience of leading or co-leading multiple RSAs and implementing road safety infrastructure interventions.
+Experience in technical documentation, BoQ/specification review and site supervision.
+Experience coordinating with government and public-sector stakeholders.
+Proficiency in English and Hindi. 
+Willingness to travel extensively to project locations.
+Firms must nominate a lead expert who individually meets the essential criteria above.
+Desirable
+Working knowledge of IRC, MoRTH and BIS standards; prior work with or empanelment by NHAI, state PWDs or similar agencies.
+Experience with blackspot/crash data analysis, iRAD, GIS mapping (QGIS/ArcGIS) and AutoCAD.
+Experience in multi-location CSR, public infrastructure or social impact projects, including funder reporting.
+6. Core Competencies
+Road Safety Engineering  |  Road Safety Audits  |  Civil/Highway Engineering  | Traffic Engineering  |  Technical Specifications  |  BoQ &amp; Drawing Review  |  Quality Assurance  |  Site Inspection  |  Government Liaison &amp; Permissions  | Vendor Technical Management |  Technical Documentation  |  Risk Assessment
+7. Engagement Terms
+Type of engagement Independent consultancy (non-exclusive); not an employment
+Duration 6 Months (Renewal subject to review and Project Requirememt)
+Expected start date 20th October 2026
+Payment terms KPI and Deliverables Linked (to be decided as per Project Implementation Calendar) “Fees will be discussed with applicants after profiles are shortlisted, that payment will be linked to accepted deliverables, and that taxes/TDS apply as per law”
+Travel &amp; local conveyance Reimbursement as per Organization’s Internal Policy and Budget</t>
+        </is>
+      </c>
+      <c r="D15" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E15" s="1" t="inlineStr">
+        <is>
+          <t>Oct 15, 2026</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/eoi-invited-for-consultant-road-safety-expert-technical-bharatcares-rfp-26-00381</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="95" customHeight="1">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
           <t>RFPs Invited for Empanelment of Publishers for Procurement of E-Books for Rashtriya e-Pustakalaya National Book Trust India</t>
         </is>
       </c>
-      <c r="C15" s="1" t="inlineStr">
+      <c r="C16" s="1" t="inlineStr">
         <is>
           <t>About the RFP:
 Rashtriya e-Pustakalaya, a free National Digital Library for children and adolescents — an initiative of the Department of School Education &amp; Literacy, Ministry of Education, Government of India, implemented by the National Book Trust (NBT), India — invites Expression of Interest (EoI) for the empanelment of publishers for the selection and procurement of e-books, with the objective of enriching the platform's book collection. NBT is an autonomous body under the Ministry of Education, established in 1957 to promote literacy and reading culture in India.
@@ -1250,34 +1358,34 @@
 Must indemnify Rashtriya e-Pustakalaya/NBT-India for any IP-related claims from authors/illustrators/translators/legal owners</t>
         </is>
       </c>
-      <c r="D15" s="1" t="inlineStr">
+      <c r="D16" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E15" s="1" t="inlineStr">
+      <c r="E16" s="1" t="inlineStr">
         <is>
           <t>Oct 16, 2026</t>
         </is>
       </c>
-      <c r="F15" s="1" t="inlineStr">
+      <c r="F16" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfps-invited-for-empanelment-of-publishers-for-procurement-of-e-books-for-rashtriya-e-pustakalaya-national-book-trust-india-national-book-trust-nbt-india-rfp-26-00371</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="95" customHeight="1">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B16" s="1" t="inlineStr">
+    <row r="17" ht="95" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
         <is>
           <t>ToR - Engagement of Consultant/Vendor Individual towards implementation of Literacy Program in Telangana State</t>
         </is>
       </c>
-      <c r="C16" s="1" t="inlineStr">
+      <c r="C17" s="1" t="inlineStr">
         <is>
           <t>ANNEX A – TERMS OF REFERENCE (ToR) 
  Engagement of Consultant/Vendor (Individual) towards implementation of Literacy Program in Telangana State.
@@ -1342,34 +1450,34 @@
 Approved travel and accommodation expenses incurred for assignment-related activities shall be reimbursed by Room to Read in accordance with the consultancy reimbursement guidelines.</t>
         </is>
       </c>
-      <c r="D16" s="1" t="inlineStr">
+      <c r="D17" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E16" s="1" t="inlineStr">
+      <c r="E17" s="1" t="inlineStr">
         <is>
           <t>Oct 16, 2026</t>
         </is>
       </c>
-      <c r="F16" s="1" t="inlineStr">
+      <c r="F17" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-engagement-of-consultantvendor-individual-towards-implementation-of-literacy-program-in-telangana-state-room-to-read-india-rfp-26-00360</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="95" customHeight="1">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B17" s="1" t="inlineStr">
+    <row r="18" ht="95" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>RFPs Invited for Consultant to Develop a Technical Assistance Package for National Application of the Digital Health and AI Investment Classification Framework</t>
         </is>
       </c>
-      <c r="C17" s="1" t="inlineStr">
+      <c r="C18" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are Transform Health: a global coalition of more than 200 organisations driving the digital transformation of health to achieve universal health coverage. 
@@ -1397,34 +1505,34 @@
 Ability to manage multi-country consultancy engagements and coordinate with in-country focal points</t>
         </is>
       </c>
-      <c r="D17" s="1" t="inlineStr">
+      <c r="D18" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E17" s="1" t="inlineStr">
+      <c r="E18" s="1" t="inlineStr">
         <is>
           <t>Oct 23, 2026</t>
         </is>
       </c>
-      <c r="F17" s="1" t="inlineStr">
+      <c r="F18" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfps-invited-for-consultant-to-develop-a-technical-assistance-package-for-national-application-of-the-digital-health-and-ai-investment-classification-framework-transform-health-rfp-26-00359</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="95" customHeight="1">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="inlineStr">
+    <row r="19" ht="95" customHeight="1">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for D-Prize Global Competition Seed Funding for New Poverty-Solution Distribution Organizations</t>
         </is>
       </c>
-      <c r="C18" s="1" t="inlineStr">
+      <c r="C19" s="1" t="inlineStr">
         <is>
           <t>About the Grant:
 D-Prize seeds new organizations that distribute proven poverty solutions at the "last mile," with the aim of scaling impact. Applicants select from a range of evidence-based interventions (health, agriculture, education, water, safety, transparency, and more) and propose how they would launch or grow an organization to distribute that intervention. Top entrepreneurs receive up to $20,000 in seed funding to run a pilot and build an organization capable of scaling to reach thousands, even millions of people.
@@ -1447,34 +1555,34 @@
 Extension Deadline: 6 December 2026, midnight PT (extension registration required)</t>
         </is>
       </c>
-      <c r="D18" s="1" t="inlineStr">
+      <c r="D19" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E18" s="1" t="inlineStr">
+      <c r="E19" s="1" t="inlineStr">
         <is>
           <t>Oct 25, 2026</t>
         </is>
       </c>
-      <c r="F18" s="1" t="inlineStr">
+      <c r="F19" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-d-prize-global-competition-seed-funding-for-new-poverty-solution-distribution-organizations-d-prize-opg-26-00191</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="95" customHeight="1">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="inlineStr">
+    <row r="20" ht="95" customHeight="1">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 8th Call for Proposals Small-Size Grants Global EbA Fund</t>
         </is>
       </c>
-      <c r="C19" s="1" t="inlineStr">
+      <c r="C20" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -1537,34 +1645,34 @@
 Only successful applicants will be contacted; no individual feedback provided to unsuccessful applicants</t>
         </is>
       </c>
-      <c r="D19" s="1" t="inlineStr">
+      <c r="D20" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E19" s="1" t="inlineStr">
+      <c r="E20" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F19" s="1" t="inlineStr">
+      <c r="F20" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-8th-call-for-proposals-small-size-grants-global-eba-fund-global-eba-fund-opg-26-00177</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="95" customHeight="1">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="inlineStr">
+    <row r="21" ht="95" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Adaptive Control Frameworks to Unlock Full-Scale BNR Potential Water Research Foundation WRF</t>
         </is>
       </c>
-      <c r="C20" s="1" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Water Research Foundation (WRF) is the leading research organization advancing the science of all water to meet the evolving needs of its subscribers and the water sector. WRF is a nonprofit, charitable and educational organization which funds, manages, and publishes research on the technology, operation, and management of drinking water, wastewater, reuse, and stormwater collection, treatment and supply systems—all in pursuit of ensuring water quality and improving water services to the public.
@@ -1605,34 +1713,34 @@
 Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
         </is>
       </c>
-      <c r="D20" s="1" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E20" s="1" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F20" s="1" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-adaptive-control-frameworks-to-unlock-full-scale-bnr-potential-water-research-foundation-wrf-the-water-research-foundation-wrf-opg-26-00187</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="95" customHeight="1">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="inlineStr">
+    <row r="22" ht="95" customHeight="1">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Crossing the Divide Best Practices for Addressing Local and Privately-Owned Lateral Sewer Issues RFP 5419</t>
         </is>
       </c>
-      <c r="C21" s="1" t="inlineStr">
+      <c r="C22" s="1" t="inlineStr">
         <is>
           <t>Project Objective:
 To provide water resource recovery facilities (WRRFs) and collection system operators with an interactive manual of practice for implementing inflow and infiltration (I&amp;I) and obstruction management programs, focused on municipal and privately owned lateral sewers in complex legal, regulatory, and multi-jurisdictional environments.
@@ -1670,34 +1778,34 @@
  Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
         </is>
       </c>
-      <c r="D21" s="1" t="inlineStr">
+      <c r="D22" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E21" s="1" t="inlineStr">
+      <c r="E22" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F21" s="1" t="inlineStr">
+      <c r="F22" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-crossing-the-divide-best-practices-for-addressing-local-and-privately-owned-lateral-sewer-issues-rfp-5419-the-water-research-foundation-wrf-opg-26-00189</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="95" customHeight="1">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="inlineStr">
+    <row r="23" ht="95" customHeight="1">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Comparison of PFAS Contributions to Agricultural Systems</t>
         </is>
       </c>
-      <c r="C22" s="1" t="inlineStr">
+      <c r="C23" s="1" t="inlineStr">
         <is>
           <t>Project Objectives:
 Report per- and polyfluoroalkyl substance (PFAS) concentrations from a variety of agricultural inputs — animal manures, fertilizers, pesticides, composts, soil amendments, seed coatings, and biosolids-based products
@@ -1733,34 +1841,34 @@
  Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00) — same deadline as the other two WRF grants</t>
         </is>
       </c>
-      <c r="D22" s="1" t="inlineStr">
+      <c r="D23" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E22" s="1" t="inlineStr">
+      <c r="E23" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F22" s="1" t="inlineStr">
+      <c r="F23" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-comparison-of-pfas-contributions-to-agricultural-systems-the-water-research-foundation-wrf-opg-26-00190</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="95" customHeight="1">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B23" s="1" t="inlineStr">
+    <row r="24" ht="95" customHeight="1">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Whitley Award 2027</t>
         </is>
       </c>
-      <c r="C23" s="1" t="inlineStr">
+      <c r="C24" s="1" t="inlineStr">
         <is>
           <t>About the Grant: 
 An annual grant by the Whitley Fund for Nature (WFN) recognising grassroots conservation leaders in the Global South, providing funding to support and scale up proven, science-based solutions that deliver lasting impact for both people and nature.
@@ -1773,34 +1881,34 @@
 You do not need to be invited or nominated to apply.</t>
         </is>
       </c>
-      <c r="D23" s="1" t="inlineStr">
+      <c r="D24" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E23" s="1" t="inlineStr">
+      <c r="E24" s="1" t="inlineStr">
         <is>
           <t>Oct 30, 2026</t>
         </is>
       </c>
-      <c r="F23" s="1" t="inlineStr">
+      <c r="F24" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-whitley-award-2027-whitley-fund-for-nature-wfn-opg-26-00153</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="95" customHeight="1">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B24" s="1" t="inlineStr">
+    <row r="25" ht="95" customHeight="1">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIFAR Global Scholars Program 20272029 Cohort</t>
         </is>
       </c>
-      <c r="C24" s="1" t="inlineStr">
+      <c r="C25" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 CIFAR is a Canadian-based globally influential research organization that convenes the world’s most brilliant people across disciplines to advance transformative knowledge and solve humanity’s biggest problems, together. By supporting long-term interdisciplinary collaboration, CIFAR provides researchers with an unparalleled environment of trust, transparency and knowledge sharing. Our time-tested model inspires new directions of inquiry, accelerates discovery and yields breakthroughs across borders and academic disciplines. Through knowledge mobilization, we are catalysts for change in industry, government and society. Through our 15 research programs and the Pan-Canadian AI Strategy, CIFAR convenes close to 400 of the world’s top researchers from 141 institutions in 20 countries. CIFAR is generously supported by the governments of Canada, Alberta and Québec, as well as foundations, individuals, corporations and Canadian and international partner organizations.
@@ -1844,58 +1952,19 @@
  Application Deadline: November 4, 2026, 12:00 PM EST</t>
         </is>
       </c>
-      <c r="D24" s="1" t="inlineStr">
+      <c r="D25" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E24" s="1" t="inlineStr">
+      <c r="E25" s="1" t="inlineStr">
         <is>
           <t>Nov 4, 2026</t>
         </is>
       </c>
-      <c r="F24" s="1" t="inlineStr">
+      <c r="F25" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cifar-global-scholars-program-20272029-cohort-cifar-canadian-institute-for-advanced-research-opg-26-00183</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="95" customHeight="1">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B25" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for IWRS Teaching Innovation Award</t>
-        </is>
-      </c>
-      <c r="C25" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
- About the Grant
-The IWRS (Insect Welfare Research Society) Teaching Innovation Award supports instructors developing new approaches to teaching insect or invertebrate biology that incorporate the 3Rs (Replacement, Reduction, and Refinement) — principles for reducing animal welfare impacts in teaching and research practices.
- Purpose
-Funds support the creation and implementation of 3Rs-driven instructional materials and pedagogical approaches. Priority is given to proposals addressing common teaching practices with substantial welfare implications.
- Grant Amount
-Two awards of $2,000 USD are available annually.</t>
-        </is>
-      </c>
-      <c r="D25" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E25" s="1" t="inlineStr">
-        <is>
-          <t>Nov 15, 2026</t>
-        </is>
-      </c>
-      <c r="F25" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
         </is>
       </c>
     </row>
@@ -1949,10 +2018,49 @@
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
+          <t>Applications Invited for IWRS Teaching Innovation Award</t>
+        </is>
+      </c>
+      <c r="C27" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
+ About the Grant
+The IWRS (Insect Welfare Research Society) Teaching Innovation Award supports instructors developing new approaches to teaching insect or invertebrate biology that incorporate the 3Rs (Replacement, Reduction, and Refinement) — principles for reducing animal welfare impacts in teaching and research practices.
+ Purpose
+Funds support the creation and implementation of 3Rs-driven instructional materials and pedagogical approaches. Priority is given to proposals addressing common teaching practices with substantial welfare implications.
+ Grant Amount
+Two awards of $2,000 USD are available annually.</t>
+        </is>
+      </c>
+      <c r="D27" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E27" s="1" t="inlineStr">
+        <is>
+          <t>Nov 15, 2026</t>
+        </is>
+      </c>
+      <c r="F27" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="95" customHeight="1">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
+        <is>
           <t>Applications Invited for Medium-Size Grants Call for Proposals Global EbA Fund</t>
         </is>
       </c>
-      <c r="C27" s="1" t="inlineStr">
+      <c r="C28" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -2009,34 +2117,34 @@
 Applications submitted via online portal (link shared on the Medium-Size Grants webpage from Oct 12)</t>
         </is>
       </c>
-      <c r="D27" s="1" t="inlineStr">
+      <c r="D28" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E27" s="1" t="inlineStr">
+      <c r="E28" s="1" t="inlineStr">
         <is>
           <t>Nov 16, 2026</t>
         </is>
       </c>
-      <c r="F27" s="1" t="inlineStr">
+      <c r="F28" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-medium-size-grants-call-for-proposals-global-eba-fund-global-eba-fund-opg-26-00178</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="95" customHeight="1">
-      <c r="A28" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B28" s="1" t="inlineStr">
+    <row r="29" ht="95" customHeight="1">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIEIF Grant 2026 Climate Intervention Environmental Impact Fund</t>
         </is>
       </c>
-      <c r="C28" s="1" t="inlineStr">
+      <c r="C29" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Climate Intervention Environmental Impact Fund (CIEIF) is a philanthropic fund focused on supporting responsible climate intervention field tests. It provides grants for activities such as environmental impact assessment (EIA), predictive impact modelling, and engagement with potentially affected stakeholders, including local communities and government agencies.
@@ -2063,34 +2171,34 @@
 Potential for scaling the innovation to a globally relevant level</t>
         </is>
       </c>
-      <c r="D28" s="1" t="inlineStr">
+      <c r="D29" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E28" s="1" t="inlineStr">
+      <c r="E29" s="1" t="inlineStr">
         <is>
           <t>Dec 1, 2026</t>
         </is>
       </c>
-      <c r="F28" s="1" t="inlineStr">
+      <c r="F29" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cieif-grant-2026-climate-intervention-environmental-impact-fund-climate-intervention-environmental-impact-fund-opg-26-00155</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="95" customHeight="1">
-      <c r="A29" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B29" s="1" t="inlineStr">
+    <row r="30" ht="95" customHeight="1">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 6th Annual Seeding The Future Global Food System Challenge</t>
         </is>
       </c>
-      <c r="C29" s="1" t="inlineStr">
+      <c r="C30" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are one of the largest and most respected private organisations for development cooperation and humanitarian aid in Germany. As a politically and confessionally independent organisation, our value-oriented actions are always based on ethical principles. Our vision is clear: "Zero Hunger by 2030"
@@ -2122,34 +2230,34 @@
 Individuals with no organizational entity</t>
         </is>
       </c>
-      <c r="D29" s="1" t="inlineStr">
+      <c r="D30" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E29" s="1" t="inlineStr">
+      <c r="E30" s="1" t="inlineStr">
         <is>
           <t>Jan 1, 2027</t>
         </is>
       </c>
-      <c r="F29" s="1" t="inlineStr">
+      <c r="F30" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-6th-annual-seeding-the-future-global-food-system-challenge-welthungerhilfe-opg-26-00180</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="95" customHeight="1">
-      <c r="A30" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B30" s="1" t="inlineStr">
+    <row r="31" ht="95" customHeight="1">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for BES Training and Travel Grants</t>
         </is>
       </c>
-      <c r="C30" s="1" t="inlineStr">
+      <c r="C31" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are a global community of scientists shining a spotlight on the intricacy and value of our natural world, providing the evidence for better decisions. Our vision is for people and nature to thrive in a world that values ecology.
@@ -2188,17 +2296,17 @@
  Application Deadline (Round 2): Opens 30 April 2026, closes 17 May 2026</t>
         </is>
       </c>
-      <c r="D30" s="1" t="inlineStr">
+      <c r="D31" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E30" s="1" t="inlineStr">
+      <c r="E31" s="1" t="inlineStr">
         <is>
           <t>May 17, 2027</t>
         </is>
       </c>
-      <c r="F30" s="1" t="inlineStr">
+      <c r="F31" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-bes-training-and-travel-grants-british-ecological-society-opg-26-00181</t>
         </is>

</xml_diff>

<commit_message>
Auto update Combined.xlsx [Fri Oct  2 07:53:22 UTC 2026]
</commit_message>
<xml_diff>
--- a/output/Combined.xlsx
+++ b/output/Combined.xlsx
@@ -467,7 +467,7 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>State Project Coordinator</t>
+          <t>Country Economist [Open to internal and external applicants]</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
@@ -478,12 +478,12 @@
       <c r="D2" s="1" t="inlineStr"/>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>10/12/2026, 03:59 AM</t>
+          <t>10/15/2026, 05:00 AM</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://estm.fa.em2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1/job/37164/?location=India&amp;locationId=300000000440677&amp;locationLevel=country&amp;mode=location</t>
+          <t>https://estm.fa.em2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1/job/37241/?location=India&amp;locationId=300000000440677&amp;locationLevel=country&amp;mode=location</t>
         </is>
       </c>
     </row>
@@ -1487,34 +1487,12 @@
       </c>
       <c r="C22" s="1" t="inlineStr">
         <is>
-          <t>About the Organization
-Climate Intervention Environmental Impact Fund (CIEIF) is a philanthropic fund focused on supporting responsible climate intervention field tests. It provides grants for activities such as environmental impact assessment (EIA), predictive impact modelling, and engagement with potentially affected stakeholders, including local communities and government agencies.
-CIEIF aims to help climate-intervention projects better understand their potential technical, environmental, economic, social, public-health, and safety impacts before and during field testing. It also places importance on the scalability and global relevance of supported innovations and encourages publication of field-test results through peer-reviewed journals or externally peer-reviewed reports.
- About the Grant
-The Climate Intervention Environmental Impact Fund (CIEIF) Grant provides USD 75,000 to support proposed climate intervention field tests. The funding is specifically intended for Environmental Impact Assessment (EIA), predictive impact modelling, and/or engagement with potentially affected stakeholders, including local communities and government agencies.
-Applicants are expected to demonstrate the proposed field test’s technical readiness, environmental and social considerations, required government approvals, innovation and potential for globally relevant scalability. The application must include a proposed budget showing how the USD 75,000 will be used.
- Grant Objective
-The grant is intended to support proposed climate intervention field tests, particularly activities related to:
-Environmental Impact Assessment (EIA)
-Predictive impact modeling
-Engagement with potentially impacted stakeholders
-Local community and government engagement
-Understanding technical, environmental, economic, social, public-health, and safety challenges
-The proposed application must focus on at least one of these three core areas: EIA, predictive impact modeling, or stakeholder engagement.
- Eligible Project Focus
-The proposed field test should demonstrate:
-A clear climate-intervention concept
-Prior research indicating that the technology is ready for the proposed field test
-Potential for innovation and scalability
-A clear understanding of technical and environmental challenges
-Consideration of economic, social, public-health, and safety implications
-Relevant government permits and approvals
-Potential for scaling the innovation to a globally relevant level</t>
+          <t>No description available</t>
         </is>
       </c>
       <c r="D22" s="1" t="inlineStr">
         <is>
-          <t>Governance</t>
+          <t>Climate</t>
         </is>
       </c>
       <c r="E22" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Auto update Combined.xlsx [Sat Oct  3 07:29:09 UTC 2026]
</commit_message>
<xml_diff>
--- a/output/Combined.xlsx
+++ b/output/Combined.xlsx
@@ -1487,12 +1487,34 @@
       </c>
       <c r="C22" s="1" t="inlineStr">
         <is>
-          <t>No description available</t>
+          <t>About the Organization
+Climate Intervention Environmental Impact Fund (CIEIF) is a philanthropic fund focused on supporting responsible climate intervention field tests. It provides grants for activities such as environmental impact assessment (EIA), predictive impact modelling, and engagement with potentially affected stakeholders, including local communities and government agencies.
+CIEIF aims to help climate-intervention projects better understand their potential technical, environmental, economic, social, public-health, and safety impacts before and during field testing. It also places importance on the scalability and global relevance of supported innovations and encourages publication of field-test results through peer-reviewed journals or externally peer-reviewed reports.
+ About the Grant
+The Climate Intervention Environmental Impact Fund (CIEIF) Grant provides USD 75,000 to support proposed climate intervention field tests. The funding is specifically intended for Environmental Impact Assessment (EIA), predictive impact modelling, and/or engagement with potentially affected stakeholders, including local communities and government agencies.
+Applicants are expected to demonstrate the proposed field test’s technical readiness, environmental and social considerations, required government approvals, innovation and potential for globally relevant scalability. The application must include a proposed budget showing how the USD 75,000 will be used.
+ Grant Objective
+The grant is intended to support proposed climate intervention field tests, particularly activities related to:
+Environmental Impact Assessment (EIA)
+Predictive impact modeling
+Engagement with potentially impacted stakeholders
+Local community and government engagement
+Understanding technical, environmental, economic, social, public-health, and safety challenges
+The proposed application must focus on at least one of these three core areas: EIA, predictive impact modeling, or stakeholder engagement.
+ Eligible Project Focus
+The proposed field test should demonstrate:
+A clear climate-intervention concept
+Prior research indicating that the technology is ready for the proposed field test
+Potential for innovation and scalability
+A clear understanding of technical and environmental challenges
+Consideration of economic, social, public-health, and safety implications
+Relevant government permits and approvals
+Potential for scaling the innovation to a globally relevant level</t>
         </is>
       </c>
       <c r="D22" s="1" t="inlineStr">
         <is>
-          <t>Climate</t>
+          <t>Governance</t>
         </is>
       </c>
       <c r="E22" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Auto update Combined.xlsx [Sun Oct  4 07:42:30 UTC 2026]
</commit_message>
<xml_diff>
--- a/output/Combined.xlsx
+++ b/output/Combined.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -495,74 +495,10 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>ToR for Onboarding of consultant/agency for Innovating &amp; Scaling Reproductive Maternal Newborn and Child Health Solutions in the Last-Mile</t>
+          <t>Application Invited GFF x CIVIC VOICES Call for Proposals</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t>No description available</t>
-        </is>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>Safety</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>Oct 5, 2026</t>
-        </is>
-      </c>
-      <c r="F3" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/tor-for-onboarding-of-consultantagency-for-innovating-and-scaling-reproductive-maternal-newborn-and-child-health-solutions-in-the-last-mile-selco-foundation-rfp-26-00373</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="95" customHeight="1">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>RFP - Design and Delivery of an Electric Vehicle EV Skilling Programme in Karnataka</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>No description available</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>Learning</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="inlineStr">
-        <is>
-          <t>Oct 5, 2026</t>
-        </is>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/rfp-design-and-delivery-of-an-electric-vehicle-ev-skilling-programme-in-karnataka-wri-india-rfp-26-00361</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="95" customHeight="1">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>Application Invited GFF x CIVIC VOICES Call for Proposals</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>About us
 PATH is a global nonprofit that turns innovation into better health. For nearly 50 years, PATH has worked with countries, communities, health workers, researchers, governments, and partners to develop and deliver health innovations, from vaccines and diagnostics to strong health systems and more accessible care. By bringing together expertise in science, economics, technology, advocacy, and other fields, PATH develops and scales innovative solutions to the world’s most pressing health challenges. *PATH has become aware of scams involving false job offers.* Please advise: - PATH will never ask for a fee during any stage of the recruitment process. - All active jobs are advertised directly on our careers page: https://path.silkroad.com/epostings/. - Official PATH emails will always arrive from an @path.org address Please report any suspicious communications to careersitehelp@path.org.
@@ -579,66 +515,66 @@
 Call for proposals</t>
         </is>
       </c>
-      <c r="D5" s="1" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E5" s="1" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Oct 7, 2026</t>
         </is>
       </c>
-      <c r="F5" s="1" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/application-invited-gff-x-civic-voices-call-for-proposals-path-opg-26-00192</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="95" customHeight="1">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
+    <row r="4" ht="95" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>ToR - Catalyse Tech Reproductive Maternal Newborn &amp; Child Health</t>
         </is>
       </c>
-      <c r="C6" s="1" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>No description available</t>
         </is>
       </c>
-      <c r="D6" s="1" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E6" s="1" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>Oct 10, 2026</t>
         </is>
       </c>
-      <c r="F6" s="1" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/tor-catalyse-tech-reproductive-maternal-newborn-and-child-health-selco-foundation-rfp-26-00379</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="95" customHeight="1">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
+    <row r="5" ht="95" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>Applications Open Draper Richards Kaplan Foundation Funding for Social Enterprises</t>
         </is>
       </c>
-      <c r="C7" s="1" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>About us
 Started in 2002, Draper Richards Kaplan Foundation (DRK) is a global venture philanthropy firm supporting early stage, high impact social enterprises. Borrowed from our venture capital legacy, DRK finds, funds, and supports exceptional leaders building innovative solutions to some of the world’s most challenging social and environmental problems. Since beginning this work nearly 25 years ago, DRK has invested in more than 270 organizations that have collectively impacted over 610 million lives to date.
@@ -662,34 +598,34 @@
 Please attach a standard resume/CV for the entrepreneur(s) and/or key leadership team members (e.g., CEO, COO, ED, etc.). Applications with text bios for entrepreneurs or members of the leadership team will not be considered.</t>
         </is>
       </c>
-      <c r="D7" s="1" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>Climate</t>
         </is>
       </c>
-      <c r="E7" s="1" t="inlineStr">
+      <c r="E5" s="1" t="inlineStr">
         <is>
           <t>Oct 10, 2026</t>
         </is>
       </c>
-      <c r="F7" s="1" t="inlineStr">
+      <c r="F5" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-open-draper-richards-kaplan-foundation-funding-for-social-enterprises-draper-richards-kaplan-foundation-opg-26-00188</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="95" customHeight="1">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
+    <row r="6" ht="95" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund</t>
         </is>
       </c>
-      <c r="C8" s="1" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund
 Apply by: 13 October, 2026
@@ -714,66 +650,66 @@
  Projects should include opportunities for ServiceNow employees to volunteer in the project activation or implementation.</t>
         </is>
       </c>
-      <c r="D8" s="1" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E8" s="1" t="inlineStr">
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>Oct 13, 2026</t>
         </is>
       </c>
-      <c r="F8" s="1" t="inlineStr">
+      <c r="F6" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/apply-for-the-servicenow-community-solar-fund-changex-opg-26-00186</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="95" customHeight="1">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="inlineStr">
+    <row r="7" ht="95" customHeight="1">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>EOI invited for Consultant Road Safety Expert / Technical</t>
         </is>
       </c>
-      <c r="C9" s="1" t="inlineStr">
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>No description available</t>
         </is>
       </c>
-      <c r="D9" s="1" t="inlineStr">
+      <c r="D7" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E9" s="1" t="inlineStr">
+      <c r="E7" s="1" t="inlineStr">
         <is>
           <t>Oct 15, 2026</t>
         </is>
       </c>
-      <c r="F9" s="1" t="inlineStr">
+      <c r="F7" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/eoi-invited-for-consultant-road-safety-expert-technical-bharatcares-rfp-26-00381</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="95" customHeight="1">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
+    <row r="8" ht="95" customHeight="1">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Blue Action Fund Grant Call Mangroves Blue Carbon Markets and 30x30 in Asia</t>
         </is>
       </c>
-      <c r="C10" s="1" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Blue Action Fund is a nonprofit foundation dedicated to conserving the ocean for future generations and improving the lives of people today. To address the global financing gap in ocean conservation, Blue Action awards grants to NGOs to create, expand, or improve marine protected areas and other effective area-based conservation measures while enhancing livelihoods in coastal communities.
@@ -814,66 +750,66 @@
 Projects must receive endorsement from the relevant national authority.</t>
         </is>
       </c>
-      <c r="D10" s="1" t="inlineStr">
+      <c r="D8" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E10" s="1" t="inlineStr">
+      <c r="E8" s="1" t="inlineStr">
         <is>
           <t>Oct 16, 2026</t>
         </is>
       </c>
-      <c r="F10" s="1" t="inlineStr">
+      <c r="F8" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-blue-action-fund-grant-call-mangroves-blue-carbon-markets-and-30x30-in-asia-blue-action-fund-opg-26-00140</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="95" customHeight="1">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="inlineStr">
+    <row r="9" ht="95" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
         <is>
           <t>RFPs Invited for Consultant to Develop a Technical Assistance Package for National Application of the Digital Health and AI Investment Classification Framework</t>
         </is>
       </c>
-      <c r="C11" s="1" t="inlineStr">
+      <c r="C9" s="1" t="inlineStr">
         <is>
           <t>No description available</t>
         </is>
       </c>
-      <c r="D11" s="1" t="inlineStr">
+      <c r="D9" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E11" s="1" t="inlineStr">
+      <c r="E9" s="1" t="inlineStr">
         <is>
           <t>Oct 23, 2026</t>
         </is>
       </c>
-      <c r="F11" s="1" t="inlineStr">
+      <c r="F9" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/rfps/rfps-invited-for-consultant-to-develop-a-technical-assistance-package-for-national-application-of-the-digital-health-and-ai-investment-classification-framework-transform-health-rfp-26-00359</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="95" customHeight="1">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="inlineStr">
+    <row r="10" ht="95" customHeight="1">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for D-Prize Global Competition Seed Funding for New Poverty-Solution Distribution Organizations</t>
         </is>
       </c>
-      <c r="C12" s="1" t="inlineStr">
+      <c r="C10" s="1" t="inlineStr">
         <is>
           <t>About the Grant:
 D-Prize seeds new organizations that distribute proven poverty solutions at the "last mile," with the aim of scaling impact. Applicants select from a range of evidence-based interventions (health, agriculture, education, water, safety, transparency, and more) and propose how they would launch or grow an organization to distribute that intervention. Top entrepreneurs receive up to $20,000 in seed funding to run a pilot and build an organization capable of scaling to reach thousands, even millions of people.
@@ -896,6 +832,134 @@
 Extension Deadline: 6 December 2026, midnight PT (extension registration required)</t>
         </is>
       </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>Oct 25, 2026</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-d-prize-global-competition-seed-funding-for-new-poverty-solution-distribution-organizations-d-prize-opg-26-00191</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="95" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Crossing the Divide Best Practices for Addressing Local and Privately-Owned Lateral Sewer Issues RFP 5419</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>Project Objective:
+To provide water resource recovery facilities (WRRFs) and collection system operators with an interactive manual of practice for implementing inflow and infiltration (I&amp;I) and obstruction management programs, focused on municipal and privately owned lateral sewers in complex legal, regulatory, and multi-jurisdictional environments.
+ Background/Rationale:
+Wastewater utilities face continuing challenges providing cost-effective sewer services amid rising demand, urban redevelopment, and performance disruptors (root intrusion, pipe degradation, blockages). I&amp;I and obstruction management remain persistent, costly problems without a consolidated resource to guide program design. During wet weather, peak I&amp;I flows can increase influent flows 3–5x average. Studies suggest up to 80% of I&amp;I originates on private property, and root intrusions cause over 50% of sewer blockages globally. Program effectiveness varies widely depending on statutory authority, multi-jurisdictional overlap, enforcement mechanisms, and participant willingness.
+ Central Research Questions:
+What I&amp;I and obstruction management practices are utilities using today, and how do they vary by jurisdictional/regulatory/infrastructure/environmental conditions?
+Which factors most influence successful implementation, and what barriers commonly derail programs?
+What measurable benefits (cost avoidance, capacity recovery, reduced spill risk, improved regulatory standing) have utilities realized from successful programs?
+This project extends WRF's ongoing "State-of-Practice Manual for Inflow and Infiltration Detection and Mitigation at Street and Private Lateral Levels" (Project 5365) into I&amp;I source control and obstruction management specifically.
+ Research Approach (4 Tasks):
+Literature and Regulatory Review — Comprehensive review of legal authorities/regulations in the US and comparable international jurisdictions; catalog program elements, enforcement mechanisms, incentive structures, and legal/jurisdictional barriers
+Utility Survey and Case Study Development — Broad survey across utility size/geography/system type; select at least 5 diverse in-depth case studies with quantitative results (I&amp;I reduction %, reduced bypass pumping, reduced basement backups, cost savings, recovered capacity, reduced blockage-related spills/service calls)
+Utility Workshop — At least one invitation-only workshop with utility representatives to present survey findings and gather structured feedback on draft guidance content
+Interactive Manual of Practice — Development of a decision-support tool/web-based application/interactive PDF enabling utilities to select effective I&amp;I/obstruction program elements based on their statutory authority, jurisdictional complexity, and enforcement mechanisms
+ Expected Deliverables:
+Research report (using WRF's Research Report Template) including literature/regulatory review
+Interactive manual of practice (following Technology Deliverables Guidance)
+In-depth utility survey, state-of-the-practice report, and at least 5 standalone case studies with quantitative results
+Summary documentation of the utility workshop, including feedback and how it was incorporated
+ Project Duration: 24 months from contract start date (No-Cost Extension Policy caps extensions at 9 months beyond original schedule)
+ Eligibility to Submit:
+Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible as named participants. Not open to individuals (same institutional-applicant structure as RFP 5424).
+ Budget/Funding:
+Maximum WRF funding: $250,000
+Applicant must contribute at least 33% of the project award as additional resources (cost share, applicant in-kind, or third-party in-kind per 2 CFR Part 200.306)
+Proposals not meeting the 33% minimum match will not be accepted
+ Proposal Evaluation Criteria:
+Understanding the Problem and Responsiveness to RFP: 20 points
+Technical and Scientific Merit: 30 points
+Qualifications, Capabilities, and Management: 20 points
+Communication Plan, Deliverables, and Applicability: 15 points
+Budget and Schedule: 15 points
+ Compliance Standards: OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
+ Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
+        </is>
+      </c>
+      <c r="D11" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>Oct 26, 2026</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-crossing-the-divide-best-practices-for-addressing-local-and-privately-owned-lateral-sewer-issues-rfp-5419-the-water-research-foundation-wrf-opg-26-00189</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="95" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Comparison of PFAS Contributions to Agricultural Systems</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>Project Objectives:
+Report per- and polyfluoroalkyl substance (PFAS) concentrations from a variety of agricultural inputs — animal manures, fertilizers, pesticides, composts, soil amendments, seed coatings, and biosolids-based products
+Compare the impact of various agricultural inputs on PFAS concentration in the soil profile over varying timeframes
+Evaluate the fate and transport of different inputs to PFAS contributions in agricultural systems at field-scale
+Determine relative contributions from biosolids-based products vs. other inputs to help develop/prioritize risk management strategies
+ Background/Rationale:
+Growing concern exists over human exposure to PFAS through biosolids land application on agricultural systems, with regulatory bans on biosolids land application enacted or proposed in at least 12 U.S. states. Utilities relying on land application for biosolids management are scrambling for alternative disposal pathways. The U.S. EPA's 2026 draft guidance noted its earlier 2025 draft risk assessment of PFOA/PFOS-contaminated sewage sludge lacked important contextual information (e.g., a national survey of PFOA/PFOS concentrations). Risk assessments have focused primarily on biosolids, with less attention to PFAS contributions from other sources — manures, compost, fertilizers, pesticides, seed coatings, irrigation water, farming practices, and atmospheric deposition. A Minnesota Pollution Control Agency review found 12 inert pesticide ingredients classified as PFAS. This project aims to improve understanding of PFAS risks from the wider range of agricultural inputs to support strategic resource allocation and inform policy amid surging fertilizer prices and shifts toward local circular resources.
+ Research Approach:
+Develop a baseline of knowledge on PFAS in biosolids and non-biosolids agricultural inputs via literature review, analytical methods evaluation, and examination of manufacturing/processing pathways; identify data gaps and uncertainties
+Measure/report compound-specific PFAS concentrations and profiles in agricultural inputs using standardized methods, including precursor characteristics for source attribution where possible
+Characterize PFAS contributions via literature review, data analysis, and field sampling — comparing soil profile/plant tissue composition between fields with non-biosolids inputs vs. biosolids-applied systems; study should test hypotheses on PFAS sources, transformation, retention, and mobility
+Optional additional focus areas: influence of soil/hydrologic/hydrochemistry conditions on PFAS behavior; degradation/transformation pathways; relative PFAS contributions across product lifecycle stages (manufacturing, bagging, delivery, etc.)
+Research approach should be hypothesis-driven, detailing specific end-user needs, and proposers are encouraged to leverage existing projects on PFAS plant uptake/fate/transport.
+ Expected Deliverables:
+Research report (WRF's Research Report Template) including: literature review, PFAS analysis of select products, risk management implications/prioritization recommendations, agriculture end-use guidance
+A webcast or workshop to share findings
+Optional additional deliverables: relative risk framework (mass input/fate/exposure/risk), decision support guide for farmers/regulators/utilities, plain language fact sheet, comparative PFAS mass input tool (spreadsheet/calculator)
+ Project Duration: 36 months from contract start date (longer than the other two WRF grants above, which were 24 months)
+ Eligibility to Submit:
+Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible. Not open to individuals (same structure as the two prior WRF grants).
+ Budget/Funding:
+Maximum WRF funding: $400,000 (the largest of the three WRF grants shared so far)
+Applicant must contribute at least 33% of the project award as additional resources (cost share, applicant in-kind, or third-party in-kind per 2 CFR Part 200.306)
+Proposals not meeting the 33% minimum match will not be accepted
+ Proposal Evaluation Criteria:
+Understanding the Problem and Responsiveness to RFP: 20 points
+Technical and Scientific Merit: 30 points
+Qualifications, Capabilities, and Management: 20 points
+Communication Plan, Deliverables, and Applicability: 15 points
+Budget and Schedule: 15 points
+ Compliance Standards: OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
+ Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00) — same deadline as the other two WRF grants</t>
+        </is>
+      </c>
       <c r="D12" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
@@ -903,12 +967,12 @@
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>Oct 25, 2026</t>
+          <t>Oct 26, 2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-d-prize-global-competition-seed-funding-for-new-poverty-solution-distribution-organizations-d-prize-opg-26-00191</t>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-comparison-of-pfas-contributions-to-agricultural-systems-the-water-research-foundation-wrf-opg-26-00190</t>
         </is>
       </c>
     </row>
@@ -988,228 +1052,10 @@
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
-          <t>Applications Invited for Crossing the Divide Best Practices for Addressing Local and Privately-Owned Lateral Sewer Issues RFP 5419</t>
+          <t>Applications Invited for Whitley Award 2027</t>
         </is>
       </c>
       <c r="C14" s="1" t="inlineStr">
-        <is>
-          <t>Project Objective:
-To provide water resource recovery facilities (WRRFs) and collection system operators with an interactive manual of practice for implementing inflow and infiltration (I&amp;I) and obstruction management programs, focused on municipal and privately owned lateral sewers in complex legal, regulatory, and multi-jurisdictional environments.
- Background/Rationale:
-Wastewater utilities face continuing challenges providing cost-effective sewer services amid rising demand, urban redevelopment, and performance disruptors (root intrusion, pipe degradation, blockages). I&amp;I and obstruction management remain persistent, costly problems without a consolidated resource to guide program design. During wet weather, peak I&amp;I flows can increase influent flows 3–5x average. Studies suggest up to 80% of I&amp;I originates on private property, and root intrusions cause over 50% of sewer blockages globally. Program effectiveness varies widely depending on statutory authority, multi-jurisdictional overlap, enforcement mechanisms, and participant willingness.
- Central Research Questions:
-What I&amp;I and obstruction management practices are utilities using today, and how do they vary by jurisdictional/regulatory/infrastructure/environmental conditions?
-Which factors most influence successful implementation, and what barriers commonly derail programs?
-What measurable benefits (cost avoidance, capacity recovery, reduced spill risk, improved regulatory standing) have utilities realized from successful programs?
-This project extends WRF's ongoing "State-of-Practice Manual for Inflow and Infiltration Detection and Mitigation at Street and Private Lateral Levels" (Project 5365) into I&amp;I source control and obstruction management specifically.
- Research Approach (4 Tasks):
-Literature and Regulatory Review — Comprehensive review of legal authorities/regulations in the US and comparable international jurisdictions; catalog program elements, enforcement mechanisms, incentive structures, and legal/jurisdictional barriers
-Utility Survey and Case Study Development — Broad survey across utility size/geography/system type; select at least 5 diverse in-depth case studies with quantitative results (I&amp;I reduction %, reduced bypass pumping, reduced basement backups, cost savings, recovered capacity, reduced blockage-related spills/service calls)
-Utility Workshop — At least one invitation-only workshop with utility representatives to present survey findings and gather structured feedback on draft guidance content
-Interactive Manual of Practice — Development of a decision-support tool/web-based application/interactive PDF enabling utilities to select effective I&amp;I/obstruction program elements based on their statutory authority, jurisdictional complexity, and enforcement mechanisms
- Expected Deliverables:
-Research report (using WRF's Research Report Template) including literature/regulatory review
-Interactive manual of practice (following Technology Deliverables Guidance)
-In-depth utility survey, state-of-the-practice report, and at least 5 standalone case studies with quantitative results
-Summary documentation of the utility workshop, including feedback and how it was incorporated
- Project Duration: 24 months from contract start date (No-Cost Extension Policy caps extensions at 9 months beyond original schedule)
- Eligibility to Submit:
-Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible as named participants. Not open to individuals (same institutional-applicant structure as RFP 5424).
- Budget/Funding:
-Maximum WRF funding: $250,000
-Applicant must contribute at least 33% of the project award as additional resources (cost share, applicant in-kind, or third-party in-kind per 2 CFR Part 200.306)
-Proposals not meeting the 33% minimum match will not be accepted
- Proposal Evaluation Criteria:
-Understanding the Problem and Responsiveness to RFP: 20 points
-Technical and Scientific Merit: 30 points
-Qualifications, Capabilities, and Management: 20 points
-Communication Plan, Deliverables, and Applicability: 15 points
-Budget and Schedule: 15 points
- Compliance Standards: OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
- Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
-        </is>
-      </c>
-      <c r="D14" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E14" s="1" t="inlineStr">
-        <is>
-          <t>Oct 26, 2026</t>
-        </is>
-      </c>
-      <c r="F14" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-crossing-the-divide-best-practices-for-addressing-local-and-privately-owned-lateral-sewer-issues-rfp-5419-the-water-research-foundation-wrf-opg-26-00189</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="95" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Comparison of PFAS Contributions to Agricultural Systems</t>
-        </is>
-      </c>
-      <c r="C15" s="1" t="inlineStr">
-        <is>
-          <t>Project Objectives:
-Report per- and polyfluoroalkyl substance (PFAS) concentrations from a variety of agricultural inputs — animal manures, fertilizers, pesticides, composts, soil amendments, seed coatings, and biosolids-based products
-Compare the impact of various agricultural inputs on PFAS concentration in the soil profile over varying timeframes
-Evaluate the fate and transport of different inputs to PFAS contributions in agricultural systems at field-scale
-Determine relative contributions from biosolids-based products vs. other inputs to help develop/prioritize risk management strategies
- Background/Rationale:
-Growing concern exists over human exposure to PFAS through biosolids land application on agricultural systems, with regulatory bans on biosolids land application enacted or proposed in at least 12 U.S. states. Utilities relying on land application for biosolids management are scrambling for alternative disposal pathways. The U.S. EPA's 2026 draft guidance noted its earlier 2025 draft risk assessment of PFOA/PFOS-contaminated sewage sludge lacked important contextual information (e.g., a national survey of PFOA/PFOS concentrations). Risk assessments have focused primarily on biosolids, with less attention to PFAS contributions from other sources — manures, compost, fertilizers, pesticides, seed coatings, irrigation water, farming practices, and atmospheric deposition. A Minnesota Pollution Control Agency review found 12 inert pesticide ingredients classified as PFAS. This project aims to improve understanding of PFAS risks from the wider range of agricultural inputs to support strategic resource allocation and inform policy amid surging fertilizer prices and shifts toward local circular resources.
- Research Approach:
-Develop a baseline of knowledge on PFAS in biosolids and non-biosolids agricultural inputs via literature review, analytical methods evaluation, and examination of manufacturing/processing pathways; identify data gaps and uncertainties
-Measure/report compound-specific PFAS concentrations and profiles in agricultural inputs using standardized methods, including precursor characteristics for source attribution where possible
-Characterize PFAS contributions via literature review, data analysis, and field sampling — comparing soil profile/plant tissue composition between fields with non-biosolids inputs vs. biosolids-applied systems; study should test hypotheses on PFAS sources, transformation, retention, and mobility
-Optional additional focus areas: influence of soil/hydrologic/hydrochemistry conditions on PFAS behavior; degradation/transformation pathways; relative PFAS contributions across product lifecycle stages (manufacturing, bagging, delivery, etc.)
-Research approach should be hypothesis-driven, detailing specific end-user needs, and proposers are encouraged to leverage existing projects on PFAS plant uptake/fate/transport.
- Expected Deliverables:
-Research report (WRF's Research Report Template) including: literature review, PFAS analysis of select products, risk management implications/prioritization recommendations, agriculture end-use guidance
-A webcast or workshop to share findings
-Optional additional deliverables: relative risk framework (mass input/fate/exposure/risk), decision support guide for farmers/regulators/utilities, plain language fact sheet, comparative PFAS mass input tool (spreadsheet/calculator)
- Project Duration: 36 months from contract start date (longer than the other two WRF grants above, which were 24 months)
- Eligibility to Submit:
-Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible. Not open to individuals (same structure as the two prior WRF grants).
- Budget/Funding:
-Maximum WRF funding: $400,000 (the largest of the three WRF grants shared so far)
-Applicant must contribute at least 33% of the project award as additional resources (cost share, applicant in-kind, or third-party in-kind per 2 CFR Part 200.306)
-Proposals not meeting the 33% minimum match will not be accepted
- Proposal Evaluation Criteria:
-Understanding the Problem and Responsiveness to RFP: 20 points
-Technical and Scientific Merit: 30 points
-Qualifications, Capabilities, and Management: 20 points
-Communication Plan, Deliverables, and Applicability: 15 points
-Budget and Schedule: 15 points
- Compliance Standards: OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
- Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00) — same deadline as the other two WRF grants</t>
-        </is>
-      </c>
-      <c r="D15" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E15" s="1" t="inlineStr">
-        <is>
-          <t>Oct 26, 2026</t>
-        </is>
-      </c>
-      <c r="F15" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-comparison-of-pfas-contributions-to-agricultural-systems-the-water-research-foundation-wrf-opg-26-00190</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="95" customHeight="1">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B16" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for 8th Call for Proposals Small-Size Grants Global EbA Fund</t>
-        </is>
-      </c>
-      <c r="C16" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
- About the Opportunity:
-The Global EbA Fund invites innovative and catalytic proposals that address systemic barriers to Ecosystem-based Adaptation (EbA) scaling — by enhancing institutional and technical capacities, quality data/evidence generation, learning networks, and investment readiness. Aligned with the IKI Strategy up to 2030 (focus on socio-ecological transformation), the Fund's primary geographic focus is ODA-eligible SIDS (Small Island Developing States) and LDCs (Least Developed Countries), though other ODA-eligible countries may be considered where proposals show exceptional ambition.
- Focus Areas:
-Overcoming upstream barriers to EbA uptake/scaling (institutional &amp; technical capacity constraints, evidence generation, knowledge exchange)
-Clear adaptation chain grounded in detailed impact chain analysis (climate hazards/risks, socioeconomic/ecological sensitivity, adaptive capacity)
-Social and environmental considerations (gender responsiveness, Indigenous Peoples' rights, local participation, environmental/social safeguards, prevention of maladaptation)
-Robust sustainability and exit strategies (long-term viability, local ownership, institutional continuity)
- Encouraged Topics:
-Investment readiness and project pipeline preparation
-Innovative technologies for EbA
-Applied and functional research
-Synergies with other EbA/Nature-based Solution (NbS) initiatives
- Grant Size: Up to USD 250,000 per grant
- Project Duration: Up to 24 months
- Eligible Applicant Types:
-Non-governmental organisations (NGOs)
-International NGOs (INGOs)
-Intergovernmental organisations (IGOs)
-Community-based organisations (CBOs)
-Indigenous People's Organisations
-Universities and academic institutions
-Research institutes and think tanks
-Private sector companies (under certain conditions; no funding for sector-specific obligations, compensatory measures, or for-profit activities)
-Consortia (must designate a clear lead "Applicant Organisation"; government entities can join a consortium but cannot receive Fund money directly)
-Note: Individuals are not eligible (e.g., no PhD study funding); UNEP and IUCN offices are also not eligible to apply.
- Key Eligibility Criteria:
-Must qualify as Ecosystem-based Adaptation (EbA) per the Fund's Qualification Criteria &amp; Quality Standards
-Must have catalytic/innovative potential
-Must clearly identify climate impacts addressed
-Falls under max 1 Strategic Objective and max 2 Action Pillars of the Fund
-Global, thematic, or targets only ODA-eligible countries
-Budget up to USD 250,000; duration up to 24 months
-Must build on existing work (not standalone/field-implementation-only projects)
-Must show sustainability post-funding
-Must partner with local institutions
-Applicant &amp; partners must be legally recognized entities with relevant experience
-Must complete Due Diligence requirements
- Evaluation Criteria (weighted):
-Ecosystem-based Adaptation (EbA) approach — 30%
-Design &amp; Methodology (Theory of Change, logframe, SMART indicators, budget coherence)
-Gender &amp; Social Inclusion (participatory approach, FPIC for Indigenous Peoples' impact)
-Innovative &amp; Catalytic Contribution — 30%
-Sustainability — 20%
-Institutional Arrangements — 20%
- Reporting Requirement: Applicants must identify at least 3 indicators from the Fund's Core Indicator Framework for their project's logframe.
- Application Package Required:
-Applicant Declaration
-Co-applicant Mandate (if applicable)
-Small-Size Grants Application Form
-Project Proposal Budget Template
-Due Diligence and Financial Capacity Questionnaire (with Annexes 1(c)(i) and 1(c)(ii) at submission stage)
- Application Language: English only (organizational documents must be translated to English
- Timeline:
-Call officially launched: August 24, 2026
-Submission window: September 28 – October 26, 2026
-Applications submitted via online portal (link shared on the Small-Size Grants webpage from Sept 28)
-Only successful applicants will be contacted; no individual feedback provided to unsuccessful applicants</t>
-        </is>
-      </c>
-      <c r="D16" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E16" s="1" t="inlineStr">
-        <is>
-          <t>Oct 26, 2026</t>
-        </is>
-      </c>
-      <c r="F16" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-8th-call-for-proposals-small-size-grants-global-eba-fund-global-eba-fund-opg-26-00177</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="95" customHeight="1">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B17" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Whitley Award 2027</t>
-        </is>
-      </c>
-      <c r="C17" s="1" t="inlineStr">
         <is>
           <t>About the Grant: 
 An annual grant by the Whitley Fund for Nature (WFN) recognising grassroots conservation leaders in the Global South, providing funding to support and scale up proven, science-based solutions that deliver lasting impact for both people and nature.
@@ -1222,34 +1068,34 @@
 You do not need to be invited or nominated to apply.</t>
         </is>
       </c>
-      <c r="D17" s="1" t="inlineStr">
+      <c r="D14" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E17" s="1" t="inlineStr">
+      <c r="E14" s="1" t="inlineStr">
         <is>
           <t>Oct 30, 2026</t>
         </is>
       </c>
-      <c r="F17" s="1" t="inlineStr">
+      <c r="F14" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-whitley-award-2027-whitley-fund-for-nature-wfn-opg-26-00153</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="95" customHeight="1">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="inlineStr">
+    <row r="15" ht="95" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIFAR Global Scholars Program 20272029 Cohort</t>
         </is>
       </c>
-      <c r="C18" s="1" t="inlineStr">
+      <c r="C15" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 CIFAR is a Canadian-based globally influential research organization that convenes the world’s most brilliant people across disciplines to advance transformative knowledge and solve humanity’s biggest problems, together. By supporting long-term interdisciplinary collaboration, CIFAR provides researchers with an unparalleled environment of trust, transparency and knowledge sharing. Our time-tested model inspires new directions of inquiry, accelerates discovery and yields breakthroughs across borders and academic disciplines. Through knowledge mobilization, we are catalysts for change in industry, government and society. Through our 15 research programs and the Pan-Canadian AI Strategy, CIFAR convenes close to 400 of the world’s top researchers from 141 institutions in 20 countries. CIFAR is generously supported by the governments of Canada, Alberta and Québec, as well as foundations, individuals, corporations and Canadian and international partner organizations.
@@ -1293,34 +1139,34 @@
  Application Deadline: November 4, 2026, 12:00 PM EST</t>
         </is>
       </c>
-      <c r="D18" s="1" t="inlineStr">
+      <c r="D15" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E18" s="1" t="inlineStr">
+      <c r="E15" s="1" t="inlineStr">
         <is>
           <t>Nov 4, 2026</t>
         </is>
       </c>
-      <c r="F18" s="1" t="inlineStr">
+      <c r="F15" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cifar-global-scholars-program-20272029-cohort-cifar-canadian-institute-for-advanced-research-opg-26-00183</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="95" customHeight="1">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="inlineStr">
+    <row r="16" ht="95" customHeight="1">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for IWRS Teaching Innovation Award</t>
         </is>
       </c>
-      <c r="C19" s="1" t="inlineStr">
+      <c r="C16" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
@@ -1332,160 +1178,34 @@
 Two awards of $2,000 USD are available annually.</t>
         </is>
       </c>
-      <c r="D19" s="1" t="inlineStr">
+      <c r="D16" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E19" s="1" t="inlineStr">
+      <c r="E16" s="1" t="inlineStr">
         <is>
           <t>Nov 15, 2026</t>
         </is>
       </c>
-      <c r="F19" s="1" t="inlineStr">
+      <c r="F16" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="95" customHeight="1">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for IWRS Teaching Innovation Award</t>
-        </is>
-      </c>
-      <c r="C20" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-Insects are one of the most numerous and diverse animal groups on Earth.
-Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice.
-About the Award
-The IWRS Teaching Innovation Award supports instructors developing new approaches to teaching invertebrate biology that incorporate the 3Rs (replacement, reduction, and refinement). It also supports the development and implementation of any novel curricula addressing invertebrate welfare and sentience across invertebrate biology, animal welfare science, and/or veterinary medicine fields.
-Grant size
-Awards up to $2,000 USD are available for approaches requiring equipment or other materials; awards up to $1,000 USD are available otherwise. Funds may be used to support any costs associated with curriculum development and implementation, including stipends, teaching tools, and related expenses. Priority is given to proposals addressing common teaching practices with substantial welfare implications.
-Who can apply for funding?
-The applicant must be an instructor teaching content related to insect or invertebrate biology at an educational institution, scientific society or museum, field-training course, or similar educational context. If you are unsure about your eligibility, contact grants@insectwelfare.com.
-The applicant can be from any discipline, country, or institution. However, we will not pay awards to recipients located in jurisdictions, countries, or regions subject to trade restrictions, embargoes, or sanctions put in place by the United Nations or the United States of America.
-IWRS staff and Advisory Group members are not eligible to apply.</t>
-        </is>
-      </c>
-      <c r="D20" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E20" s="1" t="inlineStr">
-        <is>
-          <t>Nov 15, 2026</t>
-        </is>
-      </c>
-      <c r="F20" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00166</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="95" customHeight="1">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Medium-Size Grants Call for Proposals Global EbA Fund</t>
-        </is>
-      </c>
-      <c r="C21" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
- About the Opportunity:
-The Global EbA Fund invites proposals under its General Track: Strategic Scaling and Global Influence, seeking collaborative and innovative approaches to advancing Ecosystem-based Adaptation (EbA) by addressing systemic barriers to scalability and contributing to global learning and policy dialogue. Initiatives should strengthen enabling environments and embed EbA into national frameworks that unify climate, biodiversity, land, and development priorities. Alignment with one of three priority topics is welcomed but not mandatory:
- Priority Topics:
-I. Innovative Finance Solutions for EbA — partnerships with private sector actors (financiers, innovators, local champions) to unlock private capital/blended finance for EbA, evolving EbA into profitable, scalable business models
-II. EbA for Human Development and Security — integrating EbA into national/international security frameworks for fragile and conflict-affected contexts; community co-designed interventions that reduce natural resource-related tensions and climate-induced fragility, bridging adaptation, humanitarian, development, and peacebuilding agendas
-III. Interlinkages for People-Nature-Climate-Land Synergies — strengthening operational links across the Rio Conventions (UNFCCC, CBD, UNCCD) and frameworks like the Sendai Framework on DRR, using EbA as the anchor connecting biodiversity, sustainable land management, climate adaptation, and disaster risk reduction
- Grant Size: Up to USD 500,000 per grant
- Project Duration: Up to 24 months
- Eligible Applicant Types:
-Non-governmental organisations (NGOs)
-International NGOs (INGOs)
-Intergovernmental organisations (IGOs)
-Community-based organisations (CBOs)
-Indigenous People's Organisations
-Universities and academic institutions
-Research institutes and think tanks
-Private sector companies (under certain conditions)
-Consortia (must designate a clear lead "Applicant Organisation"; government entities may join but cannot receive Fund money directly)
-Note: Individuals are not eligible; UNEP and IUCN offices are also not eligible.
- Key Eligibility Criteria:
-Must qualify as Ecosystem-based Adaptation (EbA) per the Fund's Qualification Criteria &amp; Quality Standards
-Must show catalytic/innovative potential
-Must clearly identify climate impacts addressed
-Falls under max 1 Strategic Objective and max 2 Action Pillars of the Fund
-Global, thematic, or targets only ODA-eligible countries
-Budget up to USD 500,000; duration ≤24 months
-Must build on existing work (not standalone/field-implementation-only)
-Must show sustainability post-funding
-Must partner with local institutions
-Applicant &amp; partners must be legally recognized entities with relevant experience
-Must comply with Due Diligence requirements
- Evaluation Criteria (weighted):
-Ecosystem-based Adaptation (EbA) approach — 30%
-Design &amp; Methodology (Theory of Change, logframe, SMART indicators, budget coherence)
-Gender &amp; Social Inclusion (participatory approach, FPIC for Indigenous Peoples' impact)
-Innovative &amp; Catalytic Contribution — 30%
-Sustainability — 20%
-Institutional Arrangements — 20%
- Reporting Requirement: 
-Applicants must identify at least 3 indicators from the Fund's Core Indicator Framework for their project's logframe.
- Application Package Required:
-Applicant Declaration
-Co-applicant Mandate (if applicable)
-Medium-Size Grants Application Form
-Project Proposal Budget Template
-Due Diligence and Financial Capacity Questionnaire (with Annexes 1(c)(i) and 1(c)(ii) at submission stage)
- Application Language: English only (organizational documents must be translated to English)
- Timeline:
-Call officially launched: August 24, 2026
-Submission window: October 12 – November 16, 2026
-Applications submitted via online portal (link shared on the Medium-Size Grants webpage from Oct 12)</t>
-        </is>
-      </c>
-      <c r="D21" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E21" s="1" t="inlineStr">
-        <is>
-          <t>Nov 16, 2026</t>
-        </is>
-      </c>
-      <c r="F21" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-medium-size-grants-call-for-proposals-global-eba-fund-global-eba-fund-opg-26-00178</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="95" customHeight="1">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="inlineStr">
+    <row r="17" ht="95" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIEIF Grant 2026 Climate Intervention Environmental Impact Fund</t>
         </is>
       </c>
-      <c r="C22" s="1" t="inlineStr">
+      <c r="C17" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Climate Intervention Environmental Impact Fund (CIEIF) is a philanthropic fund focused on supporting responsible climate intervention field tests. It provides grants for activities such as environmental impact assessment (EIA), predictive impact modelling, and engagement with potentially affected stakeholders, including local communities and government agencies.
@@ -1512,34 +1232,34 @@
 Potential for scaling the innovation to a globally relevant level</t>
         </is>
       </c>
-      <c r="D22" s="1" t="inlineStr">
+      <c r="D17" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E22" s="1" t="inlineStr">
+      <c r="E17" s="1" t="inlineStr">
         <is>
           <t>Dec 1, 2026</t>
         </is>
       </c>
-      <c r="F22" s="1" t="inlineStr">
+      <c r="F17" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cieif-grant-2026-climate-intervention-environmental-impact-fund-climate-intervention-environmental-impact-fund-opg-26-00155</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="95" customHeight="1">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B23" s="1" t="inlineStr">
+    <row r="18" ht="95" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Oneness Revival Team ORT NGO Grant Programme 2026</t>
         </is>
       </c>
-      <c r="C23" s="1" t="inlineStr">
+      <c r="C18" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Oneness Revival Team (ORT) is a dedicated non-governmental organization (NGO) committed to supporting, funding, and empowering other NGOs that are striving to create meaningful change in communities worldwide. We believe that grassroots organizations and charitable initiatives are at the heart of sustainable development, yet many of them face challenges in accessing essential resources, funding, and strategic partnerships to scale their impact. ORT was founded with the vision of bridging this gap, ensuring that non-profits and humanitarian projects have the necessary tools to succeed.
@@ -1583,34 +1303,34 @@
 Submit a detailed project proposal, budget, and expected outcomes.</t>
         </is>
       </c>
-      <c r="D23" s="1" t="inlineStr">
+      <c r="D18" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E23" s="1" t="inlineStr">
+      <c r="E18" s="1" t="inlineStr">
         <is>
           <t>Dec 20, 2026</t>
         </is>
       </c>
-      <c r="F23" s="1" t="inlineStr">
+      <c r="F18" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-oneness-revival-team-ort-ngo-grant-programme-2026-oneness-revival-team-ort-opg-26-00143</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="95" customHeight="1">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B24" s="1" t="inlineStr">
+    <row r="19" ht="95" customHeight="1">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 6th Annual Seeding The Future Global Food System Challenge</t>
         </is>
       </c>
-      <c r="C24" s="1" t="inlineStr">
+      <c r="C19" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are one of the largest and most respected private organisations for development cooperation and humanitarian aid in Germany. As a politically and confessionally independent organisation, our value-oriented actions are always based on ethical principles. Our vision is clear: "Zero Hunger by 2030"
@@ -1642,34 +1362,34 @@
 Individuals with no organizational entity</t>
         </is>
       </c>
-      <c r="D24" s="1" t="inlineStr">
+      <c r="D19" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E24" s="1" t="inlineStr">
+      <c r="E19" s="1" t="inlineStr">
         <is>
           <t>Jan 1, 2027</t>
         </is>
       </c>
-      <c r="F24" s="1" t="inlineStr">
+      <c r="F19" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-6th-annual-seeding-the-future-global-food-system-challenge-welthungerhilfe-opg-26-00180</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="95" customHeight="1">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B25" s="1" t="inlineStr">
+    <row r="20" ht="95" customHeight="1">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Microbiota &amp; Women's Health International Call for Projects</t>
         </is>
       </c>
-      <c r="C25" s="1" t="inlineStr">
+      <c r="C20" s="1" t="inlineStr">
         <is>
           <t>About the Grant
 An annual international research grant by the Biocodex Microbiota Foundation (BMF), rewarding research proposals on the microbiota and its implications in Women's Health and Disease. This year's theme: "Unraveling male-female genital microbiome interactions: mechanisms, transmission, and impact on vaginal dysbiosis."
@@ -1686,34 +1406,34 @@
 €200,000 annually — awarded to researchers within universities, hospitals, or other research settings to finance equipment, operations, or staffing costs. Grants are NOT awarded to individuals directly (must be institutionally affiliated). Institution's overhead costs capped at 10%.</t>
         </is>
       </c>
-      <c r="D25" s="1" t="inlineStr">
+      <c r="D20" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E25" s="1" t="inlineStr">
+      <c r="E20" s="1" t="inlineStr">
         <is>
           <t>Jan 15, 2027</t>
         </is>
       </c>
-      <c r="F25" s="1" t="inlineStr">
+      <c r="F20" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-microbiota-and-womens-health-international-call-for-projects-biocodex-microbiota-foundation-bmf-opg-26-00152</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="95" customHeight="1">
-      <c r="A26" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B26" s="1" t="inlineStr">
+    <row r="21" ht="95" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for BES Training and Travel Grants</t>
         </is>
       </c>
-      <c r="C26" s="1" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are a global community of scientists shining a spotlight on the intricacy and value of our natural world, providing the evidence for better decisions. Our vision is for people and nature to thrive in a world that values ecology.
@@ -1752,17 +1472,17 @@
  Application Deadline (Round 2): Opens 30 April 2026, closes 17 May 2026</t>
         </is>
       </c>
-      <c r="D26" s="1" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E26" s="1" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>May 17, 2027</t>
         </is>
       </c>
-      <c r="F26" s="1" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-bes-training-and-travel-grants-british-ecological-society-opg-26-00181</t>
         </is>

</xml_diff>

<commit_message>
Auto update Combined.xlsx [Mon Oct  5 08:07:56 UTC 2026]
</commit_message>
<xml_diff>
--- a/output/Combined.xlsx
+++ b/output/Combined.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -539,42 +539,10 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>ToR - Catalyse Tech Reproductive Maternal Newborn &amp; Child Health</t>
+          <t>Applications Open Draper Richards Kaplan Foundation Funding for Social Enterprises</t>
         </is>
       </c>
       <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>No description available</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>Safety</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="inlineStr">
-        <is>
-          <t>Oct 10, 2026</t>
-        </is>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/tor-catalyse-tech-reproductive-maternal-newborn-and-child-health-selco-foundation-rfp-26-00379</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="95" customHeight="1">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>Applications Open Draper Richards Kaplan Foundation Funding for Social Enterprises</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>About us
 Started in 2002, Draper Richards Kaplan Foundation (DRK) is a global venture philanthropy firm supporting early stage, high impact social enterprises. Borrowed from our venture capital legacy, DRK finds, funds, and supports exceptional leaders building innovative solutions to some of the world’s most challenging social and environmental problems. Since beginning this work nearly 25 years ago, DRK has invested in more than 270 organizations that have collectively impacted over 610 million lives to date.
@@ -598,9 +566,41 @@
 Please attach a standard resume/CV for the entrepreneur(s) and/or key leadership team members (e.g., CEO, COO, ED, etc.). Applications with text bios for entrepreneurs or members of the leadership team will not be considered.</t>
         </is>
       </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Climate</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Oct 10, 2026</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-open-draper-richards-kaplan-foundation-funding-for-social-enterprises-draper-richards-kaplan-foundation-opg-26-00188</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="95" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>ToR - Catalyse Tech Reproductive Maternal Newborn &amp; Child Health</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>No description available</t>
+        </is>
+      </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>Climate</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr">
@@ -610,7 +610,7 @@
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/grants/applications-open-draper-richards-kaplan-foundation-funding-for-social-enterprises-draper-richards-kaplan-foundation-opg-26-00188</t>
+          <t>https://onepurpos.in/openings/rfps/tor-catalyse-tech-reproductive-maternal-newborn-and-child-health-selco-foundation-rfp-26-00379</t>
         </is>
       </c>
     </row>
@@ -706,63 +706,27 @@
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>Applications Invited for Blue Action Fund Grant Call Mangroves Blue Carbon Markets and 30x30 in Asia</t>
+          <t>RFPs Invited for Consultant to Develop a Technical Assistance Package for National Application of the Digital Health and AI Investment Classification Framework</t>
         </is>
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>About the Organization
-Blue Action Fund is a nonprofit foundation dedicated to conserving the ocean for future generations and improving the lives of people today. To address the global financing gap in ocean conservation, Blue Action awards grants to NGOs to create, expand, or improve marine protected areas and other effective area-based conservation measures while enhancing livelihoods in coastal communities.
- About the Grant
-The Blue Action Fund’s Mangroves, Blue Carbon Markets, and 30x30 in Asia Grant Call is a funding initiative that supports projects focused on the protection, restoration, and sustainable management of mangrove ecosystems in Asia.
-The grant aims to support high-impact conservation projects that combine area-based conservation approaches, blue carbon development, climate action, biodiversity protection, and sustainable livelihoods for coastal communities.
-The funding window supports projects that contribute to the Kunming-Montreal Global Biodiversity Framework’s 30x30 target and advance climate change mitigation through high-integrity blue carbon initiatives.
-Eligible projects should focus on:
-Establishing or improving management of protected areas (PAs) and Other Effective Area-Based Conservation Measures (OECMs).
-Restoring and conserving mangrove ecosystems.
-Developing credible blue carbon projects toward carbon crediting.
-Strengthening coastal community livelihoods, participation, and equitable benefit-sharing.
-Building long-term financial sustainability for conservation efforts.
-The grant is open to eligible NGOs and NGO consortia implementing projects in India, Indonesia, the Philippines, or Vietnam. Selected projects can receive funding support of EUR 2 million to EUR 4 million and must be completed within 5 years or less.
- Grant Objectives
-The key objectives of the grant are:
-To protect and restore mangrove ecosystems.
-To support biodiversity conservation and climate change mitigation.
-To develop high-integrity blue carbon projects.
-To strengthen protected areas (PAs) and Other Effective Area-Based Conservation Measures (OECMs).
-To improve livelihoods and participation of coastal communities.
-To promote sustainable financing mechanisms for long-term conservation.
-To support the development of credible carbon credit pathways.
- Eligibility Criteria
-Eligible applicants must:
-Be charitable non-government organisations (NGOs) or consortia of NGOs.
-Applicants should have:
-Proven experience in mangrove conservation/restoration.
-Experience in environmental protection and sustainable livelihoods.
-Experience with community engagement and stakeholder processes.
-Capacity to manage environmental and social safeguards.
- Additional requirements:
-Projects must be located in India, Indonesia, Philippines, or Vietnam.
-Projects should cover mangrove ecosystems of at least 1,000 hectares.
-Projects must demonstrate technical readiness for blue carbon development.
-NGOs must provide minimum 25% match funding of total project costs.
-Projects must have prior feasibility or preparatory assessments.
-Projects must receive endorsement from the relevant national authority.</t>
+          <t>No description available</t>
         </is>
       </c>
       <c r="D8" s="1" t="inlineStr">
         <is>
-          <t>Governance</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>Oct 16, 2026</t>
+          <t>Oct 23, 2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-blue-action-fund-grant-call-mangroves-blue-carbon-markets-and-30x30-in-asia-blue-action-fund-opg-26-00140</t>
+          <t>https://onepurpos.in/openings/rfps/rfps-invited-for-consultant-to-develop-a-technical-assistance-package-for-national-application-of-the-digital-health-and-ai-investment-classification-framework-transform-health-rfp-26-00359</t>
         </is>
       </c>
     </row>
@@ -774,42 +738,10 @@
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
-          <t>RFPs Invited for Consultant to Develop a Technical Assistance Package for National Application of the Digital Health and AI Investment Classification Framework</t>
+          <t>Applications Invited for D-Prize Global Competition Seed Funding for New Poverty-Solution Distribution Organizations</t>
         </is>
       </c>
       <c r="C9" s="1" t="inlineStr">
-        <is>
-          <t>No description available</t>
-        </is>
-      </c>
-      <c r="D9" s="1" t="inlineStr">
-        <is>
-          <t>Safety</t>
-        </is>
-      </c>
-      <c r="E9" s="1" t="inlineStr">
-        <is>
-          <t>Oct 23, 2026</t>
-        </is>
-      </c>
-      <c r="F9" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/rfps-invited-for-consultant-to-develop-a-technical-assistance-package-for-national-application-of-the-digital-health-and-ai-investment-classification-framework-transform-health-rfp-26-00359</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="95" customHeight="1">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for D-Prize Global Competition Seed Funding for New Poverty-Solution Distribution Organizations</t>
-        </is>
-      </c>
-      <c r="C10" s="1" t="inlineStr">
         <is>
           <t>About the Grant:
 D-Prize seeds new organizations that distribute proven poverty solutions at the "last mile," with the aim of scaling impact. Applicants select from a range of evidence-based interventions (health, agriculture, education, water, safety, transparency, and more) and propose how they would launch or grow an organization to distribute that intervention. Top entrepreneurs receive up to $20,000 in seed funding to run a pilot and build an organization capable of scaling to reach thousands, even millions of people.
@@ -832,6 +764,69 @@
 Extension Deadline: 6 December 2026, midnight PT (extension registration required)</t>
         </is>
       </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>Oct 25, 2026</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-d-prize-global-competition-seed-funding-for-new-poverty-solution-distribution-organizations-d-prize-opg-26-00191</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="95" customHeight="1">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Comparison of PFAS Contributions to Agricultural Systems</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>Project Objectives:
+Report per- and polyfluoroalkyl substance (PFAS) concentrations from a variety of agricultural inputs — animal manures, fertilizers, pesticides, composts, soil amendments, seed coatings, and biosolids-based products
+Compare the impact of various agricultural inputs on PFAS concentration in the soil profile over varying timeframes
+Evaluate the fate and transport of different inputs to PFAS contributions in agricultural systems at field-scale
+Determine relative contributions from biosolids-based products vs. other inputs to help develop/prioritize risk management strategies
+ Background/Rationale:
+Growing concern exists over human exposure to PFAS through biosolids land application on agricultural systems, with regulatory bans on biosolids land application enacted or proposed in at least 12 U.S. states. Utilities relying on land application for biosolids management are scrambling for alternative disposal pathways. The U.S. EPA's 2026 draft guidance noted its earlier 2025 draft risk assessment of PFOA/PFOS-contaminated sewage sludge lacked important contextual information (e.g., a national survey of PFOA/PFOS concentrations). Risk assessments have focused primarily on biosolids, with less attention to PFAS contributions from other sources — manures, compost, fertilizers, pesticides, seed coatings, irrigation water, farming practices, and atmospheric deposition. A Minnesota Pollution Control Agency review found 12 inert pesticide ingredients classified as PFAS. This project aims to improve understanding of PFAS risks from the wider range of agricultural inputs to support strategic resource allocation and inform policy amid surging fertilizer prices and shifts toward local circular resources.
+ Research Approach:
+Develop a baseline of knowledge on PFAS in biosolids and non-biosolids agricultural inputs via literature review, analytical methods evaluation, and examination of manufacturing/processing pathways; identify data gaps and uncertainties
+Measure/report compound-specific PFAS concentrations and profiles in agricultural inputs using standardized methods, including precursor characteristics for source attribution where possible
+Characterize PFAS contributions via literature review, data analysis, and field sampling — comparing soil profile/plant tissue composition between fields with non-biosolids inputs vs. biosolids-applied systems; study should test hypotheses on PFAS sources, transformation, retention, and mobility
+Optional additional focus areas: influence of soil/hydrologic/hydrochemistry conditions on PFAS behavior; degradation/transformation pathways; relative PFAS contributions across product lifecycle stages (manufacturing, bagging, delivery, etc.)
+Research approach should be hypothesis-driven, detailing specific end-user needs, and proposers are encouraged to leverage existing projects on PFAS plant uptake/fate/transport.
+ Expected Deliverables:
+Research report (WRF's Research Report Template) including: literature review, PFAS analysis of select products, risk management implications/prioritization recommendations, agriculture end-use guidance
+A webcast or workshop to share findings
+Optional additional deliverables: relative risk framework (mass input/fate/exposure/risk), decision support guide for farmers/regulators/utilities, plain language fact sheet, comparative PFAS mass input tool (spreadsheet/calculator)
+ Project Duration: 36 months from contract start date (longer than the other two WRF grants above, which were 24 months)
+ Eligibility to Submit:
+Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible. Not open to individuals (same structure as the two prior WRF grants).
+ Budget/Funding:
+Maximum WRF funding: $400,000 (the largest of the three WRF grants shared so far)
+Applicant must contribute at least 33% of the project award as additional resources (cost share, applicant in-kind, or third-party in-kind per 2 CFR Part 200.306)
+Proposals not meeting the 33% minimum match will not be accepted
+ Proposal Evaluation Criteria:
+Understanding the Problem and Responsiveness to RFP: 20 points
+Technical and Scientific Merit: 30 points
+Qualifications, Capabilities, and Management: 20 points
+Communication Plan, Deliverables, and Applicability: 15 points
+Budget and Schedule: 15 points
+ Compliance Standards: OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
+ Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00) — same deadline as the other two WRF grants</t>
+        </is>
+      </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
@@ -839,12 +834,12 @@
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>Oct 25, 2026</t>
+          <t>Oct 26, 2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-d-prize-global-competition-seed-funding-for-new-poverty-solution-distribution-organizations-d-prize-opg-26-00191</t>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-comparison-of-pfas-contributions-to-agricultural-systems-the-water-research-foundation-wrf-opg-26-00190</t>
         </is>
       </c>
     </row>
@@ -921,73 +916,10 @@
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
-          <t>Applications Invited for Comparison of PFAS Contributions to Agricultural Systems</t>
+          <t>Applications Invited for Adaptive Control Frameworks to Unlock Full-Scale BNR Potential Water Research Foundation WRF</t>
         </is>
       </c>
       <c r="C12" s="1" t="inlineStr">
-        <is>
-          <t>Project Objectives:
-Report per- and polyfluoroalkyl substance (PFAS) concentrations from a variety of agricultural inputs — animal manures, fertilizers, pesticides, composts, soil amendments, seed coatings, and biosolids-based products
-Compare the impact of various agricultural inputs on PFAS concentration in the soil profile over varying timeframes
-Evaluate the fate and transport of different inputs to PFAS contributions in agricultural systems at field-scale
-Determine relative contributions from biosolids-based products vs. other inputs to help develop/prioritize risk management strategies
- Background/Rationale:
-Growing concern exists over human exposure to PFAS through biosolids land application on agricultural systems, with regulatory bans on biosolids land application enacted or proposed in at least 12 U.S. states. Utilities relying on land application for biosolids management are scrambling for alternative disposal pathways. The U.S. EPA's 2026 draft guidance noted its earlier 2025 draft risk assessment of PFOA/PFOS-contaminated sewage sludge lacked important contextual information (e.g., a national survey of PFOA/PFOS concentrations). Risk assessments have focused primarily on biosolids, with less attention to PFAS contributions from other sources — manures, compost, fertilizers, pesticides, seed coatings, irrigation water, farming practices, and atmospheric deposition. A Minnesota Pollution Control Agency review found 12 inert pesticide ingredients classified as PFAS. This project aims to improve understanding of PFAS risks from the wider range of agricultural inputs to support strategic resource allocation and inform policy amid surging fertilizer prices and shifts toward local circular resources.
- Research Approach:
-Develop a baseline of knowledge on PFAS in biosolids and non-biosolids agricultural inputs via literature review, analytical methods evaluation, and examination of manufacturing/processing pathways; identify data gaps and uncertainties
-Measure/report compound-specific PFAS concentrations and profiles in agricultural inputs using standardized methods, including precursor characteristics for source attribution where possible
-Characterize PFAS contributions via literature review, data analysis, and field sampling — comparing soil profile/plant tissue composition between fields with non-biosolids inputs vs. biosolids-applied systems; study should test hypotheses on PFAS sources, transformation, retention, and mobility
-Optional additional focus areas: influence of soil/hydrologic/hydrochemistry conditions on PFAS behavior; degradation/transformation pathways; relative PFAS contributions across product lifecycle stages (manufacturing, bagging, delivery, etc.)
-Research approach should be hypothesis-driven, detailing specific end-user needs, and proposers are encouraged to leverage existing projects on PFAS plant uptake/fate/transport.
- Expected Deliverables:
-Research report (WRF's Research Report Template) including: literature review, PFAS analysis of select products, risk management implications/prioritization recommendations, agriculture end-use guidance
-A webcast or workshop to share findings
-Optional additional deliverables: relative risk framework (mass input/fate/exposure/risk), decision support guide for farmers/regulators/utilities, plain language fact sheet, comparative PFAS mass input tool (spreadsheet/calculator)
- Project Duration: 36 months from contract start date (longer than the other two WRF grants above, which were 24 months)
- Eligibility to Submit:
-Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible. Not open to individuals (same structure as the two prior WRF grants).
- Budget/Funding:
-Maximum WRF funding: $400,000 (the largest of the three WRF grants shared so far)
-Applicant must contribute at least 33% of the project award as additional resources (cost share, applicant in-kind, or third-party in-kind per 2 CFR Part 200.306)
-Proposals not meeting the 33% minimum match will not be accepted
- Proposal Evaluation Criteria:
-Understanding the Problem and Responsiveness to RFP: 20 points
-Technical and Scientific Merit: 30 points
-Qualifications, Capabilities, and Management: 20 points
-Communication Plan, Deliverables, and Applicability: 15 points
-Budget and Schedule: 15 points
- Compliance Standards: OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
- Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00) — same deadline as the other two WRF grants</t>
-        </is>
-      </c>
-      <c r="D12" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E12" s="1" t="inlineStr">
-        <is>
-          <t>Oct 26, 2026</t>
-        </is>
-      </c>
-      <c r="F12" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-comparison-of-pfas-contributions-to-agricultural-systems-the-water-research-foundation-wrf-opg-26-00190</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="95" customHeight="1">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B13" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Adaptive Control Frameworks to Unlock Full-Scale BNR Potential Water Research Foundation WRF</t>
-        </is>
-      </c>
-      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Water Research Foundation (WRF) is the leading research organization advancing the science of all water to meet the evolving needs of its subscribers and the water sector. WRF is a nonprofit, charitable and educational organization which funds, manages, and publishes research on the technology, operation, and management of drinking water, wastewater, reuse, and stormwater collection, treatment and supply systems—all in pursuit of ensuring water quality and improving water services to the public.
@@ -1028,74 +960,34 @@
 Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
         </is>
       </c>
-      <c r="D13" s="1" t="inlineStr">
+      <c r="D12" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E13" s="1" t="inlineStr">
+      <c r="E12" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F13" s="1" t="inlineStr">
+      <c r="F12" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-adaptive-control-frameworks-to-unlock-full-scale-bnr-potential-water-research-foundation-wrf-the-water-research-foundation-wrf-opg-26-00187</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="95" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
+    <row r="13" ht="95" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>onepurpos</t>
         </is>
       </c>
-      <c r="B14" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Whitley Award 2027</t>
-        </is>
-      </c>
-      <c r="C14" s="1" t="inlineStr">
-        <is>
-          <t>About the Grant: 
-An annual grant by the Whitley Fund for Nature (WFN) recognising grassroots conservation leaders in the Global South, providing funding to support and scale up proven, science-based solutions that deliver lasting impact for both people and nature.
- About the Award 
-Whitley Awards support grassroots conservation leaders in the Global South. Through funding, training and profile, they help conservationists scale up effective projects that are founded in science and carried out with communities. Whitley Awards are for dynamic, mid-career conservationists who are leading vital conservation projects.
- Grant Amount: £50,000 in project funding over one year
- Eligibility
-Winners are nationals of the country in which they are working, seeking to scale up proven work that is embedded in the local community and would benefit from further funding, a profile boost, and international support.
-Projects must involve communities at the grassroots level and deliver practical action that is founded on science.
-You do not need to be invited or nominated to apply.</t>
-        </is>
-      </c>
-      <c r="D14" s="1" t="inlineStr">
-        <is>
-          <t>Learning</t>
-        </is>
-      </c>
-      <c r="E14" s="1" t="inlineStr">
-        <is>
-          <t>Oct 30, 2026</t>
-        </is>
-      </c>
-      <c r="F14" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-whitley-award-2027-whitley-fund-for-nature-wfn-opg-26-00153</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="95" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="inlineStr">
+      <c r="B13" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIFAR Global Scholars Program 20272029 Cohort</t>
         </is>
       </c>
-      <c r="C15" s="1" t="inlineStr">
+      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 CIFAR is a Canadian-based globally influential research organization that convenes the world’s most brilliant people across disciplines to advance transformative knowledge and solve humanity’s biggest problems, together. By supporting long-term interdisciplinary collaboration, CIFAR provides researchers with an unparalleled environment of trust, transparency and knowledge sharing. Our time-tested model inspires new directions of inquiry, accelerates discovery and yields breakthroughs across borders and academic disciplines. Through knowledge mobilization, we are catalysts for change in industry, government and society. Through our 15 research programs and the Pan-Canadian AI Strategy, CIFAR convenes close to 400 of the world’s top researchers from 141 institutions in 20 countries. CIFAR is generously supported by the governments of Canada, Alberta and Québec, as well as foundations, individuals, corporations and Canadian and international partner organizations.
@@ -1139,301 +1031,34 @@
  Application Deadline: November 4, 2026, 12:00 PM EST</t>
         </is>
       </c>
-      <c r="D15" s="1" t="inlineStr">
+      <c r="D13" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E15" s="1" t="inlineStr">
+      <c r="E13" s="1" t="inlineStr">
         <is>
           <t>Nov 4, 2026</t>
         </is>
       </c>
-      <c r="F15" s="1" t="inlineStr">
+      <c r="F13" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cifar-global-scholars-program-20272029-cohort-cifar-canadian-institute-for-advanced-research-opg-26-00183</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="95" customHeight="1">
-      <c r="A16" s="1" t="inlineStr">
+    <row r="14" ht="95" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
         <is>
           <t>onepurpos</t>
         </is>
       </c>
-      <c r="B16" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for IWRS Teaching Innovation Award</t>
-        </is>
-      </c>
-      <c r="C16" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
- About the Grant
-The IWRS (Insect Welfare Research Society) Teaching Innovation Award supports instructors developing new approaches to teaching insect or invertebrate biology that incorporate the 3Rs (Replacement, Reduction, and Refinement) — principles for reducing animal welfare impacts in teaching and research practices.
- Purpose
-Funds support the creation and implementation of 3Rs-driven instructional materials and pedagogical approaches. Priority is given to proposals addressing common teaching practices with substantial welfare implications.
- Grant Amount
-Two awards of $2,000 USD are available annually.</t>
-        </is>
-      </c>
-      <c r="D16" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E16" s="1" t="inlineStr">
-        <is>
-          <t>Nov 15, 2026</t>
-        </is>
-      </c>
-      <c r="F16" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="95" customHeight="1">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B17" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for CIEIF Grant 2026 Climate Intervention Environmental Impact Fund</t>
-        </is>
-      </c>
-      <c r="C17" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-Climate Intervention Environmental Impact Fund (CIEIF) is a philanthropic fund focused on supporting responsible climate intervention field tests. It provides grants for activities such as environmental impact assessment (EIA), predictive impact modelling, and engagement with potentially affected stakeholders, including local communities and government agencies.
-CIEIF aims to help climate-intervention projects better understand their potential technical, environmental, economic, social, public-health, and safety impacts before and during field testing. It also places importance on the scalability and global relevance of supported innovations and encourages publication of field-test results through peer-reviewed journals or externally peer-reviewed reports.
- About the Grant
-The Climate Intervention Environmental Impact Fund (CIEIF) Grant provides USD 75,000 to support proposed climate intervention field tests. The funding is specifically intended for Environmental Impact Assessment (EIA), predictive impact modelling, and/or engagement with potentially affected stakeholders, including local communities and government agencies.
-Applicants are expected to demonstrate the proposed field test’s technical readiness, environmental and social considerations, required government approvals, innovation and potential for globally relevant scalability. The application must include a proposed budget showing how the USD 75,000 will be used.
- Grant Objective
-The grant is intended to support proposed climate intervention field tests, particularly activities related to:
-Environmental Impact Assessment (EIA)
-Predictive impact modeling
-Engagement with potentially impacted stakeholders
-Local community and government engagement
-Understanding technical, environmental, economic, social, public-health, and safety challenges
-The proposed application must focus on at least one of these three core areas: EIA, predictive impact modeling, or stakeholder engagement.
- Eligible Project Focus
-The proposed field test should demonstrate:
-A clear climate-intervention concept
-Prior research indicating that the technology is ready for the proposed field test
-Potential for innovation and scalability
-A clear understanding of technical and environmental challenges
-Consideration of economic, social, public-health, and safety implications
-Relevant government permits and approvals
-Potential for scaling the innovation to a globally relevant level</t>
-        </is>
-      </c>
-      <c r="D17" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E17" s="1" t="inlineStr">
-        <is>
-          <t>Dec 1, 2026</t>
-        </is>
-      </c>
-      <c r="F17" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-cieif-grant-2026-climate-intervention-environmental-impact-fund-climate-intervention-environmental-impact-fund-opg-26-00155</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="95" customHeight="1">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Oneness Revival Team ORT NGO Grant Programme 2026</t>
-        </is>
-      </c>
-      <c r="C18" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-Oneness Revival Team (ORT) is a dedicated non-governmental organization (NGO) committed to supporting, funding, and empowering other NGOs that are striving to create meaningful change in communities worldwide. We believe that grassroots organizations and charitable initiatives are at the heart of sustainable development, yet many of them face challenges in accessing essential resources, funding, and strategic partnerships to scale their impact. ORT was founded with the vision of bridging this gap, ensuring that non-profits and humanitarian projects have the necessary tools to succeed.
-At ORT, we are passionate about collaboration, capacity-building, and sustainable impact. By providing financial assistance, mentorship, training, and access to global networks, we help NGOs amplify their reach, improve operational efficiency, and achieve long-term success in their respective fields. Our support extends to a diverse range of causes, including education, healthcare, poverty alleviation, environmental conservation, human rights, disaster relief, and community development.
-Our approach goes beyond just financial aid—we believe in fostering strong, strategic partnerships that enable organizations to work more efficiently and maximize their contributions to society. Through our grant programs, fundraising support, advocacy efforts, and technical assistance, we create an ecosystem where NGOs can thrive and drive transformational change.
-Whether through direct funding, professional development programs, or collaborative initiatives, ORT is committed to helping non-profits overcome barriers, strengthen their impact, and create a better future for the communities they serve. By working together, we can ensure that every organization with a mission to create positive change has the opportunity to flourish and make a lasting difference.
- About the Grant
-The Oneness Revival Team (ORT) NGO Grant Programme 2026 is the fourth annual global grant cycle designed to support registered NGOs with limited operating budgets. The programme provides funding to strengthen organizational capacity, launch or expand community projects, and promote sustainable development through two funding streams: SEED Grant and THRIVE Grant.
- Grant Objectives
-Strengthen grassroots NGOs.
-Support sustainable community development.
-Build organizational capacity.
-Expand successful community programmes.
-Promote advocacy and community outreach.
-Improve long-term sustainability of NGOs.
- Grant Types
-1. SEED Grant (1 Year)
-For:
-NGOs that have never received ORT funding.
-NGOs applying for project or general support.
-Funding may be used for:
-Launching new projects.
-Scaling existing initiatives.
-Capacity building.
-Community outreach.
-Advocacy activities. 
- 2. THRIVE Grant (1 Year)
-For:
-NGOs previously funded by ORT and in good standing.
-Funding may be used for:
-Expanding successful programmes.
-Long-term sustainability.
-Strategic organizational growth.
-Community transformation initiatives.
- Eligibility Criteria
-Applicants must:
-Be a registered NGO / non-profit organization.
-Have an annual operating budget below USD 50,000 (note: the page introduction mentions USD 100,000, but the eligibility section specifies below USD 50,000). 
-Demonstrate measurable community impact.
-Maintain transparent financial management.
-Submit a detailed project proposal, budget, and expected outcomes.</t>
-        </is>
-      </c>
-      <c r="D18" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E18" s="1" t="inlineStr">
-        <is>
-          <t>Dec 20, 2026</t>
-        </is>
-      </c>
-      <c r="F18" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-oneness-revival-team-ort-ngo-grant-programme-2026-oneness-revival-team-ort-opg-26-00143</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="95" customHeight="1">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for 6th Annual Seeding The Future Global Food System Challenge</t>
-        </is>
-      </c>
-      <c r="C19" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-We are one of the largest and most respected private organisations for development cooperation and humanitarian aid in Germany. As a politically and confessionally independent organisation, our value-oriented actions are always based on ethical principles. Our vision is clear: "Zero Hunger by 2030"
- About the Opportunity:
-The Global Food System Challenge recognizes and supports breakthrough innovations that can spark transformations of our food systems, with a particular focus on addressing critical challenges in the Global South. It calls on scientists, engineers, innovators, entrepreneurs, and multidisciplinary teams from NGOs, non-profits, social enterprises, universities, research institutions, and small/emerging for-profit enterprises to submit game-changing innovations that transform food systems.
- Innovation Focus Area (must benefit at least one, ideally more domains):
-Innovations leading to safe and nutritious food for a healthy diet
-Innovations leading to sustainable/regenerative practices keeping food systems within planetary boundaries (including food waste/loss reduction)
-Innovations leading to equitable access to food that is affordable, appealing, and trusted
- Award Levels (three tiers, applicant selects which to apply for):
-Award Amount Number Available Requirement
-Seed Grant $25,000 each Up to 8 For high-potential ideas with prototype/initial proof of concept demonstrating feasibility; must benefit ≥1, ideally 2 domains
-Growth Grant $100,000 each Up to 3 For innovations proven "doable" with economic feasibility at scale and high-impact potential; must benefit ≥2, ideally 3 domains
-Seeding The Future Grand Prize $250,000 each Up to 2 For scalable, economically feasible, trusted innovations with major impact potential; must benefit ≥2, ideally 3 domains
-Eligibility:
-Non-profits/NGOs (any country)
-Academic/research institutions (any country)
-Early-stage or emerging for-profit companies/social enterprises (any country)
-Excludes entities from countries under comprehensive U.S./German sanctions (currently: Afghanistan, Belarus, Crimea, Cuba, Iran, Myanmar, North Korea, Russia, Sevastopol, Sudan, South Sudan, Syria, Kherson/Donetsk/Luhansk/Zaporizhzhia regions of Ukraine, Venezuela)
-Individuals are not eligible — teams of students/researchers may participate as part of an organization's submission
-For-profit applicants: must be early-stage/pre-Series A, financial assets not exceeding $10M
- What Will NOT Be Funded:
-Projects harming food safety, sustainability, or unlikely to be accepted by end-users
-Funds supporting large for-profit entities' commercial R&amp;D/manufacturing/sales
-Non-scalable initiatives with limited long-term impact
-Large for-profit entities (post-Series A)
-Purely theoretical concepts with no experiments/proof of concept
-Political campaigns, capital campaigns, or lobbying
-Individuals with no organizational entity</t>
-        </is>
-      </c>
-      <c r="D19" s="1" t="inlineStr">
-        <is>
-          <t>Safety</t>
-        </is>
-      </c>
-      <c r="E19" s="1" t="inlineStr">
-        <is>
-          <t>Jan 1, 2027</t>
-        </is>
-      </c>
-      <c r="F19" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-6th-annual-seeding-the-future-global-food-system-challenge-welthungerhilfe-opg-26-00180</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="95" customHeight="1">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Microbiota &amp; Women's Health International Call for Projects</t>
-        </is>
-      </c>
-      <c r="C20" s="1" t="inlineStr">
-        <is>
-          <t>About the Grant
-An annual international research grant by the Biocodex Microbiota Foundation (BMF), rewarding research proposals on the microbiota and its implications in Women's Health and Disease. This year's theme: "Unraveling male-female genital microbiome interactions: mechanisms, transmission, and impact on vaginal dysbiosis."
- Theme/Scope
-Proposals could include, but are not limited to, mechanistic studies elucidating how the penile microbiome contributes to the establishment, persistence, and recurrence of vaginal dysbiosis, including bacterial vaginosis. Areas of interest include microbial transmission dynamics during sexual activity, niche adaptation and persistence of BV-associated taxa in the penile environment, and the functional consequences of these interactions for vaginal community stability.
-Studies evaluating how current and emerging interventions (antibiotics, topical or systemic partner therapies, circumcision, or live biotherapeutic products) alter penile microbial ecology and influence treatment response and recurrence risk in female partners are also encouraged.
- Purpose: From 2025, the Biocodex Microbiota Foundation rewards international research proposals involving the microbiota and its implication in Women's Health and Disease. Every year, the call for proposals covers a specific theme chosen by an International Scientific Committee. Either clinical or fundamental research proposals can be submitted. Maximum project duration: 3 years.
- Eligibility
-Open to MDs, PhDs, or Pharm-Ds working in the subject area (gynecology, obstetrics, microbiology, infectious diseases, internal medicine, oncology, etc.).
-No geographic restrictions — all countries are eligible.
-A principal investigator who received a Women's Health International grant from BMF cannot reapply for this award for three years. However, winners of another BMF grant category can apply for this grant.
-Members of the Women's Health International Scientific Committee and their laboratory members are not allowed to apply as Principal Investigators.
- Grant Amount
-€200,000 annually — awarded to researchers within universities, hospitals, or other research settings to finance equipment, operations, or staffing costs. Grants are NOT awarded to individuals directly (must be institutionally affiliated). Institution's overhead costs capped at 10%.</t>
-        </is>
-      </c>
-      <c r="D20" s="1" t="inlineStr">
-        <is>
-          <t>Safety</t>
-        </is>
-      </c>
-      <c r="E20" s="1" t="inlineStr">
-        <is>
-          <t>Jan 15, 2027</t>
-        </is>
-      </c>
-      <c r="F20" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-microbiota-and-womens-health-international-call-for-projects-biocodex-microbiota-foundation-bmf-opg-26-00152</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="95" customHeight="1">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="inlineStr">
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for BES Training and Travel Grants</t>
         </is>
       </c>
-      <c r="C21" s="1" t="inlineStr">
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are a global community of scientists shining a spotlight on the intricacy and value of our natural world, providing the evidence for better decisions. Our vision is for people and nature to thrive in a world that values ecology.
@@ -1472,17 +1097,17 @@
  Application Deadline (Round 2): Opens 30 April 2026, closes 17 May 2026</t>
         </is>
       </c>
-      <c r="D21" s="1" t="inlineStr">
+      <c r="D14" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E21" s="1" t="inlineStr">
+      <c r="E14" s="1" t="inlineStr">
         <is>
           <t>May 17, 2027</t>
         </is>
       </c>
-      <c r="F21" s="1" t="inlineStr">
+      <c r="F14" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-bes-training-and-travel-grants-british-ecological-society-opg-26-00181</t>
         </is>

</xml_diff>

<commit_message>
Auto update Combined.xlsx [Tue Oct  6 08:28:53 UTC 2026]
</commit_message>
<xml_diff>
--- a/output/Combined.xlsx
+++ b/output/Combined.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -495,39 +495,27 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>Application Invited GFF x CIVIC VOICES Call for Proposals</t>
+          <t>ToR - Catalyse Tech Reproductive Maternal Newborn &amp; Child Health</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>About us
-PATH is a global nonprofit that turns innovation into better health. For nearly 50 years, PATH has worked with countries, communities, health workers, researchers, governments, and partners to develop and deliver health innovations, from vaccines and diagnostics to strong health systems and more accessible care. By bringing together expertise in science, economics, technology, advocacy, and other fields, PATH develops and scales innovative solutions to the world’s most pressing health challenges. *PATH has become aware of scams involving false job offers.* Please advise: - PATH will never ask for a fee during any stage of the recruitment process. - All active jobs are advertised directly on our careers page: https://path.silkroad.com/epostings/. - Official PATH emails will always arrive from an @path.org address Please report any suspicious communications to careersitehelp@path.org.
-  Civil society and youth-led organizations are essential partners in improving health and nutrition outcomes for women, children, and adolescents. Yet too often, barriers to participation limit their influence.
-The World Bank Group’s GFF × CIVIC partnership—a joint initiative of the Global Financing Facility for Women, Children and Adolescents (GFF) and the CIVIC: The Civil Society and Social Innovation Alliance—works to help close that gap.
-Through its first pillar, the initiative is supporting a consortium led by PATH—in partnership with the African Institute for Development Policy (AFIDEP) and the Organisation of African Youth (OAY), working together as VOICES (Voices Organizing for Inclusive Civic Engagement and Sustainability)—to strengthen civil society engagement, coalition-building, and youth leadership around domestic resource mobilization for women’s, children’s and adolescent health and nutrition. To advance these objectives, the VOICES consortium will award subgrants to local CSOs and youth-led organizations in up to 22 African countries.
-Funding opportunity
-Up to USD 3,350,000 in financial support will be awarded across up to 22 African countries.
-Recipients must be local CSOs or youth-led organizations and/or community-based organizations.
-Each partnership must include at least 2 and no more than 3 organizations, with at least 1 being a youth-led organization.
-Up to 18-month grants, along with advocacy training, budget analysis technical assistance, and mentorship.
- Application deadline
-Applications close Wednesday, October 7th, 2026 at 23:59 East Africa Time. For more information, including submission details and launch event materials, visit our resource page.
-Call for proposals</t>
+          <t>No description available</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Governance</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Oct 7, 2026</t>
+          <t>Oct 10, 2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/grants/application-invited-gff-x-civic-voices-call-for-proposals-path-opg-26-00192</t>
+          <t>https://onepurpos.in/openings/rfps/tor-catalyse-tech-reproductive-maternal-newborn-and-child-health-selco-foundation-rfp-26-00379</t>
         </is>
       </c>
     </row>
@@ -590,42 +578,10 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>ToR - Catalyse Tech Reproductive Maternal Newborn &amp; Child Health</t>
+          <t>Apply for the ServiceNow Community Solar Fund</t>
         </is>
       </c>
       <c r="C5" s="1" t="inlineStr">
-        <is>
-          <t>No description available</t>
-        </is>
-      </c>
-      <c r="D5" s="1" t="inlineStr">
-        <is>
-          <t>Safety</t>
-        </is>
-      </c>
-      <c r="E5" s="1" t="inlineStr">
-        <is>
-          <t>Oct 10, 2026</t>
-        </is>
-      </c>
-      <c r="F5" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/tor-catalyse-tech-reproductive-maternal-newborn-and-child-health-selco-foundation-rfp-26-00379</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="95" customHeight="1">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>Apply for the ServiceNow Community Solar Fund</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund
 Apply by: 13 October, 2026
@@ -650,19 +606,51 @@
  Projects should include opportunities for ServiceNow employees to volunteer in the project activation or implementation.</t>
         </is>
       </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>Oct 13, 2026</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/apply-for-the-servicenow-community-solar-fund-changex-opg-26-00186</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="95" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>EOI invited for Consultant Road Safety Expert / Technical</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>No description available</t>
+        </is>
+      </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>Governance</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>Oct 13, 2026</t>
+          <t>Oct 15, 2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/grants/apply-for-the-servicenow-community-solar-fund-changex-opg-26-00186</t>
+          <t>https://onepurpos.in/openings/rfps/eoi-invited-for-consultant-road-safety-expert-technical-bharatcares-rfp-26-00381</t>
         </is>
       </c>
     </row>
@@ -674,27 +662,40 @@
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>EOI invited for Consultant Road Safety Expert / Technical</t>
+          <t>Application Invited For Partnering with Local organizations for Screening and Early care awardees</t>
         </is>
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>No description available</t>
+          <t>About the Organization
+We are a not-for-profit public health organization working towards transforming lives for improved health and well-being through locally driven solutions. We have worked in more than 20 states of India with an aim to build the skills of healthcare providers, strengthen management capacity and help create sustainable systems to improve access to quality health services. We work closely with communities and key actors on sustainable solutions for public health challenges: - Non-Communicable Diseases - Women, Adolescent and Child health - Nutrition - Infectious diseases - Environmental Health - Emergency Health and Disaster Response We focus on building public health capacity and community actions for better health outcomes. We work collaboratively with stakeholders, leveraging partnerships and influencing policies and practices. Drawing on our experiences and recognizing the unique needs of each region in India, We work in partnership with key stakeholders to design and deliver targeted responses.
+ Fund design
+The first cohort funds up to five agencies for 12 months (December 2026 – November 2027), backed by PPHF technical support for each agency.
+ Three support pillars 
+1. Screening and continuity of care. Each agency runs community-based screening of adults aged 30+ for hypertension, diabetes and oral, breast and cervical cancer, aligned with the national NCD programme. It tracks every positive case through referral, diagnosis, treatment initiation and followup. Each agency holds 100 screening camps over 12 months, screening 80–100 adults per camp: about 8,000–10,000 people per agency and up to 40,000–50,000 across five agencies. 
+2. Mentoring. PPHF provides each agency with a dedicated mentor, programme tools, training modules and communication materials, along with monthly review calls, field visits and a quarterly cohort learning session. Mentoring covers programme quality, data use and government engagement. 
+3. Capacity building. Agencies receive training for their staff plus organisational development in governance, finance, M&amp;E, safeguarding and resource mobilisation.
+ Eligibility 
+Registered in India as a trust, society or Section 8 company for at least three years, with operations in the proposed district 
+Valid 12A and 80G registration and PAN.  
+Audited financial statements for the last three years; annual expenditure between ₹10 lakh and ₹50 lakh 
+Demonstrated community health work; prior NCD experience preferred, not required 
+Not blacklisted by any government body or donor; no PPHF Board, PAC or staff member on its governing body.</t>
         </is>
       </c>
       <c r="D7" s="1" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Governance</t>
         </is>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>Oct 15, 2026</t>
+          <t>Oct 16, 2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/rfps/eoi-invited-for-consultant-road-safety-expert-technical-bharatcares-rfp-26-00381</t>
+          <t>https://onepurpos.in/openings/grants/application-invited-for-partnering-with-local-organizations-for-screening-and-early-care-awardees-people-to-people-health-foundation-opg-26-00195</t>
         </is>
       </c>
     </row>
@@ -706,27 +707,50 @@
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>RFPs Invited for Consultant to Develop a Technical Assistance Package for National Application of the Digital Health and AI Investment Classification Framework</t>
+          <t>Application Invited for SIDBI Innovation Challenge Fund SICF</t>
         </is>
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>No description available</t>
+          <t>About the Organization
+Set up on April 2, 1990 under an Act of Indian Parliament as a principal financial institution for: -- Promotion -- Financing and -- Development of industries in the MSME sector and -- Co-ordinating the functions of other institutions engaged in similar activities. Provision and Charter: SIDBI was established on April 2, 1990. The Charter establishing it, The Small Industries Development Bank of India Act, 1989 envisaged SIDBI to be "the principal financial institution for the promotion, financing and development of industry in the small-scale sector and to co-ordinate the functions of the institutions engaged in the promotion, financing or developing industry in the small-scale sector and for matters connected therewith or incidental thereto". Business Domain of SIDBI: The business domain of SIDBI consists of small-scale industrial units, which contributes significantly to the national economy in terms of production, employment and exports. Business Strategy of SIDBI: The business strategy of SIDBI is to address the financial and non-financial gaps in the MSME ecosystem. Financial support to MSMEs is provided by way of (a) indirect finance / refinance to banks / financial institutions for onward lending to MSMEs and (b) direct finance in the niche areas like risk capital, sustainable finance, receivable financing, service sector financing, etc.
+ About the Grant
+The SIDBI Innovation Challenge Fund (SICF) is a distinctive, forward-looking digital platform designed to catalyze transformative ideas and drive measurable developmental impact. Conceived as a competitive mechanism, SICF actively seeks to crowd-source pioneering, outcome-oriented solutions that address pressing socio-economic challenges.
+Rooted in SIDBI's mandate as a development finance institution and its commitment to inclusive growth and sustainable development, the Fund supports visionary entities that are not only aligned with development agendas but are also equipped to translate ideas into scalable impact. SICF empowers innovators, enterprises, and changemakers by bridging critical funding gaps and enabling the successful implementation of breakthrough solutions.
+At its core, SICF champions the ethos of Inclusive, Innovative, and Impactful (I3) interventions. It prioritizes projects that:
+Foster sustainable enterprise creation,
+Leverage cutting-edge innovation and technology, and
+Mobilize market-driven ecosystems to unlock economic opportunities for underserved and aspiring communities.
+More than a funding mechanism, SICF is an enabler of change—an ecosystem that nurtures bold thinking, rewards ingenuity, and accelerates the journey from concept to impact. By aligning capital with purpose, SICF strives to build resilient, future-ready solutions that contribute meaningfully to India's development narrative.
+Under windows of SICF, 28 inclusive, innovative, and impactful projects have been supported for capacity building, enterprise creation, market linkage, credit connect and job creation. In all, SIDBI is transforming more than 12,000 lives through various innovative interventions. The beneficiaries supported through SICF mostly comprise of Women, Tribals, Divyangjans, Artisans, Disaster Victims, Manual Scavengers, etc.
+ Objectives
+Simplify: Make complex MSME information easy to understand.
+Contextualise: Deliver AI-enabled guidance tailored to each enterprise.
+Act: Convert information into digital journeys and clear next steps.
+Link: Connect MSMEs with finance, institutions and expert support.
+Expand: Build multilingual, mobile-first solutions for wider adoption.
+ Financial Support
+Application Category: Scale-up / Replicable Interventions
+Fund Support: Fund support upto ₹2 Crore may be considered for the implementation.
+ Theme for the proposed cohort:
+Artificial Intelligence enabled Prototype Solutions for MSME Lifecycle Support
+ Sustainable Development Goals Catered
+The programs supported under the Challenge Fund have made a tangible contribution to the UN's 11 Sustainable Development Goals through various pilot and scale-up interventions. By aligning with the SDGs, the initiatives have helped communities as well as the environment holistically.</t>
         </is>
       </c>
       <c r="D8" s="1" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Governance</t>
         </is>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>Oct 23, 2026</t>
+          <t>Oct 16, 2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/rfps/rfps-invited-for-consultant-to-develop-a-technical-assistance-package-for-national-application-of-the-digital-health-and-ai-investment-classification-framework-transform-health-rfp-26-00359</t>
+          <t>https://onepurpos.in/openings/grants/application-invited-for-sidbi-innovation-challenge-fund-sicf-small-industries-development-bank-of-india-opg-26-00194</t>
         </is>
       </c>
     </row>
@@ -738,10 +762,92 @@
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
+          <t>RFPs Invited for Consultant to Develop a Technical Assistance Package for National Application of the Digital Health and AI Investment Classification Framework</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>No description available</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>Oct 23, 2026</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/rfps-invited-for-consultant-to-develop-a-technical-assistance-package-for-national-application-of-the-digital-health-and-ai-investment-classification-framework-transform-health-rfp-26-00359</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="95" customHeight="1">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Inclusivity Research Grant IRG</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+Anusandhan National Research Foundation (ANRF) - established through an  Act of Parliament: ANRF Act, 2023, to provide high-level strategic directions for research, innovation, and entrepreneurship in the fields of natural sciences, including mathematical sciences, engineering and technology, environmental and earth sciences, health and agriculture, and scientific and technological interfaces of humanities and social sciences.
+ About the Grant:
+Anusandhan National Research Foundation (ANRF) was established through an Act of Parliament (ANRF Act 2023) to undertake initiatives seeding, growing, and facilitating research at academic and research institutions. In its effort to facilitate equal participation of researchers from all sectors of society, ANRF has initiated the Inclusivity Research Grant (IRG) scheme, providing funding support to researchers belonging to the Scheduled Caste/Scheduled Tribe category to undertake research in frontier areas of science and engineering. It aims to provide a platform for researchers to further their capacity and move on to mainstream research programs. IRG subsumes the erstwhile SERB scheme "Empowerment and Equity Opportunities for Excellence in Science (EMEQ)," with enhanced support and flexible norms.
+ Nature of Support:
+Funding up to Rs. 60 lakh plus overheads, for a period of three years
+Flexibility to utilize resources under the recurring head; flexibility in manpower recruitment; enhanced travel, contingency, and overhead charges
+Support for expenses related to open access publications and patent filing charges
+International travel for project-related activities permitted (within the travel head limit)
+ Eligibility:
+Applicant must be an Indian National
+Must be an active researcher belonging to the Scheduled Caste or Scheduled Tribe category, working on a regular basis in an academic institution/national lab or any other recognized R&amp;D institution in Science and Engineering
+Must hold a PhD degree in Science or Engineering, or MD/MS/MDS degree
+Must have at least 4 years of service remaining before superannuation as of the proposal submission date
+Researchers with ongoing projects under IRG/erstwhile EMEQ scheme are not eligible
+Co-investigators are not allowed
+An investigator may avail an IRG project a maximum of 3 times in their career (including EMEQ projects of erstwhile SERB)
+ Qualification: PhD in Science/Engineering, or MD/MS/MDS
+ Experience Bracket: Active researcher (regular position) with minimum 4 years of service remaining before superannuation</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>Oct 24, 2026</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-inclusivity-research-grant-irg-anusandhan-national-research-foundation-opg-26-00193</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="95" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
           <t>Applications Invited for D-Prize Global Competition Seed Funding for New Poverty-Solution Distribution Organizations</t>
         </is>
       </c>
-      <c r="C9" s="1" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>About the Grant:
 D-Prize seeds new organizations that distribute proven poverty solutions at the "last mile," with the aim of scaling impact. Applicants select from a range of evidence-based interventions (health, agriculture, education, water, safety, transparency, and more) and propose how they would launch or grow an organization to distribute that intervention. Top entrepreneurs receive up to $20,000 in seed funding to run a pilot and build an organization capable of scaling to reach thousands, even millions of people.
@@ -764,147 +870,19 @@
 Extension Deadline: 6 December 2026, midnight PT (extension registration required)</t>
         </is>
       </c>
-      <c r="D9" s="1" t="inlineStr">
+      <c r="D11" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E9" s="1" t="inlineStr">
+      <c r="E11" s="1" t="inlineStr">
         <is>
           <t>Oct 25, 2026</t>
         </is>
       </c>
-      <c r="F9" s="1" t="inlineStr">
+      <c r="F11" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-d-prize-global-competition-seed-funding-for-new-poverty-solution-distribution-organizations-d-prize-opg-26-00191</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="95" customHeight="1">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Comparison of PFAS Contributions to Agricultural Systems</t>
-        </is>
-      </c>
-      <c r="C10" s="1" t="inlineStr">
-        <is>
-          <t>Project Objectives:
-Report per- and polyfluoroalkyl substance (PFAS) concentrations from a variety of agricultural inputs — animal manures, fertilizers, pesticides, composts, soil amendments, seed coatings, and biosolids-based products
-Compare the impact of various agricultural inputs on PFAS concentration in the soil profile over varying timeframes
-Evaluate the fate and transport of different inputs to PFAS contributions in agricultural systems at field-scale
-Determine relative contributions from biosolids-based products vs. other inputs to help develop/prioritize risk management strategies
- Background/Rationale:
-Growing concern exists over human exposure to PFAS through biosolids land application on agricultural systems, with regulatory bans on biosolids land application enacted or proposed in at least 12 U.S. states. Utilities relying on land application for biosolids management are scrambling for alternative disposal pathways. The U.S. EPA's 2026 draft guidance noted its earlier 2025 draft risk assessment of PFOA/PFOS-contaminated sewage sludge lacked important contextual information (e.g., a national survey of PFOA/PFOS concentrations). Risk assessments have focused primarily on biosolids, with less attention to PFAS contributions from other sources — manures, compost, fertilizers, pesticides, seed coatings, irrigation water, farming practices, and atmospheric deposition. A Minnesota Pollution Control Agency review found 12 inert pesticide ingredients classified as PFAS. This project aims to improve understanding of PFAS risks from the wider range of agricultural inputs to support strategic resource allocation and inform policy amid surging fertilizer prices and shifts toward local circular resources.
- Research Approach:
-Develop a baseline of knowledge on PFAS in biosolids and non-biosolids agricultural inputs via literature review, analytical methods evaluation, and examination of manufacturing/processing pathways; identify data gaps and uncertainties
-Measure/report compound-specific PFAS concentrations and profiles in agricultural inputs using standardized methods, including precursor characteristics for source attribution where possible
-Characterize PFAS contributions via literature review, data analysis, and field sampling — comparing soil profile/plant tissue composition between fields with non-biosolids inputs vs. biosolids-applied systems; study should test hypotheses on PFAS sources, transformation, retention, and mobility
-Optional additional focus areas: influence of soil/hydrologic/hydrochemistry conditions on PFAS behavior; degradation/transformation pathways; relative PFAS contributions across product lifecycle stages (manufacturing, bagging, delivery, etc.)
-Research approach should be hypothesis-driven, detailing specific end-user needs, and proposers are encouraged to leverage existing projects on PFAS plant uptake/fate/transport.
- Expected Deliverables:
-Research report (WRF's Research Report Template) including: literature review, PFAS analysis of select products, risk management implications/prioritization recommendations, agriculture end-use guidance
-A webcast or workshop to share findings
-Optional additional deliverables: relative risk framework (mass input/fate/exposure/risk), decision support guide for farmers/regulators/utilities, plain language fact sheet, comparative PFAS mass input tool (spreadsheet/calculator)
- Project Duration: 36 months from contract start date (longer than the other two WRF grants above, which were 24 months)
- Eligibility to Submit:
-Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible. Not open to individuals (same structure as the two prior WRF grants).
- Budget/Funding:
-Maximum WRF funding: $400,000 (the largest of the three WRF grants shared so far)
-Applicant must contribute at least 33% of the project award as additional resources (cost share, applicant in-kind, or third-party in-kind per 2 CFR Part 200.306)
-Proposals not meeting the 33% minimum match will not be accepted
- Proposal Evaluation Criteria:
-Understanding the Problem and Responsiveness to RFP: 20 points
-Technical and Scientific Merit: 30 points
-Qualifications, Capabilities, and Management: 20 points
-Communication Plan, Deliverables, and Applicability: 15 points
-Budget and Schedule: 15 points
- Compliance Standards: OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
- Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00) — same deadline as the other two WRF grants</t>
-        </is>
-      </c>
-      <c r="D10" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E10" s="1" t="inlineStr">
-        <is>
-          <t>Oct 26, 2026</t>
-        </is>
-      </c>
-      <c r="F10" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-comparison-of-pfas-contributions-to-agricultural-systems-the-water-research-foundation-wrf-opg-26-00190</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="95" customHeight="1">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Crossing the Divide Best Practices for Addressing Local and Privately-Owned Lateral Sewer Issues RFP 5419</t>
-        </is>
-      </c>
-      <c r="C11" s="1" t="inlineStr">
-        <is>
-          <t>Project Objective:
-To provide water resource recovery facilities (WRRFs) and collection system operators with an interactive manual of practice for implementing inflow and infiltration (I&amp;I) and obstruction management programs, focused on municipal and privately owned lateral sewers in complex legal, regulatory, and multi-jurisdictional environments.
- Background/Rationale:
-Wastewater utilities face continuing challenges providing cost-effective sewer services amid rising demand, urban redevelopment, and performance disruptors (root intrusion, pipe degradation, blockages). I&amp;I and obstruction management remain persistent, costly problems without a consolidated resource to guide program design. During wet weather, peak I&amp;I flows can increase influent flows 3–5x average. Studies suggest up to 80% of I&amp;I originates on private property, and root intrusions cause over 50% of sewer blockages globally. Program effectiveness varies widely depending on statutory authority, multi-jurisdictional overlap, enforcement mechanisms, and participant willingness.
- Central Research Questions:
-What I&amp;I and obstruction management practices are utilities using today, and how do they vary by jurisdictional/regulatory/infrastructure/environmental conditions?
-Which factors most influence successful implementation, and what barriers commonly derail programs?
-What measurable benefits (cost avoidance, capacity recovery, reduced spill risk, improved regulatory standing) have utilities realized from successful programs?
-This project extends WRF's ongoing "State-of-Practice Manual for Inflow and Infiltration Detection and Mitigation at Street and Private Lateral Levels" (Project 5365) into I&amp;I source control and obstruction management specifically.
- Research Approach (4 Tasks):
-Literature and Regulatory Review — Comprehensive review of legal authorities/regulations in the US and comparable international jurisdictions; catalog program elements, enforcement mechanisms, incentive structures, and legal/jurisdictional barriers
-Utility Survey and Case Study Development — Broad survey across utility size/geography/system type; select at least 5 diverse in-depth case studies with quantitative results (I&amp;I reduction %, reduced bypass pumping, reduced basement backups, cost savings, recovered capacity, reduced blockage-related spills/service calls)
-Utility Workshop — At least one invitation-only workshop with utility representatives to present survey findings and gather structured feedback on draft guidance content
-Interactive Manual of Practice — Development of a decision-support tool/web-based application/interactive PDF enabling utilities to select effective I&amp;I/obstruction program elements based on their statutory authority, jurisdictional complexity, and enforcement mechanisms
- Expected Deliverables:
-Research report (using WRF's Research Report Template) including literature/regulatory review
-Interactive manual of practice (following Technology Deliverables Guidance)
-In-depth utility survey, state-of-the-practice report, and at least 5 standalone case studies with quantitative results
-Summary documentation of the utility workshop, including feedback and how it was incorporated
- Project Duration: 24 months from contract start date (No-Cost Extension Policy caps extensions at 9 months beyond original schedule)
- Eligibility to Submit:
-Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible as named participants. Not open to individuals (same institutional-applicant structure as RFP 5424).
- Budget/Funding:
-Maximum WRF funding: $250,000
-Applicant must contribute at least 33% of the project award as additional resources (cost share, applicant in-kind, or third-party in-kind per 2 CFR Part 200.306)
-Proposals not meeting the 33% minimum match will not be accepted
- Proposal Evaluation Criteria:
-Understanding the Problem and Responsiveness to RFP: 20 points
-Technical and Scientific Merit: 30 points
-Qualifications, Capabilities, and Management: 20 points
-Communication Plan, Deliverables, and Applicability: 15 points
-Budget and Schedule: 15 points
- Compliance Standards: OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
- Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
-        </is>
-      </c>
-      <c r="D11" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E11" s="1" t="inlineStr">
-        <is>
-          <t>Oct 26, 2026</t>
-        </is>
-      </c>
-      <c r="F11" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-crossing-the-divide-best-practices-for-addressing-local-and-privately-owned-lateral-sewer-issues-rfp-5419-the-water-research-foundation-wrf-opg-26-00189</t>
         </is>
       </c>
     </row>
@@ -984,10 +962,268 @@
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
+          <t>Applications Invited for Comparison of PFAS Contributions to Agricultural Systems</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>Project Objectives:
+Report per- and polyfluoroalkyl substance (PFAS) concentrations from a variety of agricultural inputs — animal manures, fertilizers, pesticides, composts, soil amendments, seed coatings, and biosolids-based products
+Compare the impact of various agricultural inputs on PFAS concentration in the soil profile over varying timeframes
+Evaluate the fate and transport of different inputs to PFAS contributions in agricultural systems at field-scale
+Determine relative contributions from biosolids-based products vs. other inputs to help develop/prioritize risk management strategies
+ Background/Rationale:
+Growing concern exists over human exposure to PFAS through biosolids land application on agricultural systems, with regulatory bans on biosolids land application enacted or proposed in at least 12 U.S. states. Utilities relying on land application for biosolids management are scrambling for alternative disposal pathways. The U.S. EPA's 2026 draft guidance noted its earlier 2025 draft risk assessment of PFOA/PFOS-contaminated sewage sludge lacked important contextual information (e.g., a national survey of PFOA/PFOS concentrations). Risk assessments have focused primarily on biosolids, with less attention to PFAS contributions from other sources — manures, compost, fertilizers, pesticides, seed coatings, irrigation water, farming practices, and atmospheric deposition. A Minnesota Pollution Control Agency review found 12 inert pesticide ingredients classified as PFAS. This project aims to improve understanding of PFAS risks from the wider range of agricultural inputs to support strategic resource allocation and inform policy amid surging fertilizer prices and shifts toward local circular resources.
+ Research Approach:
+Develop a baseline of knowledge on PFAS in biosolids and non-biosolids agricultural inputs via literature review, analytical methods evaluation, and examination of manufacturing/processing pathways; identify data gaps and uncertainties
+Measure/report compound-specific PFAS concentrations and profiles in agricultural inputs using standardized methods, including precursor characteristics for source attribution where possible
+Characterize PFAS contributions via literature review, data analysis, and field sampling — comparing soil profile/plant tissue composition between fields with non-biosolids inputs vs. biosolids-applied systems; study should test hypotheses on PFAS sources, transformation, retention, and mobility
+Optional additional focus areas: influence of soil/hydrologic/hydrochemistry conditions on PFAS behavior; degradation/transformation pathways; relative PFAS contributions across product lifecycle stages (manufacturing, bagging, delivery, etc.)
+Research approach should be hypothesis-driven, detailing specific end-user needs, and proposers are encouraged to leverage existing projects on PFAS plant uptake/fate/transport.
+ Expected Deliverables:
+Research report (WRF's Research Report Template) including: literature review, PFAS analysis of select products, risk management implications/prioritization recommendations, agriculture end-use guidance
+A webcast or workshop to share findings
+Optional additional deliverables: relative risk framework (mass input/fate/exposure/risk), decision support guide for farmers/regulators/utilities, plain language fact sheet, comparative PFAS mass input tool (spreadsheet/calculator)
+ Project Duration: 36 months from contract start date (longer than the other two WRF grants above, which were 24 months)
+ Eligibility to Submit:
+Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible. Not open to individuals (same structure as the two prior WRF grants).
+ Budget/Funding:
+Maximum WRF funding: $400,000 (the largest of the three WRF grants shared so far)
+Applicant must contribute at least 33% of the project award as additional resources (cost share, applicant in-kind, or third-party in-kind per 2 CFR Part 200.306)
+Proposals not meeting the 33% minimum match will not be accepted
+ Proposal Evaluation Criteria:
+Understanding the Problem and Responsiveness to RFP: 20 points
+Technical and Scientific Merit: 30 points
+Qualifications, Capabilities, and Management: 20 points
+Communication Plan, Deliverables, and Applicability: 15 points
+Budget and Schedule: 15 points
+ Compliance Standards: OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
+ Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00) — same deadline as the other two WRF grants</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>Oct 26, 2026</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-comparison-of-pfas-contributions-to-agricultural-systems-the-water-research-foundation-wrf-opg-26-00190</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="95" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for 8th Call for Proposals Small-Size Grants Global EbA Fund</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
+ About the Opportunity:
+The Global EbA Fund invites innovative and catalytic proposals that address systemic barriers to Ecosystem-based Adaptation (EbA) scaling — by enhancing institutional and technical capacities, quality data/evidence generation, learning networks, and investment readiness. Aligned with the IKI Strategy up to 2030 (focus on socio-ecological transformation), the Fund's primary geographic focus is ODA-eligible SIDS (Small Island Developing States) and LDCs (Least Developed Countries), though other ODA-eligible countries may be considered where proposals show exceptional ambition.
+ Focus Areas:
+Overcoming upstream barriers to EbA uptake/scaling (institutional &amp; technical capacity constraints, evidence generation, knowledge exchange)
+Clear adaptation chain grounded in detailed impact chain analysis (climate hazards/risks, socioeconomic/ecological sensitivity, adaptive capacity)
+Social and environmental considerations (gender responsiveness, Indigenous Peoples' rights, local participation, environmental/social safeguards, prevention of maladaptation)
+Robust sustainability and exit strategies (long-term viability, local ownership, institutional continuity)
+ Encouraged Topics:
+Investment readiness and project pipeline preparation
+Innovative technologies for EbA
+Applied and functional research
+Synergies with other EbA/Nature-based Solution (NbS) initiatives
+ Grant Size: Up to USD 250,000 per grant
+ Project Duration: Up to 24 months
+ Eligible Applicant Types:
+Non-governmental organisations (NGOs)
+International NGOs (INGOs)
+Intergovernmental organisations (IGOs)
+Community-based organisations (CBOs)
+Indigenous People's Organisations
+Universities and academic institutions
+Research institutes and think tanks
+Private sector companies (under certain conditions; no funding for sector-specific obligations, compensatory measures, or for-profit activities)
+Consortia (must designate a clear lead "Applicant Organisation"; government entities can join a consortium but cannot receive Fund money directly)
+Note: Individuals are not eligible (e.g., no PhD study funding); UNEP and IUCN offices are also not eligible to apply.
+ Key Eligibility Criteria:
+Must qualify as Ecosystem-based Adaptation (EbA) per the Fund's Qualification Criteria &amp; Quality Standards
+Must have catalytic/innovative potential
+Must clearly identify climate impacts addressed
+Falls under max 1 Strategic Objective and max 2 Action Pillars of the Fund
+Global, thematic, or targets only ODA-eligible countries
+Budget up to USD 250,000; duration up to 24 months
+Must build on existing work (not standalone/field-implementation-only projects)
+Must show sustainability post-funding
+Must partner with local institutions
+Applicant &amp; partners must be legally recognized entities with relevant experience
+Must complete Due Diligence requirements
+ Evaluation Criteria (weighted):
+Ecosystem-based Adaptation (EbA) approach — 30%
+Design &amp; Methodology (Theory of Change, logframe, SMART indicators, budget coherence)
+Gender &amp; Social Inclusion (participatory approach, FPIC for Indigenous Peoples' impact)
+Innovative &amp; Catalytic Contribution — 30%
+Sustainability — 20%
+Institutional Arrangements — 20%
+ Reporting Requirement: Applicants must identify at least 3 indicators from the Fund's Core Indicator Framework for their project's logframe.
+ Application Package Required:
+Applicant Declaration
+Co-applicant Mandate (if applicable)
+Small-Size Grants Application Form
+Project Proposal Budget Template
+Due Diligence and Financial Capacity Questionnaire (with Annexes 1(c)(i) and 1(c)(ii) at submission stage)
+ Application Language: English only (organizational documents must be translated to English
+ Timeline:
+Call officially launched: August 24, 2026
+Submission window: September 28 – October 26, 2026
+Applications submitted via online portal (link shared on the Small-Size Grants webpage from Sept 28)
+Only successful applicants will be contacted; no individual feedback provided to unsuccessful applicants</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>Oct 26, 2026</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-8th-call-for-proposals-small-size-grants-global-eba-fund-global-eba-fund-opg-26-00177</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="95" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Crossing the Divide Best Practices for Addressing Local and Privately-Owned Lateral Sewer Issues RFP 5419</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>Project Objective:
+To provide water resource recovery facilities (WRRFs) and collection system operators with an interactive manual of practice for implementing inflow and infiltration (I&amp;I) and obstruction management programs, focused on municipal and privately owned lateral sewers in complex legal, regulatory, and multi-jurisdictional environments.
+ Background/Rationale:
+Wastewater utilities face continuing challenges providing cost-effective sewer services amid rising demand, urban redevelopment, and performance disruptors (root intrusion, pipe degradation, blockages). I&amp;I and obstruction management remain persistent, costly problems without a consolidated resource to guide program design. During wet weather, peak I&amp;I flows can increase influent flows 3–5x average. Studies suggest up to 80% of I&amp;I originates on private property, and root intrusions cause over 50% of sewer blockages globally. Program effectiveness varies widely depending on statutory authority, multi-jurisdictional overlap, enforcement mechanisms, and participant willingness.
+ Central Research Questions:
+What I&amp;I and obstruction management practices are utilities using today, and how do they vary by jurisdictional/regulatory/infrastructure/environmental conditions?
+Which factors most influence successful implementation, and what barriers commonly derail programs?
+What measurable benefits (cost avoidance, capacity recovery, reduced spill risk, improved regulatory standing) have utilities realized from successful programs?
+This project extends WRF's ongoing "State-of-Practice Manual for Inflow and Infiltration Detection and Mitigation at Street and Private Lateral Levels" (Project 5365) into I&amp;I source control and obstruction management specifically.
+ Research Approach (4 Tasks):
+Literature and Regulatory Review — Comprehensive review of legal authorities/regulations in the US and comparable international jurisdictions; catalog program elements, enforcement mechanisms, incentive structures, and legal/jurisdictional barriers
+Utility Survey and Case Study Development — Broad survey across utility size/geography/system type; select at least 5 diverse in-depth case studies with quantitative results (I&amp;I reduction %, reduced bypass pumping, reduced basement backups, cost savings, recovered capacity, reduced blockage-related spills/service calls)
+Utility Workshop — At least one invitation-only workshop with utility representatives to present survey findings and gather structured feedback on draft guidance content
+Interactive Manual of Practice — Development of a decision-support tool/web-based application/interactive PDF enabling utilities to select effective I&amp;I/obstruction program elements based on their statutory authority, jurisdictional complexity, and enforcement mechanisms
+ Expected Deliverables:
+Research report (using WRF's Research Report Template) including literature/regulatory review
+Interactive manual of practice (following Technology Deliverables Guidance)
+In-depth utility survey, state-of-the-practice report, and at least 5 standalone case studies with quantitative results
+Summary documentation of the utility workshop, including feedback and how it was incorporated
+ Project Duration: 24 months from contract start date (No-Cost Extension Policy caps extensions at 9 months beyond original schedule)
+ Eligibility to Submit:
+Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible as named participants. Not open to individuals (same institutional-applicant structure as RFP 5424).
+ Budget/Funding:
+Maximum WRF funding: $250,000
+Applicant must contribute at least 33% of the project award as additional resources (cost share, applicant in-kind, or third-party in-kind per 2 CFR Part 200.306)
+Proposals not meeting the 33% minimum match will not be accepted
+ Proposal Evaluation Criteria:
+Understanding the Problem and Responsiveness to RFP: 20 points
+Technical and Scientific Merit: 30 points
+Qualifications, Capabilities, and Management: 20 points
+Communication Plan, Deliverables, and Applicability: 15 points
+Budget and Schedule: 15 points
+ Compliance Standards: OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
+ Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
+        </is>
+      </c>
+      <c r="D15" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E15" s="1" t="inlineStr">
+        <is>
+          <t>Oct 26, 2026</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-crossing-the-divide-best-practices-for-addressing-local-and-privately-owned-lateral-sewer-issues-rfp-5419-the-water-research-foundation-wrf-opg-26-00189</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="95" customHeight="1">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Whitley Award 2027</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t>About the Grant: 
+An annual grant by the Whitley Fund for Nature (WFN) recognising grassroots conservation leaders in the Global South, providing funding to support and scale up proven, science-based solutions that deliver lasting impact for both people and nature.
+ About the Award 
+Whitley Awards support grassroots conservation leaders in the Global South. Through funding, training and profile, they help conservationists scale up effective projects that are founded in science and carried out with communities. Whitley Awards are for dynamic, mid-career conservationists who are leading vital conservation projects.
+ Grant Amount: £50,000 in project funding over one year
+ Eligibility
+Winners are nationals of the country in which they are working, seeking to scale up proven work that is embedded in the local community and would benefit from further funding, a profile boost, and international support.
+Projects must involve communities at the grassroots level and deliver practical action that is founded on science.
+You do not need to be invited or nominated to apply.</t>
+        </is>
+      </c>
+      <c r="D16" s="1" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E16" s="1" t="inlineStr">
+        <is>
+          <t>Oct 30, 2026</t>
+        </is>
+      </c>
+      <c r="F16" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-whitley-award-2027-whitley-fund-for-nature-wfn-opg-26-00153</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="95" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
           <t>Applications Invited for CIFAR Global Scholars Program 20272029 Cohort</t>
         </is>
       </c>
-      <c r="C13" s="1" t="inlineStr">
+      <c r="C17" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 CIFAR is a Canadian-based globally influential research organization that convenes the world’s most brilliant people across disciplines to advance transformative knowledge and solve humanity’s biggest problems, together. By supporting long-term interdisciplinary collaboration, CIFAR provides researchers with an unparalleled environment of trust, transparency and knowledge sharing. Our time-tested model inspires new directions of inquiry, accelerates discovery and yields breakthroughs across borders and academic disciplines. Through knowledge mobilization, we are catalysts for change in industry, government and society. Through our 15 research programs and the Pan-Canadian AI Strategy, CIFAR convenes close to 400 of the world’s top researchers from 141 institutions in 20 countries. CIFAR is generously supported by the governments of Canada, Alberta and Québec, as well as foundations, individuals, corporations and Canadian and international partner organizations.
@@ -1031,34 +1267,312 @@
  Application Deadline: November 4, 2026, 12:00 PM EST</t>
         </is>
       </c>
-      <c r="D13" s="1" t="inlineStr">
+      <c r="D17" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E13" s="1" t="inlineStr">
+      <c r="E17" s="1" t="inlineStr">
         <is>
           <t>Nov 4, 2026</t>
         </is>
       </c>
-      <c r="F13" s="1" t="inlineStr">
+      <c r="F17" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cifar-global-scholars-program-20272029-cohort-cifar-canadian-institute-for-advanced-research-opg-26-00183</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="95" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="inlineStr">
+    <row r="18" ht="95" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for IWRS Teaching Innovation Award</t>
+        </is>
+      </c>
+      <c r="C18" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
+ About the Grant
+The IWRS (Insect Welfare Research Society) Teaching Innovation Award supports instructors developing new approaches to teaching insect or invertebrate biology that incorporate the 3Rs (Replacement, Reduction, and Refinement) — principles for reducing animal welfare impacts in teaching and research practices.
+ Purpose
+Funds support the creation and implementation of 3Rs-driven instructional materials and pedagogical approaches. Priority is given to proposals addressing common teaching practices with substantial welfare implications.
+ Grant Amount
+Two awards of $2,000 USD are available annually.</t>
+        </is>
+      </c>
+      <c r="D18" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E18" s="1" t="inlineStr">
+        <is>
+          <t>Nov 15, 2026</t>
+        </is>
+      </c>
+      <c r="F18" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="95" customHeight="1">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for IWRS Teaching Innovation Award</t>
+        </is>
+      </c>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+Insects are one of the most numerous and diverse animal groups on Earth.
+Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice.
+About the Award
+The IWRS Teaching Innovation Award supports instructors developing new approaches to teaching invertebrate biology that incorporate the 3Rs (replacement, reduction, and refinement). It also supports the development and implementation of any novel curricula addressing invertebrate welfare and sentience across invertebrate biology, animal welfare science, and/or veterinary medicine fields.
+Grant size
+Awards up to $2,000 USD are available for approaches requiring equipment or other materials; awards up to $1,000 USD are available otherwise. Funds may be used to support any costs associated with curriculum development and implementation, including stipends, teaching tools, and related expenses. Priority is given to proposals addressing common teaching practices with substantial welfare implications.
+Who can apply for funding?
+The applicant must be an instructor teaching content related to insect or invertebrate biology at an educational institution, scientific society or museum, field-training course, or similar educational context. If you are unsure about your eligibility, contact grants@insectwelfare.com.
+The applicant can be from any discipline, country, or institution. However, we will not pay awards to recipients located in jurisdictions, countries, or regions subject to trade restrictions, embargoes, or sanctions put in place by the United Nations or the United States of America.
+IWRS staff and Advisory Group members are not eligible to apply.</t>
+        </is>
+      </c>
+      <c r="D19" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E19" s="1" t="inlineStr">
+        <is>
+          <t>Nov 15, 2026</t>
+        </is>
+      </c>
+      <c r="F19" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00166</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="95" customHeight="1">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Medium-Size Grants Call for Proposals Global EbA Fund</t>
+        </is>
+      </c>
+      <c r="C20" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
+ About the Opportunity:
+The Global EbA Fund invites proposals under its General Track: Strategic Scaling and Global Influence, seeking collaborative and innovative approaches to advancing Ecosystem-based Adaptation (EbA) by addressing systemic barriers to scalability and contributing to global learning and policy dialogue. Initiatives should strengthen enabling environments and embed EbA into national frameworks that unify climate, biodiversity, land, and development priorities. Alignment with one of three priority topics is welcomed but not mandatory:
+ Priority Topics:
+I. Innovative Finance Solutions for EbA — partnerships with private sector actors (financiers, innovators, local champions) to unlock private capital/blended finance for EbA, evolving EbA into profitable, scalable business models
+II. EbA for Human Development and Security — integrating EbA into national/international security frameworks for fragile and conflict-affected contexts; community co-designed interventions that reduce natural resource-related tensions and climate-induced fragility, bridging adaptation, humanitarian, development, and peacebuilding agendas
+III. Interlinkages for People-Nature-Climate-Land Synergies — strengthening operational links across the Rio Conventions (UNFCCC, CBD, UNCCD) and frameworks like the Sendai Framework on DRR, using EbA as the anchor connecting biodiversity, sustainable land management, climate adaptation, and disaster risk reduction
+ Grant Size: Up to USD 500,000 per grant
+ Project Duration: Up to 24 months
+ Eligible Applicant Types:
+Non-governmental organisations (NGOs)
+International NGOs (INGOs)
+Intergovernmental organisations (IGOs)
+Community-based organisations (CBOs)
+Indigenous People's Organisations
+Universities and academic institutions
+Research institutes and think tanks
+Private sector companies (under certain conditions)
+Consortia (must designate a clear lead "Applicant Organisation"; government entities may join but cannot receive Fund money directly)
+Note: Individuals are not eligible; UNEP and IUCN offices are also not eligible.
+ Key Eligibility Criteria:
+Must qualify as Ecosystem-based Adaptation (EbA) per the Fund's Qualification Criteria &amp; Quality Standards
+Must show catalytic/innovative potential
+Must clearly identify climate impacts addressed
+Falls under max 1 Strategic Objective and max 2 Action Pillars of the Fund
+Global, thematic, or targets only ODA-eligible countries
+Budget up to USD 500,000; duration ≤24 months
+Must build on existing work (not standalone/field-implementation-only)
+Must show sustainability post-funding
+Must partner with local institutions
+Applicant &amp; partners must be legally recognized entities with relevant experience
+Must comply with Due Diligence requirements
+ Evaluation Criteria (weighted):
+Ecosystem-based Adaptation (EbA) approach — 30%
+Design &amp; Methodology (Theory of Change, logframe, SMART indicators, budget coherence)
+Gender &amp; Social Inclusion (participatory approach, FPIC for Indigenous Peoples' impact)
+Innovative &amp; Catalytic Contribution — 30%
+Sustainability — 20%
+Institutional Arrangements — 20%
+ Reporting Requirement: 
+Applicants must identify at least 3 indicators from the Fund's Core Indicator Framework for their project's logframe.
+ Application Package Required:
+Applicant Declaration
+Co-applicant Mandate (if applicable)
+Medium-Size Grants Application Form
+Project Proposal Budget Template
+Due Diligence and Financial Capacity Questionnaire (with Annexes 1(c)(i) and 1(c)(ii) at submission stage)
+ Application Language: English only (organizational documents must be translated to English)
+ Timeline:
+Call officially launched: August 24, 2026
+Submission window: October 12 – November 16, 2026
+Applications submitted via online portal (link shared on the Medium-Size Grants webpage from Oct 12)</t>
+        </is>
+      </c>
+      <c r="D20" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E20" s="1" t="inlineStr">
+        <is>
+          <t>Nov 16, 2026</t>
+        </is>
+      </c>
+      <c r="F20" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-medium-size-grants-call-for-proposals-global-eba-fund-global-eba-fund-opg-26-00178</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="95" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for CIEIF Grant 2026 Climate Intervention Environmental Impact Fund</t>
+        </is>
+      </c>
+      <c r="C21" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+Climate Intervention Environmental Impact Fund (CIEIF) is a philanthropic fund focused on supporting responsible climate intervention field tests. It provides grants for activities such as environmental impact assessment (EIA), predictive impact modelling, and engagement with potentially affected stakeholders, including local communities and government agencies.
+CIEIF aims to help climate-intervention projects better understand their potential technical, environmental, economic, social, public-health, and safety impacts before and during field testing. It also places importance on the scalability and global relevance of supported innovations and encourages publication of field-test results through peer-reviewed journals or externally peer-reviewed reports.
+ About the Grant
+The Climate Intervention Environmental Impact Fund (CIEIF) Grant provides USD 75,000 to support proposed climate intervention field tests. The funding is specifically intended for Environmental Impact Assessment (EIA), predictive impact modelling, and/or engagement with potentially affected stakeholders, including local communities and government agencies.
+Applicants are expected to demonstrate the proposed field test’s technical readiness, environmental and social considerations, required government approvals, innovation and potential for globally relevant scalability. The application must include a proposed budget showing how the USD 75,000 will be used.
+ Grant Objective
+The grant is intended to support proposed climate intervention field tests, particularly activities related to:
+Environmental Impact Assessment (EIA)
+Predictive impact modeling
+Engagement with potentially impacted stakeholders
+Local community and government engagement
+Understanding technical, environmental, economic, social, public-health, and safety challenges
+The proposed application must focus on at least one of these three core areas: EIA, predictive impact modeling, or stakeholder engagement.
+ Eligible Project Focus
+The proposed field test should demonstrate:
+A clear climate-intervention concept
+Prior research indicating that the technology is ready for the proposed field test
+Potential for innovation and scalability
+A clear understanding of technical and environmental challenges
+Consideration of economic, social, public-health, and safety implications
+Relevant government permits and approvals
+Potential for scaling the innovation to a globally relevant level</t>
+        </is>
+      </c>
+      <c r="D21" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E21" s="1" t="inlineStr">
+        <is>
+          <t>Dec 1, 2026</t>
+        </is>
+      </c>
+      <c r="F21" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-cieif-grant-2026-climate-intervention-environmental-impact-fund-climate-intervention-environmental-impact-fund-opg-26-00155</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="95" customHeight="1">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for 6th Annual Seeding The Future Global Food System Challenge</t>
+        </is>
+      </c>
+      <c r="C22" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+We are one of the largest and most respected private organisations for development cooperation and humanitarian aid in Germany. As a politically and confessionally independent organisation, our value-oriented actions are always based on ethical principles. Our vision is clear: "Zero Hunger by 2030"
+ About the Opportunity:
+The Global Food System Challenge recognizes and supports breakthrough innovations that can spark transformations of our food systems, with a particular focus on addressing critical challenges in the Global South. It calls on scientists, engineers, innovators, entrepreneurs, and multidisciplinary teams from NGOs, non-profits, social enterprises, universities, research institutions, and small/emerging for-profit enterprises to submit game-changing innovations that transform food systems.
+ Innovation Focus Area (must benefit at least one, ideally more domains):
+Innovations leading to safe and nutritious food for a healthy diet
+Innovations leading to sustainable/regenerative practices keeping food systems within planetary boundaries (including food waste/loss reduction)
+Innovations leading to equitable access to food that is affordable, appealing, and trusted
+ Award Levels (three tiers, applicant selects which to apply for):
+Award Amount Number Available Requirement
+Seed Grant $25,000 each Up to 8 For high-potential ideas with prototype/initial proof of concept demonstrating feasibility; must benefit ≥1, ideally 2 domains
+Growth Grant $100,000 each Up to 3 For innovations proven "doable" with economic feasibility at scale and high-impact potential; must benefit ≥2, ideally 3 domains
+Seeding The Future Grand Prize $250,000 each Up to 2 For scalable, economically feasible, trusted innovations with major impact potential; must benefit ≥2, ideally 3 domains
+Eligibility:
+Non-profits/NGOs (any country)
+Academic/research institutions (any country)
+Early-stage or emerging for-profit companies/social enterprises (any country)
+Excludes entities from countries under comprehensive U.S./German sanctions (currently: Afghanistan, Belarus, Crimea, Cuba, Iran, Myanmar, North Korea, Russia, Sevastopol, Sudan, South Sudan, Syria, Kherson/Donetsk/Luhansk/Zaporizhzhia regions of Ukraine, Venezuela)
+Individuals are not eligible — teams of students/researchers may participate as part of an organization's submission
+For-profit applicants: must be early-stage/pre-Series A, financial assets not exceeding $10M
+ What Will NOT Be Funded:
+Projects harming food safety, sustainability, or unlikely to be accepted by end-users
+Funds supporting large for-profit entities' commercial R&amp;D/manufacturing/sales
+Non-scalable initiatives with limited long-term impact
+Large for-profit entities (post-Series A)
+Purely theoretical concepts with no experiments/proof of concept
+Political campaigns, capital campaigns, or lobbying
+Individuals with no organizational entity</t>
+        </is>
+      </c>
+      <c r="D22" s="1" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="E22" s="1" t="inlineStr">
+        <is>
+          <t>Jan 1, 2027</t>
+        </is>
+      </c>
+      <c r="F22" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-6th-annual-seeding-the-future-global-food-system-challenge-welthungerhilfe-opg-26-00180</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="95" customHeight="1">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for BES Training and Travel Grants</t>
         </is>
       </c>
-      <c r="C14" s="1" t="inlineStr">
+      <c r="C23" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are a global community of scientists shining a spotlight on the intricacy and value of our natural world, providing the evidence for better decisions. Our vision is for people and nature to thrive in a world that values ecology.
@@ -1097,17 +1611,17 @@
  Application Deadline (Round 2): Opens 30 April 2026, closes 17 May 2026</t>
         </is>
       </c>
-      <c r="D14" s="1" t="inlineStr">
+      <c r="D23" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E14" s="1" t="inlineStr">
+      <c r="E23" s="1" t="inlineStr">
         <is>
           <t>May 17, 2027</t>
         </is>
       </c>
-      <c r="F14" s="1" t="inlineStr">
+      <c r="F23" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-bes-training-and-travel-grants-british-ecological-society-opg-26-00181</t>
         </is>

</xml_diff>

<commit_message>
Auto update Combined.xlsx [Wed Oct  7 08:04:38 UTC 2026]
</commit_message>
<xml_diff>
--- a/output/Combined.xlsx
+++ b/output/Combined.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1220,10 +1220,42 @@
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
+          <t>RFPs Invited for Arts-Integrated National School Projects Arts Education from Government-aided and Non-profit Schools in India</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>No description available</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>Oct 30, 2026</t>
+        </is>
+      </c>
+      <c r="F17" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/rfps-invited-for-arts-integrated-national-school-projects-arts-education-from-government-aided-and-non-profit-schools-in-india-india-foundation-for-the-arts-rfp-26-00385</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="95" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
+        <is>
           <t>Applications Invited for CIFAR Global Scholars Program 20272029 Cohort</t>
         </is>
       </c>
-      <c r="C17" s="1" t="inlineStr">
+      <c r="C18" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 CIFAR is a Canadian-based globally influential research organization that convenes the world’s most brilliant people across disciplines to advance transformative knowledge and solve humanity’s biggest problems, together. By supporting long-term interdisciplinary collaboration, CIFAR provides researchers with an unparalleled environment of trust, transparency and knowledge sharing. Our time-tested model inspires new directions of inquiry, accelerates discovery and yields breakthroughs across borders and academic disciplines. Through knowledge mobilization, we are catalysts for change in industry, government and society. Through our 15 research programs and the Pan-Canadian AI Strategy, CIFAR convenes close to 400 of the world’s top researchers from 141 institutions in 20 countries. CIFAR is generously supported by the governments of Canada, Alberta and Québec, as well as foundations, individuals, corporations and Canadian and international partner organizations.
@@ -1267,34 +1299,34 @@
  Application Deadline: November 4, 2026, 12:00 PM EST</t>
         </is>
       </c>
-      <c r="D17" s="1" t="inlineStr">
+      <c r="D18" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E17" s="1" t="inlineStr">
+      <c r="E18" s="1" t="inlineStr">
         <is>
           <t>Nov 4, 2026</t>
         </is>
       </c>
-      <c r="F17" s="1" t="inlineStr">
+      <c r="F18" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cifar-global-scholars-program-20272029-cohort-cifar-canadian-institute-for-advanced-research-opg-26-00183</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="95" customHeight="1">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="inlineStr">
+    <row r="19" ht="95" customHeight="1">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for IWRS Teaching Innovation Award</t>
         </is>
       </c>
-      <c r="C18" s="1" t="inlineStr">
+      <c r="C19" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
@@ -1306,34 +1338,34 @@
 Two awards of $2,000 USD are available annually.</t>
         </is>
       </c>
-      <c r="D18" s="1" t="inlineStr">
+      <c r="D19" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E18" s="1" t="inlineStr">
+      <c r="E19" s="1" t="inlineStr">
         <is>
           <t>Nov 15, 2026</t>
         </is>
       </c>
-      <c r="F18" s="1" t="inlineStr">
+      <c r="F19" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="95" customHeight="1">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="inlineStr">
+    <row r="20" ht="95" customHeight="1">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for IWRS Teaching Innovation Award</t>
         </is>
       </c>
-      <c r="C19" s="1" t="inlineStr">
+      <c r="C20" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Insects are one of the most numerous and diverse animal groups on Earth.
@@ -1348,34 +1380,34 @@
 IWRS staff and Advisory Group members are not eligible to apply.</t>
         </is>
       </c>
-      <c r="D19" s="1" t="inlineStr">
+      <c r="D20" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E19" s="1" t="inlineStr">
+      <c r="E20" s="1" t="inlineStr">
         <is>
           <t>Nov 15, 2026</t>
         </is>
       </c>
-      <c r="F19" s="1" t="inlineStr">
+      <c r="F20" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00166</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="95" customHeight="1">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="inlineStr">
+    <row r="21" ht="95" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Medium-Size Grants Call for Proposals Global EbA Fund</t>
         </is>
       </c>
-      <c r="C20" s="1" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -1432,34 +1464,34 @@
 Applications submitted via online portal (link shared on the Medium-Size Grants webpage from Oct 12)</t>
         </is>
       </c>
-      <c r="D20" s="1" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E20" s="1" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>Nov 16, 2026</t>
         </is>
       </c>
-      <c r="F20" s="1" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-medium-size-grants-call-for-proposals-global-eba-fund-global-eba-fund-opg-26-00178</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="95" customHeight="1">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="inlineStr">
+    <row r="22" ht="95" customHeight="1">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIEIF Grant 2026 Climate Intervention Environmental Impact Fund</t>
         </is>
       </c>
-      <c r="C21" s="1" t="inlineStr">
+      <c r="C22" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Climate Intervention Environmental Impact Fund (CIEIF) is a philanthropic fund focused on supporting responsible climate intervention field tests. It provides grants for activities such as environmental impact assessment (EIA), predictive impact modelling, and engagement with potentially affected stakeholders, including local communities and government agencies.
@@ -1486,34 +1518,34 @@
 Potential for scaling the innovation to a globally relevant level</t>
         </is>
       </c>
-      <c r="D21" s="1" t="inlineStr">
+      <c r="D22" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E21" s="1" t="inlineStr">
+      <c r="E22" s="1" t="inlineStr">
         <is>
           <t>Dec 1, 2026</t>
         </is>
       </c>
-      <c r="F21" s="1" t="inlineStr">
+      <c r="F22" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cieif-grant-2026-climate-intervention-environmental-impact-fund-climate-intervention-environmental-impact-fund-opg-26-00155</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="95" customHeight="1">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="inlineStr">
+    <row r="23" ht="95" customHeight="1">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 6th Annual Seeding The Future Global Food System Challenge</t>
         </is>
       </c>
-      <c r="C22" s="1" t="inlineStr">
+      <c r="C23" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are one of the largest and most respected private organisations for development cooperation and humanitarian aid in Germany. As a politically and confessionally independent organisation, our value-oriented actions are always based on ethical principles. Our vision is clear: "Zero Hunger by 2030"
@@ -1545,34 +1577,34 @@
 Individuals with no organizational entity</t>
         </is>
       </c>
-      <c r="D22" s="1" t="inlineStr">
+      <c r="D23" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E22" s="1" t="inlineStr">
+      <c r="E23" s="1" t="inlineStr">
         <is>
           <t>Jan 1, 2027</t>
         </is>
       </c>
-      <c r="F22" s="1" t="inlineStr">
+      <c r="F23" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-6th-annual-seeding-the-future-global-food-system-challenge-welthungerhilfe-opg-26-00180</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="95" customHeight="1">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B23" s="1" t="inlineStr">
+    <row r="24" ht="95" customHeight="1">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for BES Training and Travel Grants</t>
         </is>
       </c>
-      <c r="C23" s="1" t="inlineStr">
+      <c r="C24" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are a global community of scientists shining a spotlight on the intricacy and value of our natural world, providing the evidence for better decisions. Our vision is for people and nature to thrive in a world that values ecology.
@@ -1611,17 +1643,17 @@
  Application Deadline (Round 2): Opens 30 April 2026, closes 17 May 2026</t>
         </is>
       </c>
-      <c r="D23" s="1" t="inlineStr">
+      <c r="D24" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E23" s="1" t="inlineStr">
+      <c r="E24" s="1" t="inlineStr">
         <is>
           <t>May 17, 2027</t>
         </is>
       </c>
-      <c r="F23" s="1" t="inlineStr">
+      <c r="F24" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-bes-training-and-travel-grants-british-ecological-society-opg-26-00181</t>
         </is>

</xml_diff>

<commit_message>
Auto update Combined.xlsx [Thu Oct  8 08:19:54 UTC 2026]
</commit_message>
<xml_diff>
--- a/output/Combined.xlsx
+++ b/output/Combined.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -527,61 +527,10 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>Applications Open Draper Richards Kaplan Foundation Funding for Social Enterprises</t>
+          <t>Apply for the ServiceNow Community Solar Fund</t>
         </is>
       </c>
       <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>About us
-Started in 2002, Draper Richards Kaplan Foundation (DRK) is a global venture philanthropy firm supporting early stage, high impact social enterprises. Borrowed from our venture capital legacy, DRK finds, funds, and supports exceptional leaders building innovative solutions to some of the world’s most challenging social and environmental problems. Since beginning this work nearly 25 years ago, DRK has invested in more than 270 organizations that have collectively impacted over 610 million lives to date.
-Draper Richards Kaplan Foundation accepts applications for funding year-round. Completing an application is the first step of our process and allows us to get to know you and your social enterprise so we can begin assessing your organization’s alignment with our funding thesis.
-To help make this process manageable and accessible, we have designed the application to be relatively simple and minimally burdensome. The online application should take about 30-60 minutes to complete. If you would like to save your progress and resume later, please be sure to check the box at the top of the online form to save your information.
-Please upload with your application a written executive summary, pitch deck, or business plan document addressing the following topics. Please feel free to reuse or repurpose existing materials if you feel that they would provide relevant information.
-Any additional materials (e.g., financials, impact reports, etc.) are welcome, but completely optional.
-Problem and Solution
-Please succinctly describe the mission and objectives of the organization.
-Please describe the social problem your organization addresses.
-Please describe the solution your organization provides.
-Impact
-Please explain how your organization solves (or contributes to solving) the social problem in a way that improves on existing efforts.
-Please explain how your solution supports an underserved population, including the benefits that population has seen from your pilot(s).
-Please explain how your approach is unique, including in comparison to other initiatives or organizations addressing the same problem if possible/relevant.
-Please describe the organization’s tangible results to date, detailing how you plan to measure organizational outcomes and success in the future.
-Scale
-Please explain how you plan to scale the organization over time.
-Please explain the main sources of earned income that your organization will use to sustain your work over time.
-Leader
-Please attach a standard resume/CV for the entrepreneur(s) and/or key leadership team members (e.g., CEO, COO, ED, etc.). Applications with text bios for entrepreneurs or members of the leadership team will not be considered.</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>Climate</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="inlineStr">
-        <is>
-          <t>Oct 10, 2026</t>
-        </is>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-open-draper-richards-kaplan-foundation-funding-for-social-enterprises-draper-richards-kaplan-foundation-opg-26-00188</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="95" customHeight="1">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>Apply for the ServiceNow Community Solar Fund</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund
 Apply by: 13 October, 2026
@@ -606,19 +555,51 @@
  Projects should include opportunities for ServiceNow employees to volunteer in the project activation or implementation.</t>
         </is>
       </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Oct 13, 2026</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/apply-for-the-servicenow-community-solar-fund-changex-opg-26-00186</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="95" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>EOI invited for Consultant Road Safety Expert / Technical</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>No description available</t>
+        </is>
+      </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>Governance</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>Oct 13, 2026</t>
+          <t>Oct 15, 2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/grants/apply-for-the-servicenow-community-solar-fund-changex-opg-26-00186</t>
+          <t>https://onepurpos.in/openings/rfps/eoi-invited-for-consultant-road-safety-expert-technical-bharatcares-rfp-26-00381</t>
         </is>
       </c>
     </row>
@@ -630,27 +611,46 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>EOI invited for Consultant Road Safety Expert / Technical</t>
+          <t>Applications Invited for Research Grants on Indigenous Research on Climate Change</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>No description available</t>
+          <t>About the Organization
+Center for Indigenous Peoples' Research and Development (CIPRED) has been carrying out Indigenous-led research, documentation, publication, and evidence-based policy advocacy for securing Indigenous Peoples' inherent rights to protect, promote, recognize, and continue traditional knowledge, skills, cultural values, and customary self-governance systems that have been contributing for sustaining traditional livelihoods (food and economy), natural resource management, climate change resilience, biodiversity, and sustainable development. CIPRED has been involved in the layers of activities at community, national and international levels in partnership and collaboration with Indigenous Peoples' Organization (IPOs), relevant agencies including Government, Bilateral and Multilateral agencies, research institutions, Universities, and Local Community Organization.
+ Purpose: 
+Concerning the ongoing severe impacts of climate change that we have been experiencing every day particularly the recent floods in Nepal, this call aims to encourage youth and students to carry out their research and documentation on the theme of climate change in relation to Indigenous Peoples in South Asia.
+ Eligibility: 
+The grant is open for youth and women researchers and students below 35 years with their education and research backgrounds on Indigenous Peoples.
+ Scope of the study/research: 
+The concept note is expected on the theme of climate change in relation to Indigenous Peoples on the following thematic topics:
+Food and Economy 
+Culture and Heritage 
+Customary Governance and Tenure Rights 
+Conservation and Biodiversity 
+Language and Education
+ This research will be expected to be completed by December 2026
+ Concept Notes: 
+The concept note of the study should cover the clear rational and objective of the study and indicate where the study will be carried out and how the researchers would support to the community they are working with.
+ Funding Information: 
+The study is awarded Rs. 100,000 (One Lakh Nepali Rupees Only) for each aplicant. Applicants can be individual or in group. However, we encourage to apply in group. Note: We are expecting to receive applications from South Asia and selecting 10 best concept notes who meet the objectives of this call.
+ Deadline: 
+The deadline for the submission of the concept note is on 16 October 2026. Only shortlisted candidates will be informed in advance for their presentation.</t>
         </is>
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Governance</t>
         </is>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>Oct 15, 2026</t>
+          <t>Oct 16, 2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/rfps/eoi-invited-for-consultant-road-safety-expert-technical-bharatcares-rfp-26-00381</t>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-research-grants-on-indigenous-research-on-climate-change-center-for-indigenous-peoples-research-and-development-opg-26-00197</t>
         </is>
       </c>
     </row>
@@ -844,60 +844,10 @@
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
-          <t>Applications Invited for D-Prize Global Competition Seed Funding for New Poverty-Solution Distribution Organizations</t>
+          <t>Applications Invited for Adaptive Control Frameworks to Unlock Full-Scale BNR Potential Water Research Foundation WRF</t>
         </is>
       </c>
       <c r="C11" s="1" t="inlineStr">
-        <is>
-          <t>About the Grant:
-D-Prize seeds new organizations that distribute proven poverty solutions at the "last mile," with the aim of scaling impact. Applicants select from a range of evidence-based interventions (health, agriculture, education, water, safety, transparency, and more) and propose how they would launch or grow an organization to distribute that intervention. Top entrepreneurs receive up to $20,000 in seed funding to run a pilot and build an organization capable of scaling to reach thousands, even millions of people.
- Intervention Areas (sample — 20+ tracks available):
-Health: Childhood Diarrhea Treatment, DMPA-SC (contraceptive) initiatives, Reading Glasses, Kangaroo Care, Oxygen access, Maternal Health, Child Immunization, Prevention of Mother-to-Child HIV Transmission, Patient Identification
-Education: Teaching at the Right Level, ConnectEd Phone-based Tutoring, Sugar Daddy Awareness
-Agriculture: Post-Harvest Support, Quality Inputs, Water Filters, custom agriculture proposals
-Livelihoods/Governance: Poverty Graduation, Government Transparency, Road Safety, Childcare
-"Propose Your Own": pitch a distribution model for any credible, evidence-based poverty intervention not listed
- Eligibility:
-New organizations only — most awardees are first-time entrepreneurs who have not yet launched or raised outside funding
-Applicants from low- and middle-income countries especially encouraged
-Organizations with more than 18 months of full-time operations or more than $30,000 USD already raised are typically not supported
-Existing organizations considered only if their core focus is distributing an existing, evidence-based poverty intervention
- Qualification: Not specified (open to entrepreneurs of any background; evaluated on quality of distribution concept and execution ability)
- Experience Bracket: Early-stage/first-time entrepreneurs preferred; not aimed at established organizations
- Application Deadline:
-Early Submission: 25 October 2026, midnight PT
-Regular Submission: 15 November 2026, midnight PT
-Extension Deadline: 6 December 2026, midnight PT (extension registration required)</t>
-        </is>
-      </c>
-      <c r="D11" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E11" s="1" t="inlineStr">
-        <is>
-          <t>Oct 25, 2026</t>
-        </is>
-      </c>
-      <c r="F11" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-d-prize-global-competition-seed-funding-for-new-poverty-solution-distribution-organizations-d-prize-opg-26-00191</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="95" customHeight="1">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Adaptive Control Frameworks to Unlock Full-Scale BNR Potential Water Research Foundation WRF</t>
-        </is>
-      </c>
-      <c r="C12" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Water Research Foundation (WRF) is the leading research organization advancing the science of all water to meet the evolving needs of its subscribers and the water sector. WRF is a nonprofit, charitable and educational organization which funds, manages, and publishes research on the technology, operation, and management of drinking water, wastewater, reuse, and stormwater collection, treatment and supply systems—all in pursuit of ensuring water quality and improving water services to the public.
@@ -938,34 +888,34 @@
 Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
         </is>
       </c>
-      <c r="D12" s="1" t="inlineStr">
+      <c r="D11" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E12" s="1" t="inlineStr">
+      <c r="E11" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F12" s="1" t="inlineStr">
+      <c r="F11" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-adaptive-control-frameworks-to-unlock-full-scale-bnr-potential-water-research-foundation-wrf-the-water-research-foundation-wrf-opg-26-00187</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="95" customHeight="1">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B13" s="1" t="inlineStr">
+    <row r="12" ht="95" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Comparison of PFAS Contributions to Agricultural Systems</t>
         </is>
       </c>
-      <c r="C13" s="1" t="inlineStr">
+      <c r="C12" s="1" t="inlineStr">
         <is>
           <t>Project Objectives:
 Report per- and polyfluoroalkyl substance (PFAS) concentrations from a variety of agricultural inputs — animal manures, fertilizers, pesticides, composts, soil amendments, seed coatings, and biosolids-based products
@@ -1001,34 +951,34 @@
  Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00) — same deadline as the other two WRF grants</t>
         </is>
       </c>
-      <c r="D13" s="1" t="inlineStr">
+      <c r="D12" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E13" s="1" t="inlineStr">
+      <c r="E12" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F13" s="1" t="inlineStr">
+      <c r="F12" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-comparison-of-pfas-contributions-to-agricultural-systems-the-water-research-foundation-wrf-opg-26-00190</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="95" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="inlineStr">
+    <row r="13" ht="95" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 8th Call for Proposals Small-Size Grants Global EbA Fund</t>
         </is>
       </c>
-      <c r="C14" s="1" t="inlineStr">
+      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -1091,34 +1041,34 @@
 Only successful applicants will be contacted; no individual feedback provided to unsuccessful applicants</t>
         </is>
       </c>
-      <c r="D14" s="1" t="inlineStr">
+      <c r="D13" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E14" s="1" t="inlineStr">
+      <c r="E13" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F14" s="1" t="inlineStr">
+      <c r="F13" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-8th-call-for-proposals-small-size-grants-global-eba-fund-global-eba-fund-opg-26-00177</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="95" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="inlineStr">
+    <row r="14" ht="95" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Crossing the Divide Best Practices for Addressing Local and Privately-Owned Lateral Sewer Issues RFP 5419</t>
         </is>
       </c>
-      <c r="C15" s="1" t="inlineStr">
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>Project Objective:
 To provide water resource recovery facilities (WRRFs) and collection system operators with an interactive manual of practice for implementing inflow and infiltration (I&amp;I) and obstruction management programs, focused on municipal and privately owned lateral sewers in complex legal, regulatory, and multi-jurisdictional environments.
@@ -1156,6 +1106,38 @@
  Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
         </is>
       </c>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>Oct 26, 2026</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-crossing-the-divide-best-practices-for-addressing-local-and-privately-owned-lateral-sewer-issues-rfp-5419-the-water-research-foundation-wrf-opg-26-00189</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="95" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>RFPs Invited for Arts-Integrated National School Projects Arts Education from Government-aided and Non-profit Schools in India</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>No description available</t>
+        </is>
+      </c>
       <c r="D15" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
@@ -1163,12 +1145,12 @@
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>Oct 26, 2026</t>
+          <t>Oct 30, 2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-crossing-the-divide-best-practices-for-addressing-local-and-privately-owned-lateral-sewer-issues-rfp-5419-the-water-research-foundation-wrf-opg-26-00189</t>
+          <t>https://onepurpos.in/openings/rfps/rfps-invited-for-arts-integrated-national-school-projects-arts-education-from-government-aided-and-non-profit-schools-in-india-india-foundation-for-the-arts-rfp-26-00385</t>
         </is>
       </c>
     </row>
@@ -1180,82 +1162,10 @@
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
-          <t>Applications Invited for Whitley Award 2027</t>
+          <t>Applications Invited for CIFAR Global Scholars Program 20272029 Cohort</t>
         </is>
       </c>
       <c r="C16" s="1" t="inlineStr">
-        <is>
-          <t>About the Grant: 
-An annual grant by the Whitley Fund for Nature (WFN) recognising grassroots conservation leaders in the Global South, providing funding to support and scale up proven, science-based solutions that deliver lasting impact for both people and nature.
- About the Award 
-Whitley Awards support grassroots conservation leaders in the Global South. Through funding, training and profile, they help conservationists scale up effective projects that are founded in science and carried out with communities. Whitley Awards are for dynamic, mid-career conservationists who are leading vital conservation projects.
- Grant Amount: £50,000 in project funding over one year
- Eligibility
-Winners are nationals of the country in which they are working, seeking to scale up proven work that is embedded in the local community and would benefit from further funding, a profile boost, and international support.
-Projects must involve communities at the grassroots level and deliver practical action that is founded on science.
-You do not need to be invited or nominated to apply.</t>
-        </is>
-      </c>
-      <c r="D16" s="1" t="inlineStr">
-        <is>
-          <t>Learning</t>
-        </is>
-      </c>
-      <c r="E16" s="1" t="inlineStr">
-        <is>
-          <t>Oct 30, 2026</t>
-        </is>
-      </c>
-      <c r="F16" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-whitley-award-2027-whitley-fund-for-nature-wfn-opg-26-00153</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="95" customHeight="1">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B17" s="1" t="inlineStr">
-        <is>
-          <t>RFPs Invited for Arts-Integrated National School Projects Arts Education from Government-aided and Non-profit Schools in India</t>
-        </is>
-      </c>
-      <c r="C17" s="1" t="inlineStr">
-        <is>
-          <t>No description available</t>
-        </is>
-      </c>
-      <c r="D17" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E17" s="1" t="inlineStr">
-        <is>
-          <t>Oct 30, 2026</t>
-        </is>
-      </c>
-      <c r="F17" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/rfps-invited-for-arts-integrated-national-school-projects-arts-education-from-government-aided-and-non-profit-schools-in-india-india-foundation-for-the-arts-rfp-26-00385</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="95" customHeight="1">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for CIFAR Global Scholars Program 20272029 Cohort</t>
-        </is>
-      </c>
-      <c r="C18" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 CIFAR is a Canadian-based globally influential research organization that convenes the world’s most brilliant people across disciplines to advance transformative knowledge and solve humanity’s biggest problems, together. By supporting long-term interdisciplinary collaboration, CIFAR provides researchers with an unparalleled environment of trust, transparency and knowledge sharing. Our time-tested model inspires new directions of inquiry, accelerates discovery and yields breakthroughs across borders and academic disciplines. Through knowledge mobilization, we are catalysts for change in industry, government and society. Through our 15 research programs and the Pan-Canadian AI Strategy, CIFAR convenes close to 400 of the world’s top researchers from 141 institutions in 20 countries. CIFAR is generously supported by the governments of Canada, Alberta and Québec, as well as foundations, individuals, corporations and Canadian and international partner organizations.
@@ -1299,34 +1209,89 @@
  Application Deadline: November 4, 2026, 12:00 PM EST</t>
         </is>
       </c>
-      <c r="D18" s="1" t="inlineStr">
+      <c r="D16" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E18" s="1" t="inlineStr">
+      <c r="E16" s="1" t="inlineStr">
         <is>
           <t>Nov 4, 2026</t>
         </is>
       </c>
-      <c r="F18" s="1" t="inlineStr">
+      <c r="F16" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cifar-global-scholars-program-20272029-cohort-cifar-canadian-institute-for-advanced-research-opg-26-00183</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="95" customHeight="1">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="inlineStr">
+    <row r="17" ht="95" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Regular Grant Programme 2026-27</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>About the Organization
+World Cancer Research Fund examines how diet, weight and physical activity affect your risk of developing and surviving cancer. As part of an international network of charities, we have been funding life-saving research, influencing global public health policy and educating the public since 1982.
+ About the Grant
+The Regular Grant Programme supports innovative and original research into the role of diet, nutrition, body composition and physical activity in cancer prevention or cancer survivorship. For the 2026-27 call, sleep is also included as a primary exposure. From autumn 2026, WCRF International manages grants on behalf of the whole WCRF network: WCRF UK, Wereld Kanker Onderzoek Fonds (Netherlands) and the American Institute for Cancer Research (US).
+ Grant types
+  Investigator-initiated grants Pilot and feasibility grants
+Funding Up to £500,000 Up to £60,000
+Duration Up to 4 years Up to 2 years
+Eligible organisations Anywhere in the world Anywhere in the world
+Eligible applicants Lead applicant must hold a research position at the host institution for the whole project Same
+ Research priority areas (2026-27)
+Applications must focus on at least one of these six areas. They may span more than one if scientifically justified, and the main alignment must be clear. Alignment with a priority area does not replace the usual requirements for scientific quality, fit with WCRF's remit, feasibility and impact.
+Integrative oncology: diet, physical activity, body composition, sleep, prehabilitation and other supportive-care interventions alongside conventional treatment, in childhood and adulthood. Outcomes include treatment tolerance and toxicity, quality of life, physical function, symptom control, recurrence and longer-term health. Loosely defined complementary therapies without a clear link to WCRF's remit or a strong scientific rationale are out of scope.
+Lifestyle and weight-loss medications: how diet, physical activity and behavioural support combine with weight-loss medications (including GLP-1-related medicines) across prevention, treatment and survivorship. This covers cancer-specific benefits and risks, the timing, duration and discontinuation of medication, separating drug effects from weight loss and lifestyle effects, and inequalities in access.
+Early-onset cancers: explaining rising incidence of cancers diagnosed at 18-50 years, and whether their modifiable risk factors and biology differ from later-life cancers.
+Early-life exposures: how modifiable exposures from preconception through adolescence affect later cancer risk. Studies should define the exposure precisely, use robust methods for familial and socioeconomic confounding, and where possible combine epidemiology with biomarker or mechanistic evidence.
+Ingested contaminants: contaminants in food and drinking water (endocrine-disrupting chemicals, pesticides, heavy metals, persistent organic pollutants, micro- and nano-plastics) with a clear, evidence-based rationale for cancer relevance. Studies should consider cumulative exposure and mixtures, and credible biological or causal pathways.
+Ultra-processed foods: whether and how ultra-processed food affects cancer risk and survivorship, going beyond broad classification systems to specific processing characteristics, additives or food structure. Exposure data must reflect contemporary products and consumption. Applications that don't account for changes in food formulation and consumption over time will not be considered.
+ Key dates
+Step Date
+Letter of Intent (LOI) stage opens 5 October 2026, 9:00 AM BST (UK time)
+LOI stage closes 13 November 2026, 5:00 PM GMT (UK time) (= 10:30 PM IST)
+LOI outcomes communicated February 2027
+Final funding decisions (after Board approval) End of September 2027</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>Nov 13, 2026</t>
+        </is>
+      </c>
+      <c r="F17" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-regular-grant-programme-2026-27-world-cancer-research-fund-opg-26-00196</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="95" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for IWRS Teaching Innovation Award</t>
         </is>
       </c>
-      <c r="C19" s="1" t="inlineStr">
+      <c r="C18" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
@@ -1338,34 +1303,34 @@
 Two awards of $2,000 USD are available annually.</t>
         </is>
       </c>
-      <c r="D19" s="1" t="inlineStr">
+      <c r="D18" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E19" s="1" t="inlineStr">
+      <c r="E18" s="1" t="inlineStr">
         <is>
           <t>Nov 15, 2026</t>
         </is>
       </c>
-      <c r="F19" s="1" t="inlineStr">
+      <c r="F18" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="95" customHeight="1">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="inlineStr">
+    <row r="19" ht="95" customHeight="1">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for IWRS Teaching Innovation Award</t>
         </is>
       </c>
-      <c r="C20" s="1" t="inlineStr">
+      <c r="C19" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Insects are one of the most numerous and diverse animal groups on Earth.
@@ -1380,34 +1345,34 @@
 IWRS staff and Advisory Group members are not eligible to apply.</t>
         </is>
       </c>
-      <c r="D20" s="1" t="inlineStr">
+      <c r="D19" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E20" s="1" t="inlineStr">
+      <c r="E19" s="1" t="inlineStr">
         <is>
           <t>Nov 15, 2026</t>
         </is>
       </c>
-      <c r="F20" s="1" t="inlineStr">
+      <c r="F19" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00166</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="95" customHeight="1">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="inlineStr">
+    <row r="20" ht="95" customHeight="1">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Medium-Size Grants Call for Proposals Global EbA Fund</t>
         </is>
       </c>
-      <c r="C21" s="1" t="inlineStr">
+      <c r="C20" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -1464,34 +1429,34 @@
 Applications submitted via online portal (link shared on the Medium-Size Grants webpage from Oct 12)</t>
         </is>
       </c>
-      <c r="D21" s="1" t="inlineStr">
+      <c r="D20" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E21" s="1" t="inlineStr">
+      <c r="E20" s="1" t="inlineStr">
         <is>
           <t>Nov 16, 2026</t>
         </is>
       </c>
-      <c r="F21" s="1" t="inlineStr">
+      <c r="F20" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-medium-size-grants-call-for-proposals-global-eba-fund-global-eba-fund-opg-26-00178</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="95" customHeight="1">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="inlineStr">
+    <row r="21" ht="95" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for CIEIF Grant 2026 Climate Intervention Environmental Impact Fund</t>
         </is>
       </c>
-      <c r="C22" s="1" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Climate Intervention Environmental Impact Fund (CIEIF) is a philanthropic fund focused on supporting responsible climate intervention field tests. It provides grants for activities such as environmental impact assessment (EIA), predictive impact modelling, and engagement with potentially affected stakeholders, including local communities and government agencies.
@@ -1518,34 +1483,34 @@
 Potential for scaling the innovation to a globally relevant level</t>
         </is>
       </c>
-      <c r="D22" s="1" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E22" s="1" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>Dec 1, 2026</t>
         </is>
       </c>
-      <c r="F22" s="1" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cieif-grant-2026-climate-intervention-environmental-impact-fund-climate-intervention-environmental-impact-fund-opg-26-00155</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="95" customHeight="1">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B23" s="1" t="inlineStr">
+    <row r="22" ht="95" customHeight="1">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 6th Annual Seeding The Future Global Food System Challenge</t>
         </is>
       </c>
-      <c r="C23" s="1" t="inlineStr">
+      <c r="C22" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are one of the largest and most respected private organisations for development cooperation and humanitarian aid in Germany. As a politically and confessionally independent organisation, our value-oriented actions are always based on ethical principles. Our vision is clear: "Zero Hunger by 2030"
@@ -1577,34 +1542,34 @@
 Individuals with no organizational entity</t>
         </is>
       </c>
-      <c r="D23" s="1" t="inlineStr">
+      <c r="D22" s="1" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="E23" s="1" t="inlineStr">
+      <c r="E22" s="1" t="inlineStr">
         <is>
           <t>Jan 1, 2027</t>
         </is>
       </c>
-      <c r="F23" s="1" t="inlineStr">
+      <c r="F22" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-6th-annual-seeding-the-future-global-food-system-challenge-welthungerhilfe-opg-26-00180</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="95" customHeight="1">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B24" s="1" t="inlineStr">
+    <row r="23" ht="95" customHeight="1">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for BES Training and Travel Grants</t>
         </is>
       </c>
-      <c r="C24" s="1" t="inlineStr">
+      <c r="C23" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 We are a global community of scientists shining a spotlight on the intricacy and value of our natural world, providing the evidence for better decisions. Our vision is for people and nature to thrive in a world that values ecology.
@@ -1643,17 +1608,17 @@
  Application Deadline (Round 2): Opens 30 April 2026, closes 17 May 2026</t>
         </is>
       </c>
-      <c r="D24" s="1" t="inlineStr">
+      <c r="D23" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E24" s="1" t="inlineStr">
+      <c r="E23" s="1" t="inlineStr">
         <is>
           <t>May 17, 2027</t>
         </is>
       </c>
-      <c r="F24" s="1" t="inlineStr">
+      <c r="F23" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-bes-training-and-travel-grants-british-ecological-society-opg-26-00181</t>
         </is>

</xml_diff>

<commit_message>
Auto update Combined.xlsx [Fri Oct  9 08:21:26 UTC 2026]
</commit_message>
<xml_diff>
--- a/output/Combined.xlsx
+++ b/output/Combined.xlsx
@@ -495,42 +495,10 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>ToR - Catalyse Tech Reproductive Maternal Newborn &amp; Child Health</t>
+          <t>Apply for the ServiceNow Community Solar Fund</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t>No description available</t>
-        </is>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>Safety</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>Oct 10, 2026</t>
-        </is>
-      </c>
-      <c r="F3" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/rfps/tor-catalyse-tech-reproductive-maternal-newborn-and-child-health-selco-foundation-rfp-26-00379</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="95" customHeight="1">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>Apply for the ServiceNow Community Solar Fund</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>Apply for the ServiceNow Community Solar Fund
 Apply by: 13 October, 2026
@@ -555,19 +523,51 @@
  Projects should include opportunities for ServiceNow employees to volunteer in the project activation or implementation.</t>
         </is>
       </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Oct 13, 2026</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/apply-for-the-servicenow-community-solar-fund-changex-opg-26-00186</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="95" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>EOI for Mobile Medical Health Unit MMHU Vehicle on Rental Basis Jorhat District Assam</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>No description available</t>
+        </is>
+      </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>Governance</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>Oct 13, 2026</t>
+          <t>Oct 15, 2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/grants/apply-for-the-servicenow-community-solar-fund-changex-opg-26-00186</t>
+          <t>https://onepurpos.in/openings/rfps/eoi-for-mobile-medical-health-unit-mmhu-vehicle-on-rental-basis-jorhat-district-assam-bharatcares-rfp-26-00386</t>
         </is>
       </c>
     </row>
@@ -662,7 +662,7 @@
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>Application Invited For Partnering with Local organizations for Screening and Early care awardees</t>
+          <t>Application Invited For PPHF Pulse Fund - Partnering with Local organizations for Screening and Early care</t>
         </is>
       </c>
       <c r="C7" s="1" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/grants/application-invited-for-partnering-with-local-organizations-for-screening-and-early-care-awardees-people-to-people-health-foundation-opg-26-00195</t>
+          <t>https://onepurpos.in/openings/grants/application-invited-for-pphf-pulse-fund-partnering-with-local-organizations-for-screening-and-early-care-people-to-people-health-foundation-opg-26-00195</t>
         </is>
       </c>
     </row>
@@ -844,10 +844,125 @@
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
+          <t>Applications Invited for D-Prize Global Competition Seed Funding for New Poverty-Solution Distribution Organizations</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>About the Grant:
+D-Prize seeds new organizations that distribute proven poverty solutions at the "last mile," with the aim of scaling impact. Applicants select from a range of evidence-based interventions (health, agriculture, education, water, safety, transparency, and more) and propose how they would launch or grow an organization to distribute that intervention. Top entrepreneurs receive up to $20,000 in seed funding to run a pilot and build an organization capable of scaling to reach thousands, even millions of people.
+ Intervention Areas (sample — 20+ tracks available):
+Health: Childhood Diarrhea Treatment, DMPA-SC (contraceptive) initiatives, Reading Glasses, Kangaroo Care, Oxygen access, Maternal Health, Child Immunization, Prevention of Mother-to-Child HIV Transmission, Patient Identification
+Education: Teaching at the Right Level, ConnectEd Phone-based Tutoring, Sugar Daddy Awareness
+Agriculture: Post-Harvest Support, Quality Inputs, Water Filters, custom agriculture proposals
+Livelihoods/Governance: Poverty Graduation, Government Transparency, Road Safety, Childcare
+"Propose Your Own": pitch a distribution model for any credible, evidence-based poverty intervention not listed
+ Eligibility:
+New organizations only — most awardees are first-time entrepreneurs who have not yet launched or raised outside funding
+Applicants from low- and middle-income countries especially encouraged
+Organizations with more than 18 months of full-time operations or more than $30,000 USD already raised are typically not supported
+Existing organizations considered only if their core focus is distributing an existing, evidence-based poverty intervention
+ Qualification: Not specified (open to entrepreneurs of any background; evaluated on quality of distribution concept and execution ability)
+ Experience Bracket: Early-stage/first-time entrepreneurs preferred; not aimed at established organizations
+ Application Deadline:
+Early Submission: 25 October 2026, midnight PT
+Regular Submission: 15 November 2026, midnight PT
+Extension Deadline: 6 December 2026, midnight PT (extension registration required)</t>
+        </is>
+      </c>
+      <c r="D11" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>Oct 25, 2026</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-d-prize-global-competition-seed-funding-for-new-poverty-solution-distribution-organizations-d-prize-opg-26-00191</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="95" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Crossing the Divide Best Practices for Addressing Local and Privately-Owned Lateral Sewer Issues RFP 5419</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>Project Objective:
+To provide water resource recovery facilities (WRRFs) and collection system operators with an interactive manual of practice for implementing inflow and infiltration (I&amp;I) and obstruction management programs, focused on municipal and privately owned lateral sewers in complex legal, regulatory, and multi-jurisdictional environments.
+ Background/Rationale:
+Wastewater utilities face continuing challenges providing cost-effective sewer services amid rising demand, urban redevelopment, and performance disruptors (root intrusion, pipe degradation, blockages). I&amp;I and obstruction management remain persistent, costly problems without a consolidated resource to guide program design. During wet weather, peak I&amp;I flows can increase influent flows 3–5x average. Studies suggest up to 80% of I&amp;I originates on private property, and root intrusions cause over 50% of sewer blockages globally. Program effectiveness varies widely depending on statutory authority, multi-jurisdictional overlap, enforcement mechanisms, and participant willingness.
+ Central Research Questions:
+What I&amp;I and obstruction management practices are utilities using today, and how do they vary by jurisdictional/regulatory/infrastructure/environmental conditions?
+Which factors most influence successful implementation, and what barriers commonly derail programs?
+What measurable benefits (cost avoidance, capacity recovery, reduced spill risk, improved regulatory standing) have utilities realized from successful programs?
+This project extends WRF's ongoing "State-of-Practice Manual for Inflow and Infiltration Detection and Mitigation at Street and Private Lateral Levels" (Project 5365) into I&amp;I source control and obstruction management specifically.
+ Research Approach (4 Tasks):
+Literature and Regulatory Review — Comprehensive review of legal authorities/regulations in the US and comparable international jurisdictions; catalog program elements, enforcement mechanisms, incentive structures, and legal/jurisdictional barriers
+Utility Survey and Case Study Development — Broad survey across utility size/geography/system type; select at least 5 diverse in-depth case studies with quantitative results (I&amp;I reduction %, reduced bypass pumping, reduced basement backups, cost savings, recovered capacity, reduced blockage-related spills/service calls)
+Utility Workshop — At least one invitation-only workshop with utility representatives to present survey findings and gather structured feedback on draft guidance content
+Interactive Manual of Practice — Development of a decision-support tool/web-based application/interactive PDF enabling utilities to select effective I&amp;I/obstruction program elements based on their statutory authority, jurisdictional complexity, and enforcement mechanisms
+ Expected Deliverables:
+Research report (using WRF's Research Report Template) including literature/regulatory review
+Interactive manual of practice (following Technology Deliverables Guidance)
+In-depth utility survey, state-of-the-practice report, and at least 5 standalone case studies with quantitative results
+Summary documentation of the utility workshop, including feedback and how it was incorporated
+ Project Duration: 24 months from contract start date (No-Cost Extension Policy caps extensions at 9 months beyond original schedule)
+ Eligibility to Submit:
+Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible as named participants. Not open to individuals (same institutional-applicant structure as RFP 5424).
+ Budget/Funding:
+Maximum WRF funding: $250,000
+Applicant must contribute at least 33% of the project award as additional resources (cost share, applicant in-kind, or third-party in-kind per 2 CFR Part 200.306)
+Proposals not meeting the 33% minimum match will not be accepted
+ Proposal Evaluation Criteria:
+Understanding the Problem and Responsiveness to RFP: 20 points
+Technical and Scientific Merit: 30 points
+Qualifications, Capabilities, and Management: 20 points
+Communication Plan, Deliverables, and Applicability: 15 points
+Budget and Schedule: 15 points
+ Compliance Standards: OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
+ Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>Oct 26, 2026</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-crossing-the-divide-best-practices-for-addressing-local-and-privately-owned-lateral-sewer-issues-rfp-5419-the-water-research-foundation-wrf-opg-26-00189</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="95" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
           <t>Applications Invited for Adaptive Control Frameworks to Unlock Full-Scale BNR Potential Water Research Foundation WRF</t>
         </is>
       </c>
-      <c r="C11" s="1" t="inlineStr">
+      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Water Research Foundation (WRF) is the leading research organization advancing the science of all water to meet the evolving needs of its subscribers and the water sector. WRF is a nonprofit, charitable and educational organization which funds, manages, and publishes research on the technology, operation, and management of drinking water, wastewater, reuse, and stormwater collection, treatment and supply systems—all in pursuit of ensuring water quality and improving water services to the public.
@@ -888,97 +1003,34 @@
 Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
         </is>
       </c>
-      <c r="D11" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E11" s="1" t="inlineStr">
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F11" s="1" t="inlineStr">
+      <c r="F13" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-adaptive-control-frameworks-to-unlock-full-scale-bnr-potential-water-research-foundation-wrf-the-water-research-foundation-wrf-opg-26-00187</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="95" customHeight="1">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Comparison of PFAS Contributions to Agricultural Systems</t>
-        </is>
-      </c>
-      <c r="C12" s="1" t="inlineStr">
-        <is>
-          <t>Project Objectives:
-Report per- and polyfluoroalkyl substance (PFAS) concentrations from a variety of agricultural inputs — animal manures, fertilizers, pesticides, composts, soil amendments, seed coatings, and biosolids-based products
-Compare the impact of various agricultural inputs on PFAS concentration in the soil profile over varying timeframes
-Evaluate the fate and transport of different inputs to PFAS contributions in agricultural systems at field-scale
-Determine relative contributions from biosolids-based products vs. other inputs to help develop/prioritize risk management strategies
- Background/Rationale:
-Growing concern exists over human exposure to PFAS through biosolids land application on agricultural systems, with regulatory bans on biosolids land application enacted or proposed in at least 12 U.S. states. Utilities relying on land application for biosolids management are scrambling for alternative disposal pathways. The U.S. EPA's 2026 draft guidance noted its earlier 2025 draft risk assessment of PFOA/PFOS-contaminated sewage sludge lacked important contextual information (e.g., a national survey of PFOA/PFOS concentrations). Risk assessments have focused primarily on biosolids, with less attention to PFAS contributions from other sources — manures, compost, fertilizers, pesticides, seed coatings, irrigation water, farming practices, and atmospheric deposition. A Minnesota Pollution Control Agency review found 12 inert pesticide ingredients classified as PFAS. This project aims to improve understanding of PFAS risks from the wider range of agricultural inputs to support strategic resource allocation and inform policy amid surging fertilizer prices and shifts toward local circular resources.
- Research Approach:
-Develop a baseline of knowledge on PFAS in biosolids and non-biosolids agricultural inputs via literature review, analytical methods evaluation, and examination of manufacturing/processing pathways; identify data gaps and uncertainties
-Measure/report compound-specific PFAS concentrations and profiles in agricultural inputs using standardized methods, including precursor characteristics for source attribution where possible
-Characterize PFAS contributions via literature review, data analysis, and field sampling — comparing soil profile/plant tissue composition between fields with non-biosolids inputs vs. biosolids-applied systems; study should test hypotheses on PFAS sources, transformation, retention, and mobility
-Optional additional focus areas: influence of soil/hydrologic/hydrochemistry conditions on PFAS behavior; degradation/transformation pathways; relative PFAS contributions across product lifecycle stages (manufacturing, bagging, delivery, etc.)
-Research approach should be hypothesis-driven, detailing specific end-user needs, and proposers are encouraged to leverage existing projects on PFAS plant uptake/fate/transport.
- Expected Deliverables:
-Research report (WRF's Research Report Template) including: literature review, PFAS analysis of select products, risk management implications/prioritization recommendations, agriculture end-use guidance
-A webcast or workshop to share findings
-Optional additional deliverables: relative risk framework (mass input/fate/exposure/risk), decision support guide for farmers/regulators/utilities, plain language fact sheet, comparative PFAS mass input tool (spreadsheet/calculator)
- Project Duration: 36 months from contract start date (longer than the other two WRF grants above, which were 24 months)
- Eligibility to Submit:
-Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible. Not open to individuals (same structure as the two prior WRF grants).
- Budget/Funding:
-Maximum WRF funding: $400,000 (the largest of the three WRF grants shared so far)
-Applicant must contribute at least 33% of the project award as additional resources (cost share, applicant in-kind, or third-party in-kind per 2 CFR Part 200.306)
-Proposals not meeting the 33% minimum match will not be accepted
- Proposal Evaluation Criteria:
-Understanding the Problem and Responsiveness to RFP: 20 points
-Technical and Scientific Merit: 30 points
-Qualifications, Capabilities, and Management: 20 points
-Communication Plan, Deliverables, and Applicability: 15 points
-Budget and Schedule: 15 points
- Compliance Standards: OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
- Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00) — same deadline as the other two WRF grants</t>
-        </is>
-      </c>
-      <c r="D12" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E12" s="1" t="inlineStr">
-        <is>
-          <t>Oct 26, 2026</t>
-        </is>
-      </c>
-      <c r="F12" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-comparison-of-pfas-contributions-to-agricultural-systems-the-water-research-foundation-wrf-opg-26-00190</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="95" customHeight="1">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B13" s="1" t="inlineStr">
+    <row r="14" ht="95" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for 8th Call for Proposals Small-Size Grants Global EbA Fund</t>
         </is>
       </c>
-      <c r="C13" s="1" t="inlineStr">
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
@@ -1041,59 +1093,57 @@
 Only successful applicants will be contacted; no individual feedback provided to unsuccessful applicants</t>
         </is>
       </c>
-      <c r="D13" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E13" s="1" t="inlineStr">
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F13" s="1" t="inlineStr">
+      <c r="F14" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-8th-call-for-proposals-small-size-grants-global-eba-fund-global-eba-fund-opg-26-00177</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="95" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Crossing the Divide Best Practices for Addressing Local and Privately-Owned Lateral Sewer Issues RFP 5419</t>
-        </is>
-      </c>
-      <c r="C14" s="1" t="inlineStr">
-        <is>
-          <t>Project Objective:
-To provide water resource recovery facilities (WRRFs) and collection system operators with an interactive manual of practice for implementing inflow and infiltration (I&amp;I) and obstruction management programs, focused on municipal and privately owned lateral sewers in complex legal, regulatory, and multi-jurisdictional environments.
+    <row r="15" ht="95" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Comparison of PFAS Contributions to Agricultural Systems</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>Project Objectives:
+Report per- and polyfluoroalkyl substance (PFAS) concentrations from a variety of agricultural inputs — animal manures, fertilizers, pesticides, composts, soil amendments, seed coatings, and biosolids-based products
+Compare the impact of various agricultural inputs on PFAS concentration in the soil profile over varying timeframes
+Evaluate the fate and transport of different inputs to PFAS contributions in agricultural systems at field-scale
+Determine relative contributions from biosolids-based products vs. other inputs to help develop/prioritize risk management strategies
  Background/Rationale:
-Wastewater utilities face continuing challenges providing cost-effective sewer services amid rising demand, urban redevelopment, and performance disruptors (root intrusion, pipe degradation, blockages). I&amp;I and obstruction management remain persistent, costly problems without a consolidated resource to guide program design. During wet weather, peak I&amp;I flows can increase influent flows 3–5x average. Studies suggest up to 80% of I&amp;I originates on private property, and root intrusions cause over 50% of sewer blockages globally. Program effectiveness varies widely depending on statutory authority, multi-jurisdictional overlap, enforcement mechanisms, and participant willingness.
- Central Research Questions:
-What I&amp;I and obstruction management practices are utilities using today, and how do they vary by jurisdictional/regulatory/infrastructure/environmental conditions?
-Which factors most influence successful implementation, and what barriers commonly derail programs?
-What measurable benefits (cost avoidance, capacity recovery, reduced spill risk, improved regulatory standing) have utilities realized from successful programs?
-This project extends WRF's ongoing "State-of-Practice Manual for Inflow and Infiltration Detection and Mitigation at Street and Private Lateral Levels" (Project 5365) into I&amp;I source control and obstruction management specifically.
- Research Approach (4 Tasks):
-Literature and Regulatory Review — Comprehensive review of legal authorities/regulations in the US and comparable international jurisdictions; catalog program elements, enforcement mechanisms, incentive structures, and legal/jurisdictional barriers
-Utility Survey and Case Study Development — Broad survey across utility size/geography/system type; select at least 5 diverse in-depth case studies with quantitative results (I&amp;I reduction %, reduced bypass pumping, reduced basement backups, cost savings, recovered capacity, reduced blockage-related spills/service calls)
-Utility Workshop — At least one invitation-only workshop with utility representatives to present survey findings and gather structured feedback on draft guidance content
-Interactive Manual of Practice — Development of a decision-support tool/web-based application/interactive PDF enabling utilities to select effective I&amp;I/obstruction program elements based on their statutory authority, jurisdictional complexity, and enforcement mechanisms
+Growing concern exists over human exposure to PFAS through biosolids land application on agricultural systems, with regulatory bans on biosolids land application enacted or proposed in at least 12 U.S. states. Utilities relying on land application for biosolids management are scrambling for alternative disposal pathways. The U.S. EPA's 2026 draft guidance noted its earlier 2025 draft risk assessment of PFOA/PFOS-contaminated sewage sludge lacked important contextual information (e.g., a national survey of PFOA/PFOS concentrations). Risk assessments have focused primarily on biosolids, with less attention to PFAS contributions from other sources — manures, compost, fertilizers, pesticides, seed coatings, irrigation water, farming practices, and atmospheric deposition. A Minnesota Pollution Control Agency review found 12 inert pesticide ingredients classified as PFAS. This project aims to improve understanding of PFAS risks from the wider range of agricultural inputs to support strategic resource allocation and inform policy amid surging fertilizer prices and shifts toward local circular resources.
+ Research Approach:
+Develop a baseline of knowledge on PFAS in biosolids and non-biosolids agricultural inputs via literature review, analytical methods evaluation, and examination of manufacturing/processing pathways; identify data gaps and uncertainties
+Measure/report compound-specific PFAS concentrations and profiles in agricultural inputs using standardized methods, including precursor characteristics for source attribution where possible
+Characterize PFAS contributions via literature review, data analysis, and field sampling — comparing soil profile/plant tissue composition between fields with non-biosolids inputs vs. biosolids-applied systems; study should test hypotheses on PFAS sources, transformation, retention, and mobility
+Optional additional focus areas: influence of soil/hydrologic/hydrochemistry conditions on PFAS behavior; degradation/transformation pathways; relative PFAS contributions across product lifecycle stages (manufacturing, bagging, delivery, etc.)
+Research approach should be hypothesis-driven, detailing specific end-user needs, and proposers are encouraged to leverage existing projects on PFAS plant uptake/fate/transport.
  Expected Deliverables:
-Research report (using WRF's Research Report Template) including literature/regulatory review
-Interactive manual of practice (following Technology Deliverables Guidance)
-In-depth utility survey, state-of-the-practice report, and at least 5 standalone case studies with quantitative results
-Summary documentation of the utility workshop, including feedback and how it was incorporated
- Project Duration: 24 months from contract start date (No-Cost Extension Policy caps extensions at 9 months beyond original schedule)
+Research report (WRF's Research Report Template) including: literature review, PFAS analysis of select products, risk management implications/prioritization recommendations, agriculture end-use guidance
+A webcast or workshop to share findings
+Optional additional deliverables: relative risk framework (mass input/fate/exposure/risk), decision support guide for farmers/regulators/utilities, plain language fact sheet, comparative PFAS mass input tool (spreadsheet/calculator)
+ Project Duration: 36 months from contract start date (longer than the other two WRF grants above, which were 24 months)
  Eligibility to Submit:
-Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible as named participants. Not open to individuals (same institutional-applicant structure as RFP 5424).
+Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible. Not open to individuals (same structure as the two prior WRF grants).
  Budget/Funding:
-Maximum WRF funding: $250,000
+Maximum WRF funding: $400,000 (the largest of the three WRF grants shared so far)
 Applicant must contribute at least 33% of the project award as additional resources (cost share, applicant in-kind, or third-party in-kind per 2 CFR Part 200.306)
 Proposals not meeting the 33% minimum match will not be accepted
  Proposal Evaluation Criteria:
@@ -1103,54 +1153,22 @@
 Communication Plan, Deliverables, and Applicability: 15 points
 Budget and Schedule: 15 points
  Compliance Standards: OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
- Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
-        </is>
-      </c>
-      <c r="D14" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E14" s="1" t="inlineStr">
+ Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00) — same deadline as the other two WRF grants</t>
+        </is>
+      </c>
+      <c r="D15" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E15" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F14" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-crossing-the-divide-best-practices-for-addressing-local-and-privately-owned-lateral-sewer-issues-rfp-5419-the-water-research-foundation-wrf-opg-26-00189</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="95" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="inlineStr">
-        <is>
-          <t>RFPs Invited for Arts-Integrated National School Projects Arts Education from Government-aided and Non-profit Schools in India</t>
-        </is>
-      </c>
-      <c r="C15" s="1" t="inlineStr">
-        <is>
-          <t>No description available</t>
-        </is>
-      </c>
-      <c r="D15" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E15" s="1" t="inlineStr">
-        <is>
-          <t>Oct 30, 2026</t>
-        </is>
-      </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/rfps/rfps-invited-for-arts-integrated-national-school-projects-arts-education-from-government-aided-and-non-profit-schools-in-india-india-foundation-for-the-arts-rfp-26-00385</t>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-comparison-of-pfas-contributions-to-agricultural-systems-the-water-research-foundation-wrf-opg-26-00190</t>
         </is>
       </c>
     </row>
@@ -1162,10 +1180,42 @@
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
+          <t>RFPs Invited for Arts-Integrated National School Projects Arts Education from Government-aided and Non-profit Schools in India</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t>No description available</t>
+        </is>
+      </c>
+      <c r="D16" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E16" s="1" t="inlineStr">
+        <is>
+          <t>Oct 30, 2026</t>
+        </is>
+      </c>
+      <c r="F16" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/rfps/rfps-invited-for-arts-integrated-national-school-projects-arts-education-from-government-aided-and-non-profit-schools-in-india-india-foundation-for-the-arts-rfp-26-00385</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="95" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
           <t>Applications Invited for CIFAR Global Scholars Program 20272029 Cohort</t>
         </is>
       </c>
-      <c r="C16" s="1" t="inlineStr">
+      <c r="C17" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 CIFAR is a Canadian-based globally influential research organization that convenes the world’s most brilliant people across disciplines to advance transformative knowledge and solve humanity’s biggest problems, together. By supporting long-term interdisciplinary collaboration, CIFAR provides researchers with an unparalleled environment of trust, transparency and knowledge sharing. Our time-tested model inspires new directions of inquiry, accelerates discovery and yields breakthroughs across borders and academic disciplines. Through knowledge mobilization, we are catalysts for change in industry, government and society. Through our 15 research programs and the Pan-Canadian AI Strategy, CIFAR convenes close to 400 of the world’s top researchers from 141 institutions in 20 countries. CIFAR is generously supported by the governments of Canada, Alberta and Québec, as well as foundations, individuals, corporations and Canadian and international partner organizations.
@@ -1209,34 +1259,34 @@
  Application Deadline: November 4, 2026, 12:00 PM EST</t>
         </is>
       </c>
-      <c r="D16" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E16" s="1" t="inlineStr">
+      <c r="D17" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="inlineStr">
         <is>
           <t>Nov 4, 2026</t>
         </is>
       </c>
-      <c r="F16" s="1" t="inlineStr">
+      <c r="F17" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-cifar-global-scholars-program-20272029-cohort-cifar-canadian-institute-for-advanced-research-opg-26-00183</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="95" customHeight="1">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B17" s="1" t="inlineStr">
+    <row r="18" ht="95" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Regular Grant Programme 2026-27</t>
         </is>
       </c>
-      <c r="C17" s="1" t="inlineStr">
+      <c r="C18" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 World Cancer Research Fund examines how diet, weight and physical activity affect your risk of developing and surviving cancer. As part of an international network of charities, we have been funding life-saving research, influencing global public health policy and educating the public since 1982.
@@ -1264,34 +1314,34 @@
 Final funding decisions (after Board approval) End of September 2027</t>
         </is>
       </c>
-      <c r="D17" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E17" s="1" t="inlineStr">
+      <c r="D18" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E18" s="1" t="inlineStr">
         <is>
           <t>Nov 13, 2026</t>
         </is>
       </c>
-      <c r="F17" s="1" t="inlineStr">
+      <c r="F18" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-regular-grant-programme-2026-27-world-cancer-research-fund-opg-26-00196</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="95" customHeight="1">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="inlineStr">
+    <row r="19" ht="95" customHeight="1">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for IWRS Teaching Innovation Award</t>
         </is>
       </c>
-      <c r="C18" s="1" t="inlineStr">
+      <c r="C19" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Insects are one of the most numerous and diverse animal groups on Earth. Still, we understand very little about how to measure their welfare. Insects are managed in many contexts that may present welfare concerns: as ‘mini-livestock’ farmed for food and feed, in waste management, as agricultural pests or invasive species, in research and educational settings, for medical purposes, as targets of conservation actions, and more. Scientific research is urgently needed to understand how to factor the welfare needs of individual insects into policy and practice. The Insect Welfare Research Society is an academic-led research society founded in March 2023. The society aims to support 1) the global insect welfare research community and 2) the incorporation of evidence-based information on insect welfare into policy and practice by relevant stakeholders. We also support welfare research on both terrestrial invertebrates (e.g., spiders and other arachnids, myriapods like millipedes, gastropod molluscs, etc.) and aquatic invertebrates (e.g., shrimp/prawns, horseshoe crabs, cephalopod molluscs, etc.). Support for founding the IWRS was provided by Open Philanthropy. The IWRS’s is a 501(c)3 nonprofit incorporated in the State of Delaware. Our EIN is 93-3393218. All work is independently conducted by the IWRS.
@@ -1303,34 +1353,34 @@
 Two awards of $2,000 USD are available annually.</t>
         </is>
       </c>
-      <c r="D18" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E18" s="1" t="inlineStr">
+      <c r="D19" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E19" s="1" t="inlineStr">
         <is>
           <t>Nov 15, 2026</t>
         </is>
       </c>
-      <c r="F18" s="1" t="inlineStr">
+      <c r="F19" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00169</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="95" customHeight="1">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="inlineStr">
+    <row r="20" ht="95" customHeight="1">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for IWRS Teaching Innovation Award</t>
         </is>
       </c>
-      <c r="C19" s="1" t="inlineStr">
+      <c r="C20" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 Insects are one of the most numerous and diverse animal groups on Earth.
@@ -1345,103 +1395,19 @@
 IWRS staff and Advisory Group members are not eligible to apply.</t>
         </is>
       </c>
-      <c r="D19" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E19" s="1" t="inlineStr">
+      <c r="D20" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E20" s="1" t="inlineStr">
         <is>
           <t>Nov 15, 2026</t>
         </is>
       </c>
-      <c r="F19" s="1" t="inlineStr">
+      <c r="F20" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-iwrs-teaching-innovation-award-insect-welfare-research-society-opg-26-00166</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="95" customHeight="1">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Medium-Size Grants Call for Proposals Global EbA Fund</t>
-        </is>
-      </c>
-      <c r="C20" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
- About the Opportunity:
-The Global EbA Fund invites proposals under its General Track: Strategic Scaling and Global Influence, seeking collaborative and innovative approaches to advancing Ecosystem-based Adaptation (EbA) by addressing systemic barriers to scalability and contributing to global learning and policy dialogue. Initiatives should strengthen enabling environments and embed EbA into national frameworks that unify climate, biodiversity, land, and development priorities. Alignment with one of three priority topics is welcomed but not mandatory:
- Priority Topics:
-I. Innovative Finance Solutions for EbA — partnerships with private sector actors (financiers, innovators, local champions) to unlock private capital/blended finance for EbA, evolving EbA into profitable, scalable business models
-II. EbA for Human Development and Security — integrating EbA into national/international security frameworks for fragile and conflict-affected contexts; community co-designed interventions that reduce natural resource-related tensions and climate-induced fragility, bridging adaptation, humanitarian, development, and peacebuilding agendas
-III. Interlinkages for People-Nature-Climate-Land Synergies — strengthening operational links across the Rio Conventions (UNFCCC, CBD, UNCCD) and frameworks like the Sendai Framework on DRR, using EbA as the anchor connecting biodiversity, sustainable land management, climate adaptation, and disaster risk reduction
- Grant Size: Up to USD 500,000 per grant
- Project Duration: Up to 24 months
- Eligible Applicant Types:
-Non-governmental organisations (NGOs)
-International NGOs (INGOs)
-Intergovernmental organisations (IGOs)
-Community-based organisations (CBOs)
-Indigenous People's Organisations
-Universities and academic institutions
-Research institutes and think tanks
-Private sector companies (under certain conditions)
-Consortia (must designate a clear lead "Applicant Organisation"; government entities may join but cannot receive Fund money directly)
-Note: Individuals are not eligible; UNEP and IUCN offices are also not eligible.
- Key Eligibility Criteria:
-Must qualify as Ecosystem-based Adaptation (EbA) per the Fund's Qualification Criteria &amp; Quality Standards
-Must show catalytic/innovative potential
-Must clearly identify climate impacts addressed
-Falls under max 1 Strategic Objective and max 2 Action Pillars of the Fund
-Global, thematic, or targets only ODA-eligible countries
-Budget up to USD 500,000; duration ≤24 months
-Must build on existing work (not standalone/field-implementation-only)
-Must show sustainability post-funding
-Must partner with local institutions
-Applicant &amp; partners must be legally recognized entities with relevant experience
-Must comply with Due Diligence requirements
- Evaluation Criteria (weighted):
-Ecosystem-based Adaptation (EbA) approach — 30%
-Design &amp; Methodology (Theory of Change, logframe, SMART indicators, budget coherence)
-Gender &amp; Social Inclusion (participatory approach, FPIC for Indigenous Peoples' impact)
-Innovative &amp; Catalytic Contribution — 30%
-Sustainability — 20%
-Institutional Arrangements — 20%
- Reporting Requirement: 
-Applicants must identify at least 3 indicators from the Fund's Core Indicator Framework for their project's logframe.
- Application Package Required:
-Applicant Declaration
-Co-applicant Mandate (if applicable)
-Medium-Size Grants Application Form
-Project Proposal Budget Template
-Due Diligence and Financial Capacity Questionnaire (with Annexes 1(c)(i) and 1(c)(ii) at submission stage)
- Application Language: English only (organizational documents must be translated to English)
- Timeline:
-Call officially launched: August 24, 2026
-Submission window: October 12 – November 16, 2026
-Applications submitted via online portal (link shared on the Medium-Size Grants webpage from Oct 12)</t>
-        </is>
-      </c>
-      <c r="D20" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E20" s="1" t="inlineStr">
-        <is>
-          <t>Nov 16, 2026</t>
-        </is>
-      </c>
-      <c r="F20" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-medium-size-grants-call-for-proposals-global-eba-fund-global-eba-fund-opg-26-00178</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update Combined.xlsx [Sat Oct 10 08:01:48 UTC 2026]
</commit_message>
<xml_diff>
--- a/output/Combined.xlsx
+++ b/output/Combined.xlsx
@@ -894,75 +894,10 @@
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
-          <t>Applications Invited for Crossing the Divide Best Practices for Addressing Local and Privately-Owned Lateral Sewer Issues RFP 5419</t>
+          <t>Applications Invited for Adaptive Control Frameworks to Unlock Full-Scale BNR Potential Water Research Foundation WRF</t>
         </is>
       </c>
       <c r="C12" s="1" t="inlineStr">
-        <is>
-          <t>Project Objective:
-To provide water resource recovery facilities (WRRFs) and collection system operators with an interactive manual of practice for implementing inflow and infiltration (I&amp;I) and obstruction management programs, focused on municipal and privately owned lateral sewers in complex legal, regulatory, and multi-jurisdictional environments.
- Background/Rationale:
-Wastewater utilities face continuing challenges providing cost-effective sewer services amid rising demand, urban redevelopment, and performance disruptors (root intrusion, pipe degradation, blockages). I&amp;I and obstruction management remain persistent, costly problems without a consolidated resource to guide program design. During wet weather, peak I&amp;I flows can increase influent flows 3–5x average. Studies suggest up to 80% of I&amp;I originates on private property, and root intrusions cause over 50% of sewer blockages globally. Program effectiveness varies widely depending on statutory authority, multi-jurisdictional overlap, enforcement mechanisms, and participant willingness.
- Central Research Questions:
-What I&amp;I and obstruction management practices are utilities using today, and how do they vary by jurisdictional/regulatory/infrastructure/environmental conditions?
-Which factors most influence successful implementation, and what barriers commonly derail programs?
-What measurable benefits (cost avoidance, capacity recovery, reduced spill risk, improved regulatory standing) have utilities realized from successful programs?
-This project extends WRF's ongoing "State-of-Practice Manual for Inflow and Infiltration Detection and Mitigation at Street and Private Lateral Levels" (Project 5365) into I&amp;I source control and obstruction management specifically.
- Research Approach (4 Tasks):
-Literature and Regulatory Review — Comprehensive review of legal authorities/regulations in the US and comparable international jurisdictions; catalog program elements, enforcement mechanisms, incentive structures, and legal/jurisdictional barriers
-Utility Survey and Case Study Development — Broad survey across utility size/geography/system type; select at least 5 diverse in-depth case studies with quantitative results (I&amp;I reduction %, reduced bypass pumping, reduced basement backups, cost savings, recovered capacity, reduced blockage-related spills/service calls)
-Utility Workshop — At least one invitation-only workshop with utility representatives to present survey findings and gather structured feedback on draft guidance content
-Interactive Manual of Practice — Development of a decision-support tool/web-based application/interactive PDF enabling utilities to select effective I&amp;I/obstruction program elements based on their statutory authority, jurisdictional complexity, and enforcement mechanisms
- Expected Deliverables:
-Research report (using WRF's Research Report Template) including literature/regulatory review
-Interactive manual of practice (following Technology Deliverables Guidance)
-In-depth utility survey, state-of-the-practice report, and at least 5 standalone case studies with quantitative results
-Summary documentation of the utility workshop, including feedback and how it was incorporated
- Project Duration: 24 months from contract start date (No-Cost Extension Policy caps extensions at 9 months beyond original schedule)
- Eligibility to Submit:
-Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible as named participants. Not open to individuals (same institutional-applicant structure as RFP 5424).
- Budget/Funding:
-Maximum WRF funding: $250,000
-Applicant must contribute at least 33% of the project award as additional resources (cost share, applicant in-kind, or third-party in-kind per 2 CFR Part 200.306)
-Proposals not meeting the 33% minimum match will not be accepted
- Proposal Evaluation Criteria:
-Understanding the Problem and Responsiveness to RFP: 20 points
-Technical and Scientific Merit: 30 points
-Qualifications, Capabilities, and Management: 20 points
-Communication Plan, Deliverables, and Applicability: 15 points
-Budget and Schedule: 15 points
- Compliance Standards: OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
- Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
-        </is>
-      </c>
-      <c r="D12" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E12" s="1" t="inlineStr">
-        <is>
-          <t>Oct 26, 2026</t>
-        </is>
-      </c>
-      <c r="F12" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-crossing-the-divide-best-practices-for-addressing-local-and-privately-owned-lateral-sewer-issues-rfp-5419-the-water-research-foundation-wrf-opg-26-00189</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="95" customHeight="1">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B13" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for Adaptive Control Frameworks to Unlock Full-Scale BNR Potential Water Research Foundation WRF</t>
-        </is>
-      </c>
-      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>About the Organization
 The Water Research Foundation (WRF) is the leading research organization advancing the science of all water to meet the evolving needs of its subscribers and the water sector. WRF is a nonprofit, charitable and educational organization which funds, manages, and publishes research on the technology, operation, and management of drinking water, wastewater, reuse, and stormwater collection, treatment and supply systems—all in pursuit of ensuring water quality and improving water services to the public.
@@ -1003,124 +938,34 @@
 Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
         </is>
       </c>
-      <c r="D13" s="1" t="inlineStr">
+      <c r="D12" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="E13" s="1" t="inlineStr">
+      <c r="E12" s="1" t="inlineStr">
         <is>
           <t>Oct 26, 2026</t>
         </is>
       </c>
-      <c r="F13" s="1" t="inlineStr">
+      <c r="F12" s="1" t="inlineStr">
         <is>
           <t>https://onepurpos.in/openings/grants/applications-invited-for-adaptive-control-frameworks-to-unlock-full-scale-bnr-potential-water-research-foundation-wrf-the-water-research-foundation-wrf-opg-26-00187</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="95" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="inlineStr">
-        <is>
-          <t>Applications Invited for 8th Call for Proposals Small-Size Grants Global EbA Fund</t>
-        </is>
-      </c>
-      <c r="C14" s="1" t="inlineStr">
-        <is>
-          <t>About the Organization
-The Global EbA Fund is a funding mechanism for supporting innovative approaches to Ecosystem-based Adaptation (EbA). Led by IUCN and UNEP, the IKI-supported Fund is structured to support catalytic initiatives to help to overcome identified barriers to upscaling EbA. Furthermore, it is expected that the Fund will address the gaps in knowledge and planning for EbA, as well as to increase access to public and private funding for catalytic adaptation interventions. The Fund will prioritize filling in resourcing and knowledge gaps with a broad thematic focus on innovation and urgency, thus encouraging creative solutions and partnerships among funding applicants and the wider EbA community. By supporting catalytic interventions, the Fund will address research gaps, pilot innovative EbA approaches, engage in strategic EbA policy mainstreaming, and incentivise innovative finance mechanisms and private sector EbA investment.
- About the Opportunity:
-The Global EbA Fund invites innovative and catalytic proposals that address systemic barriers to Ecosystem-based Adaptation (EbA) scaling — by enhancing institutional and technical capacities, quality data/evidence generation, learning networks, and investment readiness. Aligned with the IKI Strategy up to 2030 (focus on socio-ecological transformation), the Fund's primary geographic focus is ODA-eligible SIDS (Small Island Developing States) and LDCs (Least Developed Countries), though other ODA-eligible countries may be considered where proposals show exceptional ambition.
- Focus Areas:
-Overcoming upstream barriers to EbA uptake/scaling (institutional &amp; technical capacity constraints, evidence generation, knowledge exchange)
-Clear adaptation chain grounded in detailed impact chain analysis (climate hazards/risks, socioeconomic/ecological sensitivity, adaptive capacity)
-Social and environmental considerations (gender responsiveness, Indigenous Peoples' rights, local participation, environmental/social safeguards, prevention of maladaptation)
-Robust sustainability and exit strategies (long-term viability, local ownership, institutional continuity)
- Encouraged Topics:
-Investment readiness and project pipeline preparation
-Innovative technologies for EbA
-Applied and functional research
-Synergies with other EbA/Nature-based Solution (NbS) initiatives
- Grant Size: Up to USD 250,000 per grant
- Project Duration: Up to 24 months
- Eligible Applicant Types:
-Non-governmental organisations (NGOs)
-International NGOs (INGOs)
-Intergovernmental organisations (IGOs)
-Community-based organisations (CBOs)
-Indigenous People's Organisations
-Universities and academic institutions
-Research institutes and think tanks
-Private sector companies (under certain conditions; no funding for sector-specific obligations, compensatory measures, or for-profit activities)
-Consortia (must designate a clear lead "Applicant Organisation"; government entities can join a consortium but cannot receive Fund money directly)
-Note: Individuals are not eligible (e.g., no PhD study funding); UNEP and IUCN offices are also not eligible to apply.
- Key Eligibility Criteria:
-Must qualify as Ecosystem-based Adaptation (EbA) per the Fund's Qualification Criteria &amp; Quality Standards
-Must have catalytic/innovative potential
-Must clearly identify climate impacts addressed
-Falls under max 1 Strategic Objective and max 2 Action Pillars of the Fund
-Global, thematic, or targets only ODA-eligible countries
-Budget up to USD 250,000; duration up to 24 months
-Must build on existing work (not standalone/field-implementation-only projects)
-Must show sustainability post-funding
-Must partner with local institutions
-Applicant &amp; partners must be legally recognized entities with relevant experience
-Must complete Due Diligence requirements
- Evaluation Criteria (weighted):
-Ecosystem-based Adaptation (EbA) approach — 30%
-Design &amp; Methodology (Theory of Change, logframe, SMART indicators, budget coherence)
-Gender &amp; Social Inclusion (participatory approach, FPIC for Indigenous Peoples' impact)
-Innovative &amp; Catalytic Contribution — 30%
-Sustainability — 20%
-Institutional Arrangements — 20%
- Reporting Requirement: Applicants must identify at least 3 indicators from the Fund's Core Indicator Framework for their project's logframe.
- Application Package Required:
-Applicant Declaration
-Co-applicant Mandate (if applicable)
-Small-Size Grants Application Form
-Project Proposal Budget Template
-Due Diligence and Financial Capacity Questionnaire (with Annexes 1(c)(i) and 1(c)(ii) at submission stage)
- Application Language: English only (organizational documents must be translated to English
- Timeline:
-Call officially launched: August 24, 2026
-Submission window: September 28 – October 26, 2026
-Applications submitted via online portal (link shared on the Small-Size Grants webpage from Sept 28)
-Only successful applicants will be contacted; no individual feedback provided to unsuccessful applicants</t>
-        </is>
-      </c>
-      <c r="D14" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E14" s="1" t="inlineStr">
-        <is>
-          <t>Oct 26, 2026</t>
-        </is>
-      </c>
-      <c r="F14" s="1" t="inlineStr">
-        <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-8th-call-for-proposals-small-size-grants-global-eba-fund-global-eba-fund-opg-26-00177</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="95" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>onepurpos</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="inlineStr">
+    <row r="13" ht="95" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
         <is>
           <t>Applications Invited for Comparison of PFAS Contributions to Agricultural Systems</t>
         </is>
       </c>
-      <c r="C15" s="1" t="inlineStr">
+      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>Project Objectives:
 Report per- and polyfluoroalkyl substance (PFAS) concentrations from a variety of agricultural inputs — animal manures, fertilizers, pesticides, composts, soil amendments, seed coatings, and biosolids-based products
@@ -1156,6 +1001,103 @@
  Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00) — same deadline as the other two WRF grants</t>
         </is>
       </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>Oct 26, 2026</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-comparison-of-pfas-contributions-to-agricultural-systems-the-water-research-foundation-wrf-opg-26-00190</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="95" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>Applications Invited for Crossing the Divide Best Practices for Addressing Local and Privately-Owned Lateral Sewer Issues RFP 5419</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>Project Objective:
+To provide water resource recovery facilities (WRRFs) and collection system operators with an interactive manual of practice for implementing inflow and infiltration (I&amp;I) and obstruction management programs, focused on municipal and privately owned lateral sewers in complex legal, regulatory, and multi-jurisdictional environments.
+ Background/Rationale:
+Wastewater utilities face continuing challenges providing cost-effective sewer services amid rising demand, urban redevelopment, and performance disruptors (root intrusion, pipe degradation, blockages). I&amp;I and obstruction management remain persistent, costly problems without a consolidated resource to guide program design. During wet weather, peak I&amp;I flows can increase influent flows 3–5x average. Studies suggest up to 80% of I&amp;I originates on private property, and root intrusions cause over 50% of sewer blockages globally. Program effectiveness varies widely depending on statutory authority, multi-jurisdictional overlap, enforcement mechanisms, and participant willingness.
+ Central Research Questions:
+What I&amp;I and obstruction management practices are utilities using today, and how do they vary by jurisdictional/regulatory/infrastructure/environmental conditions?
+Which factors most influence successful implementation, and what barriers commonly derail programs?
+What measurable benefits (cost avoidance, capacity recovery, reduced spill risk, improved regulatory standing) have utilities realized from successful programs?
+This project extends WRF's ongoing "State-of-Practice Manual for Inflow and Infiltration Detection and Mitigation at Street and Private Lateral Levels" (Project 5365) into I&amp;I source control and obstruction management specifically.
+ Research Approach (4 Tasks):
+Literature and Regulatory Review — Comprehensive review of legal authorities/regulations in the US and comparable international jurisdictions; catalog program elements, enforcement mechanisms, incentive structures, and legal/jurisdictional barriers
+Utility Survey and Case Study Development — Broad survey across utility size/geography/system type; select at least 5 diverse in-depth case studies with quantitative results (I&amp;I reduction %, reduced bypass pumping, reduced basement backups, cost savings, recovered capacity, reduced blockage-related spills/service calls)
+Utility Workshop — At least one invitation-only workshop with utility representatives to present survey findings and gather structured feedback on draft guidance content
+Interactive Manual of Practice — Development of a decision-support tool/web-based application/interactive PDF enabling utilities to select effective I&amp;I/obstruction program elements based on their statutory authority, jurisdictional complexity, and enforcement mechanisms
+ Expected Deliverables:
+Research report (using WRF's Research Report Template) including literature/regulatory review
+Interactive manual of practice (following Technology Deliverables Guidance)
+In-depth utility survey, state-of-the-practice report, and at least 5 standalone case studies with quantitative results
+Summary documentation of the utility workshop, including feedback and how it was incorporated
+ Project Duration: 24 months from contract start date (No-Cost Extension Policy caps extensions at 9 months beyond original schedule)
+ Eligibility to Submit:
+Open to both U.S.-based and non-U.S.-based entities — educational institutions, research organizations, governmental agencies, consultants, or for-profit entities. Researchers late on any ongoing WRF-sponsored studies (without approved no-cost extensions) are not eligible as named participants. Not open to individuals (same institutional-applicant structure as RFP 5424).
+ Budget/Funding:
+Maximum WRF funding: $250,000
+Applicant must contribute at least 33% of the project award as additional resources (cost share, applicant in-kind, or third-party in-kind per 2 CFR Part 200.306)
+Proposals not meeting the 33% minimum match will not be accepted
+ Proposal Evaluation Criteria:
+Understanding the Problem and Responsiveness to RFP: 20 points
+Technical and Scientific Merit: 30 points
+Qualifications, Capabilities, and Management: 20 points
+Communication Plan, Deliverables, and Applicability: 15 points
+Budget and Schedule: 15 points
+ Compliance Standards: OMB Uniform Grants Guidance (2 CFR Part 200) and 48 CFR 31.2 for commercial organizations
+ Application Deadline: October 26, 2026, 3:00 PM Mountain Time (GMT-07:00)</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>Oct 26, 2026</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr">
+        <is>
+          <t>https://onepurpos.in/openings/grants/applications-invited-for-crossing-the-divide-best-practices-for-addressing-local-and-privately-owned-lateral-sewer-issues-rfp-5419-the-water-research-foundation-wrf-opg-26-00189</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="95" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>onepurpos</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>RFPs Invited for Arts-Integrated National School Projects Arts Education from Government-aided and Non-profit Schools in India</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>No description available</t>
+        </is>
+      </c>
       <c r="D15" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
@@ -1163,12 +1105,12 @@
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>Oct 26, 2026</t>
+          <t>Oct 30, 2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://onepurpos.in/openings/grants/applications-invited-for-comparison-of-pfas-contributions-to-agricultural-systems-the-water-research-foundation-wrf-opg-26-00190</t>
+          <t>https://onepurpos.in/openings/rfps/rfps-invited-for-arts-integrated-national-school-projects-arts-education-from-government-aided-and-non-profit-schools-in-india-india-foundation-for-the-arts-rfp-26-00385</t>
 